<commit_message>
docs(testing): mark TC-BUILD-08 as passed from CI run
Mobile CI on frontend PR #27 succeeded, including the new Android
debug APK build step.

Refs: adhoc-20261007-android-desugaring

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -19,8 +19,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -127,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -135,7 +135,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -183,6 +183,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -908,7 +911,7 @@
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="21" t="n">
         <v>46303</v>
       </c>
     </row>
@@ -1517,7 +1520,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="74" customHeight="1">
+    <row r="16" ht="90.5" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>TC-BUILD-08</t>
@@ -1549,19 +1552,23 @@
           <t>Mọi bước xanh, gồm "Build Android APK (debug)"</t>
         </is>
       </c>
-      <c r="G16" s="8" t="inlineStr"/>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>PR frontend #27, run 37658903070 trên e897a56: conclusion=success; mọi bước success, gồm "Build Android APK (debug)" (✓ Built build/app/outputs/flutter-apk/app-debug.apk), thời gian job 5m44s</t>
+        </is>
+      </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>AC5 · manual · cần push nhánh và mở PR</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="74" customHeight="1">
+          <t>AC5 · manual (GitHub Actions) · evidence/ci-pr27.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="173" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
           <t>TC-BUILD-09</t>
@@ -1601,7 +1608,7 @@
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>Error Guessing · manual · máy implement dùng Flutter master cũ hơn (Dart 3.12) nên không kiểm được</t>
+          <t>Error Guessing · manual · máy implement dùng Flutter master cũ hơn (Dart 3.12) nên không kiểm được. Bằng chứng gián tiếp: CI PR #27 (Flutter stable 3.x) chạy flutter pub get báo "Got dependencies!", không đổi phụ thuộc nào (evidence/ci-pr27.log); chưa chạy đúng --enforce-lockfile</t>
         </is>
       </c>
     </row>
@@ -1837,7 +1844,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="123.5" customHeight="1">
+    <row r="11" ht="156.5" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Build ứng dụng Android</t>
@@ -1872,7 +1879,7 @@
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>Lỗi Critical (APK không build được do flutter_local_notifications cần desugaring và flutter_timezone 2.x dùng API Registrar đã bị gỡ) đã sửa ở task adhoc-20261007-android-desugaring. Còn Pending: CI chạy trên PR và kiểm lockfile bằng Flutter stable của team.</t>
+          <t>Lỗi Critical (APK không build được do flutter_local_notifications cần desugaring và flutter_timezone 2.x dùng API Registrar đã bị gỡ) đã sửa ở task adhoc-20261007-android-desugaring (frontend PR #27, CI xanh gồm bước build APK). Còn Pending: kiểm lockfile bằng --enforce-lockfile với Flutter stable.</t>
         </is>
       </c>
       <c r="I11" s="11" t="inlineStr">

</xml_diff>

<commit_message>
test(qa): add catalog CRUD test cases
Refs: 2.13
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -7,10 +7,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android build" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog CRUD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Android build'!$A$8:$I$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalog CRUD'!$A$8:$I$29</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -127,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -187,6 +189,9 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -346,12 +351,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11</f>
+              <f>'Report'!$A$11:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$11</f>
+              <f>'Report'!$D$11:$D$12</f>
             </numRef>
           </val>
         </ser>
@@ -370,12 +375,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11</f>
+              <f>'Report'!$A$11:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$11</f>
+              <f>'Report'!$E$11:$E$12</f>
             </numRef>
           </val>
         </ser>
@@ -394,12 +399,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11</f>
+              <f>'Report'!$A$11:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$11</f>
+              <f>'Report'!$F$11:$F$12</f>
             </numRef>
           </val>
         </ser>
@@ -480,7 +485,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$3:$D$4</f>
+              <f>'Report'!$E$3:$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -502,7 +507,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>13</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -524,7 +529,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>13</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3240000"/>
@@ -1680,7 +1685,1433 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:T35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Admin Medication Catalog CRUD (CATCRUD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46303</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Quyền gọi Admin Medication CRUD</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="57.5" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối người chưa đăng nhập trên toàn bộ endpoint CRUD</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Không gửi danh tính xác thực.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Lần lượt gọi POST, GET danh sách, GET chi tiết, PATCH và DELETE /admin/medications.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>med_id=1; name=Panadol</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi request trả 401.</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Năm trường hợp tham số hóa đều trả 401.</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · Decision Table (R1) · test_admin_endpoints_require_auth_401</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>vai trò</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>admin đã xác thực</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>không có danh tính
+user is_admin=false</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>6
+7</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Có danh tính?</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="57.5" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối user không phải admin trên toàn bộ endpoint CRUD</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>User đã xác thực với is_admin=false.</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Lần lượt gọi năm endpoint Admin Medication CRUD.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>med_id=1; name=Panadol</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi request trả 403 và {"detail":"Admin only"}.</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Năm trường hợp đều trả 403 và đúng detail.</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · Decision Table (R2) · test_admin_endpoints_reject_non_admin_403</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>độ dài 1..255</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>rỗng
+dài hơn 255 ký tự</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>8
+9</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>is_admin?</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="57.5" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Tạo thuốc với payload hợp lệ</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực; repository trả thuốc id=101.</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi POST /admin/medications với đầy đủ thông tin thuốc.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>name=Paracetamol 500mg; source=dav_drugbank; source_ref=VN-12345-20</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Trả 201 và dữ liệu thuốc id=101.</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Trả 201; id, name và source_ref đúng.</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · EP (1,1) · Decision Table (R3) · test_create_medication_success</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>source/source_ref</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>cùng có giá trị
+cùng null</t>
+        </is>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>3
+4</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>chỉ có source
+chỉ có source_ref</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>10
+11</t>
+        </is>
+      </c>
+      <c r="Q11" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T11" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="57.5" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-BVA-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối tên thuốc rỗng</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực.</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi POST /admin/medications.
+2. Xác minh repository không được khởi tạo.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>name=(blank)</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Trả 422; không ghi repository.</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Trả 422; SqlCatalog không được gọi.</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (2) · BVA (min-1) · test_create_validation_empty_name_rejected</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>med_id</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>thuốc đang hoạt động</t>
+        </is>
+      </c>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N12" s="10" t="inlineStr">
+        <is>
+          <t>không tồn tại hoặc đã xóa mềm</t>
+        </is>
+      </c>
+      <c r="O12" s="10" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S12" s="11" t="inlineStr"/>
+      <c r="T12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13" ht="41" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-BVA-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Chấp nhận tên thuốc dài một ký tự</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực.</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi POST /admin/medications.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>name=A</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Trả 201 nếu repository tạo thành công.</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr"/>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · EP (1) · BVA (min) · manual</t>
+        </is>
+      </c>
+      <c r="Q13" s="10" t="inlineStr">
+        <is>
+          <t>403 Admin only</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="inlineStr"/>
+      <c r="S13" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="41" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-BVA-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Chấp nhận tên thuốc dài 255 ký tự</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực.</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi POST /admin/medications.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>name=a*255</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Trả 201 nếu repository tạo thành công.</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr"/>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · EP (1) · BVA (max) · manual</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>Cho phép xử lý CRUD</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr"/>
+      <c r="S14" s="11" t="inlineStr"/>
+      <c r="T14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="41" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-BVA-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối tên thuốc dài 256 ký tự</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực.</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi POST /admin/medications.
+2. Xác minh repository không ghi dữ liệu.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>name=a*256</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Trả 422; không ghi repository.</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (2) · BVA (max+1) · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="57.5" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối payload chỉ có source</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực.</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi POST /admin/medications.
+2. Xác minh repository không được khởi tạo.</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>name=Paracetamol 500mg; source=dav_drugbank; source_ref=null</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Trả 422; không ghi repository.</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Trả 422; SqlCatalog không được gọi.</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (3) · test_create_validation_source_pair_enforced</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="41" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối payload chỉ có source_ref</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực.</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi POST /admin/medications.
+2. Xác minh repository không được khởi tạo.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>name=Paracetamol 500mg; source=null; source_ref=REF-001</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Trả 422; không ghi repository.</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Trả 422; SqlCatalog không được gọi.</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (4) · test_create_validation_source_pair_enforced</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="57.5" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Liệt kê thuốc theo từ khóa và phân trang</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực; repository có một thuốc Amlodipin đang hoạt động.</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi GET /admin/medications?q=amlo&amp;skip=0&amp;limit=10.
+2. Đối chiếu tham số repository.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>q=amlo; skip=0; limit=10</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Trả 200, total=1, đúng item; repository nhận amlo, 0, 10.</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Trả đúng dữ liệu và repository nhận đúng tham số.</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · EP (1) · test_list_medications_pagination_and_query</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="41" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-BVA-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối limit bằng 0</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực.</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi GET /admin/medications?limit=0.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>limit=0</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Trả 422.</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr"/>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · BVA (min-1) · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="41" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-BVA-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Chấp nhận limit bằng 1</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực.</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi GET /admin/medications?limit=1.</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>limit=1</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Trả 200 và tối đa một item.</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr"/>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · BVA (min) · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="41" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-BVA-13</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Chấp nhận limit bằng 100</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực.</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi GET /admin/medications?limit=100.</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>limit=100</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Trả 200 và tối đa 100 item.</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr"/>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · BVA (max) · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="41" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-BVA-14</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối limit bằng 101</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực.</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi GET /admin/medications?limit=101.</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>limit=101</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Trả 422.</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr"/>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · BVA (max+1) · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="41" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Lấy chi tiết thuốc đang hoạt động</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực; thuốc id=42 đang hoạt động.</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi GET /admin/medications/42.</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>med_id=42</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Trả 200 với thuốc id=42.</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Trả 200 với Berberin id=42.</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (1) · test_get_medication_detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="41" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-16</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Trả 404 khi lấy thuốc không tồn tại</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực; repository không tìm thấy thuốc.</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi GET /admin/medications/999.</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>med_id=999</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Trả 404 với Medication not found.</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Trả 404 với đúng detail.</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (2) · test_get_medication_not_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="41" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-17</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Cập nhật thuốc đang hoạt động</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực; thuốc id=42 đang hoạt động.</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi PATCH /admin/medications/42.</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>name=Berberin 100mg</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Trả 200 với tên đã cập nhật.</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Trả 200 với name=Berberin 100mg.</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (1) · test_update_medication_success</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="41" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-18</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Trả 404 khi cập nhật thuốc không tồn tại</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực; repository không tìm thấy thuốc.</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi PATCH /admin/medications/999.</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>name=Unknown</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Trả 404 với Medication not found.</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Trả 404 với đúng detail.</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (2) · test_update_medication_not_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="41" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-19</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Xóa mềm thuốc đang hoạt động</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực; thuốc id=42 đang hoạt động.</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi DELETE /admin/medications/42.
+2. Đối chiếu lời gọi repository.</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>med_id=42</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Trả 204 không body; repository soft_delete id=42.</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Trả 204 không body; repository nhận id=42.</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · EP (1) · test_delete_medication_soft_delete</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="57.5" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-20</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Trả 404 khi xóa thuốc không tồn tại hoặc đã xóa mềm</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Admin đã xác thực; repository báo không xóa được thuốc id=42.</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi DELETE /admin/medications/42.</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>med_id=42</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Trả 404 với Medication not found.</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Trả 404 với đúng detail.</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · EP (2) · test_delete_medication_soft_delete</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="41" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATCRUD-21</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Chạy toàn bộ unit và architecture test backend</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Backend ở nhánh feat/2.13 với dependency đã cài.</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy pytest tests/unit tests/architecture.</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>380 tests</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Tất cả test pass.</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>380 pass; catalog 19/19 và architecture 11/11 pass.</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · Error Guessing · pytest tests/unit tests/architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32">
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H32" s="13">
+        <f>COUNTIF(H9:H29,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H33" s="13">
+        <f>COUNTIF(H9:H29,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="G34" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H34" s="13">
+        <f>COUNTIF(H9:H29,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H35" s="13">
+        <f>SUM(H32:H34)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I29"/>
+  <conditionalFormatting sqref="H9:H29">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1709,6 +3140,11 @@
       </c>
       <c r="D2" s="15" t="inlineStr">
         <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
@@ -1728,8 +3164,12 @@
         <f>'Android build'!$H$20</f>
         <v/>
       </c>
-      <c r="D3" s="15">
-        <f>SUM(C3:C3)</f>
+      <c r="D3" s="11">
+        <f>'Catalog CRUD'!$H$32</f>
+        <v/>
+      </c>
+      <c r="E3" s="15">
+        <f>SUM(C3:D3)</f>
         <v/>
       </c>
     </row>
@@ -1744,8 +3184,12 @@
         <f>'Android build'!$H$21</f>
         <v/>
       </c>
-      <c r="D4" s="15">
-        <f>SUM(C4:C4)</f>
+      <c r="D4" s="11">
+        <f>'Catalog CRUD'!$H$33</f>
+        <v/>
+      </c>
+      <c r="E4" s="15">
+        <f>SUM(C4:D4)</f>
         <v/>
       </c>
     </row>
@@ -1760,8 +3204,12 @@
         <f>C3+C4</f>
         <v/>
       </c>
-      <c r="D5" s="15">
-        <f>SUM(C5:C5)</f>
+      <c r="D5" s="11">
+        <f>D3+D4</f>
+        <v/>
+      </c>
+      <c r="E5" s="15">
+        <f>SUM(C5:D5)</f>
         <v/>
       </c>
     </row>
@@ -1776,8 +3224,12 @@
         <f>'Android build'!$H$22</f>
         <v/>
       </c>
-      <c r="D6" s="15">
-        <f>SUM(C6:C6)</f>
+      <c r="D6" s="11">
+        <f>'Catalog CRUD'!$H$34</f>
+        <v/>
+      </c>
+      <c r="E6" s="15">
+        <f>SUM(C6:D6)</f>
         <v/>
       </c>
     </row>
@@ -1792,8 +3244,12 @@
         <f>C5+C6</f>
         <v/>
       </c>
-      <c r="D7" s="15">
-        <f>SUM(C7:C7)</f>
+      <c r="D7" s="11">
+        <f>D5+D6</f>
+        <v/>
+      </c>
+      <c r="E7" s="15">
+        <f>SUM(C7:D7)</f>
         <v/>
       </c>
     </row>
@@ -1888,55 +3344,99 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="19" t="inlineStr">
+    <row r="12" ht="74" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Admin Medication Catalog CRUD</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Kiểm thử CRUD, phân trang, validation và phân quyền quản trị danh mục thuốc.</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Catalog CRUD</t>
+        </is>
+      </c>
+      <c r="D12" s="18">
+        <f>IFERROR(('Catalog CRUD'!$H$35-'Catalog CRUD'!$H$34)/'Catalog CRUD'!$H$35,0)</f>
+        <v/>
+      </c>
+      <c r="E12" s="18">
+        <f>IFERROR('Catalog CRUD'!$H$32/'Catalog CRUD'!$H$35,0)</f>
+        <v/>
+      </c>
+      <c r="F12" s="18">
+        <f>IFERROR('Catalog CRUD'!$H$33/'Catalog CRUD'!$H$35,0)</f>
+        <v/>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>19 test catalog pass; toàn bộ 380 unit và architecture test pass.</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
         <is>
           <t>Bug Report</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="20" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="20" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="B35" s="20" t="inlineStr">
+      <c r="B36" s="20" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C35" s="20" t="inlineStr">
+      <c r="C36" s="20" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="D35" s="20" t="inlineStr">
+      <c r="D36" s="20" t="inlineStr">
         <is>
           <t>Input Data</t>
         </is>
       </c>
-      <c r="E35" s="20" t="inlineStr">
+      <c r="E36" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F35" s="20" t="inlineStr">
+      <c r="F36" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="G35" s="20" t="inlineStr">
+      <c r="G36" s="20" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="H35" s="20" t="inlineStr">
+      <c r="H36" s="20" t="inlineStr">
         <is>
           <t>Name of Tester</t>
         </is>
       </c>
-      <c r="I35" s="20" t="inlineStr">
+      <c r="I36" s="20" t="inlineStr">
         <is>
           <t>Logs</t>
         </is>
@@ -1947,17 +3447,17 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:A5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11">
+  <conditionalFormatting sqref="F11:F12">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11">
+  <conditionalFormatting sqref="G11:G12">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>OR(G11="Critical",G11="High")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G36">
+  <conditionalFormatting sqref="G37">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
@@ -1969,10 +3469,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G11:G12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="G36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Unit Test Login User
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -7,10 +7,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android build" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đăng nhập người dùng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Android build'!$A$8:$I$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Đăng nhập người dùng'!$A$8:$I$56</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -127,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -187,6 +189,9 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -346,12 +351,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11</f>
+              <f>'Report'!$A$11:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$11</f>
+              <f>'Report'!$D$11:$D$12</f>
             </numRef>
           </val>
         </ser>
@@ -370,12 +375,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11</f>
+              <f>'Report'!$A$11:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$11</f>
+              <f>'Report'!$E$11:$E$12</f>
             </numRef>
           </val>
         </ser>
@@ -394,12 +399,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11</f>
+              <f>'Report'!$A$11:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$11</f>
+              <f>'Report'!$F$11:$F$12</f>
             </numRef>
           </val>
         </ser>
@@ -502,7 +507,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>13</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -524,7 +529,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>13</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3240000"/>
@@ -1680,7 +1685,2982 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:W62"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="8" customWidth="1" min="22" max="22"/>
+    <col width="8" customWidth="1" min="23" max="23"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập người dùng (LOGIN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46303</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Kết quả POST /auth/mobile/verify</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="W8" s="5" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="156.5" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Đăng nhập lại bằng email OTP với tài khoản đã có hồ sơ</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Tài khoản email đã đăng nhập OTP một lần và hoàn thiện hồ sơ</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Lấy mã OTP mới cho email
+2. POST /auth/mobile/verify {email, token}</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>email: it-login-&lt;ngẫu nhiên&gt;@example.com; token: mã 6 số từ Supabase</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>200; user_id trùng lần đầu; profile_complete=true; session.session_type="mobile"; expires_in = 864000 ± 60; không có field supabase, không có refresh_token; bảng users có đúng 1 dòng cho email</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · Decision Table (R6) · EP (4,6) · test_returning_email_user_same_id_profile_complete__AC1</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>Số nội địa 0xxxxxxxxx
+Số quốc tế +84xxxxxxxxx
+Có khoảng trắng, gạch, khoảng trắng hai đầu</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1
+2
+3</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>84… thiếu dấu +
+Có ngoặc hoặc chữ
+Chữ số Unicode (full-width, Ả Rập)
+Khoảng trắng không ngắt ở giữa
+Độ dài &lt; 9 hoặc &gt; 16 ký tự (kể cả +)
+Sai kiểu JSON (số, mảng, object, bool)</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>13
+14
+15
+16
+17
+18</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Định danh hợp lệ?</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90.5" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Đăng nhập bằng số điện thoại dạng nội địa</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Số thử test_otp 84900000001 = 123456 trên Supabase local</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/verify {phone: "0900000001", token: "123456"}
+2. Đọc users.phone_number của user_id trả về</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>phone: 0900000001; token: 123456</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>200; users.phone_number = "+84900000001"</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>200; phone_number = +84900000001</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · EP (1,6) · test_local_phone_format_logs_in_and_wrong_otp_401__AC2</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>Email chữ thường
+Có chữ hoa hoặc khoảng trắng hai đầu</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>4
+5</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>Sai định dạng (thiếu @, thiếu tên miền, nhiều @, có khoảng trắng)
+Rỗng hoặc chỉ khoảng trắng (không có phone)</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>19
+20</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>Mã OTP đúng?</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90.5" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Xác thực số điện thoại với mã OTP sai</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Như TC-LOGIN-02</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/verify {phone: "0900000001", token: "000000"}</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>token: 000000</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>401 {"detail":"Invalid credentials"}; không chứa msg, error_code, otp_expired của Supabase</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>401 {"detail":"Invalid credentials"}</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · Decision Table (R2) · EP (21) · test_local_phone_format_logs_in_and_wrong_otp_401__AC2</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>token (OTP)</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>Đúng mã 6 chữ số</t>
+        </is>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>Sai mã 6 chữ số
+Rỗng
+Chỉ khoảng trắng
+Sai độ dài, có chữ, rất dài
+Chuỗi injection/ký tự đặc biệt</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>21
+22
+23
+24
+25</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>Tài khoản</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T11" s="11" t="inlineStr">
+        <is>
+          <t>Đã xóa</t>
+        </is>
+      </c>
+      <c r="U11" s="11" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="V11" s="11" t="inlineStr">
+        <is>
+          <t>Thường, chưa có hồ sơ</t>
+        </is>
+      </c>
+      <c r="W11" s="11" t="inlineStr">
+        <is>
+          <t>Thường, đủ hồ sơ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="90.5" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile App bằng tài khoản admin</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Tài khoản có users.system_role = 'admin'</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Lấy mã OTP email của admin
+2. POST /auth/mobile/verify {email, token}</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>email: it-login-admin-&lt;ngẫu nhiên&gt;@example.com</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>403 {"detail":"admin_must_use_web"}; không cấp session</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>403 {"detail":"admin_must_use_web"}, không có session</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · Decision Table (R4) · test_admin_account_on_mobile_forbidden__AC3</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>ho_ten</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>Tiếng Việt có dấu
+Emoji
+Chuỗi SQL/HTML/template (lưu như dữ liệu)
+Dài đúng 255 ký tự</t>
+        </is>
+      </c>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>7
+8
+9
+10</t>
+        </is>
+      </c>
+      <c r="N12" s="10" t="inlineStr">
+        <is>
+          <t>Rỗng hoặc chỉ khoảng trắng
+Dài &gt; 255 ký tự
+Có ký tự NUL</t>
+        </is>
+      </c>
+      <c r="O12" s="10" t="inlineStr">
+        <is>
+          <t>26
+27
+28</t>
+        </is>
+      </c>
+      <c r="Q12" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="V12" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="W12" s="5" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="74" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Dùng phiên cũ và đăng nhập lại sau khi tài khoản bị xóa</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>User đã đăng nhập, đang giữ phiên mobile hợp lệ</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Đặt users.erased_at = now() (xóa trường định danh như SqlUsers.erase)
+2. POST /auth/profile với phiên cũ
+3. POST /auth/mobile/verify với mã OTP mới</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Phiên mobile còn hạn</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Cả hai request trả 401 ngay ở request kế tiếp; không cấp session</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>401 và 401, không có session</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · State Transition (đang có phiên → bị xóa) · Decision Table (R3) · test_erased_user_session_and_relogin_rejected__AC4</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>ngay_sinh</t>
+        </is>
+      </c>
+      <c r="L13" s="10" t="inlineStr">
+        <is>
+          <t>Từ 1900-01-01 tới hôm nay theo giờ Asia/Ho_Chi_Minh</t>
+        </is>
+      </c>
+      <c r="M13" s="10" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="N13" s="10" t="inlineStr">
+        <is>
+          <t>Sau hôm nay (giờ VN)
+Trước 1900-01-01
+Ngày không tồn tại hoặc sai định dạng</t>
+        </is>
+      </c>
+      <c r="O13" s="10" t="inlineStr">
+        <is>
+          <t>29
+30
+31</t>
+        </is>
+      </c>
+      <c r="Q13" s="10" t="inlineStr">
+        <is>
+          <t>422 (invalid_phone / invalid_email / login_identifier_required)</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S13" s="11" t="inlineStr"/>
+      <c r="T13" s="11" t="inlineStr"/>
+      <c r="U13" s="11" t="inlineStr"/>
+      <c r="V13" s="11" t="inlineStr"/>
+      <c r="W13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="74" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Đăng nhập với nhiều cách viết của cùng một số điện thoại</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Số thử test_otp</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/verify lần lượt với từng dạng số, token 123456
+2. So user_id các lần
+3. Đếm users có phone_number = +84900000001</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>0900000001 | +84900000001 | +84 900 000 001 | 0900-000-001 | "  0900000001  "</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Mọi lần 200 với cùng một user_id; đúng 1 dòng users, phone_number = +84900000001</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>5/5 lần 200, cùng user_id; 1 dòng users</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · EP (1,2,3) · test_phone_formats_same_user__AC5</t>
+        </is>
+      </c>
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>gioi_tinh</t>
+        </is>
+      </c>
+      <c r="L14" s="10" t="inlineStr">
+        <is>
+          <t>nam / nu / khac (không phân biệt hoa thường)</t>
+        </is>
+      </c>
+      <c r="M14" s="10" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="N14" s="10" t="inlineStr">
+        <is>
+          <t>Giá trị khác, rỗng, chuỗi injection</t>
+        </is>
+      </c>
+      <c r="O14" s="10" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>401 Invalid credentials / không cấp phiên</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr"/>
+      <c r="S14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U14" s="11" t="inlineStr"/>
+      <c r="V14" s="11" t="inlineStr"/>
+      <c r="W14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="74" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Gửi số điện thoại sai định dạng tới OTP và verify</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/otp {phone}
+2. POST /auth/mobile/verify {phone, token: 123456}
+3. Đếm auth.users trước/sau</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>84900000001 | (+84)900000001 | 09abc12345 | +84 900\u00a0000 001 | + | 0</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_phone"} ở cả hai endpoint; không tạo user trên Supabase</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>422 invalid_phone ở cả 12 request; auth.users không đổi</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (13,14,16) · test_invalid_phone_rejected_before_provider__AC6</t>
+        </is>
+      </c>
+      <c r="Q15" s="10" t="inlineStr">
+        <is>
+          <t>403 admin_must_use_web</t>
+        </is>
+      </c>
+      <c r="R15" s="11" t="inlineStr"/>
+      <c r="S15" s="11" t="inlineStr"/>
+      <c r="T15" s="11" t="inlineStr"/>
+      <c r="U15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="V15" s="11" t="inlineStr"/>
+      <c r="W15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16" ht="74" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Số thử test_otp</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
+2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>phone: 0900000001 + ký tự \n</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · Error Guessing · test_invalid_phone_rejected_before_provider__AC6[0900000001\n-*]</t>
+        </is>
+      </c>
+      <c r="Q16" s="10" t="inlineStr">
+        <is>
+          <t>200, phiên mobile 10 ngày, profile_complete=false</t>
+        </is>
+      </c>
+      <c r="R16" s="11" t="inlineStr"/>
+      <c r="S16" s="11" t="inlineStr"/>
+      <c r="T16" s="11" t="inlineStr"/>
+      <c r="U16" s="11" t="inlineStr"/>
+      <c r="V16" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="W16" s="11" t="inlineStr"/>
+    </row>
+    <row r="17" ht="57.5" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Gửi số điện thoại ngay ngoài giới hạn độ dài</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/otp và /auth/mobile/verify với từng số</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>+8490000 (8 ký tự) | +8490000000000000 (17 ký tự)</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_phone"}</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>422 invalid_phone</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · BVA (min-1, max+1) · EP (17) · test_invalid_phone_rejected_before_provider__AC6</t>
+        </is>
+      </c>
+      <c r="Q17" s="10" t="inlineStr">
+        <is>
+          <t>200, phiên mobile 10 ngày, profile_complete=true</t>
+        </is>
+      </c>
+      <c r="R17" s="11" t="inlineStr"/>
+      <c r="S17" s="11" t="inlineStr"/>
+      <c r="T17" s="11" t="inlineStr"/>
+      <c r="U17" s="11" t="inlineStr"/>
+      <c r="V17" s="11" t="inlineStr"/>
+      <c r="W17" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="57.5" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Gửi số điện thoại đúng giới hạn độ dài</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/otp {phone}
+2. POST /auth/mobile/verify {phone, token: 123456}</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>+84900000 (9 ký tự) | +849000000000000 (16 ký tự)</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Không bị backend trả invalid_phone; không 5xx ngoài 503; không lộ nội dung Supabase</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Không có invalid_phone; mã trạng thái &lt; 500 hoặc 503; không lộ nội dung</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · BVA (min, max) · EP (2) · test_phone_length_boundaries_accepted_by_backend__AC6</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="57.5" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/otp {phone}
+2. POST /auth/mobile/verify {phone, token: 123456}</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · EP (15) · test_unicode_digit_phone_rejected__AC7</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="90.5" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Đăng nhập email với chữ hoa và khoảng trắng hai đầu</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Tài khoản email chữ thường user.test+&lt;tag&gt;@example.com</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/verify {email: "User.Test+&lt;tag&gt;@Example.COM", token}
+2. POST /auth/mobile/verify {email: "  user.test+&lt;tag&gt;@example.com  ", token mới}
+3. Đọc users.email</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Hai cách viết của cùng email</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Cả hai 200, cùng user_id; users.email lưu chữ thường</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>200, 200, cùng user_id; email chữ thường</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (4,5) · test_email_case_and_spaces_same_user__AC8</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="57.5" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-13</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Gửi email sai định dạng tới OTP và verify</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/otp {email}
+2. POST /auth/mobile/verify {email, token: 123456}</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>abc | a@b | a@@b.com | a b@c.com | @example.com | a@example.</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_email"}</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>422 invalid_email ở cả 12 request</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (19) · test_invalid_email_rejected__AC8</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="57.5" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-14</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Gửi email rỗng hoặc chỉ khoảng trắng, không có số điện thoại</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/otp {email}
+2. POST /auth/mobile/verify {email, token: 123456}</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>(blank) | "   "</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail":"login_identifier_required"}</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>422 login_identifier_required</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (20) · Decision Table (R1) · test_invalid_email_rejected__AC8</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="41" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Gửi email rất dài và email có dấu tiếng Việt</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/otp {email}</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>a*300@example.com (312 ký tự) | nguyễn@example.com</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Không 5xx ngoài 503; không lộ nội dung Supabase</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Mã &lt; 500 hoặc 503; không lộ nội dung</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · Error Guessing · test_long_and_unicode_email_no_5xx__AC8</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="41" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-16</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Xác thực với mã OTP rỗng</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Tài khoản email mới</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/verify {email, token: ""}</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>token: (blank)</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · EP (22) · test_empty_token_422__AC9</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="57.5" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-17</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Xác thực với mã OTP chỉ có khoảng trắng</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Tài khoản email mới, chưa có dòng users</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/verify {email, token: "   "}
+2. Đếm users theo email</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>token: "   "</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>401; không tạo dòng users</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>401; 0 dòng users</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · EP (23) · test_blank_token_401_no_user__AC9</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="57.5" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-18</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Xác thực với mã OTP sai độ dài, có chữ hoặc rất dài</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Tài khoản email mới, chưa có dòng users</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/verify {email, token} cho từng giá trị</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>12345 | 1234567 | abcdef | "1"*1000</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>401 hoặc 422; không 5xx; không lộ nội dung; không tạo dòng users</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>401/422; không 5xx; 0 dòng users</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · BVA (min-1, max+1) · EP (24) · test_malformed_tokens_no_5xx__AC9</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="90.5" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-19</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Gửi trường sai kiểu JSON</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Phiên mobile hợp lệ cho /auth/profile</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/otp với phone/email là số, mảng, object, true
+2. POST /auth/mobile/verify với token sai kiểu
+3. POST /auth/profile với ho_ten/gioi_tinh sai kiểu</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>900000001 | ["0900000001"] | {"v": "0900000001"} | true</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>4xx (422); không 5xx; không lộ chi tiết nội bộ</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>422 ở cả 20 request</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · EP (18) · test_wrong_json_types_no_5xx__AC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="41" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-20</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Gửi body hỏng, rỗng hoặc sai Content-Type</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Phiên mobile hợp lệ cho /auth/profile</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. POST tới /auth/mobile/otp, /auth/mobile/verify, /auth/profile với từng loại body</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>"{not json" | (blank) | text/plain "phone=0900000001"</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>4xx; không 5xx</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>422 ở cả 9 request</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · Error Guessing · test_malformed_body_no_5xx__AC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="90.5" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-21</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Gửi field thừa để leo quyền hoặc ghi vào user khác</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Tài khoản email mới; một user khác B chưa có hồ sơ</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/verify {email, token, system_role: "admin", user_id: &lt;B&gt;}
+2. POST /auth/profile (phiên vừa cấp) {hồ sơ hợp lệ, user_id: &lt;B&gt;, system_role: "admin"}
+3. Đọc users của mình và của B</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>system_role: admin; user_id: id của B</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Verify 200 với user_id của chính mình; profile 204; system_role vẫn 'user'; hồ sơ chỉ ghi vào mình, B không đổi</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · Error Guessing (leo quyền) · test_extra_fields_have_no_effect__AC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="90.5" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-22</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Gửi chuỗi SQL injection và chuỗi độc hại vào số điện thoại và email</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/otp {phone: &lt;chuỗi&gt;}
+2. POST /auth/mobile/otp {email: &lt;chuỗi&gt;}
+3. Đo thời gian phản hồi; kiểm bảng users</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>' OR '1'='1 | admin'-- | '); DROP TABLE users;-- | 1; SELECT pg_sleep(5)-- | &lt;script&gt;alert(1)&lt;/script&gt; | ${7*7} | abc\u0000def</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>422; &lt; 3 giây; không có Traceback, psycopg, sqlalchemy, syntax error trong phản hồi; bảng users còn và số dòng không đổi</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>422 ở cả 14 request, &lt; 3 giây, không lộ; users còn, số dòng không đổi</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · Error Guessing (bảo mật) · test_injection_in_identifier_rejected_no_leak__AC11, test_injection_group_leaves_users_table_intact__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="41" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-23</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Gửi chuỗi injection làm mã OTP</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Tài khoản email mới, chưa có dòng users</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/verify {email, token: &lt;chuỗi&gt;}</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>7 chuỗi như TC-LOGIN-22</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>401 hoặc 422; không 5xx; không lộ; không tạo dòng users</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>401/422 ở cả 7 request; không lộ; 0 dòng users</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · EP (25) · test_injection_in_token_no_5xx_no_leak__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="57.5" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-24</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Lưu họ tên là chuỗi SQL/HTML/template</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>User có phiên mobile, chưa có hồ sơ</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ho_ten: &lt;chuỗi&gt;, ngày sinh, giới tính hợp lệ}
+2. Đọc users.full_name</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>6 chuỗi đầu của TC-LOGIN-22 (không có NUL)</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>204; full_name lưu nguyên văn chuỗi; &lt; 3 giây; bảng users còn</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>204; lưu nguyên văn cả 6 chuỗi</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · EP (9) · test_injection_in_full_name_stored_verbatim__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="57.5" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-25</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Lưu họ tên có ký tự NUL</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>User có phiên mobile, chưa có hồ sơ</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>ho_ten: abc\u0000def</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>500 Internal Server Error</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · EP (28) · Error Guessing · test_injection_in_full_name_stored_verbatim__AC11[nul]</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="41" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-26</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Gửi chuỗi injection làm giới tính</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>User có phiên mobile, chưa có hồ sơ</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {gioi_tinh: &lt;chuỗi&gt;}</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>7 chuỗi như TC-LOGIN-22</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_gender"}; hồ sơ không đổi</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>422 invalid_gender; full_name vẫn NULL</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · EP (32) · test_injection_in_gender_rejected__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="41" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-27</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Lưu họ tên tiếng Việt có dấu và có emoji</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>User có phiên mobile, chưa có hồ sơ</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ho_ten}
+2. Đọc users.full_name</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Ấn | Bà Lan 👵🏻💊</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>204; lưu đúng nguyên văn</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>204; lưu đúng</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · EP (7,8) · test_profile_valid_classes_saved__AC12</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="41" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-28</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Lưu giới tính viết hoa</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>User có phiên mobile, chưa có hồ sơ</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {gioi_tinh: "NAM"}
+2. Đọc users.gender</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>gioi_tinh: NAM</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>204; gender = 'nam'</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>204; gender = nam</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · EP (12) · test_profile_valid_classes_saved__AC12</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="57.5" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-29</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Lưu họ tên dài đúng 255 ký tự</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>User có phiên mobile, chưa có hồ sơ</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ho_ten: A*255}</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>A*255</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>204; lưu đủ 255 ký tự</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>204; lưu đủ</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · BVA (max) · EP (10) · test_profile_valid_classes_saved__AC12</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="57.5" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-30</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Lưu họ tên dài 256 ký tự</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>User có phiên mobile, chưa có hồ sơ</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ho_ten: A*256}</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>A*256</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>204, đã lưu</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · BVA (max+1) · EP (27) · test_profile_limits_255_and_1900__AC12[ten-256]</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="57.5" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-31</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Lưu ngày sinh 1900-01-01</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>User có phiên mobile, chưa có hồ sơ</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ngay_sinh: "1900-01-01"}</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>1900-01-01</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>204; date_of_birth = 1900-01-01</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>204; lưu đúng</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · BVA (min) · EP (11) · test_profile_valid_classes_saved__AC12</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="74" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-32</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Lưu ngày sinh trước 1900-01-01</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>User có phiên mobile, chưa có hồ sơ</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ngay_sinh}</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>1899-12-31 | 0001-01-01</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>204 ở cả hai giá trị, đã lưu</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · BVA (min-1) · EP (30) · test_profile_limits_255_and_1900__AC12[ngay-1899-12-31, ngay-0001-01-01]</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="90.5" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-33</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Gửi hồ sơ có họ tên, giới tính hoặc ngày sinh không hợp lệ</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>User có phiên mobile, chưa có hồ sơ</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile với từng giá trị
+2. Đọc users.full_name</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>ho_ten (blank) | "   " → invalid_full_name; gioi_tinh x | (blank) → invalid_gender; ngay_sinh 2026-02-30 | 30/01/1990 | abc</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>422 (detail tương ứng); full_name vẫn NULL (profile_complete vẫn false)</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>422 đúng detail ở cả 7 trường hợp; full_name NULL</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · EP (26,31,32) · test_profile_invalid_classes_422_db_unchanged__AC12</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="57.5" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-34</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Lưu ngày sinh là hôm nay lúc 12:00 giờ Việt Nam</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Đồng hồ server cố định 2026-10-08 12:00 (+07:00)</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>ngay_sinh: 2026-10-08</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I42" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · BVA (max) · EP (11) · test_birth_date_today_in_vietnam_accepted__AC12[12h-gio-VN]</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="57.5" customHeight="1">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-35</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Đồng hồ server cố định 2026-10-08 00:30 (+07:00) = 2026-10-07 17:30 UTC</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>ngay_sinh: 2026-10-08</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_date_of_birth"}</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · BVA (max) · EP (11) · test_birth_date_today_in_vietnam_accepted__AC12[0h30-gio-VN]</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="57.5" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-36</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Lưu ngày sinh là ngày mai theo giờ Việt Nam</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Đồng hồ server cố định 2026-10-08 12:00 (+07:00)</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ngay_sinh: "2026-10-09"}</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>ngay_sinh: 2026-10-09</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_date_of_birth"}; hồ sơ không đổi</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>422 invalid_date_of_birth; full_name NULL</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I44" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · BVA (max+1) · EP (29) · test_birth_date_tomorrow_in_vietnam_rejected__AC12</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="90.5" customHeight="1">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-37</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Gọi API cần đăng nhập với bearer thiếu, sai hoặc giả mạo</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>User chưa có hồ sơ</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile với từng header Authorization
+2. Đọc users.full_name</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>không có header | Basic &lt;token&gt; | "Bearer " | Bearer ' OR '1'='1 | token sửa chữ ký | token hết hạn (11 ngày trước) | token ký bằng secret khác</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>401 ở mọi trường hợp; hồ sơ không đổi</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>401 ở cả 7 trường hợp; full_name NULL</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I45" s="8" t="inlineStr">
+        <is>
+          <t>AC13 · Error Guessing (bảo mật) · test_bad_bearer_401_db_unchanged__AC13</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="140" customHeight="1">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-38</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Đăng nhập lần đầu trên app: hồ sơ, consent, vào Trang chủ</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>Backend + Supabase local; emulator; số thử chưa có hồ sơ, consent health_data đã rút</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở app, tab Số điện thoại, nhập 0900000001
+2. Tick đồng ý điều khoản, bấm "Gửi mã OTP"
+3. Nhập 123456
+4. Màn "Hoàn thiện hồ sơ": nhập Nguyễn Văn Ấn, chọn ngày sinh, chọn Nam, bấm "Lưu và tiếp tục"
+5. Màn "Quyền riêng tư của bạn": bật dữ liệu sức khỏe, bấm "Tiếp tục"</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>0900000001 / 123456; họ tên Nguyễn Văn Ấn</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>Vào Trang chủ; DB: users.full_name = 'Nguyễn Văn Ấn', phone_number = +84900000001, đúng 1 dòng</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>Vào Trang chủ; DB đúng</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I46" s="8" t="inlineStr">
+        <is>
+          <t>AC16 · State Transition (chưa hồ sơ → đủ hồ sơ) · E2E login_new_user_test.dart · evidence/test-e2e.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="41" customHeight="1">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-39</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Mở lại app khi còn phiên đăng nhập</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Đã qua TC-LOGIN-38</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>1. Khởi động lại app (dựng lại toàn bộ app với cùng bộ nhớ thiết bị)</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Phiên đã lưu trong secure storage</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>Vào thẳng Trang chủ, không hỏi OTP</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>Vào thẳng Trang chủ</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I47" s="8" t="inlineStr">
+        <is>
+          <t>AC17 · E2E login_new_user_test.dart · evidence/test-e2e.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="41" customHeight="1">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-40</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Đăng xuất rồi mở lại app</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở Trang chủ</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>1. Tab "Hồ sơ" → "Đăng xuất"
+2. Khởi động lại app</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>Về màn Đăng nhập; mở lại vẫn ở màn Đăng nhập</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I48" s="8" t="inlineStr">
+        <is>
+          <t>AC18 · E2E login_new_user_test.dart · evidence/test-e2e.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="57.5" customHeight="1">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-41</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Nhập mã OTP sai rồi nhập lại mã đúng trên app</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Số thử đã có hồ sơ và consent</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhập 0900000001, gửi mã
+2. Nhập 000000
+3. Nhập lại 123456</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>000000 rồi 123456</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>Sau mã sai: hiện "Mã OTP không đúng hoặc đã hết hạn", vẫn ở màn OTP; sau mã đúng: vào Trang chủ</t>
+        </is>
+      </c>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I49" s="8" t="inlineStr">
+        <is>
+          <t>AC19 · E2E login_errors_test.dart · evidence/test-e2e.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="74" customHeight="1">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-42</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>Như TC-LOGIN-41, đang ở màn OTP sau lần nhập 000000</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạm vào ô mã OTP
+2. Theo dõi request backend nhận được</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Ô đang chứa 000000</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
+        </is>
+      </c>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I50" s="8" t="inlineStr">
+        <is>
+          <t>AC19 · Error Guessing (bấm/chạm lặp) · E2E login_errors_test.dart</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="74" customHeight="1">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-43</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Nhập số điện thoại không hợp lệ trên màn Đăng nhập</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Mở app, chưa đăng nhập, đã tick điều khoản</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhập abc, bấm "Gửi mã OTP"
+2. Nhập 12, bấm "Gửi mã OTP"</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>abc | 12</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>abc: ô chỉ nhận chữ số nên rỗng → "Vui lòng nhập số điện thoại"; 12: "Số điện thoại không hợp lệ (9-11 chữ số)"; không sang màn OTP</t>
+        </is>
+      </c>
+      <c r="G51" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I51" s="8" t="inlineStr">
+        <is>
+          <t>AC20 · EP (14,17) · E2E login_errors_test.dart</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="57.5" customHeight="1">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-44</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Nhập số điện thoại có khoảng trắng trên app</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>Như TC-LOGIN-43</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhập 0900 000 001
+2. Bấm "Gửi mã OTP", nhập 123456</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>0900 000 001</t>
+        </is>
+      </c>
+      <c r="F52" s="8" t="inlineStr">
+        <is>
+          <t>Ô hiển thị "090 000 0001"; đăng nhập vào Trang chủ; DB vẫn 1 dòng users, cùng user_id với TC-LOGIN-38</t>
+        </is>
+      </c>
+      <c r="G52" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I52" s="8" t="inlineStr">
+        <is>
+          <t>AC20 · EP (3) · E2E login_errors_test.dart · evidence/test-e2e.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="90.5" customHeight="1">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-45</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Hoàn thiện hồ sơ trên app với họ tên rỗng rồi họ tên là chuỗi injection</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>Số thử chưa có hồ sơ (đã có consent)</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập, màn Hoàn thiện hồ sơ
+2. Chọn ngày sinh, giới tính Nữ, để trống họ tên, bấm "Lưu và tiếp tục"
+3. Nhập họ tên '); DROP TABLE users;--, bấm "Lưu và tiếp tục"</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>(blank) rồi '); DROP TABLE users;--</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>Lần 1: hiện "Vui lòng nhập họ tên", ở lại màn; lần 2: vào Trang chủ; DB lưu nguyên văn chuỗi, bảng users còn, số dòng không giảm</t>
+        </is>
+      </c>
+      <c r="G53" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H53" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I53" s="8" t="inlineStr">
+        <is>
+          <t>AC20 · EP (9,26) · E2E profile_input_test.dart · evidence/test-e2e.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="90.5" customHeight="1">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-46</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Chạy script E2E khi thiếu điều kiện môi trường</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>Không có Supabase local hoặc không có emulator</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>1. backend/.venv/Scripts/python.exe tests/e2e/mobile_login/run_e2e.py</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="F54" s="8" t="inlineStr">
+        <is>
+          <t>Thoát mã 2 với "LỖI MÔI TRƯỜNG: …"; không chạy flutter, không báo pass; output không chứa key/token/mật khẩu</t>
+        </is>
+      </c>
+      <c r="G54" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi (unit test test_run_e2e.py, 16 pass)</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I54" s="8" t="inlineStr">
+        <is>
+          <t>AC21 · test_main_exits_2_when_environment_missing, test_pick_device_*, test_require_local_*, test_redact_* · evidence/test-tests-unit.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="74" customHeight="1">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-47</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Gõ lại mã OTP bằng bàn phím thật sau khi nhập sai</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>Điện thoại hoặc emulator, app nối backend có Supabase; đang ở màn OTP sau khi nhập mã sai</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạm vào ô mã
+2. Xóa mã cũ bằng phím xóa
+3. Gõ mã đúng bằng bàn phím</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Mã đúng của số đang dùng</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>Mã mới hiện trong ô và app vào Trang chủ</t>
+        </is>
+      </c>
+      <c r="G55" s="8" t="inlineStr"/>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I55" s="8" t="inlineStr">
+        <is>
+          <t>AC19 · manual · integration_test không gõ lại được vào ô sau khi app bỏ focus nên E2E đặt mã qua controller</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="57.5" customHeight="1">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-48</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Tắt hẳn app (force stop) rồi mở lại khi còn phiên</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập trên thiết bị</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>1. Cài đặt → Ứng dụng → DrugTime → Buộc dừng
+2. Mở lại app từ màn hình chính</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="F56" s="8" t="inlineStr">
+        <is>
+          <t>Vào thẳng Trang chủ, không hỏi OTP</t>
+        </is>
+      </c>
+      <c r="G56" s="8" t="inlineStr"/>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I56" s="8" t="inlineStr">
+        <is>
+          <t>AC17 · manual · integration_test chỉ dựng lại app trong cùng tiến trình</t>
+        </is>
+      </c>
+    </row>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59">
+      <c r="G59" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H59" s="13">
+        <f>COUNTIF(H9:H56,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="G60" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H60" s="13">
+        <f>COUNTIF(H9:H56,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="G61" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H61" s="13">
+        <f>COUNTIF(H9:H56,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="G62" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H62" s="13">
+        <f>SUM(H59:H61)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I56"/>
+  <conditionalFormatting sqref="H9:H56">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1725,7 +4705,7 @@
         </is>
       </c>
       <c r="C3" s="11">
-        <f>'Android build'!$H$20</f>
+        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59</f>
         <v/>
       </c>
       <c r="D3" s="15">
@@ -1741,7 +4721,7 @@
         </is>
       </c>
       <c r="C4" s="11">
-        <f>'Android build'!$H$21</f>
+        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60</f>
         <v/>
       </c>
       <c r="D4" s="15">
@@ -1773,7 +4753,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr"/>
       <c r="C6" s="11">
-        <f>'Android build'!$H$22</f>
+        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61</f>
         <v/>
       </c>
       <c r="D6" s="15">
@@ -1888,57 +4868,440 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="19" t="inlineStr">
+    <row r="12" ht="189.5" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Đăng nhập người dùng</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile App bằng OTP (số điện thoại hoặc email), hoàn thiện hồ sơ lần đầu, phiên đăng nhập và đăng xuất — user thường, không gồm admin</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Đăng nhập người dùng</t>
+        </is>
+      </c>
+      <c r="D12" s="18">
+        <f>IFERROR(('Đăng nhập người dùng'!$H$62-'Đăng nhập người dùng'!$H$61)/'Đăng nhập người dùng'!$H$62,0)</f>
+        <v/>
+      </c>
+      <c r="E12" s="18">
+        <f>IFERROR('Đăng nhập người dùng'!$H$59/'Đăng nhập người dùng'!$H$62,0)</f>
+        <v/>
+      </c>
+      <c r="F12" s="18">
+        <f>IFERROR('Đăng nhập người dùng'!$H$60/'Đăng nhập người dùng'!$H$62,0)</f>
+        <v/>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Luồng chính (đăng nhập, hồ sơ, consent, mở lại app, đăng xuất) và mọi kiểm tra quyền/bearer đạt, cả ở API lẫn E2E trên emulator. 7 Fail gồm lỗi kiểm tra đầu vào ở biên (chữ số Unicode, họ tên &gt; 255, ngày sinh &lt; 1900, ký tự NUL gây 500), lỗi múi giờ khi kiểm ngày sinh (dùng UTC), app gửi lại mã OTP sai khi chạm ô, và một kỳ vọng AC6 cần chốt lại (ký tự xuống dòng cuối số điện thoại).</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
         <is>
           <t>Bug Report</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="20" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="20" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="B35" s="20" t="inlineStr">
+      <c r="B36" s="20" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C35" s="20" t="inlineStr">
+      <c r="C36" s="20" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="D35" s="20" t="inlineStr">
+      <c r="D36" s="20" t="inlineStr">
         <is>
           <t>Input Data</t>
         </is>
       </c>
-      <c r="E35" s="20" t="inlineStr">
+      <c r="E36" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F35" s="20" t="inlineStr">
+      <c r="F36" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="G35" s="20" t="inlineStr">
+      <c r="G36" s="20" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="H35" s="20" t="inlineStr">
+      <c r="H36" s="20" t="inlineStr">
         <is>
           <t>Name of Tester</t>
         </is>
       </c>
-      <c r="I35" s="20" t="inlineStr">
+      <c r="I36" s="20" t="inlineStr">
         <is>
           <t>Logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="123.5" customHeight="1">
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-08</t>
+        </is>
+      </c>
+      <c r="B37" s="22" t="inlineStr">
+        <is>
+          <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
+        </is>
+      </c>
+      <c r="C37" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
+2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
+        </is>
+      </c>
+      <c r="D37" s="22" t="inlineStr">
+        <is>
+          <t>phone: 0900000001 + ký tự \n</t>
+        </is>
+      </c>
+      <c r="E37" s="22" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
+        </is>
+      </c>
+      <c r="F37" s="22" t="inlineStr">
+        <is>
+          <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
+        </is>
+      </c>
+      <c r="G37" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H37" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I37" s="22" t="inlineStr">
+        <is>
+          <t>Nghi vấn — kỳ vọng AC6 mâu thuẫn AC5: backend `_validate_required_text` (sign_in.py:178) `strip()` mọi ký tự trắng hai đầu, nên \n cuối được xử lý như khoảng trắng hai đầu mà AC5 coi là hợp lệ. Cần người dùng chốt: sửa AC6 hoặc sửa backend
+Log: evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="123.5" customHeight="1">
+      <c r="A38" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-11</t>
+        </is>
+      </c>
+      <c r="B38" s="22" t="inlineStr">
+        <is>
+          <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
+        </is>
+      </c>
+      <c r="C38" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/otp {phone}
+2. POST /auth/mobile/verify {phone, token: 123456}</t>
+        </is>
+      </c>
+      <c r="D38" s="22" t="inlineStr">
+        <is>
+          <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
+        </is>
+      </c>
+      <c r="E38" s="22" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
+        </is>
+      </c>
+      <c r="F38" s="22" t="inlineStr">
+        <is>
+          <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
+        </is>
+      </c>
+      <c r="G38" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H38" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I38" s="22" t="inlineStr">
+        <is>
+          <t>`_normalize_phone` (sign_in.py:197–206) kiểm bằng `str.isdigit()`, nhận cả chữ số Unicode, nên số lọt qua kiểm tra và gửi tới Supabase. Ô nhập của app chỉ cho 0-9 nên người dùng app không gặp; lỗi ở tầng API
+Log: evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="189.5" customHeight="1">
+      <c r="A39" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-25</t>
+        </is>
+      </c>
+      <c r="B39" s="22" t="inlineStr">
+        <is>
+          <t>Lưu họ tên có ký tự NUL</t>
+        </is>
+      </c>
+      <c r="C39" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
+        </is>
+      </c>
+      <c r="D39" s="22" t="inlineStr">
+        <is>
+          <t>ho_ten: abc\u0000def</t>
+        </is>
+      </c>
+      <c r="E39" s="22" t="inlineStr">
+        <is>
+          <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
+        </is>
+      </c>
+      <c r="F39" s="22" t="inlineStr">
+        <is>
+          <t>500 Internal Server Error</t>
+        </is>
+      </c>
+      <c r="G39" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H39" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I39" s="22" t="inlineStr">
+        <is>
+          <t>`_validate_required_text` (sign_in.py:178) không chặn ký tự điều khiển; PostgreSQL từ chối NUL trong cột text: `psycopg.DataError: PostgreSQL text fields cannot contain NUL (0x00) bytes` ở `UPDATE users SET full_name…` (SqlUsers.update_profile); không có handler cho DataError nên thành 500. Câu SQL có tham số nên không phải lỗ hổng SQL injection
+Log: evidence/test-integration.log, evidence/test-probe-nul.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="90.5" customHeight="1">
+      <c r="A40" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-30</t>
+        </is>
+      </c>
+      <c r="B40" s="22" t="inlineStr">
+        <is>
+          <t>Lưu họ tên dài 256 ký tự</t>
+        </is>
+      </c>
+      <c r="C40" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ho_ten: A*256}</t>
+        </is>
+      </c>
+      <c r="D40" s="22" t="inlineStr">
+        <is>
+          <t>A*256</t>
+        </is>
+      </c>
+      <c r="E40" s="22" t="inlineStr">
+        <is>
+          <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
+        </is>
+      </c>
+      <c r="F40" s="22" t="inlineStr">
+        <is>
+          <t>204, đã lưu</t>
+        </is>
+      </c>
+      <c r="G40" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H40" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I40" s="22" t="inlineStr">
+        <is>
+          <t>Không có giới hạn độ dài họ tên: `_validate_profile` (sign_in.py) chỉ kiểm rỗng; cột users.full_name kiểu text không giới hạn
+Log: evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="90.5" customHeight="1">
+      <c r="A41" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-32</t>
+        </is>
+      </c>
+      <c r="B41" s="22" t="inlineStr">
+        <is>
+          <t>Lưu ngày sinh trước 1900-01-01</t>
+        </is>
+      </c>
+      <c r="C41" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ngay_sinh}</t>
+        </is>
+      </c>
+      <c r="D41" s="22" t="inlineStr">
+        <is>
+          <t>1899-12-31 | 0001-01-01</t>
+        </is>
+      </c>
+      <c r="E41" s="22" t="inlineStr">
+        <is>
+          <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
+        </is>
+      </c>
+      <c r="F41" s="22" t="inlineStr">
+        <is>
+          <t>204 ở cả hai giá trị, đã lưu</t>
+        </is>
+      </c>
+      <c r="G41" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H41" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I41" s="22" t="inlineStr">
+        <is>
+          <t>`_validate_birth_date` (sign_in.py:229–231) chỉ chặn ngày tương lai, không có cận dưới. App mobile đã giới hạn date picker từ 1900 nên chỉ gặp khi gọi API trực tiếp
+Log: evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="123.5" customHeight="1">
+      <c r="A42" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-35</t>
+        </is>
+      </c>
+      <c r="B42" s="22" t="inlineStr">
+        <is>
+          <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
+        </is>
+      </c>
+      <c r="C42" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
+        </is>
+      </c>
+      <c r="D42" s="22" t="inlineStr">
+        <is>
+          <t>ngay_sinh: 2026-10-08</t>
+        </is>
+      </c>
+      <c r="E42" s="22" t="inlineStr">
+        <is>
+          <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
+        </is>
+      </c>
+      <c r="F42" s="22" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_date_of_birth"}</t>
+        </is>
+      </c>
+      <c r="G42" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H42" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I42" s="22" t="inlineStr">
+        <is>
+          <t>`_validate_birth_date` (sign_in.py:230) so với `now.date()` trong khi `now()` (shared/clock.py) trả giờ UTC: từ 00:00 đến 07:00 giờ VN, "hôm nay" bị coi là ngày mai. Vi phạm bất biến 7 (múi giờ cố định Asia/Ho_Chi_Minh)
+Log: evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="173" customHeight="1">
+      <c r="A43" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-42</t>
+        </is>
+      </c>
+      <c r="B43" s="22" t="inlineStr">
+        <is>
+          <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
+        </is>
+      </c>
+      <c r="C43" s="22" t="inlineStr">
+        <is>
+          <t>1. Chạm vào ô mã OTP
+2. Theo dõi request backend nhận được</t>
+        </is>
+      </c>
+      <c r="D43" s="22" t="inlineStr">
+        <is>
+          <t>Ô đang chứa 000000</t>
+        </is>
+      </c>
+      <c r="E43" s="22" t="inlineStr">
+        <is>
+          <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
+        </is>
+      </c>
+      <c r="F43" s="22" t="inlineStr">
+        <is>
+          <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
+        </is>
+      </c>
+      <c r="G43" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H43" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I43" s="22" t="inlineStr">
+        <is>
+          <t>`OtpPinInput._handleTextChange` (frontend/mobile/lib/features/auth/presentation/widgets/otp_pin_input.dart:66–72) chạy với mọi thông báo của controller, kể cả khi chỉ đổi vị trí con trỏ lúc chạm ô, và gọi onCompleted hễ ô đủ 6 số → gửi lại mã sai, tốn hạn mức token_verifications
+Log: evidence/test-e2e.log (mục "request backend trong pha 2"), evidence/implement-P10-run-phase2-requests.log</t>
         </is>
       </c>
     </row>
@@ -1947,17 +5310,17 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:A5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11">
+  <conditionalFormatting sqref="F11:F12">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11">
+  <conditionalFormatting sqref="G11:G12">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>OR(G11="Critical",G11="High")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G36">
+  <conditionalFormatting sqref="G37:G43">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
@@ -1969,10 +5332,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G11:G12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="G36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G37:G43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(testing): add medication schedule test cases
Sheets "Lịch uống thuốc" (SCHED) and "Tải lịch uống" (SCHEDSYNC) in Test_Cases.xlsx;
Report sheet rebuilt.

Refs: 2.04

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -1,18 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android build" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đăng nhập người dùng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Android build" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Đăng nhập người dùng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Lịch uống thuốc" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tải lịch uống" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Report" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Android build'!$A$8:$I$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Đăng nhập người dùng'!$A$8:$I$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lịch uống thuốc'!$A$8:$I$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Tải lịch uống'!$A$8:$I$29</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -315,13 +319,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -345,18 +349,18 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$12</f>
+              <f>'Report'!$A$11:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$11:$D$12</f>
+              <f>'Report'!$D$11:$D$14</f>
             </numRef>
           </val>
         </ser>
@@ -369,18 +373,18 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$12</f>
+              <f>'Report'!$A$11:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$11:$E$12</f>
+              <f>'Report'!$E$11:$E$14</f>
             </numRef>
           </val>
         </ser>
@@ -393,18 +397,18 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$12</f>
+              <f>'Report'!$A$11:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$11:$F$12</f>
+              <f>'Report'!$F$11:$F$14</f>
             </numRef>
           </val>
         </ser>
@@ -450,13 +454,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -474,7 +478,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -502,12 +506,12 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>16</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -517,9 +521,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -529,7 +533,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>16</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3240000"/>
@@ -539,9 +543,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -4660,7 +4664,4132 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:V54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="8" customWidth="1" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Quản lý lịch uống thuốc (SCHED)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46304</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Kết quả thao tác ghi lịch theo trạng thái thuốc</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="74" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Thêm giờ uống 12:00 cho thuốc theo giờ</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Người bệnh P có consent health_data; thuốc X có lịch 08:00, 20:00 cả tuần</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /medications/{X}/schedules với body
+2. Đọc lịch của X trong DB</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>{"intake_time": "12:00"}</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>201; schedules 08:00, 12:00, 20:00; lịch mới cả tuần, reminder_enabled true, effective_from = thời điểm request; doses_per_day = 3; 08:00, 20:00 giữ id</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>201, đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · EP (1) · Decision Table (R5) · test_add_schedule__AC1[None]</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>intake_time</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>HH:MM 24 giờ, chưa có lịch mở cùng giờ</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>Thiếu
+Sai định dạng (8:00, 7h, 24:00, 12:60)
+Trùng giờ một lịch đang mở khác</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>7
+8
+9</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Thuốc đã ngừng?</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="74" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Thêm giờ uống tắt nhắc</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Như TC-SCHED-01</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /medications/{X}/schedules với body</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>{"intake_time": "12:00", "reminder_enabled": false}</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>201; lịch 12:00 có reminder_enabled false</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>201, reminder_enabled false</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · EP (2) · test_add_schedule__AC1[False]</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>reminder_enabled</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>true
+false
+Không gửi (mặc định true khi thêm)</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>2
+3
+4</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>Chuỗi "false"
+null hoặc số 0</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>10
+11</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>Thuốc as_needed?</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="74" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Thêm giờ trùng một lịch đang mở</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Như TC-SCHED-01</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /medications/{X}/schedules với body
+2. So dữ liệu thuốc, lịch trước và sau</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>{"intake_time": "08:00"}</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail": "schedule_time_conflict"}; không ghi gì</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>422 schedule_time_conflict; DB không đổi</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · EP (5) · Decision Table (R3) · test_add_schedule_rejected_writes_nothing__AC2</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>days_of_week (PATCH /medications/{id})</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>1–7 phần tử, giá trị 1..7, không trùng</t>
+        </is>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>Mảng rỗng
+Giá trị ngoài 1..7
+Phần tử trùng
+Gửi cho thuốc as_needed</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>12
+13
+14
+15</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>Trùng giờ lịch mở?</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U11" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V11" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="74" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Thêm giờ với body sai cấu trúc</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Như TC-SCHED-01</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi lần lượt từng body tới POST /medications/{X}/schedules</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>{} ; {"intake_time": "24:00"} ; {"intake_time": "08:00", "days_of_week": [1]} ; {"intake_time": "09:00", "foo": 1}</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>422, detail là mảng lỗi theo field; không ghi gì</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>422 mảng lỗi cho cả 4 body; DB không đổi</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · EP (3,4) · test_add_schedule_rejected_writes_nothing__AC2</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>schedule_id</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>Lịch đang mở của đúng thuốc</t>
+        </is>
+      </c>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N12" s="10" t="inlineStr">
+        <is>
+          <t>Lịch đã đóng
+Lịch của thuốc khác
+Id không tồn tại</t>
+        </is>
+      </c>
+      <c r="O12" s="10" t="inlineStr">
+        <is>
+          <t>16
+17
+18</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
+        <is>
+          <t>Đã có 6 lịch mở?</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S12" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T12" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V12" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="41" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-BVA-01</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Thêm giờ ở biên dưới và trên của ngày</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Thuốc có lịch 12:00</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /medications/{X}/schedules với 00:00
+2. Lặp lại với thuốc khác và 23:59</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>00:00 ; 23:59</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>201 cả hai</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>201 cả hai (evidence/testcase-bva-manual.log)</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · BVA (min, max) · manual (scratch/bva_check.py)</t>
+        </is>
+      </c>
+      <c r="Q13" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T13" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U13" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="V13" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="74" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-BVA-02</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Thêm giờ ở biên trên + 1</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Như TC-SCHED-01</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /medications/{X}/schedules</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>{"intake_time": "24:00"}</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>422 mảng lỗi</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>422 mảng lỗi</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · BVA (max+1) · test_add_schedule_rejected_writes_nothing__AC2; test_schedule_structural_errors_422_array</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>422 medication_stopped</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S14" s="11" t="inlineStr"/>
+      <c r="T14" s="11" t="inlineStr"/>
+      <c r="U14" s="11" t="inlineStr"/>
+      <c r="V14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="41" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-BVA-03</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Thêm lịch thứ 6 (biên trên số lịch)</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Thuốc có 5 lịch mở</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /medications/{X}/schedules 16:00</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>{"intake_time": "16:00"}</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>201; doses_per_day = 6</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>201; doses_per_day 6 (evidence/testcase-bva-manual.log)</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · BVA (max) · manual (scratch/bva_check.py)</t>
+        </is>
+      </c>
+      <c r="Q15" s="10" t="inlineStr">
+        <is>
+          <t>422 medication_rule_violation</t>
+        </is>
+      </c>
+      <c r="R15" s="11" t="inlineStr"/>
+      <c r="S15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T15" s="11" t="inlineStr"/>
+      <c r="U15" s="11" t="inlineStr"/>
+      <c r="V15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16" ht="57.5" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-BVA-04</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Thêm lịch thứ 7 (biên trên + 1)</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Thuốc có 6 lịch mở</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /medications/{X}/schedules 18:00</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>{"intake_time": "18:00"}</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail": "schedule_limit_reached"}; không ghi gì</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>422 schedule_limit_reached; lịch không đổi</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · BVA (max+1) · Decision Table (R4) · test_add_schedule_limit_reached__AC2</t>
+        </is>
+      </c>
+      <c r="Q16" s="10" t="inlineStr">
+        <is>
+          <t>422 schedule_time_conflict</t>
+        </is>
+      </c>
+      <c r="R16" s="11" t="inlineStr"/>
+      <c r="S16" s="11" t="inlineStr"/>
+      <c r="T16" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U16" s="11" t="inlineStr"/>
+      <c r="V16" s="11" t="inlineStr"/>
+    </row>
+    <row r="17" ht="57.5" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-05</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Thêm giờ cho thuốc dùng khi cần</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Thuốc W as_needed</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /medications/{W}/schedules</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>{"intake_time": "08:00"}</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail": "medication_rule_violation"}; không có lịch</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>422 medication_rule_violation</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · Decision Table (R2) · test_add_schedule_as_needed_422__AC2</t>
+        </is>
+      </c>
+      <c r="Q17" s="10" t="inlineStr">
+        <is>
+          <t>422 schedule_limit_reached</t>
+        </is>
+      </c>
+      <c r="R17" s="11" t="inlineStr"/>
+      <c r="S17" s="11" t="inlineStr"/>
+      <c r="T17" s="11" t="inlineStr"/>
+      <c r="U17" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="V17" s="11" t="inlineStr"/>
+    </row>
+    <row r="18" ht="57.5" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-06</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Ghi lịch của thuốc đã ngừng</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Thuốc X đã ngừng (PATCH stopped true)</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /medications/{X}/schedules
+2. PATCH /medications/{X}/schedules/{S1}
+3. DELETE /medications/{X}/schedules/{S1}</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>12:00 ; {"intake_time": "07:00"} ; (blank)</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Cả ba 422 {"detail": "medication_stopped"}; không ghi gì</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>422 medication_stopped cả ba; DB không đổi</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · Decision Table (R1) · test_stopped_medication_schedule_writes_422__AC8</t>
+        </is>
+      </c>
+      <c r="Q18" s="10" t="inlineStr">
+        <is>
+          <t>201, thêm lịch</t>
+        </is>
+      </c>
+      <c r="R18" s="11" t="inlineStr"/>
+      <c r="S18" s="11" t="inlineStr"/>
+      <c r="T18" s="11" t="inlineStr"/>
+      <c r="U18" s="11" t="inlineStr"/>
+      <c r="V18" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="74" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-07</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Đổi giờ một lịch, lịch cũ đóng chứ không xoá</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>X có S1 08:00, S2 20:00; một liều quá khứ trỏ S1</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH /medications/{X}/schedules/{S1}
+2. Đọc lịch và dose_logs trong DB</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>{"intake_time": "07:00"}</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>200; S1 có ended_at, vẫn còn dòng; lịch 07:00 id mới, effective_from = ended_at(S1), giữ ngày và nhắc; S2 không đổi; doses_per_day 2; liều cũ vẫn trỏ S1</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>200, đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · test_edit_time_versions_schedule_and_keeps_dose_logs__AC3</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="57.5" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-08</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Tắt rồi bật nhắc một giờ</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Như TC-SCHED-07</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH S1 reminder_enabled false
+2. PATCH lịch mới reminder_enabled true</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>{"reminder_enabled": false} ; {"reminder_enabled": true}</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lần 200, đóng lịch cũ và tạo lịch 08:00 id mới với trạng thái nhắc mới; luôn còn 2 lịch mở</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>200 cả hai; 2 lịch mở, 4 dòng lịch</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (1,2) · test_toggle_reminder_versions_schedule__AC4</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="57.5" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-09</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Sửa lịch với giá trị giống hiện tại</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>S2 20:00 nhắc bật</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH /medications/{X}/schedules/{S2} với từng body</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>{"reminder_enabled": true} ; {"intake_time": "20:00"} ; cả hai</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>200; S2 giữ id; DB không đổi</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>200; DB không đổi</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · test_edit_same_values_noop__AC4</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="74" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-10</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Sửa lịch sang giờ trùng lịch khác hoặc body sai</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Như TC-SCHED-07</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH /medications/{X}/schedules/{S1} với từng body</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>{"intake_time": "20:00"} ; {} ; {"intake_time": "7h"} ; {"reminder_enabled": false, "x": 1}</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>422 (schedule_time_conflict cho body đầu, mảng lỗi cho phần còn lại); không ghi gì</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · EP (5,3) · test_edit_invalid_writes_nothing__AC5</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="74" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-11</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Sửa hoặc hủy lịch đã đóng, lịch thuốc khác, id không tồn tại</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>S1 đã bị thay (sau TC-SCHED-07); P có thuốc khác Y</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH và DELETE /medications/{X}/schedules/{id} với từng id</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>S1 (đã đóng) ; lịch của Y ; 4611686018427387904</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>404 {"detail": "medication_schedule_not_found"}; không lịch nào đổi</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>404 cả 6 lần; DB không đổi</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (schedule_id: không hợp lệ) · test_closed_or_foreign_schedule_404_changes_nothing__AC6</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="41" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-12</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Hủy một giờ uống</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>X có S1, S2</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. DELETE /medications/{X}/schedules/{S2}
+2. GET /medications/{X}</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>200; schedules chỉ còn S1; S2 có ended_at; doses_per_day 1; liều không đổi</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>200, đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · test_remove_schedule__AC7</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="41" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-13</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Hủy lịch mở cuối cùng</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>X chỉ còn S1</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. DELETE /medications/{X}/schedules/{S1}</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail": "last_schedule_not_removable"}; lịch vẫn mở</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>422 last_schedule_not_removable</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · test_remove_last_schedule_422__AC8</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="74" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-14</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Đổi ngày uống trong tuần</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>X có S1 08:00 nhắc bật, S2 20:00 nhắc tắt</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH /medications/{X}
+2. Gửi lại cùng ngày
+3. PATCH kèm intake_times</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>{"days_of_week": [5,1,3]} ; [1,3,5] ; {"intake_times": ["09:00"], "days_of_week": [6,7]}</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Lần 1: 200, lịch mới 08:00 và 20:00 ngày [1,3,5], giữ nhắc, cùng effective_from = ended_at lịch cũ; lần 2: không đổi lịch; lần 3: lịch 09:00 ngày [6,7]</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · EP (days: hợp lệ) · test_patch_days_of_week__AC9</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="74" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-15</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Đổi ngày uống với giá trị sai</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Như TC-SCHED-14</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH /medications/{X} với từng body</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>[] ; [8] ; [1,1] ; chuyển sang as_needed kèm days_of_week [1]</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>422 (mảng lỗi, hoặc medication_rule_violation cho body cuối); không ghi gì</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · EP (days: không hợp lệ) · test_patch_days_invalid_writes_nothing__AC9; test_patch_days_on_as_needed_422__AC9</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="57.5" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-BVA-05</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Đổi ngày uống ở biên 1, 7 và 0, 8</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Thuốc có lịch 08:00</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH /medications/{X} với từng giá trị</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>[1] ; [7] ; [0] ; [8]</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>[1], [7]: 200; [0], [8]: 422</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>200, 200, 422, 422 (evidence/testcase-bva-manual.log)</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · BVA (min, max, min-1, max+1) · manual (scratch/bva_check.py)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="41" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-16</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Đổi giờ qua PATCH /medications giữ trạng thái nhắc</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>S2 20:00 đang tắt nhắc</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH /medications/{X}</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>{"intake_times": ["08:00","20:00","22:00"]}</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>08:00 bật, 20:00 tắt, 22:00 bật</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · test_patch_times_keeps_reminder__AC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="57.5" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-17</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Hai request thêm cùng giờ gửi đồng thời</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Như TC-SCHED-01</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi song song hai POST /medications/{X}/schedules 12:00</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>{"intake_time": "12:00"} ×2</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Một 201, một 422; đúng một lịch 12:00 mở; doses_per_day = số lịch mở</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>[201, 422]; một lịch 12:00 (5/5 lần lặp)</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · đoán lỗi (gửi trùng) · test_two_adds_same_time_one_wins__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="41" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-18</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Hủy hai lịch còn lại đồng thời</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>X có S1, S2</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi song song DELETE S1 và DELETE S2</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Một 200, một 422; còn đúng một lịch mở</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>[200, 422]; 1 lịch mở (5/5 lần lặp)</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · test_remove_both_schedules_one_wins__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="57.5" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-19</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Sửa một lịch và đổi ngày đồng thời</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>X có S1, S2</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi song song PATCH S1 07:00 và PATCH /medications/{X} days [2,4]</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>{"intake_time": "07:00"} ; {"days_of_week": [2,4]}</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Không 5xx; đổi ngày 200; sửa lịch 200 hoặc 404; mọi lịch mở có ngày [2,4], không trùng giờ</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng (5/5 lần lặp)</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · test_edit_schedule_and_change_days_serialized__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="41" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-20</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Lỗi giữa chừng khi tạo lịch mới thì không đổi gì</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Giả lập lỗi khi chèn lịch mới</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH S1 07:00
+2. PATCH /medications/{X} days [1]</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>add_schedules ném lỗi</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>500; lịch cũ vẫn mở, không có lịch mới (rollback)</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>500; DB không đổi</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>AC17 · test_failure_after_close_rolls_back__AC17</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="74" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-21</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Sửa lịch có liều đã xác nhận sớm</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Liều của S1 có giờ dự kiến 10 phút sau thời điểm hiện tại đã được ghi (da_uong)</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH S1 tắt nhắc (lần khác: đổi giờ 07:55)
+2. Đọc lịch và liều</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>{"reminder_enabled": false} ; {"intake_time": "07:55"}</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>ended_at(S1) = giờ dự kiến + 1 giây; lịch mới effective_from = ended_at(S1); liều vẫn thuộc S1 và nằm trong [effective_from, ended_at) của S1</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>AC20 · QD-16 · test_early_dose_edit_shifts_boundary__AC20</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="57.5" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-22</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Đổi ngày hoặc đổi giờ cả thuốc khi có liều xác nhận sớm</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Như TC-SCHED-21</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH /medications/{X} days [1,2] (lần khác: intake_times 09:00, 21:00)</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>{"days_of_week": [1,2]} ; {"intake_times": ["09:00","21:00"]}</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>S1 đóng tại giờ dự kiến + 1 giây, S2 đóng sớm hơn; mọi lịch mới bắt đầu tại ended_at(S1)</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>AC20 · test_early_dose_bulk_replace_starts_after_dose__AC20</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="57.5" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-23</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Hủy lịch có liều sớm rồi thêm lại cùng giờ</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Như TC-SCHED-21</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>1. DELETE S1
+2. POST 08:00</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>(blank) ; {"intake_time": "08:00"}</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>ended_at(S1) = giờ dự kiến + 1 giây; lịch 08:00 mới có effective_from = ended_at(S1), không chồng khoảng hiệu lực</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>AC21 · test_delete_then_add_same_time_no_overlap__AC21</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="107" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-24</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Ngừng rồi dùng lại thuốc ngay sau khi có lịch hiệu lực ở tương lai</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Như TC-SCHED-21, S1 vừa được thay bằng lịch tắt nhắc</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH /medications/{X} stopped true
+2. PATCH /medications/{X} stopped false</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>{"stopped": true} ; {"stopped": false}</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Cả hai 200 (không lỗi CHECK); dùng lại mở 08:00 tắt nhắc và 20:00 bật nhắc; lịch 08:00 mới bắt đầu ngay sau giờ dự kiến của liều sớm; liều nằm trong khoảng hiệu lực của lịch nó trỏ tới; không giờ dự kiến nào thuộc hai lịch</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng (vòng 3)</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>AC25 · M1 của review · test_stop_and_reactivate_after_future_replacement</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="90.5" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-25</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Ngừng, chuyển sang khi cần, hoặc xoá thuốc khi có liều xác nhận sớm</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Liều của S1 có giờ dự kiến 10 phút sau thời điểm hiện tại đã được ghi (da_uong); X có S1 08:00, S2 20:00</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH /medications/{X} stopped true (lần khác: chuyển as_needed; DELETE /medications/{X})
+2. Đọc lịch, liều, thuốc trong DB</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>{"stopped": true} ; {"dosing_mode": "as_needed", "max_doses_per_day": 2} ; DELETE</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>ended_at(S1) = giờ dự kiến của liều + 1 giây; S2 đóng tại thời điểm request; liều vẫn nằm trong khoảng hiệu lực của S1; ended_at/deleted_at của thuốc = thời điểm request</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng cả 3 thao tác</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>AC24 · QD-16 · R1 · test_stop_switch_or_delete_after_early_dose_keeps_dose_inside__AC24</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="74" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-26</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Ngừng rồi dùng lại thuốc trước giờ của liều xác nhận sớm</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Liều của S1 có giờ dự kiến 10 phút sau thời điểm hiện tại đã được ghi (da_uong); X có S1 08:00, S2 20:00</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH stopped true
+2. PATCH stopped false
+3. Đọc lịch trong DB</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>{"stopped": true} ; {"stopped": false}</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>200; mở lại 08:00 và 20:00; lịch 08:00 mới bắt đầu tại ended_at(S1) (sau liều); 20:00 bắt đầu tại thời điểm dùng lại; không giờ dự kiến nào thuộc hai lịch</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng (trước khi sửa R1: lịch 08:00 mới phủ giờ của liều, evidence/review-R1-repro.log)</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>AC25 · R1 · test_reactivate_after_early_dose_no_overlap__AC25</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="90.5" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-27</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Chuyển sang khi cần rồi về theo giờ trước giờ của liều xác nhận sớm</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Liều của S1 có giờ dự kiến 10 phút sau thời điểm hiện tại đã được ghi (da_uong); X có S1 08:00, S2 20:00</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH chuyển as_needed
+2. PATCH chuyển scheduled với intake_times 08:00, 20:00</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>{"dosing_mode": "as_needed", "max_doses_per_day": 2} ; {"dosing_mode": "scheduled", "intake_times": ["08:00","20:00"]}</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Lịch 08:00 mới bắt đầu tại ended_at(S1) (sau liều); 20:00 tại thời điểm request; không giờ dự kiến nào thuộc hai lịch</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng (trước khi sửa R1: lịch 08:00 mới phủ giờ của liều)</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>AC26 · R1 · test_back_to_scheduled_after_early_dose_no_overlap__AC26</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="90.5" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-28</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Dùng lại thuốc khi cần đã chuyển từ theo giờ sau liều xác nhận sớm</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Liều của S1 có giờ dự kiến 10 phút sau thời điểm hiện tại đã được ghi (da_uong); X có S1 08:00, S2 20:00</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH chuyển as_needed
+2. PATCH stopped true
+3. PATCH stopped false
+4. Đọc lịch trong DB</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>{"dosing_mode": "as_needed", "max_doses_per_day": 2} ; {"stopped": true} ; {"stopped": false}</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>200; dosing_mode as_needed, status active, schedules []; không có lịch mở trong DB; liều vẫn nằm trong khoảng hiệu lực của S1</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng (trước khi sửa R2: schedules có lịch 08:00 mở, evidence/review-v3-asneeded-repro.log)</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="inlineStr">
+        <is>
+          <t>R2 của review vòng 3 · contract 'Thuốc as_needed: không tạo lịch' · test_reactivate_as_needed_after_early_dose_opens_no_schedule__R2</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="90.5" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-29</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Dùng lại thuốc sau khi đổi cả bộ giờ uống sau liều xác nhận sớm rồi ngừng</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Liều của S1 có giờ dự kiến 10 phút sau thời điểm hiện tại đã được ghi (da_uong); X theo giờ có S1 08:00, S2 20:00 cả tuần, đang dùng</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH /medications/X đổi intake_times
+2. PATCH /medications/X stopped true
+3. PATCH /medications/X stopped false
+4. Đọc response và lịch trong DB</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>{"intake_times": ["07:00", "22:00"]} ; {"stopped": true} ; {"stopped": false}</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>200; schedules gồm đủ 07:00 và 22:00; doses_per_day = 2 = số lịch mở; liều vẫn nằm trong khoảng hiệu lực của S1; không giờ dự kiến nào thuộc hai lịch</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng (trước khi sửa R3: chỉ mở lại 22:00, doses_per_day 2, evidence/review-final-fuzz.log seed 43)</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I42" s="8" t="inlineStr">
+        <is>
+          <t>AC27 · R3 của review vòng 4 · test_reactivate_after_bulk_change_after_early_dose_keeps_all__AC27[intake_times]</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="90.5" customHeight="1">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-30</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Dùng lại thuốc sau khi đổi ngày uống sau liều xác nhận sớm rồi ngừng</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Liều của S1 có giờ dự kiến 10 phút sau thời điểm hiện tại đã được ghi (da_uong); X theo giờ có S1 08:00, S2 20:00 cả tuần, đang dùng</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH /medications/X đổi days_of_week
+2. PATCH /medications/X stopped true
+3. PATCH /medications/X stopped false</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>{"days_of_week": [1, 2]} ; {"stopped": true} ; {"stopped": false}</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>200; schedules 08:00 và 20:00 với days_of_week [1, 2]; doses_per_day = 2; không chồng khoảng hiệu lực</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="inlineStr">
+        <is>
+          <t>AC27 · R3 · test_reactivate_after_bulk_change_after_early_dose_keeps_all__AC27[days_of_week]</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="90.5" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-31</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Dùng lại thuốc sau khi sửa/xóa từng lịch tạo lịch hiệu lực ở tương lai</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Liều của S1 có giờ dự kiến 10 phút sau thời điểm hiện tại đã được ghi (da_uong); X theo giờ có S1 08:00, S2 20:00 cả tuần, đang dùng</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>1. Ca 1: PATCH lịch S1 đổi giờ 07:55, rồi POST thêm 12:00
+2. Ca 2: DELETE lịch S1, rồi POST thêm 08:00
+3. PATCH stopped true, rồi stopped false</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Ca 1: {"intake_time": "07:55"} ; {"intake_time": "12:00"}. Ca 2: {"intake_time": "08:00"}</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>Ca 1: schedules 07:55, 12:00, 20:00, doses_per_day 3. Ca 2: schedules 08:00, 20:00, doses_per_day 2. Liều trong khoảng của S1; không chồng lịch</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng ở cả 2 ca</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I44" s="8" t="inlineStr">
+        <is>
+          <t>AC27 · test_reactivate_after_single_schedule_writes_with_future_schedule__AC27</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="107" customHeight="1">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-32</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Không mở lại lịch đã bị thay trước khi ngừng; chỉ lịch đóng do ngừng mang dấu</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>X theo giờ có S1 08:00, S2 20:00, đang dùng; không có liều sớm</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH lịch S1 đổi giờ 07:00
+2. PATCH /medications/X stopped true
+3. Đọc closed_by_stop_at của các lịch trong DB
+4. PATCH /medications/X stopped false</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>{"intake_time": "07:00"} ; {"stopped": true} ; {"stopped": false}</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>S1 (đóng vì sửa) có closed_by_stop_at NULL; các lịch đóng lúc ngừng có closed_by_stop_at = ended_at của thuốc; dùng lại: schedules 07:00, 20:00, doses_per_day 2; response không có field closed_by_stop_at; lịch mở lại không mang dấu</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I45" s="8" t="inlineStr">
+        <is>
+          <t>AC28 · M3 · test_reactivate_skips_schedules_replaced_before_stop_and_marks__AC28</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="74" customHeight="1">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-33</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Dùng lại thuốc đã ngừng trước khi chạy migration (dữ liệu chưa có dấu)</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>X đã ngừng; dấu closed_by_stop_at của mọi lịch đặt về NULL (giả lập dữ liệu trước migration 20261009065232)</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy câu UPDATE điền dữ liệu của file migration
+2. Kiểm closed_by_stop_at = ended_at của thuốc
+3. PATCH /medications/X stopped false</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>{"stopped": false}</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>Mọi lịch đóng lúc ngừng được đánh dấu lại; 200; schedules 08:00, 20:00; doses_per_day 2 (như hành vi 2.01). supabase db reset chạy hết migration không lỗi</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng; db reset OK (evidence/implement-v4-db-reset.log)</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I46" s="8" t="inlineStr">
+        <is>
+          <t>AC29 · test_backfill_marks_pre_migration_stop__AC29</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="57.5" customHeight="1">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-34</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Chặn dấu đóng do ngừng trên lịch đang mở</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>X có lịch S1 đang mở</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>1. UPDATE medication_schedules SET closed_by_stop_at = now() WHERE id = S1</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>closed_by_stop_at = now(), ended_at NULL</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>DB từ chối: vi phạm medication_schedules_closed_by_stop_chk</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>IntegrityError medication_schedules_closed_by_stop_chk</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I47" s="8" t="inlineStr">
+        <is>
+          <t>AC29 · Đoán lỗi (ràng buộc DB) · test_marker_requires_closed_schedule_check</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="90.5" customHeight="1">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHED-35</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Giữ bất biến lịch trên chuỗi thao tác ngẫu nhiên có seed cố định</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi chuỗi: một thuốc theo giờ mới tạo (08:00, 20:00)</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy 10 bước ngẫu nhiên theo seed: thêm/sửa/xóa từng lịch, bật/tắt nhắc, đổi giờ, đổi ngày, ngừng, dùng lại, chuyển chế độ, ghi liều xác nhận sớm
+2. Sau mỗi bước kiểm bất biến I1–I5</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Seed 0–49 và 96, 97, 178, 198 (gồm 5 seed đã tìm ra R3: 43, 96, 97, 178, 198)</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>I1 không giờ dự kiến thuộc hai lịch; I2 liều trong khoảng của lịch nó trỏ tới; I3 thuốc khi cần/đã ngừng không có lịch mở; I4 doses_per_day = số lịch mở, giờ không trùng; I5 không 5xx</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>54/54 chuỗi giữ bất biến (bản 200 seed ở implement: 200/200; trước khi sửa R3: 195/200)</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I48" s="8" t="inlineStr">
+        <is>
+          <t>AC30 · Chuyển trạng thái (ngẫu nhiên) · test_random_sequences_keep_invariants__AC30</t>
+        </is>
+      </c>
+    </row>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51">
+      <c r="G51" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H51" s="13">
+        <f>COUNTIF(H9:H48,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="G52" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H52" s="13">
+        <f>COUNTIF(H9:H48,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="G53" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H53" s="13">
+        <f>COUNTIF(H9:H48,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="G54" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H54" s="13">
+        <f>SUM(H51:H53)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I48"/>
+  <conditionalFormatting sqref="H9:H48">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:W35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="8" customWidth="1" min="22" max="22"/>
+    <col width="8" customWidth="1" min="23" max="23"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Tải lịch uống và phân quyền dữ liệu thuốc (SCHEDSYNC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46304</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Quyền đọc GET /patients/{patient_id}/schedules</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="W8" s="5" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="90.5" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Người bệnh tải lịch của chính mình</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>P có X (S1, S2 mở; S0 đóng 10 ngày trước; S9 đóng 40 ngày trước), Y đã ngừng, Z đã xoá, W khi cần; người khác có thuốc</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /patients/{P}/schedules</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>(không query)</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>200; items gồm S1, S2, S0, lịch của Y, sắp theo id; không có S9, Z, W, người khác; mỗi phần tử đủ 11 field, ended_at null khi mở; next_cursor null; không ghi access_logs</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · Decision Table (R1) · test_patient_reads_own_schedules__AC12</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>limit</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>1..200
+Không gửi (mặc định 100)</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1
+2</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>0
+201
+Không phải số</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>5
+6
+7</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Người gọi là chính người bệnh?</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="74" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Người bệnh chưa có lịch nào</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>P không có thuốc</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /patients/{P}/schedules</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>200 {"items": [], "next_cursor": null}</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · test_patient_without_schedules_gets_empty_page__AC12</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>cursor</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>next_cursor của trang trước, cùng người bệnh</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>Chuỗi rác
+Base64 không phải JSON hợp lệ
+Con trỏ của người bệnh khác
+Chuỗi rỗng</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>8
+9
+10
+11</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>Consent health_data còn hiệu lực?</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="57.5" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Tải theo trang với limit 2</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>P có 5 lịch</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. GET limit=2
+2. Gửi next_cursor cho tới khi null</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>limit=2</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>3 trang (2, 2, 1); hợp các trang bằng kết quả không phân trang</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>3 trang, đúng thứ tự</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC23 · EP (limit: hợp lệ; cursor: hợp lệ) · test_pagination__AC23</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>UUID của tài khoản tồn tại</t>
+        </is>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>Không phải UUID
+UUID không có tài khoản</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>12
+13</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>Liên kết active + bật chia sẻ + consent family_sharing?</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U11" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W11" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="41" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-BVA-01</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>limit ở biên 1 và 200</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>P có 2 lịch</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. GET limit=1
+2. GET limit=200</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>1 ; 200</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>200; limit 1 trả 1 lịch và có next_cursor; limit 200 trả 2 lịch, next_cursor null</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng (evidence/testcase-bva-manual.log)</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC23 · BVA (min, max) · manual (scratch/bva_check.py)</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
+        <is>
+          <t>Người gọi là admin?</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S12" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T12" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U12" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V12" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="41" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-BVA-02</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>limit ở biên 0 và 201</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>P bất kỳ</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. GET limit=0
+2. GET limit=201</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>0 ; 201</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>422 mảng lỗi</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>422 cả hai</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC23 · BVA (min-1, max+1) · test_limit_out_of_range_422__AC23</t>
+        </is>
+      </c>
+      <c r="Q13" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T13" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U13" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="V13" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="W13" s="5" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="74" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-04</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Con trỏ hỏng hoặc của người bệnh khác</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>P bất kỳ</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. GET với từng cursor</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>!!! ; abc ; eyJhIjoxfQ ; con trỏ mã hoá cho UUID khác</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail": "invalid_cursor"}</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>422 invalid_cursor cả 4</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC23 · EP (cursor: không hợp lệ) · test_bad_cursor_422__AC23; test_cursor_of_other_patient_422__AC23</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>200, không ghi log</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S14" s="11" t="inlineStr"/>
+      <c r="T14" s="11" t="inlineStr"/>
+      <c r="U14" s="11" t="inlineStr"/>
+      <c r="V14" s="11" t="inlineStr"/>
+      <c r="W14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="57.5" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-05</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Người thân hợp lệ tải lịch qua nhiều trang</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>F có liên kết active, bật chia sẻ; P có consent health_data, family_sharing</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. F GET limit=2 tới trang cuối</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>limit=2</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>200 mọi trang; mỗi trang một dòng access_logs allowed, actor_role family</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC13 · Decision Table (R3) · test_family_allowed_logged_each_page__AC13</t>
+        </is>
+      </c>
+      <c r="Q15" s="10" t="inlineStr">
+        <is>
+          <t>403 consent_revoked</t>
+        </is>
+      </c>
+      <c r="R15" s="11" t="inlineStr"/>
+      <c r="S15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T15" s="11" t="inlineStr"/>
+      <c r="U15" s="11" t="inlineStr"/>
+      <c r="V15" s="11" t="inlineStr"/>
+      <c r="W15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16" ht="57.5" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-06</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Admin tải lịch của người bệnh (QD-32)</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Admin không có liên kết với P</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. Admin GET /patients/{P}/schedules</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>403 {"detail": "khong_co_quyen"}; access_logs denied, actor_role admin</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC13 · AC22 · Decision Table (R6) · test_admin_denied_logged__AC13</t>
+        </is>
+      </c>
+      <c r="Q16" s="10" t="inlineStr">
+        <is>
+          <t>200 + access_logs allowed (family)</t>
+        </is>
+      </c>
+      <c r="R16" s="11" t="inlineStr"/>
+      <c r="S16" s="11" t="inlineStr"/>
+      <c r="T16" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U16" s="11" t="inlineStr"/>
+      <c r="V16" s="11" t="inlineStr"/>
+      <c r="W16" s="11" t="inlineStr"/>
+    </row>
+    <row r="17" ht="74" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-07</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Người lạ tải lịch của người bệnh</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Q không có liên kết với P</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Q GET /patients/{P}/schedules</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>403 khong_co_quyen; không lộ items; access_logs denied (actor Q, patient P, scope danh_sach_thuoc)</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC13 · Decision Table (R4) · kịch bản 'truy cập chéo khi không có liên kết' · test_unlinked_user_denied_logged__AC13</t>
+        </is>
+      </c>
+      <c r="Q17" s="10" t="inlineStr">
+        <is>
+          <t>403 khong_co_quyen + access_logs denied</t>
+        </is>
+      </c>
+      <c r="R17" s="11" t="inlineStr"/>
+      <c r="S17" s="11" t="inlineStr"/>
+      <c r="T17" s="11" t="inlineStr"/>
+      <c r="U17" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="V17" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="W17" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="57.5" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-08</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Người thân thiếu consent hoặc bị tắt chia sẻ</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Liên kết có một trong: tắt chia sẻ, thiếu family_sharing, thiếu health_data</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. F GET /patients/{P}/schedules</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>3 trường hợp</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>403; một dòng denied khong_co_quyen</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng cả 3</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC13 · Decision Table (R4, R5) · test_family_missing_consent_or_sharing_off_denied</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="41" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-09</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Người thân đổi patient_id sang người bệnh khác</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>F liên kết với P, không liên kết với R</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. F GET /patients/{R}/schedules</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>patient_id = R</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>403; dòng denied ghi cho R; không có log cho P</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Cross-patient · test_family_swaps_patient_id_denied</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="74" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-10</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Rút quyền giữa hai trang</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>F đã tải trang 1</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. Rút health_data / family_sharing / tắt chia sẻ / hủy liên kết
+2. F gửi trang 2 với next_cursor</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>4 trường hợp</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Trang 2 trả 403; nhật ký: allowed rồi denied</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng cả 4</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC14 · kịch bản 'rút consent hoặc hủy liên kết → 403 ngay' · test_revoke_between_pages_403__AC14</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="41" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-11</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Ghi access log thất bại khi người thân đọc</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Giả lập lỗi ghi access_logs allowed</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. F GET /patients/{P}/schedules</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>append_allowed ném lỗi</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>500; response không chứa dữ liệu lịch</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>500, không có dữ liệu</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Fail-closed · test_allowed_log_failure_fails_request</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="74" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-12</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Người thân, admin, người lạ gọi endpoint ghi lịch</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>X của P</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. POST schedules
+2. PATCH schedule
+3. DELETE schedule
+4. PATCH /medications/{X} days_of_week</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>3 vai × 4 endpoint</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>403 khong_co_quyen cả 4; 4 dòng denied với vai thực tế; X không đổi</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AC15 · test_write_endpoints_denied_for_family_admin_stranger__AC15</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="57.5" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-13</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Người bệnh đã rút consent health_data ghi hoặc đọc lịch</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>P rút health_data</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi 4 endpoint ghi
+2. GET /patients/{P}/schedules</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>403 {"detail": "consent_revoked"}; không ghi gì</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AC15 · Decision Table (R2) · test_self_revoked_consent_cannot_write__AC15</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="57.5" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-14</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>patient_id không ứng với tài khoản nào</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Người dùng thường hoặc admin</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /patients/{UUID ngẫu nhiên}/schedules</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>uuid4 chưa có</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>403 khong_co_quyen; không có dòng access_logs; không 5xx</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng cả hai vai</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>AC16 · EP (patient_id: UUID không có tài khoản) · test_unknown_patient_403_without_log__AC16</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="57.5" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-15</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Gọi không có token hoặc token sai; thuốc đã xoá</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>X của P</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi 4 endpoint không có header và với 'Bearer x'
+2. Xoá X rồi gọi 3 endpoint ghi lịch</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>(blank) ; Bearer x</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>401 khi thiếu hoặc sai token; 404 user_medication_not_found khi thuốc đã xoá</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>AC16 · test_unauthenticated_401_and_unknown_medication_404__AC16</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="57.5" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-16</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>patient_id sai định dạng</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /patients/abc/schedules</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>422 mảng lỗi</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>422 mảng lỗi</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>AC16 · EP (patient_id: không phải UUID) · tests/unit test_patient_id_must_be_uuid</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="57.5" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-17</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Admin xem một thuốc của người bệnh (QD-32)</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>X của P; admin không có liên kết</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. Admin GET /medications/{X}
+2. Admin PATCH /medications/{X}</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>{"quantity_per_dose": 3}</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>403 cả hai; 2 dòng denied actor_role admin</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AC22 · test_admin_get_medication_403_denied__AC22; test_admin_cannot_read_or_write__AC15_QD32</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="57.5" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-18</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Admin xác nhận liều hộ (QD-32)</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Lịch S1 của P; admin không có liên kết</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. Admin POST /doses/batch với một liều của S1</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>schedule_id = S1, scheduled_at = 5 phút trước</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>200; item result failed, http_status 403; không có dose_logs; access_logs denied admin, scope lich_su_tuan_thu</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như kỳ vọng</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AC22 · test_admin_dose_batch_rejected__AC22</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="57.5" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-SCHEDSYNC-19</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>App người thân không lưu lịch xuống máy (QD-29)</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>App mobile của người thân đã nối GET /patients/{id}/schedules</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. Người thân mở lịch của người bệnh
+2. Tắt mạng, đóng và mở lại app
+3. Kiểm tra CSDL cục bộ</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Không có lịch của người bệnh trong CSDL cục bộ; chỉ giữ trong phiên</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr"/>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>QD-29 · manual · cần app mobile (chưa có task nối API)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32">
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H32" s="13">
+        <f>COUNTIF(H9:H29,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H33" s="13">
+        <f>COUNTIF(H9:H29,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="G34" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H34" s="13">
+        <f>COUNTIF(H9:H29,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H35" s="13">
+        <f>SUM(H32:H34)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I29"/>
+  <conditionalFormatting sqref="H9:H29">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4705,7 +8834,7 @@
         </is>
       </c>
       <c r="C3" s="11">
-        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59</f>
+        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59+'Lịch uống thuốc'!$H$51+'Tải lịch uống'!$H$32</f>
         <v/>
       </c>
       <c r="D3" s="15">
@@ -4721,7 +8850,7 @@
         </is>
       </c>
       <c r="C4" s="11">
-        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60</f>
+        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60+'Lịch uống thuốc'!$H$52+'Tải lịch uống'!$H$33</f>
         <v/>
       </c>
       <c r="D4" s="15">
@@ -4753,7 +8882,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr"/>
       <c r="C6" s="11">
-        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61</f>
+        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61+'Lịch uống thuốc'!$H$53+'Tải lịch uống'!$H$34</f>
         <v/>
       </c>
       <c r="D6" s="15">
@@ -4912,393 +9041,481 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="19" t="inlineStr">
+    <row r="13" ht="222.5" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Quản lý lịch uống thuốc</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Backend API thêm, sửa, hủy từng giờ uống; bật/tắt nhắc; đổi ngày uống trong tuần; mốc hiệu lực khi có liều xác nhận sớm (QD-16). Chỉ chính người bệnh được ghi.</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Lịch uống thuốc</t>
+        </is>
+      </c>
+      <c r="D13" s="18">
+        <f>IFERROR(('Lịch uống thuốc'!$H$54-'Lịch uống thuốc'!$H$53)/'Lịch uống thuốc'!$H$54,0)</f>
+        <v/>
+      </c>
+      <c r="E13" s="18">
+        <f>IFERROR('Lịch uống thuốc'!$H$51/'Lịch uống thuốc'!$H$54,0)</f>
+        <v/>
+      </c>
+      <c r="F13" s="18">
+        <f>IFERROR('Lịch uống thuốc'!$H$52/'Lịch uống thuốc'!$H$54,0)</f>
+        <v/>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động và kiểm tra biên đạt trên Supabase local. Đã sửa và có test cho các lỗi review R1 (sinh trùng liều khi ngừng/dùng lại sau liều xác nhận sớm), R2 (dùng lại thuốc khi cần mở lịch cũ), R3 (dùng lại mất lịch sau khi đổi cả bộ giờ/ngày sau liều sớm; sửa bằng migration closed_by_stop_at) và M3 (doses_per_day sau khi dùng lại). Có test bất biến trên chuỗi thao tác ngẫu nhiên. Chưa phủ: race giữa xác nhận liều sớm và sửa lịch (2.10).</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="90.5" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Tải lịch uống và phân quyền dữ liệu thuốc</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>GET /patients/{patient_id}/schedules (lịch đang mở và đóng trong 30 ngày, phân trang con trỏ); phân quyền ghi lịch; QD-32 admin không đọc dữ liệu y tế; patient_id không tồn tại.</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Tải lịch uống</t>
+        </is>
+      </c>
+      <c r="D14" s="18">
+        <f>IFERROR(('Tải lịch uống'!$H$35-'Tải lịch uống'!$H$34)/'Tải lịch uống'!$H$35,0)</f>
+        <v/>
+      </c>
+      <c r="E14" s="18">
+        <f>IFERROR('Tải lịch uống'!$H$32/'Tải lịch uống'!$H$35,0)</f>
+        <v/>
+      </c>
+      <c r="F14" s="18">
+        <f>IFERROR('Tải lịch uống'!$H$33/'Tải lịch uống'!$H$35,0)</f>
+        <v/>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ ca phân quyền đạt, mỗi ca kiểm cả response lẫn access_logs. Quy tắc QD-29 (app người thân không lưu xuống máy) là quy tắc client, chưa kiểm được ở backend.</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="19" t="inlineStr">
         <is>
           <t>Bug Report</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="20" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="20" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="B36" s="20" t="inlineStr">
+      <c r="B38" s="20" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C36" s="20" t="inlineStr">
+      <c r="C38" s="20" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="D36" s="20" t="inlineStr">
+      <c r="D38" s="20" t="inlineStr">
         <is>
           <t>Input Data</t>
         </is>
       </c>
-      <c r="E36" s="20" t="inlineStr">
+      <c r="E38" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F36" s="20" t="inlineStr">
+      <c r="F38" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="G36" s="20" t="inlineStr">
+      <c r="G38" s="20" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="H36" s="20" t="inlineStr">
+      <c r="H38" s="20" t="inlineStr">
         <is>
           <t>Name of Tester</t>
         </is>
       </c>
-      <c r="I36" s="20" t="inlineStr">
+      <c r="I38" s="20" t="inlineStr">
         <is>
           <t>Logs</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="123.5" customHeight="1">
-      <c r="A37" s="22" t="inlineStr">
+    <row r="39" ht="123.5" customHeight="1">
+      <c r="A39" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-08</t>
         </is>
       </c>
-      <c r="B37" s="22" t="inlineStr">
+      <c r="B39" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
         </is>
       </c>
-      <c r="C37" s="22" t="inlineStr">
+      <c r="C39" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
 2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
         </is>
       </c>
-      <c r="D37" s="22" t="inlineStr">
+      <c r="D39" s="22" t="inlineStr">
         <is>
           <t>phone: 0900000001 + ký tự \n</t>
         </is>
       </c>
-      <c r="E37" s="22" t="inlineStr">
+      <c r="E39" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F37" s="22" t="inlineStr">
+      <c r="F39" s="22" t="inlineStr">
         <is>
           <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
         </is>
       </c>
-      <c r="G37" s="22" t="inlineStr">
+      <c r="G39" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H37" s="22" t="inlineStr">
+      <c r="H39" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I37" s="22" t="inlineStr">
+      <c r="I39" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn — kỳ vọng AC6 mâu thuẫn AC5: backend `_validate_required_text` (sign_in.py:178) `strip()` mọi ký tự trắng hai đầu, nên \n cuối được xử lý như khoảng trắng hai đầu mà AC5 coi là hợp lệ. Cần người dùng chốt: sửa AC6 hoặc sửa backend
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="123.5" customHeight="1">
-      <c r="A38" s="22" t="inlineStr">
+    <row r="40" ht="123.5" customHeight="1">
+      <c r="A40" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-11</t>
         </is>
       </c>
-      <c r="B38" s="22" t="inlineStr">
+      <c r="B40" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
         </is>
       </c>
-      <c r="C38" s="22" t="inlineStr">
+      <c r="C40" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone}
 2. POST /auth/mobile/verify {phone, token: 123456}</t>
         </is>
       </c>
-      <c r="D38" s="22" t="inlineStr">
+      <c r="D40" s="22" t="inlineStr">
         <is>
           <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
         </is>
       </c>
-      <c r="E38" s="22" t="inlineStr">
+      <c r="E40" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
         </is>
       </c>
-      <c r="F38" s="22" t="inlineStr">
+      <c r="F40" s="22" t="inlineStr">
         <is>
           <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
         </is>
       </c>
-      <c r="G38" s="22" t="inlineStr">
+      <c r="G40" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H38" s="22" t="inlineStr">
+      <c r="H40" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I38" s="22" t="inlineStr">
+      <c r="I40" s="22" t="inlineStr">
         <is>
           <t>`_normalize_phone` (sign_in.py:197–206) kiểm bằng `str.isdigit()`, nhận cả chữ số Unicode, nên số lọt qua kiểm tra và gửi tới Supabase. Ô nhập của app chỉ cho 0-9 nên người dùng app không gặp; lỗi ở tầng API
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="189.5" customHeight="1">
-      <c r="A39" s="22" t="inlineStr">
+    <row r="41" ht="189.5" customHeight="1">
+      <c r="A41" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-25</t>
         </is>
       </c>
-      <c r="B39" s="22" t="inlineStr">
+      <c r="B41" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên có ký tự NUL</t>
         </is>
       </c>
-      <c r="C39" s="22" t="inlineStr">
+      <c r="C41" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
         </is>
       </c>
-      <c r="D39" s="22" t="inlineStr">
+      <c r="D41" s="22" t="inlineStr">
         <is>
           <t>ho_ten: abc\u0000def</t>
         </is>
       </c>
-      <c r="E39" s="22" t="inlineStr">
+      <c r="E41" s="22" t="inlineStr">
         <is>
           <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
         </is>
       </c>
-      <c r="F39" s="22" t="inlineStr">
+      <c r="F41" s="22" t="inlineStr">
         <is>
           <t>500 Internal Server Error</t>
         </is>
       </c>
-      <c r="G39" s="22" t="inlineStr">
+      <c r="G41" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H39" s="22" t="inlineStr">
+      <c r="H41" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I39" s="22" t="inlineStr">
+      <c r="I41" s="22" t="inlineStr">
         <is>
           <t>`_validate_required_text` (sign_in.py:178) không chặn ký tự điều khiển; PostgreSQL từ chối NUL trong cột text: `psycopg.DataError: PostgreSQL text fields cannot contain NUL (0x00) bytes` ở `UPDATE users SET full_name…` (SqlUsers.update_profile); không có handler cho DataError nên thành 500. Câu SQL có tham số nên không phải lỗ hổng SQL injection
 Log: evidence/test-integration.log, evidence/test-probe-nul.log</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="90.5" customHeight="1">
-      <c r="A40" s="22" t="inlineStr">
+    <row r="42" ht="90.5" customHeight="1">
+      <c r="A42" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-30</t>
         </is>
       </c>
-      <c r="B40" s="22" t="inlineStr">
+      <c r="B42" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên dài 256 ký tự</t>
         </is>
       </c>
-      <c r="C40" s="22" t="inlineStr">
+      <c r="C42" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: A*256}</t>
         </is>
       </c>
-      <c r="D40" s="22" t="inlineStr">
+      <c r="D42" s="22" t="inlineStr">
         <is>
           <t>A*256</t>
         </is>
       </c>
-      <c r="E40" s="22" t="inlineStr">
+      <c r="E42" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F40" s="22" t="inlineStr">
+      <c r="F42" s="22" t="inlineStr">
         <is>
           <t>204, đã lưu</t>
         </is>
       </c>
-      <c r="G40" s="22" t="inlineStr">
+      <c r="G42" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H40" s="22" t="inlineStr">
+      <c r="H42" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I40" s="22" t="inlineStr">
+      <c r="I42" s="22" t="inlineStr">
         <is>
           <t>Không có giới hạn độ dài họ tên: `_validate_profile` (sign_in.py) chỉ kiểm rỗng; cột users.full_name kiểu text không giới hạn
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="90.5" customHeight="1">
-      <c r="A41" s="22" t="inlineStr">
+    <row r="43" ht="90.5" customHeight="1">
+      <c r="A43" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-32</t>
         </is>
       </c>
-      <c r="B41" s="22" t="inlineStr">
+      <c r="B43" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh trước 1900-01-01</t>
         </is>
       </c>
-      <c r="C41" s="22" t="inlineStr">
+      <c r="C43" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh}</t>
         </is>
       </c>
-      <c r="D41" s="22" t="inlineStr">
+      <c r="D43" s="22" t="inlineStr">
         <is>
           <t>1899-12-31 | 0001-01-01</t>
         </is>
       </c>
-      <c r="E41" s="22" t="inlineStr">
+      <c r="E43" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
         </is>
       </c>
-      <c r="F41" s="22" t="inlineStr">
+      <c r="F43" s="22" t="inlineStr">
         <is>
           <t>204 ở cả hai giá trị, đã lưu</t>
         </is>
       </c>
-      <c r="G41" s="22" t="inlineStr">
+      <c r="G43" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H41" s="22" t="inlineStr">
+      <c r="H43" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I41" s="22" t="inlineStr">
+      <c r="I43" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:229–231) chỉ chặn ngày tương lai, không có cận dưới. App mobile đã giới hạn date picker từ 1900 nên chỉ gặp khi gọi API trực tiếp
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="123.5" customHeight="1">
-      <c r="A42" s="22" t="inlineStr">
+    <row r="44" ht="123.5" customHeight="1">
+      <c r="A44" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-35</t>
         </is>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B44" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
         </is>
       </c>
-      <c r="C42" s="22" t="inlineStr">
+      <c r="C44" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
         </is>
       </c>
-      <c r="D42" s="22" t="inlineStr">
+      <c r="D44" s="22" t="inlineStr">
         <is>
           <t>ngay_sinh: 2026-10-08</t>
         </is>
       </c>
-      <c r="E42" s="22" t="inlineStr">
+      <c r="E44" s="22" t="inlineStr">
         <is>
           <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
         </is>
       </c>
-      <c r="F42" s="22" t="inlineStr">
+      <c r="F44" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_date_of_birth"}</t>
         </is>
       </c>
-      <c r="G42" s="22" t="inlineStr">
+      <c r="G44" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H42" s="22" t="inlineStr">
+      <c r="H44" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I42" s="22" t="inlineStr">
+      <c r="I44" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:230) so với `now.date()` trong khi `now()` (shared/clock.py) trả giờ UTC: từ 00:00 đến 07:00 giờ VN, "hôm nay" bị coi là ngày mai. Vi phạm bất biến 7 (múi giờ cố định Asia/Ho_Chi_Minh)
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="173" customHeight="1">
-      <c r="A43" s="22" t="inlineStr">
+    <row r="45" ht="173" customHeight="1">
+      <c r="A45" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-42</t>
         </is>
       </c>
-      <c r="B43" s="22" t="inlineStr">
+      <c r="B45" s="22" t="inlineStr">
         <is>
           <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
         </is>
       </c>
-      <c r="C43" s="22" t="inlineStr">
+      <c r="C45" s="22" t="inlineStr">
         <is>
           <t>1. Chạm vào ô mã OTP
 2. Theo dõi request backend nhận được</t>
         </is>
       </c>
-      <c r="D43" s="22" t="inlineStr">
+      <c r="D45" s="22" t="inlineStr">
         <is>
           <t>Ô đang chứa 000000</t>
         </is>
       </c>
-      <c r="E43" s="22" t="inlineStr">
+      <c r="E45" s="22" t="inlineStr">
         <is>
           <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
         </is>
       </c>
-      <c r="F43" s="22" t="inlineStr">
+      <c r="F45" s="22" t="inlineStr">
         <is>
           <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
         </is>
       </c>
-      <c r="G43" s="22" t="inlineStr">
+      <c r="G45" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H43" s="22" t="inlineStr">
+      <c r="H45" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I43" s="22" t="inlineStr">
+      <c r="I45" s="22" t="inlineStr">
         <is>
           <t>`OtpPinInput._handleTextChange` (frontend/mobile/lib/features/auth/presentation/widgets/otp_pin_input.dart:66–72) chạy với mọi thông báo của controller, kể cả khi chỉ đổi vị trí con trỏ lúc chạm ô, và gọi onCompleted hễ ô đủ 6 số → gửi lại mã sai, tốn hạn mức token_verifications
 Log: evidence/test-e2e.log (mục "request backend trong pha 2"), evidence/implement-P10-run-phase2-requests.log</t>
@@ -5310,17 +9527,17 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:A5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11:F12">
+  <conditionalFormatting sqref="F11:F14">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11:G12">
+  <conditionalFormatting sqref="G11:G14">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>OR(G11="Critical",G11="High")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G37:G43">
+  <conditionalFormatting sqref="G39:G45">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
@@ -5332,10 +9549,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G11:G12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G11:G14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="G37:G43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G39:G45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(testing): add interaction catalog CRUD test cases
Refs: 2.16

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -10,13 +10,19 @@
     <sheet name="Đăng nhập người dùng" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Lịch uống thuốc" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Tải lịch uống" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Report" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Tương tác thuốc-thuốc" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Tương tác thuốc-thực phẩm" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Tra cứu hoạt chất" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Report" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Android build'!$A$8:$I$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Đăng nhập người dùng'!$A$8:$I$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lịch uống thuốc'!$A$8:$I$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Tải lịch uống'!$A$8:$I$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tương tác thuốc-thuốc'!$A$8:$I$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Tương tác thuốc-thực phẩm'!$A$8:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Tra cứu hoạt chất'!$A$8:$I$14</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -355,12 +361,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$14</f>
+              <f>'Report'!$A$11:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$11:$D$14</f>
+              <f>'Report'!$D$11:$D$17</f>
             </numRef>
           </val>
         </ser>
@@ -379,12 +385,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$14</f>
+              <f>'Report'!$A$11:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$11:$E$14</f>
+              <f>'Report'!$E$11:$E$17</f>
             </numRef>
           </val>
         </ser>
@@ -403,12 +409,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$14</f>
+              <f>'Report'!$A$11:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$11:$F$14</f>
+              <f>'Report'!$F$11:$F$17</f>
             </numRef>
           </val>
         </ser>
@@ -511,7 +517,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>16</row>
+      <row>19</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -533,7 +539,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>16</row>
+      <row>19</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3240000"/>
@@ -8789,7 +8795,3860 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:U55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Danh mục tương tác thuốc-thuốc (admin) (DDIRULE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46307</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Quyền gọi endpoint /admin/drug-interactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="107" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Tạo quy tắc chống chỉ định giữa hai hoạt chất trong danh mục</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập admin (phiên admin_web); hoạt chất X, Y có trong danh mục</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /admin/drug-interactions với A = X, B = Y, chong_chi_dinh, mức 4, tranh_phoi_hop, mô tả, nguồn
+2. Kiểm dòng DB của phiên bản vừa tạo</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>{ingredient_a_id: X, ingredient_b_id: Y, interaction_type: chong_chi_dinh, severity_level: 4, handling_type: tranh_phoi_hop}</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>201; version = 1, state = current; ingredient_a/ingredient_b có id và standard_name; verification_status = da_xac_minh; updated_by.id = admin. DB: ingredient_b_in_table_a = co, deleted_at rỗng, created_by = admin</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>201 và các giá trị đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · EP (1) · test_create_with_catalog_ingredient_b__AC1</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>Hoạt chất B</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>ingredient_b_id có trong danh mục, khác A
+ingredient_b_external_name (chất ngoài danh mục)</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1
+2</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>gửi cả hai
+không gửi cả hai
+id không tồn tại
+B trùng A</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>9
+10
+11
+12</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Có token hợp lệ?</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="57.5" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Tạo quy tắc với hoạt chất B là chất ngoài danh mục</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Admin; hoạt chất X có trong danh mục</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /admin/drug-interactions với ingredient_b_external_name = "Rượu", không gửi ingredient_b_id</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>ingredient_b_external_name: Rượu</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>201; ingredient_b = null, ingredient_b_external_name = Rượu; DB: ingredient_b_id rỗng, ingredient_b_in_table_a = khong</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>201, DB đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · EP (2) · test_create_with_external_ingredient_b__AC2</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>severity_level</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>1–4</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>&lt; 1
+&gt; 4
+chong_chi_dinh mà khác 4</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>13
+14
+15</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>system_role = admin?</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="107" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Tạo, thay và giữ ngưỡng liều của quy tắc phụ thuộc liều</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Admin; hoạt chất X, Y</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. POST với 2 ngưỡng (A 0–100 mg/ngày mức 2; B ≥300 mg/ngày mức 4)
+2. GET /admin/drug-interactions/{id}
+3. PATCH gửi dose_thresholds 1 ngưỡng (A 50–60)
+4. PATCH chỉ đổi description</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>dose_thresholds như bước</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>GET trả đủ 2 ngưỡng; sau PATCH thứ nhất chỉ còn ngưỡng 50–60; sau PATCH thứ hai ngưỡng giữ nguyên</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · test_dose_thresholds_create_replace_keep__AC3</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>min_interval_hours</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>null
+0 &lt; số giờ ≤ 168 với cach_gio</t>
+        </is>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>4
+5</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>≤ 0
+&gt; 168
+có giá trị mà handling_type khác cach_gio</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>16
+17
+18</t>
+        </is>
+      </c>
+      <c r="Q11" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T11" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="123.5" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối tạo quy tắc có A trùng B</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Admin; hoạt chất X</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. POST với ingredient_a_id = ingredient_b_id = X
+2. Đếm quy tắc và ngưỡng chạm X</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>A = B = X</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail": "same_ingredient"}; không có dòng mới</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>422 same_ingredient; số dòng không đổi</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (12) · test_validation_errors_write_nothing__AC4</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>dose_thresholds</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>0–20 ngưỡng hợp lệ với phu_thuoc_lieu</t>
+        </is>
+      </c>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N12" s="10" t="inlineStr">
+        <is>
+          <t>&gt; 20 ngưỡng
+min_dose &gt; max_dose
+thiếu cả min và max
+liều âm
+ingredient_ref = B khi B ngoài danh mục
+có ngưỡng với chong_chi_dinh</t>
+        </is>
+      </c>
+      <c r="O12" s="10" t="inlineStr">
+        <is>
+          <t>19
+20
+21
+22
+23
+24</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S12" s="11" t="inlineStr"/>
+      <c r="T12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13" ht="41" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối tạo quy tắc với id hoạt chất không tồn tại</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. POST với ingredient_b_id = 2000000000</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>ingredient_b_id: 2000000000</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail": "active_ingredient_not_found"}; không có dòng mới</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>422 active_ingredient_not_found</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (11) · test_validation_errors_write_nothing__AC4</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>verification_status (request)</t>
+        </is>
+      </c>
+      <c r="L13" s="10" t="inlineStr">
+        <is>
+          <t>không gửi</t>
+        </is>
+      </c>
+      <c r="M13" s="10" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="N13" s="10" t="inlineStr">
+        <is>
+          <t>gửi bất kỳ giá trị</t>
+        </is>
+      </c>
+      <c r="O13" s="10" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="Q13" s="10" t="inlineStr">
+        <is>
+          <t>403 admin_only, không ghi gì</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="inlineStr"/>
+      <c r="S13" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="41" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối gửi cả ingredient_b_id và ingredient_b_external_name</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Admin; X, Y</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. POST với cả ingredient_b_id = Y và ingredient_b_external_name = Rượu</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>cả hai field B</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>422 ValidationError (detail là mảng lỗi theo field); không có dòng mới</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>422 ValidationError</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (9) · test_validation_errors_write_nothing__AC4</t>
+        </is>
+      </c>
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>expected_version (PATCH/DELETE)</t>
+        </is>
+      </c>
+      <c r="L14" s="10" t="inlineStr">
+        <is>
+          <t>bằng phiên bản hiện hành</t>
+        </is>
+      </c>
+      <c r="M14" s="10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="N14" s="10" t="inlineStr">
+        <is>
+          <t>phiên bản cũ
+thiếu</t>
+        </is>
+      </c>
+      <c r="O14" s="10" t="inlineStr">
+        <is>
+          <t>26
+27</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>Xử lý theo nghiệp vụ</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr"/>
+      <c r="S14" s="11" t="inlineStr"/>
+      <c r="T14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="41" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối không gửi hoạt chất B</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Admin; X</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. POST không có ingredient_b_id lẫn ingredient_b_external_name</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>thiếu B</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>422 ValidationError</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>422 ValidationError</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (10) · test_create_without_b_422 (unit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="41" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối chống chỉ định với mức độ khác 4</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Admin; X, Y</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. POST interaction_type = chong_chi_dinh, severity_level = 2</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>chong_chi_dinh, mức 2</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail": "contraindication_severity_mismatch"}</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>422 contraindication_severity_mismatch</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (15) · test_validation_errors_write_nothing__AC4</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="41" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối chống chỉ định kèm ngưỡng liều</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Admin; X, Y</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. POST chong_chi_dinh, mức 4, có 1 ngưỡng</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>chong_chi_dinh + dose_thresholds[1]</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail": "threshold_not_allowed"}</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>422 threshold_not_allowed</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (24) · test_validation_errors_write_nothing__AC4</t>
+        </is>
+      </c>
+      <c r="Q17" s="4" t="inlineStr">
+        <is>
+          <t>Kết quả PATCH theo phiên bản và nội dung</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="41" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối ngưỡng có min_dose lớn hơn max_dose</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Admin; X, Y</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. POST với ngưỡng min_dose = 100, max_dose = 50</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>min 100, max 50</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail": "threshold_range_invalid"}</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>422 threshold_range_invalid</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (20) · test_validation_errors_write_nothing__AC4</t>
+        </is>
+      </c>
+      <c r="Q18" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R18" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S18" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T18" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U18" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="41" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối ngưỡng thiếu cả min_dose và max_dose</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Admin; X, Y</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. POST với ngưỡng không có min_dose, max_dose</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>ngưỡng không có khoảng liều</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>422 ValidationError</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>422 ValidationError</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (21) · test_validation_errors_write_nothing__AC4</t>
+        </is>
+      </c>
+      <c r="Q19" s="10" t="inlineStr">
+        <is>
+          <t>Quy tắc tồn tại, chưa xóa?</t>
+        </is>
+      </c>
+      <c r="R19" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S19" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T19" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U19" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="41" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối ngưỡng có liều âm</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Admin; X, Y</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. POST với ngưỡng min_dose = -1</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>min_dose: -1</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>422 ValidationError</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>422 ValidationError</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (22) · test_create_structure_errors_422 (unit)</t>
+        </is>
+      </c>
+      <c r="Q20" s="10" t="inlineStr">
+        <is>
+          <t>expected_version = hiện hành?</t>
+        </is>
+      </c>
+      <c r="R20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S20" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T20" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U20" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="57.5" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-13</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối ngưỡng cho hoạt chất B khi B là chất ngoài danh mục</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Admin; X</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. POST B = Rượu (tên ngoài), ngưỡng ingredient_ref = B
+2. Đếm dòng chạm X</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>ingredient_ref: B</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail": "threshold_ref_invalid"}; không có dòng mới</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>422 threshold_ref_invalid; 0 dòng</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (23) · test_threshold_for_external_b_rejected__AC4</t>
+        </is>
+      </c>
+      <c r="Q21" s="10" t="inlineStr">
+        <is>
+          <t>Nội dung khác hiện hành?</t>
+        </is>
+      </c>
+      <c r="R21" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S21" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T21" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U21" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="74" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-14</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối gửi verification_status khi tạo và khi sửa</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Admin; X, Y</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. POST có verification_status = cho_duyet
+2. Tạo quy tắc hợp lệ rồi PATCH có verification_status
+3. Đọc verification_status trong DB</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>verification_status: cho_duyet / x</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Cả hai 422 ValidationError; DB chỉ có da_xac_minh</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>422 cả hai; DB = [da_xac_minh]</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AC15, AC16 · EP (25) · test_verification_status_not_writable__AC15_AC16</t>
+        </is>
+      </c>
+      <c r="Q22" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R22" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S22" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T22" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U22" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="41" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Báo trùng khi tạo cặp hoạt chất đảo thứ tự hoặc tên ngoài khác hoa thường</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Admin; đã có quy tắc (X, Y) và (X, "Rượu")</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. POST (Y, X)
+2. POST (X, "rượu")</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>cặp đảo chiều; tên ngoài viết thường</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>409 {"detail": "interaction_rule_exists"} cho cả hai; không có dòng mới</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>409 interaction_rule_exists; vẫn 2 quy tắc</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · Đoán lỗi · test_duplicate_pair_conflict__AC5</t>
+        </is>
+      </c>
+      <c r="Q23" s="10" t="inlineStr">
+        <is>
+          <t>404 interaction_rule_not_found</t>
+        </is>
+      </c>
+      <c r="R23" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S23" s="11" t="inlineStr"/>
+      <c r="T23" s="11" t="inlineStr"/>
+      <c r="U23" s="11" t="inlineStr"/>
+    </row>
+    <row r="24" ht="74" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-16</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Hai request tạo cùng cặp chạy đồng thời chỉ một thành công</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Admin; X, Y chưa có quy tắc; một giao dịch khác đang giữ cặp (X, Y) chưa commit</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi đồng thời POST (X, Y) và POST (Y, X)
+2. Chờ tới khi cả hai đang chờ khóa DB
+3. Rollback giao dịch đang giữ
+4. Đếm quy tắc mở của cặp</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>2 request song song</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Một 201, một 409; đúng 1 quy tắc mở cho cặp</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>[201, 409]; 1 quy tắc</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · Chạy đua · test_concurrent_create_one_wins__AC6</t>
+        </is>
+      </c>
+      <c r="Q24" s="10" t="inlineStr">
+        <is>
+          <t>409 version_conflict</t>
+        </is>
+      </c>
+      <c r="R24" s="11" t="inlineStr"/>
+      <c r="S24" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T24" s="11" t="inlineStr"/>
+      <c r="U24" s="11" t="inlineStr"/>
+    </row>
+    <row r="25" ht="107" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-17</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Xóa mềm quy tắc: ẩn khỏi danh sách, giữ dòng và ngưỡng, tạo lại được</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Admin; quy tắc Q (phiên bản 1, 1 ngưỡng)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. DELETE /admin/drug-interactions/{id}?expected_version=1
+2. Kiểm DB
+3. GET, PATCH, DELETE lại Q
+4. GET danh sách lọc theo X
+5. POST lại cùng cặp</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>expected_version: 1</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>204 rỗng; DB còn dòng, deleted_at và deleted_by = admin, ngưỡng còn; GET/PATCH/DELETE 404 interaction_rule_not_found; danh sách rỗng; tạo lại 201 với mã mới</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>AC7, AC24 · Chuyển trạng thái (current → deleted) · test_soft_delete_hides_keeps_rows_and_allows_recreate__AC7</t>
+        </is>
+      </c>
+      <c r="Q25" s="10" t="inlineStr">
+        <is>
+          <t>200, giữ phiên bản</t>
+        </is>
+      </c>
+      <c r="R25" s="11" t="inlineStr"/>
+      <c r="S25" s="11" t="inlineStr"/>
+      <c r="T25" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U25" s="11" t="inlineStr"/>
+    </row>
+    <row r="26" ht="123.5" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-18</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Lọc, phân trang và sắp xếp danh sách quy tắc</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Admin; 3 quy tắc chạm hoạt chất Alpha (một ở vị trí B), 1 quy tắc tên ngoài; thuốc phối hợp chứa hai hoạt chất</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. GET ?ingredient_id=Alpha
+2. Thêm severity_level, interaction_type
+3. limit=2, skip=2
+4. q viết hoa khác tên
+5. q theo tên ngoài
+6. medication_id của thuốc phối hợp và của thuốc chưa có hoạt chất</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>các bộ lọc như bước</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ các quy tắc mở khớp lọc; mới sửa trước; total không tính phân trang; q không phân biệt hoa thường; medication_id khớp bất kỳ hoạt chất của thuốc; thuốc chưa có hoạt chất → rỗng</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>AC8, AC26 · test_list_filters_paging_total_order__AC8_AC26</t>
+        </is>
+      </c>
+      <c r="Q26" s="10" t="inlineStr">
+        <is>
+          <t>200, phiên bản mới, bản cũ superseded</t>
+        </is>
+      </c>
+      <c r="R26" s="11" t="inlineStr"/>
+      <c r="S26" s="11" t="inlineStr"/>
+      <c r="T26" s="11" t="inlineStr"/>
+      <c r="U26" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="123.5" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-19</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Sửa nội dung giữ field khác; không đổi được cặp hoạt chất</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Admin; quy tắc phụ thuộc liều có 1 ngưỡng</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH expected_version=1, severity_level=3, description
+2. PATCH gửi ingredient_a_id / ingredient_b_id / ingredient_b_external_name
+3. PATCH đổi sang chong_chi_dinh mức 4 khi còn ngưỡng
+4. PATCH như trên kèm dose_thresholds: []</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>như bước</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>200 với 2 field đổi, field khác giữ; đổi cặp 422 ValidationError; còn ngưỡng 422 threshold_not_allowed; kèm [] thì 200 và không còn ngưỡng</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · test_patch_content_and_reject_pair_change__AC9</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="90.5" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-20</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Chặn người chưa đăng nhập và tài khoản không phải admin</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>User thường; không token</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi lần lượt mọi endpoint /admin/drug-interactions..., /admin/drug-food-interactions, /admin/active-ingredients không token
+2. Gọi lại bằng phiên của user thường
+3. Đếm access_logs trước/sau</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>9 route</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>401 khi không token; 403 {"detail": "admin_only"} với user thường; access_logs không đổi; POST của user thường không ghi dòng nào</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · Decision Table (R1, R2) · test_auth_401_and_non_admin_403__AC11, test_non_admin_write_changes_nothing__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="123.5" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-21</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Uống cách giờ: số giờ không bắt buộc, chỉ đi với cach_gio</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Admin; các hoạt chất mới</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. POST cach_gio + 2 giờ
+2. POST cach_gio không số giờ
+3. POST tranh_phoi_hop / can_theo_doi / giam_lieu kèm 2 giờ
+4. PATCH đổi cach_gio → can_theo_doi khi còn số giờ
+5. PATCH như trên kèm min_interval_hours: null</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>như bước</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>201 với 2; 201 với null; 422 min_interval_not_allowed và không ghi; PATCH 422 min_interval_not_allowed; kèm null thì 200</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>AC27 · EP (4, 5, 18) · test_min_interval_rules__AC27</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="41" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-BVA-01</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Biên severity_level</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>1. POST với severity_level = 0, 1, 4 (chong_chi_dinh), 5</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>0 / 1 / 4 / 5</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>0 → 422; 1 → 201; 4 → 201; 5 → 422</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · BVA (min-1, min, max, max+1) · test_create_boundaries</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="41" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-BVA-02</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Biên min_interval_hours</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Admin; handling_type = cach_gio</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>1. POST với min_interval_hours = 0, 0.5, 168, 169</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>0 / 0.5 / 168 / 169</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>0 → 422; 0.5 → 201; 168 → 201; 169 → 422</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>AC27 · BVA (min-1, min, max, max+1) · test_create_boundaries</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="41" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-BVA-03</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Biên độ dài description và source</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>1. POST description dài 4000 và 4001
+2. POST source dài 500 và 501</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>a*4000 / a*4001 / s*500 / s*501</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>4000 → 201, 4001 → 422; 500 → 201, 501 → 422</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>BVA (max, max+1) · test_create_boundaries</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="41" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-BVA-04</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Biên số ngưỡng liều</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>1. POST với 20 ngưỡng
+2. POST với 21 ngưỡng</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>20 / 21 ngưỡng</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>20 → 201 và trả đủ 20; 21 → 422</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>BVA (max, max+1) · test_create_boundaries</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="57.5" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-BVA-05</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Biên limit của danh sách</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /admin/drug-interactions?limit=0, 1, 100, 101</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>0 / 1 / 100 / 101</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>0 → 422; 1 → 200; 100 → 200; 101 → 422</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · BVA (min-1, min, max, max+1) · test_list_limit_boundaries</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="90.5" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-22</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Sửa tạo phiên bản mới, phiên bản cũ giữ nguyên nội dung</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Admin; quy tắc R phiên bản 1</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH expected_version=1, severity_level=3
+2. So dòng DB phiên bản 1 trước và sau</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>severity_level: 3</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>200: cùng id, version = 2, version_id mới, updated_by = admin; DB có 2 dòng, phiên bản 1 nội dung không đổi và superseded_at có giá trị</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>AC18 · Decision Table bảng 2 (R4) · Chuyển trạng thái (current → superseded) · test_patch_creates_new_version_old_unchanged__AC18</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="57.5" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-23</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Ngưỡng liều thuộc từng phiên bản</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Admin; quy tắc có 2 ngưỡng</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH chỉ đổi description
+2. PATCH gửi 1 ngưỡng mới
+3. Đọc ngưỡng của từng phiên bản trong DB</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>như bước</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>Phiên bản 2 có 2 ngưỡng id mới; phiên bản 3 có 1 ngưỡng; ngưỡng của phiên bản 1 không đổi</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>AC19 · test_thresholds_belong_to_each_version__AC19</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="57.5" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-24</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối sửa/xóa với expected_version cũ</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Admin; quy tắc đã lên phiên bản 2</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH expected_version=1
+2. DELETE ?expected_version=1</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>expected_version: 1</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>409 {"detail": "version_conflict"} cho cả hai; DB không đổi</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>409 version_conflict; vẫn 2 phiên bản, chưa xóa</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>AC20 · EP (26) · Decision Table bảng 2 (R2) · test_stale_expected_version_conflict__AC20</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="90.5" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-25</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Hai admin sửa cùng phiên bản đồng thời chỉ một thành công</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Admin; quy tắc phiên bản 1; một giao dịch khác giữ khóa quy tắc</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi đồng thời hai PATCH expected_version=1 với mô tả khác nhau
+2. Chờ tới khi cả hai đang chờ khóa DB
+3. Thả khóa
+4. Đếm phiên bản</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>2 request song song</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>Một 200, một 409; đúng 2 phiên bản, 1 phiên bản mở</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>[200, 409]; phiên bản [1, 2]</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>AC20 · Chạy đua · test_concurrent_patch_same_version_one_wins__AC20</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="57.5" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-26</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Sửa với giá trị giống hệt không tạo phiên bản</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Admin; quy tắc phiên bản 1 có 2 ngưỡng</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH expected_version=1 với severity_level, description và dose_thresholds giống hệt (đảo thứ tự ngưỡng)</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>giá trị hiện tại</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>200; version = 1, version_id không đổi; DB vẫn 1 dòng</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>AC21 · Decision Table bảng 2 (R3) · test_noop_patch_keeps_version__AC21</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="107" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-27</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Xem lịch sử và một phiên bản sau khi quy tắc bị xóa</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Admin; quy tắc qua 3 phiên bản rồi bị xóa mềm</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /admin/drug-interactions/{id}/versions
+2. GET /admin/drug-interaction-versions/{version_id của phiên bản 1}
+3. GET với mã/id không tồn tại</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>như bước</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>3 phiên bản mới nhất trước: deleted/superseded/superseded, mỗi phiên bản đủ ngưỡng, phiên bản cuối có deleted_by; phiên bản 1 đúng nội dung cũ; 404 interaction_version_not_found / interaction_rule_not_found</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>AC23 · test_history_and_version_lookup_after_delete__AC23</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="57.5" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-28</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>created_at giữ thời điểm tạo phiên bản 1; updated_at theo phiên bản hiện hành</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Admin; quy tắc phiên bản 1</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH đổi source
+2. GET chi tiết</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>source: Dược thư</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>created_at không đổi; updated_at ≥ trước; chi tiết trả version 2 với source mới</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="inlineStr">
+        <is>
+          <t>AC26 · test_created_at_and_updated_at__AC26</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="74" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-29</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>DB chặn sửa nội dung phiên bản với mọi role</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Quy tắc phiên bản 1 có 1 ngưỡng (chèn trực tiếp DB)</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>1. UPDATE severity_level bằng api_role
+2. Bằng worker_role
+3. Bằng postgres
+4. Đọc lại severity_level</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>SET severity_level = 4</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>api_role, worker_role: permission denied; postgres: "version content is immutable"; giá trị không đổi</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I42" s="8" t="inlineStr">
+        <is>
+          <t>AC22 · test_content_update_rejected_for_every_role__AC22</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="90.5" customHeight="1">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-30</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>DB chỉ cho đóng phiên bản một lần, không cho vừa thay vừa xóa</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Quy tắc phiên bản 1</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>1. api_role: SET superseded_at
+2. postgres: SET deleted_at, rồi SET superseded_at lần nữa
+3. postgres: SET superseded_at và deleted_at cùng lúc trên quy tắc khác</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>như bước</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>Lần đầu thành công; sau đó "closed and immutable"; cùng lúc: vi phạm CHECK state_chk</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="inlineStr">
+        <is>
+          <t>AC22 · Chuyển trạng thái (superseded → * bị cấm) · test_close_once_then_immutable__AC22, test_superseded_and_deleted_together_rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="74" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-31</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>DB chặn DELETE và TRUNCATE quy tắc và ngưỡng</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Quy tắc có ngưỡng</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>1. postgres: DELETE quy tắc / ngưỡng
+2. api_role: DELETE
+3. postgres: TRUNCATE (trong giao dịch, rollback)</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>như bước</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>postgres: "... is not allowed on the versioned interaction catalog"; api_role: permission denied</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I44" s="8" t="inlineStr">
+        <is>
+          <t>AC22 · test_delete_and_truncate_rejected__AC22</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="74" customHeight="1">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-32</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>DB chặn sửa ngưỡng và thêm ngưỡng vào phiên bản đã có</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Quy tắc có 1 ngưỡng</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>1. postgres: UPDATE ngưỡng
+2. api_role: INSERT ngưỡng cho phiên bản đã có (giao dịch khác)
+3. Đếm ngưỡng</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>như bước</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>UPDATE: not allowed; INSERT: "... created in the same transaction"; vẫn 1 ngưỡng</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I45" s="8" t="inlineStr">
+        <is>
+          <t>AC22, AC19 · test_thresholds_immutable_and_only_added_with_new_version__AC22_AC19</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="57.5" customHeight="1">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-33</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Quyền tối thiểu: worker_role chỉ đọc; anon/authenticated không đọc được</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>Quy tắc có sẵn</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>1. worker_role: SELECT, INSERT, UPDATE superseded_at
+2. SET ROLE anon / authenticated rồi SELECT</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>như bước</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>worker_role đọc được, ghi bị permission denied; anon/authenticated permission denied</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I46" s="8" t="inlineStr">
+        <is>
+          <t>AC22 · test_worker_role_read_only, test_client_roles_cannot_read</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="90.5" customHeight="1">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-34</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Dòng chèn kiểu cũ thành phiên bản 1 hợp lệ; chặn chèn phiên bản đóng hoặc thiếu rule_id</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>DB sau migration</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>1. INSERT kiểu cũ (không cột mới)
+2. INSERT có deleted_at
+3. INSERT version = 2 không rule_id</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>như bước</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>rule_id = id, version 1, mở; "must be inserted open"; "needs an existing rule_id"</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi. Backfill dữ liệu có trước migration kiểm ở implement (33/33)</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I47" s="8" t="inlineStr">
+        <is>
+          <t>AC25 · test_old_style_insert_becomes_open_version_1__AC25, test_insert_closed_or_versionless_rejected; evidence/impl-check-migration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="57.5" customHeight="1">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-35</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Unique cặp chỉ tính phiên bản mở</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Quy tắc (A, B) mở</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>1. INSERT (B, A)
+2. Xóa mềm (A, B)
+3. INSERT (B, A) lần nữa</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>như bước</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>Lần đầu vi phạm active_ingredient_interactions_pair_uq; sau xóa mềm chèn được</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I48" s="8" t="inlineStr">
+        <is>
+          <t>AC24 · test_pair_unique_only_among_open_versions__AC24</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="57.5" customHeight="1">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>TC-DDIRULE-36</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Response khớp contract (operationId, mã trạng thái, field)</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>api_contract/openapi.json (đã duyệt)</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>1. So OpenAPI sinh từ app với contract cho 15 operation</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>15 operation</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>operationId, mã trạng thái, shape request/response, tham số query khớp; bảng mức độ 1–4 có trong contract</t>
+        </is>
+      </c>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>28 test pass</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I49" s="8" t="inlineStr">
+        <is>
+          <t>AC14, AC17 · test_contract_interaction.py (unit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52">
+      <c r="G52" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H52" s="13">
+        <f>COUNTIF(H9:H49,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="G53" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H53" s="13">
+        <f>COUNTIF(H9:H49,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="G54" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H54" s="13">
+        <f>COUNTIF(H9:H49,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="G55" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H55" s="13">
+        <f>SUM(H52:H54)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I49"/>
+  <conditionalFormatting sqref="H9:H49">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Danh mục tương tác thuốc-thực phẩm (admin) (DFIRULE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46307</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="123.5" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-DFIRULE-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Tạo, xem, sửa, xóa mềm, xem lịch sử, tạo lại quy tắc thực phẩm</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Admin; hoạt chất có trong danh mục</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /admin/drug-food-interactions
+2. GET chi tiết
+3. PATCH expected_version=1 đổi food_to_avoid, reason, severity_level
+4. DELETE ?expected_version=2
+5. GET chi tiết, GET lịch sử, GET phiên bản 1
+6. POST lại cùng thực phẩm</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>food_to_avoid: Nước bưởi chùm → Rượu</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>201 version 1; GET bằng response tạo; 200 version 2; DB có 2 phiên bản, bản 1 superseded; 204; 404; lịch sử deleted/superseded; phiên bản 1 giữ Nước bưởi chùm; tạo lại 201</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC10, AC7, AC18 · Chuyển trạng thái · test_crud_flow__AC10</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>ingredient_id</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>có trong danh mục</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>không tồn tại
+gửi khi sửa</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>3
+4</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90.5" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-DFIRULE-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối dữ liệu sai và không ghi gì</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. POST với hoạt chất không tồn tại
+2. food_to_avoid chỉ khoảng trắng
+3. severity_level = 5
+4. có verification_status
+5. thiếu source</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>như bước</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>422 (hoạt chất không tồn tại: {"detail": "active_ingredient_not_found"}); không có dòng mới</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC10, AC4, AC15 · EP (3, 5) · test_validation_errors_write_nothing__AC10_AC4</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>food_to_avoid</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>1–200 ký tự, có ký tự không phải khoảng trắng</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>chỉ khoảng trắng
+trùng (không phân biệt hoa thường) với quy tắc mở của cùng hoạt chất</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>5
+6</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="57.5" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-DFIRULE-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Báo trùng thực phẩm không phân biệt hoa thường</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Admin; đã có (hoạt chất H, "Bưởi")</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. POST (H, "BƯỞI")
+2. POST (hoạt chất khác, "Bưởi")</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>BƯỞI</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>409 interaction_rule_exists; hoạt chất khác thì 201</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC10, AC5 · EP (6) · test_duplicate_food_case_insensitive__AC10_AC5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="57.5" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-DFIRULE-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Sửa thực phẩm thành trùng với quy tắc khác bị từ chối và không ghi gì</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Admin; hoạt chất H có "Sữa" và "Rượu"</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH quy tắc "Rượu" đổi food_to_avoid = "sữa"
+2. Đọc phiên bản trong DB</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>food_to_avoid: sữa</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>409 interaction_rule_exists; vẫn 1 phiên bản, phiên bản 1 vẫn mở (giao dịch rollback)</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC10, AC5 · EP (6) · Đoán lỗi · test_patch_food_to_duplicate_conflict_writes_nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="57.5" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-DFIRULE-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Không đổi được hoạt chất; phiên bản cũ bị từ chối</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Admin; quy tắc phiên bản 1</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH gửi ingredient_id
+2. PATCH hợp lệ lên phiên bản 2
+3. PATCH expected_version=1</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>như bước</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>422 ValidationError; 200; 409 version_conflict</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC10, AC9, AC20 · EP (4) · test_patch_rejects_ingredient_change_and_stale_version</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="107" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-DFIRULE-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Lọc và phân trang quy tắc thực phẩm</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Admin; 2 quy tắc của hoạt chất Simva, 1 của hoạt chất khác</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. GET ?ingredient_id
+2. thêm severity_level
+3. q viết hoa theo tên hoạt chất
+4. q theo food_to_avoid
+5. medication_id
+6. limit=1&amp;skip=1</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>như bước</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Đúng tập kết quả, mới sửa trước, total đúng</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC10, AC8 · test_filters__AC10_AC8</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17">
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H17" s="13">
+        <f>COUNTIF(H9:H14,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H18" s="13">
+        <f>COUNTIF(H9:H14,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H19" s="13">
+        <f>COUNTIF(H9:H14,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H20" s="13">
+        <f>SUM(H17:H19)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I14"/>
+  <conditionalFormatting sqref="H9:H14">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Tra cứu hoạt chất (admin) (INGRED)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46307</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="74" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-INGRED-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Tìm hoạt chất theo tên chuẩn và theo tên gọi khác</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Admin; hoạt chất Warfarin-&lt;tag&gt; có alias Coumadin-&lt;tag&gt;; Other-&lt;tag&gt;</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /admin/active-ingredients?q=WARFARIN-&lt;tag&gt; (viết hoa)
+2. q=coumadin-&lt;tag&gt;
+3. q=&lt;tag&gt;</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>như bước</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Trả đúng Warfarin kèm aliases; theo alias trả Warfarin; theo tag trả cả hai, sắp theo tên</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · EP (1, 2) · test_search_by_name_and_alias__AC12</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>q</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>khớp một phần tên chuẩn
+khớp một phần alias</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1
+2</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>chuỗi rỗng
+ký tự wildcard % _ (phải khớp nguyên văn)</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>4
+5</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="41" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-INGRED-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Ký tự wildcard trong từ khóa được khớp nguyên văn</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Admin; hoạt chất plain-&lt;tag&gt;</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. GET q=%&lt;tag&gt;
+2. GET q=_lain-&lt;tag&gt;</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>% và _</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>total = 0 cho cả hai</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · EP (5) · Đoán lỗi · test_wildcards_are_literal</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>medication_id</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>thuốc có hoạt chất</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>thuốc không tồn tại
+thuốc chưa ánh xạ hoạt chất</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>6
+7</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="41" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-INGRED-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Xem hoạt chất của một thuốc phối hợp</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Admin; thuốc chứa hai hoạt chất</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. GET ?medication_id
+2. GET ?medication_id&amp;limit=1</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>thuốc 2 hoạt chất</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Trả đúng 2 hoạt chất, total 2; limit 1 trả 1 với total 2</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC12, Q7 · EP (3) · test_by_medication__AC12</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="57.5" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-INGRED-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Thuốc không tồn tại hoặc chưa ánh xạ hoạt chất trả danh sách rỗng</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. GET ?medication_id=2000000000
+2. GET ?medication_id=&lt;thuốc chưa có hoạt chất&gt;</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>như bước</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>200 {"items": [], "total": 0}</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · EP (6, 7) · test_unknown_or_unmapped_medication_empty__AC12</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="41" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-INGRED-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối tham số query sai</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. GET ?limit=0, ?limit=101, ?skip=-1, ?q=</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>như bước</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>422 cho từng trường hợp</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · EP (4) · BVA · test_bad_query_422 (unit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="41" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-INGRED-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Chặn không token và tài khoản không phải admin</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Không token; user thường</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /admin/active-ingredients không token
+2. GET bằng phiên user thường</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>401; 403 {"detail": "admin_only"}</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · test_auth_401_and_non_admin_403__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17">
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H17" s="13">
+        <f>COUNTIF(H9:H14,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H18" s="13">
+        <f>COUNTIF(H9:H14,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H19" s="13">
+        <f>COUNTIF(H9:H14,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H20" s="13">
+        <f>SUM(H17:H19)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I14"/>
+  <conditionalFormatting sqref="H9:H14">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8834,7 +12693,7 @@
         </is>
       </c>
       <c r="C3" s="11">
-        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59+'Lịch uống thuốc'!$H$51+'Tải lịch uống'!$H$32</f>
+        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59+'Lịch uống thuốc'!$H$51+'Tải lịch uống'!$H$32+'Tương tác thuốc-thuốc'!$H$52+'Tương tác thuốc-thực phẩm'!$H$17+'Tra cứu hoạt chất'!$H$17</f>
         <v/>
       </c>
       <c r="D3" s="15">
@@ -8850,7 +12709,7 @@
         </is>
       </c>
       <c r="C4" s="11">
-        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60+'Lịch uống thuốc'!$H$52+'Tải lịch uống'!$H$33</f>
+        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60+'Lịch uống thuốc'!$H$52+'Tải lịch uống'!$H$33+'Tương tác thuốc-thuốc'!$H$53+'Tương tác thuốc-thực phẩm'!$H$18+'Tra cứu hoạt chất'!$H$18</f>
         <v/>
       </c>
       <c r="D4" s="15">
@@ -8882,7 +12741,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr"/>
       <c r="C6" s="11">
-        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61+'Lịch uống thuốc'!$H$53+'Tải lịch uống'!$H$34</f>
+        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61+'Lịch uống thuốc'!$H$53+'Tải lịch uống'!$H$34+'Tương tác thuốc-thuốc'!$H$54+'Tương tác thuốc-thực phẩm'!$H$19+'Tra cứu hoạt chất'!$H$19</f>
         <v/>
       </c>
       <c r="D6" s="15">
@@ -9129,393 +12988,525 @@
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="19" t="inlineStr">
+    <row r="15" ht="90.5" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Danh mục tương tác thuốc-thuốc (admin)</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Admin thêm, xem, sửa (tạo phiên bản mới), xóa mềm quy tắc tương tác giữa hai hoạt chất, kèm ngưỡng liều; xem lịch sử phiên bản (task 2.16, PB05).</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Tương tác thuốc-thuốc</t>
+        </is>
+      </c>
+      <c r="D15" s="18">
+        <f>IFERROR(('Tương tác thuốc-thuốc'!$H$55-'Tương tác thuốc-thuốc'!$H$54)/'Tương tác thuốc-thuốc'!$H$55,0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="18">
+        <f>IFERROR('Tương tác thuốc-thuốc'!$H$52/'Tương tác thuốc-thuốc'!$H$55,0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="18">
+        <f>IFERROR('Tương tác thuốc-thuốc'!$H$53/'Tương tác thuốc-thuốc'!$H$55,0)</f>
+        <v/>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động (tích hợp với Postgres thật, app chạy bằng api_role) pass. Không có lỗi sản phẩm.</t>
+        </is>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="107" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Danh mục tương tác thuốc-thực phẩm (admin)</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Admin thêm, xem, sửa (tạo phiên bản mới), xóa mềm quy tắc tương tác giữa hoạt chất và thực phẩm (task 2.16, PB05).</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Tương tác thuốc-thực phẩm</t>
+        </is>
+      </c>
+      <c r="D16" s="18">
+        <f>IFERROR(('Tương tác thuốc-thực phẩm'!$H$20-'Tương tác thuốc-thực phẩm'!$H$19)/'Tương tác thuốc-thực phẩm'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="18">
+        <f>IFERROR('Tương tác thuốc-thực phẩm'!$H$17/'Tương tác thuốc-thực phẩm'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="F16" s="18">
+        <f>IFERROR('Tương tác thuốc-thực phẩm'!$H$18/'Tương tác thuốc-thực phẩm'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động pass. Không có lỗi sản phẩm.</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90.5" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Tra cứu hoạt chất (admin)</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Admin tìm hoạt chất theo tên chuẩn hoặc tên gọi khác, hoặc xem hoạt chất của một thuốc, để chọn khi nhập quy tắc tương tác (task 2.16).</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Tra cứu hoạt chất</t>
+        </is>
+      </c>
+      <c r="D17" s="18">
+        <f>IFERROR(('Tra cứu hoạt chất'!$H$20-'Tra cứu hoạt chất'!$H$19)/'Tra cứu hoạt chất'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="E17" s="18">
+        <f>IFERROR('Tra cứu hoạt chất'!$H$17/'Tra cứu hoạt chất'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="F17" s="18">
+        <f>IFERROR('Tra cứu hoạt chất'!$H$18/'Tra cứu hoạt chất'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động pass.</t>
+        </is>
+      </c>
+      <c r="I17" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="19" t="inlineStr">
         <is>
           <t>Bug Report</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="20" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="20" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="B38" s="20" t="inlineStr">
+      <c r="B41" s="20" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C38" s="20" t="inlineStr">
+      <c r="C41" s="20" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="D38" s="20" t="inlineStr">
+      <c r="D41" s="20" t="inlineStr">
         <is>
           <t>Input Data</t>
         </is>
       </c>
-      <c r="E38" s="20" t="inlineStr">
+      <c r="E41" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F38" s="20" t="inlineStr">
+      <c r="F41" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="G38" s="20" t="inlineStr">
+      <c r="G41" s="20" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="H38" s="20" t="inlineStr">
+      <c r="H41" s="20" t="inlineStr">
         <is>
           <t>Name of Tester</t>
         </is>
       </c>
-      <c r="I38" s="20" t="inlineStr">
+      <c r="I41" s="20" t="inlineStr">
         <is>
           <t>Logs</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="123.5" customHeight="1">
-      <c r="A39" s="22" t="inlineStr">
+    <row r="42" ht="123.5" customHeight="1">
+      <c r="A42" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-08</t>
         </is>
       </c>
-      <c r="B39" s="22" t="inlineStr">
+      <c r="B42" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
         </is>
       </c>
-      <c r="C39" s="22" t="inlineStr">
+      <c r="C42" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
 2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
         </is>
       </c>
-      <c r="D39" s="22" t="inlineStr">
+      <c r="D42" s="22" t="inlineStr">
         <is>
           <t>phone: 0900000001 + ký tự \n</t>
         </is>
       </c>
-      <c r="E39" s="22" t="inlineStr">
+      <c r="E42" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F39" s="22" t="inlineStr">
+      <c r="F42" s="22" t="inlineStr">
         <is>
           <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
         </is>
       </c>
-      <c r="G39" s="22" t="inlineStr">
+      <c r="G42" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H39" s="22" t="inlineStr">
+      <c r="H42" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I39" s="22" t="inlineStr">
+      <c r="I42" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn — kỳ vọng AC6 mâu thuẫn AC5: backend `_validate_required_text` (sign_in.py:178) `strip()` mọi ký tự trắng hai đầu, nên \n cuối được xử lý như khoảng trắng hai đầu mà AC5 coi là hợp lệ. Cần người dùng chốt: sửa AC6 hoặc sửa backend
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="123.5" customHeight="1">
-      <c r="A40" s="22" t="inlineStr">
+    <row r="43" ht="123.5" customHeight="1">
+      <c r="A43" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-11</t>
         </is>
       </c>
-      <c r="B40" s="22" t="inlineStr">
+      <c r="B43" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
         </is>
       </c>
-      <c r="C40" s="22" t="inlineStr">
+      <c r="C43" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone}
 2. POST /auth/mobile/verify {phone, token: 123456}</t>
         </is>
       </c>
-      <c r="D40" s="22" t="inlineStr">
+      <c r="D43" s="22" t="inlineStr">
         <is>
           <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
         </is>
       </c>
-      <c r="E40" s="22" t="inlineStr">
+      <c r="E43" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
         </is>
       </c>
-      <c r="F40" s="22" t="inlineStr">
+      <c r="F43" s="22" t="inlineStr">
         <is>
           <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
         </is>
       </c>
-      <c r="G40" s="22" t="inlineStr">
+      <c r="G43" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H40" s="22" t="inlineStr">
+      <c r="H43" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I40" s="22" t="inlineStr">
+      <c r="I43" s="22" t="inlineStr">
         <is>
           <t>`_normalize_phone` (sign_in.py:197–206) kiểm bằng `str.isdigit()`, nhận cả chữ số Unicode, nên số lọt qua kiểm tra và gửi tới Supabase. Ô nhập của app chỉ cho 0-9 nên người dùng app không gặp; lỗi ở tầng API
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="189.5" customHeight="1">
-      <c r="A41" s="22" t="inlineStr">
+    <row r="44" ht="189.5" customHeight="1">
+      <c r="A44" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-25</t>
         </is>
       </c>
-      <c r="B41" s="22" t="inlineStr">
+      <c r="B44" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên có ký tự NUL</t>
         </is>
       </c>
-      <c r="C41" s="22" t="inlineStr">
+      <c r="C44" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
         </is>
       </c>
-      <c r="D41" s="22" t="inlineStr">
+      <c r="D44" s="22" t="inlineStr">
         <is>
           <t>ho_ten: abc\u0000def</t>
         </is>
       </c>
-      <c r="E41" s="22" t="inlineStr">
+      <c r="E44" s="22" t="inlineStr">
         <is>
           <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
         </is>
       </c>
-      <c r="F41" s="22" t="inlineStr">
+      <c r="F44" s="22" t="inlineStr">
         <is>
           <t>500 Internal Server Error</t>
         </is>
       </c>
-      <c r="G41" s="22" t="inlineStr">
+      <c r="G44" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H41" s="22" t="inlineStr">
+      <c r="H44" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I41" s="22" t="inlineStr">
+      <c r="I44" s="22" t="inlineStr">
         <is>
           <t>`_validate_required_text` (sign_in.py:178) không chặn ký tự điều khiển; PostgreSQL từ chối NUL trong cột text: `psycopg.DataError: PostgreSQL text fields cannot contain NUL (0x00) bytes` ở `UPDATE users SET full_name…` (SqlUsers.update_profile); không có handler cho DataError nên thành 500. Câu SQL có tham số nên không phải lỗ hổng SQL injection
 Log: evidence/test-integration.log, evidence/test-probe-nul.log</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="90.5" customHeight="1">
-      <c r="A42" s="22" t="inlineStr">
+    <row r="45" ht="90.5" customHeight="1">
+      <c r="A45" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-30</t>
         </is>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B45" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên dài 256 ký tự</t>
         </is>
       </c>
-      <c r="C42" s="22" t="inlineStr">
+      <c r="C45" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: A*256}</t>
         </is>
       </c>
-      <c r="D42" s="22" t="inlineStr">
+      <c r="D45" s="22" t="inlineStr">
         <is>
           <t>A*256</t>
         </is>
       </c>
-      <c r="E42" s="22" t="inlineStr">
+      <c r="E45" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F42" s="22" t="inlineStr">
+      <c r="F45" s="22" t="inlineStr">
         <is>
           <t>204, đã lưu</t>
         </is>
       </c>
-      <c r="G42" s="22" t="inlineStr">
+      <c r="G45" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H42" s="22" t="inlineStr">
+      <c r="H45" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I42" s="22" t="inlineStr">
+      <c r="I45" s="22" t="inlineStr">
         <is>
           <t>Không có giới hạn độ dài họ tên: `_validate_profile` (sign_in.py) chỉ kiểm rỗng; cột users.full_name kiểu text không giới hạn
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="90.5" customHeight="1">
-      <c r="A43" s="22" t="inlineStr">
+    <row r="46" ht="90.5" customHeight="1">
+      <c r="A46" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-32</t>
         </is>
       </c>
-      <c r="B43" s="22" t="inlineStr">
+      <c r="B46" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh trước 1900-01-01</t>
         </is>
       </c>
-      <c r="C43" s="22" t="inlineStr">
+      <c r="C46" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh}</t>
         </is>
       </c>
-      <c r="D43" s="22" t="inlineStr">
+      <c r="D46" s="22" t="inlineStr">
         <is>
           <t>1899-12-31 | 0001-01-01</t>
         </is>
       </c>
-      <c r="E43" s="22" t="inlineStr">
+      <c r="E46" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
         </is>
       </c>
-      <c r="F43" s="22" t="inlineStr">
+      <c r="F46" s="22" t="inlineStr">
         <is>
           <t>204 ở cả hai giá trị, đã lưu</t>
         </is>
       </c>
-      <c r="G43" s="22" t="inlineStr">
+      <c r="G46" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H43" s="22" t="inlineStr">
+      <c r="H46" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I43" s="22" t="inlineStr">
+      <c r="I46" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:229–231) chỉ chặn ngày tương lai, không có cận dưới. App mobile đã giới hạn date picker từ 1900 nên chỉ gặp khi gọi API trực tiếp
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="123.5" customHeight="1">
-      <c r="A44" s="22" t="inlineStr">
+    <row r="47" ht="123.5" customHeight="1">
+      <c r="A47" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-35</t>
         </is>
       </c>
-      <c r="B44" s="22" t="inlineStr">
+      <c r="B47" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
         </is>
       </c>
-      <c r="C44" s="22" t="inlineStr">
+      <c r="C47" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
         </is>
       </c>
-      <c r="D44" s="22" t="inlineStr">
+      <c r="D47" s="22" t="inlineStr">
         <is>
           <t>ngay_sinh: 2026-10-08</t>
         </is>
       </c>
-      <c r="E44" s="22" t="inlineStr">
+      <c r="E47" s="22" t="inlineStr">
         <is>
           <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
         </is>
       </c>
-      <c r="F44" s="22" t="inlineStr">
+      <c r="F47" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_date_of_birth"}</t>
         </is>
       </c>
-      <c r="G44" s="22" t="inlineStr">
+      <c r="G47" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H44" s="22" t="inlineStr">
+      <c r="H47" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I44" s="22" t="inlineStr">
+      <c r="I47" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:230) so với `now.date()` trong khi `now()` (shared/clock.py) trả giờ UTC: từ 00:00 đến 07:00 giờ VN, "hôm nay" bị coi là ngày mai. Vi phạm bất biến 7 (múi giờ cố định Asia/Ho_Chi_Minh)
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="173" customHeight="1">
-      <c r="A45" s="22" t="inlineStr">
+    <row r="48" ht="173" customHeight="1">
+      <c r="A48" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-42</t>
         </is>
       </c>
-      <c r="B45" s="22" t="inlineStr">
+      <c r="B48" s="22" t="inlineStr">
         <is>
           <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
         </is>
       </c>
-      <c r="C45" s="22" t="inlineStr">
+      <c r="C48" s="22" t="inlineStr">
         <is>
           <t>1. Chạm vào ô mã OTP
 2. Theo dõi request backend nhận được</t>
         </is>
       </c>
-      <c r="D45" s="22" t="inlineStr">
+      <c r="D48" s="22" t="inlineStr">
         <is>
           <t>Ô đang chứa 000000</t>
         </is>
       </c>
-      <c r="E45" s="22" t="inlineStr">
+      <c r="E48" s="22" t="inlineStr">
         <is>
           <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
         </is>
       </c>
-      <c r="F45" s="22" t="inlineStr">
+      <c r="F48" s="22" t="inlineStr">
         <is>
           <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
         </is>
       </c>
-      <c r="G45" s="22" t="inlineStr">
+      <c r="G48" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H45" s="22" t="inlineStr">
+      <c r="H48" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I45" s="22" t="inlineStr">
+      <c r="I48" s="22" t="inlineStr">
         <is>
           <t>`OtpPinInput._handleTextChange` (frontend/mobile/lib/features/auth/presentation/widgets/otp_pin_input.dart:66–72) chạy với mọi thông báo của controller, kể cả khi chỉ đổi vị trí con trỏ lúc chạm ô, và gọi onCompleted hễ ô đủ 6 số → gửi lại mã sai, tốn hạn mức token_verifications
 Log: evidence/test-e2e.log (mục "request backend trong pha 2"), evidence/implement-P10-run-phase2-requests.log</t>
@@ -9527,17 +13518,17 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:A5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11:F14">
+  <conditionalFormatting sqref="F11:F17">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11:G14">
+  <conditionalFormatting sqref="G11:G17">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>OR(G11="Critical",G11="High")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G39:G45">
+  <conditionalFormatting sqref="G42:G48">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
@@ -9549,10 +13540,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G11:G14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G11:G17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="G39:G45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G42:G48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
test(catalog): record sync E2E failures and pending crash case
Refs: 2.22-sync-job-e2e
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -8,11 +8,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android build" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đăng nhập người dùng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog sync E2E" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Android build'!$A$8:$I$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Đăng nhập người dùng'!$A$8:$I$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Catalog sync E2E'!$A$8:$I$40</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -351,12 +353,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$12</f>
+              <f>'Report'!$A$11:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$11:$D$12</f>
+              <f>'Report'!$D$11:$D$13</f>
             </numRef>
           </val>
         </ser>
@@ -375,12 +377,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$12</f>
+              <f>'Report'!$A$11:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$11:$E$12</f>
+              <f>'Report'!$E$11:$E$13</f>
             </numRef>
           </val>
         </ser>
@@ -399,12 +401,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$12</f>
+              <f>'Report'!$A$11:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$11:$F$12</f>
+              <f>'Report'!$F$11:$F$13</f>
             </numRef>
           </val>
         </ser>
@@ -485,7 +487,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$3:$D$4</f>
+              <f>'Report'!$E$3:$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -507,7 +509,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>15</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -529,7 +531,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>15</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3240000"/>
@@ -4660,7 +4662,2105 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:U46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Đồng bộ danh mục thuốc E2E (CATSYNC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46304</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Lập lịch source</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="140" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Đồng bộ lần đầu từ Beat qua broker thật</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC1
+2. Đối chiếu test_beat_triggers_first_sync_and_commits_snapshot__AC1 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>source=dav_drugbank; snapshot 10 thuốc E2E-001..010; thuốc thứ 10 withdrawn; Unicode và khoảng trắng</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Một sync scheduler; 10 thuốc normalize đúng; inserted=10, updated=0, failed=0; run thanh_cong/finished_at; tick/delivery/HTTP liên kết cùng ledger.</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-a61765b49491.json; evidence/test-a61765b49491-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · EP (1,2,3,4,5) · Decision Table (R1) · test_beat_triggers_first_sync_and_commits_snapshot__AC1</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>dav_drugbank</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>qd_5948 chưa hỗ trợ</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Source đang running?</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="140" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Bỏ qua sync khi thành công chưa đủ 7 ngày</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC2
+2. Đối chiếu test_recent_success_suppresses_sync_after_completed_tick__AC2[518400] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>age_seconds=518400</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Tick hoàn tất, không catalog.sync/HTTP/run mới; thời điểm quan sát vẫn nhỏ hơn 604800 giây.</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Tick đã hoàn tất; không phát catalog.sync, không HTTP; chỉ còn run success đã seed. evidence/test-integration.log; evidence/test-case-328d86da3570.json; evidence/test-328d86da3570-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · BVA (dưới ngưỡng) · Decision Table (R2) · test_recent_success_suppresses_sync_after_completed_tick__AC2[518400]</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>snapshot</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>10 thuốc Unicode có withdrawn</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>items=[]
+thiếu name
+thiếu source_ref</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>7
+8
+9</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>Có success trước?</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="140" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Bỏ qua sync khi thành công chưa đủ 7 ngày</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC2
+2. Đối chiếu test_recent_success_suppresses_sync_after_completed_tick__AC2[604740] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>age_seconds=604740</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Tick hoàn tất, không catalog.sync/HTTP/run mới; thời điểm quan sát vẫn nhỏ hơn 604800 giây.</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Tick đã hoàn tất; không phát catalog.sync, không HTTP; chỉ còn run success đã seed. evidence/test-integration.log; evidence/test-case-348d637587e3.json; evidence/test-348d637587e3-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · BVA (dưới ngưỡng) · Decision Table (R2) · test_recent_success_suppresses_sync_after_completed_tick__AC2[604740]</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>HTTP status</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>429
+500
+400/404/422</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>10
+11
+12</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>Tuổi success</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S11" s="11" t="inlineStr">
+        <is>
+          <t>&lt;7 ngày</t>
+        </is>
+      </c>
+      <c r="T11" s="11" t="inlineStr">
+        <is>
+          <t>&gt;=7 ngày</t>
+        </is>
+      </c>
+      <c r="U11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="140" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Chạy sync khi thành công đủ hoặc quá 7 ngày</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC2
+2. Đối chiếu test_seven_day_success_is_due__AC2[604800] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>age_seconds=604800</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Beat tick enqueue đúng một sync; thuốc đúng; run mới thanh_cong, inserted=10.</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200]; run statuses=["thanh_cong","dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-7dcadc29d94b.json; evidence/test-7dcadc29d94b-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · BVA (ngưỡng/ngưỡng+60) · Decision Table (R3) · test_seven_day_success_is_due__AC2[604800]</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>environment</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>Linux + Python&gt;=3.12 + Docker local</t>
+        </is>
+      </c>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N12" s="10" t="inlineStr">
+        <is>
+          <t>Windows native
+remote/malformed URL hoặc Docker TCP/SSH</t>
+        </is>
+      </c>
+      <c r="O12" s="10" t="inlineStr">
+        <is>
+          <t>13
+14</t>
+        </is>
+      </c>
+      <c r="Q12" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="140" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Chạy sync khi thành công đủ hoặc quá 7 ngày</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC2
+2. Đối chiếu test_seven_day_success_is_due__AC2[604860] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>age_seconds=604860</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Beat tick enqueue đúng một sync; thuốc đúng; run mới thanh_cong, inserted=10.</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200]; run statuses=["thanh_cong","dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-9e8caeaa27f2.json; evidence/test-9e8caeaa27f2-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · BVA (ngưỡng/ngưỡng+60) · Decision Table (R3) · test_seven_day_success_is_due__AC2[604860]</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>ownership</t>
+        </is>
+      </c>
+      <c r="L13" s="10" t="inlineStr">
+        <is>
+          <t>DB marker và labels khớp</t>
+        </is>
+      </c>
+      <c r="M13" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N13" s="10" t="inlineStr">
+        <is>
+          <t>DB name/marker sai
+Compose/run labels sai</t>
+        </is>
+      </c>
+      <c r="O13" s="10" t="inlineStr">
+        <is>
+          <t>15
+16</t>
+        </is>
+      </c>
+      <c r="Q13" s="10" t="inlineStr">
+        <is>
+          <t>Enqueue catalog.sync</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S13" s="11" t="inlineStr"/>
+      <c r="T13" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="140" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Chặn tick và message trùng khi source đang chạy</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC3
+2. Đối chiếu test_running_source_suppresses_tick_and_duplicate_message__AC3 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Worker concurrency=2; giữ HTTP đầu ≤20s; publish duplicate cùng source</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Một run/fetch; tick và duplicate đã hoàn tất không tạo run/fetch chồng; thả HTTP có một success, thuốc đúng.</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200]; run statuses=["dang_chay"]; medications=0; deliveries=2. evidence/test-integration.log; evidence/test-case-9d6eedf72a76.json; evidence/test-9d6eedf72a76-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · Decision Table (R4) · State (dang_chay→thanh_cong) · test_running_source_suppresses_tick_and_duplicate_message__AC3</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>Không enqueue</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr"/>
+      <c r="S14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T14" s="11" t="inlineStr"/>
+      <c r="U14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="140" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Giữ ID thuốc khi chạy sync lặp</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC4
+2. Đối chiếu test_repeated_broker_sync_preserves_medication_ids__AC4 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Hai catalog.sync qua RabbitMQ; cùng snapshot 10 thuốc</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>10 source_ref duy nhất; ID giữ nguyên; counters lần 1=10/0/0, lần 2=0/10/0; không run running.</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200]; run statuses=["dang_chay"]; medications=0; deliveries=1. Sync đầu không ghi được thuốc nên chưa tới bước so ID lần hai. evidence/test-integration.log; evidence/test-case-4c83c671ad57.json; evidence/test-4c83c671ad57-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (1,2) · đoán lỗi gửi lặp · test_repeated_broker_sync_preserves_medication_ids__AC4</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="140" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Retry lỗi tạm thời rồi đồng bộ thành công</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC5
+2. Đối chiếu test_transient_http_retries_then_succeeds__AC5[429] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>HTTP=[429,429,429,200]</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Cùng task ID; retries 0→1→2→3; ba run that_bai, một thanh_cong; 10 thuốc; không retry thứ 5.</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[429]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-1cdcf1e60087.json; evidence/test-1cdcf1e60087-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · EP (10) · BVA (retry 0..3) · State (dang_chay→that_bai; dang_chay→thanh_cong) · test_transient_http_retries_then_succeeds__AC5[429]</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="140" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Dừng retry sau bốn attempt lỗi</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC5
+2. Đối chiếu test_transient_http_exhausts_four_attempts__AC5[429] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>HTTP luôn 429; quan sát thêm 10s sau terminal task</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Đúng bốn run/HTTP với finished_at; retries 0..3; không attempt 5, thuốc hoặc run dang_chay.</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[429]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-bffd8e518f38.json; evidence/test-bffd8e518f38-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · EP (10) · BVA (retry max/max+1) · test_transient_http_exhausts_four_attempts__AC5[429]</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="140" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Retry lỗi tạm thời rồi đồng bộ thành công</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC5
+2. Đối chiếu test_transient_http_retries_then_succeeds__AC5[500] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>HTTP=[500,500,500,200]</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Cùng task ID; retries 0→1→2→3; ba run that_bai, một thanh_cong; 10 thuốc; không retry thứ 5.</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[500]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-ada0c520b6bc.json; evidence/test-ada0c520b6bc-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · EP (11) · BVA (retry 0..3) · State (dang_chay→that_bai; dang_chay→thanh_cong) · test_transient_http_retries_then_succeeds__AC5[500]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="140" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Dừng retry sau bốn attempt lỗi</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC5
+2. Đối chiếu test_transient_http_exhausts_four_attempts__AC5[500] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>HTTP luôn 500; quan sát thêm 10s sau terminal task</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Đúng bốn run/HTTP với finished_at; retries 0..3; không attempt 5, thuốc hoặc run dang_chay.</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[500]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-51baed685b8d.json; evidence/test-51baed685b8d-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · EP (11) · BVA (retry max/max+1) · test_transient_http_exhausts_four_attempts__AC5[500]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="140" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Dừng lỗi HTTP cố định không retry</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC6
+2. Đối chiếu test_permanent_http_failure_has_no_retry__AC6[400] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>HTTP=400</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Một attempt/run that_bai có error_details/finished_at; không thuốc, HTTP hoặc retry tiếp theo.</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[400]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-74f89a8ac834.json; evidence/test-74f89a8ac834-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (12) · State (dang_chay→that_bai) · test_permanent_http_failure_has_no_retry__AC6[400]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="140" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-13</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Dừng lỗi HTTP cố định không retry</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC6
+2. Đối chiếu test_permanent_http_failure_has_no_retry__AC6[404] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>HTTP=404</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Một attempt/run that_bai có error_details/finished_at; không thuốc, HTTP hoặc retry tiếp theo.</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[404]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-8365039e1953.json; evidence/test-8365039e1953-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (12) · State (dang_chay→that_bai) · test_permanent_http_failure_has_no_retry__AC6[404]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="140" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-14</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Dừng lỗi HTTP cố định không retry</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC6
+2. Đối chiếu test_permanent_http_failure_has_no_retry__AC6[422] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>HTTP=422</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Một attempt/run that_bai có error_details/finished_at; không thuốc, HTTP hoặc retry tiếp theo.</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[422]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-0f684cdce3bb.json; evidence/test-0f684cdce3bb-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (12) · State (dang_chay→that_bai) · test_permanent_http_failure_has_no_retry__AC6[422]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="140" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối source chưa hỗ trợ</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC6
+2. Đối chiếu test_unsupported_source_has_no_retry_or_run__AC6 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>source=qd_5948</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Task lỗi unsupported catalog source; không run/HTTP/thuốc/retry.</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Task qd_5948 lỗi unsupported catalog source; không HTTP/run/thuốc, một delivery và không retry. evidence/test-integration.log; evidence/test-case-f584fcaccaa2.json; evidence/test-f584fcaccaa2-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (6) · test_unsupported_source_has_no_retry_or_run__AC6</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="140" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-16</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Kết thúc thất bại khi không có thuốc hợp lệ</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC6
+2. Đối chiếu test_no_valid_records_finishes_failed_without_retry__AC6[items0] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>items=[]</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Một run that_bai có finished_at/error_details; không thuốc/retry; không suy số HTTP bằng số run vì fetcher có phân trang.</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-a4b501f0afae.json; evidence/test-a4b501f0afae-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (7) · State (dang_chay→that_bai) · test_no_valid_records_finishes_failed_without_retry__AC6[items0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="140" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-17</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Kết thúc thất bại khi không có thuốc hợp lệ</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC6
+2. Đối chiếu test_no_valid_records_finishes_failed_without_retry__AC6[items1] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>items=[{"tenThuoc":"thiếu mã"}]</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Một run that_bai có finished_at/error_details; không thuốc/retry; không suy số HTTP bằng số run vì fetcher có phân trang.</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200,200,200,200,200,200,200,200,200,200]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-ee7e4efcc999.json; evidence/test-ee7e4efcc999-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (9) · State (dang_chay→that_bai) · test_no_valid_records_finishes_failed_without_retry__AC6[items1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="140" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-18</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Kết thúc thất bại khi không có thuốc hợp lệ</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC6
+2. Đối chiếu test_no_valid_records_finishes_failed_without_retry__AC6[items2] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>items=[{"soDangKy":"thiếu tên"}]</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Một run that_bai có finished_at/error_details; không thuốc/retry; không suy số HTTP bằng số run vì fetcher có phân trang.</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200,200,200,200,200,200,200,200,200,200]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-6d3163f60486.json; evidence/test-6d3163f60486-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (8) · State (dang_chay→that_bai) · test_no_valid_records_finishes_failed_without_retry__AC6[items2]</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="140" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-19</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Khôi phục sau Worker mất trước commit thuốc</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC7
+2. Đối chiếu test_worker_loss_before_commit_redelivers_and_recovers__AC7 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>HTTP hold; run dang_chay đã commit; thuốc rỗng; broker unacked=1; SIGKILL owned group</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Broker redelivers cùng ID/redelivered=true; cuối có 10 thuốc và success, không run treo/trùng; không chỉnh run thủ công để pass.</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200]; run statuses=["dang_chay"]; medications=0; deliveries=2. Cùng task ID được broker giao lại với redelivered=true, Worker báo succeeded nhưng run vẫn dang_chay, không thuốc. evidence/test-integration.log; evidence/test-case-e13de4a4b0bf.json; evidence/test-e13de4a4b0bf-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · đoán lỗi crash · State (dang_chay→recovery); nghi vấn run treo chưa tái hiện · test_worker_loss_before_commit_redelivers_and_recovers__AC7</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="140" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-20</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Giữ dữ liệu sau commit nhưng trước ack</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC8
+2. Đối chiếu test_worker_loss_after_commit_before_ack_is_idempotent__AC8 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Arm gate trước publish; DB thuốc/run đã commit; ack bị giữ; broker unacked=1; kill/restart</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Cùng ID redelivered=true; dữ liệu/ID thuốc không mất/trùng; run mới kết thúc; không gửi task thay thế.</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr"/>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · đoán lỗi crash · State (committed→redelivered) · test_worker_loss_after_commit_before_ack_is_idempotent__AC8 · Blocked: sync chưa commit thành công; chưa kiểm chứng crash sau commit, không phải skip.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="140" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-21</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Đối chiếu quyền và thuộc tính delivery thực tế</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC9
+2. Đối chiếu test_local_execution_role_and_delivery_properties__AC9 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Worker fetch bị giữ; pg_stat_activity; durable celery queue; delivery_mode=2</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Kết nối Worker thực là worker_role; unacked=1; payload chỉ source/trigger; cùng process báo Asia/Ho_Chi_Minh/no result backend/prefetch=1.</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Assert thực tế worker_role, durable queue, delivery_mode=2, unacked=1, payload chỉ source/triggered_by, timezone Asia/Ho_Chi_Minh, result backend=None, prefetch=1 đều đạt. Sync sau thả HTTP có lỗi quyền ghi riêng ở AC1. evidence/test-integration.log; evidence/test-case-65621e7b470e.json; evidence/test-65621e7b470e-worker-0.log</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · EP (4,5) · test_local_execution_role_and_delivery_properties__AC9</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="140" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-22</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Dọn tài nguyên sau lỗi và giữ sentinel ngoài case</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Linux/WSL2 Python ≥3.12 + Docker local; DB/queue do runner tạo mới; không dùng production.</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC10
+2. Đối chiếu test_failure_cleanup_removes_only_owned_resources__AC10 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Tạo sentinel vhost; lỗi assertion khi owned Worker đang fetch</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Owned group dừng, connection/vhost đã dọn; sentinel còn; marker DB suite nguyên; cleanup lỗi trả nonzero.</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Case cleanup đạt: owned process/vhost được dọn, sentinel còn và DB marker nguyên. evidence/test-integration.log; evidence/test-cleanup-final.log</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · đoán lỗi timeout/cleanup · test_failure_cleanup_removes_only_owned_resources__AC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="189.5" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-23</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Chặn URL/context ngoài loopback</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Python Windows có dependency backend/pytest; không cần Docker.</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy backend/.venv/Scripts/python.exe -X utf8 -B -m pytest tests/e2e/catalog_sync/test_harness.py -q -p no:cacheprovider
+2. Đối chiếu test_preflight_rejects_remote_urls__AC10; test_preflight_rejects_remote_docker_context__AC10 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>URL trống; remote; localhost; 127.0.0.1.evil; thiếu port; ssh/tcp Docker</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>PrerequisiteError trước tạo/ghi tài nguyên; literal loopback và socket local là giới hạn.</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Nhóm helper tương ứng đã đạt trong 59/59 unit tests trên Windows và Linux, không warning (thread warning được coi là lỗi). evidence/test-catalog-unit.log; evidence/test-catalog-unit-linux.log.</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · EP (14) · test_preflight_rejects_remote_urls__AC10; test_preflight_rejects_remote_docker_context__AC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="206" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-24</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Chặn marker/nhãn sở hữu sai</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Python Windows có dependency backend/pytest; không cần Docker.</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy backend/.venv/Scripts/python.exe -X utf8 -B -m pytest tests/e2e/catalog_sync/test_harness.py -q -p no:cacheprovider
+2. Đối chiếu test_ownership_guard_rejects_wrong_database_or_manifest__AC10; test_ownership_accepts_only_matching_marker_and_resource_labels__AC10 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>database=postgres; marker=other; labels={}; run label=other</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>verify_owner từ chối; trường hợp khớp đầy đủ mới qua.</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Nhóm helper tương ứng đã đạt trong 59/59 unit tests trên Windows và Linux, không warning (thread warning được coi là lỗi). evidence/test-catalog-unit.log; evidence/test-catalog-unit-linux.log.</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · EP (5,15,16) · test_ownership_guard_rejects_wrong_database_or_manifest__AC10; test_ownership_accepts_only_matching_marker_and_resource_labels__AC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="173" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-25</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Cô lập env Worker khỏi cấu hình production</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Python Windows có dependency backend/pytest; không cần Docker.</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy backend/.venv/Scripts/python.exe -X utf8 -B -m pytest tests/e2e/catalog_sync/test_harness.py -q -p no:cacheprovider
+2. Đối chiếu test_env_isolated_from_production_settings__AC10 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Env cha chứa production-secret ở DATABASE_URL/LLM_API_KEY/HTTP_PROXY/PYTHONPATH</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Env con chỉ loopback/test/empty key; không HTTP_PROXY hoặc giá trị production-secret.</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Nhóm helper tương ứng đã đạt trong 59/59 unit tests trên Windows và Linux, không warning (thread warning được coi là lỗi). evidence/test-catalog-unit.log; evidence/test-catalog-unit-linux.log.</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · đoán lỗi bí mật · test_env_isolated_from_production_settings__AC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="206" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-26</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Che bí mật trước khi ghi log</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Python Windows có dependency backend/pytest; không cần Docker.</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy backend/.venv/Scripts/python.exe -X utf8 -B -m pytest tests/e2e/catalog_sync/test_harness.py -q -p no:cacheprovider
+2. Đối chiếu test_redaction_precedes_all_log_sinks__AC11; test_stream_redacts_secrets_split_across_writes__AC11; test_auth_frames_are_forwarded_but_never_retained__AC11 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>URL credential, Bearer, JWT, api_key, secret chia hai write(); AMQP Start-Ok</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>Không secret ở file/screen/observer; stream giữ dòng chưa hoàn chỉnh cho đến khi redact.</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Nhóm helper tương ứng đã đạt trong 59/59 unit tests trên Windows và Linux, không warning (thread warning được coi là lỗi). evidence/test-catalog-unit.log; evidence/test-catalog-unit-linux.log.</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · đoán lỗi bí mật · test_redaction_precedes_all_log_sinks__AC11; test_stream_redacts_secrets_split_across_writes__AC11; test_auth_frames_are_forwarded_but_never_retained__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="206" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-27</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Ghép frame và giữ ack đúng delivery</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Python Windows có dependency backend/pytest; không cần Docker.</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy backend/.venv/Scripts/python.exe -X utf8 -B -m pytest tests/e2e/catalog_sync/test_harness.py -q -p no:cacheprovider
+2. Đối chiếu test_amqp_frame_assembly_and_task_correlation__AC8; test_ack_gate_preserves_target_and_forwards_heartbeats__AC8; test_proxy_closes_connections_without_flushing_held_acks__AC8 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>TCP split/gộp; multi-channel; multiple/tag=0; same ID redelivery; tag reuse</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>Ack mục tiêu giữ, heartbeat/ack khác forward; close không flush ack; correlation theo connection/channel/tag.</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Nhóm helper tương ứng đã đạt trong 59/59 unit tests trên Windows và Linux, không warning (thread warning được coi là lỗi). evidence/test-catalog-unit.log; evidence/test-catalog-unit-linux.log.</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · đoán lỗi giao thức; helper AC8 · test_amqp_frame_assembly_and_task_correlation__AC8; test_ack_gate_preserves_target_and_forwards_heartbeats__AC8; test_proxy_closes_connections_without_flushing_held_acks__AC8</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="206" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-28</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối cleanup tài nguyên không sở hữu</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Python Windows có dependency backend/pytest; không cần Docker.</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy backend/.venv/Scripts/python.exe -X utf8 -B -m pytest tests/e2e/catalog_sync/test_harness.py -q -p no:cacheprovider
+2. Đối chiếu test_cleanup_continues_after_process_error_and_taints_infra__AC10; test_cleanup_refuses_unowned_vhost__AC10; test_process_cleanup_refuses_unowned_group__AC10 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>PGID≠PID; unowned vhost; process stop phát sinh lỗi</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>Không kill/delete unowned; vẫn thử dọn owned vhost sau process error; taint infra và trả lỗi.</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>Nhóm helper tương ứng đã đạt trong 59/59 unit tests trên Windows và Linux, không warning (thread warning được coi là lỗi). evidence/test-catalog-unit.log; evidence/test-catalog-unit-linux.log.</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · đoán lỗi cleanup; helper AC10 · test_cleanup_continues_after_process_error_and_taints_infra__AC10; test_cleanup_refuses_unowned_vhost__AC10; test_process_cleanup_refuses_unowned_group__AC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="206" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-29</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Chặn timeout và kết quả đến sau deadline</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Python Windows có dependency backend/pytest; không cần Docker.</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy backend/.venv/Scripts/python.exe -X utf8 -B -m pytest tests/e2e/catalog_sync/test_harness.py -q -p no:cacheprovider
+2. Đối chiếu test_deadline_is_bounded_by_parent__AC10; test_late_success_cannot_escape_deadline__AC10; test_wait_timeout_does_not_report_success__AC10 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Clock 0→4→5; child timeout20/parent5; commit trả true ở giây6</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Deadline con≤cha; hết hạn hoặc late commit không báo thành công.</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Nhóm helper tương ứng đã đạt trong 59/59 unit tests trên Windows và Linux, không warning (thread warning được coi là lỗi). evidence/test-catalog-unit.log; evidence/test-catalog-unit-linux.log.</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · BVA (deadline−1/deadline/deadline+1) · test_deadline_is_bounded_by_parent__AC10; test_late_success_cannot_escape_deadline__AC10; test_wait_timeout_does_not_report_success__AC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="222.5" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-30</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Phân biệt pass với chưa thực thi/thiếu môi trường</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Python Windows có dependency backend/pytest; không cần Docker.</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy backend/.venv/Scripts/python.exe -X utf8 -B -m pytest tests/e2e/catalog_sync/test_harness.py -q -p no:cacheprovider
+2. Đối chiếu test_runner_exit_codes_require_executed_cases__AC10; test_runner_bootstrap_failure_is_exit_two__AC10; test_runner_missing_environment_is_exit_two__AC10; test_runner_native_windows_refuses_before_resources__AC10 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>zero/collect/skip/pytest fail/bootstrap fail/cleanup fail/native Windows</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>0 chỉ mọi selected case thực thi đạt; 1 test/cleanup fail; 2 thiếu môi trường. Windows bị chặn trước Docker mutation.</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>Nhóm helper tương ứng đã đạt trong 59/59 unit tests trên Windows và Linux, không warning (thread warning được coi là lỗi). evidence/test-catalog-unit.log; evidence/test-catalog-unit-linux.log.</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · EP (13) · test_runner_exit_codes_require_executed_cases__AC10; test_runner_bootstrap_failure_is_exit_two__AC10; test_runner_missing_environment_is_exit_two__AC10; test_runner_native_windows_refuses_before_resources__AC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="173" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-31</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Chọn đúng AC1 khi chạy một phần</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Python Windows có dependency backend/pytest; không cần Docker.</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy backend/.venv/Scripts/python.exe -X utf8 -B -m pytest tests/e2e/catalog_sync/test_harness.py -q -p no:cacheprovider
+2. Đối chiếu test_case_selection_does_not_confuse_ac_one_and_ten__AC11 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Hai node tên __AC1 và __AC10; chọn AC1</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ chọn __AC1; báo partial=true; không tính AC10 vào lượt AC1.</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>Nhóm helper tương ứng đã đạt trong 59/59 unit tests trên Windows và Linux, không warning (thread warning được coi là lỗi). evidence/test-catalog-unit.log; evidence/test-catalog-unit-linux.log.</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · đoán lỗi chọn case · test_case_selection_does_not_confuse_ac_one_and_ten__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="140" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>TC-CATSYNC-32</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm bàn giao E2E và workbook đầy đủ</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Linux/Docker chạy được E2E; Python có openpyxl; workbook tổng đã đọc.</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy toàn catalog runner và đọc kết quả/evidence cho từng AC.
+2. Chạy python .agents/scripts/testcase_xlsx.py validate|build|merge 2.22-sync-job-e2e lần lượt.
+3. Kiểm giữ sheet BUILD/LOGIN; số Pass/Fail/Pending, Bug Report và Test Report khớp log; xác nhận scope.</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>11 AC; code mới CATSYNC; workbook tổng có BUILD, LOGIN.</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Có lệnh tái chạy, versions/hash/evidence sanitize, AC mapping; workbook task/tổng dựng/gộp thành công; Pending được nêu; Fail chỉ khi tái hiện thật.</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>Đã có lệnh tái chạy, 11 AC mapping, DB/ledger/Worker evidence sanitize và báo cáo ba nhóm High. validate/build/merge bằng Python toàn cục có openpyxl exit 0; kiểm workbook giữ BUILD/LOGIN và số CATSYNC/Bug Report khớp spec. evidence/testcase-xlsx.log; evidence/test-docs-check.log; 05-test-report.md.</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · manual · không tính spec JSON là Excel đã dựng</t>
+        </is>
+      </c>
+    </row>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43">
+      <c r="G43" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H43" s="13">
+        <f>COUNTIF(H9:H40,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="G44" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H44" s="13">
+        <f>COUNTIF(H9:H40,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="G45" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H45" s="13">
+        <f>COUNTIF(H9:H40,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="G46" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H46" s="13">
+        <f>SUM(H43:H45)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I40"/>
+  <conditionalFormatting sqref="H9:H40">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4689,6 +6789,11 @@
       </c>
       <c r="D2" s="15" t="inlineStr">
         <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
@@ -4708,8 +6813,12 @@
         <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59</f>
         <v/>
       </c>
-      <c r="D3" s="15">
-        <f>SUM(C3:C3)</f>
+      <c r="D3" s="11">
+        <f>'Catalog sync E2E'!$H$43</f>
+        <v/>
+      </c>
+      <c r="E3" s="15">
+        <f>SUM(C3:D3)</f>
         <v/>
       </c>
     </row>
@@ -4724,8 +6833,12 @@
         <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60</f>
         <v/>
       </c>
-      <c r="D4" s="15">
-        <f>SUM(C4:C4)</f>
+      <c r="D4" s="11">
+        <f>'Catalog sync E2E'!$H$44</f>
+        <v/>
+      </c>
+      <c r="E4" s="15">
+        <f>SUM(C4:D4)</f>
         <v/>
       </c>
     </row>
@@ -4740,8 +6853,12 @@
         <f>C3+C4</f>
         <v/>
       </c>
-      <c r="D5" s="15">
-        <f>SUM(C5:C5)</f>
+      <c r="D5" s="11">
+        <f>D3+D4</f>
+        <v/>
+      </c>
+      <c r="E5" s="15">
+        <f>SUM(C5:D5)</f>
         <v/>
       </c>
     </row>
@@ -4756,8 +6873,12 @@
         <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61</f>
         <v/>
       </c>
-      <c r="D6" s="15">
-        <f>SUM(C6:C6)</f>
+      <c r="D6" s="11">
+        <f>'Catalog sync E2E'!$H$45</f>
+        <v/>
+      </c>
+      <c r="E6" s="15">
+        <f>SUM(C6:D6)</f>
         <v/>
       </c>
     </row>
@@ -4772,8 +6893,12 @@
         <f>C5+C6</f>
         <v/>
       </c>
-      <c r="D7" s="15">
-        <f>SUM(C7:C7)</f>
+      <c r="D7" s="11">
+        <f>D5+D6</f>
+        <v/>
+      </c>
+      <c r="E7" s="15">
+        <f>SUM(C7:D7)</f>
         <v/>
       </c>
     </row>
@@ -4912,396 +7037,1240 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="19" t="inlineStr">
+    <row r="13" ht="140" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Đồng bộ danh mục thuốc E2E</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Beat → RabbitMQ → Worker prefork → DAV local → PostgreSQL thật; retry/crash/ownership.</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Catalog sync E2E</t>
+        </is>
+      </c>
+      <c r="D13" s="18">
+        <f>IFERROR(('Catalog sync E2E'!$H$46-'Catalog sync E2E'!$H$45)/'Catalog sync E2E'!$H$46,0)</f>
+        <v/>
+      </c>
+      <c r="E13" s="18">
+        <f>IFERROR('Catalog sync E2E'!$H$43/'Catalog sync E2E'!$H$46,0)</f>
+        <v/>
+      </c>
+      <c r="F13" s="18">
+        <f>IFERROR('Catalog sync E2E'!$H$44/'Catalog sync E2E'!$H$46,0)</f>
+        <v/>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>Toàn E2E: 22 executed, 5 Pass, 16 lỗi sản phẩm, 1 blocked (AC8) — pytest 17 fail/5 pass, exit1. Ba nhóm root cause High; Bug Report sinh 16 dòng cho 16 test case Fail. AC8 Pending vì chưa đạt commit-before-ack. Helper Windows/Linux đều 59 pass; kết quả helper không thay E2E.</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
         <is>
           <t>Bug Report</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="20" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="20" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="B36" s="20" t="inlineStr">
+      <c r="B37" s="20" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C36" s="20" t="inlineStr">
+      <c r="C37" s="20" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="D36" s="20" t="inlineStr">
+      <c r="D37" s="20" t="inlineStr">
         <is>
           <t>Input Data</t>
         </is>
       </c>
-      <c r="E36" s="20" t="inlineStr">
+      <c r="E37" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F36" s="20" t="inlineStr">
+      <c r="F37" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="G36" s="20" t="inlineStr">
+      <c r="G37" s="20" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="H36" s="20" t="inlineStr">
+      <c r="H37" s="20" t="inlineStr">
         <is>
           <t>Name of Tester</t>
         </is>
       </c>
-      <c r="I36" s="20" t="inlineStr">
+      <c r="I37" s="20" t="inlineStr">
         <is>
           <t>Logs</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="123.5" customHeight="1">
-      <c r="A37" s="22" t="inlineStr">
+    <row r="38" ht="123.5" customHeight="1">
+      <c r="A38" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-08</t>
         </is>
       </c>
-      <c r="B37" s="22" t="inlineStr">
+      <c r="B38" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
         </is>
       </c>
-      <c r="C37" s="22" t="inlineStr">
+      <c r="C38" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
 2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
         </is>
       </c>
-      <c r="D37" s="22" t="inlineStr">
+      <c r="D38" s="22" t="inlineStr">
         <is>
           <t>phone: 0900000001 + ký tự \n</t>
         </is>
       </c>
-      <c r="E37" s="22" t="inlineStr">
+      <c r="E38" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F37" s="22" t="inlineStr">
+      <c r="F38" s="22" t="inlineStr">
         <is>
           <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
         </is>
       </c>
-      <c r="G37" s="22" t="inlineStr">
+      <c r="G38" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H37" s="22" t="inlineStr">
+      <c r="H38" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I37" s="22" t="inlineStr">
+      <c r="I38" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn — kỳ vọng AC6 mâu thuẫn AC5: backend `_validate_required_text` (sign_in.py:178) `strip()` mọi ký tự trắng hai đầu, nên \n cuối được xử lý như khoảng trắng hai đầu mà AC5 coi là hợp lệ. Cần người dùng chốt: sửa AC6 hoặc sửa backend
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="123.5" customHeight="1">
-      <c r="A38" s="22" t="inlineStr">
+    <row r="39" ht="123.5" customHeight="1">
+      <c r="A39" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-11</t>
         </is>
       </c>
-      <c r="B38" s="22" t="inlineStr">
+      <c r="B39" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
         </is>
       </c>
-      <c r="C38" s="22" t="inlineStr">
+      <c r="C39" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone}
 2. POST /auth/mobile/verify {phone, token: 123456}</t>
         </is>
       </c>
-      <c r="D38" s="22" t="inlineStr">
+      <c r="D39" s="22" t="inlineStr">
         <is>
           <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
         </is>
       </c>
-      <c r="E38" s="22" t="inlineStr">
+      <c r="E39" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
         </is>
       </c>
-      <c r="F38" s="22" t="inlineStr">
+      <c r="F39" s="22" t="inlineStr">
         <is>
           <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
         </is>
       </c>
-      <c r="G38" s="22" t="inlineStr">
+      <c r="G39" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H38" s="22" t="inlineStr">
+      <c r="H39" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I38" s="22" t="inlineStr">
+      <c r="I39" s="22" t="inlineStr">
         <is>
           <t>`_normalize_phone` (sign_in.py:197–206) kiểm bằng `str.isdigit()`, nhận cả chữ số Unicode, nên số lọt qua kiểm tra và gửi tới Supabase. Ô nhập của app chỉ cho 0-9 nên người dùng app không gặp; lỗi ở tầng API
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="189.5" customHeight="1">
-      <c r="A39" s="22" t="inlineStr">
+    <row r="40" ht="189.5" customHeight="1">
+      <c r="A40" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-25</t>
         </is>
       </c>
-      <c r="B39" s="22" t="inlineStr">
+      <c r="B40" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên có ký tự NUL</t>
         </is>
       </c>
-      <c r="C39" s="22" t="inlineStr">
+      <c r="C40" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
         </is>
       </c>
-      <c r="D39" s="22" t="inlineStr">
+      <c r="D40" s="22" t="inlineStr">
         <is>
           <t>ho_ten: abc\u0000def</t>
         </is>
       </c>
-      <c r="E39" s="22" t="inlineStr">
+      <c r="E40" s="22" t="inlineStr">
         <is>
           <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
         </is>
       </c>
-      <c r="F39" s="22" t="inlineStr">
+      <c r="F40" s="22" t="inlineStr">
         <is>
           <t>500 Internal Server Error</t>
         </is>
       </c>
-      <c r="G39" s="22" t="inlineStr">
+      <c r="G40" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H39" s="22" t="inlineStr">
+      <c r="H40" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I39" s="22" t="inlineStr">
+      <c r="I40" s="22" t="inlineStr">
         <is>
           <t>`_validate_required_text` (sign_in.py:178) không chặn ký tự điều khiển; PostgreSQL từ chối NUL trong cột text: `psycopg.DataError: PostgreSQL text fields cannot contain NUL (0x00) bytes` ở `UPDATE users SET full_name…` (SqlUsers.update_profile); không có handler cho DataError nên thành 500. Câu SQL có tham số nên không phải lỗ hổng SQL injection
 Log: evidence/test-integration.log, evidence/test-probe-nul.log</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="90.5" customHeight="1">
-      <c r="A40" s="22" t="inlineStr">
+    <row r="41" ht="90.5" customHeight="1">
+      <c r="A41" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-30</t>
         </is>
       </c>
-      <c r="B40" s="22" t="inlineStr">
+      <c r="B41" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên dài 256 ký tự</t>
         </is>
       </c>
-      <c r="C40" s="22" t="inlineStr">
+      <c r="C41" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: A*256}</t>
         </is>
       </c>
-      <c r="D40" s="22" t="inlineStr">
+      <c r="D41" s="22" t="inlineStr">
         <is>
           <t>A*256</t>
         </is>
       </c>
-      <c r="E40" s="22" t="inlineStr">
+      <c r="E41" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F40" s="22" t="inlineStr">
+      <c r="F41" s="22" t="inlineStr">
         <is>
           <t>204, đã lưu</t>
         </is>
       </c>
-      <c r="G40" s="22" t="inlineStr">
+      <c r="G41" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H40" s="22" t="inlineStr">
+      <c r="H41" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I40" s="22" t="inlineStr">
+      <c r="I41" s="22" t="inlineStr">
         <is>
           <t>Không có giới hạn độ dài họ tên: `_validate_profile` (sign_in.py) chỉ kiểm rỗng; cột users.full_name kiểu text không giới hạn
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="90.5" customHeight="1">
-      <c r="A41" s="22" t="inlineStr">
+    <row r="42" ht="90.5" customHeight="1">
+      <c r="A42" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-32</t>
         </is>
       </c>
-      <c r="B41" s="22" t="inlineStr">
+      <c r="B42" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh trước 1900-01-01</t>
         </is>
       </c>
-      <c r="C41" s="22" t="inlineStr">
+      <c r="C42" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh}</t>
         </is>
       </c>
-      <c r="D41" s="22" t="inlineStr">
+      <c r="D42" s="22" t="inlineStr">
         <is>
           <t>1899-12-31 | 0001-01-01</t>
         </is>
       </c>
-      <c r="E41" s="22" t="inlineStr">
+      <c r="E42" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
         </is>
       </c>
-      <c r="F41" s="22" t="inlineStr">
+      <c r="F42" s="22" t="inlineStr">
         <is>
           <t>204 ở cả hai giá trị, đã lưu</t>
         </is>
       </c>
-      <c r="G41" s="22" t="inlineStr">
+      <c r="G42" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H41" s="22" t="inlineStr">
+      <c r="H42" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I41" s="22" t="inlineStr">
+      <c r="I42" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:229–231) chỉ chặn ngày tương lai, không có cận dưới. App mobile đã giới hạn date picker từ 1900 nên chỉ gặp khi gọi API trực tiếp
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="123.5" customHeight="1">
-      <c r="A42" s="22" t="inlineStr">
+    <row r="43" ht="123.5" customHeight="1">
+      <c r="A43" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-35</t>
         </is>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B43" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
         </is>
       </c>
-      <c r="C42" s="22" t="inlineStr">
+      <c r="C43" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
         </is>
       </c>
-      <c r="D42" s="22" t="inlineStr">
+      <c r="D43" s="22" t="inlineStr">
         <is>
           <t>ngay_sinh: 2026-10-08</t>
         </is>
       </c>
-      <c r="E42" s="22" t="inlineStr">
+      <c r="E43" s="22" t="inlineStr">
         <is>
           <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
         </is>
       </c>
-      <c r="F42" s="22" t="inlineStr">
+      <c r="F43" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_date_of_birth"}</t>
         </is>
       </c>
-      <c r="G42" s="22" t="inlineStr">
+      <c r="G43" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H42" s="22" t="inlineStr">
+      <c r="H43" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I42" s="22" t="inlineStr">
+      <c r="I43" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:230) so với `now.date()` trong khi `now()` (shared/clock.py) trả giờ UTC: từ 00:00 đến 07:00 giờ VN, "hôm nay" bị coi là ngày mai. Vi phạm bất biến 7 (múi giờ cố định Asia/Ho_Chi_Minh)
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="173" customHeight="1">
-      <c r="A43" s="22" t="inlineStr">
+    <row r="44" ht="173" customHeight="1">
+      <c r="A44" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-42</t>
         </is>
       </c>
-      <c r="B43" s="22" t="inlineStr">
+      <c r="B44" s="22" t="inlineStr">
         <is>
           <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
         </is>
       </c>
-      <c r="C43" s="22" t="inlineStr">
+      <c r="C44" s="22" t="inlineStr">
         <is>
           <t>1. Chạm vào ô mã OTP
 2. Theo dõi request backend nhận được</t>
         </is>
       </c>
-      <c r="D43" s="22" t="inlineStr">
+      <c r="D44" s="22" t="inlineStr">
         <is>
           <t>Ô đang chứa 000000</t>
         </is>
       </c>
-      <c r="E43" s="22" t="inlineStr">
+      <c r="E44" s="22" t="inlineStr">
         <is>
           <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
         </is>
       </c>
-      <c r="F43" s="22" t="inlineStr">
+      <c r="F44" s="22" t="inlineStr">
         <is>
           <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
         </is>
       </c>
-      <c r="G43" s="22" t="inlineStr">
+      <c r="G44" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H43" s="22" t="inlineStr">
+      <c r="H44" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I43" s="22" t="inlineStr">
+      <c r="I44" s="22" t="inlineStr">
         <is>
           <t>`OtpPinInput._handleTextChange` (frontend/mobile/lib/features/auth/presentation/widgets/otp_pin_input.dart:66–72) chạy với mọi thông báo của controller, kể cả khi chỉ đổi vị trí con trỏ lúc chạm ô, và gọi onCompleted hễ ô đủ 6 số → gửi lại mã sai, tốn hạn mức token_verifications
 Log: evidence/test-e2e.log (mục "request backend trong pha 2"), evidence/implement-P10-run-phase2-requests.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="222.5" customHeight="1">
+      <c r="A45" s="22" t="inlineStr">
+        <is>
+          <t>BUG-CATSYNC-01</t>
+        </is>
+      </c>
+      <c r="B45" s="22" t="inlineStr">
+        <is>
+          <t>Đồng bộ lần đầu từ Beat qua broker thật</t>
+        </is>
+      </c>
+      <c r="C45" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC1
+2. Đối chiếu test_beat_triggers_first_sync_and_commits_snapshot__AC1 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="D45" s="22" t="inlineStr">
+        <is>
+          <t>source=dav_drugbank; snapshot 10 thuốc E2E-001..010; thuốc thứ 10 withdrawn; Unicode và khoảng trắng</t>
+        </is>
+      </c>
+      <c r="E45" s="22" t="inlineStr">
+        <is>
+          <t>Một sync scheduler; 10 thuốc normalize đúng; inserted=10, updated=0, failed=0; run thanh_cong/finished_at; tick/delivery/HTTP liên kết cùng ledger.</t>
+        </is>
+      </c>
+      <c r="F45" s="22" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-a61765b49491.json; evidence/test-a61765b49491-worker-0.log</t>
+        </is>
+      </c>
+      <c r="G45" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H45" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I45" s="22" t="inlineStr">
+        <is>
+          <t>CAT-E2E-01/02 đã tái hiện: migration catalog search revoke quyền PUBLIC và chỉ grant api_role, worker_role thiếu EXECUTE catalog_search_key nên INSERT thuốc lỗi InsufficientPrivilege; fail_run tiếp tục lỗi IndeterminateDatatype, run giữ dang_chay.
+Log: evidence/test-integration.log; evidence/test-case-a61765b49491.json; evidence/test-a61765b49491-worker-0.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="222.5" customHeight="1">
+      <c r="A46" s="22" t="inlineStr">
+        <is>
+          <t>BUG-CATSYNC-04</t>
+        </is>
+      </c>
+      <c r="B46" s="22" t="inlineStr">
+        <is>
+          <t>Chạy sync khi thành công đủ hoặc quá 7 ngày</t>
+        </is>
+      </c>
+      <c r="C46" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC2
+2. Đối chiếu test_seven_day_success_is_due__AC2[604800] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="D46" s="22" t="inlineStr">
+        <is>
+          <t>age_seconds=604800</t>
+        </is>
+      </c>
+      <c r="E46" s="22" t="inlineStr">
+        <is>
+          <t>Beat tick enqueue đúng một sync; thuốc đúng; run mới thanh_cong, inserted=10.</t>
+        </is>
+      </c>
+      <c r="F46" s="22" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200]; run statuses=["thanh_cong","dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-7dcadc29d94b.json; evidence/test-7dcadc29d94b-worker-0.log</t>
+        </is>
+      </c>
+      <c r="G46" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H46" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I46" s="22" t="inlineStr">
+        <is>
+          <t>CAT-E2E-01/02 đã tái hiện: migration catalog search revoke quyền PUBLIC và chỉ grant api_role, worker_role thiếu EXECUTE catalog_search_key nên INSERT thuốc lỗi InsufficientPrivilege; fail_run tiếp tục lỗi IndeterminateDatatype, run giữ dang_chay.
+Log: evidence/test-integration.log; evidence/test-case-7dcadc29d94b.json; evidence/test-7dcadc29d94b-worker-0.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="222.5" customHeight="1">
+      <c r="A47" s="22" t="inlineStr">
+        <is>
+          <t>BUG-CATSYNC-05</t>
+        </is>
+      </c>
+      <c r="B47" s="22" t="inlineStr">
+        <is>
+          <t>Chạy sync khi thành công đủ hoặc quá 7 ngày</t>
+        </is>
+      </c>
+      <c r="C47" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC2
+2. Đối chiếu test_seven_day_success_is_due__AC2[604860] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="D47" s="22" t="inlineStr">
+        <is>
+          <t>age_seconds=604860</t>
+        </is>
+      </c>
+      <c r="E47" s="22" t="inlineStr">
+        <is>
+          <t>Beat tick enqueue đúng một sync; thuốc đúng; run mới thanh_cong, inserted=10.</t>
+        </is>
+      </c>
+      <c r="F47" s="22" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200]; run statuses=["thanh_cong","dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-9e8caeaa27f2.json; evidence/test-9e8caeaa27f2-worker-0.log</t>
+        </is>
+      </c>
+      <c r="G47" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H47" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I47" s="22" t="inlineStr">
+        <is>
+          <t>CAT-E2E-01/02 đã tái hiện: migration catalog search revoke quyền PUBLIC và chỉ grant api_role, worker_role thiếu EXECUTE catalog_search_key nên INSERT thuốc lỗi InsufficientPrivilege; fail_run tiếp tục lỗi IndeterminateDatatype, run giữ dang_chay.
+Log: evidence/test-integration.log; evidence/test-case-9e8caeaa27f2.json; evidence/test-9e8caeaa27f2-worker-0.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="222.5" customHeight="1">
+      <c r="A48" s="22" t="inlineStr">
+        <is>
+          <t>BUG-CATSYNC-06</t>
+        </is>
+      </c>
+      <c r="B48" s="22" t="inlineStr">
+        <is>
+          <t>Chặn tick và message trùng khi source đang chạy</t>
+        </is>
+      </c>
+      <c r="C48" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC3
+2. Đối chiếu test_running_source_suppresses_tick_and_duplicate_message__AC3 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="D48" s="22" t="inlineStr">
+        <is>
+          <t>Worker concurrency=2; giữ HTTP đầu ≤20s; publish duplicate cùng source</t>
+        </is>
+      </c>
+      <c r="E48" s="22" t="inlineStr">
+        <is>
+          <t>Một run/fetch; tick và duplicate đã hoàn tất không tạo run/fetch chồng; thả HTTP có một success, thuốc đúng.</t>
+        </is>
+      </c>
+      <c r="F48" s="22" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200]; run statuses=["dang_chay"]; medications=0; deliveries=2. evidence/test-integration.log; evidence/test-case-9d6eedf72a76.json; evidence/test-9d6eedf72a76-worker-0.log</t>
+        </is>
+      </c>
+      <c r="G48" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H48" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I48" s="22" t="inlineStr">
+        <is>
+          <t>CAT-E2E-01/02 đã tái hiện: migration catalog search revoke quyền PUBLIC và chỉ grant api_role, worker_role thiếu EXECUTE catalog_search_key nên INSERT thuốc lỗi InsufficientPrivilege; fail_run tiếp tục lỗi IndeterminateDatatype, run giữ dang_chay.
+Log: evidence/test-integration.log; evidence/test-case-9d6eedf72a76.json; evidence/test-9d6eedf72a76-worker-0.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="222.5" customHeight="1">
+      <c r="A49" s="22" t="inlineStr">
+        <is>
+          <t>BUG-CATSYNC-07</t>
+        </is>
+      </c>
+      <c r="B49" s="22" t="inlineStr">
+        <is>
+          <t>Giữ ID thuốc khi chạy sync lặp</t>
+        </is>
+      </c>
+      <c r="C49" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC4
+2. Đối chiếu test_repeated_broker_sync_preserves_medication_ids__AC4 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="D49" s="22" t="inlineStr">
+        <is>
+          <t>Hai catalog.sync qua RabbitMQ; cùng snapshot 10 thuốc</t>
+        </is>
+      </c>
+      <c r="E49" s="22" t="inlineStr">
+        <is>
+          <t>10 source_ref duy nhất; ID giữ nguyên; counters lần 1=10/0/0, lần 2=0/10/0; không run running.</t>
+        </is>
+      </c>
+      <c r="F49" s="22" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200]; run statuses=["dang_chay"]; medications=0; deliveries=1. Sync đầu không ghi được thuốc nên chưa tới bước so ID lần hai. evidence/test-integration.log; evidence/test-case-4c83c671ad57.json; evidence/test-4c83c671ad57-worker-0.log</t>
+        </is>
+      </c>
+      <c r="G49" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H49" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I49" s="22" t="inlineStr">
+        <is>
+          <t>CAT-E2E-01/02 đã tái hiện: migration catalog search revoke quyền PUBLIC và chỉ grant api_role, worker_role thiếu EXECUTE catalog_search_key nên INSERT thuốc lỗi InsufficientPrivilege; fail_run tiếp tục lỗi IndeterminateDatatype, run giữ dang_chay.
+Log: evidence/test-integration.log; evidence/test-case-4c83c671ad57.json; evidence/test-4c83c671ad57-worker-0.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="222.5" customHeight="1">
+      <c r="A50" s="22" t="inlineStr">
+        <is>
+          <t>BUG-CATSYNC-08</t>
+        </is>
+      </c>
+      <c r="B50" s="22" t="inlineStr">
+        <is>
+          <t>Retry lỗi tạm thời rồi đồng bộ thành công</t>
+        </is>
+      </c>
+      <c r="C50" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC5
+2. Đối chiếu test_transient_http_retries_then_succeeds__AC5[429] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="D50" s="22" t="inlineStr">
+        <is>
+          <t>HTTP=[429,429,429,200]</t>
+        </is>
+      </c>
+      <c r="E50" s="22" t="inlineStr">
+        <is>
+          <t>Cùng task ID; retries 0→1→2→3; ba run that_bai, một thanh_cong; 10 thuốc; không retry thứ 5.</t>
+        </is>
+      </c>
+      <c r="F50" s="22" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[429]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-1cdcf1e60087.json; evidence/test-1cdcf1e60087-worker-0.log</t>
+        </is>
+      </c>
+      <c r="G50" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H50" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I50" s="22" t="inlineStr">
+        <is>
+          <t>CAT-E2E-02 đã tái hiện: repository.fail_run dùng jsonb_build_object('message', :error), PostgreSQL không suy ra kiểu tham số $1 (IndeterminateDatatype). Ghi thất bại rollback, run dang_chay; ProgrammingError che lỗi HTTP/validation, không retry transient.
+Log: evidence/test-integration.log; evidence/test-case-1cdcf1e60087.json; evidence/test-1cdcf1e60087-worker-0.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="222.5" customHeight="1">
+      <c r="A51" s="22" t="inlineStr">
+        <is>
+          <t>BUG-CATSYNC-09</t>
+        </is>
+      </c>
+      <c r="B51" s="22" t="inlineStr">
+        <is>
+          <t>Dừng retry sau bốn attempt lỗi</t>
+        </is>
+      </c>
+      <c r="C51" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC5
+2. Đối chiếu test_transient_http_exhausts_four_attempts__AC5[429] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="D51" s="22" t="inlineStr">
+        <is>
+          <t>HTTP luôn 429; quan sát thêm 10s sau terminal task</t>
+        </is>
+      </c>
+      <c r="E51" s="22" t="inlineStr">
+        <is>
+          <t>Đúng bốn run/HTTP với finished_at; retries 0..3; không attempt 5, thuốc hoặc run dang_chay.</t>
+        </is>
+      </c>
+      <c r="F51" s="22" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[429]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-bffd8e518f38.json; evidence/test-bffd8e518f38-worker-0.log</t>
+        </is>
+      </c>
+      <c r="G51" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H51" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I51" s="22" t="inlineStr">
+        <is>
+          <t>CAT-E2E-02 đã tái hiện: repository.fail_run dùng jsonb_build_object('message', :error), PostgreSQL không suy ra kiểu tham số $1 (IndeterminateDatatype). Ghi thất bại rollback, run dang_chay; ProgrammingError che lỗi HTTP/validation, không retry transient.
+Log: evidence/test-integration.log; evidence/test-case-bffd8e518f38.json; evidence/test-bffd8e518f38-worker-0.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="222.5" customHeight="1">
+      <c r="A52" s="22" t="inlineStr">
+        <is>
+          <t>BUG-CATSYNC-10</t>
+        </is>
+      </c>
+      <c r="B52" s="22" t="inlineStr">
+        <is>
+          <t>Retry lỗi tạm thời rồi đồng bộ thành công</t>
+        </is>
+      </c>
+      <c r="C52" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC5
+2. Đối chiếu test_transient_http_retries_then_succeeds__AC5[500] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="D52" s="22" t="inlineStr">
+        <is>
+          <t>HTTP=[500,500,500,200]</t>
+        </is>
+      </c>
+      <c r="E52" s="22" t="inlineStr">
+        <is>
+          <t>Cùng task ID; retries 0→1→2→3; ba run that_bai, một thanh_cong; 10 thuốc; không retry thứ 5.</t>
+        </is>
+      </c>
+      <c r="F52" s="22" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[500]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-ada0c520b6bc.json; evidence/test-ada0c520b6bc-worker-0.log</t>
+        </is>
+      </c>
+      <c r="G52" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H52" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I52" s="22" t="inlineStr">
+        <is>
+          <t>CAT-E2E-02 đã tái hiện: repository.fail_run dùng jsonb_build_object('message', :error), PostgreSQL không suy ra kiểu tham số $1 (IndeterminateDatatype). Ghi thất bại rollback, run dang_chay; ProgrammingError che lỗi HTTP/validation, không retry transient.
+Log: evidence/test-integration.log; evidence/test-case-ada0c520b6bc.json; evidence/test-ada0c520b6bc-worker-0.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="222.5" customHeight="1">
+      <c r="A53" s="22" t="inlineStr">
+        <is>
+          <t>BUG-CATSYNC-11</t>
+        </is>
+      </c>
+      <c r="B53" s="22" t="inlineStr">
+        <is>
+          <t>Dừng retry sau bốn attempt lỗi</t>
+        </is>
+      </c>
+      <c r="C53" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC5
+2. Đối chiếu test_transient_http_exhausts_four_attempts__AC5[500] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="D53" s="22" t="inlineStr">
+        <is>
+          <t>HTTP luôn 500; quan sát thêm 10s sau terminal task</t>
+        </is>
+      </c>
+      <c r="E53" s="22" t="inlineStr">
+        <is>
+          <t>Đúng bốn run/HTTP với finished_at; retries 0..3; không attempt 5, thuốc hoặc run dang_chay.</t>
+        </is>
+      </c>
+      <c r="F53" s="22" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[500]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-51baed685b8d.json; evidence/test-51baed685b8d-worker-0.log</t>
+        </is>
+      </c>
+      <c r="G53" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H53" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I53" s="22" t="inlineStr">
+        <is>
+          <t>CAT-E2E-02 đã tái hiện: repository.fail_run dùng jsonb_build_object('message', :error), PostgreSQL không suy ra kiểu tham số $1 (IndeterminateDatatype). Ghi thất bại rollback, run dang_chay; ProgrammingError che lỗi HTTP/validation, không retry transient.
+Log: evidence/test-integration.log; evidence/test-case-51baed685b8d.json; evidence/test-51baed685b8d-worker-0.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="222.5" customHeight="1">
+      <c r="A54" s="22" t="inlineStr">
+        <is>
+          <t>BUG-CATSYNC-12</t>
+        </is>
+      </c>
+      <c r="B54" s="22" t="inlineStr">
+        <is>
+          <t>Dừng lỗi HTTP cố định không retry</t>
+        </is>
+      </c>
+      <c r="C54" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC6
+2. Đối chiếu test_permanent_http_failure_has_no_retry__AC6[400] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="D54" s="22" t="inlineStr">
+        <is>
+          <t>HTTP=400</t>
+        </is>
+      </c>
+      <c r="E54" s="22" t="inlineStr">
+        <is>
+          <t>Một attempt/run that_bai có error_details/finished_at; không thuốc, HTTP hoặc retry tiếp theo.</t>
+        </is>
+      </c>
+      <c r="F54" s="22" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[400]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-74f89a8ac834.json; evidence/test-74f89a8ac834-worker-0.log</t>
+        </is>
+      </c>
+      <c r="G54" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H54" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I54" s="22" t="inlineStr">
+        <is>
+          <t>CAT-E2E-02 đã tái hiện: repository.fail_run dùng jsonb_build_object('message', :error), PostgreSQL không suy ra kiểu tham số $1 (IndeterminateDatatype). Ghi thất bại rollback, run dang_chay; ProgrammingError che lỗi HTTP/validation, không retry transient.
+Log: evidence/test-integration.log; evidence/test-case-74f89a8ac834.json; evidence/test-74f89a8ac834-worker-0.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="222.5" customHeight="1">
+      <c r="A55" s="22" t="inlineStr">
+        <is>
+          <t>BUG-CATSYNC-13</t>
+        </is>
+      </c>
+      <c r="B55" s="22" t="inlineStr">
+        <is>
+          <t>Dừng lỗi HTTP cố định không retry</t>
+        </is>
+      </c>
+      <c r="C55" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC6
+2. Đối chiếu test_permanent_http_failure_has_no_retry__AC6[404] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="D55" s="22" t="inlineStr">
+        <is>
+          <t>HTTP=404</t>
+        </is>
+      </c>
+      <c r="E55" s="22" t="inlineStr">
+        <is>
+          <t>Một attempt/run that_bai có error_details/finished_at; không thuốc, HTTP hoặc retry tiếp theo.</t>
+        </is>
+      </c>
+      <c r="F55" s="22" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[404]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-8365039e1953.json; evidence/test-8365039e1953-worker-0.log</t>
+        </is>
+      </c>
+      <c r="G55" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H55" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I55" s="22" t="inlineStr">
+        <is>
+          <t>CAT-E2E-02 đã tái hiện: repository.fail_run dùng jsonb_build_object('message', :error), PostgreSQL không suy ra kiểu tham số $1 (IndeterminateDatatype). Ghi thất bại rollback, run dang_chay; ProgrammingError che lỗi HTTP/validation, không retry transient.
+Log: evidence/test-integration.log; evidence/test-case-8365039e1953.json; evidence/test-8365039e1953-worker-0.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="222.5" customHeight="1">
+      <c r="A56" s="22" t="inlineStr">
+        <is>
+          <t>BUG-CATSYNC-14</t>
+        </is>
+      </c>
+      <c r="B56" s="22" t="inlineStr">
+        <is>
+          <t>Dừng lỗi HTTP cố định không retry</t>
+        </is>
+      </c>
+      <c r="C56" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC6
+2. Đối chiếu test_permanent_http_failure_has_no_retry__AC6[422] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="D56" s="22" t="inlineStr">
+        <is>
+          <t>HTTP=422</t>
+        </is>
+      </c>
+      <c r="E56" s="22" t="inlineStr">
+        <is>
+          <t>Một attempt/run that_bai có error_details/finished_at; không thuốc, HTTP hoặc retry tiếp theo.</t>
+        </is>
+      </c>
+      <c r="F56" s="22" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[422]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-0f684cdce3bb.json; evidence/test-0f684cdce3bb-worker-0.log</t>
+        </is>
+      </c>
+      <c r="G56" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H56" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I56" s="22" t="inlineStr">
+        <is>
+          <t>CAT-E2E-02 đã tái hiện: repository.fail_run dùng jsonb_build_object('message', :error), PostgreSQL không suy ra kiểu tham số $1 (IndeterminateDatatype). Ghi thất bại rollback, run dang_chay; ProgrammingError che lỗi HTTP/validation, không retry transient.
+Log: evidence/test-integration.log; evidence/test-case-0f684cdce3bb.json; evidence/test-0f684cdce3bb-worker-0.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="239" customHeight="1">
+      <c r="A57" s="22" t="inlineStr">
+        <is>
+          <t>BUG-CATSYNC-16</t>
+        </is>
+      </c>
+      <c r="B57" s="22" t="inlineStr">
+        <is>
+          <t>Kết thúc thất bại khi không có thuốc hợp lệ</t>
+        </is>
+      </c>
+      <c r="C57" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC6
+2. Đối chiếu test_no_valid_records_finishes_failed_without_retry__AC6[items0] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="D57" s="22" t="inlineStr">
+        <is>
+          <t>items=[]</t>
+        </is>
+      </c>
+      <c r="E57" s="22" t="inlineStr">
+        <is>
+          <t>Một run that_bai có finished_at/error_details; không thuốc/retry; không suy số HTTP bằng số run vì fetcher có phân trang.</t>
+        </is>
+      </c>
+      <c r="F57" s="22" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-a4b501f0afae.json; evidence/test-a4b501f0afae-worker-0.log</t>
+        </is>
+      </c>
+      <c r="G57" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H57" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I57" s="22" t="inlineStr">
+        <is>
+          <t>CAT-E2E-02 đã tái hiện: repository.fail_run dùng jsonb_build_object('message', :error), PostgreSQL không suy ra kiểu tham số $1 (IndeterminateDatatype). Ghi thất bại rollback, run dang_chay; ProgrammingError che lỗi HTTP/validation, không retry transient.
+Log: evidence/test-integration.log; evidence/test-case-a4b501f0afae.json; evidence/test-a4b501f0afae-worker-0.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="239" customHeight="1">
+      <c r="A58" s="22" t="inlineStr">
+        <is>
+          <t>BUG-CATSYNC-17</t>
+        </is>
+      </c>
+      <c r="B58" s="22" t="inlineStr">
+        <is>
+          <t>Kết thúc thất bại khi không có thuốc hợp lệ</t>
+        </is>
+      </c>
+      <c r="C58" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC6
+2. Đối chiếu test_no_valid_records_finishes_failed_without_retry__AC6[items1] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="D58" s="22" t="inlineStr">
+        <is>
+          <t>items=[{"tenThuoc":"thiếu mã"}]</t>
+        </is>
+      </c>
+      <c r="E58" s="22" t="inlineStr">
+        <is>
+          <t>Một run that_bai có finished_at/error_details; không thuốc/retry; không suy số HTTP bằng số run vì fetcher có phân trang.</t>
+        </is>
+      </c>
+      <c r="F58" s="22" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200,200,200,200,200,200,200,200,200,200]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-ee7e4efcc999.json; evidence/test-ee7e4efcc999-worker-0.log</t>
+        </is>
+      </c>
+      <c r="G58" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H58" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I58" s="22" t="inlineStr">
+        <is>
+          <t>CAT-E2E-02 đã tái hiện: repository.fail_run dùng jsonb_build_object('message', :error), PostgreSQL không suy ra kiểu tham số $1 (IndeterminateDatatype). Ghi thất bại rollback, run dang_chay; ProgrammingError che lỗi HTTP/validation, không retry transient.
+Log: evidence/test-integration.log; evidence/test-case-ee7e4efcc999.json; evidence/test-ee7e4efcc999-worker-0.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="239" customHeight="1">
+      <c r="A59" s="22" t="inlineStr">
+        <is>
+          <t>BUG-CATSYNC-18</t>
+        </is>
+      </c>
+      <c r="B59" s="22" t="inlineStr">
+        <is>
+          <t>Kết thúc thất bại khi không có thuốc hợp lệ</t>
+        </is>
+      </c>
+      <c r="C59" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC6
+2. Đối chiếu test_no_valid_records_finishes_failed_without_retry__AC6[items2] với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="D59" s="22" t="inlineStr">
+        <is>
+          <t>items=[{"soDangKy":"thiếu tên"}]</t>
+        </is>
+      </c>
+      <c r="E59" s="22" t="inlineStr">
+        <is>
+          <t>Một run that_bai có finished_at/error_details; không thuốc/retry; không suy số HTTP bằng số run vì fetcher có phân trang.</t>
+        </is>
+      </c>
+      <c r="F59" s="22" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200,200,200,200,200,200,200,200,200,200]; run statuses=["dang_chay"]; medications=0; deliveries=1. evidence/test-integration.log; evidence/test-case-6d3163f60486.json; evidence/test-6d3163f60486-worker-0.log</t>
+        </is>
+      </c>
+      <c r="G59" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H59" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I59" s="22" t="inlineStr">
+        <is>
+          <t>CAT-E2E-02 đã tái hiện: repository.fail_run dùng jsonb_build_object('message', :error), PostgreSQL không suy ra kiểu tham số $1 (IndeterminateDatatype). Ghi thất bại rollback, run dang_chay; ProgrammingError che lỗi HTTP/validation, không retry transient.
+Log: evidence/test-integration.log; evidence/test-case-6d3163f60486.json; evidence/test-6d3163f60486-worker-0.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="255.5" customHeight="1">
+      <c r="A60" s="22" t="inlineStr">
+        <is>
+          <t>BUG-CATSYNC-19</t>
+        </is>
+      </c>
+      <c r="B60" s="22" t="inlineStr">
+        <is>
+          <t>Khôi phục sau Worker mất trước commit thuốc</t>
+        </is>
+      </c>
+      <c r="C60" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ gốc superproject chạy python tests/e2e/catalog_sync/run_e2e.py --case AC7
+2. Đối chiếu test_worker_loss_before_commit_redelivers_and_recovers__AC7 với dữ liệu nêu dưới; đọc ledger/HTTP/DB JSON trong work/2.22-sync-job-e2e/evidence/.
+3. Kiểm mã thoát, số executed và cleanup; không tính collect/preflight là E2E pass.</t>
+        </is>
+      </c>
+      <c r="D60" s="22" t="inlineStr">
+        <is>
+          <t>HTTP hold; run dang_chay đã commit; thuốc rỗng; broker unacked=1; SIGKILL owned group</t>
+        </is>
+      </c>
+      <c r="E60" s="22" t="inlineStr">
+        <is>
+          <t>Broker redelivers cùng ID/redelivered=true; cuối có 10 thuốc và success, không run treo/trùng; không chỉnh run thủ công để pass.</t>
+        </is>
+      </c>
+      <c r="F60" s="22" t="inlineStr">
+        <is>
+          <t>HTTP statuses=[200]; run statuses=["dang_chay"]; medications=0; deliveries=2. Cùng task ID được broker giao lại với redelivered=true, Worker báo succeeded nhưng run vẫn dang_chay, không thuốc. evidence/test-integration.log; evidence/test-case-e13de4a4b0bf.json; evidence/test-e13de4a4b0bf-worker-0.log</t>
+        </is>
+      </c>
+      <c r="G60" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H60" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I60" s="22" t="inlineStr">
+        <is>
+          <t>CAT-E2E-03 đã tái hiện: start_run đã commit trước fetch; SIGKILL giữ run dang_chay. Broker redelivers cùng ID nhưng start_run conflict trả None và service return, không phục hồi/finish run.
+Log: evidence/test-integration.log; evidence/test-case-e13de4a4b0bf.json; evidence/test-e13de4a4b0bf-worker-0.log</t>
         </is>
       </c>
     </row>
@@ -5310,17 +8279,17 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:A5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11:F12">
+  <conditionalFormatting sqref="F11:F13">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11:G12">
+  <conditionalFormatting sqref="G11:G13">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>OR(G11="Critical",G11="High")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G37:G43">
+  <conditionalFormatting sqref="G38:G60">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
@@ -5332,10 +8301,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G11:G12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G11:G13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="G37:G43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G38:G60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs: align link code docs with QD-04 and add LINKCODE test cases
- Backlog: PB15 and PB19 acceptance criteria, task 3.12 and 3.13
  descriptions now follow QD-04 (one fixed, non-expiring code per user;
  entering a code only creates a pending link request)
- Schema v11: link_codes matches the new migration (UNIQUE per user,
  code format CHECK, narrowed grants)
- Test cases: new sheet "Mã liên kết người thân" (LINKCODE), 33 cases

Refs: 3.10

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Android build" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Đăng nhập người dùng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Lịch uống thuốc" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Tải lịch uống" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Tương tác thuốc-thuốc" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Tương tác thuốc-thực phẩm" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Tra cứu hoạt chất" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Report" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android build" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đăng nhập người dùng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lịch uống thuốc" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tải lịch uống" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tương tác thuốc-thuốc" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tương tác thuốc-thực phẩm" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tra cứu hoạt chất" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mã liên kết người thân" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Android build'!$A$8:$I$17</definedName>
@@ -23,6 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tương tác thuốc-thuốc'!$A$8:$I$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Tương tác thuốc-thực phẩm'!$A$8:$I$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Tra cứu hoạt chất'!$A$8:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Mã liên kết người thân'!$A$8:$I$41</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -325,13 +327,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -355,18 +357,18 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$17</f>
+              <f>'Report'!$A$11:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$11:$D$17</f>
+              <f>'Report'!$D$11:$D$18</f>
             </numRef>
           </val>
         </ser>
@@ -379,18 +381,18 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$17</f>
+              <f>'Report'!$A$11:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$11:$E$17</f>
+              <f>'Report'!$E$11:$E$18</f>
             </numRef>
           </val>
         </ser>
@@ -403,18 +405,18 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$17</f>
+              <f>'Report'!$A$11:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$11:$F$17</f>
+              <f>'Report'!$F$11:$F$18</f>
             </numRef>
           </val>
         </ser>
@@ -460,13 +462,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -484,7 +486,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -512,12 +514,12 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>19</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -527,9 +529,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -539,7 +541,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>19</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3240000"/>
@@ -549,9 +551,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -12648,7 +12650,2060 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:U47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Mã liên kết người thân (LINKCODE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Kết quả GET /family/link-code</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="107" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Lấy mã liên kết lần đầu khi user chưa có mã</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>User thường đã đăng nhập (phiên mobile), chưa có dòng link_codes</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /family/link-code với header Authorization của user
+2. Kiểm bảng link_codes theo patient_user_id</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Authorization: Bearer &lt;phiên mobile của U&gt;</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>200; body chỉ có code (10 ký tự khớp ^[A-HJKMNP-Z2-9]{10}$) và qr_payload; DB có đúng 1 dòng link_codes của U với code trùng response</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>200, body {code, qr_payload} đúng định dạng; đúng 1 dòng link_codes của U</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · EP (1) · Decision Table (R4) · test_first_call_creates_one_row__AC1</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>Phiên gọi (header Authorization)</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>Phiên mobile hợp lệ của tài khoản cá nhân</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>Không có header
+Token sai
+Token của tài khoản đã xóa dữ liệu
+Token của user không tồn tại
+Phiên của tài khoản admin</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>3
+4
+5
+6
+7</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Phiên hợp lệ, tài khoản còn?</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="57.5" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Gọi lại nhiều lần trả đúng mã cũ</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>User U đã có mã C (đã gọi endpoint một lần)</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /family/link-code 3 lần với phiên của U
+2. Kiểm bảng link_codes của U</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>3 lần gọi liên tiếp</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Cả 3 lần 200 với cùng body; vẫn 1 dòng, code và created_at không đổi</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>3 lần 200, body giống hệt lần đầu; 1 dòng, created_at không đổi</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · Decision Table (R3) · test_repeated_calls_return_same_code__AC2</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>Mã liên kết (code)</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>10 ký tự thuộc A–Z, 2–9, bỏ 0 O 1 I L</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>Có ký tự dễ nhầm 0, O, 1, I, L
+Chữ thường
+Độ dài khác 10</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>8
+9
+10</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>Tài khoản admin?</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="107" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Chờ request khác đang tạo mã cho cùng user rồi trả đúng mã đó</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>User U chưa có mã; một kết nối khác đã INSERT mã M cho U trong transaction chưa commit</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /family/link-code của U trong thread riêng
+2. Xác nhận request đang chờ khóa (pg_stat_activity)
+3. Commit transaction của kết nối kia
+4. Đợi request trả về</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>M = mã ngẫu nhiên hợp lệ</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>200 với code = M; DB chỉ có 1 dòng của U; không 5xx</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Request chờ khóa, sau commit trả 200 với code = M; 1 dòng. Chạy lặp 5 lần đều pass</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · Đoán lỗi (chạy đua) · test_waits_for_concurrent_insert_and_returns_its_code__AC3</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>User đã có mã?</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U11" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="57.5" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Hai request đầu tiên gửi đồng thời nhận cùng một mã</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>User U chưa có mã</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi đồng thời 2 request GET /family/link-code của U (Barrier)
+2. Kiểm bảng link_codes của U</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>2 thread cùng phiên của U</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Cả hai 200, cùng body; đúng 1 dòng của U</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Cả hai 200, cùng code; 1 dòng. Chạy lặp 5 lần đều pass</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · Đoán lỗi (gửi trùng) · test_parallel_first_calls_same_code__AC3</t>
+        </is>
+      </c>
+      <c r="Q12" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="41" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Sinh 10.000 mã đều đúng độ dài và bảng ký tự</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Không cần DB</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi generate_code() 10.000 lần
+2. Kiểm độ dài và ký tự của từng mã</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>10.000 mã</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Mọi mã dài 10, chỉ gồm ký tự trong ALPHABET; không trùng nhau</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>10.000 mã dài 10, đúng bảng ký tự, không trùng</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (1) · test_generate_code_length_and_alphabet__AC4</t>
+        </is>
+      </c>
+      <c r="Q13" s="10" t="inlineStr">
+        <is>
+          <t>401, không ghi gì</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S13" s="11" t="inlineStr"/>
+      <c r="T13" s="11" t="inlineStr"/>
+      <c r="U13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="57.5" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Bảng ký tự không chứa ký tự dễ nhầm</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Không cần DB</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. Đọc ALPHABET
+2. So với tập 0 O 1 I L</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>ALPHABET = ABCDEFGHJKMNPQRSTUVWXYZ23456789</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>31 ký tự phân biệt; không có 0, O, 1, I, L</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>31 ký tự, không có ký tự dễ nhầm</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (2) · test_alphabet_excludes_confusable_characters__AC4</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>403 khong_co_quyen, không ghi gì</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr"/>
+      <c r="S14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T14" s="11" t="inlineStr"/>
+      <c r="U14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="90.5" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Mã được sinh bằng nguồn ngẫu nhiên an toàn</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Không cần DB</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. Kiểm giá trị mặc định của generate_code
+2. Quét mã nguồn module family tìm import random</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>src/drugtime/modules/family/**</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Mặc định dùng secrets.choice; không file nào import random</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Mặc định secrets.choice; không có import random</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · Đoán lỗi (bảo mật) · test_generate_code_defaults_to_secrets_choice__AC4, test_family_module_does_not_import_random__AC4</t>
+        </is>
+      </c>
+      <c r="Q15" s="10" t="inlineStr">
+        <is>
+          <t>200, trả mã cũ, không ghi gì</t>
+        </is>
+      </c>
+      <c r="R15" s="11" t="inlineStr"/>
+      <c r="S15" s="11" t="inlineStr"/>
+      <c r="T15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16" ht="57.5" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Tách mã từ qr_payload được đúng code</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>User thường đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /family/link-code
+2. Phân tích qr_payload như URL, lấy tham số code</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>qr_payload trong response</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>qr_payload = drugtime://link?code=&lt;code&gt;; scheme drugtime, host link, tham số code = code</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Đúng định dạng; tham số code bằng code của response</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · test_qr_payload_contains_code__AC5, test_qr_payload_roundtrip__AC5</t>
+        </is>
+      </c>
+      <c r="Q16" s="10" t="inlineStr">
+        <is>
+          <t>200, sinh và lưu một mã mới</t>
+        </is>
+      </c>
+      <c r="R16" s="11" t="inlineStr"/>
+      <c r="S16" s="11" t="inlineStr"/>
+      <c r="T16" s="11" t="inlineStr"/>
+      <c r="U16" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90.5" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Không lấy được hoặc tạo mã cho user khác bằng tham số query</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Hai user thường U, V; V chưa có mã</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. U gọi GET /family/link-code
+2. U gọi GET /family/link-code?patient_user_id=&lt;V&gt;&amp;user_id=&lt;V&gt;
+3. Kiểm link_codes của V
+4. V gọi GET /family/link-code</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>patient_user_id = id của V</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Lần 2 vẫn trả mã của U; V không có dòng nào cho tới khi V tự gọi; mã của V khác mã của U</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Trả mã của U; V không có dòng; sau đó V nhận mã riêng, khác mã của U</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · Đoán lỗi (truy cập dữ liệu người khác) · test_codes_are_per_user_and_query_ignored__AC6</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="57.5" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Sinh lại khi mã trùng với mã của user khác</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Mã đầu tiên sinh ra đã thuộc user khác (fake repository)</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi use case get_link_code với generate trả lần lượt mã đã có rồi mã mới</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>TAKEN23456 (đã có), FRESH23456</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Trả FRESH23456; insert được gọi 2 lần</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Trả FRESH23456 sau 2 lần insert</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · Đoán lỗi (trùng mã) · test_retries_on_code_collision__AC7</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="74" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Trả 503 link_code_unavailable khi trùng mã ở cả 5 lần thử</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Mọi mã sinh ra đều đã thuộc user khác (fake repository)</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi use case get_link_code với generate luôn trả mã đã có</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>TAKEN23456 × 5</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>ServiceUnavailable("link_code_unavailable") (HTTP 503) sau đúng 5 lần insert; không lưu gì; message không chứa mã</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>ServiceUnavailable link_code_unavailable sau 5 lần; không lưu; message không có mã</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · AC10 · BVA (max = 5 lần thử) · test_gives_up_after_max_attempts_503__AC7, test_errors_do_not_contain_code__AC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="57.5" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Gọi không có header Authorization</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Không đăng nhập</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /family/link-code không có header Authorization
+2. Đếm dòng link_codes trước và sau</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>401; số dòng link_codes không đổi</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>401; không có dòng mới</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (2) · Decision Table (R1) · test_unauthenticated_401_no_row__AC8[no_header]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="57.5" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-13</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Gọi với token sai</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Không có phiên hợp lệ</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /family/link-code với Authorization: Bearer not-a-valid-token</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Bearer not-a-valid-token</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>401; không có dòng mới</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>401; không có dòng mới</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (3) · Decision Table (R1) · test_unauthenticated_401_no_row__AC8[bad_token]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="57.5" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-14</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Gọi bằng token của tài khoản đã xóa dữ liệu</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>User U có phiên mobile hợp lệ, sau đó users.erased_at được đặt</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /family/link-code với token của U</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Token đúng chữ ký, tài khoản đã xóa</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>401; U không có dòng link_codes</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>401; không có dòng</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (4) · Decision Table (R1) · test_unauthenticated_401_no_row__AC8[erased_account]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="57.5" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Gọi bằng token của user không tồn tại</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Token đúng chữ ký với sub là UUID ngẫu nhiên không có trong users</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /family/link-code với token đó</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>sub = uuid4() ngẫu nhiên</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (5) · test_unknown_user_token_401</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="74" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-16</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Tài khoản admin bị từ chối lấy mã</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Tài khoản admin có phiên admin_web</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /family/link-code với phiên admin
+2. Đếm dòng link_codes trước và sau</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Phiên admin_web</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>403 {"detail": "khong_co_quyen"}; không có dòng mới</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>403 {"detail": "khong_co_quyen"}; không có dòng mới</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · EP (6) · Decision Table (R2) · test_admin_403_khong_co_quyen_no_row__AC9, test_admin_forbidden_before_any_query__AC9</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="57.5" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-17</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Mã và qr_payload không xuất hiện trong log ứng dụng</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Logger drugtime ở mức DEBUG</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi GET /family/link-code 2 lần (sinh mã, rồi lấy lại)
+2. Tìm code và qr_payload trong log bắt được</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>caplog</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Không dòng log nào chứa code hay qr_payload</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Không có</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · Đoán lỗi (bí mật) · test_code_not_logged__AC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="57.5" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-18</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Bảng link_codes sau migration chỉ còn cột của mô hình mã cố định</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>supabase db reset (10 migration)</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. Đọc information_schema.columns và pg_indexes của link_codes</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Cột: id, patient_user_id, code, created_at; index: link_codes_code_key, link_codes_patient_user_id_key, link_codes_pkey</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · test_link_codes_columns_after_migration__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="41" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-19</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>DB từ chối mã thứ hai cho cùng một user</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>User U đã có một dòng link_codes</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. INSERT dòng link_codes thứ hai cho U với mã khác</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Mã ngẫu nhiên hợp lệ</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Lỗi vi phạm link_codes_patient_user_id_key; U vẫn 1 dòng</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Lỗi link_codes_patient_user_id_key; vẫn 1 dòng</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · test_second_code_for_same_user_rejected__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="41" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-20</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>DB từ chối mã trùng của hai user khác nhau</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>User U có mã C</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. INSERT dòng link_codes cho user V với cùng mã C</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>C của U</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Lỗi vi phạm link_codes_code_key; V không có dòng</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Lỗi link_codes_code_key; V không có dòng</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · test_duplicate_code_rejected__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="123.5" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-21</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Migration dọn trùng giữ đúng dòng mới nhất và xóa mã sai định dạng</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>DB reset về 20261011164026 (trước migration), schema cũ. A: 2 mã hợp lệ (cách nhau 1 ngày); B: 1 mã hợp lệ; C: chỉ có mã sai định dạng; D: mã hợp lệ (cũ hơn) + mã sai định dạng (mới hơn)</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. supabase migration up --local
+2. Đọc link_codes của A, B, C, D
+3. supabase db reset lại đầy đủ</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>A: AAAAAAAAA2 (cũ), AAAAAAAAA3 (mới); B: BBBBBBBBB2; C: LEGACYIO01; D: DDDDDDDDD2 (cũ), legacy-d0 (mới)</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>A còn AAAAAAAAA3; B còn BBBBBBBBB2; C không còn dòng; D còn DDDDDDDDD2</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>A: AAAAAAAAA3; B: BBBBBBBBB2; C: không có dòng; D: DDDDDDDDD2</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · Review F1 · Chuyển trạng thái (schema cũ → mới) · scratch/verify_link_codes_dedupe.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="57.5" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-22</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>api_role chỉ đọc và tạo được mã</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Kết nối bằng api_role; mỗi thao tác trong transaction riêng rồi rollback</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>1. SELECT, INSERT, UPDATE, DELETE trên link_codes bằng api_role</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>SELECT, INSERT thành công; UPDATE, DELETE bị từ chối (permission denied)</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>AC13 · test_role_grants_on_link_codes__AC13[api_role-*]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="57.5" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-23</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>worker_role chỉ đọc và xóa được mã</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Kết nối bằng worker_role; mỗi thao tác trong transaction riêng rồi rollback</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>1. SELECT, INSERT, UPDATE, DELETE trên link_codes bằng worker_role</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>SELECT, DELETE thành công; INSERT, UPDATE bị từ chối (permission denied)</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>AC13 · test_role_grants_on_link_codes__AC13[worker_role-*]</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="74" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-24</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Xóa dữ liệu user xóa đúng mã của user đó</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>User U và V đều có mã</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy family.eraser.erase_user(U) bằng kết nối worker_role
+2. Đọc link_codes của U và V</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Không lỗi; U không còn mã; mã của V còn nguyên</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Không lỗi; U hết mã; V còn mã</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>AC14 · test_family_eraser_deletes_only_that_users_code__AC14, test_sql_erase_deletes_link_code_without_family_column__AC14</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="57.5" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-25</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>OpenAPI của app khớp hợp đồng api_contract</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>api_contract/openapi.json có GET /family/link-code</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>1. So operationId, tập response code, hình dạng và ràng buộc response 200 giữa app và contract</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>operationId getMyLinkCode; response ⊆; code/qr_payload cùng pattern, minLength, maxLength; additionalProperties false</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Khớp</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>AC15 · test_operation_matches_contract__AC15, test_link_code_constraints_match_contract__AC15</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="41" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-BVA-01</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Contract từ chối mã 9 ký tự</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Schema LinkCode trong api_contract/openapi.json</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>1. Validate body có code 9 ký tự với schema LinkCode</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>code = ABCDEFGHJ</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>Bị từ chối</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Bị từ chối</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · BVA (min-1) · EP (4) · scratch/check_link_code.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="41" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-BVA-02</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Contract nhận mã đúng 10 ký tự</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Schema LinkCode</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>1. Validate body có code 10 ký tự hợp lệ</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>code = ABCDEFGHJK</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>Hợp lệ</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Hợp lệ</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · BVA (min = max) · EP (1) · scratch/check_link_code.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="41" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-BVA-03</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Contract từ chối mã 11 ký tự</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Schema LinkCode</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>1. Validate body có code 11 ký tự</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>code = ABCDEFGHJKM</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>Bị từ chối</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>Bị từ chối</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · BVA (max+1) · EP (4) · scratch/check_link_code.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="57.5" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-26</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Contract từ chối mã có ký tự dễ nhầm hoặc chữ thường</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Schema LinkCode</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>1. Validate lần lượt mã chứa O, I, L, 0, 1 và mã chữ thường</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>ABCDEFGHJO, ABCDEFGHJI, ABCDEFGHJL, ABCDEFGHJ0, ABCDEFGHJ1, abcdefghjk</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Cả 6 bị từ chối</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Cả 6 bị từ chối</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (2,3) · scratch/check_link_code.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="90.5" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-27</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Backlog và tài liệu schema khớp QD-04, giữ nguyên biểu đồ</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>docs trên nhánh feat/3.10-qr-referral-code-generation-api</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy scratch/update_backlog_xlsx.py (kiểm so với bản gốc)
+2. Mở backlog bằng Excel (chỉ đọc)
+3. grep block link_codes trong drugtime_schema_v11.sql</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Product-and-Sprint-backlog-DrugTime.xlsx, drugtime_schema_v11.sql</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>PB15, PB19, mô tả 3.12, 3.13 là chuỗi mới; không còn 24h, /links/generate, /links/redeem; 107 phần, 12 chart; Excel mở không báo sửa file; schema không còn expires_at, is_used, family_user_id</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>ALL OK; Excel mở được, 18 sheet, 12 chart; schema đúng</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>AC17 · manual + script</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="107" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-28</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Toàn bộ unit test, architecture test và ruff toàn repo pass</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>backend trên nhánh task; venv backend/.venv</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>1. pytest tests/unit tests/architecture -q
+2. ruff check .
+3. So với baseline trước khi sửa code</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>pytest và ruff đều pass</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>697 pass, 1 fail (tests/unit/test_app.py::test_doses_batch_openapi_uses_contract_shape: NameError paths); ruff toàn repo 21 lỗi ở module khác. Fail và lỗi ruff đã có trước khi task sửa code; file của task pass ruff</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>AC16 · implement-baseline-unit.log, implement-final-backend.log, implement-ruff.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="74" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-29</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>DB từ chối lưu mã sai định dạng</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>supabase db reset (migration có link_codes_code_format_check); user U chưa có mã</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>1. INSERT link_codes cho U với từng mã sai định dạng
+2. Đọc link_codes của U</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>LEGACYIO01 (ký tự dễ nhầm) | abcdefghjk (chữ thường) | ABCDEFGHJ (9 ký tự) | ABCDEFGHJKM (11 ký tự)</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Cả 4 lần bị từ chối với lỗi vi phạm link_codes_code_format_check; U không có dòng nào</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>Cả 4 bị từ chối bởi link_codes_code_format_check; U không có dòng</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · Review F1 · EP (2,3,4) · BVA (min-1, max+1) · test_code_format_check_rejects_invalid_code__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="90.5" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCODE-30</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>User không bị kẹt khi có mã kiểu cũ sai định dạng</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>DB theo migration mới; thử chèn mã kiểu cũ LEGACYIO01 cho user U (trước bản sửa: chèn được và API trả 500 vĩnh viễn)</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>1. INSERT link_codes(U, 'LEGACYIO01')
+2. GET /family/link-code của U hai lần</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>LEGACYIO01</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>INSERT bị từ chối (link_codes_code_format_check); hai lần gọi đều 200 với cùng một mã mới hợp lệ</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>INSERT bị từ chối; 200 cả hai lần, cùng mã 6QQDTXZBHK</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · AC2 · Review F1 · Đoán lỗi (dữ liệu cũ) · scratch/probe_legacy_code.py (trước sửa: evidence/review-probe-legacy-code.log, 500 × 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44">
+      <c r="G44" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H44" s="13">
+        <f>COUNTIF(H9:H41,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="G45" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H45" s="13">
+        <f>COUNTIF(H9:H41,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="G46" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H46" s="13">
+        <f>COUNTIF(H9:H41,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="G47" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H47" s="13">
+        <f>SUM(H44:H46)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I41"/>
+  <conditionalFormatting sqref="H9:H41">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12693,7 +14748,7 @@
         </is>
       </c>
       <c r="C3" s="11">
-        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59+'Lịch uống thuốc'!$H$51+'Tải lịch uống'!$H$32+'Tương tác thuốc-thuốc'!$H$52+'Tương tác thuốc-thực phẩm'!$H$17+'Tra cứu hoạt chất'!$H$17</f>
+        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59+'Lịch uống thuốc'!$H$51+'Tải lịch uống'!$H$32+'Tương tác thuốc-thuốc'!$H$52+'Tương tác thuốc-thực phẩm'!$H$17+'Tra cứu hoạt chất'!$H$17+'Mã liên kết người thân'!$H$44</f>
         <v/>
       </c>
       <c r="D3" s="15">
@@ -12709,7 +14764,7 @@
         </is>
       </c>
       <c r="C4" s="11">
-        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60+'Lịch uống thuốc'!$H$52+'Tải lịch uống'!$H$33+'Tương tác thuốc-thuốc'!$H$53+'Tương tác thuốc-thực phẩm'!$H$18+'Tra cứu hoạt chất'!$H$18</f>
+        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60+'Lịch uống thuốc'!$H$52+'Tải lịch uống'!$H$33+'Tương tác thuốc-thuốc'!$H$53+'Tương tác thuốc-thực phẩm'!$H$18+'Tra cứu hoạt chất'!$H$18+'Mã liên kết người thân'!$H$45</f>
         <v/>
       </c>
       <c r="D4" s="15">
@@ -12741,7 +14796,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr"/>
       <c r="C6" s="11">
-        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61+'Lịch uống thuốc'!$H$53+'Tải lịch uống'!$H$34+'Tương tác thuốc-thuốc'!$H$54+'Tương tác thuốc-thực phẩm'!$H$19+'Tra cứu hoạt chất'!$H$19</f>
+        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61+'Lịch uống thuốc'!$H$53+'Tải lịch uống'!$H$34+'Tương tác thuốc-thuốc'!$H$54+'Tương tác thuốc-thực phẩm'!$H$19+'Tra cứu hoạt chất'!$H$19+'Mã liên kết người thân'!$H$46</f>
         <v/>
       </c>
       <c r="D6" s="15">
@@ -13120,396 +15175,490 @@
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="19" t="inlineStr">
+    <row r="18" ht="156.5" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Mã liên kết người thân</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>User lấy mã liên kết cố định, không hết hạn của mình (kèm QR payload) để mời người thân: GET /family/link-code; mỗi user đúng một mã (QD-04, QD-34). Task 3.10, PB15.</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Mã liên kết người thân</t>
+        </is>
+      </c>
+      <c r="D18" s="18">
+        <f>IFERROR(('Mã liên kết người thân'!$H$47-'Mã liên kết người thân'!$H$46)/'Mã liên kết người thân'!$H$47,0)</f>
+        <v/>
+      </c>
+      <c r="E18" s="18">
+        <f>IFERROR('Mã liên kết người thân'!$H$44/'Mã liên kết người thân'!$H$47,0)</f>
+        <v/>
+      </c>
+      <c r="F18" s="18">
+        <f>IFERROR('Mã liên kết người thân'!$H$45/'Mã liên kết người thân'!$H$47,0)</f>
+        <v/>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động của chức năng (tích hợp với Postgres thật, app chạy bằng api_role; unit; contract) pass, kể cả sau bản sửa F1 của review (mã kiểu cũ sai định dạng bị xóa khi migrate, DB có CHECK định dạng). Một Fail: bộ unit test toàn repo và ruff toàn repo còn lỗi có sẵn trên main ở module khác, không do task này.</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="19" t="inlineStr">
         <is>
           <t>Bug Report</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="20" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="B41" s="20" t="inlineStr">
+      <c r="B42" s="20" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C41" s="20" t="inlineStr">
+      <c r="C42" s="20" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="D41" s="20" t="inlineStr">
+      <c r="D42" s="20" t="inlineStr">
         <is>
           <t>Input Data</t>
         </is>
       </c>
-      <c r="E41" s="20" t="inlineStr">
+      <c r="E42" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F41" s="20" t="inlineStr">
+      <c r="F42" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="G41" s="20" t="inlineStr">
+      <c r="G42" s="20" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="H41" s="20" t="inlineStr">
+      <c r="H42" s="20" t="inlineStr">
         <is>
           <t>Name of Tester</t>
         </is>
       </c>
-      <c r="I41" s="20" t="inlineStr">
+      <c r="I42" s="20" t="inlineStr">
         <is>
           <t>Logs</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="123.5" customHeight="1">
-      <c r="A42" s="22" t="inlineStr">
+    <row r="43" ht="123.5" customHeight="1">
+      <c r="A43" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-08</t>
         </is>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B43" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
         </is>
       </c>
-      <c r="C42" s="22" t="inlineStr">
+      <c r="C43" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
 2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
         </is>
       </c>
-      <c r="D42" s="22" t="inlineStr">
+      <c r="D43" s="22" t="inlineStr">
         <is>
           <t>phone: 0900000001 + ký tự \n</t>
         </is>
       </c>
-      <c r="E42" s="22" t="inlineStr">
+      <c r="E43" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F42" s="22" t="inlineStr">
+      <c r="F43" s="22" t="inlineStr">
         <is>
           <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
         </is>
       </c>
-      <c r="G42" s="22" t="inlineStr">
+      <c r="G43" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H42" s="22" t="inlineStr">
+      <c r="H43" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I42" s="22" t="inlineStr">
+      <c r="I43" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn — kỳ vọng AC6 mâu thuẫn AC5: backend `_validate_required_text` (sign_in.py:178) `strip()` mọi ký tự trắng hai đầu, nên \n cuối được xử lý như khoảng trắng hai đầu mà AC5 coi là hợp lệ. Cần người dùng chốt: sửa AC6 hoặc sửa backend
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="123.5" customHeight="1">
-      <c r="A43" s="22" t="inlineStr">
+    <row r="44" ht="123.5" customHeight="1">
+      <c r="A44" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-11</t>
         </is>
       </c>
-      <c r="B43" s="22" t="inlineStr">
+      <c r="B44" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
         </is>
       </c>
-      <c r="C43" s="22" t="inlineStr">
+      <c r="C44" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone}
 2. POST /auth/mobile/verify {phone, token: 123456}</t>
         </is>
       </c>
-      <c r="D43" s="22" t="inlineStr">
+      <c r="D44" s="22" t="inlineStr">
         <is>
           <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
         </is>
       </c>
-      <c r="E43" s="22" t="inlineStr">
+      <c r="E44" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
         </is>
       </c>
-      <c r="F43" s="22" t="inlineStr">
+      <c r="F44" s="22" t="inlineStr">
         <is>
           <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
         </is>
       </c>
-      <c r="G43" s="22" t="inlineStr">
+      <c r="G44" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H43" s="22" t="inlineStr">
+      <c r="H44" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I43" s="22" t="inlineStr">
+      <c r="I44" s="22" t="inlineStr">
         <is>
           <t>`_normalize_phone` (sign_in.py:197–206) kiểm bằng `str.isdigit()`, nhận cả chữ số Unicode, nên số lọt qua kiểm tra và gửi tới Supabase. Ô nhập của app chỉ cho 0-9 nên người dùng app không gặp; lỗi ở tầng API
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="189.5" customHeight="1">
-      <c r="A44" s="22" t="inlineStr">
+    <row r="45" ht="189.5" customHeight="1">
+      <c r="A45" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-25</t>
         </is>
       </c>
-      <c r="B44" s="22" t="inlineStr">
+      <c r="B45" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên có ký tự NUL</t>
         </is>
       </c>
-      <c r="C44" s="22" t="inlineStr">
+      <c r="C45" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
         </is>
       </c>
-      <c r="D44" s="22" t="inlineStr">
+      <c r="D45" s="22" t="inlineStr">
         <is>
           <t>ho_ten: abc\u0000def</t>
         </is>
       </c>
-      <c r="E44" s="22" t="inlineStr">
+      <c r="E45" s="22" t="inlineStr">
         <is>
           <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
         </is>
       </c>
-      <c r="F44" s="22" t="inlineStr">
+      <c r="F45" s="22" t="inlineStr">
         <is>
           <t>500 Internal Server Error</t>
         </is>
       </c>
-      <c r="G44" s="22" t="inlineStr">
+      <c r="G45" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H44" s="22" t="inlineStr">
+      <c r="H45" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I44" s="22" t="inlineStr">
+      <c r="I45" s="22" t="inlineStr">
         <is>
           <t>`_validate_required_text` (sign_in.py:178) không chặn ký tự điều khiển; PostgreSQL từ chối NUL trong cột text: `psycopg.DataError: PostgreSQL text fields cannot contain NUL (0x00) bytes` ở `UPDATE users SET full_name…` (SqlUsers.update_profile); không có handler cho DataError nên thành 500. Câu SQL có tham số nên không phải lỗ hổng SQL injection
 Log: evidence/test-integration.log, evidence/test-probe-nul.log</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="90.5" customHeight="1">
-      <c r="A45" s="22" t="inlineStr">
+    <row r="46" ht="90.5" customHeight="1">
+      <c r="A46" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-30</t>
         </is>
       </c>
-      <c r="B45" s="22" t="inlineStr">
+      <c r="B46" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên dài 256 ký tự</t>
         </is>
       </c>
-      <c r="C45" s="22" t="inlineStr">
+      <c r="C46" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: A*256}</t>
         </is>
       </c>
-      <c r="D45" s="22" t="inlineStr">
+      <c r="D46" s="22" t="inlineStr">
         <is>
           <t>A*256</t>
         </is>
       </c>
-      <c r="E45" s="22" t="inlineStr">
+      <c r="E46" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F45" s="22" t="inlineStr">
+      <c r="F46" s="22" t="inlineStr">
         <is>
           <t>204, đã lưu</t>
         </is>
       </c>
-      <c r="G45" s="22" t="inlineStr">
+      <c r="G46" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H45" s="22" t="inlineStr">
+      <c r="H46" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I45" s="22" t="inlineStr">
+      <c r="I46" s="22" t="inlineStr">
         <is>
           <t>Không có giới hạn độ dài họ tên: `_validate_profile` (sign_in.py) chỉ kiểm rỗng; cột users.full_name kiểu text không giới hạn
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="90.5" customHeight="1">
-      <c r="A46" s="22" t="inlineStr">
+    <row r="47" ht="90.5" customHeight="1">
+      <c r="A47" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-32</t>
         </is>
       </c>
-      <c r="B46" s="22" t="inlineStr">
+      <c r="B47" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh trước 1900-01-01</t>
         </is>
       </c>
-      <c r="C46" s="22" t="inlineStr">
+      <c r="C47" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh}</t>
         </is>
       </c>
-      <c r="D46" s="22" t="inlineStr">
+      <c r="D47" s="22" t="inlineStr">
         <is>
           <t>1899-12-31 | 0001-01-01</t>
         </is>
       </c>
-      <c r="E46" s="22" t="inlineStr">
+      <c r="E47" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
         </is>
       </c>
-      <c r="F46" s="22" t="inlineStr">
+      <c r="F47" s="22" t="inlineStr">
         <is>
           <t>204 ở cả hai giá trị, đã lưu</t>
         </is>
       </c>
-      <c r="G46" s="22" t="inlineStr">
+      <c r="G47" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H46" s="22" t="inlineStr">
+      <c r="H47" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I46" s="22" t="inlineStr">
+      <c r="I47" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:229–231) chỉ chặn ngày tương lai, không có cận dưới. App mobile đã giới hạn date picker từ 1900 nên chỉ gặp khi gọi API trực tiếp
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="123.5" customHeight="1">
-      <c r="A47" s="22" t="inlineStr">
+    <row r="48" ht="123.5" customHeight="1">
+      <c r="A48" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-35</t>
         </is>
       </c>
-      <c r="B47" s="22" t="inlineStr">
+      <c r="B48" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
         </is>
       </c>
-      <c r="C47" s="22" t="inlineStr">
+      <c r="C48" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
         </is>
       </c>
-      <c r="D47" s="22" t="inlineStr">
+      <c r="D48" s="22" t="inlineStr">
         <is>
           <t>ngay_sinh: 2026-10-08</t>
         </is>
       </c>
-      <c r="E47" s="22" t="inlineStr">
+      <c r="E48" s="22" t="inlineStr">
         <is>
           <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
         </is>
       </c>
-      <c r="F47" s="22" t="inlineStr">
+      <c r="F48" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_date_of_birth"}</t>
         </is>
       </c>
-      <c r="G47" s="22" t="inlineStr">
+      <c r="G48" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H47" s="22" t="inlineStr">
+      <c r="H48" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I47" s="22" t="inlineStr">
+      <c r="I48" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:230) so với `now.date()` trong khi `now()` (shared/clock.py) trả giờ UTC: từ 00:00 đến 07:00 giờ VN, "hôm nay" bị coi là ngày mai. Vi phạm bất biến 7 (múi giờ cố định Asia/Ho_Chi_Minh)
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="173" customHeight="1">
-      <c r="A48" s="22" t="inlineStr">
+    <row r="49" ht="173" customHeight="1">
+      <c r="A49" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-42</t>
         </is>
       </c>
-      <c r="B48" s="22" t="inlineStr">
+      <c r="B49" s="22" t="inlineStr">
         <is>
           <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
         </is>
       </c>
-      <c r="C48" s="22" t="inlineStr">
+      <c r="C49" s="22" t="inlineStr">
         <is>
           <t>1. Chạm vào ô mã OTP
 2. Theo dõi request backend nhận được</t>
         </is>
       </c>
-      <c r="D48" s="22" t="inlineStr">
+      <c r="D49" s="22" t="inlineStr">
         <is>
           <t>Ô đang chứa 000000</t>
         </is>
       </c>
-      <c r="E48" s="22" t="inlineStr">
+      <c r="E49" s="22" t="inlineStr">
         <is>
           <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
         </is>
       </c>
-      <c r="F48" s="22" t="inlineStr">
+      <c r="F49" s="22" t="inlineStr">
         <is>
           <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
         </is>
       </c>
-      <c r="G48" s="22" t="inlineStr">
+      <c r="G49" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H48" s="22" t="inlineStr">
+      <c r="H49" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I48" s="22" t="inlineStr">
+      <c r="I49" s="22" t="inlineStr">
         <is>
           <t>`OtpPinInput._handleTextChange` (frontend/mobile/lib/features/auth/presentation/widgets/otp_pin_input.dart:66–72) chạy với mọi thông báo của controller, kể cả khi chỉ đổi vị trí con trỏ lúc chạm ô, và gọi onCompleted hễ ô đủ 6 số → gửi lại mã sai, tốn hạn mức token_verifications
 Log: evidence/test-e2e.log (mục "request backend trong pha 2"), evidence/implement-P10-run-phase2-requests.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="189.5" customHeight="1">
+      <c r="A50" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LINKCODE-28</t>
+        </is>
+      </c>
+      <c r="B50" s="22" t="inlineStr">
+        <is>
+          <t>Toàn bộ unit test, architecture test và ruff toàn repo pass</t>
+        </is>
+      </c>
+      <c r="C50" s="22" t="inlineStr">
+        <is>
+          <t>1. pytest tests/unit tests/architecture -q
+2. ruff check .
+3. So với baseline trước khi sửa code</t>
+        </is>
+      </c>
+      <c r="D50" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E50" s="22" t="inlineStr">
+        <is>
+          <t>pytest và ruff đều pass</t>
+        </is>
+      </c>
+      <c r="F50" s="22" t="inlineStr">
+        <is>
+          <t>697 pass, 1 fail (tests/unit/test_app.py::test_doses_batch_openapi_uses_contract_shape: NameError paths); ruff toàn repo 21 lỗi ở module khác. Fail và lỗi ruff đã có trước khi task sửa code; file của task pass ruff</t>
+        </is>
+      </c>
+      <c r="G50" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H50" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I50" s="22" t="inlineStr">
+        <is>
+          <t>Có sẵn trên main, không do task 3.10: test_app.py dòng 43–44 dùng biến paths chưa định nghĩa; ruff báo lỗi ở catalog/*, consent/adapters/outbound/job_queue.py, runtime/job_runner.py (F821 health chưa import, nghi vấn làm Worker lỗi khi ghi heartbeat), worker.py, tests/unit/test_catalog_crud.py
+Log: evidence/implement-final-backend.log</t>
         </is>
       </c>
     </row>
@@ -13518,17 +15667,17 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:A5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11:F17">
+  <conditionalFormatting sqref="F11:F18">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11:G17">
+  <conditionalFormatting sqref="G11:G18">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>OR(G11="Critical",G11="High")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G42:G48">
+  <conditionalFormatting sqref="G43:G50">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
@@ -13540,10 +15689,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G11:G17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G11:G18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="G42:G48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G43:G50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
test(medication): record catalog selection results
Refs: 3.05
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Android build" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Đăng nhập người dùng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Lịch uống thuốc" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Tải lịch uống" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Tương tác thuốc-thuốc" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Tương tác thuốc-thực phẩm" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Tra cứu hoạt chất" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Report" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android build" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đăng nhập người dùng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lịch uống thuốc" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tải lịch uống" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tương tác thuốc-thuốc" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tương tác thuốc-thực phẩm" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tra cứu hoạt chất" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chọn thuốc danh mục" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hồi quy xác nhận liều" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Android build'!$A$8:$I$17</definedName>
@@ -23,6 +25,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tương tác thuốc-thuốc'!$A$8:$I$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Tương tác thuốc-thực phẩm'!$A$8:$I$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Tra cứu hoạt chất'!$A$8:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Chọn thuốc danh mục'!$A$8:$I$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Hồi quy xác nhận liều'!$A$8:$I$9</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -325,13 +329,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -355,18 +359,18 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$17</f>
+              <f>'Report'!$A$11:$A$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$11:$D$17</f>
+              <f>'Report'!$D$11:$D$19</f>
             </numRef>
           </val>
         </ser>
@@ -379,18 +383,18 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$17</f>
+              <f>'Report'!$A$11:$A$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$11:$E$17</f>
+              <f>'Report'!$E$11:$E$19</f>
             </numRef>
           </val>
         </ser>
@@ -403,18 +407,18 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$17</f>
+              <f>'Report'!$A$11:$A$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$11:$F$17</f>
+              <f>'Report'!$F$11:$F$19</f>
             </numRef>
           </val>
         </ser>
@@ -460,13 +464,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -484,7 +488,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -495,7 +499,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$3:$D$4</f>
+              <f>'Report'!$E$3:$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -512,12 +516,12 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>19</row>
+      <row>21</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -527,9 +531,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -539,7 +543,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>19</row>
+      <row>21</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3240000"/>
@@ -549,9 +553,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1689,6 +1693,1079 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>TEST REPORT</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Executed</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="C3" s="11">
+        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59+'Lịch uống thuốc'!$H$51+'Tải lịch uống'!$H$32+'Tương tác thuốc-thuốc'!$H$52+'Tương tác thuốc-thực phẩm'!$H$17+'Tra cứu hoạt chất'!$H$17</f>
+        <v/>
+      </c>
+      <c r="D3" s="11">
+        <f>'Chọn thuốc danh mục'!$H$40+'Hồi quy xác nhận liều'!$H$12</f>
+        <v/>
+      </c>
+      <c r="E3" s="15">
+        <f>SUM(C3:D3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="n"/>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="C4" s="11">
+        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60+'Lịch uống thuốc'!$H$52+'Tải lịch uống'!$H$33+'Tương tác thuốc-thuốc'!$H$53+'Tương tác thuốc-thực phẩm'!$H$18+'Tra cứu hoạt chất'!$H$18</f>
+        <v/>
+      </c>
+      <c r="D4" s="11">
+        <f>'Chọn thuốc danh mục'!$H$41+'Hồi quy xác nhận liều'!$H$13</f>
+        <v/>
+      </c>
+      <c r="E4" s="15">
+        <f>SUM(C4:D4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="n"/>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>(Total) Test executed (Passed + Failed)</t>
+        </is>
+      </c>
+      <c r="C5" s="11">
+        <f>C3+C4</f>
+        <v/>
+      </c>
+      <c r="D5" s="11">
+        <f>D3+D4</f>
+        <v/>
+      </c>
+      <c r="E5" s="15">
+        <f>SUM(C5:D5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr"/>
+      <c r="C6" s="11">
+        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61+'Lịch uống thuốc'!$H$53+'Tải lịch uống'!$H$34+'Tương tác thuốc-thuốc'!$H$54+'Tương tác thuốc-thực phẩm'!$H$19+'Tra cứu hoạt chất'!$H$19</f>
+        <v/>
+      </c>
+      <c r="D6" s="11">
+        <f>'Chọn thuốc danh mục'!$H$42+'Hồi quy xác nhận liều'!$H$14</f>
+        <v/>
+      </c>
+      <c r="E6" s="15">
+        <f>SUM(C6:D6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>(Sub-total) Test Planned</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr"/>
+      <c r="C7" s="11">
+        <f>C5+C6</f>
+        <v/>
+      </c>
+      <c r="D7" s="11">
+        <f>D5+D6</f>
+        <v/>
+      </c>
+      <c r="E7" s="15">
+        <f>SUM(C7:D7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Function</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Sheet Name</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>% TCs Executed</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>% TCs Passed</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>% TCs Failed</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Done by</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="156.5" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Build ứng dụng Android</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Build APK debug của Mobile App từ nhánh main (cấu hình Gradle, desugaring, plugin native) và bước build trong CI</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Android build</t>
+        </is>
+      </c>
+      <c r="D11" s="18">
+        <f>IFERROR(('Android build'!$H$23-'Android build'!$H$22)/'Android build'!$H$23,0)</f>
+        <v/>
+      </c>
+      <c r="E11" s="18">
+        <f>IFERROR('Android build'!$H$20/'Android build'!$H$23,0)</f>
+        <v/>
+      </c>
+      <c r="F11" s="18">
+        <f>IFERROR('Android build'!$H$21/'Android build'!$H$23,0)</f>
+        <v/>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Lỗi Critical (APK không build được do flutter_local_notifications cần desugaring và flutter_timezone 2.x dùng API Registrar đã bị gỡ) đã sửa ở task adhoc-20261007-android-desugaring (frontend PR #27, CI xanh gồm bước build APK). Còn Pending: kiểm lockfile bằng --enforce-lockfile với Flutter stable.</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="189.5" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Đăng nhập người dùng</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile App bằng OTP (số điện thoại hoặc email), hoàn thiện hồ sơ lần đầu, phiên đăng nhập và đăng xuất — user thường, không gồm admin</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Đăng nhập người dùng</t>
+        </is>
+      </c>
+      <c r="D12" s="18">
+        <f>IFERROR(('Đăng nhập người dùng'!$H$62-'Đăng nhập người dùng'!$H$61)/'Đăng nhập người dùng'!$H$62,0)</f>
+        <v/>
+      </c>
+      <c r="E12" s="18">
+        <f>IFERROR('Đăng nhập người dùng'!$H$59/'Đăng nhập người dùng'!$H$62,0)</f>
+        <v/>
+      </c>
+      <c r="F12" s="18">
+        <f>IFERROR('Đăng nhập người dùng'!$H$60/'Đăng nhập người dùng'!$H$62,0)</f>
+        <v/>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Luồng chính (đăng nhập, hồ sơ, consent, mở lại app, đăng xuất) và mọi kiểm tra quyền/bearer đạt, cả ở API lẫn E2E trên emulator. 7 Fail gồm lỗi kiểm tra đầu vào ở biên (chữ số Unicode, họ tên &gt; 255, ngày sinh &lt; 1900, ký tự NUL gây 500), lỗi múi giờ khi kiểm ngày sinh (dùng UTC), app gửi lại mã OTP sai khi chạm ô, và một kỳ vọng AC6 cần chốt lại (ký tự xuống dòng cuối số điện thoại).</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="222.5" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Quản lý lịch uống thuốc</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Backend API thêm, sửa, hủy từng giờ uống; bật/tắt nhắc; đổi ngày uống trong tuần; mốc hiệu lực khi có liều xác nhận sớm (QD-16). Chỉ chính người bệnh được ghi.</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Lịch uống thuốc</t>
+        </is>
+      </c>
+      <c r="D13" s="18">
+        <f>IFERROR(('Lịch uống thuốc'!$H$54-'Lịch uống thuốc'!$H$53)/'Lịch uống thuốc'!$H$54,0)</f>
+        <v/>
+      </c>
+      <c r="E13" s="18">
+        <f>IFERROR('Lịch uống thuốc'!$H$51/'Lịch uống thuốc'!$H$54,0)</f>
+        <v/>
+      </c>
+      <c r="F13" s="18">
+        <f>IFERROR('Lịch uống thuốc'!$H$52/'Lịch uống thuốc'!$H$54,0)</f>
+        <v/>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động và kiểm tra biên đạt trên Supabase local. Đã sửa và có test cho các lỗi review R1 (sinh trùng liều khi ngừng/dùng lại sau liều xác nhận sớm), R2 (dùng lại thuốc khi cần mở lịch cũ), R3 (dùng lại mất lịch sau khi đổi cả bộ giờ/ngày sau liều sớm; sửa bằng migration closed_by_stop_at) và M3 (doses_per_day sau khi dùng lại). Có test bất biến trên chuỗi thao tác ngẫu nhiên. Chưa phủ: race giữa xác nhận liều sớm và sửa lịch (2.10).</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="90.5" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Tải lịch uống và phân quyền dữ liệu thuốc</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>GET /patients/{patient_id}/schedules (lịch đang mở và đóng trong 30 ngày, phân trang con trỏ); phân quyền ghi lịch; QD-32 admin không đọc dữ liệu y tế; patient_id không tồn tại.</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Tải lịch uống</t>
+        </is>
+      </c>
+      <c r="D14" s="18">
+        <f>IFERROR(('Tải lịch uống'!$H$35-'Tải lịch uống'!$H$34)/'Tải lịch uống'!$H$35,0)</f>
+        <v/>
+      </c>
+      <c r="E14" s="18">
+        <f>IFERROR('Tải lịch uống'!$H$32/'Tải lịch uống'!$H$35,0)</f>
+        <v/>
+      </c>
+      <c r="F14" s="18">
+        <f>IFERROR('Tải lịch uống'!$H$33/'Tải lịch uống'!$H$35,0)</f>
+        <v/>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ ca phân quyền đạt, mỗi ca kiểm cả response lẫn access_logs. Quy tắc QD-29 (app người thân không lưu xuống máy) là quy tắc client, chưa kiểm được ở backend.</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="90.5" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Danh mục tương tác thuốc-thuốc (admin)</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Admin thêm, xem, sửa (tạo phiên bản mới), xóa mềm quy tắc tương tác giữa hai hoạt chất, kèm ngưỡng liều; xem lịch sử phiên bản (task 2.16, PB05).</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Tương tác thuốc-thuốc</t>
+        </is>
+      </c>
+      <c r="D15" s="18">
+        <f>IFERROR(('Tương tác thuốc-thuốc'!$H$55-'Tương tác thuốc-thuốc'!$H$54)/'Tương tác thuốc-thuốc'!$H$55,0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="18">
+        <f>IFERROR('Tương tác thuốc-thuốc'!$H$52/'Tương tác thuốc-thuốc'!$H$55,0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="18">
+        <f>IFERROR('Tương tác thuốc-thuốc'!$H$53/'Tương tác thuốc-thuốc'!$H$55,0)</f>
+        <v/>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động (tích hợp với Postgres thật, app chạy bằng api_role) pass. Không có lỗi sản phẩm.</t>
+        </is>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="107" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Danh mục tương tác thuốc-thực phẩm (admin)</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Admin thêm, xem, sửa (tạo phiên bản mới), xóa mềm quy tắc tương tác giữa hoạt chất và thực phẩm (task 2.16, PB05).</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Tương tác thuốc-thực phẩm</t>
+        </is>
+      </c>
+      <c r="D16" s="18">
+        <f>IFERROR(('Tương tác thuốc-thực phẩm'!$H$20-'Tương tác thuốc-thực phẩm'!$H$19)/'Tương tác thuốc-thực phẩm'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="18">
+        <f>IFERROR('Tương tác thuốc-thực phẩm'!$H$17/'Tương tác thuốc-thực phẩm'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="F16" s="18">
+        <f>IFERROR('Tương tác thuốc-thực phẩm'!$H$18/'Tương tác thuốc-thực phẩm'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động pass. Không có lỗi sản phẩm.</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90.5" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Tra cứu hoạt chất (admin)</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Admin tìm hoạt chất theo tên chuẩn hoặc tên gọi khác, hoặc xem hoạt chất của một thuốc, để chọn khi nhập quy tắc tương tác (task 2.16).</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Tra cứu hoạt chất</t>
+        </is>
+      </c>
+      <c r="D17" s="18">
+        <f>IFERROR(('Tra cứu hoạt chất'!$H$20-'Tra cứu hoạt chất'!$H$19)/'Tra cứu hoạt chất'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="E17" s="18">
+        <f>IFERROR('Tra cứu hoạt chất'!$H$17/'Tra cứu hoạt chất'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="F17" s="18">
+        <f>IFERROR('Tra cứu hoạt chất'!$H$18/'Tra cứu hoạt chất'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động pass.</t>
+        </is>
+      </c>
+      <c r="I17" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="123.5" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Tìm và chọn thuốc khi nhập thuốc</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Sheet tìm/chọn danh mục trong form thêm thuốc, không gồm tra cứu độc lập.</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Chọn thuốc danh mục</t>
+        </is>
+      </c>
+      <c r="D18" s="18">
+        <f>IFERROR(('Chọn thuốc danh mục'!$H$43-'Chọn thuốc danh mục'!$H$42)/'Chọn thuốc danh mục'!$H$43,0)</f>
+        <v/>
+      </c>
+      <c r="E18" s="18">
+        <f>IFERROR('Chọn thuốc danh mục'!$H$40/'Chọn thuốc danh mục'!$H$43,0)</f>
+        <v/>
+      </c>
+      <c r="F18" s="18">
+        <f>IFERROR('Chọn thuốc danh mục'!$H$41/'Chọn thuốc danh mục'!$H$43,0)</f>
+        <v/>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>29 Pass, 0 Fail, 0 Pending cho phạm vi tìm/chọn thuốc. Ba case cuối được chạy 2026-10-13 bằng harness biên và Flutter drive Android nối API/DB local thật; không bao gồm login. Kết quả toàn suite/backend Auth và REGDOSE báo riêng trong 05.</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="90.5" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Hồi quy xác nhận liều</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Sai khác test–API phát hiện khi chạy bộ tích hợp rộng của task 3.05; ngoài chức năng tìm/chọn thuốc.</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Hồi quy xác nhận liều</t>
+        </is>
+      </c>
+      <c r="D19" s="18">
+        <f>IFERROR(('Hồi quy xác nhận liều'!$H$15-'Hồi quy xác nhận liều'!$H$14)/'Hồi quy xác nhận liều'!$H$15,0)</f>
+        <v/>
+      </c>
+      <c r="E19" s="18">
+        <f>IFERROR('Hồi quy xác nhận liều'!$H$12/'Hồi quy xác nhận liều'!$H$15,0)</f>
+        <v/>
+      </c>
+      <c r="F19" s="18">
+        <f>IFERROR('Hồi quy xác nhận liều'!$H$13/'Hồi quy xác nhận liều'!$H$15,0)</f>
+        <v/>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>Một test Fail lặp lại; chưa kết luận sản phẩm sai hay kỳ vọng test đã cũ. Không sửa backend trong task 3.05.</t>
+        </is>
+      </c>
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>Bug Report</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>Bug ID</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C43" s="20" t="inlineStr">
+        <is>
+          <t>Steps to Reproduce</t>
+        </is>
+      </c>
+      <c r="D43" s="20" t="inlineStr">
+        <is>
+          <t>Input Data</t>
+        </is>
+      </c>
+      <c r="E43" s="20" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="F43" s="20" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="G43" s="20" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="H43" s="20" t="inlineStr">
+        <is>
+          <t>Name of Tester</t>
+        </is>
+      </c>
+      <c r="I43" s="20" t="inlineStr">
+        <is>
+          <t>Logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="123.5" customHeight="1">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-08</t>
+        </is>
+      </c>
+      <c r="B44" s="22" t="inlineStr">
+        <is>
+          <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
+        </is>
+      </c>
+      <c r="C44" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
+2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
+        </is>
+      </c>
+      <c r="D44" s="22" t="inlineStr">
+        <is>
+          <t>phone: 0900000001 + ký tự \n</t>
+        </is>
+      </c>
+      <c r="E44" s="22" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
+        </is>
+      </c>
+      <c r="F44" s="22" t="inlineStr">
+        <is>
+          <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
+        </is>
+      </c>
+      <c r="G44" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H44" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I44" s="22" t="inlineStr">
+        <is>
+          <t>Nghi vấn — kỳ vọng AC6 mâu thuẫn AC5: backend `_validate_required_text` (sign_in.py:178) `strip()` mọi ký tự trắng hai đầu, nên \n cuối được xử lý như khoảng trắng hai đầu mà AC5 coi là hợp lệ. Cần người dùng chốt: sửa AC6 hoặc sửa backend
+Log: evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="123.5" customHeight="1">
+      <c r="A45" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-11</t>
+        </is>
+      </c>
+      <c r="B45" s="22" t="inlineStr">
+        <is>
+          <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
+        </is>
+      </c>
+      <c r="C45" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/otp {phone}
+2. POST /auth/mobile/verify {phone, token: 123456}</t>
+        </is>
+      </c>
+      <c r="D45" s="22" t="inlineStr">
+        <is>
+          <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
+        </is>
+      </c>
+      <c r="E45" s="22" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
+        </is>
+      </c>
+      <c r="F45" s="22" t="inlineStr">
+        <is>
+          <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
+        </is>
+      </c>
+      <c r="G45" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H45" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I45" s="22" t="inlineStr">
+        <is>
+          <t>`_normalize_phone` (sign_in.py:197–206) kiểm bằng `str.isdigit()`, nhận cả chữ số Unicode, nên số lọt qua kiểm tra và gửi tới Supabase. Ô nhập của app chỉ cho 0-9 nên người dùng app không gặp; lỗi ở tầng API
+Log: evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="189.5" customHeight="1">
+      <c r="A46" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-25</t>
+        </is>
+      </c>
+      <c r="B46" s="22" t="inlineStr">
+        <is>
+          <t>Lưu họ tên có ký tự NUL</t>
+        </is>
+      </c>
+      <c r="C46" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
+        </is>
+      </c>
+      <c r="D46" s="22" t="inlineStr">
+        <is>
+          <t>ho_ten: abc\u0000def</t>
+        </is>
+      </c>
+      <c r="E46" s="22" t="inlineStr">
+        <is>
+          <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
+        </is>
+      </c>
+      <c r="F46" s="22" t="inlineStr">
+        <is>
+          <t>500 Internal Server Error</t>
+        </is>
+      </c>
+      <c r="G46" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H46" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I46" s="22" t="inlineStr">
+        <is>
+          <t>`_validate_required_text` (sign_in.py:178) không chặn ký tự điều khiển; PostgreSQL từ chối NUL trong cột text: `psycopg.DataError: PostgreSQL text fields cannot contain NUL (0x00) bytes` ở `UPDATE users SET full_name…` (SqlUsers.update_profile); không có handler cho DataError nên thành 500. Câu SQL có tham số nên không phải lỗ hổng SQL injection
+Log: evidence/test-integration.log, evidence/test-probe-nul.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="90.5" customHeight="1">
+      <c r="A47" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-30</t>
+        </is>
+      </c>
+      <c r="B47" s="22" t="inlineStr">
+        <is>
+          <t>Lưu họ tên dài 256 ký tự</t>
+        </is>
+      </c>
+      <c r="C47" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ho_ten: A*256}</t>
+        </is>
+      </c>
+      <c r="D47" s="22" t="inlineStr">
+        <is>
+          <t>A*256</t>
+        </is>
+      </c>
+      <c r="E47" s="22" t="inlineStr">
+        <is>
+          <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
+        </is>
+      </c>
+      <c r="F47" s="22" t="inlineStr">
+        <is>
+          <t>204, đã lưu</t>
+        </is>
+      </c>
+      <c r="G47" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H47" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I47" s="22" t="inlineStr">
+        <is>
+          <t>Không có giới hạn độ dài họ tên: `_validate_profile` (sign_in.py) chỉ kiểm rỗng; cột users.full_name kiểu text không giới hạn
+Log: evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="90.5" customHeight="1">
+      <c r="A48" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-32</t>
+        </is>
+      </c>
+      <c r="B48" s="22" t="inlineStr">
+        <is>
+          <t>Lưu ngày sinh trước 1900-01-01</t>
+        </is>
+      </c>
+      <c r="C48" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ngay_sinh}</t>
+        </is>
+      </c>
+      <c r="D48" s="22" t="inlineStr">
+        <is>
+          <t>1899-12-31 | 0001-01-01</t>
+        </is>
+      </c>
+      <c r="E48" s="22" t="inlineStr">
+        <is>
+          <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
+        </is>
+      </c>
+      <c r="F48" s="22" t="inlineStr">
+        <is>
+          <t>204 ở cả hai giá trị, đã lưu</t>
+        </is>
+      </c>
+      <c r="G48" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H48" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I48" s="22" t="inlineStr">
+        <is>
+          <t>`_validate_birth_date` (sign_in.py:229–231) chỉ chặn ngày tương lai, không có cận dưới. App mobile đã giới hạn date picker từ 1900 nên chỉ gặp khi gọi API trực tiếp
+Log: evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="123.5" customHeight="1">
+      <c r="A49" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-35</t>
+        </is>
+      </c>
+      <c r="B49" s="22" t="inlineStr">
+        <is>
+          <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
+        </is>
+      </c>
+      <c r="C49" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
+        </is>
+      </c>
+      <c r="D49" s="22" t="inlineStr">
+        <is>
+          <t>ngay_sinh: 2026-10-08</t>
+        </is>
+      </c>
+      <c r="E49" s="22" t="inlineStr">
+        <is>
+          <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
+        </is>
+      </c>
+      <c r="F49" s="22" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_date_of_birth"}</t>
+        </is>
+      </c>
+      <c r="G49" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H49" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I49" s="22" t="inlineStr">
+        <is>
+          <t>`_validate_birth_date` (sign_in.py:230) so với `now.date()` trong khi `now()` (shared/clock.py) trả giờ UTC: từ 00:00 đến 07:00 giờ VN, "hôm nay" bị coi là ngày mai. Vi phạm bất biến 7 (múi giờ cố định Asia/Ho_Chi_Minh)
+Log: evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="173" customHeight="1">
+      <c r="A50" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-42</t>
+        </is>
+      </c>
+      <c r="B50" s="22" t="inlineStr">
+        <is>
+          <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
+        </is>
+      </c>
+      <c r="C50" s="22" t="inlineStr">
+        <is>
+          <t>1. Chạm vào ô mã OTP
+2. Theo dõi request backend nhận được</t>
+        </is>
+      </c>
+      <c r="D50" s="22" t="inlineStr">
+        <is>
+          <t>Ô đang chứa 000000</t>
+        </is>
+      </c>
+      <c r="E50" s="22" t="inlineStr">
+        <is>
+          <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
+        </is>
+      </c>
+      <c r="F50" s="22" t="inlineStr">
+        <is>
+          <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
+        </is>
+      </c>
+      <c r="G50" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H50" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I50" s="22" t="inlineStr">
+        <is>
+          <t>`OtpPinInput._handleTextChange` (frontend/mobile/lib/features/auth/presentation/widgets/otp_pin_input.dart:66–72) chạy với mọi thông báo của controller, kể cả khi chỉ đổi vị trí con trỏ lúc chạm ô, và gọi onCompleted hễ ô đủ 6 số → gửi lại mã sai, tốn hạn mức token_verifications
+Log: evidence/test-e2e.log (mục "request backend trong pha 2"), evidence/implement-P10-run-phase2-requests.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="239" customHeight="1">
+      <c r="A51" s="22" t="inlineStr">
+        <is>
+          <t>BUG-REGDOSE-01</t>
+        </is>
+      </c>
+      <c r="B51" s="22" t="inlineStr">
+        <is>
+          <t>Đối chiếu scheduled_at có giây khi xác nhận liều</t>
+        </is>
+      </c>
+      <c r="C51" s="22" t="inlineStr">
+        <is>
+          <t>1. Từ backend chạy .venv/Scripts/python.exe -m pytest tests/integration/test_dose_confirmation_api.py::test_post_doses_batch_creates_dose_log_for_authenticated_patient__AC1_AC10_AC18 -q -ra.
+2. Fixture POST /doses/batch với danh sách một item ở Test Data.
+3. Đối chiếu items[0].scheduled_at với kỳ vọng test hiện có.</t>
+        </is>
+      </c>
+      <c r="D51" s="22" t="inlineStr">
+        <is>
+          <t>client_uuid: UUID mới; schedule_id: fixture; scheduled_at=2026-10-02T01:00:59.999Z; taken_at=2026-10-02T01:05:59.999Z</t>
+        </is>
+      </c>
+      <c r="E51" s="22" t="inlineStr">
+        <is>
+          <t>Theo test hiện có: HTTP 200, synced, da_uong và scheduled_at=2026-10-02T01:00:00Z.</t>
+        </is>
+      </c>
+      <c r="F51" s="22" t="inlineStr">
+        <is>
+          <t>HTTP 200, synced, da_uong; scheduled_at=2026-10-02T01:00:59.999000Z. Fail trong suite DB và lặp lại khi chạy riêng (1 failed trong 1.67s).</t>
+        </is>
+      </c>
+      <c r="G51" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H51" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I51" s="22" t="inlineStr">
+        <is>
+          <t>Nghi vấn kỳ vọng chuẩn hóa tới phút trong test không khớp hành vi giữ thời điểm của API; chưa xác định phía nào sai theo contract/nghiệp vụ. Chưa chứng minh mất/trùng bản ghi liều; mức Medium tạm thời cho sai khác test, phải nâng tối thiểu High nếu xác nhận mất/trùng liều.
+Log: evidence/test-integration-db.log; evidence/test-dose-mismatch-repeat.log</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:A5"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F11:F19">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G11:G19">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>OR(G11="Critical",G11="High")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G44:G51">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
+      <formula>"Critical"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2">
+      <formula>"High"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="3">
+      <formula>"Medium"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="G11:G19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Critical,High,Medium,Low"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G44:G51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Critical,High,Medium,Low"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -12648,906 +13725,2073 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:U43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
-        <is>
-          <t>TEST REPORT</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="C2" s="15" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-      <c r="D2" s="15" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Tìm và chọn thuốc khi nhập thuốc (MEDPICK)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Kết quả tìm kiếm hiện hành</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="90.5" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Mở sheet chọn thuốc từ form thêm</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạm trường Thuốc.
+2. Nhập amlo; chọn Amlodipin 5mg.
+3. Quan sát form và số lần gọi add.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Thuốc: chưa chọn</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Sheet mở; thuốc trở về form, không mở tra cứu/chi tiết và chưa tự lưu.</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test 3.05: hủy/chọn lại giữ dữ liệu sử dụng, chưa tự lưu và đúng catalog id; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC1, AC5 · Chuyển trạng thái form → sheet → form · 3.05: hủy/chọn lại giữ dữ liệu sử dụng, chưa tự lưu và đúng catalog id · evidence/test-flutter.log</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>q</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>1–100 Unicode code point sau trim</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>(blank) hoặc toàn khoảng trắng
+Trên 100 Unicode code point</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>3
+4</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Kết quả</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>Có item</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>Items rỗng</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>Lỗi mạng/validation/server</t>
+        </is>
+      </c>
+      <c r="U9" s="11" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90.5" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Giữ hướng dẫn khi từ khóa rỗng</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở sheet; không nhập.
+2. Chờ trên 300ms.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>(blank), độ dài 0</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Hiện Nhập tên thuốc hoặc hoạt chất; không gọi tìm kiếm.</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test sheet danh mục: chưa gõ thì gợi ý, không tìm; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · EP (3); BVA (min-1=0) · sheet danh mục: chưa gõ thì gợi ý, không tìm · evidence/test-flutter.log</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>Có trường nullable, giữ đúng id</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr"/>
+      <c r="O10" s="10" t="inlineStr"/>
+      <c r="Q10" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S10" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T10" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U10" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90.5" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Bỏ qua từ khóa toàn khoảng trắng</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhập ba dấu cách.
+2. Chờ 400ms; kiểm tra số request.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>q="   "</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Không gọi API; không giữ kết quả cũ.</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test empty whitespace, debounce 299/300ms and trimmed final query; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · EP (3) · empty whitespace, debounce 299/300ms and trimmed final query · evidence/test-flutter.log</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr"/>
+      <c r="M11" s="10" t="inlineStr"/>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>Lỗi mạng/HTTP, không được coi là thành công</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>Hiện kết quả và cho chọn</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S11" s="11" t="inlineStr"/>
+      <c r="T11" s="11" t="inlineStr"/>
+      <c r="U11" s="11" t="inlineStr"/>
+    </row>
+    <row r="12" ht="90.5" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Trim từ khóa một ký tự và chờ debounce</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhập A có khoảng trắng hai đầu.
+2. Chờ 299ms rồi đổi sang B có khoảng trắng.
+3. Chờ 299ms rồi thêm 1ms.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>q=" A ", sau đó " B "; 299ms + 1ms</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Không gọi trước 300ms; chỉ gửi B đã trim.</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test empty whitespace, debounce 299/300ms and trimmed final query; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · EP (1); BVA (min=1) · empty whitespace, debounce 299/300ms and trimmed final query · evidence/test-flutter.log</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
+        <is>
+          <t>Hiện không tìm thấy</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="inlineStr"/>
+      <c r="S12" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T12" s="11" t="inlineStr"/>
+      <c r="U12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13" ht="90.5" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Giữ thứ tự kết quả server</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Tìm B.
+2. Server trả second trước first.
+3. Quan sát thứ tự trên sheet.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>items: second, first</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>second nằm trước first; client không tự sắp xếp.</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test empty whitespace, debounce 299/300ms and trimmed final query; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · EP (1) · empty whitespace, debounce 299/300ms and trimmed final query · evidence/test-flutter.log</t>
+        </is>
+      </c>
+      <c r="Q13" s="10" t="inlineStr">
+        <is>
+          <t>Hiện lỗi, cho retry</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="inlineStr"/>
+      <c r="S13" s="11" t="inlineStr"/>
+      <c r="T13" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="90.5" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Xóa từ khóa và bỏ response còn chờ</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. Tìm A.
+2. Xóa từ khóa trước khi response về.
+3. Cho response A về.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>q=A → (blank); response A về sau</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Kết quả A không xuất hiện; trở về hướng dẫn.</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test clear invalidates request and dispose cancels timer or ignores response; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC2, AC9 · Chuyển trạng thái loading → initial · clear invalidates request and dispose cancels timer or ignores response · evidence/test-flutter.log</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>Xử lý phiên chung, không retry tìm</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr"/>
+      <c r="S14" s="11" t="inlineStr"/>
+      <c r="T14" s="11" t="inlineStr"/>
+      <c r="U14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="90.5" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Chỉ nhận response mới nhất trong A → B → A</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. Tìm A, B, A theo thứ tự.
+2. Trả latest cho A2 rồi stale cho A1 và lỗi mạng cho B.
+3. Quan sát kết quả và lỗi.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Request A1, B, A2; response A2, A1, lỗi B</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ latest hiển thị, không xuất hiện stale hoặc Chưa tìm được.</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test A B A: only current generation can update, including stale error; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · Đoán lỗi response sai thứ tự · A B A: only current generation can update, including stale error · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="90.5" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Đóng sheet khi còn timer và request</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. Tìm A rồi xóa.
+2. Tìm B rồi nhập C chưa đủ debounce.
+3. Đóng sheet; trả lỗi B.</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>A đang chờ; B gửi; C đang debounce</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Timer C không gửi; không exception cập nhật widget đã dispose.</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test clear invalidates request and dispose cancels timer or ignores response; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · Chuyển trạng thái sheet → disposed · clear invalidates request and dispose cancels timer or ignores response · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90.5" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Chấp nhận 99 ký tự sau trim</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhập chuỗi a dài 99 ký tự.
+2. Chờ 300ms; kiểm tra request.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>q=a*99</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Gửi q 99 ký tự; không báo quá dài.</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Harness biên 99 ký tự: 1 test pass; không request ở 299ms, gửi đúng a*99 tại 300ms sau trim. Android cũng gửi query này tới API thật. evidence/test-boundary-99.log; evidence/test-device-AC14-scroll.log.</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · EP (1) · BVA (max-1=99) · scratch/catalog_boundary_test.dart; Flutter drive Android · evidence/test-boundary-99.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90.5" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Chấp nhận 100 ký tự tiếng Việt sau trim</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhập 100 ký tự á có khoảng trắng hai đầu.
+2. Chờ 300ms; kiểm tra request.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>q=" "+á*100+" "</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Gửi đúng 100 ký tự á sau trim.</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test trimmed Unicode limit 100 allowed, 101 blocked: á; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · EP (1); BVA (max=100) · trimmed Unicode limit 100 allowed, 101 blocked: á · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="90.5" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Chặn 101 ký tự tiếng Việt và khôi phục query hợp lệ</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi query 100 ký tự rồi nhập 101 ký tự.
+2. Trả response cũ.
+3. Đổi sang valid và trả items rỗng.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>á*100 → á*101 → valid</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Không gửi query 101; bỏ response cũ; hiện Nhập tối đa 100 ký tự sau khi bỏ khoảng trắng đầu và cuối.; query valid tìm lại được.</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test trimmed Unicode limit 100 allowed, 101 blocked: á; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC9, AC10 · EP (4); BVA (max+1=101) · trimmed Unicode limit 100 allowed, 101 blocked: á · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="90.5" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Đếm Unicode ngoài BMP theo code point</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhập 100 emoji rồi 101 emoji.
+2. Quan sát số lần gọi tìm kiếm và thông báo.</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>😀*100, 😀*101</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>100 code point được gửi, 101 bị chặn, không đếm thành 200 UTF-16 unit.</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test trimmed Unicode limit 100 allowed, 101 blocked: 😀; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · EP (1,4); BVA (max=100,max+1=101) · trimmed Unicode limit 100 allowed, 101 blocked: 😀 · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="90.5" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-13</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Hiện không tìm thấy khi API trả items rỗng</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. Tìm valid.
+2. Server trả danh sách rỗng.
+3. Quan sát sheet.</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>q=valid; items=[]</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Hiện Không tìm thấy thuốc phù hợp và gợi ý đổi từ khóa; không tự tạo thuốc.</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test network retry uses current query once and clears old error; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · Decision Table (R2) · network retry uses current query once and clears old error · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="90.5" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-14</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Thử lại lỗi mạng đúng query hiện tại</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhập A; mô phỏng mất mạng.
+2. Bấm Thử lại liên tục hai lần.
+3. Cho lần retry trả latest.</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>q=" A "; lần đầu lỗi mạng, lần sau latest</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Hiện Chưa tìm được; chỉ một retry với A đã trim; lỗi được xóa khi tải.</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test network retry uses current query once and clears old error; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (5); Decision Table (R3) · network retry uses current query once and clears old error · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="90.5" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Phân biệt lỗi HTTP 422 với kết quả rỗng</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhập A.
+2. Trả lỗi validation 422.
+3. Quan sát lỗi và khả năng retry.</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>GET /catalog/medications; HTTP 422</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Hiện Chưa tìm được; không hiển thị như tìm thành công không có kết quả.</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test failure MedicationFailureKind.validation is not empty success; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · EP (5); Decision Table (R3) · failure MedicationFailureKind.validation is not empty success · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="107" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-16</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Xử lý 401 theo cơ chế phiên chung</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. Tìm A với phiên không hợp lệ.
+2. Trả 401; kiểm callback phiên và lỗi repository.
+3. Quan sát sheet.</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 401; refresh thất bại</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Callback onUnauthorized được gọi; ném unauthorized; sheet không báo kết quả rỗng hoặc cho retry tìm kiếm.</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test 3.05 search 401 throws failure rather than empty success; failure MedicationFailureKind.unauthorized is not empty success; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · EP (5); Decision Table (R4) · 3.05 search 401 throws failure rather than empty success; failure MedicationFailureKind.unauthorized is not empty success · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="90.5" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-17</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Giữ lỗi timeout và lỗi server</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi searchCatalog với mỗi status đã nêu.
+2. Quan sát kết quả repository.</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 408, 500, 503</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Ném failure tương ứng; không chuyển thành danh sách rỗng thành công.</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test 3.05 search 408/500/503 throws failure rather than empty success; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (5); Decision Table (R3) · 3.05 search 408/500/503 throws failure rather than empty success · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="90.5" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-18</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Giữ lỗi socket khi mất kết nối</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi searchCatalog khi server không nhận kết nối.
+2. Kiểm tra lỗi trả về.</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Ngắt kết nối server cục bộ</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Ném lỗi network thay vì trả items rỗng.</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test 3.05 search socket failure is network error; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (5) · 3.05 search socket failure is network error · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="90.5" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-19</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Hiện thông tin nhận diện và không suy diễn trường thiếu</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. Tìm A và trả hai item.
+2. Quan sát tên, 5 mg và các trường thiếu.</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Hai thuốc Cùng tên: id=1 đủ thông tin, id=2 thiếu hoạt chất/hàm lượng/dạng</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Hiện hai dòng cùng tên; 5 mg chỉ ở item đủ thông tin; không hiện null; có Chưa có thông tin hoạt chất.</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test strength, missing fields and same name distinct ids keep original item; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AC5, AC6 · EP (2); Decision Table (R1) · strength, missing fields and same name distinct ids keep original item · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="90.5" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-20</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Chọn đúng item khi hai thuốc cùng tên</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. Tìm Cùng.
+2. Chọn dòng thứ hai.
+3. Quan sát form trước Lưu.</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Cùng tên: id=1, id=200; chọn item thứ hai nullable</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Form nhận nguyên item id=200; hàm lượng trống, không tự điền y khoa, không tự lưu.</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test 3.05: chọn đúng item cùng tên, thiếu thông tin giữ trường trống không tự lưu; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AC5, AC6 · EP (2) · 3.05: chọn đúng item cùng tên, thiếu thông tin giữ trường trống không tự lưu · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="90.5" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-21</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Giữ thông tin sử dụng khi hủy rồi chọn lại</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. Chọn Amlodipin; tăng liều thành 2 và chọn 3 lần/ngày.
+2. Mở sheet rồi hủy; mở lại và chọn Losartan.
+3. Kiểm dữ liệu còn giữ, sau đó Lưu để kiểm payload.</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Amlodipin 5mg → Losartan 50mg; liều 2; 3 lần/ngày</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Hủy giữ thuốc cũ; chọn lại đổi catalog id; giữ liều/tần suất/giờ mặc định đã chọn; chưa add trước Lưu.</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test 3.05: hủy/chọn lại giữ dữ liệu sử dụng, chưa tự lưu và đúng catalog id; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>AC12, AC5 · Chuyển trạng thái chọn → hủy → chọn lại · 3.05: hủy/chọn lại giữ dữ liệu sử dụng, chưa tự lưu và đúng catalog id · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="90.5" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-22</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Cho phép chọn thuốc đang dùng và giữ cảnh báo</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>1. Tìm losartan.
+2. Quan sát nhãn Đang dùng và chọn.
+3. Quan sát form.</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Losartan 50mg đã có trong danh sách</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Giữ nhãn Đang dùng và cảnh báo đã có trong danh sách đang dùng; vẫn chọn được.</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test 3.05: hủy/chọn lại giữ dữ liệu sử dụng, chưa tự lưu và đúng catalog id; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>AC13 · Decision Table (R1) · 3.05: hủy/chọn lại giữ dữ liệu sử dụng, chưa tự lưu và đúng catalog id · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="90.5" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-23</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Gọi đúng GET và giữ id/nullable/thứ tự</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi RemoteMedicationRepository.searchCatalog.
+2. Kiểm method/path/q và item mapper.</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>q có khoảng trắng; hai item khác id, trường nullable</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>GET /catalog/medications với q trim; giữ thứ tự và id; nullable không tạo dữ liệu giả.</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test 3.05 search GET trim, server order, nullable and exact ids; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>AC3, AC5, AC6 · EP (1,2) · 3.05 search GET trim, server order, nullable and exact ids · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="90.5" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-24</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Cuộn trạng thái ở màn nhỏ có bàn phím</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở sheet ở cấu hình đã nêu.
+2. Cho lỗi mạng, cuộn tới Thử lại và bấm.
+3. Trả rỗng rồi kết quả; cuộn tới kết quả.</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Widget 320×640; scale 1.5; keyboard inset 250</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Không exception layout; retry chạm được và kết quả cuộn được. Chỉ là kiểm tra widget hỗ trợ AC14.</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Đạt các assertion trong test small screen large text with keyboard: states scroll and retry remains reachable; toàn bộ 354 test pass tại evidence/test-flutter.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>AC14 · Đoán lỗi layout · small screen large text with keyboard: states scroll and retry remains reachable · evidence/test-flutter.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="90.5" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-25</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Tìm tên/hoạt chất có dấu, không dấu và khác hoa thường trên DB thật</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>1. Reset Supabase local, không dùng DB deploy.
+2. Chạy pytest tests/integration/test_catalog_search.py -q -ra.
+3. Kiểm test_unaccented_and_case_insensitive__AC5c và response.</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Thuốc ho Bảo Thanh &lt;tag&gt;; Đồng sulfat &lt;tag&gt;; các query thuoc ho bao thanh, THUỐC HO BẢO THANH, dong sulfat, ĐỒNG SULFAT</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 200; cùng thuốc phù hợp cho các biến thể dấu và hoa thường.</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Bộ tests/integration/test_catalog_search.py đạt 14 pass, 0 fail, 0 skip trong 8.28s sau reset Supabase PostgreSQL local; evidence/test-catalog-after-reset.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (1); tích hợp DB thật · pytest tests/integration/test_catalog_search.py · evidence/test-catalog-after-reset.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="90.5" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-26</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Loại thuốc đã gỡ và kiểm limit/thứ tự ở API thật</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>1. Chuẩn bị fixture trong test_catalog_search.py.
+2. Chạy test_matches_name_and_ingredient_excludes_deleted_respects_limit__AC5 và test_prefix_first_then_name_order__AC5.</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Metformin &lt;tag&gt;, Glucophage &lt;tag&gt;; một thuốc deleted_at khác null; limit=1</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ thuốc chưa gỡ, đúng schema; limit 1; tiền tố tên được ưu tiên, sau đó thứ tự tên.</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Bộ tests/integration/test_catalog_search.py đạt 14 pass, 0 fail, 0 skip trong 8.28s sau reset Supabase PostgreSQL local; evidence/test-catalog-after-reset.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (1); tích hợp DB thật · pytest tests/integration/test_catalog_search.py · evidence/test-catalog-after-reset.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="123.5" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-27</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Chọn thuốc từ Mobile nối Backend API thật</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy app với DRUGTIME_API_BASE_URL trỏ Backend local; đăng nhập tài khoản test.
+2. Mở Thêm thuốc → Thuốc; tìm tên/hoạt chất có dấu, không dấu, hoa thường.
+3. Chọn item; đối chiếu id trong phản hồi API và form; không bấm Lưu.</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Danh mục local có tên/hoạt chất có dấu và một thuốc đã gỡ; tài khoản test</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>Chọn đúng item/id; không thấy thuốc gỡ; tìm/chọn chưa tạo thuốc cá nhân.</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>LM G710 Android 13, cấu hình màn hình/font mặc định: 5 query tên/hoạt chất có dấu/không dấu/hoa thường; đều chọn id=179, không thấy id thuốc gỡ; sheet đóng sau mỗi chọn. meds/schedules/prescriptions đều 0 trước và sau. Flutter drive exit 0. evidence/test-device-AC4.log.</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>AC4, AC5 · Flutter drive thiết bị thật + Backend API thật + PostgreSQL local; session từ fixture, không test login · evidence/test-device-AC4.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="189.5" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-28</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Đọc và chọn thuốc trên thiết bị với cỡ chữ lớn và bàn phím</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở form và sheet; bật cỡ chữ lớn trong cấu hình thiết bị.
+2. Kiểm hướng dẫn, loading, không kết quả, lỗi và retry.
+3. Tìm thuốc, cuộn và chọn kết quả; kiểm form.
+4. Khôi phục cỡ chữ ban đầu sau test.</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Điện thoại LM G710 Android 13; cỡ chữ lớn; bàn phím mở</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>Nội dung đọc/cuộn được; bàn phím không che thao tác; chọn trả đúng thuốc về form.</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>Android thật, viewport 360×616 dp, font system 1.5×, bàn phím thực tế inset 325.5 dp: kiểm initial/error 503/retry/empty/results; cuộn 120 dp tới metadata, chạm tile trong vùng thấy 44.3 dp và trả đúng id; chưa tạo thuốc. Đã đọc ảnh kết quả/metadata. Flutter drive exit 0, không exception ở lượt cuối. evidence/test-device-AC14-scroll.log; evidence/android-small-results.png; evidence/android-small-scrolled-metadata.png.</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>AC14 · Flutter drive trên thiết bị thật + agent kiểm ảnh; thay thao tác tay bằng cùng luồng tự động, không giả lập viewInsets · evidence/test-device-AC14-scroll.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="90.5" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>TC-MEDPICK-29</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Tìm chuỗi ký tự đặc biệt nguyên văn</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile; mở Danh sách thuốc → Thêm thuốc → trường Thuốc. Dữ liệu/hạ tầng theo Test Data; test tự động dùng fixture riêng.</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy test_like_wildcards_are_literal__AC6 với DB local.
+2. Kiểm items không bị wildcard khớp tất cả.</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>q=%; q=_; tên có 100% tự nhiên, a_b, axb</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ khớp ký tự nguyên văn; không mở rộng thành mọi thuốc.</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Bộ tests/integration/test_catalog_search.py đạt 14 pass, 0 fail, 0 skip trong 8.28s sau reset Supabase PostgreSQL local; evidence/test-catalog-after-reset.log (2026-10-13).</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · Đoán lỗi SQL wildcard; tích hợp DB thật · pytest tests/integration/test_catalog_search.py · evidence/test-catalog-after-reset.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40">
+      <c r="G40" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H40" s="13">
+        <f>COUNTIF(H9:H37,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="G41" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H41" s="13">
+        <f>COUNTIF(H9:H37,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="G42" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H42" s="13">
+        <f>COUNTIF(H9:H37,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="G43" s="12" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>Executed</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="C3" s="11">
-        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59+'Lịch uống thuốc'!$H$51+'Tải lịch uống'!$H$32+'Tương tác thuốc-thuốc'!$H$52+'Tương tác thuốc-thực phẩm'!$H$17+'Tra cứu hoạt chất'!$H$17</f>
+      <c r="H43" s="13">
+        <f>SUM(H40:H42)</f>
         <v/>
       </c>
-      <c r="D3" s="15">
-        <f>SUM(C3:C3)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="16" t="n"/>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="C4" s="11">
-        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60+'Lịch uống thuốc'!$H$52+'Tải lịch uống'!$H$33+'Tương tác thuốc-thuốc'!$H$53+'Tương tác thuốc-thực phẩm'!$H$18+'Tra cứu hoạt chất'!$H$18</f>
-        <v/>
-      </c>
-      <c r="D4" s="15">
-        <f>SUM(C4:C4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="17" t="n"/>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>(Total) Test executed (Passed + Failed)</t>
-        </is>
-      </c>
-      <c r="C5" s="11">
-        <f>C3+C4</f>
-        <v/>
-      </c>
-      <c r="D5" s="15">
-        <f>SUM(C5:C5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr"/>
-      <c r="C6" s="11">
-        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61+'Lịch uống thuốc'!$H$53+'Tải lịch uống'!$H$34+'Tương tác thuốc-thuốc'!$H$54+'Tương tác thuốc-thực phẩm'!$H$19+'Tra cứu hoạt chất'!$H$19</f>
-        <v/>
-      </c>
-      <c r="D6" s="15">
-        <f>SUM(C6:C6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>(Sub-total) Test Planned</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="11">
-        <f>C5+C6</f>
-        <v/>
-      </c>
-      <c r="D7" s="15">
-        <f>SUM(C7:C7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Function</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Sheet Name</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>% TCs Executed</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>% TCs Passed</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>% TCs Failed</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>Done by</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="156.5" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>Build ứng dụng Android</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Build APK debug của Mobile App từ nhánh main (cấu hình Gradle, desugaring, plugin native) và bước build trong CI</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>Android build</t>
-        </is>
-      </c>
-      <c r="D11" s="18">
-        <f>IFERROR(('Android build'!$H$23-'Android build'!$H$22)/'Android build'!$H$23,0)</f>
-        <v/>
-      </c>
-      <c r="E11" s="18">
-        <f>IFERROR('Android build'!$H$20/'Android build'!$H$23,0)</f>
-        <v/>
-      </c>
-      <c r="F11" s="18">
-        <f>IFERROR('Android build'!$H$21/'Android build'!$H$23,0)</f>
-        <v/>
-      </c>
-      <c r="G11" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>Lỗi Critical (APK không build được do flutter_local_notifications cần desugaring và flutter_timezone 2.x dùng API Registrar đã bị gỡ) đã sửa ở task adhoc-20261007-android-desugaring (frontend PR #27, CI xanh gồm bước build APK). Còn Pending: kiểm lockfile bằng --enforce-lockfile với Flutter stable.</t>
-        </is>
-      </c>
-      <c r="I11" s="11" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="189.5" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>Đăng nhập người dùng</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Đăng nhập Mobile App bằng OTP (số điện thoại hoặc email), hoàn thiện hồ sơ lần đầu, phiên đăng nhập và đăng xuất — user thường, không gồm admin</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
-        <is>
-          <t>Đăng nhập người dùng</t>
-        </is>
-      </c>
-      <c r="D12" s="18">
-        <f>IFERROR(('Đăng nhập người dùng'!$H$62-'Đăng nhập người dùng'!$H$61)/'Đăng nhập người dùng'!$H$62,0)</f>
-        <v/>
-      </c>
-      <c r="E12" s="18">
-        <f>IFERROR('Đăng nhập người dùng'!$H$59/'Đăng nhập người dùng'!$H$62,0)</f>
-        <v/>
-      </c>
-      <c r="F12" s="18">
-        <f>IFERROR('Đăng nhập người dùng'!$H$60/'Đăng nhập người dùng'!$H$62,0)</f>
-        <v/>
-      </c>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
-        <is>
-          <t>Luồng chính (đăng nhập, hồ sơ, consent, mở lại app, đăng xuất) và mọi kiểm tra quyền/bearer đạt, cả ở API lẫn E2E trên emulator. 7 Fail gồm lỗi kiểm tra đầu vào ở biên (chữ số Unicode, họ tên &gt; 255, ngày sinh &lt; 1900, ký tự NUL gây 500), lỗi múi giờ khi kiểm ngày sinh (dùng UTC), app gửi lại mã OTP sai khi chạm ô, và một kỳ vọng AC6 cần chốt lại (ký tự xuống dòng cuối số điện thoại).</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="222.5" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>Quản lý lịch uống thuốc</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Backend API thêm, sửa, hủy từng giờ uống; bật/tắt nhắc; đổi ngày uống trong tuần; mốc hiệu lực khi có liều xác nhận sớm (QD-16). Chỉ chính người bệnh được ghi.</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>Lịch uống thuốc</t>
-        </is>
-      </c>
-      <c r="D13" s="18">
-        <f>IFERROR(('Lịch uống thuốc'!$H$54-'Lịch uống thuốc'!$H$53)/'Lịch uống thuốc'!$H$54,0)</f>
-        <v/>
-      </c>
-      <c r="E13" s="18">
-        <f>IFERROR('Lịch uống thuốc'!$H$51/'Lịch uống thuốc'!$H$54,0)</f>
-        <v/>
-      </c>
-      <c r="F13" s="18">
-        <f>IFERROR('Lịch uống thuốc'!$H$52/'Lịch uống thuốc'!$H$54,0)</f>
-        <v/>
-      </c>
-      <c r="G13" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H13" s="10" t="inlineStr">
-        <is>
-          <t>Toàn bộ test tự động và kiểm tra biên đạt trên Supabase local. Đã sửa và có test cho các lỗi review R1 (sinh trùng liều khi ngừng/dùng lại sau liều xác nhận sớm), R2 (dùng lại thuốc khi cần mở lịch cũ), R3 (dùng lại mất lịch sau khi đổi cả bộ giờ/ngày sau liều sớm; sửa bằng migration closed_by_stop_at) và M3 (doses_per_day sau khi dùng lại). Có test bất biến trên chuỗi thao tác ngẫu nhiên. Chưa phủ: race giữa xác nhận liều sớm và sửa lịch (2.10).</t>
-        </is>
-      </c>
-      <c r="I13" s="11" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="90.5" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>Tải lịch uống và phân quyền dữ liệu thuốc</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>GET /patients/{patient_id}/schedules (lịch đang mở và đóng trong 30 ngày, phân trang con trỏ); phân quyền ghi lịch; QD-32 admin không đọc dữ liệu y tế; patient_id không tồn tại.</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>Tải lịch uống</t>
-        </is>
-      </c>
-      <c r="D14" s="18">
-        <f>IFERROR(('Tải lịch uống'!$H$35-'Tải lịch uống'!$H$34)/'Tải lịch uống'!$H$35,0)</f>
-        <v/>
-      </c>
-      <c r="E14" s="18">
-        <f>IFERROR('Tải lịch uống'!$H$32/'Tải lịch uống'!$H$35,0)</f>
-        <v/>
-      </c>
-      <c r="F14" s="18">
-        <f>IFERROR('Tải lịch uống'!$H$33/'Tải lịch uống'!$H$35,0)</f>
-        <v/>
-      </c>
-      <c r="G14" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
-        <is>
-          <t>Toàn bộ ca phân quyền đạt, mỗi ca kiểm cả response lẫn access_logs. Quy tắc QD-29 (app người thân không lưu xuống máy) là quy tắc client, chưa kiểm được ở backend.</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="90.5" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>Danh mục tương tác thuốc-thuốc (admin)</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Admin thêm, xem, sửa (tạo phiên bản mới), xóa mềm quy tắc tương tác giữa hai hoạt chất, kèm ngưỡng liều; xem lịch sử phiên bản (task 2.16, PB05).</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>Tương tác thuốc-thuốc</t>
-        </is>
-      </c>
-      <c r="D15" s="18">
-        <f>IFERROR(('Tương tác thuốc-thuốc'!$H$55-'Tương tác thuốc-thuốc'!$H$54)/'Tương tác thuốc-thuốc'!$H$55,0)</f>
-        <v/>
-      </c>
-      <c r="E15" s="18">
-        <f>IFERROR('Tương tác thuốc-thuốc'!$H$52/'Tương tác thuốc-thuốc'!$H$55,0)</f>
-        <v/>
-      </c>
-      <c r="F15" s="18">
-        <f>IFERROR('Tương tác thuốc-thuốc'!$H$53/'Tương tác thuốc-thuốc'!$H$55,0)</f>
-        <v/>
-      </c>
-      <c r="G15" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H15" s="10" t="inlineStr">
-        <is>
-          <t>Toàn bộ test tự động (tích hợp với Postgres thật, app chạy bằng api_role) pass. Không có lỗi sản phẩm.</t>
-        </is>
-      </c>
-      <c r="I15" s="11" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="107" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>Danh mục tương tác thuốc-thực phẩm (admin)</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>Admin thêm, xem, sửa (tạo phiên bản mới), xóa mềm quy tắc tương tác giữa hoạt chất và thực phẩm (task 2.16, PB05).</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr">
-        <is>
-          <t>Tương tác thuốc-thực phẩm</t>
-        </is>
-      </c>
-      <c r="D16" s="18">
-        <f>IFERROR(('Tương tác thuốc-thực phẩm'!$H$20-'Tương tác thuốc-thực phẩm'!$H$19)/'Tương tác thuốc-thực phẩm'!$H$20,0)</f>
-        <v/>
-      </c>
-      <c r="E16" s="18">
-        <f>IFERROR('Tương tác thuốc-thực phẩm'!$H$17/'Tương tác thuốc-thực phẩm'!$H$20,0)</f>
-        <v/>
-      </c>
-      <c r="F16" s="18">
-        <f>IFERROR('Tương tác thuốc-thực phẩm'!$H$18/'Tương tác thuốc-thực phẩm'!$H$20,0)</f>
-        <v/>
-      </c>
-      <c r="G16" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H16" s="10" t="inlineStr">
-        <is>
-          <t>Toàn bộ test tự động pass. Không có lỗi sản phẩm.</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="90.5" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>Tra cứu hoạt chất (admin)</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>Admin tìm hoạt chất theo tên chuẩn hoặc tên gọi khác, hoặc xem hoạt chất của một thuốc, để chọn khi nhập quy tắc tương tác (task 2.16).</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>Tra cứu hoạt chất</t>
-        </is>
-      </c>
-      <c r="D17" s="18">
-        <f>IFERROR(('Tra cứu hoạt chất'!$H$20-'Tra cứu hoạt chất'!$H$19)/'Tra cứu hoạt chất'!$H$20,0)</f>
-        <v/>
-      </c>
-      <c r="E17" s="18">
-        <f>IFERROR('Tra cứu hoạt chất'!$H$17/'Tra cứu hoạt chất'!$H$20,0)</f>
-        <v/>
-      </c>
-      <c r="F17" s="18">
-        <f>IFERROR('Tra cứu hoạt chất'!$H$18/'Tra cứu hoạt chất'!$H$20,0)</f>
-        <v/>
-      </c>
-      <c r="G17" s="11" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H17" s="10" t="inlineStr">
-        <is>
-          <t>Toàn bộ test tự động pass.</t>
-        </is>
-      </c>
-      <c r="I17" s="11" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="19" t="inlineStr">
-        <is>
-          <t>Bug Report</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="20" t="inlineStr">
-        <is>
-          <t>Bug ID</t>
-        </is>
-      </c>
-      <c r="B41" s="20" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C41" s="20" t="inlineStr">
-        <is>
-          <t>Steps to Reproduce</t>
-        </is>
-      </c>
-      <c r="D41" s="20" t="inlineStr">
-        <is>
-          <t>Input Data</t>
-        </is>
-      </c>
-      <c r="E41" s="20" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="F41" s="20" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="G41" s="20" t="inlineStr">
-        <is>
-          <t>Severity</t>
-        </is>
-      </c>
-      <c r="H41" s="20" t="inlineStr">
-        <is>
-          <t>Name of Tester</t>
-        </is>
-      </c>
-      <c r="I41" s="20" t="inlineStr">
-        <is>
-          <t>Logs</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="123.5" customHeight="1">
-      <c r="A42" s="22" t="inlineStr">
-        <is>
-          <t>BUG-LOGIN-08</t>
-        </is>
-      </c>
-      <c r="B42" s="22" t="inlineStr">
-        <is>
-          <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
-        </is>
-      </c>
-      <c r="C42" s="22" t="inlineStr">
-        <is>
-          <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
-2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
-        </is>
-      </c>
-      <c r="D42" s="22" t="inlineStr">
-        <is>
-          <t>phone: 0900000001 + ký tự \n</t>
-        </is>
-      </c>
-      <c r="E42" s="22" t="inlineStr">
-        <is>
-          <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
-        </is>
-      </c>
-      <c r="F42" s="22" t="inlineStr">
-        <is>
-          <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
-        </is>
-      </c>
-      <c r="G42" s="22" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H42" s="22" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-      <c r="I42" s="22" t="inlineStr">
-        <is>
-          <t>Nghi vấn — kỳ vọng AC6 mâu thuẫn AC5: backend `_validate_required_text` (sign_in.py:178) `strip()` mọi ký tự trắng hai đầu, nên \n cuối được xử lý như khoảng trắng hai đầu mà AC5 coi là hợp lệ. Cần người dùng chốt: sửa AC6 hoặc sửa backend
-Log: evidence/test-integration.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="123.5" customHeight="1">
-      <c r="A43" s="22" t="inlineStr">
-        <is>
-          <t>BUG-LOGIN-11</t>
-        </is>
-      </c>
-      <c r="B43" s="22" t="inlineStr">
-        <is>
-          <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
-        </is>
-      </c>
-      <c r="C43" s="22" t="inlineStr">
-        <is>
-          <t>1. POST /auth/mobile/otp {phone}
-2. POST /auth/mobile/verify {phone, token: 123456}</t>
-        </is>
-      </c>
-      <c r="D43" s="22" t="inlineStr">
-        <is>
-          <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
-        </is>
-      </c>
-      <c r="E43" s="22" t="inlineStr">
-        <is>
-          <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
-        </is>
-      </c>
-      <c r="F43" s="22" t="inlineStr">
-        <is>
-          <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
-        </is>
-      </c>
-      <c r="G43" s="22" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H43" s="22" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-      <c r="I43" s="22" t="inlineStr">
-        <is>
-          <t>`_normalize_phone` (sign_in.py:197–206) kiểm bằng `str.isdigit()`, nhận cả chữ số Unicode, nên số lọt qua kiểm tra và gửi tới Supabase. Ô nhập của app chỉ cho 0-9 nên người dùng app không gặp; lỗi ở tầng API
-Log: evidence/test-integration.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="189.5" customHeight="1">
-      <c r="A44" s="22" t="inlineStr">
-        <is>
-          <t>BUG-LOGIN-25</t>
-        </is>
-      </c>
-      <c r="B44" s="22" t="inlineStr">
-        <is>
-          <t>Lưu họ tên có ký tự NUL</t>
-        </is>
-      </c>
-      <c r="C44" s="22" t="inlineStr">
-        <is>
-          <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
-        </is>
-      </c>
-      <c r="D44" s="22" t="inlineStr">
-        <is>
-          <t>ho_ten: abc\u0000def</t>
-        </is>
-      </c>
-      <c r="E44" s="22" t="inlineStr">
-        <is>
-          <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
-        </is>
-      </c>
-      <c r="F44" s="22" t="inlineStr">
-        <is>
-          <t>500 Internal Server Error</t>
-        </is>
-      </c>
-      <c r="G44" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H44" s="22" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-      <c r="I44" s="22" t="inlineStr">
-        <is>
-          <t>`_validate_required_text` (sign_in.py:178) không chặn ký tự điều khiển; PostgreSQL từ chối NUL trong cột text: `psycopg.DataError: PostgreSQL text fields cannot contain NUL (0x00) bytes` ở `UPDATE users SET full_name…` (SqlUsers.update_profile); không có handler cho DataError nên thành 500. Câu SQL có tham số nên không phải lỗ hổng SQL injection
-Log: evidence/test-integration.log, evidence/test-probe-nul.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="90.5" customHeight="1">
-      <c r="A45" s="22" t="inlineStr">
-        <is>
-          <t>BUG-LOGIN-30</t>
-        </is>
-      </c>
-      <c r="B45" s="22" t="inlineStr">
-        <is>
-          <t>Lưu họ tên dài 256 ký tự</t>
-        </is>
-      </c>
-      <c r="C45" s="22" t="inlineStr">
-        <is>
-          <t>1. POST /auth/profile {ho_ten: A*256}</t>
-        </is>
-      </c>
-      <c r="D45" s="22" t="inlineStr">
-        <is>
-          <t>A*256</t>
-        </is>
-      </c>
-      <c r="E45" s="22" t="inlineStr">
-        <is>
-          <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
-        </is>
-      </c>
-      <c r="F45" s="22" t="inlineStr">
-        <is>
-          <t>204, đã lưu</t>
-        </is>
-      </c>
-      <c r="G45" s="22" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H45" s="22" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-      <c r="I45" s="22" t="inlineStr">
-        <is>
-          <t>Không có giới hạn độ dài họ tên: `_validate_profile` (sign_in.py) chỉ kiểm rỗng; cột users.full_name kiểu text không giới hạn
-Log: evidence/test-integration.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="90.5" customHeight="1">
-      <c r="A46" s="22" t="inlineStr">
-        <is>
-          <t>BUG-LOGIN-32</t>
-        </is>
-      </c>
-      <c r="B46" s="22" t="inlineStr">
-        <is>
-          <t>Lưu ngày sinh trước 1900-01-01</t>
-        </is>
-      </c>
-      <c r="C46" s="22" t="inlineStr">
-        <is>
-          <t>1. POST /auth/profile {ngay_sinh}</t>
-        </is>
-      </c>
-      <c r="D46" s="22" t="inlineStr">
-        <is>
-          <t>1899-12-31 | 0001-01-01</t>
-        </is>
-      </c>
-      <c r="E46" s="22" t="inlineStr">
-        <is>
-          <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
-        </is>
-      </c>
-      <c r="F46" s="22" t="inlineStr">
-        <is>
-          <t>204 ở cả hai giá trị, đã lưu</t>
-        </is>
-      </c>
-      <c r="G46" s="22" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H46" s="22" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-      <c r="I46" s="22" t="inlineStr">
-        <is>
-          <t>`_validate_birth_date` (sign_in.py:229–231) chỉ chặn ngày tương lai, không có cận dưới. App mobile đã giới hạn date picker từ 1900 nên chỉ gặp khi gọi API trực tiếp
-Log: evidence/test-integration.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="123.5" customHeight="1">
-      <c r="A47" s="22" t="inlineStr">
-        <is>
-          <t>BUG-LOGIN-35</t>
-        </is>
-      </c>
-      <c r="B47" s="22" t="inlineStr">
-        <is>
-          <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
-        </is>
-      </c>
-      <c r="C47" s="22" t="inlineStr">
-        <is>
-          <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
-        </is>
-      </c>
-      <c r="D47" s="22" t="inlineStr">
-        <is>
-          <t>ngay_sinh: 2026-10-08</t>
-        </is>
-      </c>
-      <c r="E47" s="22" t="inlineStr">
-        <is>
-          <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
-        </is>
-      </c>
-      <c r="F47" s="22" t="inlineStr">
-        <is>
-          <t>422 {"detail":"invalid_date_of_birth"}</t>
-        </is>
-      </c>
-      <c r="G47" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H47" s="22" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-      <c r="I47" s="22" t="inlineStr">
-        <is>
-          <t>`_validate_birth_date` (sign_in.py:230) so với `now.date()` trong khi `now()` (shared/clock.py) trả giờ UTC: từ 00:00 đến 07:00 giờ VN, "hôm nay" bị coi là ngày mai. Vi phạm bất biến 7 (múi giờ cố định Asia/Ho_Chi_Minh)
-Log: evidence/test-integration.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="173" customHeight="1">
-      <c r="A48" s="22" t="inlineStr">
-        <is>
-          <t>BUG-LOGIN-42</t>
-        </is>
-      </c>
-      <c r="B48" s="22" t="inlineStr">
-        <is>
-          <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
-        </is>
-      </c>
-      <c r="C48" s="22" t="inlineStr">
-        <is>
-          <t>1. Chạm vào ô mã OTP
-2. Theo dõi request backend nhận được</t>
-        </is>
-      </c>
-      <c r="D48" s="22" t="inlineStr">
-        <is>
-          <t>Ô đang chứa 000000</t>
-        </is>
-      </c>
-      <c r="E48" s="22" t="inlineStr">
-        <is>
-          <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
-        </is>
-      </c>
-      <c r="F48" s="22" t="inlineStr">
-        <is>
-          <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
-        </is>
-      </c>
-      <c r="G48" s="22" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H48" s="22" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-      <c r="I48" s="22" t="inlineStr">
-        <is>
-          <t>`OtpPinInput._handleTextChange` (frontend/mobile/lib/features/auth/presentation/widgets/otp_pin_input.dart:66–72) chạy với mọi thông báo của controller, kể cả khi chỉ đổi vị trí con trỏ lúc chạm ô, và gọi onCompleted hễ ô đủ 6 số → gửi lại mã sai, tốn hạn mức token_verifications
-Log: evidence/test-e2e.log (mục "request backend trong pha 2"), evidence/implement-P10-run-phase2-requests.log</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:A5"/>
-  </mergeCells>
-  <conditionalFormatting sqref="F11:F17">
-    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
-      <formula>0.2</formula>
+  <autoFilter ref="A8:I37"/>
+  <conditionalFormatting sqref="H9:H37">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11:G17">
-    <cfRule type="expression" priority="2" dxfId="0">
-      <formula>OR(G11="Critical",G11="High")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G42:G48">
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
-      <formula>"Critical"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2">
-      <formula>"High"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="3">
-      <formula>"Medium"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation sqref="G11:G17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Critical,High,Medium,Low"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G42:G48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Critical,High,Medium,Low"</formula1>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Hồi quy xác nhận liều (REGDOSE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="156.5" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-REGDOSE-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Đối chiếu scheduled_at có giây khi xác nhận liều</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Supabase PostgreSQL local đã reset và migration hiện hành; fixture tạo patient/schedule/consent riêng và override identity.current_user cho patient.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ backend chạy .venv/Scripts/python.exe -m pytest tests/integration/test_dose_confirmation_api.py::test_post_doses_batch_creates_dose_log_for_authenticated_patient__AC1_AC10_AC18 -q -ra.
+2. Fixture POST /doses/batch với danh sách một item ở Test Data.
+3. Đối chiếu items[0].scheduled_at với kỳ vọng test hiện có.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>client_uuid: UUID mới; schedule_id: fixture; scheduled_at=2026-10-02T01:00:59.999Z; taken_at=2026-10-02T01:05:59.999Z</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Theo test hiện có: HTTP 200, synced, da_uong và scheduled_at=2026-10-02T01:00:00Z.</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 200, synced, da_uong; scheduled_at=2026-10-02T01:00:59.999000Z. Fail trong suite DB và lặp lại khi chạy riêng (1 failed trong 1.67s).</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Ngoài AC task 3.05; AC1_AC10_AC18 của test backend hiện có · Đoán lỗi độ chính xác thời gian · test_post_doses_batch_creates_dose_log_for_authenticated_patient__AC1_AC10_AC18</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12">
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H12" s="13">
+        <f>COUNTIF(H9:H9,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H13" s="13">
+        <f>COUNTIF(H9:H9,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H14" s="13">
+        <f>COUNTIF(H9:H9,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H15" s="13">
+        <f>SUM(H12:H14)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I9"/>
+  <conditionalFormatting sqref="H9">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
test: add API contract sync cases
Refs: adhoc-20261015-api-contract-sync
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -16,7 +16,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mã liên kết người thân" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chọn thuốc danh mục" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hồi quy xác nhận liều" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Contract Sync" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Android build'!$A$8:$I$17</definedName>
@@ -29,6 +30,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Mã liên kết người thân'!$A$8:$I$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Chọn thuốc danh mục'!$A$8:$I$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Hồi quy xác nhận liều'!$A$8:$I$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'API Contract Sync'!$A$8:$I$20</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -367,12 +369,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$20</f>
+              <f>'Report'!$A$11:$A$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$11:$D$20</f>
+              <f>'Report'!$D$11:$D$21</f>
             </numRef>
           </val>
         </ser>
@@ -391,12 +393,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$20</f>
+              <f>'Report'!$A$11:$A$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$11:$E$20</f>
+              <f>'Report'!$E$11:$E$21</f>
             </numRef>
           </val>
         </ser>
@@ -415,12 +417,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$20</f>
+              <f>'Report'!$A$11:$A$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$11:$F$20</f>
+              <f>'Report'!$F$11:$F$21</f>
             </numRef>
           </val>
         </ser>
@@ -523,7 +525,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>22</row>
+      <row>23</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -545,7 +547,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>22</row>
+      <row>23</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3240000"/>
@@ -1941,7 +1943,1086 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:T26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Đồng bộ API contract (APIC) (APIC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Quyền truy cập lịch và hồ sơ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="90.5" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-APIC-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Đối chiếu nguồn và phân loại từng delta contract</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Có requirement, contract đã duyệt, operation-schema inventory và snapshot protected 3.16.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở inventory và contract diff.
+2. Truy từng operation/schema mục tiêu tới commit lịch sử hoặc quyết định đã duyệt.
+3. Đối chiếu snapshot protected và ghi rõ khôi phục, mới hoặc mâu thuẫn.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Các operation/schema trong inventory của task.</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Mọi delta có nguồn và phân loại; phần protected 3.16 không đổi.</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr"/>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · manual</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>OpenAPI references</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>Mọi $ref resolve trong document</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>Dangling local $ref</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Caller là patient hoặc caregiver được liên kết?</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>Patient</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>Caregiver</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90.5" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-APIC-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra family link và interaction contract</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Backend dependency và OpenAPI contract task có sẵn.</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy `pytest tests/unit/test_contract_family.py tests/unit/test_contract_interaction.py -q -p no:cacheprovider`.
+2. Đọc kết quả assertions về LinkCode và interaction schemas/operations.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Contract family link và 15 interaction operations.</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Toàn bộ parity assertions pass; LinkCode, query bounds, severity và semantics Q1 đúng contract.</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Implementation evidence: 58 passed, 3 failed toàn parity suite; các lỗi thuộc profile Cache-Control được nêu ở TC-APIC-04.</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · EP (1) · `evidence/implement-P4-parity.log`</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>operationId</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>Mỗi operationId duy nhất</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>operationId trùng giữa hai operation</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>Consent/sharing hợp lệ?</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="74" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-APIC-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra medication và schedule contract</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Backend dependency và OpenAPI contract task có sẵn.</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy `pytest tests/unit/test_contract_medication.py -q -p no:cacheprovider`.
+2. Xem assertions về days_of_week, schedule status/body, query bounds và auth.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>ISO weekday 1..7; giới hạn schedule theo contract.</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Parity test pass; DELETE schedule trả 200 với UserMedication.</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Implementation evidence: suite parity gộp pass cho medication; tổng parity còn ba failure profile Cache-Control.</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · BVA (min/max theo contract) · `evidence/implement-P4-parity.log`</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>profile condition id</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>Condition id của caller</t>
+        </is>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>ID của người khác hoặc không tồn tại</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="Q11" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="74" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-APIC-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra profile và condition contract</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Backend dependency và OpenAPI contract task có sẵn.</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy `pytest tests/unit/test_contract_profile.py -q -p no:cacheprovider`.
+2. Kiểm tra response headers, required/nullability, bearer security và semantics 403/404.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>GET/PUT profile; GET/POST/PATCH/DELETE conditions.</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Toàn bộ profile parity pass, gồm Cache-Control theo contract.</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>3 profile operation thất bại do Cache-Control const ở runtime so với enum trong contract; lỗi được giữ lại theo phạm vi đã duyệt.</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · `evidence/implement-P4-parity.log`</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
+        <is>
+          <t>Được phép; response và audit theo contract</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S12" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="74" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-APIC-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Bảo toàn family-link 3.16</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Checkout backend 3.16 chứa overlay được bảo vệ và snapshot requirement.</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy `pytest tests/unit/test_contract_family_links.py -q -p no:cacheprovider` trên checkout 3.16.
+2. Đối chiếu snapshot protected trước/sau.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Ba operation và sáu schema family-link.</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Mười parity assertions pass; protected fragments deep-equal snapshot.</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>10 passed theo `evidence/implement-family-links.log`; snapshot protected được giữ nguyên theo implement record.</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · `evidence/implement-family-links.log`</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="90.5" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-APIC-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra refs, operationId và schema semantics</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Test semantic regression mới nằm trong linked worktree backend.</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy `pytest tests/unit/test_contract_openapi_semantics.py -q -p no:cacheprovider`.
+2. Xem kiểm tra dangling refs, operationId, bearer security, ValidationError và bounds/nullability.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>OpenAPI contract và fixture hợp lệ/lỗi của semantic tests.</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Document hợp lệ pass; các fixture mồ côi/trùng/mất security hoặc envelope bị đổi bị phát hiện.</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>5 passed trong implement stage.</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (1,2) · `evidence/implement-P3.log`</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="90.5" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-APIC-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Xác nhận PEP, consent và audit cho schedule/profile</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Supabase local có schema task và integration fixtures.</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy toàn bộ integration suite.
+2. Đối chiếu các case allow/deny, revoke và audit trong kết quả.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Patient/caregiver, liên kết, sharing và consent theo fixture từng test.</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>PEP quyết định mỗi request; deny 403 có denied audit, revoke chặn request kế tiếp và audit fail-closed.</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Các suite AC7 trong plan đều pass trong full integration: patient_schedules_access, profile_access, migration_access_self_audit, medication_schedules, medication_schedule_invariants và profile_api.</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · Decision Table (R1,R2) · evidence/test-integration.log</t>
+        </is>
+      </c>
+      <c r="Q15" s="4" t="inlineStr">
+        <is>
+          <t>Profile condition và quyền truy cập</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="107" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-APIC-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Rà soát ngoại lệ Q1 và quyết định profile Q2</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Requirement ghi Q1/Q2 đã được người dùng chốt và stage contract approved.</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. Xác nhận interaction publishing có hiệu lực ngay, không bước duyệt, và nêu ngoại lệ QD-37.
+2. Xác nhận condition ngoài caller/không tồn tại trả 404 user_condition_not_found; PEP deny vẫn 403.</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Q1, Q2 trong requirement và contract đã duyệt.</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Không biến code/test thành nguồn quyết định; ngoại lệ được nêu rõ để reviewer xác nhận.</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr"/>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · manual</t>
+        </is>
+      </c>
+      <c r="Q16" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R16" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S16" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T16" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="57.5" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-APIC-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Xem kết quả full unit và phân loại lỗi còn lại</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Có full unit/architecture evidence từ implement stage.</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Đọc `evidence/implement-final-backend.log`.
+2. Xác nhận số pass/fail và phân loại các lỗi nằm ngoài phạm vi/mismatch đã ghi.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Toàn bộ backend unit và architecture suites.</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Không có failure bị che; lỗi nền và mismatch được báo riêng.</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>815 passed, 9 failed: ba Cache-Control mismatch và sáu lỗi auth trả 422 thay vì 401.</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · `evidence/implement-final-backend.log`</t>
+        </is>
+      </c>
+      <c r="Q17" s="10" t="inlineStr">
+        <is>
+          <t>PEP/consent cho phép?</t>
+        </is>
+      </c>
+      <c r="R17" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S17" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T17" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90.5" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-APIC-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Chạy toàn bộ integration suite trong stage test</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Local Postgres lắng nghe trên 127.0.0.1:54322.</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy pytest tests/integration -vv -p no:cacheprovider từ linked worktree.
+2. Lưu summary và phân loại toàn bộ failure/skip.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Toàn bộ 686 collected tests trong tests/integration.</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Suite kết thúc có summary đầy đủ; mọi lỗi và skip được phân loại riêng, không bị che.</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>524 passed, 2 failed, 159 skipped, 1 xpassed; 5,860 warnings; 18:47. Hai lỗi được ghi tại TC-APIC-11 và TC-APIC-12. 159 test auth skip do supabase status -o env trả non-zero.</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC7, AC9 · evidence/test-integration.log</t>
+        </is>
+      </c>
+      <c r="Q18" s="10" t="inlineStr">
+        <is>
+          <t>Condition thuộc caller và tồn tại?</t>
+        </is>
+      </c>
+      <c r="R18" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S18" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T18" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="90.5" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-APIC-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra test admin role revocation cho catalog sync history</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Local integration DB đã có schema/catalog sync.</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy test_admin_role_revocation_applies_on_next_request__AC8 trong toàn bộ integration suite.
+2. Gửi GET /admin/catalog/sync-runs với admin session do fixture tạo.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Nguồn sync fixture qd_5948.</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Request đầu trả 200 trước khi thu hồi admin role.</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Request phát sinh ValueError: qd_5948 is not a valid CatalogSyncSource trước khi assertion status hoàn tất.</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · test_admin_role_revocation_applies_on_next_request__AC8 · evidence/test-integration.log</t>
+        </is>
+      </c>
+      <c r="Q19" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T19" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="74" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-APIC-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra timestamp của dose batch</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Local integration DB và patient schedule fixture hoạt động.</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy test_post_doses_batch_creates_dose_log_for_authenticated_patient__AC1_AC10_AC18.
+2. Gửi dose batch và so timestamp response với scheduled time.</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Scheduled time 2026-10-02T01:00:00Z.</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Dose log trả đúng scheduled time 2026-10-02T01:00:00Z.</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Response trả 2026-10-02T01:00:59.999000Z; assertion không khớp kỳ vọng.</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · test_post_doses_batch_creates_dose_log_for_authenticated_patient__AC1_AC10_AC18 · evidence/test-integration.log</t>
+        </is>
+      </c>
+      <c r="Q20" s="10" t="inlineStr">
+        <is>
+          <t>403 theo PEP/consent</t>
+        </is>
+      </c>
+      <c r="R20" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S20" s="11" t="inlineStr"/>
+      <c r="T20" s="11" t="inlineStr"/>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="Q21" s="10" t="inlineStr">
+        <is>
+          <t>Thành công theo operation</t>
+        </is>
+      </c>
+      <c r="R21" s="11" t="inlineStr"/>
+      <c r="S21" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T21" s="11" t="inlineStr"/>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="Q22" s="10" t="inlineStr">
+        <is>
+          <t>404 user_condition_not_found</t>
+        </is>
+      </c>
+      <c r="R22" s="11" t="inlineStr"/>
+      <c r="S22" s="11" t="inlineStr"/>
+      <c r="T22" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H23" s="13">
+        <f>COUNTIF(H9:H20,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H24" s="13">
+        <f>COUNTIF(H9:H20,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H25" s="13">
+        <f>COUNTIF(H9:H20,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H26" s="13">
+        <f>SUM(H23:H25)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I20"/>
+  <conditionalFormatting sqref="H9:H20">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1995,7 +3076,7 @@
         <v/>
       </c>
       <c r="D3" s="11">
-        <f>'Chọn thuốc danh mục'!$H$40+'Hồi quy xác nhận liều'!$H$12</f>
+        <f>'Chọn thuốc danh mục'!$H$40+'Hồi quy xác nhận liều'!$H$12+'API Contract Sync'!$H$23</f>
         <v/>
       </c>
       <c r="E3" s="15">
@@ -2015,7 +3096,7 @@
         <v/>
       </c>
       <c r="D4" s="11">
-        <f>'Chọn thuốc danh mục'!$H$41+'Hồi quy xác nhận liều'!$H$13</f>
+        <f>'Chọn thuốc danh mục'!$H$41+'Hồi quy xác nhận liều'!$H$13+'API Contract Sync'!$H$24</f>
         <v/>
       </c>
       <c r="E4" s="15">
@@ -2055,7 +3136,7 @@
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>'Chọn thuốc danh mục'!$H$42+'Hồi quy xác nhận liều'!$H$14</f>
+        <f>'Chọn thuốc danh mục'!$H$42+'Hồi quy xác nhận liều'!$H$14+'API Contract Sync'!$H$25</f>
         <v/>
       </c>
       <c r="E6" s="15">
@@ -2570,496 +3651,736 @@
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="19" t="inlineStr">
+    <row r="21" ht="107" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>Đồng bộ API contract (APIC)</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Khôi phục OpenAPI có truy vết, giữ semantics và xác nhận contract với backend.</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>API Contract Sync</t>
+        </is>
+      </c>
+      <c r="D21" s="18">
+        <f>IFERROR(('API Contract Sync'!$H$26-'API Contract Sync'!$H$25)/'API Contract Sync'!$H$26,0)</f>
+        <v/>
+      </c>
+      <c r="E21" s="18">
+        <f>IFERROR('API Contract Sync'!$H$23/'API Contract Sync'!$H$26,0)</f>
+        <v/>
+      </c>
+      <c r="F21" s="18">
+        <f>IFERROR('API Contract Sync'!$H$24/'API Contract Sync'!$H$26,0)</f>
+        <v/>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>Full integration: 524 passed, 2 failed, 159 skipped, 1 xpassed. AC7 suites pass; unrelated catalog sync and dose batch failures are recorded separately. Parity and full unit/architecture retain documented mismatches.</t>
+        </is>
+      </c>
+      <c r="I21" s="11" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="19" t="inlineStr">
         <is>
           <t>Bug Report</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="20" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="20" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="B44" s="20" t="inlineStr">
+      <c r="B45" s="20" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C44" s="20" t="inlineStr">
+      <c r="C45" s="20" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="D44" s="20" t="inlineStr">
+      <c r="D45" s="20" t="inlineStr">
         <is>
           <t>Input Data</t>
         </is>
       </c>
-      <c r="E44" s="20" t="inlineStr">
+      <c r="E45" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F44" s="20" t="inlineStr">
+      <c r="F45" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="G44" s="20" t="inlineStr">
+      <c r="G45" s="20" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="H44" s="20" t="inlineStr">
+      <c r="H45" s="20" t="inlineStr">
         <is>
           <t>Name of Tester</t>
         </is>
       </c>
-      <c r="I44" s="20" t="inlineStr">
+      <c r="I45" s="20" t="inlineStr">
         <is>
           <t>Logs</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="123.5" customHeight="1">
-      <c r="A45" s="22" t="inlineStr">
+    <row r="46" ht="123.5" customHeight="1">
+      <c r="A46" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-08</t>
         </is>
       </c>
-      <c r="B45" s="22" t="inlineStr">
+      <c r="B46" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
         </is>
       </c>
-      <c r="C45" s="22" t="inlineStr">
+      <c r="C46" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
 2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
         </is>
       </c>
-      <c r="D45" s="22" t="inlineStr">
+      <c r="D46" s="22" t="inlineStr">
         <is>
           <t>phone: 0900000001 + ký tự \n</t>
         </is>
       </c>
-      <c r="E45" s="22" t="inlineStr">
+      <c r="E46" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F45" s="22" t="inlineStr">
+      <c r="F46" s="22" t="inlineStr">
         <is>
           <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
         </is>
       </c>
-      <c r="G45" s="22" t="inlineStr">
+      <c r="G46" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H45" s="22" t="inlineStr">
+      <c r="H46" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I45" s="22" t="inlineStr">
+      <c r="I46" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn — kỳ vọng AC6 mâu thuẫn AC5: backend `_validate_required_text` (sign_in.py:178) `strip()` mọi ký tự trắng hai đầu, nên \n cuối được xử lý như khoảng trắng hai đầu mà AC5 coi là hợp lệ. Cần người dùng chốt: sửa AC6 hoặc sửa backend
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="123.5" customHeight="1">
-      <c r="A46" s="22" t="inlineStr">
+    <row r="47" ht="123.5" customHeight="1">
+      <c r="A47" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-11</t>
         </is>
       </c>
-      <c r="B46" s="22" t="inlineStr">
+      <c r="B47" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
         </is>
       </c>
-      <c r="C46" s="22" t="inlineStr">
+      <c r="C47" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone}
 2. POST /auth/mobile/verify {phone, token: 123456}</t>
         </is>
       </c>
-      <c r="D46" s="22" t="inlineStr">
+      <c r="D47" s="22" t="inlineStr">
         <is>
           <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
         </is>
       </c>
-      <c r="E46" s="22" t="inlineStr">
+      <c r="E47" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
         </is>
       </c>
-      <c r="F46" s="22" t="inlineStr">
+      <c r="F47" s="22" t="inlineStr">
         <is>
           <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
         </is>
       </c>
-      <c r="G46" s="22" t="inlineStr">
+      <c r="G47" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H46" s="22" t="inlineStr">
+      <c r="H47" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I46" s="22" t="inlineStr">
+      <c r="I47" s="22" t="inlineStr">
         <is>
           <t>`_normalize_phone` (sign_in.py:197–206) kiểm bằng `str.isdigit()`, nhận cả chữ số Unicode, nên số lọt qua kiểm tra và gửi tới Supabase. Ô nhập của app chỉ cho 0-9 nên người dùng app không gặp; lỗi ở tầng API
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="189.5" customHeight="1">
-      <c r="A47" s="22" t="inlineStr">
+    <row r="48" ht="189.5" customHeight="1">
+      <c r="A48" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-25</t>
         </is>
       </c>
-      <c r="B47" s="22" t="inlineStr">
+      <c r="B48" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên có ký tự NUL</t>
         </is>
       </c>
-      <c r="C47" s="22" t="inlineStr">
+      <c r="C48" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
         </is>
       </c>
-      <c r="D47" s="22" t="inlineStr">
+      <c r="D48" s="22" t="inlineStr">
         <is>
           <t>ho_ten: abc\u0000def</t>
         </is>
       </c>
-      <c r="E47" s="22" t="inlineStr">
+      <c r="E48" s="22" t="inlineStr">
         <is>
           <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
         </is>
       </c>
-      <c r="F47" s="22" t="inlineStr">
+      <c r="F48" s="22" t="inlineStr">
         <is>
           <t>500 Internal Server Error</t>
         </is>
       </c>
-      <c r="G47" s="22" t="inlineStr">
+      <c r="G48" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H47" s="22" t="inlineStr">
+      <c r="H48" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I47" s="22" t="inlineStr">
+      <c r="I48" s="22" t="inlineStr">
         <is>
           <t>`_validate_required_text` (sign_in.py:178) không chặn ký tự điều khiển; PostgreSQL từ chối NUL trong cột text: `psycopg.DataError: PostgreSQL text fields cannot contain NUL (0x00) bytes` ở `UPDATE users SET full_name…` (SqlUsers.update_profile); không có handler cho DataError nên thành 500. Câu SQL có tham số nên không phải lỗ hổng SQL injection
 Log: evidence/test-integration.log, evidence/test-probe-nul.log</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="90.5" customHeight="1">
-      <c r="A48" s="22" t="inlineStr">
+    <row r="49" ht="90.5" customHeight="1">
+      <c r="A49" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-30</t>
         </is>
       </c>
-      <c r="B48" s="22" t="inlineStr">
+      <c r="B49" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên dài 256 ký tự</t>
         </is>
       </c>
-      <c r="C48" s="22" t="inlineStr">
+      <c r="C49" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: A*256}</t>
         </is>
       </c>
-      <c r="D48" s="22" t="inlineStr">
+      <c r="D49" s="22" t="inlineStr">
         <is>
           <t>A*256</t>
         </is>
       </c>
-      <c r="E48" s="22" t="inlineStr">
+      <c r="E49" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F48" s="22" t="inlineStr">
+      <c r="F49" s="22" t="inlineStr">
         <is>
           <t>204, đã lưu</t>
         </is>
       </c>
-      <c r="G48" s="22" t="inlineStr">
+      <c r="G49" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H48" s="22" t="inlineStr">
+      <c r="H49" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I48" s="22" t="inlineStr">
+      <c r="I49" s="22" t="inlineStr">
         <is>
           <t>Không có giới hạn độ dài họ tên: `_validate_profile` (sign_in.py) chỉ kiểm rỗng; cột users.full_name kiểu text không giới hạn
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="90.5" customHeight="1">
-      <c r="A49" s="22" t="inlineStr">
+    <row r="50" ht="90.5" customHeight="1">
+      <c r="A50" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-32</t>
         </is>
       </c>
-      <c r="B49" s="22" t="inlineStr">
+      <c r="B50" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh trước 1900-01-01</t>
         </is>
       </c>
-      <c r="C49" s="22" t="inlineStr">
+      <c r="C50" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh}</t>
         </is>
       </c>
-      <c r="D49" s="22" t="inlineStr">
+      <c r="D50" s="22" t="inlineStr">
         <is>
           <t>1899-12-31 | 0001-01-01</t>
         </is>
       </c>
-      <c r="E49" s="22" t="inlineStr">
+      <c r="E50" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
         </is>
       </c>
-      <c r="F49" s="22" t="inlineStr">
+      <c r="F50" s="22" t="inlineStr">
         <is>
           <t>204 ở cả hai giá trị, đã lưu</t>
         </is>
       </c>
-      <c r="G49" s="22" t="inlineStr">
+      <c r="G50" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H49" s="22" t="inlineStr">
+      <c r="H50" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I49" s="22" t="inlineStr">
+      <c r="I50" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:229–231) chỉ chặn ngày tương lai, không có cận dưới. App mobile đã giới hạn date picker từ 1900 nên chỉ gặp khi gọi API trực tiếp
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="123.5" customHeight="1">
-      <c r="A50" s="22" t="inlineStr">
+    <row r="51" ht="123.5" customHeight="1">
+      <c r="A51" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-35</t>
         </is>
       </c>
-      <c r="B50" s="22" t="inlineStr">
+      <c r="B51" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
         </is>
       </c>
-      <c r="C50" s="22" t="inlineStr">
+      <c r="C51" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
         </is>
       </c>
-      <c r="D50" s="22" t="inlineStr">
+      <c r="D51" s="22" t="inlineStr">
         <is>
           <t>ngay_sinh: 2026-10-08</t>
         </is>
       </c>
-      <c r="E50" s="22" t="inlineStr">
+      <c r="E51" s="22" t="inlineStr">
         <is>
           <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
         </is>
       </c>
-      <c r="F50" s="22" t="inlineStr">
+      <c r="F51" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_date_of_birth"}</t>
         </is>
       </c>
-      <c r="G50" s="22" t="inlineStr">
+      <c r="G51" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H50" s="22" t="inlineStr">
+      <c r="H51" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I50" s="22" t="inlineStr">
+      <c r="I51" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:230) so với `now.date()` trong khi `now()` (shared/clock.py) trả giờ UTC: từ 00:00 đến 07:00 giờ VN, "hôm nay" bị coi là ngày mai. Vi phạm bất biến 7 (múi giờ cố định Asia/Ho_Chi_Minh)
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="173" customHeight="1">
-      <c r="A51" s="22" t="inlineStr">
+    <row r="52" ht="173" customHeight="1">
+      <c r="A52" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-42</t>
         </is>
       </c>
-      <c r="B51" s="22" t="inlineStr">
+      <c r="B52" s="22" t="inlineStr">
         <is>
           <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
         </is>
       </c>
-      <c r="C51" s="22" t="inlineStr">
+      <c r="C52" s="22" t="inlineStr">
         <is>
           <t>1. Chạm vào ô mã OTP
 2. Theo dõi request backend nhận được</t>
         </is>
       </c>
-      <c r="D51" s="22" t="inlineStr">
+      <c r="D52" s="22" t="inlineStr">
         <is>
           <t>Ô đang chứa 000000</t>
         </is>
       </c>
-      <c r="E51" s="22" t="inlineStr">
+      <c r="E52" s="22" t="inlineStr">
         <is>
           <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
         </is>
       </c>
-      <c r="F51" s="22" t="inlineStr">
+      <c r="F52" s="22" t="inlineStr">
         <is>
           <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
         </is>
       </c>
-      <c r="G51" s="22" t="inlineStr">
+      <c r="G52" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H51" s="22" t="inlineStr">
+      <c r="H52" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I51" s="22" t="inlineStr">
+      <c r="I52" s="22" t="inlineStr">
         <is>
           <t>`OtpPinInput._handleTextChange` (frontend/mobile/lib/features/auth/presentation/widgets/otp_pin_input.dart:66–72) chạy với mọi thông báo của controller, kể cả khi chỉ đổi vị trí con trỏ lúc chạm ô, và gọi onCompleted hễ ô đủ 6 số → gửi lại mã sai, tốn hạn mức token_verifications
 Log: evidence/test-e2e.log (mục "request backend trong pha 2"), evidence/implement-P10-run-phase2-requests.log</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="189.5" customHeight="1">
-      <c r="A52" s="22" t="inlineStr">
+    <row r="53" ht="189.5" customHeight="1">
+      <c r="A53" s="22" t="inlineStr">
         <is>
           <t>BUG-LINKCODE-28</t>
         </is>
       </c>
-      <c r="B52" s="22" t="inlineStr">
+      <c r="B53" s="22" t="inlineStr">
         <is>
           <t>Toàn bộ unit test, architecture test và ruff toàn repo pass</t>
         </is>
       </c>
-      <c r="C52" s="22" t="inlineStr">
+      <c r="C53" s="22" t="inlineStr">
         <is>
           <t>1. pytest tests/unit tests/architecture -q
 2. ruff check .
 3. So với baseline trước khi sửa code</t>
         </is>
       </c>
-      <c r="D52" s="22" t="inlineStr">
+      <c r="D53" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E52" s="22" t="inlineStr">
+      <c r="E53" s="22" t="inlineStr">
         <is>
           <t>pytest và ruff đều pass</t>
         </is>
       </c>
-      <c r="F52" s="22" t="inlineStr">
+      <c r="F53" s="22" t="inlineStr">
         <is>
           <t>697 pass, 1 fail (tests/unit/test_app.py::test_doses_batch_openapi_uses_contract_shape: NameError paths); ruff toàn repo 21 lỗi ở module khác. Fail và lỗi ruff đã có trước khi task sửa code; file của task pass ruff</t>
         </is>
       </c>
-      <c r="G52" s="22" t="inlineStr">
+      <c r="G53" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H52" s="22" t="inlineStr">
+      <c r="H53" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I52" s="22" t="inlineStr">
+      <c r="I53" s="22" t="inlineStr">
         <is>
           <t>Có sẵn trên main, không do task 3.10: test_app.py dòng 43–44 dùng biến paths chưa định nghĩa; ruff báo lỗi ở catalog/*, consent/adapters/outbound/job_queue.py, runtime/job_runner.py (F821 health chưa import, nghi vấn làm Worker lỗi khi ghi heartbeat), worker.py, tests/unit/test_catalog_crud.py
 Log: evidence/implement-final-backend.log</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="239" customHeight="1">
-      <c r="A53" s="22" t="inlineStr">
+    <row r="54" ht="239" customHeight="1">
+      <c r="A54" s="22" t="inlineStr">
         <is>
           <t>BUG-REGDOSE-01</t>
         </is>
       </c>
-      <c r="B53" s="22" t="inlineStr">
+      <c r="B54" s="22" t="inlineStr">
         <is>
           <t>Đối chiếu scheduled_at có giây khi xác nhận liều</t>
         </is>
       </c>
-      <c r="C53" s="22" t="inlineStr">
+      <c r="C54" s="22" t="inlineStr">
         <is>
           <t>1. Từ backend chạy .venv/Scripts/python.exe -m pytest tests/integration/test_dose_confirmation_api.py::test_post_doses_batch_creates_dose_log_for_authenticated_patient__AC1_AC10_AC18 -q -ra.
 2. Fixture POST /doses/batch với danh sách một item ở Test Data.
 3. Đối chiếu items[0].scheduled_at với kỳ vọng test hiện có.</t>
         </is>
       </c>
-      <c r="D53" s="22" t="inlineStr">
+      <c r="D54" s="22" t="inlineStr">
         <is>
           <t>client_uuid: UUID mới; schedule_id: fixture; scheduled_at=2026-10-02T01:00:59.999Z; taken_at=2026-10-02T01:05:59.999Z</t>
         </is>
       </c>
-      <c r="E53" s="22" t="inlineStr">
+      <c r="E54" s="22" t="inlineStr">
         <is>
           <t>Theo test hiện có: HTTP 200, synced, da_uong và scheduled_at=2026-10-02T01:00:00Z.</t>
         </is>
       </c>
-      <c r="F53" s="22" t="inlineStr">
+      <c r="F54" s="22" t="inlineStr">
         <is>
           <t>HTTP 200, synced, da_uong; scheduled_at=2026-10-02T01:00:59.999000Z. Fail trong suite DB và lặp lại khi chạy riêng (1 failed trong 1.67s).</t>
         </is>
       </c>
-      <c r="G53" s="22" t="inlineStr">
+      <c r="G54" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H53" s="22" t="inlineStr">
+      <c r="H54" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I53" s="22" t="inlineStr">
+      <c r="I54" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn kỳ vọng chuẩn hóa tới phút trong test không khớp hành vi giữ thời điểm của API; chưa xác định phía nào sai theo contract/nghiệp vụ. Chưa chứng minh mất/trùng bản ghi liều; mức Medium tạm thời cho sai khác test, phải nâng tối thiểu High nếu xác nhận mất/trùng liều.
 Log: evidence/test-integration-db.log; evidence/test-dose-mismatch-repeat.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="123.5" customHeight="1">
+      <c r="A55" s="22" t="inlineStr">
+        <is>
+          <t>BUG-APIC-04</t>
+        </is>
+      </c>
+      <c r="B55" s="22" t="inlineStr">
+        <is>
+          <t>Kiểm tra profile và condition contract</t>
+        </is>
+      </c>
+      <c r="C55" s="22" t="inlineStr">
+        <is>
+          <t>1. Chạy `pytest tests/unit/test_contract_profile.py -q -p no:cacheprovider`.
+2. Kiểm tra response headers, required/nullability, bearer security và semantics 403/404.</t>
+        </is>
+      </c>
+      <c r="D55" s="22" t="inlineStr">
+        <is>
+          <t>GET/PUT profile; GET/POST/PATCH/DELETE conditions.</t>
+        </is>
+      </c>
+      <c r="E55" s="22" t="inlineStr">
+        <is>
+          <t>Toàn bộ profile parity pass, gồm Cache-Control theo contract.</t>
+        </is>
+      </c>
+      <c r="F55" s="22" t="inlineStr">
+        <is>
+          <t>3 profile operation thất bại do Cache-Control const ở runtime so với enum trong contract; lỗi được giữ lại theo phạm vi đã duyệt.</t>
+        </is>
+      </c>
+      <c r="G55" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H55" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I55" s="22" t="inlineStr">
+        <is>
+          <t>Đã xác định mismatch giữa metadata Cache-Control của generated runtime OpenAPI và contract chuẩn.
+Log: evidence/implement-P4-parity.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="90.5" customHeight="1">
+      <c r="A56" s="22" t="inlineStr">
+        <is>
+          <t>BUG-APIC-09</t>
+        </is>
+      </c>
+      <c r="B56" s="22" t="inlineStr">
+        <is>
+          <t>Xem kết quả full unit và phân loại lỗi còn lại</t>
+        </is>
+      </c>
+      <c r="C56" s="22" t="inlineStr">
+        <is>
+          <t>1. Đọc `evidence/implement-final-backend.log`.
+2. Xác nhận số pass/fail và phân loại các lỗi nằm ngoài phạm vi/mismatch đã ghi.</t>
+        </is>
+      </c>
+      <c r="D56" s="22" t="inlineStr">
+        <is>
+          <t>Toàn bộ backend unit và architecture suites.</t>
+        </is>
+      </c>
+      <c r="E56" s="22" t="inlineStr">
+        <is>
+          <t>Không có failure bị che; lỗi nền và mismatch được báo riêng.</t>
+        </is>
+      </c>
+      <c r="F56" s="22" t="inlineStr">
+        <is>
+          <t>815 passed, 9 failed: ba Cache-Control mismatch và sáu lỗi auth trả 422 thay vì 401.</t>
+        </is>
+      </c>
+      <c r="G56" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H56" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I56" s="22" t="inlineStr">
+        <is>
+          <t>Ba failure contract-runtime Cache-Control đã xác định; sáu lỗi auth 422 thay vì 401 còn là lỗi hiện có ngoài phạm vi, nguyên nhân gốc chưa xác định trong task này.
+Log: evidence/implement-final-backend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="123.5" customHeight="1">
+      <c r="A57" s="22" t="inlineStr">
+        <is>
+          <t>BUG-APIC-11</t>
+        </is>
+      </c>
+      <c r="B57" s="22" t="inlineStr">
+        <is>
+          <t>Kiểm tra test admin role revocation cho catalog sync history</t>
+        </is>
+      </c>
+      <c r="C57" s="22" t="inlineStr">
+        <is>
+          <t>1. Chạy test_admin_role_revocation_applies_on_next_request__AC8 trong toàn bộ integration suite.
+2. Gửi GET /admin/catalog/sync-runs với admin session do fixture tạo.</t>
+        </is>
+      </c>
+      <c r="D57" s="22" t="inlineStr">
+        <is>
+          <t>Nguồn sync fixture qd_5948.</t>
+        </is>
+      </c>
+      <c r="E57" s="22" t="inlineStr">
+        <is>
+          <t>Request đầu trả 200 trước khi thu hồi admin role.</t>
+        </is>
+      </c>
+      <c r="F57" s="22" t="inlineStr">
+        <is>
+          <t>Request phát sinh ValueError: qd_5948 is not a valid CatalogSyncSource trước khi assertion status hoàn tất.</t>
+        </is>
+      </c>
+      <c r="G57" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H57" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I57" s="22" t="inlineStr">
+        <is>
+          <t>Nguyên nhân gốc chưa xác định; nghi vấn fixture dùng catalog sync source không có trong enum CatalogSyncSource.
+Log: evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="123.5" customHeight="1">
+      <c r="A58" s="22" t="inlineStr">
+        <is>
+          <t>BUG-APIC-12</t>
+        </is>
+      </c>
+      <c r="B58" s="22" t="inlineStr">
+        <is>
+          <t>Kiểm tra timestamp của dose batch</t>
+        </is>
+      </c>
+      <c r="C58" s="22" t="inlineStr">
+        <is>
+          <t>1. Chạy test_post_doses_batch_creates_dose_log_for_authenticated_patient__AC1_AC10_AC18.
+2. Gửi dose batch và so timestamp response với scheduled time.</t>
+        </is>
+      </c>
+      <c r="D58" s="22" t="inlineStr">
+        <is>
+          <t>Scheduled time 2026-10-02T01:00:00Z.</t>
+        </is>
+      </c>
+      <c r="E58" s="22" t="inlineStr">
+        <is>
+          <t>Dose log trả đúng scheduled time 2026-10-02T01:00:00Z.</t>
+        </is>
+      </c>
+      <c r="F58" s="22" t="inlineStr">
+        <is>
+          <t>Response trả 2026-10-02T01:00:59.999000Z; assertion không khớp kỳ vọng.</t>
+        </is>
+      </c>
+      <c r="G58" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H58" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I58" s="22" t="inlineStr">
+        <is>
+          <t>Nguyên nhân gốc chưa xác định; nghi vấn time-window selection trả cuối cửa sổ một phút thay vì scheduled time.
+Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
@@ -3068,17 +4389,17 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:A5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11:F20">
+  <conditionalFormatting sqref="F11:F21">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11:G20">
+  <conditionalFormatting sqref="G11:G21">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>OR(G11="Critical",G11="High")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G45:G53">
+  <conditionalFormatting sqref="G46:G58">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
@@ -3090,10 +4411,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G11:G20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G11:G21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="G45:G53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G46:G58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(test): add profile auth test cases and update testcase book
Refs: adhoc-20261016-profile-auth-test-fixture
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -17,7 +17,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chọn thuốc danh mục" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hồi quy xác nhận liều" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Contract Sync" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profile auth test" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Android build'!$A$8:$I$17</definedName>
@@ -31,6 +32,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Chọn thuốc danh mục'!$A$8:$I$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Hồi quy xác nhận liều'!$A$8:$I$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'API Contract Sync'!$A$8:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Profile auth test'!$A$8:$I$12</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -369,12 +371,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$21</f>
+              <f>'Report'!$A$11:$A$22</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$11:$D$21</f>
+              <f>'Report'!$D$11:$D$22</f>
             </numRef>
           </val>
         </ser>
@@ -393,12 +395,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$21</f>
+              <f>'Report'!$A$11:$A$22</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$11:$E$21</f>
+              <f>'Report'!$E$11:$E$22</f>
             </numRef>
           </val>
         </ser>
@@ -417,12 +419,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$21</f>
+              <f>'Report'!$A$11:$A$22</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$11:$F$21</f>
+              <f>'Report'!$F$11:$F$22</f>
             </numRef>
           </val>
         </ser>
@@ -525,7 +527,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>23</row>
+      <row>24</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -547,7 +549,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>23</row>
+      <row>24</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3240000"/>
@@ -3022,7 +3024,611 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:U18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Cấu hình xác thực test hồ sơ sức khỏe (PROFAUTH)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Xử lý xác thực theo loại token và cấu hình secret</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="123.5" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-PROFAUTH-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Xác thực thất bại với Bearer token không hợp lệ tới 6 endpoint profile/conditions khi có fixture secret</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Backend unit test client nạp fixture autouse session_secret (SESSION_JWT_SECRET được cấu hình).</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Khởi tạo FastAPI TestClient từ create_app() với override get_uow.
+2. Gửi request kèm header Authorization: Bearer not-a-real-token tới GET /profile, PUT /profile, POST /profile/conditions, PATCH /profile/conditions/1, DELETE /profile/conditions/1, GET /conditions.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Authorization: Bearer not-a-real-token</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Tất cả 6 endpoint đều trả về HTTP 401 Unauthorized với chi tiết 'Invalid or expired session', không ném 422.</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>6/6 test case pass, trả về HTTP 401 Unauthorized (log evidence/implement-P3.log)</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · Decision Table (R1) · test_invalid_or_erased_auth[invalid-*]</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>Authorization header</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>Bearer token hợp lệ có sub (erased=False)</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>(blank) không gửi header
+Bearer token không hợp lệ (not-a-real-token)
+Bearer token của tài khoản đã bị xóa (erased=True)</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>2
+3
+4</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Loại token</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>erased</t>
+        </is>
+      </c>
+      <c r="U9" s="11" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90.5" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-PROFAUTH-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Xác thực thất bại với Bearer token của tài khoản đã bị xóa (erased=True)</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Backend unit test client với fixture autouse session_secret và mock SqlUsers trả về user có erased=True.</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Khởi tạo TestClient với dependency override SqlUsers trả về user có erased=True.
+2. Gửi request kèm header Authorization: Bearer not-a-real-token tới các endpoint profile/conditions.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Authorization: Bearer not-a-real-token; user.erased=True</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Tất cả endpoint trả về HTTP 401 Unauthorized.</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>6/6 test case pass, trả về HTTP 401 Unauthorized (log evidence/implement-P3.log)</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · Decision Table (R3) · test_invalid_or_erased_auth[erased-*]</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>SESSION_JWT_SECRET đã cấu hình?</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90.5" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-PROFAUTH-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Xác thực thất bại khi không gửi Authorization header tới các endpoint profile/conditions</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>App backend khởi tạo với get_uow mock, không cung cấp thông tin xác thực.</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Khởi tạo TestClient.
+2. Gửi request không có header Authorization tới GET /profile, PUT /profile, POST /profile/conditions, PATCH /profile/conditions/1, DELETE /profile/conditions/1, GET /conditions.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Server từ chối truy cập và trả về HTTP 401 Unauthorized cho tất cả các thao tác.</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>6/6 test case pass, trả về HTTP 401 Unauthorized (log evidence/implement-P3.log)</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · EP (2) · test_unauthenticated_all_operations</t>
+        </is>
+      </c>
+      <c r="Q11" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T11" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U11" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="74" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-PROFAUTH-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Toàn bộ test suite test_profile_http pass và cô lập cache get_settings</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Môi trường pytest với fixture session_secret thực hiện get_settings.cache_clear() trước (setup) và sau (teardown).</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy lệnh pytest backend/tests/unit/test_profile_http.py.
+2. Quan sát kết quả kiểm thử và cảnh báo nếu có.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Toàn bộ 54 ca test trong test_profile_http.py</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>54/54 ca test pass (100%), không có test nào fail hoặc error do thiếu cấu hình secret hay rò rỉ cache settings giữa các test.</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>54 passed, 1 warning trong 7.98s (log evidence/implement-P3.log)</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · test_profile_http.py suite</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S12" s="11" t="inlineStr"/>
+      <c r="T12" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="Q13" s="10" t="inlineStr">
+        <is>
+          <t>HTTP 422 DomainError (lỗi cũ)</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="inlineStr"/>
+      <c r="S13" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T13" s="11" t="inlineStr"/>
+      <c r="U13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>HTTP 200/201/204 Success</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr"/>
+      <c r="S14" s="11" t="inlineStr"/>
+      <c r="T14" s="11" t="inlineStr"/>
+      <c r="U14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H15" s="13">
+        <f>COUNTIF(H9:H12,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H16" s="13">
+        <f>COUNTIF(H9:H12,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H17" s="13">
+        <f>COUNTIF(H9:H12,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H18" s="13">
+        <f>SUM(H15:H17)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I12"/>
+  <conditionalFormatting sqref="H9:H12">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3076,7 +3682,7 @@
         <v/>
       </c>
       <c r="D3" s="11">
-        <f>'Chọn thuốc danh mục'!$H$40+'Hồi quy xác nhận liều'!$H$12+'API Contract Sync'!$H$23</f>
+        <f>'Chọn thuốc danh mục'!$H$40+'Hồi quy xác nhận liều'!$H$12+'API Contract Sync'!$H$23+'Profile auth test'!$H$15</f>
         <v/>
       </c>
       <c r="E3" s="15">
@@ -3096,7 +3702,7 @@
         <v/>
       </c>
       <c r="D4" s="11">
-        <f>'Chọn thuốc danh mục'!$H$41+'Hồi quy xác nhận liều'!$H$13+'API Contract Sync'!$H$24</f>
+        <f>'Chọn thuốc danh mục'!$H$41+'Hồi quy xác nhận liều'!$H$13+'API Contract Sync'!$H$24+'Profile auth test'!$H$16</f>
         <v/>
       </c>
       <c r="E4" s="15">
@@ -3136,7 +3742,7 @@
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>'Chọn thuốc danh mục'!$H$42+'Hồi quy xác nhận liều'!$H$14+'API Contract Sync'!$H$25</f>
+        <f>'Chọn thuốc danh mục'!$H$42+'Hồi quy xác nhận liều'!$H$14+'API Contract Sync'!$H$25+'Profile auth test'!$H$17</f>
         <v/>
       </c>
       <c r="E6" s="15">
@@ -3695,689 +4301,733 @@
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="19" t="inlineStr">
+    <row r="22" ht="90.5" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Cấu hình xác thực test hồ sơ sức khỏe</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Fixture cấu hình SESSION_JWT_SECRET và cô lập cache cho các test case xác thực profile_http</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Profile auth test</t>
+        </is>
+      </c>
+      <c r="D22" s="18">
+        <f>IFERROR(('Profile auth test'!$H$18-'Profile auth test'!$H$17)/'Profile auth test'!$H$18,0)</f>
+        <v/>
+      </c>
+      <c r="E22" s="18">
+        <f>IFERROR('Profile auth test'!$H$15/'Profile auth test'!$H$18,0)</f>
+        <v/>
+      </c>
+      <c r="F22" s="18">
+        <f>IFERROR('Profile auth test'!$H$16/'Profile auth test'!$H$18,0)</f>
+        <v/>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>Đã khắc phục lỗi thiếu secret fixture khiến 6 ca test invalid auth trả về 422 thay vì 401; toàn bộ 54/54 test pass.</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="19" t="inlineStr">
         <is>
           <t>Bug Report</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="20" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="20" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="B45" s="20" t="inlineStr">
+      <c r="B46" s="20" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C45" s="20" t="inlineStr">
+      <c r="C46" s="20" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="D45" s="20" t="inlineStr">
+      <c r="D46" s="20" t="inlineStr">
         <is>
           <t>Input Data</t>
         </is>
       </c>
-      <c r="E45" s="20" t="inlineStr">
+      <c r="E46" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F45" s="20" t="inlineStr">
+      <c r="F46" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="G45" s="20" t="inlineStr">
+      <c r="G46" s="20" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="H45" s="20" t="inlineStr">
+      <c r="H46" s="20" t="inlineStr">
         <is>
           <t>Name of Tester</t>
         </is>
       </c>
-      <c r="I45" s="20" t="inlineStr">
+      <c r="I46" s="20" t="inlineStr">
         <is>
           <t>Logs</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="123.5" customHeight="1">
-      <c r="A46" s="22" t="inlineStr">
+    <row r="47" ht="123.5" customHeight="1">
+      <c r="A47" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-08</t>
         </is>
       </c>
-      <c r="B46" s="22" t="inlineStr">
+      <c r="B47" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
         </is>
       </c>
-      <c r="C46" s="22" t="inlineStr">
+      <c r="C47" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
 2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
         </is>
       </c>
-      <c r="D46" s="22" t="inlineStr">
+      <c r="D47" s="22" t="inlineStr">
         <is>
           <t>phone: 0900000001 + ký tự \n</t>
         </is>
       </c>
-      <c r="E46" s="22" t="inlineStr">
+      <c r="E47" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F46" s="22" t="inlineStr">
+      <c r="F47" s="22" t="inlineStr">
         <is>
           <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
         </is>
       </c>
-      <c r="G46" s="22" t="inlineStr">
+      <c r="G47" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H46" s="22" t="inlineStr">
+      <c r="H47" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I46" s="22" t="inlineStr">
+      <c r="I47" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn — kỳ vọng AC6 mâu thuẫn AC5: backend `_validate_required_text` (sign_in.py:178) `strip()` mọi ký tự trắng hai đầu, nên \n cuối được xử lý như khoảng trắng hai đầu mà AC5 coi là hợp lệ. Cần người dùng chốt: sửa AC6 hoặc sửa backend
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="123.5" customHeight="1">
-      <c r="A47" s="22" t="inlineStr">
+    <row r="48" ht="123.5" customHeight="1">
+      <c r="A48" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-11</t>
         </is>
       </c>
-      <c r="B47" s="22" t="inlineStr">
+      <c r="B48" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
         </is>
       </c>
-      <c r="C47" s="22" t="inlineStr">
+      <c r="C48" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone}
 2. POST /auth/mobile/verify {phone, token: 123456}</t>
         </is>
       </c>
-      <c r="D47" s="22" t="inlineStr">
+      <c r="D48" s="22" t="inlineStr">
         <is>
           <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
         </is>
       </c>
-      <c r="E47" s="22" t="inlineStr">
+      <c r="E48" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
         </is>
       </c>
-      <c r="F47" s="22" t="inlineStr">
+      <c r="F48" s="22" t="inlineStr">
         <is>
           <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
         </is>
       </c>
-      <c r="G47" s="22" t="inlineStr">
+      <c r="G48" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H47" s="22" t="inlineStr">
+      <c r="H48" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I47" s="22" t="inlineStr">
+      <c r="I48" s="22" t="inlineStr">
         <is>
           <t>`_normalize_phone` (sign_in.py:197–206) kiểm bằng `str.isdigit()`, nhận cả chữ số Unicode, nên số lọt qua kiểm tra và gửi tới Supabase. Ô nhập của app chỉ cho 0-9 nên người dùng app không gặp; lỗi ở tầng API
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="189.5" customHeight="1">
-      <c r="A48" s="22" t="inlineStr">
+    <row r="49" ht="189.5" customHeight="1">
+      <c r="A49" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-25</t>
         </is>
       </c>
-      <c r="B48" s="22" t="inlineStr">
+      <c r="B49" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên có ký tự NUL</t>
         </is>
       </c>
-      <c r="C48" s="22" t="inlineStr">
+      <c r="C49" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
         </is>
       </c>
-      <c r="D48" s="22" t="inlineStr">
+      <c r="D49" s="22" t="inlineStr">
         <is>
           <t>ho_ten: abc\u0000def</t>
         </is>
       </c>
-      <c r="E48" s="22" t="inlineStr">
+      <c r="E49" s="22" t="inlineStr">
         <is>
           <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
         </is>
       </c>
-      <c r="F48" s="22" t="inlineStr">
+      <c r="F49" s="22" t="inlineStr">
         <is>
           <t>500 Internal Server Error</t>
         </is>
       </c>
-      <c r="G48" s="22" t="inlineStr">
+      <c r="G49" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H48" s="22" t="inlineStr">
+      <c r="H49" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I48" s="22" t="inlineStr">
+      <c r="I49" s="22" t="inlineStr">
         <is>
           <t>`_validate_required_text` (sign_in.py:178) không chặn ký tự điều khiển; PostgreSQL từ chối NUL trong cột text: `psycopg.DataError: PostgreSQL text fields cannot contain NUL (0x00) bytes` ở `UPDATE users SET full_name…` (SqlUsers.update_profile); không có handler cho DataError nên thành 500. Câu SQL có tham số nên không phải lỗ hổng SQL injection
 Log: evidence/test-integration.log, evidence/test-probe-nul.log</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="90.5" customHeight="1">
-      <c r="A49" s="22" t="inlineStr">
+    <row r="50" ht="90.5" customHeight="1">
+      <c r="A50" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-30</t>
         </is>
       </c>
-      <c r="B49" s="22" t="inlineStr">
+      <c r="B50" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên dài 256 ký tự</t>
         </is>
       </c>
-      <c r="C49" s="22" t="inlineStr">
+      <c r="C50" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: A*256}</t>
         </is>
       </c>
-      <c r="D49" s="22" t="inlineStr">
+      <c r="D50" s="22" t="inlineStr">
         <is>
           <t>A*256</t>
         </is>
       </c>
-      <c r="E49" s="22" t="inlineStr">
+      <c r="E50" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F49" s="22" t="inlineStr">
+      <c r="F50" s="22" t="inlineStr">
         <is>
           <t>204, đã lưu</t>
         </is>
       </c>
-      <c r="G49" s="22" t="inlineStr">
+      <c r="G50" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H49" s="22" t="inlineStr">
+      <c r="H50" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I49" s="22" t="inlineStr">
+      <c r="I50" s="22" t="inlineStr">
         <is>
           <t>Không có giới hạn độ dài họ tên: `_validate_profile` (sign_in.py) chỉ kiểm rỗng; cột users.full_name kiểu text không giới hạn
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="90.5" customHeight="1">
-      <c r="A50" s="22" t="inlineStr">
+    <row r="51" ht="90.5" customHeight="1">
+      <c r="A51" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-32</t>
         </is>
       </c>
-      <c r="B50" s="22" t="inlineStr">
+      <c r="B51" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh trước 1900-01-01</t>
         </is>
       </c>
-      <c r="C50" s="22" t="inlineStr">
+      <c r="C51" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh}</t>
         </is>
       </c>
-      <c r="D50" s="22" t="inlineStr">
+      <c r="D51" s="22" t="inlineStr">
         <is>
           <t>1899-12-31 | 0001-01-01</t>
         </is>
       </c>
-      <c r="E50" s="22" t="inlineStr">
+      <c r="E51" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
         </is>
       </c>
-      <c r="F50" s="22" t="inlineStr">
+      <c r="F51" s="22" t="inlineStr">
         <is>
           <t>204 ở cả hai giá trị, đã lưu</t>
         </is>
       </c>
-      <c r="G50" s="22" t="inlineStr">
+      <c r="G51" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H50" s="22" t="inlineStr">
+      <c r="H51" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I50" s="22" t="inlineStr">
+      <c r="I51" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:229–231) chỉ chặn ngày tương lai, không có cận dưới. App mobile đã giới hạn date picker từ 1900 nên chỉ gặp khi gọi API trực tiếp
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="123.5" customHeight="1">
-      <c r="A51" s="22" t="inlineStr">
+    <row r="52" ht="123.5" customHeight="1">
+      <c r="A52" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-35</t>
         </is>
       </c>
-      <c r="B51" s="22" t="inlineStr">
+      <c r="B52" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
         </is>
       </c>
-      <c r="C51" s="22" t="inlineStr">
+      <c r="C52" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
         </is>
       </c>
-      <c r="D51" s="22" t="inlineStr">
+      <c r="D52" s="22" t="inlineStr">
         <is>
           <t>ngay_sinh: 2026-10-08</t>
         </is>
       </c>
-      <c r="E51" s="22" t="inlineStr">
+      <c r="E52" s="22" t="inlineStr">
         <is>
           <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
         </is>
       </c>
-      <c r="F51" s="22" t="inlineStr">
+      <c r="F52" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_date_of_birth"}</t>
         </is>
       </c>
-      <c r="G51" s="22" t="inlineStr">
+      <c r="G52" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H51" s="22" t="inlineStr">
+      <c r="H52" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I51" s="22" t="inlineStr">
+      <c r="I52" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:230) so với `now.date()` trong khi `now()` (shared/clock.py) trả giờ UTC: từ 00:00 đến 07:00 giờ VN, "hôm nay" bị coi là ngày mai. Vi phạm bất biến 7 (múi giờ cố định Asia/Ho_Chi_Minh)
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="173" customHeight="1">
-      <c r="A52" s="22" t="inlineStr">
+    <row r="53" ht="173" customHeight="1">
+      <c r="A53" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-42</t>
         </is>
       </c>
-      <c r="B52" s="22" t="inlineStr">
+      <c r="B53" s="22" t="inlineStr">
         <is>
           <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
         </is>
       </c>
-      <c r="C52" s="22" t="inlineStr">
+      <c r="C53" s="22" t="inlineStr">
         <is>
           <t>1. Chạm vào ô mã OTP
 2. Theo dõi request backend nhận được</t>
         </is>
       </c>
-      <c r="D52" s="22" t="inlineStr">
+      <c r="D53" s="22" t="inlineStr">
         <is>
           <t>Ô đang chứa 000000</t>
         </is>
       </c>
-      <c r="E52" s="22" t="inlineStr">
+      <c r="E53" s="22" t="inlineStr">
         <is>
           <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
         </is>
       </c>
-      <c r="F52" s="22" t="inlineStr">
+      <c r="F53" s="22" t="inlineStr">
         <is>
           <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
         </is>
       </c>
-      <c r="G52" s="22" t="inlineStr">
+      <c r="G53" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H52" s="22" t="inlineStr">
+      <c r="H53" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I52" s="22" t="inlineStr">
+      <c r="I53" s="22" t="inlineStr">
         <is>
           <t>`OtpPinInput._handleTextChange` (frontend/mobile/lib/features/auth/presentation/widgets/otp_pin_input.dart:66–72) chạy với mọi thông báo của controller, kể cả khi chỉ đổi vị trí con trỏ lúc chạm ô, và gọi onCompleted hễ ô đủ 6 số → gửi lại mã sai, tốn hạn mức token_verifications
 Log: evidence/test-e2e.log (mục "request backend trong pha 2"), evidence/implement-P10-run-phase2-requests.log</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="189.5" customHeight="1">
-      <c r="A53" s="22" t="inlineStr">
+    <row r="54" ht="189.5" customHeight="1">
+      <c r="A54" s="22" t="inlineStr">
         <is>
           <t>BUG-LINKCODE-28</t>
         </is>
       </c>
-      <c r="B53" s="22" t="inlineStr">
+      <c r="B54" s="22" t="inlineStr">
         <is>
           <t>Toàn bộ unit test, architecture test và ruff toàn repo pass</t>
         </is>
       </c>
-      <c r="C53" s="22" t="inlineStr">
+      <c r="C54" s="22" t="inlineStr">
         <is>
           <t>1. pytest tests/unit tests/architecture -q
 2. ruff check .
 3. So với baseline trước khi sửa code</t>
         </is>
       </c>
-      <c r="D53" s="22" t="inlineStr">
+      <c r="D54" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E53" s="22" t="inlineStr">
+      <c r="E54" s="22" t="inlineStr">
         <is>
           <t>pytest và ruff đều pass</t>
         </is>
       </c>
-      <c r="F53" s="22" t="inlineStr">
+      <c r="F54" s="22" t="inlineStr">
         <is>
           <t>697 pass, 1 fail (tests/unit/test_app.py::test_doses_batch_openapi_uses_contract_shape: NameError paths); ruff toàn repo 21 lỗi ở module khác. Fail và lỗi ruff đã có trước khi task sửa code; file của task pass ruff</t>
         </is>
       </c>
-      <c r="G53" s="22" t="inlineStr">
+      <c r="G54" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H53" s="22" t="inlineStr">
+      <c r="H54" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I53" s="22" t="inlineStr">
+      <c r="I54" s="22" t="inlineStr">
         <is>
           <t>Có sẵn trên main, không do task 3.10: test_app.py dòng 43–44 dùng biến paths chưa định nghĩa; ruff báo lỗi ở catalog/*, consent/adapters/outbound/job_queue.py, runtime/job_runner.py (F821 health chưa import, nghi vấn làm Worker lỗi khi ghi heartbeat), worker.py, tests/unit/test_catalog_crud.py
 Log: evidence/implement-final-backend.log</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="239" customHeight="1">
-      <c r="A54" s="22" t="inlineStr">
+    <row r="55" ht="239" customHeight="1">
+      <c r="A55" s="22" t="inlineStr">
         <is>
           <t>BUG-REGDOSE-01</t>
         </is>
       </c>
-      <c r="B54" s="22" t="inlineStr">
+      <c r="B55" s="22" t="inlineStr">
         <is>
           <t>Đối chiếu scheduled_at có giây khi xác nhận liều</t>
         </is>
       </c>
-      <c r="C54" s="22" t="inlineStr">
+      <c r="C55" s="22" t="inlineStr">
         <is>
           <t>1. Từ backend chạy .venv/Scripts/python.exe -m pytest tests/integration/test_dose_confirmation_api.py::test_post_doses_batch_creates_dose_log_for_authenticated_patient__AC1_AC10_AC18 -q -ra.
 2. Fixture POST /doses/batch với danh sách một item ở Test Data.
 3. Đối chiếu items[0].scheduled_at với kỳ vọng test hiện có.</t>
         </is>
       </c>
-      <c r="D54" s="22" t="inlineStr">
+      <c r="D55" s="22" t="inlineStr">
         <is>
           <t>client_uuid: UUID mới; schedule_id: fixture; scheduled_at=2026-10-02T01:00:59.999Z; taken_at=2026-10-02T01:05:59.999Z</t>
         </is>
       </c>
-      <c r="E54" s="22" t="inlineStr">
+      <c r="E55" s="22" t="inlineStr">
         <is>
           <t>Theo test hiện có: HTTP 200, synced, da_uong và scheduled_at=2026-10-02T01:00:00Z.</t>
         </is>
       </c>
-      <c r="F54" s="22" t="inlineStr">
+      <c r="F55" s="22" t="inlineStr">
         <is>
           <t>HTTP 200, synced, da_uong; scheduled_at=2026-10-02T01:00:59.999000Z. Fail trong suite DB và lặp lại khi chạy riêng (1 failed trong 1.67s).</t>
         </is>
       </c>
-      <c r="G54" s="22" t="inlineStr">
+      <c r="G55" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H54" s="22" t="inlineStr">
+      <c r="H55" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I54" s="22" t="inlineStr">
+      <c r="I55" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn kỳ vọng chuẩn hóa tới phút trong test không khớp hành vi giữ thời điểm của API; chưa xác định phía nào sai theo contract/nghiệp vụ. Chưa chứng minh mất/trùng bản ghi liều; mức Medium tạm thời cho sai khác test, phải nâng tối thiểu High nếu xác nhận mất/trùng liều.
 Log: evidence/test-integration-db.log; evidence/test-dose-mismatch-repeat.log</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="123.5" customHeight="1">
-      <c r="A55" s="22" t="inlineStr">
+    <row r="56" ht="123.5" customHeight="1">
+      <c r="A56" s="22" t="inlineStr">
         <is>
           <t>BUG-APIC-04</t>
         </is>
       </c>
-      <c r="B55" s="22" t="inlineStr">
+      <c r="B56" s="22" t="inlineStr">
         <is>
           <t>Kiểm tra profile và condition contract</t>
         </is>
       </c>
-      <c r="C55" s="22" t="inlineStr">
+      <c r="C56" s="22" t="inlineStr">
         <is>
           <t>1. Chạy `pytest tests/unit/test_contract_profile.py -q -p no:cacheprovider`.
 2. Kiểm tra response headers, required/nullability, bearer security và semantics 403/404.</t>
         </is>
       </c>
-      <c r="D55" s="22" t="inlineStr">
+      <c r="D56" s="22" t="inlineStr">
         <is>
           <t>GET/PUT profile; GET/POST/PATCH/DELETE conditions.</t>
         </is>
       </c>
-      <c r="E55" s="22" t="inlineStr">
+      <c r="E56" s="22" t="inlineStr">
         <is>
           <t>Toàn bộ profile parity pass, gồm Cache-Control theo contract.</t>
         </is>
       </c>
-      <c r="F55" s="22" t="inlineStr">
+      <c r="F56" s="22" t="inlineStr">
         <is>
           <t>3 profile operation thất bại do Cache-Control const ở runtime so với enum trong contract; lỗi được giữ lại theo phạm vi đã duyệt.</t>
         </is>
       </c>
-      <c r="G55" s="22" t="inlineStr">
+      <c r="G56" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H55" s="22" t="inlineStr">
+      <c r="H56" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I55" s="22" t="inlineStr">
+      <c r="I56" s="22" t="inlineStr">
         <is>
           <t>Đã xác định mismatch giữa metadata Cache-Control của generated runtime OpenAPI và contract chuẩn.
 Log: evidence/implement-P4-parity.log</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="90.5" customHeight="1">
-      <c r="A56" s="22" t="inlineStr">
+    <row r="57" ht="90.5" customHeight="1">
+      <c r="A57" s="22" t="inlineStr">
         <is>
           <t>BUG-APIC-09</t>
         </is>
       </c>
-      <c r="B56" s="22" t="inlineStr">
+      <c r="B57" s="22" t="inlineStr">
         <is>
           <t>Xem kết quả full unit và phân loại lỗi còn lại</t>
         </is>
       </c>
-      <c r="C56" s="22" t="inlineStr">
+      <c r="C57" s="22" t="inlineStr">
         <is>
           <t>1. Đọc `evidence/implement-final-backend.log`.
 2. Xác nhận số pass/fail và phân loại các lỗi nằm ngoài phạm vi/mismatch đã ghi.</t>
         </is>
       </c>
-      <c r="D56" s="22" t="inlineStr">
+      <c r="D57" s="22" t="inlineStr">
         <is>
           <t>Toàn bộ backend unit và architecture suites.</t>
         </is>
       </c>
-      <c r="E56" s="22" t="inlineStr">
+      <c r="E57" s="22" t="inlineStr">
         <is>
           <t>Không có failure bị che; lỗi nền và mismatch được báo riêng.</t>
         </is>
       </c>
-      <c r="F56" s="22" t="inlineStr">
+      <c r="F57" s="22" t="inlineStr">
         <is>
           <t>815 passed, 9 failed: ba Cache-Control mismatch và sáu lỗi auth trả 422 thay vì 401.</t>
         </is>
       </c>
-      <c r="G56" s="22" t="inlineStr">
+      <c r="G57" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H56" s="22" t="inlineStr">
+      <c r="H57" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I56" s="22" t="inlineStr">
+      <c r="I57" s="22" t="inlineStr">
         <is>
           <t>Ba failure contract-runtime Cache-Control đã xác định; sáu lỗi auth 422 thay vì 401 còn là lỗi hiện có ngoài phạm vi, nguyên nhân gốc chưa xác định trong task này.
 Log: evidence/implement-final-backend.log</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="123.5" customHeight="1">
-      <c r="A57" s="22" t="inlineStr">
+    <row r="58" ht="123.5" customHeight="1">
+      <c r="A58" s="22" t="inlineStr">
         <is>
           <t>BUG-APIC-11</t>
         </is>
       </c>
-      <c r="B57" s="22" t="inlineStr">
+      <c r="B58" s="22" t="inlineStr">
         <is>
           <t>Kiểm tra test admin role revocation cho catalog sync history</t>
         </is>
       </c>
-      <c r="C57" s="22" t="inlineStr">
+      <c r="C58" s="22" t="inlineStr">
         <is>
           <t>1. Chạy test_admin_role_revocation_applies_on_next_request__AC8 trong toàn bộ integration suite.
 2. Gửi GET /admin/catalog/sync-runs với admin session do fixture tạo.</t>
         </is>
       </c>
-      <c r="D57" s="22" t="inlineStr">
+      <c r="D58" s="22" t="inlineStr">
         <is>
           <t>Nguồn sync fixture qd_5948.</t>
         </is>
       </c>
-      <c r="E57" s="22" t="inlineStr">
+      <c r="E58" s="22" t="inlineStr">
         <is>
           <t>Request đầu trả 200 trước khi thu hồi admin role.</t>
         </is>
       </c>
-      <c r="F57" s="22" t="inlineStr">
+      <c r="F58" s="22" t="inlineStr">
         <is>
           <t>Request phát sinh ValueError: qd_5948 is not a valid CatalogSyncSource trước khi assertion status hoàn tất.</t>
         </is>
       </c>
-      <c r="G57" s="22" t="inlineStr">
+      <c r="G58" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H57" s="22" t="inlineStr">
+      <c r="H58" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I57" s="22" t="inlineStr">
+      <c r="I58" s="22" t="inlineStr">
         <is>
           <t>Nguyên nhân gốc chưa xác định; nghi vấn fixture dùng catalog sync source không có trong enum CatalogSyncSource.
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="123.5" customHeight="1">
-      <c r="A58" s="22" t="inlineStr">
+    <row r="59" ht="123.5" customHeight="1">
+      <c r="A59" s="22" t="inlineStr">
         <is>
           <t>BUG-APIC-12</t>
         </is>
       </c>
-      <c r="B58" s="22" t="inlineStr">
+      <c r="B59" s="22" t="inlineStr">
         <is>
           <t>Kiểm tra timestamp của dose batch</t>
         </is>
       </c>
-      <c r="C58" s="22" t="inlineStr">
+      <c r="C59" s="22" t="inlineStr">
         <is>
           <t>1. Chạy test_post_doses_batch_creates_dose_log_for_authenticated_patient__AC1_AC10_AC18.
 2. Gửi dose batch và so timestamp response với scheduled time.</t>
         </is>
       </c>
-      <c r="D58" s="22" t="inlineStr">
+      <c r="D59" s="22" t="inlineStr">
         <is>
           <t>Scheduled time 2026-10-02T01:00:00Z.</t>
         </is>
       </c>
-      <c r="E58" s="22" t="inlineStr">
+      <c r="E59" s="22" t="inlineStr">
         <is>
           <t>Dose log trả đúng scheduled time 2026-10-02T01:00:00Z.</t>
         </is>
       </c>
-      <c r="F58" s="22" t="inlineStr">
+      <c r="F59" s="22" t="inlineStr">
         <is>
           <t>Response trả 2026-10-02T01:00:59.999000Z; assertion không khớp kỳ vọng.</t>
         </is>
       </c>
-      <c r="G58" s="22" t="inlineStr">
+      <c r="G59" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H58" s="22" t="inlineStr">
+      <c r="H59" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I58" s="22" t="inlineStr">
+      <c r="I59" s="22" t="inlineStr">
         <is>
           <t>Nguyên nhân gốc chưa xác định; nghi vấn time-window selection trả cuối cửa sổ một phút thay vì scheduled time.
 Log: evidence/test-integration.log</t>
@@ -4389,17 +5039,17 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:A5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11:F21">
+  <conditionalFormatting sqref="F11:F22">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11:G21">
+  <conditionalFormatting sqref="G11:G22">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>OR(G11="Critical",G11="High")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G46:G58">
+  <conditionalFormatting sqref="G47:G59">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
@@ -4411,10 +5061,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G11:G21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G11:G22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="G46:G58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G47:G59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
test: add test cases spreadsheet for Team1 DTU quality and testing
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android build" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đăng nhập người dùng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lịch uống thuốc" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tải lịch uống" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tương tác thuốc-thuốc" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tương tác thuốc-thực phẩm" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tra cứu hoạt chất" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mã liên kết người thân" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chọn thuốc danh mục" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hồi quy xác nhận liều" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Contract Sync" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profile auth test" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Android build" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Đăng nhập người dùng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Lịch uống thuốc" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tải lịch uống" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Tương tác thuốc-thuốc" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Tương tác thuốc-thực phẩm" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Tra cứu hoạt chất" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Mã liên kết người thân" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Chọn thuốc danh mục" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Hồi quy xác nhận liều" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="API Contract Sync" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Profile auth test" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Xử lý liên kết và consent" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Report" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Android build'!$A$8:$I$17</definedName>
@@ -33,6 +34,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Hồi quy xác nhận liều'!$A$8:$I$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'API Contract Sync'!$A$8:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Profile auth test'!$A$8:$I$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Xử lý liên kết và consent'!$A$8:$I$41</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -335,13 +337,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -365,18 +367,18 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$22</f>
+              <f>'Report'!$A$11:$A$23</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$11:$D$22</f>
+              <f>'Report'!$D$11:$D$23</f>
             </numRef>
           </val>
         </ser>
@@ -389,18 +391,18 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$22</f>
+              <f>'Report'!$A$11:$A$23</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$11:$E$22</f>
+              <f>'Report'!$E$11:$E$23</f>
             </numRef>
           </val>
         </ser>
@@ -413,18 +415,18 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$22</f>
+              <f>'Report'!$A$11:$A$23</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$11:$F$22</f>
+              <f>'Report'!$F$11:$F$23</f>
             </numRef>
           </val>
         </ser>
@@ -470,13 +472,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -494,7 +496,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -522,12 +524,12 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>24</row>
+      <row>25</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -537,9 +539,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -549,7 +551,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>24</row>
+      <row>25</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3240000"/>
@@ -559,9 +561,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -3628,7 +3630,2431 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:V47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="8" customWidth="1" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Xem và xử lý yêu cầu liên kết với consent (LINKCONSENT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Quyết định duyệt yêu cầu liên kết (POST /family/links/{id}/approve)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="107" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Yêu cầu liên kết pending không cấp quyền truy cập dữ liệu y tế</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Bệnh nhân P có pending link gửi từ người thân F, chưa xác nhận consent; P có thuốc trong danh sách</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Người thân F gửi GET /medications/{user_med_id} của bệnh nhân P với token của F</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>user_med_id của patient P, Authorization Bearer của F</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden, detail 'khong_co_quyen'; access_logs ghi nhận 1 dòng denied</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden; detail: khong_co_quyen; 1 access_log denied</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · test_pending_grants_no_access__AC1</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>status (query GET /family/links)</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>(blank)
+active
+rejected
+revoked
+trùng lặp nhiều status
+kèm query lạ patient_id</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>7
+8
+9
+10
+11
+12</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Link tồn tại và trạng thái pending?</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="74" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Bệnh nhân duyệt yêu cầu pending kèm xác nhận consent người thân</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Link trạng thái pending giữa P và F; P có consent family_sharing đang hiệu lực</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Bệnh nhân P gửi POST /family/links/{link_id}/approve kèm family_user_id của F, consent_confirmed=true, document_version='2026-10-v1'</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>family_user_id=F, consent_confirmed=true, document_version='2026-10-v1'</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK, status='active', sharing_enabled=false; DB lưu 1 bản ghi vào family_link_consent_confirmations</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK; status='active'; confirmation được ghi nhận</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · Decision Table 1 (R1) · test_approve_success_persists_evidence_and_activates_link__AC2</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>family_user_id (body POST approve)</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>UUID hợp lệ khớp đúng người thân trong link pending</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>(blank)
+không phải UUID
+UUID người lạ
+UUID chính caller</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>13
+14
+15
+16</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>Caller là patient sở hữu link?</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="74" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối duyệt khi thiếu xác nhận consent_confirmed hoặc sai version</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Link trạng thái pending</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi POST /family/links/{link_id}/approve với consent_confirmed=false hoặc version cũ/lạ</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>consent_confirmed=false hoặc document_version='outdated_v0'</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity; link vẫn pending; không tạo bằng chứng mới</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity; link giữ nguyên pending</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · Decision Table 1 (R2) · test_approve_outdated_version_and_false_confirmation_422__AC3</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>consent_confirmed (body POST approve)</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>false
+null
+1
+chuỗi 'true'</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>17
+18
+19
+20</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>Patient có consent family_sharing hiệu lực?</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T11" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="57.5" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Chặn người khác hoặc admin duyệt hộ yêu cầu liên kết</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Link pending thuộc về bệnh nhân P</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Người thân F, admin hoặc người lạ X gọi POST /family/links/{link_id}/approve</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Token của F/Admin/Stranger</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden, detail 'khong_co_quyen'; ghi audit event denied</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden; audit event denied được ghi</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · Decision Table 1 (R4) · test_approve_denied_caller_matrix__AC4_AC10_AC16</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>document_version (body POST approve)</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-v1 (phiên bản hiện hành)</t>
+        </is>
+      </c>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N12" s="10" t="inlineStr">
+        <is>
+          <t>(blank)
+độ dài 65 ký tự (quá 64)
+phiên bản cũ/lạ</t>
+        </is>
+      </c>
+      <c r="O12" s="10" t="inlineStr">
+        <is>
+          <t>21
+22
+23</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
+        <is>
+          <t>consent_confirmed = true và đúng version?</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S12" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T12" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U12" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V12" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="74" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Gửi lại approve cùng payload trên link đã active (replay idempotent)</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Link đã active với bằng chứng consent hợp lệ</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi lại đúng payload POST /family/links/{link_id}/approve</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Cùng family_user_id, consent_confirmed=true, document_version cũ</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK, trả trạng thái hiện tại; không tạo thêm bản ghi confirmation thứ hai</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK; confirmation giữ nguyên 1 bản ghi</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · AC9 · test_approve_replay_idempotent_with_same_evidence__AC5_AC9</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>link_id (path param)</t>
+        </is>
+      </c>
+      <c r="L13" s="10" t="inlineStr">
+        <is>
+          <t>1
+9223372036854775807</t>
+        </is>
+      </c>
+      <c r="M13" s="10" t="inlineStr">
+        <is>
+          <t>5
+6</t>
+        </is>
+      </c>
+      <c r="N13" s="10" t="inlineStr">
+        <is>
+          <t>0
+-1
+9223372036854775808 (quá int64)
+chuỗi abc</t>
+        </is>
+      </c>
+      <c r="O13" s="10" t="inlineStr">
+        <is>
+          <t>24
+25
+26
+27</t>
+        </is>
+      </c>
+      <c r="Q13" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T13" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U13" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="V13" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="107" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Phân quyền đọc dữ liệu y tế sau khi duyệt và chặn quyền ghi thay</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Link active giữa P và F</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. Khi sharing_enabled=false: F gửi GET /medications/{id}
+2. Khi sharing_enabled=true: F gửi GET /medications/{id}
+3. Khi sharing_enabled=true: F gửi PATCH /medications/{id}</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>user_med_id của P</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Bước 1: 403 denied log; Bước 2: 200 allowed log; Bước 3: 403 denied log</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Bước 1: 403; Bước 2: 200; Bước 3: 403</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · Decision Table 2 · test_approved_link_with_sharing_off_gets_403_and_denied_log__AC6</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>200 OK + active + lưu bằng chứng consent_confirmations</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S14" s="11" t="inlineStr"/>
+      <c r="T14" s="11" t="inlineStr"/>
+      <c r="U14" s="11" t="inlineStr"/>
+      <c r="V14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="90.5" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Rút consent hoặc hủy link có hiệu lực ngay ở request tiếp theo với cùng JWT</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>F đang đọc dữ liệu y tế thành công với JWT token</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. F gửi GET /medications/{id} -&gt; 200
+2. P rút consent family_sharing hoặc revoked link
+3. F gửi lại GET /medications/{id} với cùng token JWT cũ</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Cùng Authorization Bearer token của F</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden; access_logs ghi nhận 1 allowed và 1 denied</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden; log ghi nhận allowed rồi denied</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · test_revocation_takes_effect_immediately_same_jwt__AC7</t>
+        </is>
+      </c>
+      <c r="Q15" s="10" t="inlineStr">
+        <is>
+          <t>422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="R15" s="11" t="inlineStr"/>
+      <c r="S15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T15" s="11" t="inlineStr"/>
+      <c r="U15" s="11" t="inlineStr"/>
+      <c r="V15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16" ht="57.5" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Chặn duyệt trên link đã rejected hoặc revoked</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Link có trạng thái rejected hoặc revoked</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi POST /family/links/{link_id}/approve</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>link_id của link rejected/revoked</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 409 Conflict, detail 'invalid_link_transition'; không đổi trạng thái link</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 409 Conflict; status không đổi</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · Decision Table 1 (R5) · test_approve_rejected_or_revoked_conflict_409__AC8</t>
+        </is>
+      </c>
+      <c r="Q16" s="10" t="inlineStr">
+        <is>
+          <t>403 Forbidden (consent_missing hoặc khong_co_quyen)</t>
+        </is>
+      </c>
+      <c r="R16" s="11" t="inlineStr"/>
+      <c r="S16" s="11" t="inlineStr"/>
+      <c r="T16" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U16" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="V16" s="11" t="inlineStr"/>
+    </row>
+    <row r="17" ht="57.5" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Xử lý tương tranh hai yêu cầu approve đồng thời</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Link pending</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi 2 request approve đồng thời cho cùng 1 link</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>2 thread đồng thời</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Cả hai nhận 200, DB chỉ lưu đúng 1 bản ghi bằng chứng duy nhất</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Cả 2 HTTP 200; đúng 1 bản ghi confirmation</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · AC9 · test_concurrent_approve_same_payload_both_200_single_evidence__AC5_AC9</t>
+        </is>
+      </c>
+      <c r="Q17" s="10" t="inlineStr">
+        <is>
+          <t>409 Conflict hoặc 404 Not Found</t>
+        </is>
+      </c>
+      <c r="R17" s="11" t="inlineStr"/>
+      <c r="S17" s="11" t="inlineStr"/>
+      <c r="T17" s="11" t="inlineStr"/>
+      <c r="U17" s="11" t="inlineStr"/>
+      <c r="V17" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="57.5" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Chặn người thân đọc dữ liệu thuốc của bệnh nhân khác</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>F là người thân của P1; P2 có đơn thuốc riêng</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. F gửi GET /medications/{id_P2}</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>id thuốc của P2, token của F</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden, detail 'khong_co_quyen'; ghi denied access_logs cho P2</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden; ghi denied log cho P2</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · test_family_cannot_read_other_patient_medication__AC6_AC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="90.5" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Bảo toàn dữ liệu link legacy và chặn approve khi thiếu bằng chứng</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Link active legacy được tạo trước migration (không có confirmation)</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. Kiểm tra DB: link legacy vẫn tồn tại, không bị tự động backfill
+2. Gửi POST /family/links/{link_id}/approve trên link legacy
+3. Kiểm tra query Worker sharing_family_ids</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>link_id của link legacy</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Bước 1: không có confirmation; Bước 2: 409 consent_confirmation_missing; Bước 3: loại bỏ khỏi sharing</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Bước 1: không evidence; Bước 2: 409; Bước 3: loại bỏ</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · test_legacy_links_preserved_without_backfill__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="74" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Bệnh nhân xem danh sách yêu cầu liên kết pending của chính mình</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Bệnh nhân có 2 yêu cầu pending, 1 active, 1 rejected, và có yêu cầu của patient khác</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. Bệnh nhân gửi GET /family/links?status=pending</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>query status=pending</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK, trả items chỉ gồm 2 pending của caller, thông tin người gửi tối thiểu (id, name, requested_at); không lộ email, số điện thoại hay mã liên kết</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK; items chỉ chứa pending của caller, không lộ dữ liệu nhạy cảm</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · test_list_own_pending_minimal_order_without_consents__AC12_AC13</t>
+        </is>
+      </c>
+      <c r="Q20" s="4" t="inlineStr">
+        <is>
+          <t>Phân quyền truy cập dữ liệu y tế người thân qua PEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="57.5" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-13</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Xem danh sách pending khi chưa có yêu cầu hoặc chưa có consent</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Bệnh nhân chưa có yêu cầu pending nào hoặc chưa cấp consent family_sharing</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /family/links?status=pending</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>query status=pending</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK, trả items rỗng []</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK; items=[]</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AC13 · test_list_pending_empty_returns_200_items_empty__AC13</t>
+        </is>
+      </c>
+      <c r="Q21" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S21" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T21" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U21" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="V21" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="57.5" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-14</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Bệnh nhân từ chối yêu cầu liên kết pending (POST reject)</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Link trạng thái pending</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. Bệnh nhân gửi POST /family/links/{link_id}/reject</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>link_id của pending link</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK, status='rejected', có rejected_at; không tạo confirmation; yêu cầu biến mất khỏi danh sách pending</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK; status='rejected'; không confirmation; biến mất khỏi GET pending</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AC14 · test_reject_without_consent_and_replay_idempotent__AC14_AC15</t>
+        </is>
+      </c>
+      <c r="Q22" s="10" t="inlineStr">
+        <is>
+          <t>Link trạng thái active?</t>
+        </is>
+      </c>
+      <c r="R22" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S22" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T22" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U22" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V22" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="57.5" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Gửi lại reject trên link đã rejected (idempotent) và chặn reject link active/revoked</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Link đã rejected hoặc active</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi lại reject trên link đã rejected
+2. Gửi reject trên link active hoặc revoked</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>link_id tương ứng</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Bước 1: HTTP 200 OK giữ nguyên rejected_at cũ; Bước 2: HTTP 409 Conflict</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Bước 1: 200 với rejected_at cũ; Bước 2: 409 Conflict</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AC15 · test_reject_active_or_revoked_conflict_409__AC15</t>
+        </is>
+      </c>
+      <c r="Q23" s="10" t="inlineStr">
+        <is>
+          <t>Có bằng chứng consent confirmation đúng cặp?</t>
+        </is>
+      </c>
+      <c r="R23" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S23" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T23" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U23" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V23" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="57.5" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-16</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Chặn người khác hoặc admin từ chối hộ yêu cầu của bệnh nhân</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Link pending của bệnh nhân P</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. Người thân F hoặc admin gửi POST /family/links/{link_id}/reject</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Token của F/Admin</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden, detail 'khong_co_quyen'; ghi audit event denied; link không đổi</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden; audit event denied được ghi</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>AC16 · test_strict_http_inputs_and_forbidden_cases__AC12_AC16</t>
+        </is>
+      </c>
+      <c r="Q24" s="10" t="inlineStr">
+        <is>
+          <t>sharing_enabled = true?</t>
+        </is>
+      </c>
+      <c r="R24" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S24" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T24" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="57.5" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-17</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Xử lý tương tranh giữa approve và reject cho cùng một pending link</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Link pending</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi 1 request approve và 1 request reject đồng thời cho cùng 1 link</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>2 thread đồng thời</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ 1 request nhận 200, request còn lại nhận 409 Conflict; không có trạng thái mâu thuẫn</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>1 request 200, 1 request 409; DB nhất quán</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>AC17 · test_concurrent_approve_and_reject_one_wins_other_409__AC17</t>
+        </is>
+      </c>
+      <c r="Q25" s="10" t="inlineStr">
+        <is>
+          <t>Patient có đủ consent (health_data + family_sharing)?</t>
+        </is>
+      </c>
+      <c r="R25" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S25" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T25" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U25" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V25" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="57.5" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-18</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Xử lý lỗi commit/lưu trữ và cơ chế append-only cho bảng audit/evidence</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>DB gặp sự cố mất kết nối hoặc rollback</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. Giả lập lỗi commit khi duyệt link
+2. Kiểm tra thao tác UPDATE/DELETE/TRUNCATE trên 2 bảng mới với 6 role</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>OperationalError</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Bước 1: HTTP 503 service_unavailable và rollback hoàn toàn; Bước 2: Trigger chặn mọi thao tác sửa/xóa</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Bước 1: 503 service_unavailable; Bước 2: 56 ca kiểm tra trigger/RLS đều pass</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>AC18 · test_storage_commit_failure_returns_503_and_rolls_back__AC18</t>
+        </is>
+      </c>
+      <c r="Q26" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R26" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S26" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T26" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U26" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="V26" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="41" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-BVA-01</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra giá trị biên link_id = 0 (min - 1)</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Hệ thống đang hoạt động</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi POST /family/links/0/approve</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>link_id=0</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>BVA (min-1) · test_path_bounds</t>
+        </is>
+      </c>
+      <c r="Q27" s="10" t="inlineStr">
+        <is>
+          <t>200 OK + access_logs allowed</t>
+        </is>
+      </c>
+      <c r="R27" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S27" s="11" t="inlineStr"/>
+      <c r="T27" s="11" t="inlineStr"/>
+      <c r="U27" s="11" t="inlineStr"/>
+      <c r="V27" s="11" t="inlineStr"/>
+    </row>
+    <row r="28" ht="41" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-BVA-02</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra giá trị biên link_id = 1 (min)</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Không có link id 1 trong DB</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi POST /family/links/1/approve với payload hợp lệ</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>link_id=1</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found (path hợp lệ, vượt qua validation)</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>BVA (min) · test_approve_not_found_404</t>
+        </is>
+      </c>
+      <c r="Q28" s="10" t="inlineStr">
+        <is>
+          <t>403 Forbidden + access_logs denied</t>
+        </is>
+      </c>
+      <c r="R28" s="11" t="inlineStr"/>
+      <c r="S28" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T28" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U28" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="V28" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="41" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-BVA-03</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra giá trị biên link_id = 9223372036854775807 (max int64)</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Không có link id max trong DB</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi POST /family/links/9223372036854775807/approve</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>link_id=9223372036854775807</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found (vượt qua validation int64)</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>BVA (max) · test_path_bounds</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="41" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-BVA-04</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra giá trị biên link_id = 9223372036854775808 (max + 1)</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Hệ thống đang hoạt động</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi POST /family/links/9223372036854775808/approve</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>link_id=9223372036854775808</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity (vượt giới hạn int64)</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>BVA (max+1) · test_path_bounds</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="41" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-BVA-05</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra giá trị biên độ dài document_version = 65 ký tự (max + 1)</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Link pending</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi POST approve với document_version dài 65 ký tự</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>document_version='a'*65</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity (chuỗi dài quá 64 ký tự)</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>BVA (max+1) · test_body_version_bounds</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="41" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-EP-01</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>GET /family/links thiếu query parameter status</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /family/links</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Không query param</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>EP (invalid) · test_missing_query</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="41" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-EP-02</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>GET /family/links với status khác pending</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /family/links?status=active</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>status=active</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>EP (invalid) · test_invalid_status_query</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="41" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-EP-03</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>GET /family/links truyền lặp nhiều tham số status</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /family/links?status=pending&amp;status=pending</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>status lặp</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>EP (invalid) · test_repeated_status_query</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="41" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-EP-04</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>GET /family/links truyền thêm tham số lạ patient_id</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /family/links?status=pending&amp;patient_id=other_uuid</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>patient_id query param</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>EP (invalid) · test_extra_query_forbidden</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="41" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-EP-05</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>POST approve truyền thêm trường không xác định trong body</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Link pending</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi POST approve kèm trường lạ 'extra_field': 'value'</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>extra_field in json</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity (extra_forbidden)</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>EP (invalid) · test_extra_body_fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="41" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-EP-06</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>POST reject có gửi kèm body nội dung</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Link pending</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi POST /family/links/{id}/reject kèm body json {}</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>body = {}</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity (reject không nhận body)</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>EP (invalid) · test_reject_body_forbidden</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="107" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-SEC-01</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Chặn truy cập API khi chưa cung cấp token xác thực</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Chưa đăng nhập</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /family/links?status=pending không Authorization header
+2. POST /family/links/1/approve không Authorization header
+3. POST /family/links/1/reject không Authorization header</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Không token</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized cho cả 3 thao tác</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>Security · test_missing_session_is_401</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="41" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-SEC-02</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Admin bị chặn trước khi tra cứu dữ liệu (QD-32)</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Caller có system_role = 'admin'</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>1. Admin gọi GET/approve/reject</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Token admin</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden; ghi denied audit trước khi chạm DB caregiver_links</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden; denied audit ghi trước lookup</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>Security · test_admin_http_denies_before_lookup_and_audits</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="41" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-SEC-03</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra phân quyền worker_role tối thiểu trên DB</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Role worker_role trên PostgreSQL</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>1. Kiểm tra privilege của worker_role trên 2 bảng mới</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>worker_role</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ có SELECT trên confirmations; không có quyền trên audit_events</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ SELECT confirmations; không có quyền audit_events</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>Security · test_worker_role_privileges_restricted__AC18</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="57.5" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-SEC-04</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Trigger append-only chặn UPDATE/DELETE/TRUNCATE với mọi role</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Hai bảng mới có dữ liệu</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>1. Thực hiện lệnh UPDATE/DELETE/TRUNCATE dưới role postgres, anon, authenticated, service_role, api_role, worker_role</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>6 roles, 3 operations</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>Tất cả đều bị trigger chặn ném lỗi DBAPIError</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>Trigger chặn toàn bộ 18 tổ hợp role × operation</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="inlineStr">
+        <is>
+          <t>Security · test_append_only_triggers_block_all_roles__AC18</t>
+        </is>
+      </c>
+    </row>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44">
+      <c r="G44" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H44" s="13">
+        <f>COUNTIF(H9:H41,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="G45" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H45" s="13">
+        <f>COUNTIF(H9:H41,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="G46" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H46" s="13">
+        <f>COUNTIF(H9:H41,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="G47" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H47" s="13">
+        <f>SUM(H44:H46)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I41"/>
+  <conditionalFormatting sqref="H9:H41">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3682,7 +6108,7 @@
         <v/>
       </c>
       <c r="D3" s="11">
-        <f>'Chọn thuốc danh mục'!$H$40+'Hồi quy xác nhận liều'!$H$12+'API Contract Sync'!$H$23+'Profile auth test'!$H$15</f>
+        <f>'Chọn thuốc danh mục'!$H$40+'Hồi quy xác nhận liều'!$H$12+'API Contract Sync'!$H$23+'Profile auth test'!$H$15+'Xử lý liên kết và consent'!$H$44</f>
         <v/>
       </c>
       <c r="E3" s="15">
@@ -3702,7 +6128,7 @@
         <v/>
       </c>
       <c r="D4" s="11">
-        <f>'Chọn thuốc danh mục'!$H$41+'Hồi quy xác nhận liều'!$H$13+'API Contract Sync'!$H$24+'Profile auth test'!$H$16</f>
+        <f>'Chọn thuốc danh mục'!$H$41+'Hồi quy xác nhận liều'!$H$13+'API Contract Sync'!$H$24+'Profile auth test'!$H$16+'Xử lý liên kết và consent'!$H$45</f>
         <v/>
       </c>
       <c r="E4" s="15">
@@ -3742,7 +6168,7 @@
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>'Chọn thuốc danh mục'!$H$42+'Hồi quy xác nhận liều'!$H$14+'API Contract Sync'!$H$25+'Profile auth test'!$H$17</f>
+        <f>'Chọn thuốc danh mục'!$H$42+'Hồi quy xác nhận liều'!$H$14+'API Contract Sync'!$H$25+'Profile auth test'!$H$17+'Xử lý liên kết và consent'!$H$46</f>
         <v/>
       </c>
       <c r="E6" s="15">
@@ -4345,689 +6771,733 @@
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="19" t="inlineStr">
+    <row r="23" ht="107" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>Xem và xử lý yêu cầu liên kết với consent</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Bệnh nhân xem danh sách yêu cầu chờ (pending), duyệt kèm xác nhận consent người thân, hoặc từ chối yêu cầu liên kết</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Xử lý liên kết và consent</t>
+        </is>
+      </c>
+      <c r="D23" s="18">
+        <f>IFERROR(('Xử lý liên kết và consent'!$H$47-'Xử lý liên kết và consent'!$H$46)/'Xử lý liên kết và consent'!$H$47,0)</f>
+        <v/>
+      </c>
+      <c r="E23" s="18">
+        <f>IFERROR('Xử lý liên kết và consent'!$H$44/'Xử lý liên kết và consent'!$H$47,0)</f>
+        <v/>
+      </c>
+      <c r="F23" s="18">
+        <f>IFERROR('Xử lý liên kết và consent'!$H$45/'Xử lý liên kết và consent'!$H$47,0)</f>
+        <v/>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>86/86 test case tích hợp và 148/148 test unit/architecture đã chạy pass 100%; không phát hiện lỗi sản phẩm mới.</t>
+        </is>
+      </c>
+      <c r="I23" s="11" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="19" t="inlineStr">
         <is>
           <t>Bug Report</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="20" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="20" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="B46" s="20" t="inlineStr">
+      <c r="B47" s="20" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C46" s="20" t="inlineStr">
+      <c r="C47" s="20" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="D46" s="20" t="inlineStr">
+      <c r="D47" s="20" t="inlineStr">
         <is>
           <t>Input Data</t>
         </is>
       </c>
-      <c r="E46" s="20" t="inlineStr">
+      <c r="E47" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F46" s="20" t="inlineStr">
+      <c r="F47" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="G46" s="20" t="inlineStr">
+      <c r="G47" s="20" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="H46" s="20" t="inlineStr">
+      <c r="H47" s="20" t="inlineStr">
         <is>
           <t>Name of Tester</t>
         </is>
       </c>
-      <c r="I46" s="20" t="inlineStr">
+      <c r="I47" s="20" t="inlineStr">
         <is>
           <t>Logs</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="123.5" customHeight="1">
-      <c r="A47" s="22" t="inlineStr">
+    <row r="48" ht="123.5" customHeight="1">
+      <c r="A48" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-08</t>
         </is>
       </c>
-      <c r="B47" s="22" t="inlineStr">
+      <c r="B48" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
         </is>
       </c>
-      <c r="C47" s="22" t="inlineStr">
+      <c r="C48" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
 2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
         </is>
       </c>
-      <c r="D47" s="22" t="inlineStr">
+      <c r="D48" s="22" t="inlineStr">
         <is>
           <t>phone: 0900000001 + ký tự \n</t>
         </is>
       </c>
-      <c r="E47" s="22" t="inlineStr">
+      <c r="E48" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F47" s="22" t="inlineStr">
+      <c r="F48" s="22" t="inlineStr">
         <is>
           <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
         </is>
       </c>
-      <c r="G47" s="22" t="inlineStr">
+      <c r="G48" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H47" s="22" t="inlineStr">
+      <c r="H48" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I47" s="22" t="inlineStr">
+      <c r="I48" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn — kỳ vọng AC6 mâu thuẫn AC5: backend `_validate_required_text` (sign_in.py:178) `strip()` mọi ký tự trắng hai đầu, nên \n cuối được xử lý như khoảng trắng hai đầu mà AC5 coi là hợp lệ. Cần người dùng chốt: sửa AC6 hoặc sửa backend
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="123.5" customHeight="1">
-      <c r="A48" s="22" t="inlineStr">
+    <row r="49" ht="123.5" customHeight="1">
+      <c r="A49" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-11</t>
         </is>
       </c>
-      <c r="B48" s="22" t="inlineStr">
+      <c r="B49" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
         </is>
       </c>
-      <c r="C48" s="22" t="inlineStr">
+      <c r="C49" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone}
 2. POST /auth/mobile/verify {phone, token: 123456}</t>
         </is>
       </c>
-      <c r="D48" s="22" t="inlineStr">
+      <c r="D49" s="22" t="inlineStr">
         <is>
           <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
         </is>
       </c>
-      <c r="E48" s="22" t="inlineStr">
+      <c r="E49" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
         </is>
       </c>
-      <c r="F48" s="22" t="inlineStr">
+      <c r="F49" s="22" t="inlineStr">
         <is>
           <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
         </is>
       </c>
-      <c r="G48" s="22" t="inlineStr">
+      <c r="G49" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H48" s="22" t="inlineStr">
+      <c r="H49" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I48" s="22" t="inlineStr">
+      <c r="I49" s="22" t="inlineStr">
         <is>
           <t>`_normalize_phone` (sign_in.py:197–206) kiểm bằng `str.isdigit()`, nhận cả chữ số Unicode, nên số lọt qua kiểm tra và gửi tới Supabase. Ô nhập của app chỉ cho 0-9 nên người dùng app không gặp; lỗi ở tầng API
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="189.5" customHeight="1">
-      <c r="A49" s="22" t="inlineStr">
+    <row r="50" ht="189.5" customHeight="1">
+      <c r="A50" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-25</t>
         </is>
       </c>
-      <c r="B49" s="22" t="inlineStr">
+      <c r="B50" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên có ký tự NUL</t>
         </is>
       </c>
-      <c r="C49" s="22" t="inlineStr">
+      <c r="C50" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
         </is>
       </c>
-      <c r="D49" s="22" t="inlineStr">
+      <c r="D50" s="22" t="inlineStr">
         <is>
           <t>ho_ten: abc\u0000def</t>
         </is>
       </c>
-      <c r="E49" s="22" t="inlineStr">
+      <c r="E50" s="22" t="inlineStr">
         <is>
           <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
         </is>
       </c>
-      <c r="F49" s="22" t="inlineStr">
+      <c r="F50" s="22" t="inlineStr">
         <is>
           <t>500 Internal Server Error</t>
         </is>
       </c>
-      <c r="G49" s="22" t="inlineStr">
+      <c r="G50" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H49" s="22" t="inlineStr">
+      <c r="H50" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I49" s="22" t="inlineStr">
+      <c r="I50" s="22" t="inlineStr">
         <is>
           <t>`_validate_required_text` (sign_in.py:178) không chặn ký tự điều khiển; PostgreSQL từ chối NUL trong cột text: `psycopg.DataError: PostgreSQL text fields cannot contain NUL (0x00) bytes` ở `UPDATE users SET full_name…` (SqlUsers.update_profile); không có handler cho DataError nên thành 500. Câu SQL có tham số nên không phải lỗ hổng SQL injection
 Log: evidence/test-integration.log, evidence/test-probe-nul.log</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="90.5" customHeight="1">
-      <c r="A50" s="22" t="inlineStr">
+    <row r="51" ht="90.5" customHeight="1">
+      <c r="A51" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-30</t>
         </is>
       </c>
-      <c r="B50" s="22" t="inlineStr">
+      <c r="B51" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên dài 256 ký tự</t>
         </is>
       </c>
-      <c r="C50" s="22" t="inlineStr">
+      <c r="C51" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: A*256}</t>
         </is>
       </c>
-      <c r="D50" s="22" t="inlineStr">
+      <c r="D51" s="22" t="inlineStr">
         <is>
           <t>A*256</t>
         </is>
       </c>
-      <c r="E50" s="22" t="inlineStr">
+      <c r="E51" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F50" s="22" t="inlineStr">
+      <c r="F51" s="22" t="inlineStr">
         <is>
           <t>204, đã lưu</t>
         </is>
       </c>
-      <c r="G50" s="22" t="inlineStr">
+      <c r="G51" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H50" s="22" t="inlineStr">
+      <c r="H51" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I50" s="22" t="inlineStr">
+      <c r="I51" s="22" t="inlineStr">
         <is>
           <t>Không có giới hạn độ dài họ tên: `_validate_profile` (sign_in.py) chỉ kiểm rỗng; cột users.full_name kiểu text không giới hạn
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="90.5" customHeight="1">
-      <c r="A51" s="22" t="inlineStr">
+    <row r="52" ht="90.5" customHeight="1">
+      <c r="A52" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-32</t>
         </is>
       </c>
-      <c r="B51" s="22" t="inlineStr">
+      <c r="B52" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh trước 1900-01-01</t>
         </is>
       </c>
-      <c r="C51" s="22" t="inlineStr">
+      <c r="C52" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh}</t>
         </is>
       </c>
-      <c r="D51" s="22" t="inlineStr">
+      <c r="D52" s="22" t="inlineStr">
         <is>
           <t>1899-12-31 | 0001-01-01</t>
         </is>
       </c>
-      <c r="E51" s="22" t="inlineStr">
+      <c r="E52" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
         </is>
       </c>
-      <c r="F51" s="22" t="inlineStr">
+      <c r="F52" s="22" t="inlineStr">
         <is>
           <t>204 ở cả hai giá trị, đã lưu</t>
         </is>
       </c>
-      <c r="G51" s="22" t="inlineStr">
+      <c r="G52" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H51" s="22" t="inlineStr">
+      <c r="H52" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I51" s="22" t="inlineStr">
+      <c r="I52" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:229–231) chỉ chặn ngày tương lai, không có cận dưới. App mobile đã giới hạn date picker từ 1900 nên chỉ gặp khi gọi API trực tiếp
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="123.5" customHeight="1">
-      <c r="A52" s="22" t="inlineStr">
+    <row r="53" ht="123.5" customHeight="1">
+      <c r="A53" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-35</t>
         </is>
       </c>
-      <c r="B52" s="22" t="inlineStr">
+      <c r="B53" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
         </is>
       </c>
-      <c r="C52" s="22" t="inlineStr">
+      <c r="C53" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
         </is>
       </c>
-      <c r="D52" s="22" t="inlineStr">
+      <c r="D53" s="22" t="inlineStr">
         <is>
           <t>ngay_sinh: 2026-10-08</t>
         </is>
       </c>
-      <c r="E52" s="22" t="inlineStr">
+      <c r="E53" s="22" t="inlineStr">
         <is>
           <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
         </is>
       </c>
-      <c r="F52" s="22" t="inlineStr">
+      <c r="F53" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_date_of_birth"}</t>
         </is>
       </c>
-      <c r="G52" s="22" t="inlineStr">
+      <c r="G53" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H52" s="22" t="inlineStr">
+      <c r="H53" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I52" s="22" t="inlineStr">
+      <c r="I53" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:230) so với `now.date()` trong khi `now()` (shared/clock.py) trả giờ UTC: từ 00:00 đến 07:00 giờ VN, "hôm nay" bị coi là ngày mai. Vi phạm bất biến 7 (múi giờ cố định Asia/Ho_Chi_Minh)
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="173" customHeight="1">
-      <c r="A53" s="22" t="inlineStr">
+    <row r="54" ht="173" customHeight="1">
+      <c r="A54" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-42</t>
         </is>
       </c>
-      <c r="B53" s="22" t="inlineStr">
+      <c r="B54" s="22" t="inlineStr">
         <is>
           <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
         </is>
       </c>
-      <c r="C53" s="22" t="inlineStr">
+      <c r="C54" s="22" t="inlineStr">
         <is>
           <t>1. Chạm vào ô mã OTP
 2. Theo dõi request backend nhận được</t>
         </is>
       </c>
-      <c r="D53" s="22" t="inlineStr">
+      <c r="D54" s="22" t="inlineStr">
         <is>
           <t>Ô đang chứa 000000</t>
         </is>
       </c>
-      <c r="E53" s="22" t="inlineStr">
+      <c r="E54" s="22" t="inlineStr">
         <is>
           <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
         </is>
       </c>
-      <c r="F53" s="22" t="inlineStr">
+      <c r="F54" s="22" t="inlineStr">
         <is>
           <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
         </is>
       </c>
-      <c r="G53" s="22" t="inlineStr">
+      <c r="G54" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H53" s="22" t="inlineStr">
+      <c r="H54" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I53" s="22" t="inlineStr">
+      <c r="I54" s="22" t="inlineStr">
         <is>
           <t>`OtpPinInput._handleTextChange` (frontend/mobile/lib/features/auth/presentation/widgets/otp_pin_input.dart:66–72) chạy với mọi thông báo của controller, kể cả khi chỉ đổi vị trí con trỏ lúc chạm ô, và gọi onCompleted hễ ô đủ 6 số → gửi lại mã sai, tốn hạn mức token_verifications
 Log: evidence/test-e2e.log (mục "request backend trong pha 2"), evidence/implement-P10-run-phase2-requests.log</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="189.5" customHeight="1">
-      <c r="A54" s="22" t="inlineStr">
+    <row r="55" ht="189.5" customHeight="1">
+      <c r="A55" s="22" t="inlineStr">
         <is>
           <t>BUG-LINKCODE-28</t>
         </is>
       </c>
-      <c r="B54" s="22" t="inlineStr">
+      <c r="B55" s="22" t="inlineStr">
         <is>
           <t>Toàn bộ unit test, architecture test và ruff toàn repo pass</t>
         </is>
       </c>
-      <c r="C54" s="22" t="inlineStr">
+      <c r="C55" s="22" t="inlineStr">
         <is>
           <t>1. pytest tests/unit tests/architecture -q
 2. ruff check .
 3. So với baseline trước khi sửa code</t>
         </is>
       </c>
-      <c r="D54" s="22" t="inlineStr">
+      <c r="D55" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E54" s="22" t="inlineStr">
+      <c r="E55" s="22" t="inlineStr">
         <is>
           <t>pytest và ruff đều pass</t>
         </is>
       </c>
-      <c r="F54" s="22" t="inlineStr">
+      <c r="F55" s="22" t="inlineStr">
         <is>
           <t>697 pass, 1 fail (tests/unit/test_app.py::test_doses_batch_openapi_uses_contract_shape: NameError paths); ruff toàn repo 21 lỗi ở module khác. Fail và lỗi ruff đã có trước khi task sửa code; file của task pass ruff</t>
         </is>
       </c>
-      <c r="G54" s="22" t="inlineStr">
+      <c r="G55" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H54" s="22" t="inlineStr">
+      <c r="H55" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I54" s="22" t="inlineStr">
+      <c r="I55" s="22" t="inlineStr">
         <is>
           <t>Có sẵn trên main, không do task 3.10: test_app.py dòng 43–44 dùng biến paths chưa định nghĩa; ruff báo lỗi ở catalog/*, consent/adapters/outbound/job_queue.py, runtime/job_runner.py (F821 health chưa import, nghi vấn làm Worker lỗi khi ghi heartbeat), worker.py, tests/unit/test_catalog_crud.py
 Log: evidence/implement-final-backend.log</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="239" customHeight="1">
-      <c r="A55" s="22" t="inlineStr">
+    <row r="56" ht="239" customHeight="1">
+      <c r="A56" s="22" t="inlineStr">
         <is>
           <t>BUG-REGDOSE-01</t>
         </is>
       </c>
-      <c r="B55" s="22" t="inlineStr">
+      <c r="B56" s="22" t="inlineStr">
         <is>
           <t>Đối chiếu scheduled_at có giây khi xác nhận liều</t>
         </is>
       </c>
-      <c r="C55" s="22" t="inlineStr">
+      <c r="C56" s="22" t="inlineStr">
         <is>
           <t>1. Từ backend chạy .venv/Scripts/python.exe -m pytest tests/integration/test_dose_confirmation_api.py::test_post_doses_batch_creates_dose_log_for_authenticated_patient__AC1_AC10_AC18 -q -ra.
 2. Fixture POST /doses/batch với danh sách một item ở Test Data.
 3. Đối chiếu items[0].scheduled_at với kỳ vọng test hiện có.</t>
         </is>
       </c>
-      <c r="D55" s="22" t="inlineStr">
+      <c r="D56" s="22" t="inlineStr">
         <is>
           <t>client_uuid: UUID mới; schedule_id: fixture; scheduled_at=2026-10-02T01:00:59.999Z; taken_at=2026-10-02T01:05:59.999Z</t>
         </is>
       </c>
-      <c r="E55" s="22" t="inlineStr">
+      <c r="E56" s="22" t="inlineStr">
         <is>
           <t>Theo test hiện có: HTTP 200, synced, da_uong và scheduled_at=2026-10-02T01:00:00Z.</t>
         </is>
       </c>
-      <c r="F55" s="22" t="inlineStr">
+      <c r="F56" s="22" t="inlineStr">
         <is>
           <t>HTTP 200, synced, da_uong; scheduled_at=2026-10-02T01:00:59.999000Z. Fail trong suite DB và lặp lại khi chạy riêng (1 failed trong 1.67s).</t>
         </is>
       </c>
-      <c r="G55" s="22" t="inlineStr">
+      <c r="G56" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H55" s="22" t="inlineStr">
+      <c r="H56" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I55" s="22" t="inlineStr">
+      <c r="I56" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn kỳ vọng chuẩn hóa tới phút trong test không khớp hành vi giữ thời điểm của API; chưa xác định phía nào sai theo contract/nghiệp vụ. Chưa chứng minh mất/trùng bản ghi liều; mức Medium tạm thời cho sai khác test, phải nâng tối thiểu High nếu xác nhận mất/trùng liều.
 Log: evidence/test-integration-db.log; evidence/test-dose-mismatch-repeat.log</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="123.5" customHeight="1">
-      <c r="A56" s="22" t="inlineStr">
+    <row r="57" ht="123.5" customHeight="1">
+      <c r="A57" s="22" t="inlineStr">
         <is>
           <t>BUG-APIC-04</t>
         </is>
       </c>
-      <c r="B56" s="22" t="inlineStr">
+      <c r="B57" s="22" t="inlineStr">
         <is>
           <t>Kiểm tra profile và condition contract</t>
         </is>
       </c>
-      <c r="C56" s="22" t="inlineStr">
+      <c r="C57" s="22" t="inlineStr">
         <is>
           <t>1. Chạy `pytest tests/unit/test_contract_profile.py -q -p no:cacheprovider`.
 2. Kiểm tra response headers, required/nullability, bearer security và semantics 403/404.</t>
         </is>
       </c>
-      <c r="D56" s="22" t="inlineStr">
+      <c r="D57" s="22" t="inlineStr">
         <is>
           <t>GET/PUT profile; GET/POST/PATCH/DELETE conditions.</t>
         </is>
       </c>
-      <c r="E56" s="22" t="inlineStr">
+      <c r="E57" s="22" t="inlineStr">
         <is>
           <t>Toàn bộ profile parity pass, gồm Cache-Control theo contract.</t>
         </is>
       </c>
-      <c r="F56" s="22" t="inlineStr">
+      <c r="F57" s="22" t="inlineStr">
         <is>
           <t>3 profile operation thất bại do Cache-Control const ở runtime so với enum trong contract; lỗi được giữ lại theo phạm vi đã duyệt.</t>
         </is>
       </c>
-      <c r="G56" s="22" t="inlineStr">
+      <c r="G57" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H56" s="22" t="inlineStr">
+      <c r="H57" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I56" s="22" t="inlineStr">
+      <c r="I57" s="22" t="inlineStr">
         <is>
           <t>Đã xác định mismatch giữa metadata Cache-Control của generated runtime OpenAPI và contract chuẩn.
 Log: evidence/implement-P4-parity.log</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="90.5" customHeight="1">
-      <c r="A57" s="22" t="inlineStr">
+    <row r="58" ht="90.5" customHeight="1">
+      <c r="A58" s="22" t="inlineStr">
         <is>
           <t>BUG-APIC-09</t>
         </is>
       </c>
-      <c r="B57" s="22" t="inlineStr">
+      <c r="B58" s="22" t="inlineStr">
         <is>
           <t>Xem kết quả full unit và phân loại lỗi còn lại</t>
         </is>
       </c>
-      <c r="C57" s="22" t="inlineStr">
+      <c r="C58" s="22" t="inlineStr">
         <is>
           <t>1. Đọc `evidence/implement-final-backend.log`.
 2. Xác nhận số pass/fail và phân loại các lỗi nằm ngoài phạm vi/mismatch đã ghi.</t>
         </is>
       </c>
-      <c r="D57" s="22" t="inlineStr">
+      <c r="D58" s="22" t="inlineStr">
         <is>
           <t>Toàn bộ backend unit và architecture suites.</t>
         </is>
       </c>
-      <c r="E57" s="22" t="inlineStr">
+      <c r="E58" s="22" t="inlineStr">
         <is>
           <t>Không có failure bị che; lỗi nền và mismatch được báo riêng.</t>
         </is>
       </c>
-      <c r="F57" s="22" t="inlineStr">
+      <c r="F58" s="22" t="inlineStr">
         <is>
           <t>815 passed, 9 failed: ba Cache-Control mismatch và sáu lỗi auth trả 422 thay vì 401.</t>
         </is>
       </c>
-      <c r="G57" s="22" t="inlineStr">
+      <c r="G58" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H57" s="22" t="inlineStr">
+      <c r="H58" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I57" s="22" t="inlineStr">
+      <c r="I58" s="22" t="inlineStr">
         <is>
           <t>Ba failure contract-runtime Cache-Control đã xác định; sáu lỗi auth 422 thay vì 401 còn là lỗi hiện có ngoài phạm vi, nguyên nhân gốc chưa xác định trong task này.
 Log: evidence/implement-final-backend.log</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="123.5" customHeight="1">
-      <c r="A58" s="22" t="inlineStr">
+    <row r="59" ht="123.5" customHeight="1">
+      <c r="A59" s="22" t="inlineStr">
         <is>
           <t>BUG-APIC-11</t>
         </is>
       </c>
-      <c r="B58" s="22" t="inlineStr">
+      <c r="B59" s="22" t="inlineStr">
         <is>
           <t>Kiểm tra test admin role revocation cho catalog sync history</t>
         </is>
       </c>
-      <c r="C58" s="22" t="inlineStr">
+      <c r="C59" s="22" t="inlineStr">
         <is>
           <t>1. Chạy test_admin_role_revocation_applies_on_next_request__AC8 trong toàn bộ integration suite.
 2. Gửi GET /admin/catalog/sync-runs với admin session do fixture tạo.</t>
         </is>
       </c>
-      <c r="D58" s="22" t="inlineStr">
+      <c r="D59" s="22" t="inlineStr">
         <is>
           <t>Nguồn sync fixture qd_5948.</t>
         </is>
       </c>
-      <c r="E58" s="22" t="inlineStr">
+      <c r="E59" s="22" t="inlineStr">
         <is>
           <t>Request đầu trả 200 trước khi thu hồi admin role.</t>
         </is>
       </c>
-      <c r="F58" s="22" t="inlineStr">
+      <c r="F59" s="22" t="inlineStr">
         <is>
           <t>Request phát sinh ValueError: qd_5948 is not a valid CatalogSyncSource trước khi assertion status hoàn tất.</t>
         </is>
       </c>
-      <c r="G58" s="22" t="inlineStr">
+      <c r="G59" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H58" s="22" t="inlineStr">
+      <c r="H59" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I58" s="22" t="inlineStr">
+      <c r="I59" s="22" t="inlineStr">
         <is>
           <t>Nguyên nhân gốc chưa xác định; nghi vấn fixture dùng catalog sync source không có trong enum CatalogSyncSource.
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="123.5" customHeight="1">
-      <c r="A59" s="22" t="inlineStr">
+    <row r="60" ht="123.5" customHeight="1">
+      <c r="A60" s="22" t="inlineStr">
         <is>
           <t>BUG-APIC-12</t>
         </is>
       </c>
-      <c r="B59" s="22" t="inlineStr">
+      <c r="B60" s="22" t="inlineStr">
         <is>
           <t>Kiểm tra timestamp của dose batch</t>
         </is>
       </c>
-      <c r="C59" s="22" t="inlineStr">
+      <c r="C60" s="22" t="inlineStr">
         <is>
           <t>1. Chạy test_post_doses_batch_creates_dose_log_for_authenticated_patient__AC1_AC10_AC18.
 2. Gửi dose batch và so timestamp response với scheduled time.</t>
         </is>
       </c>
-      <c r="D59" s="22" t="inlineStr">
+      <c r="D60" s="22" t="inlineStr">
         <is>
           <t>Scheduled time 2026-10-02T01:00:00Z.</t>
         </is>
       </c>
-      <c r="E59" s="22" t="inlineStr">
+      <c r="E60" s="22" t="inlineStr">
         <is>
           <t>Dose log trả đúng scheduled time 2026-10-02T01:00:00Z.</t>
         </is>
       </c>
-      <c r="F59" s="22" t="inlineStr">
+      <c r="F60" s="22" t="inlineStr">
         <is>
           <t>Response trả 2026-10-02T01:00:59.999000Z; assertion không khớp kỳ vọng.</t>
         </is>
       </c>
-      <c r="G59" s="22" t="inlineStr">
+      <c r="G60" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H59" s="22" t="inlineStr">
+      <c r="H60" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I59" s="22" t="inlineStr">
+      <c r="I60" s="22" t="inlineStr">
         <is>
           <t>Nguyên nhân gốc chưa xác định; nghi vấn time-window selection trả cuối cửa sổ một phút thay vì scheduled time.
 Log: evidence/test-integration.log</t>
@@ -5039,17 +7509,17 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:A5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11:F22">
+  <conditionalFormatting sqref="F11:F23">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11:G22">
+  <conditionalFormatting sqref="G11:G23">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>OR(G11="Critical",G11="High")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G47:G59">
+  <conditionalFormatting sqref="G48:G60">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
@@ -5061,10 +7531,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G11:G22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G11:G23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="G47:G59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G48:G60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
test: add consent linking test cases
Refs: 3.16
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -34,7 +34,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Hồi quy xác nhận liều'!$A$8:$I$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'API Contract Sync'!$A$8:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Profile auth test'!$A$8:$I$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Xử lý liên kết và consent'!$A$8:$I$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Xử lý liên kết và consent'!$A$8:$I$46</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -3630,7 +3630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V47"/>
+  <dimension ref="A1:V52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5986,61 +5986,297 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44">
-      <c r="G44" s="12" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="H44" s="13">
-        <f>COUNTIF(H9:H41,"Pass")</f>
+    <row r="42" ht="57.5" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-19</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra denied audit writer lỗi và vẫn fail-closed</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Audit writer family_link_audit_events gặp lỗi khi request cần ghi denied</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>1. Giả lập audit writer lỗi
+2. Gửi request bị từ chối
+3. Kiểm tra response và DB</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Lỗi DB khi ghi denied audit</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>Request thất bại; không trả thành công; trạng thái nghiệp vụ không đổi</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>Request lỗi 500; link vẫn pending; không phát sinh audit allowed/denied</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I42" s="8" t="inlineStr">
+        <is>
+          <t>AC18 · test_denied_audit_writer_failure_fails_closed__AC18</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="57.5" customHeight="1">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-20</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra policy SELECT thực tế dưới anon và authenticated</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Hai bảng evidence và audit đã có dữ liệu thử</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập lần lượt bằng anon và authenticated
+2. Thử SELECT hai bảng mới</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Role anon, authenticated</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>Client không đọc được dữ liệu và không có policy client</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>SELECT bị PostgreSQL từ chối cho anon/authenticated trên cả hai bảng</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="inlineStr">
+        <is>
+          <t>AC18 · test_client_roles_cannot_select_link_metadata__AC18</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="57.5" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-21</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra thứ tự approve khóa consent trước khi rút consent</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Có thể điều khiển hai transaction để kiểm tra khóa consent</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>1. Cho approve giữ SHARE lock
+2. Chạy transaction rút consent
+3. Kiểm tra request y tế sau khi rút</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Hai transaction PostgreSQL đồng thời</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>Sau khi rút consent commit, request y tế kế tiếp trả 403</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="inlineStr"/>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I44" s="8" t="inlineStr">
+        <is>
+          <t>AC7, AC17 · I12; Pending được người dùng chấp nhận, chưa chạy</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="57.5" customHeight="1">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-22</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra lỗi Access Log Writer không trả dữ liệu y tế</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Request PEP hợp lệ nhưng Access Log Writer lỗi</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>1. Giả lập Access Log Writer lỗi
+2. Gửi request đọc dữ liệu y tế
+3. Kiểm tra response</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Lỗi khi ghi access_logs</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>Request thất bại và không trả dữ liệu y tế</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 500; response không chứa medication; test Access Log Writer lỗi đã pass</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I45" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · test_allowed_log_failure_fails_request</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="74" customHeight="1">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKCONSENT-23</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra migration nâng cấp trên dữ liệu legacy có sẵn</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>DB cách ly có caregiver_links legacy trước khi áp migration mới</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>1. Chụp snapshot các link legacy
+2. Áp migration mới
+3. So sánh trạng thái và evidence</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>DB cách ly trước migration</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>Dữ liệu legacy được giữ nguyên và không tự backfill confirmation</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="inlineStr"/>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I46" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · I9; Pending được người dùng chấp nhận, chưa chạy; test hiện tại xác nhận fixture legacy sau migration không backfill</t>
+        </is>
+      </c>
+    </row>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49">
+      <c r="G49" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H49" s="13">
+        <f>COUNTIF(H9:H46,"Pass")</f>
         <v/>
       </c>
     </row>
-    <row r="45">
-      <c r="G45" s="12" t="inlineStr">
+    <row r="50">
+      <c r="G50" s="12" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="H45" s="13">
-        <f>COUNTIF(H9:H41,"Fail")</f>
+      <c r="H50" s="13">
+        <f>COUNTIF(H9:H46,"Fail")</f>
         <v/>
       </c>
     </row>
-    <row r="46">
-      <c r="G46" s="12" t="inlineStr">
+    <row r="51">
+      <c r="G51" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="H46" s="13">
-        <f>COUNTIF(H9:H41,"Pending")</f>
+      <c r="H51" s="13">
+        <f>COUNTIF(H9:H46,"Pending")</f>
         <v/>
       </c>
     </row>
-    <row r="47">
-      <c r="G47" s="12" t="inlineStr">
+    <row r="52">
+      <c r="G52" s="12" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="H47" s="13">
-        <f>SUM(H44:H46)</f>
+      <c r="H52" s="13">
+        <f>SUM(H49:H51)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A8:I41"/>
-  <conditionalFormatting sqref="H9:H41">
+  <autoFilter ref="A8:I46"/>
+  <conditionalFormatting sqref="H9:H46">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Fail"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H9:H41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H9:H46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pass,Fail,Pending"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6108,7 +6344,7 @@
         <v/>
       </c>
       <c r="D3" s="11">
-        <f>'Chọn thuốc danh mục'!$H$40+'Hồi quy xác nhận liều'!$H$12+'API Contract Sync'!$H$23+'Profile auth test'!$H$15+'Xử lý liên kết và consent'!$H$44</f>
+        <f>'Chọn thuốc danh mục'!$H$40+'Hồi quy xác nhận liều'!$H$12+'API Contract Sync'!$H$23+'Profile auth test'!$H$15+'Xử lý liên kết và consent'!$H$49</f>
         <v/>
       </c>
       <c r="E3" s="15">
@@ -6128,7 +6364,7 @@
         <v/>
       </c>
       <c r="D4" s="11">
-        <f>'Chọn thuốc danh mục'!$H$41+'Hồi quy xác nhận liều'!$H$13+'API Contract Sync'!$H$24+'Profile auth test'!$H$16+'Xử lý liên kết và consent'!$H$45</f>
+        <f>'Chọn thuốc danh mục'!$H$41+'Hồi quy xác nhận liều'!$H$13+'API Contract Sync'!$H$24+'Profile auth test'!$H$16+'Xử lý liên kết và consent'!$H$50</f>
         <v/>
       </c>
       <c r="E4" s="15">
@@ -6168,7 +6404,7 @@
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>'Chọn thuốc danh mục'!$H$42+'Hồi quy xác nhận liều'!$H$14+'API Contract Sync'!$H$25+'Profile auth test'!$H$17+'Xử lý liên kết và consent'!$H$46</f>
+        <f>'Chọn thuốc danh mục'!$H$42+'Hồi quy xác nhận liều'!$H$14+'API Contract Sync'!$H$25+'Profile auth test'!$H$17+'Xử lý liên kết và consent'!$H$51</f>
         <v/>
       </c>
       <c r="E6" s="15">
@@ -6788,15 +7024,15 @@
         </is>
       </c>
       <c r="D23" s="18">
-        <f>IFERROR(('Xử lý liên kết và consent'!$H$47-'Xử lý liên kết và consent'!$H$46)/'Xử lý liên kết và consent'!$H$47,0)</f>
+        <f>IFERROR(('Xử lý liên kết và consent'!$H$52-'Xử lý liên kết và consent'!$H$51)/'Xử lý liên kết và consent'!$H$52,0)</f>
         <v/>
       </c>
       <c r="E23" s="18">
-        <f>IFERROR('Xử lý liên kết và consent'!$H$44/'Xử lý liên kết và consent'!$H$47,0)</f>
+        <f>IFERROR('Xử lý liên kết và consent'!$H$49/'Xử lý liên kết và consent'!$H$52,0)</f>
         <v/>
       </c>
       <c r="F23" s="18">
-        <f>IFERROR('Xử lý liên kết và consent'!$H$45/'Xử lý liên kết và consent'!$H$47,0)</f>
+        <f>IFERROR('Xử lý liên kết và consent'!$H$50/'Xử lý liên kết và consent'!$H$52,0)</f>
         <v/>
       </c>
       <c r="G23" s="11" t="inlineStr">
@@ -6806,7 +7042,7 @@
       </c>
       <c r="H23" s="10" t="inlineStr">
         <is>
-          <t>86/86 test case tích hợp và 148/148 test unit/architecture đã chạy pass 100%; không phát hiện lỗi sản phẩm mới.</t>
+          <t>36 Pass, 0 Fail, 2 Pending; người dùng chấp nhận giữ Pending. 105 integration tests task và regression PEP pass; các ca Pending chưa được chạy và không được tính Pass.</t>
         </is>
       </c>
       <c r="I23" s="11" t="inlineStr">

</xml_diff>

<commit_message>
docs(testing): add landing page test cases (LANDING)
Add the "Landing page" sheet to Test_Cases.xlsx: 32 test cases covering
AC1-AC16 of the landing redesign, all Pass.

Refs: adhoc-20261016-update-landing-ui

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -14,7 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tương tác thuốc-thực phẩm" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tra cứu hoạt chất" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mã liên kết người thân" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Landing page" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Android build'!$A$8:$I$17</definedName>
@@ -25,6 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Tương tác thuốc-thực phẩm'!$A$8:$I$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Tra cứu hoạt chất'!$A$8:$I$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Mã liên kết người thân'!$A$8:$I$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Landing page'!$A$8:$I$40</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -363,12 +365,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$18</f>
+              <f>'Report'!$A$11:$A$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$11:$D$18</f>
+              <f>'Report'!$D$11:$D$19</f>
             </numRef>
           </val>
         </ser>
@@ -387,12 +389,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$18</f>
+              <f>'Report'!$A$11:$A$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$11:$E$18</f>
+              <f>'Report'!$E$11:$E$19</f>
             </numRef>
           </val>
         </ser>
@@ -411,12 +413,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$18</f>
+              <f>'Report'!$A$11:$A$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$11:$F$18</f>
+              <f>'Report'!$F$11:$F$19</f>
             </numRef>
           </val>
         </ser>
@@ -519,7 +521,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>20</row>
+      <row>21</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -541,7 +543,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>20</row>
+      <row>21</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3240000"/>
@@ -1691,6 +1693,1054 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>TEST REPORT</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Executed</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="C3" s="11">
+        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59+'Lịch uống thuốc'!$H$51+'Tải lịch uống'!$H$32+'Tương tác thuốc-thuốc'!$H$52+'Tương tác thuốc-thực phẩm'!$H$17+'Tra cứu hoạt chất'!$H$17+'Mã liên kết người thân'!$H$44+'Landing page'!$H$43</f>
+        <v/>
+      </c>
+      <c r="D3" s="15">
+        <f>SUM(C3:C3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="n"/>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="C4" s="11">
+        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60+'Lịch uống thuốc'!$H$52+'Tải lịch uống'!$H$33+'Tương tác thuốc-thuốc'!$H$53+'Tương tác thuốc-thực phẩm'!$H$18+'Tra cứu hoạt chất'!$H$18+'Mã liên kết người thân'!$H$45+'Landing page'!$H$44</f>
+        <v/>
+      </c>
+      <c r="D4" s="15">
+        <f>SUM(C4:C4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="n"/>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>(Total) Test executed (Passed + Failed)</t>
+        </is>
+      </c>
+      <c r="C5" s="11">
+        <f>C3+C4</f>
+        <v/>
+      </c>
+      <c r="D5" s="15">
+        <f>SUM(C5:C5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr"/>
+      <c r="C6" s="11">
+        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61+'Lịch uống thuốc'!$H$53+'Tải lịch uống'!$H$34+'Tương tác thuốc-thuốc'!$H$54+'Tương tác thuốc-thực phẩm'!$H$19+'Tra cứu hoạt chất'!$H$19+'Mã liên kết người thân'!$H$46+'Landing page'!$H$45</f>
+        <v/>
+      </c>
+      <c r="D6" s="15">
+        <f>SUM(C6:C6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>(Sub-total) Test Planned</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr"/>
+      <c r="C7" s="11">
+        <f>C5+C6</f>
+        <v/>
+      </c>
+      <c r="D7" s="15">
+        <f>SUM(C7:C7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Function</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Sheet Name</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>% TCs Executed</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>% TCs Passed</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>% TCs Failed</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Done by</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="156.5" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Build ứng dụng Android</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Build APK debug của Mobile App từ nhánh main (cấu hình Gradle, desugaring, plugin native) và bước build trong CI</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Android build</t>
+        </is>
+      </c>
+      <c r="D11" s="18">
+        <f>IFERROR(('Android build'!$H$23-'Android build'!$H$22)/'Android build'!$H$23,0)</f>
+        <v/>
+      </c>
+      <c r="E11" s="18">
+        <f>IFERROR('Android build'!$H$20/'Android build'!$H$23,0)</f>
+        <v/>
+      </c>
+      <c r="F11" s="18">
+        <f>IFERROR('Android build'!$H$21/'Android build'!$H$23,0)</f>
+        <v/>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Lỗi Critical (APK không build được do flutter_local_notifications cần desugaring và flutter_timezone 2.x dùng API Registrar đã bị gỡ) đã sửa ở task adhoc-20261007-android-desugaring (frontend PR #27, CI xanh gồm bước build APK). Còn Pending: kiểm lockfile bằng --enforce-lockfile với Flutter stable.</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="189.5" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Đăng nhập người dùng</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Đăng nhập Mobile App bằng OTP (số điện thoại hoặc email), hoàn thiện hồ sơ lần đầu, phiên đăng nhập và đăng xuất — user thường, không gồm admin</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Đăng nhập người dùng</t>
+        </is>
+      </c>
+      <c r="D12" s="18">
+        <f>IFERROR(('Đăng nhập người dùng'!$H$62-'Đăng nhập người dùng'!$H$61)/'Đăng nhập người dùng'!$H$62,0)</f>
+        <v/>
+      </c>
+      <c r="E12" s="18">
+        <f>IFERROR('Đăng nhập người dùng'!$H$59/'Đăng nhập người dùng'!$H$62,0)</f>
+        <v/>
+      </c>
+      <c r="F12" s="18">
+        <f>IFERROR('Đăng nhập người dùng'!$H$60/'Đăng nhập người dùng'!$H$62,0)</f>
+        <v/>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Luồng chính (đăng nhập, hồ sơ, consent, mở lại app, đăng xuất) và mọi kiểm tra quyền/bearer đạt, cả ở API lẫn E2E trên emulator. 7 Fail gồm lỗi kiểm tra đầu vào ở biên (chữ số Unicode, họ tên &gt; 255, ngày sinh &lt; 1900, ký tự NUL gây 500), lỗi múi giờ khi kiểm ngày sinh (dùng UTC), app gửi lại mã OTP sai khi chạm ô, và một kỳ vọng AC6 cần chốt lại (ký tự xuống dòng cuối số điện thoại).</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="222.5" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Quản lý lịch uống thuốc</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Backend API thêm, sửa, hủy từng giờ uống; bật/tắt nhắc; đổi ngày uống trong tuần; mốc hiệu lực khi có liều xác nhận sớm (QD-16). Chỉ chính người bệnh được ghi.</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Lịch uống thuốc</t>
+        </is>
+      </c>
+      <c r="D13" s="18">
+        <f>IFERROR(('Lịch uống thuốc'!$H$54-'Lịch uống thuốc'!$H$53)/'Lịch uống thuốc'!$H$54,0)</f>
+        <v/>
+      </c>
+      <c r="E13" s="18">
+        <f>IFERROR('Lịch uống thuốc'!$H$51/'Lịch uống thuốc'!$H$54,0)</f>
+        <v/>
+      </c>
+      <c r="F13" s="18">
+        <f>IFERROR('Lịch uống thuốc'!$H$52/'Lịch uống thuốc'!$H$54,0)</f>
+        <v/>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động và kiểm tra biên đạt trên Supabase local. Đã sửa và có test cho các lỗi review R1 (sinh trùng liều khi ngừng/dùng lại sau liều xác nhận sớm), R2 (dùng lại thuốc khi cần mở lịch cũ), R3 (dùng lại mất lịch sau khi đổi cả bộ giờ/ngày sau liều sớm; sửa bằng migration closed_by_stop_at) và M3 (doses_per_day sau khi dùng lại). Có test bất biến trên chuỗi thao tác ngẫu nhiên. Chưa phủ: race giữa xác nhận liều sớm và sửa lịch (2.10).</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="90.5" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Tải lịch uống và phân quyền dữ liệu thuốc</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>GET /patients/{patient_id}/schedules (lịch đang mở và đóng trong 30 ngày, phân trang con trỏ); phân quyền ghi lịch; QD-32 admin không đọc dữ liệu y tế; patient_id không tồn tại.</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Tải lịch uống</t>
+        </is>
+      </c>
+      <c r="D14" s="18">
+        <f>IFERROR(('Tải lịch uống'!$H$35-'Tải lịch uống'!$H$34)/'Tải lịch uống'!$H$35,0)</f>
+        <v/>
+      </c>
+      <c r="E14" s="18">
+        <f>IFERROR('Tải lịch uống'!$H$32/'Tải lịch uống'!$H$35,0)</f>
+        <v/>
+      </c>
+      <c r="F14" s="18">
+        <f>IFERROR('Tải lịch uống'!$H$33/'Tải lịch uống'!$H$35,0)</f>
+        <v/>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ ca phân quyền đạt, mỗi ca kiểm cả response lẫn access_logs. Quy tắc QD-29 (app người thân không lưu xuống máy) là quy tắc client, chưa kiểm được ở backend.</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="90.5" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Danh mục tương tác thuốc-thuốc (admin)</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Admin thêm, xem, sửa (tạo phiên bản mới), xóa mềm quy tắc tương tác giữa hai hoạt chất, kèm ngưỡng liều; xem lịch sử phiên bản (task 2.16, PB05).</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Tương tác thuốc-thuốc</t>
+        </is>
+      </c>
+      <c r="D15" s="18">
+        <f>IFERROR(('Tương tác thuốc-thuốc'!$H$55-'Tương tác thuốc-thuốc'!$H$54)/'Tương tác thuốc-thuốc'!$H$55,0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="18">
+        <f>IFERROR('Tương tác thuốc-thuốc'!$H$52/'Tương tác thuốc-thuốc'!$H$55,0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="18">
+        <f>IFERROR('Tương tác thuốc-thuốc'!$H$53/'Tương tác thuốc-thuốc'!$H$55,0)</f>
+        <v/>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động (tích hợp với Postgres thật, app chạy bằng api_role) pass. Không có lỗi sản phẩm.</t>
+        </is>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="107" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Danh mục tương tác thuốc-thực phẩm (admin)</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Admin thêm, xem, sửa (tạo phiên bản mới), xóa mềm quy tắc tương tác giữa hoạt chất và thực phẩm (task 2.16, PB05).</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Tương tác thuốc-thực phẩm</t>
+        </is>
+      </c>
+      <c r="D16" s="18">
+        <f>IFERROR(('Tương tác thuốc-thực phẩm'!$H$20-'Tương tác thuốc-thực phẩm'!$H$19)/'Tương tác thuốc-thực phẩm'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="18">
+        <f>IFERROR('Tương tác thuốc-thực phẩm'!$H$17/'Tương tác thuốc-thực phẩm'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="F16" s="18">
+        <f>IFERROR('Tương tác thuốc-thực phẩm'!$H$18/'Tương tác thuốc-thực phẩm'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động pass. Không có lỗi sản phẩm.</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90.5" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Tra cứu hoạt chất (admin)</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Admin tìm hoạt chất theo tên chuẩn hoặc tên gọi khác, hoặc xem hoạt chất của một thuốc, để chọn khi nhập quy tắc tương tác (task 2.16).</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Tra cứu hoạt chất</t>
+        </is>
+      </c>
+      <c r="D17" s="18">
+        <f>IFERROR(('Tra cứu hoạt chất'!$H$20-'Tra cứu hoạt chất'!$H$19)/'Tra cứu hoạt chất'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="E17" s="18">
+        <f>IFERROR('Tra cứu hoạt chất'!$H$17/'Tra cứu hoạt chất'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="F17" s="18">
+        <f>IFERROR('Tra cứu hoạt chất'!$H$18/'Tra cứu hoạt chất'!$H$20,0)</f>
+        <v/>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động pass.</t>
+        </is>
+      </c>
+      <c r="I17" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="156.5" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Mã liên kết người thân</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>User lấy mã liên kết cố định, không hết hạn của mình (kèm QR payload) để mời người thân: GET /family/link-code; mỗi user đúng một mã (QD-04, QD-34). Task 3.10, PB15.</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Mã liên kết người thân</t>
+        </is>
+      </c>
+      <c r="D18" s="18">
+        <f>IFERROR(('Mã liên kết người thân'!$H$47-'Mã liên kết người thân'!$H$46)/'Mã liên kết người thân'!$H$47,0)</f>
+        <v/>
+      </c>
+      <c r="E18" s="18">
+        <f>IFERROR('Mã liên kết người thân'!$H$44/'Mã liên kết người thân'!$H$47,0)</f>
+        <v/>
+      </c>
+      <c r="F18" s="18">
+        <f>IFERROR('Mã liên kết người thân'!$H$45/'Mã liên kết người thân'!$H$47,0)</f>
+        <v/>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động của chức năng (tích hợp với Postgres thật, app chạy bằng api_role; unit; contract) pass, kể cả sau bản sửa F1 của review (mã kiểu cũ sai định dạng bị xóa khi migrate, DB có CHECK định dạng). Một Fail: bộ unit test toàn repo và ruff toàn repo còn lỗi có sẵn trên main ở module khác, không do task này.</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="123.5" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Landing page (giao diện mới, iPhone 3D)</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Trang chủ landing: hero iPhone 3D (Spline) + vòng icon tính năng, dải bằng chứng, scroll-story 4 tính năng, 5 thẻ tiện ích, 3 bước, an toàn, FAQ, CTA, footer; hiệu ứng GSAP</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Landing page</t>
+        </is>
+      </c>
+      <c r="D19" s="18">
+        <f>IFERROR(('Landing page'!$H$46-'Landing page'!$H$45)/'Landing page'!$H$46,0)</f>
+        <v/>
+      </c>
+      <c r="E19" s="18">
+        <f>IFERROR('Landing page'!$H$43/'Landing page'!$H$46,0)</f>
+        <v/>
+      </c>
+      <c r="F19" s="18">
+        <f>IFERROR('Landing page'!$H$44/'Landing page'!$H$46,0)</f>
+        <v/>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>32/32 Pass ở vòng test 2 (2026-10-17). Vòng 1 có 5 Fail (bàn phím / trình đọc màn hình không tới nội dung chưa cuộn tới — High; Performance mobile 77; tương phản nút mock; nhãn nút store; câu chữ icon người nhà), đã sửa ở implement P22 và chạy lại.</t>
+        </is>
+      </c>
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>Bug Report</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>Bug ID</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C43" s="20" t="inlineStr">
+        <is>
+          <t>Steps to Reproduce</t>
+        </is>
+      </c>
+      <c r="D43" s="20" t="inlineStr">
+        <is>
+          <t>Input Data</t>
+        </is>
+      </c>
+      <c r="E43" s="20" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="F43" s="20" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="G43" s="20" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="H43" s="20" t="inlineStr">
+        <is>
+          <t>Name of Tester</t>
+        </is>
+      </c>
+      <c r="I43" s="20" t="inlineStr">
+        <is>
+          <t>Logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="123.5" customHeight="1">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-08</t>
+        </is>
+      </c>
+      <c r="B44" s="22" t="inlineStr">
+        <is>
+          <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
+        </is>
+      </c>
+      <c r="C44" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
+2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
+        </is>
+      </c>
+      <c r="D44" s="22" t="inlineStr">
+        <is>
+          <t>phone: 0900000001 + ký tự \n</t>
+        </is>
+      </c>
+      <c r="E44" s="22" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
+        </is>
+      </c>
+      <c r="F44" s="22" t="inlineStr">
+        <is>
+          <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
+        </is>
+      </c>
+      <c r="G44" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H44" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I44" s="22" t="inlineStr">
+        <is>
+          <t>Nghi vấn — kỳ vọng AC6 mâu thuẫn AC5: backend `_validate_required_text` (sign_in.py:178) `strip()` mọi ký tự trắng hai đầu, nên \n cuối được xử lý như khoảng trắng hai đầu mà AC5 coi là hợp lệ. Cần người dùng chốt: sửa AC6 hoặc sửa backend
+Log: evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="123.5" customHeight="1">
+      <c r="A45" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-11</t>
+        </is>
+      </c>
+      <c r="B45" s="22" t="inlineStr">
+        <is>
+          <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
+        </is>
+      </c>
+      <c r="C45" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/mobile/otp {phone}
+2. POST /auth/mobile/verify {phone, token: 123456}</t>
+        </is>
+      </c>
+      <c r="D45" s="22" t="inlineStr">
+        <is>
+          <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
+        </is>
+      </c>
+      <c r="E45" s="22" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
+        </is>
+      </c>
+      <c r="F45" s="22" t="inlineStr">
+        <is>
+          <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
+        </is>
+      </c>
+      <c r="G45" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H45" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I45" s="22" t="inlineStr">
+        <is>
+          <t>`_normalize_phone` (sign_in.py:197–206) kiểm bằng `str.isdigit()`, nhận cả chữ số Unicode, nên số lọt qua kiểm tra và gửi tới Supabase. Ô nhập của app chỉ cho 0-9 nên người dùng app không gặp; lỗi ở tầng API
+Log: evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="189.5" customHeight="1">
+      <c r="A46" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-25</t>
+        </is>
+      </c>
+      <c r="B46" s="22" t="inlineStr">
+        <is>
+          <t>Lưu họ tên có ký tự NUL</t>
+        </is>
+      </c>
+      <c r="C46" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
+        </is>
+      </c>
+      <c r="D46" s="22" t="inlineStr">
+        <is>
+          <t>ho_ten: abc\u0000def</t>
+        </is>
+      </c>
+      <c r="E46" s="22" t="inlineStr">
+        <is>
+          <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
+        </is>
+      </c>
+      <c r="F46" s="22" t="inlineStr">
+        <is>
+          <t>500 Internal Server Error</t>
+        </is>
+      </c>
+      <c r="G46" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H46" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I46" s="22" t="inlineStr">
+        <is>
+          <t>`_validate_required_text` (sign_in.py:178) không chặn ký tự điều khiển; PostgreSQL từ chối NUL trong cột text: `psycopg.DataError: PostgreSQL text fields cannot contain NUL (0x00) bytes` ở `UPDATE users SET full_name…` (SqlUsers.update_profile); không có handler cho DataError nên thành 500. Câu SQL có tham số nên không phải lỗ hổng SQL injection
+Log: evidence/test-integration.log, evidence/test-probe-nul.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="90.5" customHeight="1">
+      <c r="A47" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-30</t>
+        </is>
+      </c>
+      <c r="B47" s="22" t="inlineStr">
+        <is>
+          <t>Lưu họ tên dài 256 ký tự</t>
+        </is>
+      </c>
+      <c r="C47" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ho_ten: A*256}</t>
+        </is>
+      </c>
+      <c r="D47" s="22" t="inlineStr">
+        <is>
+          <t>A*256</t>
+        </is>
+      </c>
+      <c r="E47" s="22" t="inlineStr">
+        <is>
+          <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
+        </is>
+      </c>
+      <c r="F47" s="22" t="inlineStr">
+        <is>
+          <t>204, đã lưu</t>
+        </is>
+      </c>
+      <c r="G47" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H47" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I47" s="22" t="inlineStr">
+        <is>
+          <t>Không có giới hạn độ dài họ tên: `_validate_profile` (sign_in.py) chỉ kiểm rỗng; cột users.full_name kiểu text không giới hạn
+Log: evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="90.5" customHeight="1">
+      <c r="A48" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-32</t>
+        </is>
+      </c>
+      <c r="B48" s="22" t="inlineStr">
+        <is>
+          <t>Lưu ngày sinh trước 1900-01-01</t>
+        </is>
+      </c>
+      <c r="C48" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ngay_sinh}</t>
+        </is>
+      </c>
+      <c r="D48" s="22" t="inlineStr">
+        <is>
+          <t>1899-12-31 | 0001-01-01</t>
+        </is>
+      </c>
+      <c r="E48" s="22" t="inlineStr">
+        <is>
+          <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
+        </is>
+      </c>
+      <c r="F48" s="22" t="inlineStr">
+        <is>
+          <t>204 ở cả hai giá trị, đã lưu</t>
+        </is>
+      </c>
+      <c r="G48" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H48" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I48" s="22" t="inlineStr">
+        <is>
+          <t>`_validate_birth_date` (sign_in.py:229–231) chỉ chặn ngày tương lai, không có cận dưới. App mobile đã giới hạn date picker từ 1900 nên chỉ gặp khi gọi API trực tiếp
+Log: evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="123.5" customHeight="1">
+      <c r="A49" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-35</t>
+        </is>
+      </c>
+      <c r="B49" s="22" t="inlineStr">
+        <is>
+          <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
+        </is>
+      </c>
+      <c r="C49" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
+        </is>
+      </c>
+      <c r="D49" s="22" t="inlineStr">
+        <is>
+          <t>ngay_sinh: 2026-10-08</t>
+        </is>
+      </c>
+      <c r="E49" s="22" t="inlineStr">
+        <is>
+          <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
+        </is>
+      </c>
+      <c r="F49" s="22" t="inlineStr">
+        <is>
+          <t>422 {"detail":"invalid_date_of_birth"}</t>
+        </is>
+      </c>
+      <c r="G49" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H49" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I49" s="22" t="inlineStr">
+        <is>
+          <t>`_validate_birth_date` (sign_in.py:230) so với `now.date()` trong khi `now()` (shared/clock.py) trả giờ UTC: từ 00:00 đến 07:00 giờ VN, "hôm nay" bị coi là ngày mai. Vi phạm bất biến 7 (múi giờ cố định Asia/Ho_Chi_Minh)
+Log: evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="173" customHeight="1">
+      <c r="A50" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LOGIN-42</t>
+        </is>
+      </c>
+      <c r="B50" s="22" t="inlineStr">
+        <is>
+          <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
+        </is>
+      </c>
+      <c r="C50" s="22" t="inlineStr">
+        <is>
+          <t>1. Chạm vào ô mã OTP
+2. Theo dõi request backend nhận được</t>
+        </is>
+      </c>
+      <c r="D50" s="22" t="inlineStr">
+        <is>
+          <t>Ô đang chứa 000000</t>
+        </is>
+      </c>
+      <c r="E50" s="22" t="inlineStr">
+        <is>
+          <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
+        </is>
+      </c>
+      <c r="F50" s="22" t="inlineStr">
+        <is>
+          <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
+        </is>
+      </c>
+      <c r="G50" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H50" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I50" s="22" t="inlineStr">
+        <is>
+          <t>`OtpPinInput._handleTextChange` (frontend/mobile/lib/features/auth/presentation/widgets/otp_pin_input.dart:66–72) chạy với mọi thông báo của controller, kể cả khi chỉ đổi vị trí con trỏ lúc chạm ô, và gọi onCompleted hễ ô đủ 6 số → gửi lại mã sai, tốn hạn mức token_verifications
+Log: evidence/test-e2e.log (mục "request backend trong pha 2"), evidence/implement-P10-run-phase2-requests.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="189.5" customHeight="1">
+      <c r="A51" s="22" t="inlineStr">
+        <is>
+          <t>BUG-LINKCODE-28</t>
+        </is>
+      </c>
+      <c r="B51" s="22" t="inlineStr">
+        <is>
+          <t>Toàn bộ unit test, architecture test và ruff toàn repo pass</t>
+        </is>
+      </c>
+      <c r="C51" s="22" t="inlineStr">
+        <is>
+          <t>1. pytest tests/unit tests/architecture -q
+2. ruff check .
+3. So với baseline trước khi sửa code</t>
+        </is>
+      </c>
+      <c r="D51" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E51" s="22" t="inlineStr">
+        <is>
+          <t>pytest và ruff đều pass</t>
+        </is>
+      </c>
+      <c r="F51" s="22" t="inlineStr">
+        <is>
+          <t>697 pass, 1 fail (tests/unit/test_app.py::test_doses_batch_openapi_uses_contract_shape: NameError paths); ruff toàn repo 21 lỗi ở module khác. Fail và lỗi ruff đã có trước khi task sửa code; file của task pass ruff</t>
+        </is>
+      </c>
+      <c r="G51" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H51" s="22" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+      <c r="I51" s="22" t="inlineStr">
+        <is>
+          <t>Có sẵn trên main, không do task 3.10: test_app.py dòng 43–44 dùng biến paths chưa định nghĩa; ruff báo lỗi ở catalog/*, consent/adapters/outbound/job_queue.py, runtime/job_runner.py (F821 health chưa import, nghi vấn làm Worker lỗi khi ghi heartbeat), worker.py, tests/unit/test_catalog_crud.py
+Log: evidence/implement-final-backend.log</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:A5"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F11:F19">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G11:G19">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>OR(G11="Critical",G11="High")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G44:G51">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
+      <formula>"Critical"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2">
+      <formula>"High"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="3">
+      <formula>"Medium"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="G11:G19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Critical,High,Medium,Low"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G44:G51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Critical,High,Medium,Low"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -14703,1000 +15753,2027 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:U46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
-        <is>
-          <t>TEST REPORT</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="C2" s="15" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Landing page (giao diện mới, iPhone 3D) (LANDING)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="D2" s="15" t="inlineStr">
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46312</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Có tải iPhone 3D (shouldLoad3D)?</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="107" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Tải iPhone 3D trên desktop sau khi nội dung chính hiển thị</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Bản build production chạy ở http://localhost:3100; trình duyệt 1440×900, prefers-reduced-motion: no-preference</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở /
+2. Đợi hero xong (phone3d--ready)
+3. Đọc thời điểm LCP và thời điểm request đầu tiên tới spline.design</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Viewport 1440×900</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Request Spline bắt đầu sau LCP; phần tử LCP là ảnh tĩnh, không phải canvas</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>LCP 1208 ms (IMG ảnh điện thoại), request Spline đầu tiên 1278 ms, trạng thái phone3d--ready</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · EP (1,4,9) · Decision Table (R1) · acceptance.mjs · evidence/test-acceptance-gpu.log</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>Độ rộng màn hình</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>≥ 1024 px (desktop: tải iPhone 3D, pin scroll-story)
+768–1023 px (tablet: ảnh tĩnh, thẻ xếp dọc)
+&lt; 768 px (mobile: ảnh tĩnh, hàng icon dưới điện thoại)</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1
+2
+3</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr"/>
+      <c r="O9" s="10" t="inlineStr"/>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Rộng ≥ 1024 px?</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="57.5" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm không nhảy layout khi scene 3D crossfade lên ảnh tĩnh</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Như TC-LANDING-01</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở /
+2. Đợi scene sẵn sàng + 4 s
+3. Đọc tổng layout-shift (CLS)</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Viewport 1440×900</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>CLS &lt; 0.1</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>CLS = 0</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · acceptance.mjs · evidence/test-acceptance-gpu.log</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>prefers-reduced-motion</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>no-preference (đủ hiệu ứng)
+reduce (không animation, nội dung ở trạng thái cuối)</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>4
+5</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr"/>
+      <c r="O10" s="10" t="inlineStr"/>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>prefers-reduced-motion: reduce?</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="74" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Mở trang trên mobile 375 px</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Bản build production chạy</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Đặt viewport 375×812
+2. Mở /
+3. Đếm request tới spline.design, kiểm cuộn ngang</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Viewport 375×812</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Hero hiện ảnh tĩnh (phone3d--idle), 0 request spline.design, không có thanh cuộn ngang</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>phone3d--idle, spline requests: 0, overflowX: false</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · EP (3) · Decision Table (R2) · probe.mjs · evidence/test-probes.log</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>Thiết bị trỏ</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>Chuột (hover: hover, pointer: fine)
+Cảm ứng (hover: none)
+Bàn phím</t>
+        </is>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>6
+7
+8</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr"/>
+      <c r="O11" s="10" t="inlineStr"/>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>Data saver bật?</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="74" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm biên độ rộng 1023 / 1024 px cho việc tải 3D</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Bộ unit test landing</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy npm test trong frontend/landing
+2. Xem các ca shouldLoad3D: biên 1023/1024, reduced motion, data saver</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>width = 1023 / 1024; reducedMotion = true; saveData = true</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>1023 → không tải; 1024 → tải; reduce → không tải; data saver → không tải</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>18/18 test pass, gồm các ca biên 1023/1024, reduced motion, data saver</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC1, AC2, AC3 · BVA (max, max+1) · Decision Table (R2, R3, R4) · capabilities.test.ts · evidence/test-static.log</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>Tài nguyên Spline</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>Tải được</t>
+        </is>
+      </c>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="N12" s="10" t="inlineStr">
+        <is>
+          <t>Bị chặn / lỗi mạng
+Quá 12 s chưa sẵn sàng</t>
+        </is>
+      </c>
+      <c r="O12" s="10" t="inlineStr">
+        <is>
+          <t>10
+11</t>
+        </is>
+      </c>
+      <c r="Q12" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="57.5" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Mở trang trên tablet 768 px</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Bản build production chạy</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Đặt viewport 768×1024
+2. Mở /
+3. Đếm request spline.design, kiểm cuộn ngang</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Viewport 768×1024</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Ảnh tĩnh, 0 request spline.design, không cuộn ngang, scroll-story không pin</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>phone3d--idle, spline requests: 0, overflowX: false, story không is-pinned</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · EP (2) · probe.mjs · evidence/test-probes.log</t>
+        </is>
+      </c>
+      <c r="Q13" s="10" t="inlineStr">
+        <is>
+          <t>Tải Spline sau LCP, crossfade lên ảnh tĩnh</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S13" s="11" t="inlineStr"/>
+      <c r="T13" s="11" t="inlineStr"/>
+      <c r="U13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="74" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Duyệt trang khi bật giảm chuyển động</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>prefers-reduced-motion: reduce</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở / ở 1440×900
+2. Chụp toàn trang
+3. Đếm phần tử data-reveal còn ẩn, kiểm pin và Spline</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>prefers-reduced-motion: reduce</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Không pin / scrub / tải 3D; mọi nội dung hiện ở trạng thái cuối</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>hiddenReveals 0/23, story không pin, phone3d--idle, 0 request Spline</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · EP (5) · Decision Table (R3) · probe.mjs · evidence/test-probes.log</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>Giữ ảnh tĩnh, không request spline.design</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr"/>
+      <c r="S14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="41" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Đếm số từ hiển thị trong main của trang chủ</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Bản build production; mốc 911 từ (giai đoạn plan)</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy count_words.py trên .next/server/app/index.html</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Ngưỡng ≤ 774 từ (giảm ≥ 15%)</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>≤ 774 từ</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>750 từ (giảm 17,7%)</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · BVA (max) · evidence/test-static.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="74" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Cuộn qua section tính năng trên desktop</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>1440×900, no-preference</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. Cuộn tới #tinh-nang
+2. Cuộn tiếp từng bước qua toàn bộ đoạn pin
+3. Ghi chương đang hiện và chấm tiến độ ở mỗi bước</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>13 điểm cuộn đều trên đoạn pin</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Section được ghim; chương hiện lần lượt 1→4, chấm tiến độ khớp</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>chapters [0,1,2,3], dots [0,1,2,3], pinned true</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · acceptance.mjs · evidence/test-acceptance-gpu.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="57.5" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm giới hạn chữ của 4 chương tính năng</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Trang chủ đã tải</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Đếm từ tiêu đề và mô tả từng chương</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Tiêu đề ≤ 6 từ, mô tả ≤ 20 từ</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Mọi chương trong giới hạn</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Tiêu đề 6/5/5/5 từ, mô tả 12/15/15/16 từ</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · BVA (max) · acceptance.mjs · evidence/test-acceptance-gpu.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="123.5" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm nội dung bắt buộc vẫn có trên trang</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Trang chủ đã tải</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. Kiểm khối 'Lưu ý y khoa bắt buộc', link tel:115
+2. Kiểm câu FAQ 'DrugTime có thay bác sĩ không?' trả lời 'Không.'
+3. Kiểm 'Dược thư Quốc gia', '5948/QĐ-BYT', 4 FAQ, 2 nút store ở CTA, 3 link pháp lý, 5 anchor</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>#tinh-nang, #cach-hoat-dong, #an-toan, #hoi-dap, #tai-app</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Đủ tất cả mục</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Đủ: medicalNote, tel115, notReplaceDoctor, duocThu, qd5948, faqCount 4, storeButtons 2, 3 link pháp lý, 5 anchor</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · acceptance.mjs · evidence/test-acceptance-gpu.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="57.5" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Bấm link navbar từ trang con /terms</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở /terms</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm 'Cách hoạt động' trên navbar
+2. Lặp lại với 'An toàn'; và 'Hỏi đáp' từ /</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>/terms → /#cach-hoat-dong, /terms → /#an-toan, / → /#hoi-dap</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Chuyển về trang chủ, section nằm ngay dưới navbar</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>URL đúng hash, section top = 96 px ở cả 3 lần</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · acceptance.mjs · evidence/test-acceptance-gpu.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="57.5" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Chấm Lighthouse Accessibility desktop và mobile</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Bản build production; Lighthouse 12; --force-prefers-no-reduced-motion</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy lighthouse mobile (mặc định)
+2. Chạy lighthouse --preset=desktop</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Ngưỡng ≥ 95</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Accessibility ≥ 95 ở cả hai</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Mobile 100 (5 lần), desktop 100</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · evidence/test-lighthouse-summary.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="156.5" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-13</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Dùng Tab đi qua toàn bộ phần tử tương tác của trang chủ</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>1440×900, no-preference, chưa cuộn trang</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhấn Tab 40 lần từ đầu trang
+2. Ghi phần tử nhận focus
+3. Kiểm cây truy cập trước khi cuộn</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Bàn phím</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Tab tới được mọi nút / link, gồm 5 thẻ tiện ích, 4 câu FAQ và link 'Cấp cứu 115'; nội dung có trong cây truy cập</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Tab lần lượt qua 5 thẻ tiện ích (17–21), link Cấp cứu 115 (22), thẻ liên hệ, 4 câu FAQ (24–27); 0 lần focus vào iframe/canvas. Trước khi cuộn: các khối có visibility: visible, opacity 0; cây truy cập có "Cấp cứu 115", "Lưu ý y khoa bắt buộc", câu FAQ 1. Focus link 115 → khối lưu ý opacity 0 → 1 (1440 và 390 px). Vòng 1 Fail (BUG-LANDING-13), đã sửa ở implement P22.</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · Đoán lỗi (bàn phím, trình đọc màn hình) · taborder.mjs, hidden-a11y.mjs, focus-reveal.mjs · evidence/test-taborder.log, evidence/test-hidden-a11y.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="74" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-14</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tương phản chữ trên trang</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Lighthouse accessibility</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. Đọc audit color-contrast</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Ngưỡng 4.5:1</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Không phần tử nào dưới 4.5:1</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Lighthouse không còn audit color-contrast lỗi (mobile 5 lần, desktop); nút mock dùng --color-safe-strong. Vòng 1 Fail 3,29:1 (BUG-LANDING-14), đã sửa.</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · evidence/test-lighthouse-summary.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="74" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tên truy cập của nút tải app khớp chữ hiển thị</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Lighthouse accessibility</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. Đọc audit label-content-name-mismatch</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>4 nút App Store / Google Play (hero + CTA)</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Tên truy cập chứa chữ hiển thị</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Lighthouse không còn audit label-content-name-mismatch; nút store không có aria-label, tên truy cập = chữ hiển thị. Vòng 1 Fail (BUG-LANDING-15), đã sửa.</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · WCAG 2.5.3 · evidence/test-lighthouse-summary.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="57.5" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-16</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm canvas / iframe của Spline không nhận focus</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>1440×900, scene 3D đã sẵn sàng</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhấn Tab 40 lần
+2. Đếm lần focus rơi vào IFRAME hoặc CANVAS, đếm phần tử không có outline</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Bàn phím</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>0 lần focus vào iframe/canvas; phần tử được focus có outline ≥ 2 px</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>iframe/canvas focused: 0; chỉ 1/40 không outline (BODY khi Tab vòng hết trang)</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · taborder.mjs · evidence/test-taborder.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="90.5" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-17</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Chấm Lighthouse Performance mobile</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Bản build production; Lighthouse 12 mobile (giả lập 4G chậm, CPU chậm)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy lighthouse mobile 5 lần
+2. Lấy trung vị điểm Performance</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Ngưỡng ≥ 85</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Performance ≥ 85</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>86 / 71 / 92 / 93 / 91, trung vị 91; LCP ≈ 3,0–3,5 s; lần 71 có TBT 917 ms (dao động máy). Vòng 1 Fail trung vị 77 (BUG-LANDING-17), đã sửa: GSAP nạp động, favicon 10 KB.</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · evidence/test-lighthouse-summary.log, evidence/test-lighthouse-mobile-run*.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="41" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-18</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm CLS và phần tử LCP trên mobile</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Lighthouse mobile</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. Đọc CLS và largest-contentful-paint-element</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>CLS &lt; 0.1</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>CLS &lt; 0.1; LCP không phải canvas 3D</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>CLS 0.005; LCP = img trong .iphone__screen (5 lần chạy mobile)</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · evidence/test-lighthouse-details.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="74" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-19</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Chạy lint, typecheck, unit test và build</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>frontend/landing, nhánh zannguyen/feat-update_frontend_landingpage</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. npm run lint
+2. npm run typecheck
+3. npm test
+4. npm run build (sau khi xóa .next)</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Cả 4 lệnh exit 0</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>lint 0, typecheck 0, vitest 18/18, build sạch 0</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · evidence/test-static.log, evidence/test-build.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="41" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-20</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Quét key / token / secret trong mã nguồn landing</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Mã nguồn landing</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. grep api key, secret, password, bearer, supabase, token= trong app/, components/, lib/</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Không có kết quả</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>no matches</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · evidence/test-static.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="57.5" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-21</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Mở trang khi request tới Spline bị chặn</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>1440×900; chặn mọi URL chứa spline.design</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở /
+2. Đợi 6 s
+3. Kiểm trạng thái hero và layout</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Network request blocking</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Ảnh tĩnh vẫn hiện, không lỗi trắng, section khác hoạt động</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>phone3d--failed, ảnh tĩnh giữ nguyên, story vẫn pin, overflowX false; console chỉ có cảnh báo của trang</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · EP (10) · probe.mjs · evidence/test-probes.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="74" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-22</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Rà màu dùng trong CSS</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Mã nguồn landing</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>1. grep mã hex / rgb() trong app/styles, globals.css, components
+2. Liệt kê chỗ dùng màu safe / caution / danger</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Không màu rời ngoài tokens.css; màu lâm sàng chỉ dùng đúng nghĩa</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Không màu rời; safe = đã uống, caution = cảnh báo tương tác, danger = lỡ liều / lưu ý y khoa / 115</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · evidence/test-static.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="57.5" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-23</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Rê chuột lên thẻ an toàn</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>1440×900, chuột</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>1. Cuộn tới #an-toan
+2. Rê chuột lên góc phải trên của thẻ đầu tiên</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Chuột</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Spotlight theo con trỏ (--mx/--my, ::before opacity 1) và thẻ nghiêng 3D</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>--mx 294px, --rx 3.48deg, --ry 5.40deg, transform matrix3d, spotlight opacity 1</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · EP (6) · acceptance.mjs · evidence/test-acceptance-gpu.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="41" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-24</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Rê chuột lên nút App Store ở hero</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>1440×900, chuột</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>1. Rê chuột tới góc trên phải nút App Store</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Chuột</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Nút bị hút về phía con trỏ (magnetic) và vệt sáng lướt qua</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>transform translate(22.1px, -6.7px); ::after chuyển tới translateX dương (204 px)</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · acceptance.mjs · evidence/test-acceptance-gpu.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="74" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-25</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Mở trang trên thiết bị cảm ứng</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Giả lập iPhone 390×844, hasTouch</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở /
+2. Kiểm class motion-hover và transform của thẻ an toàn
+3. Chạm nút App Store</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Cảm ứng</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Không bật hiệu ứng hover; nút vẫn bấm được</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>motion-hover false, thẻ transform none</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · EP (7) · acceptance.mjs · evidence/test-acceptance-gpu.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="57.5" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-26</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Cuộn hết trang và đo khung hình</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>1440×900, GPU thật (Intel Iris Xe, D3D11), scene 3D sẵn sàng</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>1. Cuộn từ đầu tới cuối trang mỗi khung 28 px
+2. Đếm requestAnimationFrame và long task</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>FPS trung bình ≥ 55; không long task &gt; 100 ms</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>59,7 FPS (3157 khung / 52,9 s); 0 long task</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>AC13 · acceptance.mjs · evidence/test-acceptance-gpu.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="74" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-27</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm scene 3D dừng vẽ khi khuất màn hình và khi tab ẩn</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>1440×900, đếm GPUQueue.submit + WebGL draw</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>1. Rê chuột trên điện thoại 2 s, đếm lệnh vẽ
+2. Cuộn xuống cuối trang 2 s, đếm
+3. Về đầu trang, giả lập tab ẩn (visibilitychange), đếm 2 s</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>Có lệnh vẽ khi hiển thị; 0 khi khuất; 0 khi tab ẩn</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>visibleDraws 2093, offscreenDraws 0, hiddenDraws 0</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>AC13 · acceptance.mjs · evidence/test-acceptance-gpu.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="90.5" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-28</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Mở icon tính năng quanh iPhone bằng chuột, bàn phím và chạm</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>1440×900 (chuột, bàn phím); 375×812 cảm ứng</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>1. Rê chuột lên icon 1, rồi icon 6, rồi ra ngoài
+2. Tab tới icon 1, nhấn Escape
+3. Ở 375 px chạm icon 3, rồi chạm ngoài</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Chuột / Tab / chạm</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lần chỉ một icon mở (aria-expanded=true) và hiện tên + mô tả; rời chuột / Escape / chạm ngoài thì đóng; 375 px không cuộn ngang</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>Hover icon 0 → chỉ icon 0 mở (rộng 253 px); hover icon 5 → chỉ icon 5; rời chuột → đóng; Tab → icon 0 mở; Escape → đóng; chạm icon 2 → mở; chạm ngoài → đóng; overflow false</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>AC14 · EP (6,7,8) · orbit-probe.mjs · evidence/test-probes.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="41" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-29</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Mở icon tính năng khi bật giảm chuyển động</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>prefers-reduced-motion: reduce, 1440×900</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>1. Rê chuột lên icon 2
+2. Đọc animation-name của nút</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>reduce</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Icon vẫn mở, không có animation bồng bềnh</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>icon 1 aria-expanded true; animation none</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>AC14, AC3 · orbit-probe.mjs · evidence/test-probes.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="74" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-30</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Đổi thẻ đang mở trong section 'Còn nhiều hơn thế'</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>1440×900 chuột; 375 px mobile</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>1. Rê chuột lên thẻ thứ 4
+2. Ở mobile, kiểm trạng thái 5 thẻ</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>5 thẻ: Báo cáo tuân thủ, Gợi ý món ăn hợp thuốc, Theo dõi nhiều người thân, Chế độ đơn giản, Tra cứu thuốc</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>Desktop: chỉ thẻ được rê mở; mobile: cả 5 thẻ mở</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>Desktop [false,false,false,true,false]; mobile [true,true,true,true,true]</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>AC15 · orbit-probe.mjs · evidence/test-probes.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="90.5" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-31</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Rà câu chữ icon hero và 5 thẻ mới theo quyết định nghiệp vụ</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Bảng 'Quyết định nghiệp vụ áp dụng' trong 01-requirement</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>1. Tìm chữ 'AI' trong FeatureOrbit / MoreFeatures
+2. Tìm 'chỉ tham khảo'
+3. Tìm con số %
+4. Đọc mô tả liên quan người thân</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>QD-41, QD-40, QD-42, QD-27/28</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>Không 'AI'; có 'chỉ tham khảo'; không con số tuân thủ; người thân được mô tả là xem / nhận báo khi được đồng ý chia sẻ</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>Không "AI", có "Chỉ tham khảo" ở cả hai, không %; thẻ: "Xem lịch uống của bố, mẹ khi họ đồng ý chia sẻ."; icon hero: "Báo người nhà khi được chia sẻ". Vòng 1 Fail (BUG-LANDING-31), đã sửa.</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>AC16 · review nội dung · evidence/test-static.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="57.5" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>TC-LANDING-32</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Mở trang khi scene Spline treo quá 12 s</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>1440×900, no-preference; request scene.splinecode bị giữ 20 s</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở /
+2. Đợi trạng thái phone3d--loading
+3. Đợi tới khi hết thời gian chờ</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Độ trễ scene 20 s (ngưỡng 12 s)</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Khoảng 12 s sau khi bắt đầu tải: chuyển phone3d--failed, gỡ canvas, ảnh tĩnh hiện đầy đủ</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>failed sau 12 981 ms; canvas đã gỡ; ảnh tĩnh opacity 1</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · EP (11) · BVA (timeout) · timeout.mjs · evidence/test-spline-timeout.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43">
+      <c r="G43" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H43" s="13">
+        <f>COUNTIF(H9:H40,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="G44" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H44" s="13">
+        <f>COUNTIF(H9:H40,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="G45" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H45" s="13">
+        <f>COUNTIF(H9:H40,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="G46" s="12" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>Executed</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="C3" s="11">
-        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59+'Lịch uống thuốc'!$H$51+'Tải lịch uống'!$H$32+'Tương tác thuốc-thuốc'!$H$52+'Tương tác thuốc-thực phẩm'!$H$17+'Tra cứu hoạt chất'!$H$17+'Mã liên kết người thân'!$H$44</f>
+      <c r="H46" s="13">
+        <f>SUM(H43:H45)</f>
         <v/>
       </c>
-      <c r="D3" s="15">
-        <f>SUM(C3:C3)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="16" t="n"/>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="C4" s="11">
-        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60+'Lịch uống thuốc'!$H$52+'Tải lịch uống'!$H$33+'Tương tác thuốc-thuốc'!$H$53+'Tương tác thuốc-thực phẩm'!$H$18+'Tra cứu hoạt chất'!$H$18+'Mã liên kết người thân'!$H$45</f>
-        <v/>
-      </c>
-      <c r="D4" s="15">
-        <f>SUM(C4:C4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="17" t="n"/>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>(Total) Test executed (Passed + Failed)</t>
-        </is>
-      </c>
-      <c r="C5" s="11">
-        <f>C3+C4</f>
-        <v/>
-      </c>
-      <c r="D5" s="15">
-        <f>SUM(C5:C5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr"/>
-      <c r="C6" s="11">
-        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61+'Lịch uống thuốc'!$H$53+'Tải lịch uống'!$H$34+'Tương tác thuốc-thuốc'!$H$54+'Tương tác thuốc-thực phẩm'!$H$19+'Tra cứu hoạt chất'!$H$19+'Mã liên kết người thân'!$H$46</f>
-        <v/>
-      </c>
-      <c r="D6" s="15">
-        <f>SUM(C6:C6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>(Sub-total) Test Planned</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="11">
-        <f>C5+C6</f>
-        <v/>
-      </c>
-      <c r="D7" s="15">
-        <f>SUM(C7:C7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Function</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Sheet Name</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>% TCs Executed</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>% TCs Passed</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>% TCs Failed</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>Done by</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="156.5" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>Build ứng dụng Android</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Build APK debug của Mobile App từ nhánh main (cấu hình Gradle, desugaring, plugin native) và bước build trong CI</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>Android build</t>
-        </is>
-      </c>
-      <c r="D11" s="18">
-        <f>IFERROR(('Android build'!$H$23-'Android build'!$H$22)/'Android build'!$H$23,0)</f>
-        <v/>
-      </c>
-      <c r="E11" s="18">
-        <f>IFERROR('Android build'!$H$20/'Android build'!$H$23,0)</f>
-        <v/>
-      </c>
-      <c r="F11" s="18">
-        <f>IFERROR('Android build'!$H$21/'Android build'!$H$23,0)</f>
-        <v/>
-      </c>
-      <c r="G11" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>Lỗi Critical (APK không build được do flutter_local_notifications cần desugaring và flutter_timezone 2.x dùng API Registrar đã bị gỡ) đã sửa ở task adhoc-20261007-android-desugaring (frontend PR #27, CI xanh gồm bước build APK). Còn Pending: kiểm lockfile bằng --enforce-lockfile với Flutter stable.</t>
-        </is>
-      </c>
-      <c r="I11" s="11" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="189.5" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>Đăng nhập người dùng</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Đăng nhập Mobile App bằng OTP (số điện thoại hoặc email), hoàn thiện hồ sơ lần đầu, phiên đăng nhập và đăng xuất — user thường, không gồm admin</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
-        <is>
-          <t>Đăng nhập người dùng</t>
-        </is>
-      </c>
-      <c r="D12" s="18">
-        <f>IFERROR(('Đăng nhập người dùng'!$H$62-'Đăng nhập người dùng'!$H$61)/'Đăng nhập người dùng'!$H$62,0)</f>
-        <v/>
-      </c>
-      <c r="E12" s="18">
-        <f>IFERROR('Đăng nhập người dùng'!$H$59/'Đăng nhập người dùng'!$H$62,0)</f>
-        <v/>
-      </c>
-      <c r="F12" s="18">
-        <f>IFERROR('Đăng nhập người dùng'!$H$60/'Đăng nhập người dùng'!$H$62,0)</f>
-        <v/>
-      </c>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
-        <is>
-          <t>Luồng chính (đăng nhập, hồ sơ, consent, mở lại app, đăng xuất) và mọi kiểm tra quyền/bearer đạt, cả ở API lẫn E2E trên emulator. 7 Fail gồm lỗi kiểm tra đầu vào ở biên (chữ số Unicode, họ tên &gt; 255, ngày sinh &lt; 1900, ký tự NUL gây 500), lỗi múi giờ khi kiểm ngày sinh (dùng UTC), app gửi lại mã OTP sai khi chạm ô, và một kỳ vọng AC6 cần chốt lại (ký tự xuống dòng cuối số điện thoại).</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="222.5" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>Quản lý lịch uống thuốc</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Backend API thêm, sửa, hủy từng giờ uống; bật/tắt nhắc; đổi ngày uống trong tuần; mốc hiệu lực khi có liều xác nhận sớm (QD-16). Chỉ chính người bệnh được ghi.</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>Lịch uống thuốc</t>
-        </is>
-      </c>
-      <c r="D13" s="18">
-        <f>IFERROR(('Lịch uống thuốc'!$H$54-'Lịch uống thuốc'!$H$53)/'Lịch uống thuốc'!$H$54,0)</f>
-        <v/>
-      </c>
-      <c r="E13" s="18">
-        <f>IFERROR('Lịch uống thuốc'!$H$51/'Lịch uống thuốc'!$H$54,0)</f>
-        <v/>
-      </c>
-      <c r="F13" s="18">
-        <f>IFERROR('Lịch uống thuốc'!$H$52/'Lịch uống thuốc'!$H$54,0)</f>
-        <v/>
-      </c>
-      <c r="G13" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H13" s="10" t="inlineStr">
-        <is>
-          <t>Toàn bộ test tự động và kiểm tra biên đạt trên Supabase local. Đã sửa và có test cho các lỗi review R1 (sinh trùng liều khi ngừng/dùng lại sau liều xác nhận sớm), R2 (dùng lại thuốc khi cần mở lịch cũ), R3 (dùng lại mất lịch sau khi đổi cả bộ giờ/ngày sau liều sớm; sửa bằng migration closed_by_stop_at) và M3 (doses_per_day sau khi dùng lại). Có test bất biến trên chuỗi thao tác ngẫu nhiên. Chưa phủ: race giữa xác nhận liều sớm và sửa lịch (2.10).</t>
-        </is>
-      </c>
-      <c r="I13" s="11" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="90.5" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>Tải lịch uống và phân quyền dữ liệu thuốc</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>GET /patients/{patient_id}/schedules (lịch đang mở và đóng trong 30 ngày, phân trang con trỏ); phân quyền ghi lịch; QD-32 admin không đọc dữ liệu y tế; patient_id không tồn tại.</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>Tải lịch uống</t>
-        </is>
-      </c>
-      <c r="D14" s="18">
-        <f>IFERROR(('Tải lịch uống'!$H$35-'Tải lịch uống'!$H$34)/'Tải lịch uống'!$H$35,0)</f>
-        <v/>
-      </c>
-      <c r="E14" s="18">
-        <f>IFERROR('Tải lịch uống'!$H$32/'Tải lịch uống'!$H$35,0)</f>
-        <v/>
-      </c>
-      <c r="F14" s="18">
-        <f>IFERROR('Tải lịch uống'!$H$33/'Tải lịch uống'!$H$35,0)</f>
-        <v/>
-      </c>
-      <c r="G14" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
-        <is>
-          <t>Toàn bộ ca phân quyền đạt, mỗi ca kiểm cả response lẫn access_logs. Quy tắc QD-29 (app người thân không lưu xuống máy) là quy tắc client, chưa kiểm được ở backend.</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="90.5" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>Danh mục tương tác thuốc-thuốc (admin)</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Admin thêm, xem, sửa (tạo phiên bản mới), xóa mềm quy tắc tương tác giữa hai hoạt chất, kèm ngưỡng liều; xem lịch sử phiên bản (task 2.16, PB05).</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>Tương tác thuốc-thuốc</t>
-        </is>
-      </c>
-      <c r="D15" s="18">
-        <f>IFERROR(('Tương tác thuốc-thuốc'!$H$55-'Tương tác thuốc-thuốc'!$H$54)/'Tương tác thuốc-thuốc'!$H$55,0)</f>
-        <v/>
-      </c>
-      <c r="E15" s="18">
-        <f>IFERROR('Tương tác thuốc-thuốc'!$H$52/'Tương tác thuốc-thuốc'!$H$55,0)</f>
-        <v/>
-      </c>
-      <c r="F15" s="18">
-        <f>IFERROR('Tương tác thuốc-thuốc'!$H$53/'Tương tác thuốc-thuốc'!$H$55,0)</f>
-        <v/>
-      </c>
-      <c r="G15" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H15" s="10" t="inlineStr">
-        <is>
-          <t>Toàn bộ test tự động (tích hợp với Postgres thật, app chạy bằng api_role) pass. Không có lỗi sản phẩm.</t>
-        </is>
-      </c>
-      <c r="I15" s="11" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="107" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>Danh mục tương tác thuốc-thực phẩm (admin)</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>Admin thêm, xem, sửa (tạo phiên bản mới), xóa mềm quy tắc tương tác giữa hoạt chất và thực phẩm (task 2.16, PB05).</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr">
-        <is>
-          <t>Tương tác thuốc-thực phẩm</t>
-        </is>
-      </c>
-      <c r="D16" s="18">
-        <f>IFERROR(('Tương tác thuốc-thực phẩm'!$H$20-'Tương tác thuốc-thực phẩm'!$H$19)/'Tương tác thuốc-thực phẩm'!$H$20,0)</f>
-        <v/>
-      </c>
-      <c r="E16" s="18">
-        <f>IFERROR('Tương tác thuốc-thực phẩm'!$H$17/'Tương tác thuốc-thực phẩm'!$H$20,0)</f>
-        <v/>
-      </c>
-      <c r="F16" s="18">
-        <f>IFERROR('Tương tác thuốc-thực phẩm'!$H$18/'Tương tác thuốc-thực phẩm'!$H$20,0)</f>
-        <v/>
-      </c>
-      <c r="G16" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H16" s="10" t="inlineStr">
-        <is>
-          <t>Toàn bộ test tự động pass. Không có lỗi sản phẩm.</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="90.5" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>Tra cứu hoạt chất (admin)</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>Admin tìm hoạt chất theo tên chuẩn hoặc tên gọi khác, hoặc xem hoạt chất của một thuốc, để chọn khi nhập quy tắc tương tác (task 2.16).</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>Tra cứu hoạt chất</t>
-        </is>
-      </c>
-      <c r="D17" s="18">
-        <f>IFERROR(('Tra cứu hoạt chất'!$H$20-'Tra cứu hoạt chất'!$H$19)/'Tra cứu hoạt chất'!$H$20,0)</f>
-        <v/>
-      </c>
-      <c r="E17" s="18">
-        <f>IFERROR('Tra cứu hoạt chất'!$H$17/'Tra cứu hoạt chất'!$H$20,0)</f>
-        <v/>
-      </c>
-      <c r="F17" s="18">
-        <f>IFERROR('Tra cứu hoạt chất'!$H$18/'Tra cứu hoạt chất'!$H$20,0)</f>
-        <v/>
-      </c>
-      <c r="G17" s="11" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H17" s="10" t="inlineStr">
-        <is>
-          <t>Toàn bộ test tự động pass.</t>
-        </is>
-      </c>
-      <c r="I17" s="11" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="156.5" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>Mã liên kết người thân</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>User lấy mã liên kết cố định, không hết hạn của mình (kèm QR payload) để mời người thân: GET /family/link-code; mỗi user đúng một mã (QD-04, QD-34). Task 3.10, PB15.</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>Mã liên kết người thân</t>
-        </is>
-      </c>
-      <c r="D18" s="18">
-        <f>IFERROR(('Mã liên kết người thân'!$H$47-'Mã liên kết người thân'!$H$46)/'Mã liên kết người thân'!$H$47,0)</f>
-        <v/>
-      </c>
-      <c r="E18" s="18">
-        <f>IFERROR('Mã liên kết người thân'!$H$44/'Mã liên kết người thân'!$H$47,0)</f>
-        <v/>
-      </c>
-      <c r="F18" s="18">
-        <f>IFERROR('Mã liên kết người thân'!$H$45/'Mã liên kết người thân'!$H$47,0)</f>
-        <v/>
-      </c>
-      <c r="G18" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H18" s="10" t="inlineStr">
-        <is>
-          <t>Toàn bộ test tự động của chức năng (tích hợp với Postgres thật, app chạy bằng api_role; unit; contract) pass, kể cả sau bản sửa F1 của review (mã kiểu cũ sai định dạng bị xóa khi migrate, DB có CHECK định dạng). Một Fail: bộ unit test toàn repo và ruff toàn repo còn lỗi có sẵn trên main ở module khác, không do task này.</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="19" t="inlineStr">
-        <is>
-          <t>Bug Report</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="20" t="inlineStr">
-        <is>
-          <t>Bug ID</t>
-        </is>
-      </c>
-      <c r="B42" s="20" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C42" s="20" t="inlineStr">
-        <is>
-          <t>Steps to Reproduce</t>
-        </is>
-      </c>
-      <c r="D42" s="20" t="inlineStr">
-        <is>
-          <t>Input Data</t>
-        </is>
-      </c>
-      <c r="E42" s="20" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="F42" s="20" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="G42" s="20" t="inlineStr">
-        <is>
-          <t>Severity</t>
-        </is>
-      </c>
-      <c r="H42" s="20" t="inlineStr">
-        <is>
-          <t>Name of Tester</t>
-        </is>
-      </c>
-      <c r="I42" s="20" t="inlineStr">
-        <is>
-          <t>Logs</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="123.5" customHeight="1">
-      <c r="A43" s="22" t="inlineStr">
-        <is>
-          <t>BUG-LOGIN-08</t>
-        </is>
-      </c>
-      <c r="B43" s="22" t="inlineStr">
-        <is>
-          <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
-        </is>
-      </c>
-      <c r="C43" s="22" t="inlineStr">
-        <is>
-          <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
-2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
-        </is>
-      </c>
-      <c r="D43" s="22" t="inlineStr">
-        <is>
-          <t>phone: 0900000001 + ký tự \n</t>
-        </is>
-      </c>
-      <c r="E43" s="22" t="inlineStr">
-        <is>
-          <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
-        </is>
-      </c>
-      <c r="F43" s="22" t="inlineStr">
-        <is>
-          <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
-        </is>
-      </c>
-      <c r="G43" s="22" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H43" s="22" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-      <c r="I43" s="22" t="inlineStr">
-        <is>
-          <t>Nghi vấn — kỳ vọng AC6 mâu thuẫn AC5: backend `_validate_required_text` (sign_in.py:178) `strip()` mọi ký tự trắng hai đầu, nên \n cuối được xử lý như khoảng trắng hai đầu mà AC5 coi là hợp lệ. Cần người dùng chốt: sửa AC6 hoặc sửa backend
-Log: evidence/test-integration.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="123.5" customHeight="1">
-      <c r="A44" s="22" t="inlineStr">
-        <is>
-          <t>BUG-LOGIN-11</t>
-        </is>
-      </c>
-      <c r="B44" s="22" t="inlineStr">
-        <is>
-          <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
-        </is>
-      </c>
-      <c r="C44" s="22" t="inlineStr">
-        <is>
-          <t>1. POST /auth/mobile/otp {phone}
-2. POST /auth/mobile/verify {phone, token: 123456}</t>
-        </is>
-      </c>
-      <c r="D44" s="22" t="inlineStr">
-        <is>
-          <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
-        </is>
-      </c>
-      <c r="E44" s="22" t="inlineStr">
-        <is>
-          <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
-        </is>
-      </c>
-      <c r="F44" s="22" t="inlineStr">
-        <is>
-          <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
-        </is>
-      </c>
-      <c r="G44" s="22" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H44" s="22" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-      <c r="I44" s="22" t="inlineStr">
-        <is>
-          <t>`_normalize_phone` (sign_in.py:197–206) kiểm bằng `str.isdigit()`, nhận cả chữ số Unicode, nên số lọt qua kiểm tra và gửi tới Supabase. Ô nhập của app chỉ cho 0-9 nên người dùng app không gặp; lỗi ở tầng API
-Log: evidence/test-integration.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="189.5" customHeight="1">
-      <c r="A45" s="22" t="inlineStr">
-        <is>
-          <t>BUG-LOGIN-25</t>
-        </is>
-      </c>
-      <c r="B45" s="22" t="inlineStr">
-        <is>
-          <t>Lưu họ tên có ký tự NUL</t>
-        </is>
-      </c>
-      <c r="C45" s="22" t="inlineStr">
-        <is>
-          <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
-        </is>
-      </c>
-      <c r="D45" s="22" t="inlineStr">
-        <is>
-          <t>ho_ten: abc\u0000def</t>
-        </is>
-      </c>
-      <c r="E45" s="22" t="inlineStr">
-        <is>
-          <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
-        </is>
-      </c>
-      <c r="F45" s="22" t="inlineStr">
-        <is>
-          <t>500 Internal Server Error</t>
-        </is>
-      </c>
-      <c r="G45" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H45" s="22" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-      <c r="I45" s="22" t="inlineStr">
-        <is>
-          <t>`_validate_required_text` (sign_in.py:178) không chặn ký tự điều khiển; PostgreSQL từ chối NUL trong cột text: `psycopg.DataError: PostgreSQL text fields cannot contain NUL (0x00) bytes` ở `UPDATE users SET full_name…` (SqlUsers.update_profile); không có handler cho DataError nên thành 500. Câu SQL có tham số nên không phải lỗ hổng SQL injection
-Log: evidence/test-integration.log, evidence/test-probe-nul.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="90.5" customHeight="1">
-      <c r="A46" s="22" t="inlineStr">
-        <is>
-          <t>BUG-LOGIN-30</t>
-        </is>
-      </c>
-      <c r="B46" s="22" t="inlineStr">
-        <is>
-          <t>Lưu họ tên dài 256 ký tự</t>
-        </is>
-      </c>
-      <c r="C46" s="22" t="inlineStr">
-        <is>
-          <t>1. POST /auth/profile {ho_ten: A*256}</t>
-        </is>
-      </c>
-      <c r="D46" s="22" t="inlineStr">
-        <is>
-          <t>A*256</t>
-        </is>
-      </c>
-      <c r="E46" s="22" t="inlineStr">
-        <is>
-          <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
-        </is>
-      </c>
-      <c r="F46" s="22" t="inlineStr">
-        <is>
-          <t>204, đã lưu</t>
-        </is>
-      </c>
-      <c r="G46" s="22" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H46" s="22" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-      <c r="I46" s="22" t="inlineStr">
-        <is>
-          <t>Không có giới hạn độ dài họ tên: `_validate_profile` (sign_in.py) chỉ kiểm rỗng; cột users.full_name kiểu text không giới hạn
-Log: evidence/test-integration.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="90.5" customHeight="1">
-      <c r="A47" s="22" t="inlineStr">
-        <is>
-          <t>BUG-LOGIN-32</t>
-        </is>
-      </c>
-      <c r="B47" s="22" t="inlineStr">
-        <is>
-          <t>Lưu ngày sinh trước 1900-01-01</t>
-        </is>
-      </c>
-      <c r="C47" s="22" t="inlineStr">
-        <is>
-          <t>1. POST /auth/profile {ngay_sinh}</t>
-        </is>
-      </c>
-      <c r="D47" s="22" t="inlineStr">
-        <is>
-          <t>1899-12-31 | 0001-01-01</t>
-        </is>
-      </c>
-      <c r="E47" s="22" t="inlineStr">
-        <is>
-          <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
-        </is>
-      </c>
-      <c r="F47" s="22" t="inlineStr">
-        <is>
-          <t>204 ở cả hai giá trị, đã lưu</t>
-        </is>
-      </c>
-      <c r="G47" s="22" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H47" s="22" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-      <c r="I47" s="22" t="inlineStr">
-        <is>
-          <t>`_validate_birth_date` (sign_in.py:229–231) chỉ chặn ngày tương lai, không có cận dưới. App mobile đã giới hạn date picker từ 1900 nên chỉ gặp khi gọi API trực tiếp
-Log: evidence/test-integration.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="123.5" customHeight="1">
-      <c r="A48" s="22" t="inlineStr">
-        <is>
-          <t>BUG-LOGIN-35</t>
-        </is>
-      </c>
-      <c r="B48" s="22" t="inlineStr">
-        <is>
-          <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
-        </is>
-      </c>
-      <c r="C48" s="22" t="inlineStr">
-        <is>
-          <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
-        </is>
-      </c>
-      <c r="D48" s="22" t="inlineStr">
-        <is>
-          <t>ngay_sinh: 2026-10-08</t>
-        </is>
-      </c>
-      <c r="E48" s="22" t="inlineStr">
-        <is>
-          <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
-        </is>
-      </c>
-      <c r="F48" s="22" t="inlineStr">
-        <is>
-          <t>422 {"detail":"invalid_date_of_birth"}</t>
-        </is>
-      </c>
-      <c r="G48" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H48" s="22" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-      <c r="I48" s="22" t="inlineStr">
-        <is>
-          <t>`_validate_birth_date` (sign_in.py:230) so với `now.date()` trong khi `now()` (shared/clock.py) trả giờ UTC: từ 00:00 đến 07:00 giờ VN, "hôm nay" bị coi là ngày mai. Vi phạm bất biến 7 (múi giờ cố định Asia/Ho_Chi_Minh)
-Log: evidence/test-integration.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="173" customHeight="1">
-      <c r="A49" s="22" t="inlineStr">
-        <is>
-          <t>BUG-LOGIN-42</t>
-        </is>
-      </c>
-      <c r="B49" s="22" t="inlineStr">
-        <is>
-          <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
-        </is>
-      </c>
-      <c r="C49" s="22" t="inlineStr">
-        <is>
-          <t>1. Chạm vào ô mã OTP
-2. Theo dõi request backend nhận được</t>
-        </is>
-      </c>
-      <c r="D49" s="22" t="inlineStr">
-        <is>
-          <t>Ô đang chứa 000000</t>
-        </is>
-      </c>
-      <c r="E49" s="22" t="inlineStr">
-        <is>
-          <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
-        </is>
-      </c>
-      <c r="F49" s="22" t="inlineStr">
-        <is>
-          <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
-        </is>
-      </c>
-      <c r="G49" s="22" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H49" s="22" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-      <c r="I49" s="22" t="inlineStr">
-        <is>
-          <t>`OtpPinInput._handleTextChange` (frontend/mobile/lib/features/auth/presentation/widgets/otp_pin_input.dart:66–72) chạy với mọi thông báo của controller, kể cả khi chỉ đổi vị trí con trỏ lúc chạm ô, và gọi onCompleted hễ ô đủ 6 số → gửi lại mã sai, tốn hạn mức token_verifications
-Log: evidence/test-e2e.log (mục "request backend trong pha 2"), evidence/implement-P10-run-phase2-requests.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="189.5" customHeight="1">
-      <c r="A50" s="22" t="inlineStr">
-        <is>
-          <t>BUG-LINKCODE-28</t>
-        </is>
-      </c>
-      <c r="B50" s="22" t="inlineStr">
-        <is>
-          <t>Toàn bộ unit test, architecture test và ruff toàn repo pass</t>
-        </is>
-      </c>
-      <c r="C50" s="22" t="inlineStr">
-        <is>
-          <t>1. pytest tests/unit tests/architecture -q
-2. ruff check .
-3. So với baseline trước khi sửa code</t>
-        </is>
-      </c>
-      <c r="D50" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E50" s="22" t="inlineStr">
-        <is>
-          <t>pytest và ruff đều pass</t>
-        </is>
-      </c>
-      <c r="F50" s="22" t="inlineStr">
-        <is>
-          <t>697 pass, 1 fail (tests/unit/test_app.py::test_doses_batch_openapi_uses_contract_shape: NameError paths); ruff toàn repo 21 lỗi ở module khác. Fail và lỗi ruff đã có trước khi task sửa code; file của task pass ruff</t>
-        </is>
-      </c>
-      <c r="G50" s="22" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H50" s="22" t="inlineStr">
-        <is>
-          <t>zannguyen</t>
-        </is>
-      </c>
-      <c r="I50" s="22" t="inlineStr">
-        <is>
-          <t>Có sẵn trên main, không do task 3.10: test_app.py dòng 43–44 dùng biến paths chưa định nghĩa; ruff báo lỗi ở catalog/*, consent/adapters/outbound/job_queue.py, runtime/job_runner.py (F821 health chưa import, nghi vấn làm Worker lỗi khi ghi heartbeat), worker.py, tests/unit/test_catalog_crud.py
-Log: evidence/implement-final-backend.log</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:A5"/>
-  </mergeCells>
-  <conditionalFormatting sqref="F11:F18">
-    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
-      <formula>0.2</formula>
+  <autoFilter ref="A8:I40"/>
+  <conditionalFormatting sqref="H9:H40">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11:G18">
-    <cfRule type="expression" priority="2" dxfId="0">
-      <formula>OR(G11="Critical",G11="High")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G43:G50">
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
-      <formula>"Critical"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2">
-      <formula>"High"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="3">
-      <formula>"Medium"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation sqref="G11:G18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Critical,High,Medium,Low"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G43:G50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Critical,High,Medium,Low"</formula1>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(testcases): add 3.14 test cases (LINKFOLLOW, INVITELINK, APPNAV)
Generated by testcase_xlsx.py merge for 3.14-mobile-scan-qr-enter-code-ui.
53 test cases: 46 Pass, 0 Fail, 7 Pending (device/production checks).

Refs: 3.14

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -18,7 +18,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hồi quy xác nhận liều" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Landing page" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yêu cầu liên kết người thân" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo dõi người thân (app)" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Link mời người thân" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Khung điều hướng app" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Android build'!$A$8:$I$17</definedName>
@@ -33,6 +36,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Hồi quy xác nhận liều'!$A$8:$I$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Landing page'!$A$8:$I$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Yêu cầu liên kết người thân'!$A$8:$I$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Theo dõi người thân (app)'!$A$8:$I$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Link mời người thân'!$A$8:$I$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Khung điều hướng app'!$A$8:$I$13</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -371,12 +377,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$22</f>
+              <f>'Report'!$A$11:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$11:$D$22</f>
+              <f>'Report'!$D$11:$D$25</f>
             </numRef>
           </val>
         </ser>
@@ -395,12 +401,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$22</f>
+              <f>'Report'!$A$11:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$11:$E$22</f>
+              <f>'Report'!$E$11:$E$25</f>
             </numRef>
           </val>
         </ser>
@@ -419,12 +425,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$22</f>
+              <f>'Report'!$A$11:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$11:$F$22</f>
+              <f>'Report'!$F$11:$F$25</f>
             </numRef>
           </val>
         </ser>
@@ -527,7 +533,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>24</row>
+      <row>27</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -549,7 +555,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>24</row>
+      <row>27</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3240000"/>
@@ -8149,7 +8155,3427 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:O49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi người thân bằng QR, mã hoặc link (mobile) (LINKFOLLOW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="123.5" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Quét QR hợp lệ của patient và gửi yêu cầu</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Người thân đã đăng nhập, cấp quyền camera, đang ở màn Quét mã QR</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Tab Người thân → Theo dõi người thân → Quét mã QR
+2. Đưa QR của patient vào khung</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>drugtime://link?code=K7M2Q9XAR4</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>App chuyển sang màn nhập mã đã điền K7M2 Q9XA R4, tự gửi đúng một yêu cầu và hiện màn "Đang chờ xác nhận"</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Scanner giả phát QR 5 lần: repository nhận đúng 1 request với mã K7M2Q9XAR4, hiện LinkRequestResultScreen</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC1, AC4, AC5 · EP (1) · scan_link_qr_screen_test: AC5</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>Nội dung QR</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>drugtime://link?code=&lt;10 ký tự hợp lệ&gt;</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>URL https (link mời)
+Văn bản thường
+Scheme hoặc host khác
+Thiếu tham số code
+code có O, I, L, 0, 1
+code chữ thường
+code sai độ dài</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>9
+10
+11
+12
+13
+14
+15</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="123.5" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Quét QR không phải mã liên kết DrugTime</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở màn Quét mã QR</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Đưa lần lượt từng QR trong Test Data vào khung</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>https://drug-time-frontend.vercel.app/link#code=K7M2Q9XAR4; hello; drugtime://link?code=k7m2q9xar4</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Hiện "Đây không phải mã liên kết DrugTime."; không gửi request nào; vẫn ở màn quét</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Hiện đúng câu cho cả 3 QR; repository 0 lần gọi</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · EP (2,3,7) · scan_link_qr_screen_test: AC2</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>Mã nhập tay</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>10 ký tự trong bảng A-H J K M N P-Z 2-9
+Có khoảng trắng, gạch nối, chữ thường (được chuẩn hóa)
+Dán chuỗi drugtime://link?code=
+Dán link mời https://&lt;host&gt;/link#code=</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>2
+3
+4
+5</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>Ít hơn 10 ký tự
+Có ký tự ngoài bảng mã (0, 1, O, I, L, ký tự đặc biệt)</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>16
+17</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="140" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Đọc nội dung QR sai định dạng contract 3.10</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi bộ đọc QR với từng chuỗi trong Test Data</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>otherapp://link?code=…; drugtime://invite?code=…; drugtime://link; code có 0/O/I/L/1; 9 và 11 ký tự</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Bộ đọc trả null cho mọi chuỗi</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>18 chuỗi không hợp lệ đều trả null</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · EP (4,5,6,8) · link_code_test: AC2</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>Phản hồi của POST /family/link-requests</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>201 pending
+200 active (gửi lại)
+409 link_request_pending</t>
+        </is>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>6
+7
+8</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>404 link_code_not_found
+422 self_link_not_allowed
+409 already_linked
+200 rejected/revoked (gửi lại)
+429 có Retry-After
+429 thiếu Retry-After
+Mất mạng / 5xx
+401</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>18
+19
+20
+21
+22
+23
+24
+25</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="41" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Nhập mã có chữ thường, khoảng trắng, gạch nối</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở màn Nhập mã liên kết</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Gõ mã trong Test Data vào ô Mã liên kết</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>k7m2 q9xa-r4</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Ô hiện K7M2 Q9XA R4; nút "Gửi yêu cầu" bật; chưa gửi request</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Ô hiện K7M2 Q9XA R4, nút bật, repository 0 lần gọi</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · EP (1,2) · enter_link_code_screen_test: AC3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="74" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Dán chuỗi QR và link mời vào ô nhập</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở màn Nhập mã liên kết</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Dán chuỗi QR
+2. Xóa ô, dán link mời</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>drugtime://link?code=K7M2Q9XAR4; https://drug-time-frontend.vercel.app/link#code=K7M2Q9XAR5</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Ô lần lượt hiện K7M2 Q9XA R4 và K7M2 Q9XA R5</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Ô hiện đúng hai mã</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC3, AC15 · EP (3,4) · enter_link_code_screen_test</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="41" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-BVA-01</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Nhập 9 ký tự (dưới biên)</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở màn Nhập mã liên kết</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. Gõ mã trong Test Data
+2. Bấm Gửi yêu cầu</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>K7M2Q9XAR</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Dưới ô hiện "Mã cần đủ 10 ký tự (còn thiếu 1)."; nút tắt; không gửi request</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Hiện đúng câu, nút tắt, repository 0 lần gọi</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · BVA (min-1) · enter_link_code_screen_test</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="41" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-BVA-02</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Nhập đúng 10 ký tự (tại biên)</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở màn Nhập mã liên kết</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. Gõ mã trong Test Data</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>K7M2Q9XAR4</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Không có lỗi dưới ô; nút bật</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Nút bật, không có lỗi</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · BVA (min/max) · enter_link_code_screen_test</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="41" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-BVA-03</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Nhập 11 ký tự (trên biên)</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở màn Nhập mã liên kết</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. Gõ mã trong Test Data</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>K7M2Q9XAR4K</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Ô chỉ giữ 10 ký tự đầu K7M2 Q9XA R4; nút bật</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Ô hiện K7M2 Q9XA R4, nút bật</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · BVA (max+1) · enter_link_code_screen_test: AC3 BVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="41" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-06</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Nhập mã có ký tự ngoài bảng mã</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở màn Nhập mã liên kết</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Gõ mã trong Test Data</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>K7M2Q9XA01</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Dưới ô hiện "Mã chỉ gồm chữ và số, không có 0, O, 1, I, L."; nút tắt</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Hiện đúng câu, nút tắt</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · EP (6) · enter_link_code_screen_test</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="57.5" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-07</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Bấm Gửi liên tục khi request đầu chưa xong</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Đã nhập mã hợp lệ; server trả chậm</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Gửi yêu cầu 3 lần liên tiếp</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>K7M2Q9XAR4</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ một request; nút tắt và có vòng xoay trong lúc chờ</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Repository 1 lần gọi; có chỉ báo đang gửi; nút tắt</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · Đoán lỗi (bấm liên tục) · enter_link_code_screen_test: AC5</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="57.5" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-08</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Gửi mã không tồn tại hoặc patient chưa bật chia sẻ</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Đã nhập mã hợp lệ</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Gửi yêu cầu</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Server trả 404 link_code_not_found</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Hiện "Mã không đúng, hoặc người thân chưa bật chia sẻ với gia đình."; ở lại màn; giữ mã</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Hiện đúng câu, vẫn ở màn nhập mã, ô vẫn K7M2 Q9XA R4</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (Phản hồi 4) · enter_link_code_screen_test: AC6</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="41" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-09</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Gửi mã của chính mình</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Đã nhập mã của chính tài khoản</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Gửi yêu cầu</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Server trả 422 self_link_not_allowed</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Hiện "Đây là mã của chính bạn."; ở lại màn</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Hiện đúng câu</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (Phản hồi 5) · enter_link_code_screen_test: AC6</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="41" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-10</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Gửi mã của người đã theo dõi</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Đã liên kết active với patient này</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Gửi yêu cầu</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Server trả 409 already_linked</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Hiện "Bạn đã theo dõi người này rồi."</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Hiện đúng câu</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (Phản hồi 6) · enter_link_code_screen_test: AC6</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="41" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-11</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Gửi khi đã có yêu cầu đang chờ với patient</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Đã gửi yêu cầu trước đó, chưa được trả lời</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Gửi yêu cầu</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Server trả 409 link_request_pending</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Hiện màn "Đang chờ xác nhận" (không báo lỗi)</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Hiện màn Đang chờ xác nhận</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AC21 · EP (Phản hồi 3) · enter_link_code_screen_test: AC21</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="74" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-12</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Gửi lại khi yêu cầu cũ đã được chấp thuận, bị từ chối, hoặc trạng thái lạ</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Lần gửi trước bị mất phản hồi</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Gửi yêu cầu</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Server trả 200 với status active; rejected; xyz</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>active: "Đã được chấp thuận"; rejected: "Yêu cầu này không còn hiệu lực. Bạn có thể gửi lại." và ở lại màn; xyz: màn Đang chờ xác nhận</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Đúng cả ba kết quả</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AC21 · EP (Phản hồi 2,7) · enter_link_code_screen_test: AC21</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="57.5" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-13</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Bị khóa vì nhập sai nhiều lần</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Đã nhập mã hợp lệ</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Gửi yêu cầu
+2. Bấm Gửi lại khi đang đếm ngược
+3. Chờ hết 900 giây</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Server trả 429 link_request_locked, Retry-After: 900</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Hiện "Bạn đã nhập sai mã nhiều lần. Thử lại sau 15:00.", đếm ngược mỗi giây; nút tắt; hết giờ nút bật lại và không tự gửi</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Hiện 15:00 rồi 14:59; bấm không gửi; sau 900 giây nút bật, repository vẫn 1 lần gọi</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>AC20 · EP (Phản hồi 8) · enter_link_code_screen_test: AC20</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="57.5" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-14</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Bị chặn 24 giờ nhưng server không gửi Retry-After</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Đã nhập mã hợp lệ</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Gửi yêu cầu</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Server trả 429 link_request_cooldown, không có Retry-After</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Hiện "Người này đã từ chối nhiều lần liên tiếp." (không có thời gian); không tự gửi</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Hiện đúng câu không kèm thời gian</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>AC20 · EP (Phản hồi 9) · enter_link_code_screen_test: AC20</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="74" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-15</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Mất mạng khi gửi rồi bấm Thử lại</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Đã nhập mã hợp lệ; mất mạng</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Gửi yêu cầu
+2. Bấm Thử lại
+3. Sửa mã thành K7M2Q9XAR5 rồi bấm Gửi</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Lỗi mạng ở cả 3 lần</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Hiện "Không kết nối được, thử lại.", nút đổi thành Thử lại; lần 2 dùng cùng client_uuid; lần 3 dùng client_uuid mới; không tự gửi lại trong nền</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>client_uuid lần 1 = lần 2, lần 3 khác; sau 1 phút vẫn 3 request</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · EP (Phản hồi 10) · Đoán lỗi (mất mạng) · enter_link_code_screen_test: AC7</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="74" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-16</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Phiên hết hạn khi gửi yêu cầu</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Token đã hết hạn</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Gửi yêu cầu</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Server trả 401</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>App về màn Đăng nhập (onUnauthorized); không hiện lỗi về mã</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>onUnauthorized được gọi 1 lần; controller không có lỗi hiển thị</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (Phản hồi 11) · remote_family_link_repository_test, link_request_controller_test: AC8</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="74" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-17</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Gửi request đúng contract 3.13</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>HTTP server giả</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi mã K7M2Q9XAR4 qua repository Remote</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>client_uuid 9b2e4c71-5d3a-4f8e-a1c6-7e0d2b9f4a58</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>POST /family/link-requests, body đúng {client_uuid, code}, header Authorization: Bearer; mọi cặp mã trạng thái/detail được ánh xạ; detail lạ → không xác định</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>9/9 test của repository Remote pass</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · remote_family_link_repository_test</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="41" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-18</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối quyền camera</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Quyền camera ở trạng thái bị từ chối</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở màn Quét mã QR
+2. Bấm Cho phép camera sau khi bật quyền</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>(không có)</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Không crash; hiện "Chưa có quyền dùng camera", nút Nhập mã; xin lại được</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Hiện giải thích và nút Nhập mã; sau khi cấp quyền camera hiện</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · Đoán lỗi · scan_link_qr_screen_test: AC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="57.5" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-19</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Quyền camera bị từ chối vĩnh viễn</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Quyền camera bị từ chối vĩnh viễn</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở màn Quét mã QR
+2. Bấm Mở Cài đặt
+3. Bấm Nhập mã</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>(không có)</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Có nút Mở Cài đặt mở trang cài đặt app; Nhập mã mở màn nhập mã</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>openSettings được gọi 1 lần; mở màn nhập mã</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · scan_link_qr_screen_test: AC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="74" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-20</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Chọn cách theo dõi người thân từ tab Người thân</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở tab Người thân
+2. Bấm Theo dõi người thân
+3. Chọn Quét mã QR / Nhập mã
+4. Từ màn quét bấm Nhập mã</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>(không có)</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Sheet có hai lựa chọn; mỗi lựa chọn mở đúng màn; từ màn quét sang được màn nhập mã</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Đúng cả ba</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · family_tab_screen_test, scan_link_qr_screen_test: AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="41" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-21</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Mở link mời khi đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập, app đang ở Trang chủ</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở link mời từ bên ngoài app</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>https://drug-time-frontend.vercel.app/link#code=K7M2Q9XAR4</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>App mở màn Nhập mã đã điền K7M2 Q9XA R4; chưa gửi cho tới khi bấm Gửi</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Màn nhập mã điền sẵn, repository 0 lần; bấm Gửi thì 1 lần</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>AC16 · invite_link_flow_test</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="41" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-22</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Mở link mời khi chưa đăng nhập</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Chưa đăng nhập, đang ở màn nhập OTP</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở link mời
+2. Nhập OTP 123456</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>https://drug-time-frontend.vercel.app/link#code=K7M2Q9XAR4</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Link chờ tới khi đăng nhập xong; sau đó mở màn nhập mã đúng mã, chưa gửi</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Sau OTP hiện màn nhập mã K7M2 Q9XA R4, repository 0 lần</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>AC16 · invite_link_flow_test</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="41" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-23</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Mở link mời sai định dạng</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở link mời trong Test Data</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>https://drug-time-frontend.vercel.app/link#code=K7M2Q9XAR0</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>Màn nhập mã trống kèm "Link mời không hợp lệ."</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Hiện đúng câu, ô trống</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>AC15, AC16 · invite_link_flow_test, link_code_test: AC15</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="57.5" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-24</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Không lưu mã liên kết xuống máy hay log</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Đã nhập mã hợp lệ</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Gửi (lỗi mạng)
+2. Bấm Thử lại
+3. Rà code tìm print/debugPrint/log và storage</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>K7M2Q9XAR4</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>Không có lời gọi secure storage hay SQLite; không có lệnh log nào in mã</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>0 lời gọi kênh flutter_secure_storage/sqflite; grep sạch</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>AC13 · Bảo mật · enter_link_code_screen_test: AC13 · evidence/implement-ac13-grep.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="74" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-25</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Quét QR thật trên Android và kiểm DB</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Thiết bị Android thật; backend main chạy local; patient đã đồng ý family_sharing và đang hiện QR</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>1. Người thân quét QR của patient
+2. Kiểm caregiver_links trong DB
+3. Quét lại cùng QR</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>QR từ màn Mã liên kết của tôi</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>Hiện màn chờ; DB có 1 dòng caregiver_links pending cho đúng cặp; lần quét 2 vẫn hiện màn chờ và DB không thêm dòng</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr"/>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · manual (cần camera, thiết bị, backend)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="41" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-26</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Bật tắt đèn flash khi quét</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Thiết bị có đèn flash, đang ở màn quét</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm nút đèn
+2. Bấm lại</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>(không có)</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Đèn bật rồi tắt; icon đổi tương ứng</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr"/>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="74" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-27</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối quyền camera trên máy thật</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>App mới cài trên Android thật</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở màn quét, chọn Không cho phép
+2. Mở lại, chọn Không cho phép và không hỏi lại
+3. Bấm Mở Cài đặt</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>(không có)</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>Không crash; lần 2 có nút Mở Cài đặt mở đúng trang cài đặt DrugTime</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr"/>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="57.5" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-28</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>App bị ẩn rồi hiện lại khi hộp thoại xin quyền camera còn mở</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Mở màn Quét mã QR lần đầu, hộp thoại xin quyền camera đang hiện</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>1. App chuyển inactive rồi resumed (hộp thoại che màn hình)
+2. Chọn Cho phép trong hộp thoại</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>(không có)</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ có đúng một yêu cầu xin quyền; sau khi cho phép thì camera hiện</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>Số lần xin quyền giữ ở 1 sau resumed và sau khi trả kết quả; scanner hiện</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · Đoán lỗi (review M1) · scan_link_qr_screen_test: AC10 (M1) resumed</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="57.5" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-29</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Xin quyền camera bị lỗi nền tảng</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Plugin quyền ném lỗi khi xin quyền</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở màn Quét mã QR</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>PlatformException ERROR_ALREADY_REQUESTING_PERMISSIONS</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Không kẹt ở vòng xoay; hiện "Chưa có quyền dùng camera" và nút Nhập mã</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>Không còn vòng xoay; hiện giải thích và nút Nhập mã</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · Đoán lỗi (review M1) · scan_link_qr_screen_test: AC10 (M1) lỗi nền tảng</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="57.5" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-30</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Chỉ kiểm lại quyền camera khi quay về từ Cài đặt</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Quyền camera bị từ chối vĩnh viễn, đang ở màn quét</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>1. Ẩn rồi hiện lại app mà không bấm Mở Cài đặt
+2. Bấm Mở Cài đặt, bật quyền camera, quay lại app</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>(không có)</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>Bước 1 không xin quyền thêm; bước 2 kiểm lại quyền đúng một lần và camera hiện</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>Bước 1 số lần xin quyền vẫn 1; bước 2 thành 2 và scanner hiện</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · Đoán lỗi (review M1) · scan_link_qr_screen_test: AC10 (M1) Cài đặt</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="74" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-31</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Sửa mã khi đang bị khóa vì nhập sai hoặc đủ yêu cầu trong ngày</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Đã gửi K7M2Q9XAR4 và bị khóa</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>1. Sửa mã thành K7M2Q9XAR5
+2. Chờ hết thời gian khóa</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Server trả 429 link_request_locked, Retry-After: 900; 429 link_request_daily_limit, Retry-After: 60</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>Câu báo và thời gian chờ vẫn hiện, nút Gửi vẫn tắt; hết giờ nút bật lại, không tự gửi</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>Vẫn hiện "Bạn đã nhập sai mã nhiều lần. Thử lại sau 15:00.", nút tắt; daily_limit giữ 60 giây rồi mở lại, repository 1 lần gọi</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I42" s="8" t="inlineStr">
+        <is>
+          <t>AC20 · Đoán lỗi (review M2) · enter_link_code_screen_test: AC20 (M2); link_request_controller_test: AC20 (M2) daily_limit</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="57.5" customHeight="1">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKFOLLOW-32</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Sửa sang mã khác khi bị chặn vì patient cũ từ chối nhiều lần</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Đã gửi K7M2Q9XAR4 và bị chặn</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>1. Sửa mã thành K7M2Q9XAR5</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Server trả 429 link_request_cooldown, Retry-After: 86400</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>Câu báo và đếm ngược biến mất; nút Gửi bật (chặn chỉ áp cho patient cũ)</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>Không còn lỗi, không còn đếm ngược, nút bật</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="inlineStr">
+        <is>
+          <t>AC20 · Đoán lỗi (review M2) · link_request_controller_test: AC20 (M2) cooldown</t>
+        </is>
+      </c>
+    </row>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46">
+      <c r="G46" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H46" s="13">
+        <f>COUNTIF(H9:H43,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="G47" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H47" s="13">
+        <f>COUNTIF(H9:H43,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="G48" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H48" s="13">
+        <f>COUNTIF(H9:H43,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="G49" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H49" s="13">
+        <f>SUM(H46:H48)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I43"/>
+  <conditionalFormatting sqref="H9:H43">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Gửi và mở link mời người thân (INVITELINK)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Màn Gửi link mời</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="107" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-INVITELINK-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Mở Gửi link mời và xem link</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập, đã đồng ý family_sharing, mã của tài khoản là K7M2Q9XAR4</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Tab Người thân → Gửi link mời</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Mã K7M2Q9XAR4</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Hiện https://drug-time-frontend.vercel.app/link#code=K7M2Q9XAR4; không có cảnh báo</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Hiện đúng link; không có cảnh báo</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC22, AC23 · Decision Table (R1) · share_invite_link_screen_test</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>Phần #code của link</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>#code=&lt;10 ký tự hợp lệ&gt;</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>Thiếu #
+Thiếu code hoặc code rỗng
+Chữ thường
+Có 0/O
+Sai độ dài
+Chứa ký tự HTML</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>2
+3
+4
+5
+6
+7</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Tải được mã?</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="41" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-INVITELINK-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Chia sẻ link mời</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở màn Gửi link mời</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Chia sẻ</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Mã K7M2Q9XAR4</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Bảng chia sẻ nhận đúng một chuỗi: câu mời + link; không có tên hay thông tin hồ sơ</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Sharer giả nhận 1 chuỗi đúng inviteShareText(link)</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC22 · share_invite_link_screen_test</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>Đã đồng ý family_sharing?</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="41" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-INVITELINK-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Sao chép link mời</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở màn Gửi link mời</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Sao chép link</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Mã K7M2Q9XAR4</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Clipboard chứa đúng link; hiện "Đã sao chép link"</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Clipboard.setData nhận đúng link; SnackBar hiện</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC22 · share_invite_link_screen_test</t>
+        </is>
+      </c>
+      <c r="Q11" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T11" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="57.5" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-INVITELINK-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Gửi link khi chưa bật chia sẻ với gia đình</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Chưa đồng ý family_sharing</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở Gửi link mời
+2. Bấm Mở Quyền riêng tư</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>(không có)</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Có cảnh báo người thân chưa gửi được yêu cầu; vẫn có nút Chia sẻ; mở được màn Quyền riêng tư</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Có cảnh báo và nút Chia sẻ; mở PrivacySettingsScreen</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC23 · Decision Table (R2) · share_invite_link_screen_test</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
+        <is>
+          <t>Hiện link, Chia sẻ, Sao chép</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S12" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13" ht="57.5" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-INVITELINK-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Không tải được mã liên kết</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>GET /family/link-code lỗi (503)</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở Gửi link mời
+2. Bấm Thử lại khi server đã ổn</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Lần 1: lỗi unavailable; lần 2: mã K7M2Q9XAR4</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Lần 1: "Chưa thể tải link mời. Vui lòng thử lại.", không có link, không có nút chia sẻ/sao chép; sau Thử lại hiện link</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Đúng cả hai lần</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC23 · Decision Table (R3) · share_invite_link_screen_test</t>
+        </is>
+      </c>
+      <c r="Q13" s="10" t="inlineStr">
+        <is>
+          <t>Cảnh báo + lối sang Quyền riêng tư</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="inlineStr"/>
+      <c r="S13" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="57.5" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-INVITELINK-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Ghép link và đọc ngược ra mã</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. Ghép link từ mã
+2. Đọc lại mã từ link</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>K7M2Q9XAR4, host drug-time-frontend.vercel.app</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Link https://drug-time-frontend.vercel.app/link#code=K7M2Q9XAR4; đọc lại được K7M2Q9XAR4</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Đúng</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC22 · link_code_test: AC22</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>Thông báo lỗi + Thử lại, không có link</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr"/>
+      <c r="S14" s="11" t="inlineStr"/>
+      <c r="T14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="74" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-INVITELINK-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Trang /link đọc phần #code</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi parseInviteHash với từng giá trị</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>#code=K7M2Q9XAR4; code=K7M2Q9XAR4; (blank); #ma=…; #code=; chữ thường; có 0/O; 9/11 ký tự; #code=&lt;script&gt;</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Hai giá trị đầu trả mã; còn lại trả null</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>4/4 test vitest pass</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC17 · EP (1-7) · landing lib/invite/linkCode.test.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="57.5" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-INVITELINK-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>HTML trang /link không lộ mã và không được lập chỉ mục</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Landing build và chạy bằng next start</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. curl http://127.0.0.1:3917/link</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>(không có)</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Có meta robots noindex, nofollow; thẻ OG chỉ có nội dung chung; không chứa mã; không có script ngoài</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>robots "noindex, nofollow"; OG chung; 0 lần xuất hiện K7M2; 0 script ngoài</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC17 · Bảo mật · evidence/implement-P16.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90.5" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-INVITELINK-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Mở trang /link trên trình duyệt</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Landing đã deploy</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở link mời trên Chrome Android và desktop
+2. Bấm Sao chép mã
+3. Xem tab Network</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>/link#code=K7M2Q9XAR4; /link#code=abc</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Hiện K7M2 Q9XA R4, nút sao chép, Mở bằng ứng dụng (chỉ Android), Tải ứng dụng, hướng dẫn iPhone; không có request tới backend hay analytics; mã sai hiện thông báo chung</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr"/>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC17 · manual (trình duyệt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="41" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-INVITELINK-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>File assetlinks.json phục vụ đúng</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Landing build và chạy bằng next start</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. curl -i http://127.0.0.1:3917/.well-known/assetlinks.json</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>(không có)</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>200, Content-Type application/json</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>200 OK, Content-Type: application/json; charset=UTF-8</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC18 (local) · evidence/implement-P16.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="74" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-INVITELINK-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>App Links được Android xác minh trên production</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Landing đã deploy lên drug-time-frontend.vercel.app; cài APK ký bằng khóa có fingerprint trong assetlinks.json</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. curl -i https://drug-time-frontend.vercel.app/.well-known/assetlinks.json
+2. adb shell pm get-app-links vn.drugtime.drugtime_mobile</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>(không có)</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>200 application/json; host drug-time-frontend.vercel.app ở trạng thái verified</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr"/>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC18 · manual (cần deploy production, Q1-A)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="74" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-INVITELINK-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Bấm link mời trong Zalo và SMS</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Android thật đã cài APK demo; landing đã lên production</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi link qua Zalo, bấm link
+2. Gửi qua SMS, bấm link
+3. Nếu Zalo mở trình duyệt riêng: bấm Mở bằng ứng dụng DrugTime</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>https://drug-time-frontend.vercel.app/link#code=&lt;mã thật&gt;</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>App mở màn nhập mã đã điền sẵn; với trình duyệt của Zalo, nút Mở bằng ứng dụng vào được app</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr"/>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC19 · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="41" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-INVITELINK-13</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Chia sẻ link qua bảng chia sẻ thật</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Android thật có Zalo</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. Tab Người thân → Gửi link mời → Chia sẻ
+2. Chọn Zalo, gửi cho một người</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>(không có)</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Zalo nhận đúng câu mời kèm link</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr"/>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AC22 · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24">
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H24" s="13">
+        <f>COUNTIF(H9:H21,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H25" s="13">
+        <f>COUNTIF(H9:H21,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H26" s="13">
+        <f>COUNTIF(H9:H21,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H27" s="13">
+        <f>SUM(H24:H26)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I21"/>
+  <conditionalFormatting sqref="H9:H21">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Khung điều hướng: tab Hồ sơ và Người thân (APPNAV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="57.5" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-APPNAV-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Mở tab Hồ sơ</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm tab Hồ sơ</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>(không có)</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Hiện màn Hồ sơ có mục Người giám sát; không có thẻ UI Catalog hay lối tắt màn Đăng nhập</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>ProfileScreen có supervisors-tile; không có UI Catalog</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC24 · app_shell_test: AC24</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="41" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-APPNAV-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Đăng xuất từ menu cài đặt của Hồ sơ</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Tab Hồ sơ → nút cài đặt → Đăng xuất</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>(không có)</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Về màn Đăng nhập; phiên bị xóa</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Hiện LoginMobileScreen; phiên null</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC24 · auth_flow_test: (e) Đăng xuất</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="41" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-APPNAV-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Menu cài đặt của Hồ sơ không còn UI Catalog</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập, ở tab Hồ sơ</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm nút cài đặt</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>(không có)</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Menu chỉ có một mục "Đăng xuất"</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>1 mục Đăng xuất</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC25 · app_shell_test: AC25</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-APPNAV-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Mở route /dev-catalog</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi onGenerateRoute với /dev-catalog</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>/dev-catalog</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Không có route (null)</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC25 · app_shell_test: AC25</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="41" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-APPNAV-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Mở tab Người thân</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm tab Người thân</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>(không có)</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Hiện các thẻ Mã liên kết của tôi, Gửi link mời, Theo dõi người thân</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Hiện FamilyTabScreen; thẻ Mã liên kết của tôi mở màn QR của 3.11</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · app_shell_test, family_tab_screen_test</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16">
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H16" s="13">
+        <f>COUNTIF(H9:H13,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H17" s="13">
+        <f>COUNTIF(H9:H13,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H18" s="13">
+        <f>COUNTIF(H9:H13,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H19" s="13">
+        <f>SUM(H16:H18)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I13"/>
+  <conditionalFormatting sqref="H9:H13">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8199,7 +11625,7 @@
         </is>
       </c>
       <c r="C3" s="11">
-        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59+'Lịch uống thuốc'!$H$51+'Tải lịch uống'!$H$32+'Tương tác thuốc-thuốc'!$H$52+'Tương tác thuốc-thực phẩm'!$H$17+'Tra cứu hoạt chất'!$H$17+'Mã liên kết người thân'!$H$47+'Landing page'!$H$43+'Yêu cầu liên kết người thân'!$H$72</f>
+        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59+'Lịch uống thuốc'!$H$51+'Tải lịch uống'!$H$32+'Tương tác thuốc-thuốc'!$H$52+'Tương tác thuốc-thực phẩm'!$H$17+'Tra cứu hoạt chất'!$H$17+'Mã liên kết người thân'!$H$47+'Landing page'!$H$43+'Yêu cầu liên kết người thân'!$H$72+'Theo dõi người thân (app)'!$H$46+'Link mời người thân'!$H$24+'Khung điều hướng app'!$H$16</f>
         <v/>
       </c>
       <c r="D3" s="11">
@@ -8219,7 +11645,7 @@
         </is>
       </c>
       <c r="C4" s="11">
-        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60+'Lịch uống thuốc'!$H$52+'Tải lịch uống'!$H$33+'Tương tác thuốc-thuốc'!$H$53+'Tương tác thuốc-thực phẩm'!$H$18+'Tra cứu hoạt chất'!$H$18+'Mã liên kết người thân'!$H$48+'Landing page'!$H$44+'Yêu cầu liên kết người thân'!$H$73</f>
+        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60+'Lịch uống thuốc'!$H$52+'Tải lịch uống'!$H$33+'Tương tác thuốc-thuốc'!$H$53+'Tương tác thuốc-thực phẩm'!$H$18+'Tra cứu hoạt chất'!$H$18+'Mã liên kết người thân'!$H$48+'Landing page'!$H$44+'Yêu cầu liên kết người thân'!$H$73+'Theo dõi người thân (app)'!$H$47+'Link mời người thân'!$H$25+'Khung điều hướng app'!$H$17</f>
         <v/>
       </c>
       <c r="D4" s="11">
@@ -8259,7 +11685,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr"/>
       <c r="C6" s="11">
-        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61+'Lịch uống thuốc'!$H$53+'Tải lịch uống'!$H$34+'Tương tác thuốc-thuốc'!$H$54+'Tương tác thuốc-thực phẩm'!$H$19+'Tra cứu hoạt chất'!$H$19+'Mã liên kết người thân'!$H$49+'Landing page'!$H$45+'Yêu cầu liên kết người thân'!$H$74</f>
+        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61+'Lịch uống thuốc'!$H$53+'Tải lịch uống'!$H$34+'Tương tác thuốc-thuốc'!$H$54+'Tương tác thuốc-thực phẩm'!$H$19+'Tra cứu hoạt chất'!$H$19+'Mã liên kết người thân'!$H$49+'Landing page'!$H$45+'Yêu cầu liên kết người thân'!$H$74+'Theo dõi người thân (app)'!$H$48+'Link mời người thân'!$H$26+'Khung điều hướng app'!$H$18</f>
         <v/>
       </c>
       <c r="D6" s="11">
@@ -8866,493 +12292,625 @@
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="19" t="inlineStr">
+    <row r="23" ht="107" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>Theo dõi người thân bằng QR, mã hoặc link (mobile)</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Người thân quét QR, nhập mã hoặc mở link mời để gửi yêu cầu liên kết tới patient (POST /family/link-requests).</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Theo dõi người thân (app)</t>
+        </is>
+      </c>
+      <c r="D23" s="18">
+        <f>IFERROR(('Theo dõi người thân (app)'!$H$49-'Theo dõi người thân (app)'!$H$48)/'Theo dõi người thân (app)'!$H$49,0)</f>
+        <v/>
+      </c>
+      <c r="E23" s="18">
+        <f>IFERROR('Theo dõi người thân (app)'!$H$46/'Theo dõi người thân (app)'!$H$49,0)</f>
+        <v/>
+      </c>
+      <c r="F23" s="18">
+        <f>IFERROR('Theo dõi người thân (app)'!$H$47/'Theo dõi người thân (app)'!$H$49,0)</f>
+        <v/>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động (widget/unit) pass trong phiên 2026-10-20. Các ca cần camera, thiết bị Android thật và backend chạy thật còn Pending.</t>
+        </is>
+      </c>
+      <c r="I23" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="90.5" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>Gửi và mở link mời người thân</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Patient chia sẻ link mời cố định https://&lt;host&gt;/link#code=&lt;mã&gt;; trang /link trên landing và App Links mở app.</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Link mời người thân</t>
+        </is>
+      </c>
+      <c r="D24" s="18">
+        <f>IFERROR(('Link mời người thân'!$H$27-'Link mời người thân'!$H$26)/'Link mời người thân'!$H$27,0)</f>
+        <v/>
+      </c>
+      <c r="E24" s="18">
+        <f>IFERROR('Link mời người thân'!$H$24/'Link mời người thân'!$H$27,0)</f>
+        <v/>
+      </c>
+      <c r="F24" s="18">
+        <f>IFERROR('Link mời người thân'!$H$25/'Link mời người thân'!$H$27,0)</f>
+        <v/>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>Phần app và hàm thuần của landing đã test tự động; kiểm trang trên trình duyệt, App Links và Zalo cần landing lên production và thiết bị thật (Pending).</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="90.5" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>Khung điều hướng: tab Hồ sơ và Người thân</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Tab Hồ sơ dùng màn Hồ sơ thật (sửa lỗi sau merge 3.11); bỏ trang UI Catalog; tab Người thân dùng FamilyTabScreen.</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Khung điều hướng app</t>
+        </is>
+      </c>
+      <c r="D25" s="18">
+        <f>IFERROR(('Khung điều hướng app'!$H$19-'Khung điều hướng app'!$H$18)/'Khung điều hướng app'!$H$19,0)</f>
+        <v/>
+      </c>
+      <c r="E25" s="18">
+        <f>IFERROR('Khung điều hướng app'!$H$16/'Khung điều hướng app'!$H$19,0)</f>
+        <v/>
+      </c>
+      <c r="F25" s="18">
+        <f>IFERROR('Khung điều hướng app'!$H$17/'Khung điều hướng app'!$H$19,0)</f>
+        <v/>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ pass; test Đăng xuất từng fail trên main nay pass.</t>
+        </is>
+      </c>
+      <c r="I25" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="19" t="inlineStr">
         <is>
           <t>Bug Report</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="20" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="20" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="B46" s="20" t="inlineStr">
+      <c r="B49" s="20" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C46" s="20" t="inlineStr">
+      <c r="C49" s="20" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="D46" s="20" t="inlineStr">
+      <c r="D49" s="20" t="inlineStr">
         <is>
           <t>Input Data</t>
         </is>
       </c>
-      <c r="E46" s="20" t="inlineStr">
+      <c r="E49" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F46" s="20" t="inlineStr">
+      <c r="F49" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="G46" s="20" t="inlineStr">
+      <c r="G49" s="20" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="H46" s="20" t="inlineStr">
+      <c r="H49" s="20" t="inlineStr">
         <is>
           <t>Name of Tester</t>
         </is>
       </c>
-      <c r="I46" s="20" t="inlineStr">
+      <c r="I49" s="20" t="inlineStr">
         <is>
           <t>Logs</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="123.5" customHeight="1">
-      <c r="A47" s="22" t="inlineStr">
+    <row r="50" ht="123.5" customHeight="1">
+      <c r="A50" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-08</t>
         </is>
       </c>
-      <c r="B47" s="22" t="inlineStr">
+      <c r="B50" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
         </is>
       </c>
-      <c r="C47" s="22" t="inlineStr">
+      <c r="C50" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
 2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
         </is>
       </c>
-      <c r="D47" s="22" t="inlineStr">
+      <c r="D50" s="22" t="inlineStr">
         <is>
           <t>phone: 0900000001 + ký tự \n</t>
         </is>
       </c>
-      <c r="E47" s="22" t="inlineStr">
+      <c r="E50" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F47" s="22" t="inlineStr">
+      <c r="F50" s="22" t="inlineStr">
         <is>
           <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
         </is>
       </c>
-      <c r="G47" s="22" t="inlineStr">
+      <c r="G50" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H47" s="22" t="inlineStr">
+      <c r="H50" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I47" s="22" t="inlineStr">
+      <c r="I50" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn — kỳ vọng AC6 mâu thuẫn AC5: backend `_validate_required_text` (sign_in.py:178) `strip()` mọi ký tự trắng hai đầu, nên \n cuối được xử lý như khoảng trắng hai đầu mà AC5 coi là hợp lệ. Cần người dùng chốt: sửa AC6 hoặc sửa backend
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="123.5" customHeight="1">
-      <c r="A48" s="22" t="inlineStr">
+    <row r="51" ht="123.5" customHeight="1">
+      <c r="A51" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-11</t>
         </is>
       </c>
-      <c r="B48" s="22" t="inlineStr">
+      <c r="B51" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
         </is>
       </c>
-      <c r="C48" s="22" t="inlineStr">
+      <c r="C51" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone}
 2. POST /auth/mobile/verify {phone, token: 123456}</t>
         </is>
       </c>
-      <c r="D48" s="22" t="inlineStr">
+      <c r="D51" s="22" t="inlineStr">
         <is>
           <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
         </is>
       </c>
-      <c r="E48" s="22" t="inlineStr">
+      <c r="E51" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
         </is>
       </c>
-      <c r="F48" s="22" t="inlineStr">
+      <c r="F51" s="22" t="inlineStr">
         <is>
           <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
         </is>
       </c>
-      <c r="G48" s="22" t="inlineStr">
+      <c r="G51" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H48" s="22" t="inlineStr">
+      <c r="H51" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I48" s="22" t="inlineStr">
+      <c r="I51" s="22" t="inlineStr">
         <is>
           <t>`_normalize_phone` (sign_in.py:197–206) kiểm bằng `str.isdigit()`, nhận cả chữ số Unicode, nên số lọt qua kiểm tra và gửi tới Supabase. Ô nhập của app chỉ cho 0-9 nên người dùng app không gặp; lỗi ở tầng API
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="189.5" customHeight="1">
-      <c r="A49" s="22" t="inlineStr">
+    <row r="52" ht="189.5" customHeight="1">
+      <c r="A52" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-25</t>
         </is>
       </c>
-      <c r="B49" s="22" t="inlineStr">
+      <c r="B52" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên có ký tự NUL</t>
         </is>
       </c>
-      <c r="C49" s="22" t="inlineStr">
+      <c r="C52" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
         </is>
       </c>
-      <c r="D49" s="22" t="inlineStr">
+      <c r="D52" s="22" t="inlineStr">
         <is>
           <t>ho_ten: abc\u0000def</t>
         </is>
       </c>
-      <c r="E49" s="22" t="inlineStr">
+      <c r="E52" s="22" t="inlineStr">
         <is>
           <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
         </is>
       </c>
-      <c r="F49" s="22" t="inlineStr">
+      <c r="F52" s="22" t="inlineStr">
         <is>
           <t>500 Internal Server Error</t>
         </is>
       </c>
-      <c r="G49" s="22" t="inlineStr">
+      <c r="G52" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H49" s="22" t="inlineStr">
+      <c r="H52" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I49" s="22" t="inlineStr">
+      <c r="I52" s="22" t="inlineStr">
         <is>
           <t>`_validate_required_text` (sign_in.py:178) không chặn ký tự điều khiển; PostgreSQL từ chối NUL trong cột text: `psycopg.DataError: PostgreSQL text fields cannot contain NUL (0x00) bytes` ở `UPDATE users SET full_name…` (SqlUsers.update_profile); không có handler cho DataError nên thành 500. Câu SQL có tham số nên không phải lỗ hổng SQL injection
 Log: evidence/test-integration.log, evidence/test-probe-nul.log</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="90.5" customHeight="1">
-      <c r="A50" s="22" t="inlineStr">
+    <row r="53" ht="90.5" customHeight="1">
+      <c r="A53" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-30</t>
         </is>
       </c>
-      <c r="B50" s="22" t="inlineStr">
+      <c r="B53" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên dài 256 ký tự</t>
         </is>
       </c>
-      <c r="C50" s="22" t="inlineStr">
+      <c r="C53" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: A*256}</t>
         </is>
       </c>
-      <c r="D50" s="22" t="inlineStr">
+      <c r="D53" s="22" t="inlineStr">
         <is>
           <t>A*256</t>
         </is>
       </c>
-      <c r="E50" s="22" t="inlineStr">
+      <c r="E53" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F50" s="22" t="inlineStr">
+      <c r="F53" s="22" t="inlineStr">
         <is>
           <t>204, đã lưu</t>
         </is>
       </c>
-      <c r="G50" s="22" t="inlineStr">
+      <c r="G53" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H50" s="22" t="inlineStr">
+      <c r="H53" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I50" s="22" t="inlineStr">
+      <c r="I53" s="22" t="inlineStr">
         <is>
           <t>Không có giới hạn độ dài họ tên: `_validate_profile` (sign_in.py) chỉ kiểm rỗng; cột users.full_name kiểu text không giới hạn
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="90.5" customHeight="1">
-      <c r="A51" s="22" t="inlineStr">
+    <row r="54" ht="90.5" customHeight="1">
+      <c r="A54" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-32</t>
         </is>
       </c>
-      <c r="B51" s="22" t="inlineStr">
+      <c r="B54" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh trước 1900-01-01</t>
         </is>
       </c>
-      <c r="C51" s="22" t="inlineStr">
+      <c r="C54" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh}</t>
         </is>
       </c>
-      <c r="D51" s="22" t="inlineStr">
+      <c r="D54" s="22" t="inlineStr">
         <is>
           <t>1899-12-31 | 0001-01-01</t>
         </is>
       </c>
-      <c r="E51" s="22" t="inlineStr">
+      <c r="E54" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
         </is>
       </c>
-      <c r="F51" s="22" t="inlineStr">
+      <c r="F54" s="22" t="inlineStr">
         <is>
           <t>204 ở cả hai giá trị, đã lưu</t>
         </is>
       </c>
-      <c r="G51" s="22" t="inlineStr">
+      <c r="G54" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H51" s="22" t="inlineStr">
+      <c r="H54" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I51" s="22" t="inlineStr">
+      <c r="I54" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:229–231) chỉ chặn ngày tương lai, không có cận dưới. App mobile đã giới hạn date picker từ 1900 nên chỉ gặp khi gọi API trực tiếp
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="123.5" customHeight="1">
-      <c r="A52" s="22" t="inlineStr">
+    <row r="55" ht="123.5" customHeight="1">
+      <c r="A55" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-35</t>
         </is>
       </c>
-      <c r="B52" s="22" t="inlineStr">
+      <c r="B55" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
         </is>
       </c>
-      <c r="C52" s="22" t="inlineStr">
+      <c r="C55" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
         </is>
       </c>
-      <c r="D52" s="22" t="inlineStr">
+      <c r="D55" s="22" t="inlineStr">
         <is>
           <t>ngay_sinh: 2026-10-08</t>
         </is>
       </c>
-      <c r="E52" s="22" t="inlineStr">
+      <c r="E55" s="22" t="inlineStr">
         <is>
           <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
         </is>
       </c>
-      <c r="F52" s="22" t="inlineStr">
+      <c r="F55" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_date_of_birth"}</t>
         </is>
       </c>
-      <c r="G52" s="22" t="inlineStr">
+      <c r="G55" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H52" s="22" t="inlineStr">
+      <c r="H55" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I52" s="22" t="inlineStr">
+      <c r="I55" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:230) so với `now.date()` trong khi `now()` (shared/clock.py) trả giờ UTC: từ 00:00 đến 07:00 giờ VN, "hôm nay" bị coi là ngày mai. Vi phạm bất biến 7 (múi giờ cố định Asia/Ho_Chi_Minh)
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="173" customHeight="1">
-      <c r="A53" s="22" t="inlineStr">
+    <row r="56" ht="173" customHeight="1">
+      <c r="A56" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-42</t>
         </is>
       </c>
-      <c r="B53" s="22" t="inlineStr">
+      <c r="B56" s="22" t="inlineStr">
         <is>
           <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
         </is>
       </c>
-      <c r="C53" s="22" t="inlineStr">
+      <c r="C56" s="22" t="inlineStr">
         <is>
           <t>1. Chạm vào ô mã OTP
 2. Theo dõi request backend nhận được</t>
         </is>
       </c>
-      <c r="D53" s="22" t="inlineStr">
+      <c r="D56" s="22" t="inlineStr">
         <is>
           <t>Ô đang chứa 000000</t>
         </is>
       </c>
-      <c r="E53" s="22" t="inlineStr">
+      <c r="E56" s="22" t="inlineStr">
         <is>
           <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
         </is>
       </c>
-      <c r="F53" s="22" t="inlineStr">
+      <c r="F56" s="22" t="inlineStr">
         <is>
           <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
         </is>
       </c>
-      <c r="G53" s="22" t="inlineStr">
+      <c r="G56" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H53" s="22" t="inlineStr">
+      <c r="H56" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I53" s="22" t="inlineStr">
+      <c r="I56" s="22" t="inlineStr">
         <is>
           <t>`OtpPinInput._handleTextChange` (frontend/mobile/lib/features/auth/presentation/widgets/otp_pin_input.dart:66–72) chạy với mọi thông báo của controller, kể cả khi chỉ đổi vị trí con trỏ lúc chạm ô, và gọi onCompleted hễ ô đủ 6 số → gửi lại mã sai, tốn hạn mức token_verifications
 Log: evidence/test-e2e.log (mục "request backend trong pha 2"), evidence/implement-P10-run-phase2-requests.log</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="222.5" customHeight="1">
-      <c r="A54" s="22" t="inlineStr">
+    <row r="57" ht="222.5" customHeight="1">
+      <c r="A57" s="22" t="inlineStr">
         <is>
           <t>BUG-LINKCODE-28</t>
         </is>
       </c>
-      <c r="B54" s="22" t="inlineStr">
+      <c r="B57" s="22" t="inlineStr">
         <is>
           <t>Toàn bộ unit test, architecture test và ruff toàn repo pass</t>
         </is>
       </c>
-      <c r="C54" s="22" t="inlineStr">
+      <c r="C57" s="22" t="inlineStr">
         <is>
           <t>1. pytest tests/unit tests/architecture -q
 2. ruff check .
 3. So với baseline trước khi sửa code</t>
         </is>
       </c>
-      <c r="D54" s="22" t="inlineStr">
+      <c r="D57" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E54" s="22" t="inlineStr">
+      <c r="E57" s="22" t="inlineStr">
         <is>
           <t>pytest và ruff đều pass</t>
         </is>
       </c>
-      <c r="F54" s="22" t="inlineStr">
+      <c r="F57" s="22" t="inlineStr">
         <is>
           <t>pytest tests/unit tests/architecture: 885 passed, 18 failed (test_contract_profile.py ×12, test_profile_http.py ×6); ruff check . 19 lỗi ở module khác. Cùng danh sách với baseline trước khi 3.13 sửa code; file của task pass ruff. Lỗi test_app.py của lần chạy 3.10 không còn</t>
         </is>
       </c>
-      <c r="G54" s="22" t="inlineStr">
+      <c r="G57" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H54" s="22" t="inlineStr">
+      <c r="H57" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I54" s="22" t="inlineStr">
+      <c r="I57" s="22" t="inlineStr">
         <is>
           <t>Có sẵn trên main, không do 3.10/3.13. Nghi vấn: 18 test profile fail vì api_contract (aea2b26) chưa có các endpoint /profile mà backend đã có (remote có nhánh fix/adhoc-20261015-api-contract-sync); 19 lỗi ruff ở catalog/*, runtime/*, worker.py, tests/unit/test_catalog_crud.py
 Log: evidence/test-unit-2.log, evidence/implement-final-backend-2.log</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="239" customHeight="1">
-      <c r="A55" s="22" t="inlineStr">
+    <row r="58" ht="239" customHeight="1">
+      <c r="A58" s="22" t="inlineStr">
         <is>
           <t>BUG-REGDOSE-01</t>
         </is>
       </c>
-      <c r="B55" s="22" t="inlineStr">
+      <c r="B58" s="22" t="inlineStr">
         <is>
           <t>Đối chiếu scheduled_at có giây khi xác nhận liều</t>
         </is>
       </c>
-      <c r="C55" s="22" t="inlineStr">
+      <c r="C58" s="22" t="inlineStr">
         <is>
           <t>1. Từ backend chạy .venv/Scripts/python.exe -m pytest tests/integration/test_dose_confirmation_api.py::test_post_doses_batch_creates_dose_log_for_authenticated_patient__AC1_AC10_AC18 -q -ra.
 2. Fixture POST /doses/batch với danh sách một item ở Test Data.
 3. Đối chiếu items[0].scheduled_at với kỳ vọng test hiện có.</t>
         </is>
       </c>
-      <c r="D55" s="22" t="inlineStr">
+      <c r="D58" s="22" t="inlineStr">
         <is>
           <t>client_uuid: UUID mới; schedule_id: fixture; scheduled_at=2026-10-02T01:00:59.999Z; taken_at=2026-10-02T01:05:59.999Z</t>
         </is>
       </c>
-      <c r="E55" s="22" t="inlineStr">
+      <c r="E58" s="22" t="inlineStr">
         <is>
           <t>Theo test hiện có: HTTP 200, synced, da_uong và scheduled_at=2026-10-02T01:00:00Z.</t>
         </is>
       </c>
-      <c r="F55" s="22" t="inlineStr">
+      <c r="F58" s="22" t="inlineStr">
         <is>
           <t>HTTP 200, synced, da_uong; scheduled_at=2026-10-02T01:00:59.999000Z. Fail trong suite DB và lặp lại khi chạy riêng (1 failed trong 1.67s).</t>
         </is>
       </c>
-      <c r="G55" s="22" t="inlineStr">
+      <c r="G58" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H55" s="22" t="inlineStr">
+      <c r="H58" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I55" s="22" t="inlineStr">
+      <c r="I58" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn kỳ vọng chuẩn hóa tới phút trong test không khớp hành vi giữ thời điểm của API; chưa xác định phía nào sai theo contract/nghiệp vụ. Chưa chứng minh mất/trùng bản ghi liều; mức Medium tạm thời cho sai khác test, phải nâng tối thiểu High nếu xác nhận mất/trùng liều.
 Log: evidence/test-integration-db.log; evidence/test-dose-mismatch-repeat.log</t>
@@ -9364,17 +12922,17 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:A5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11:F22">
+  <conditionalFormatting sqref="F11:F25">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11:G22">
+  <conditionalFormatting sqref="G11:G25">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>OR(G11="Critical",G11="High")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G47:G55">
+  <conditionalFormatting sqref="G50:G58">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
@@ -9386,10 +12944,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G11:G22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G11:G25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="G47:G55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G50:G58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(testing): add LINKAPPROVE and CAREGIVER test cases
Two new sheets in Test_Cases.xlsx for the family link approval and
caregiver management features (27 + 28 test cases); Report rebuilt.

Refs: adhoc-20261020-family-link-approval

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -21,7 +21,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo dõi người thân (app)" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Link mời người thân" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Khung điều hướng app" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Duyệt yêu cầu liên kết" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Người giám sát" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Android build'!$A$8:$I$17</definedName>
@@ -39,6 +41,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Theo dõi người thân (app)'!$A$8:$I$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Link mời người thân'!$A$8:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Khung điều hướng app'!$A$8:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Duyệt yêu cầu liên kết'!$A$8:$I$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Người giám sát'!$A$8:$I$36</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -377,12 +381,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$25</f>
+              <f>'Report'!$A$11:$A$27</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$11:$D$25</f>
+              <f>'Report'!$D$11:$D$27</f>
             </numRef>
           </val>
         </ser>
@@ -401,12 +405,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$25</f>
+              <f>'Report'!$A$11:$A$27</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$11:$E$25</f>
+              <f>'Report'!$E$11:$E$27</f>
             </numRef>
           </val>
         </ser>
@@ -425,12 +429,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$25</f>
+              <f>'Report'!$A$11:$A$27</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$11:$F$25</f>
+              <f>'Report'!$F$11:$F$27</f>
             </numRef>
           </val>
         </ser>
@@ -533,7 +537,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>29</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -555,7 +559,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>29</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3240000"/>
@@ -11575,7 +11579,3537 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:T41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Duyệt yêu cầu liên kết người thân (LINKAPPROVE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>BS-04: người thân gửi lại yêu cầu</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="74" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Xem danh sách yêu cầu đang chờ của chính mình</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Patient P có 2 yêu cầu pending từ F1 (gửi trước) và F2 (gửi sau); có thêm yêu cầu pending gửi cho patient khác</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập bằng P
+2. GET /family/links?status=pending</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>status=pending</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>200; items gồm đúng 2 mục theo thứ tự F2, F1; mỗi mục chỉ có link_id, family_user_id, family_full_name, status=pending, requested_at; có audit list_pending/allowed</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · test_list_own_pending_minimal_order_without_consents__AC12_AC13 · evidence/test-integration.log</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>family_user_id (body approve)</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>UUID đúng người gửi yêu cầu</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>UUID của người khác
+không phải UUID</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>4
+5</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Số lần bị cùng patient từ chối liên tiếp (từ lần chấp thuận gần nhất)</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>0–4</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="57.5" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Xem danh sách khi không có yêu cầu nào</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Patient không có yêu cầu pending</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /family/links?status=pending</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>status=pending</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>200; {"items": []}</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>200; {"items": []}</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · test_list_pending_empty_returns_200_items_empty__AC13 · evidence/test-integration.log</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>consent_confirmed</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>true (boolean)</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>false
+thiếu field
+"true" (chuỗi)</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>6
+7
+8</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>Còn trong 24 giờ kể từ lần từ chối thứ 5?</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90.5" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Gửi query lạ khi xem danh sách (patient_id)</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Patient đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /family/links?status=pending&amp;patient_id=&lt;UUID khác&gt;</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>patient_id=&lt;UUID patient khác&gt;</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>422 ValidationError; không gọi use case</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · Đoán lỗi (truy cập dữ liệu người khác) · test_list_rejects_missing_invalid_duplicate_or_extra_query · evidence/implement-final-backend.log</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>document_version</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-v1 (bản hiện hành)</t>
+        </is>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>(blank)
+a*65
+phiên bản khác bản hiện hành</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>9
+10
+11</t>
+        </is>
+      </c>
+      <c r="Q11" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T11" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="107" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Chấp thuận yêu cầu với xác nhận đồng ý hợp lệ</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>P đã đồng ý family_sharing 2026-10-v1; có link pending từ F</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập bằng P
+2. POST /family/links/{link_id}/approve</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>{"family_user_id": "&lt;F&gt;", "consent_confirmed": true, "document_version": "2026-10-v1"}</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>200; status=active, sharing_enabled=false, consent_confirmation.purpose=family_sharing; đúng 1 dòng family_link_consent_confirmations; link rời danh sách chờ và có trong GET /family/caregivers</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · EP (1,2,3) · test_approve_success_persists_evidence_and_activates_link__AC2, test_approved_link_moves_from_pending_to_caregivers__AC3 · evidence/test-integration.log</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
+        <is>
+          <t>201: tạo yêu cầu mới (pending)</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S12" s="11" t="inlineStr"/>
+      <c r="T12" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="74" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Chấp thuận thay bởi người thân, người lạ, admin hoặc sai family_user_id</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Link pending P←F; có người lạ X và tài khoản admin A</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. POST approve không token
+2. POST approve bằng token F, X, A
+3. POST approve bằng token P với family_user_id của X</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>family_user_id = &lt;F&gt; hoặc &lt;X&gt;</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>401 khi không token; 403 {"detail": "khong_co_quyen"} cho các trường hợp còn lại; link vẫn pending, không có bằng chứng; có audit denied</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · EP (4) · test_approve_denied_caller_matrix__AC4_AC10_AC16 · evidence/test-integration.log</t>
+        </is>
+      </c>
+      <c r="Q13" s="10" t="inlineStr">
+        <is>
+          <t>429 link_request_cooldown + Retry-After</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="inlineStr"/>
+      <c r="S13" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="90.5" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối thay bởi người thân, người lạ hoặc admin</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Link pending P←F; người lạ X; admin A</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /family/links/{link_id}/reject không token
+2. POST reject bằng token F, X, A
+3. POST reject bằng token P</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>(không có body)</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>401 khi không token; 403 khong_co_quyen với F, X, A, mỗi lượt đúng 1 audit reject/denied với actor là người gọi (admin không ghi patient/link); link vẫn pending; P từ chối được (200)</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · test_reject_denied_caller_matrix__AC5 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="74" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Chấp thuận khi patient chưa đồng ý hoặc đã rút family_sharing</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Link pending P←F; P không có consent family_sharing hiệu lực</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. POST approve bằng token P</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>body hợp lệ</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>403 {"detail": "consent_revoked"}; link vẫn pending; không có bằng chứng; audit approve/denied reason consent_revoked</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · test_approve_missing_or_revoked_patient_consent_403__AC3_AC10 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="74" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Chấp thuận với phiên bản văn bản cũ hoặc consent_confirmed=false</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Link pending P←F; P có family_sharing</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. POST approve với document_version khác bản hiện hành
+2. POST approve với consent_confirmed=false</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>document_version="wrong-version"; consent_confirmed=false</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail": "consent_document_outdated"}; 422 ValidationError; link vẫn pending</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (6,11) · test_approve_outdated_version_and_false_confirmation_422__AC3 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="107" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Gửi body chấp thuận sai cấu trúc</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Người gọi đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /family/links/1/approve với từng body sai</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>family_user_id="invalid"; thiếu consent_confirmed; consent_confirmed="true"; consent_confirmed=1; document_version=""; document_version="a"*65; field lạ patient_id</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>422 ValidationError cho mọi trường hợp; không gọi use case</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>422 cho mọi trường hợp</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (5,7,8,9,10) · BVA (min-1, max+1) · test_strict_approval_body_rejected_before_use_case · evidence/implement-final-backend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="57.5" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-BVA-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Chấp thuận với document_version dài 1 ký tự (biên dưới hợp lệ của độ dài)</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Link pending P←F; P có family_sharing</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. POST approve bằng token P</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>document_version="a"</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail": "consent_document_outdated"} (đúng độ dài nhưng không phải bản hiện hành); link vẫn pending</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr"/>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · BVA (min) · chưa có test riêng, cần chạy tay</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="41" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-BVA-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Chấp thuận với document_version dài 64 ký tự (biên trên hợp lệ của độ dài)</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Link pending P←F; P có family_sharing</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. POST approve bằng token P</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>document_version="a"*64</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail": "consent_document_outdated"}; link vẫn pending</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr"/>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · BVA (max) · chưa có test riêng, cần chạy tay</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="74" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Gửi lại chấp thuận với cùng nội dung</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Link đã được P chấp thuận</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. POST approve lần 2 với cùng body</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>body giống lần 1</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>200; cùng id/confirmed_at bằng chứng cũ; không thêm bằng chứng</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · Đoán lỗi (gửi trùng) · test_approve_replay_idempotent_with_same_evidence__AC5_AC9 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="90.5" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-13</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Chấp thuận liên kết đã bị từ chối hoặc đã hủy</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Link ở trạng thái rejected hoặc revoked</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. POST approve bằng token P</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>body hợp lệ</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>409 {"detail": "invalid_link_transition"}; trạng thái giữ nguyên</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · Chuyển trạng thái (chuyển bị cấm) · test_approve_rejected_or_revoked_conflict_409__AC8 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="90.5" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-14</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối yêu cầu đang chờ và gửi lại lệnh từ chối</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Link pending P←F; P không cần consent</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. POST reject bằng token P
+2. POST reject lần 2</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>(không có body)</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>200 status=rejected, có rejected_at; lần 2 trả 200 cùng rejected_at</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · Chuyển trạng thái (pending→rejected) · test_reject_without_consent_and_replay_idempotent__AC14_AC15 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="74" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối liên kết đang active hoặc đã hủy</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Link active hoặc revoked</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. POST reject bằng token P</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>(không có body)</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>409 {"detail": "invalid_link_transition"}</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · Chuyển trạng thái (chuyển bị cấm) · test_reject_active_or_revoked_conflict_409__AC15 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="74" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-16</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Chấp thuận và từ chối cùng lúc một yêu cầu</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Link pending P←F</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi đồng thời POST approve và POST reject bằng token P</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>body approve hợp lệ</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Một request 200, request kia 409; không có trạng thái vừa rejected vừa có bằng chứng</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>AC15 · Đoán lỗi (chạy đua) · test_concurrent_approve_and_reject_one_wins_other_409__AC17 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="123.5" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-17</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Gửi lại yêu cầu sau 5 lần bị từ chối liên tiếp qua endpoint thật</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>P có family_sharing và mã liên kết; F chưa liên kết</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. F gửi yêu cầu bằng mã của P, P từ chối; lặp 4 lần (lần 5 vẫn gửi được)
+2. P từ chối lần thứ 5
+3. F gửi lại ngay
+4. Người thân khác gửi yêu cầu
+5. Đặt giờ app = rejected_at lần 5 + 23h59
+6. Đặt giờ app = rejected_at lần 5 + 24h</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>client_uuid mới mỗi lần</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Lần 1–5: 201; sau lần từ chối thứ 5: 429 {"detail": "link_request_cooldown"}, Retry-After trong (0, 86400]; người thân khác 201; tại +23h59: 429; tại +24h: 201</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · Decision Table (R1, R2, R3) · BVA (24h-1 phút, 24h) · test_five_rejections_via_endpoint_block_24h_others_unaffected__AC9 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="74" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-18</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Chấp thuận rồi hủy liên kết làm bộ đếm từ chối về 0</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>P có family_sharing và mã liên kết; F chưa liên kết</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. Từ chối 4 lần qua endpoint
+2. F gửi, P chấp thuận, P hủy liên kết
+3. Từ chối thêm 4 lần
+4. F gửi lần thứ 10 trong ngày</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>client_uuid mới mỗi lần</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Lần gửi cuối 201 (không bị chặn); các dòng theo thứ tự: 4 rejected, 1 revoked, 4 rejected, 1 pending</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · Decision Table (R1) · test_approval_then_revoke_resets_streak_via_endpoints__AC9 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="90.5" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-19</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Hiện mục Yêu cầu theo dõi bạn trên tab Người thân</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>App mobile; có 2 yêu cầu pending, 1 người gửi không có tên</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở tab Người thân
+2. Kéo xuống để tải lại</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>requested_at = 2026-10-15T02:00:00Z</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Hiện "Yêu cầu theo dõi bạn (2)"; tên người thân và "Người dùng DrugTime" cho người không có tên; "Gửi lúc 09:00 15/10/2026"; kéo xuống gọi lại API; không có yêu cầu thì không hiện mục</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AC16 · incoming_requests_test.dart (AC16) · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="57.5" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-20</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Chuyển sang tab Người thân thì tải lại yêu cầu đang chờ</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>App mở ở tab Thuốc</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạm tab Người thân
+2. Chuyển sang tab Thuốc
+3. Chạm lại tab Người thân</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lần mở tab Người thân gọi listPendingRequests một lần; trước khi mở tab thì không gọi</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AC16 · app_shell_test.dart (AC16) · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="123.5" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-21</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Chấp thuận trên app qua bước xác nhận đồng ý</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Có yêu cầu từ Nguyễn Văn An</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Chấp thuận
+2. Kiểm nút Chấp thuận khi chưa tick
+3. Tick "Tôi đồng ý chia sẻ…" và bấm Chấp thuận
+4. Ở hộp "Đã liên kết…" chọn Để sau (lần khác chọn Bật chia sẻ)
+5. Lần khác: mở bước xác nhận rồi bấm Hủy</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>consentDocumentVersion = 2026-10-v1</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Hiện văn bản family_sharing và "Chia sẻ với: Nguyễn Văn An"; chưa tick thì nút khóa; gửi approve đúng family_user_id và 2026-10-v1; mục biến mất; Để sau không bật chia sẻ, Bật chia sẻ gọi API và báo "Đã bật chia sẻ với Nguyễn Văn An."; Hủy không gọi API</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>AC17 · incoming_requests_test.dart (AC17) · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="74" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-22</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối trên app có hộp xác nhận</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Có yêu cầu từ Nguyễn Văn An</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Từ chối rồi Hủy
+2. Bấm Từ chối rồi xác nhận Từ chối</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Hủy không gọi API; xác nhận thì gửi reject không body, mục biến mất, báo "Đã từ chối yêu cầu của Nguyễn Văn An."</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>AC18 · incoming_requests_test.dart (AC18), api_client_test.dart (post không body) · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="57.5" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-23</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Nhắc bật chia sẻ khi patient chưa đồng ý family_sharing</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Tài khoản chưa bật family_sharing; có yêu cầu đang chờ</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở tab Người thân
+2. Bấm "Mở Quyền riêng tư"</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Có dải nhắc "Cần bật \"Chia sẻ với người thân\"…"; bấm nút mở màn Quyền riêng tư; đã bật thì không có dải nhắc</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>AC19 · incoming_requests_test.dart (AC19) · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="90.5" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-24</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Xử lý lỗi khi chấp thuận trên app</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Có yêu cầu đang chờ; server trả lỗi</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>1. Chấp thuận khi server trả lần lượt 403 consent_revoked, 409, 404, 422 consent_document_outdated, lỗi mạng</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Báo đúng câu cho từng lỗi; không hiện hộp bật chia sẻ; tải lại danh sách; yêu cầu vẫn còn</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>AC22 · Đoán lỗi (mất mạng) · incoming_requests_test.dart (AC22), remote_caregiver_repository_test.dart · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="74" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-25</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Bấm liên tục khi đang gửi thao tác</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Có yêu cầu đang chờ; server phản hồi chậm</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>1. Xác nhận từ chối
+2. Trong lúc chờ bấm lại Từ chối</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Hai nút của mục bị khóa khi đang gửi; chỉ một request reject được gửi</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>AC22 · Đoán lỗi (bấm liên tục) · incoming_requests_test.dart (AC22) · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="74" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-26</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Chấp thuận yêu cầu thật trên hai thiết bị</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Hai tài khoản trên hai máy, backend đang chạy; P đã bật family_sharing</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>1. F nhập/quét mã của P
+2. P mở tab Người thân, thấy yêu cầu
+3. P chấp thuận, tick đồng ý, chọn Bật chia sẻ
+4. F gửi lại mã</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Mã liên kết của P</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>P thấy yêu cầu đúng tên F; sau chấp thuận F có trong Người giám sát với chia sẻ bật; F gửi lại mã nhận thông báo đã liên kết (409 already_linked)</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr"/>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>AC23 · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="57.5" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>TC-LINKAPPROVE-27</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối yêu cầu thật trên hai thiết bị</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Hai tài khoản trên hai máy, backend đang chạy</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>1. F gửi yêu cầu bằng mã của P
+2. P từ chối
+3. F gửi lại ngay</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Mã liên kết của P</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>Yêu cầu biến mất trên máy P; F gửi lại được ngay (201) khi chưa đủ 5 lần bị từ chối</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr"/>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>AC23 · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38">
+      <c r="G38" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H38" s="13">
+        <f>COUNTIF(H9:H35,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="G39" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H39" s="13">
+        <f>COUNTIF(H9:H35,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="G40" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H40" s="13">
+        <f>COUNTIF(H9:H35,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="G41" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H41" s="13">
+        <f>SUM(H38:H40)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I35"/>
+  <conditionalFormatting sqref="H9:H35">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Quản lý người giám sát (CAREGIVER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Người thân đọc dữ liệu sức khỏe / nhận cảnh báo của patient</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="123.5" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Xem danh sách người giám sát của chính mình</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>P có 2 liên kết chấp thuận qua API (F1 bật chia sẻ, F2 chấp thuận sau), 1 liên kết cũ không bằng chứng (F3), và các liên kết pending/rejected/revoked; có liên kết của patient khác</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập bằng P
+2. GET /family/caregivers</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>200; items theo thứ tự F2, F1, F3; mỗi mục đúng 6 field, status=active; F1 sharing_enabled=true; F3 approved_at=null; không có liên kết khác; audit list_caregivers/allowed không có link_id</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · test_list_only_own_active_ordered_minimal__AC11 · evidence/test-integration.log</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>sharing_enabled (body PATCH)</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>true
+false</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1
+2</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>"true" (chuỗi)
+1
+null
+thiếu field
+field lạ (patient_id)</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>4
+5
+6
+7
+8</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Liên kết active?</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="U9" s="11" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="140" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Xem danh sách khi chưa có người giám sát</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Tài khoản không có liên kết active</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /family/caregivers</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>200; {"items": []}</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>200; {"items": []}</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC11 · test_empty_list_returns_items_empty__AC11 · evidence/test-integration.log</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>link_id (path)</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>id liên kết active của chính mình</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>0
+-1
+abc
+9223372036854775808
+id không tồn tại
+liên kết của patient khác
+liên kết không active (pending/rejected/revoked)</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>9
+10
+11
+12
+13
+14
+15</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>Công tắc chia sẻ bật?</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="U10" s="11" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90.5" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Gửi query patient_id để xem người giám sát của người khác</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. GET /family/caregivers?patient_id=&lt;UUID khác&gt;</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>patient_id=&lt;UUID&gt;</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · Đoán lỗi (truy cập dữ liệu người khác) · test_caregivers_rejects_query_parameters__AC11 · evidence/test-integration.log</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>Patient còn đồng ý family_sharing?</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T11" s="11" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="U11" s="11" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="74" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Bật, bật lại và tắt chia sẻ</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Liên kết active chấp thuận qua API, chia sẻ đang tắt; P có family_sharing</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH /family/links/{id}/sharing true
+2. PATCH lại true
+3. PATCH false</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>{"sharing_enabled": true} / {"sharing_enabled": false}</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>200 trả Caregiver với sharing_enabled đúng giá trị; gửi lại true trả kết quả giống hệt; DB đổi theo; audit enable_sharing x2, disable_sharing</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · EP (1,2,3) · Đoán lỗi (gửi trùng) · test_enable_disable_idempotent_and_audit__AC12 · evidence/test-integration.log</t>
+        </is>
+      </c>
+      <c r="Q12" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="57.5" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Tắt chia sẻ khi đã rút family_sharing</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Liên kết active đang chia sẻ; P đã rút family_sharing</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH sharing false</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>{"sharing_enabled": false}</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>200; sharing_enabled=false</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC12 · test_disable_allowed_without_consent__AC12 · evidence/test-integration.log</t>
+        </is>
+      </c>
+      <c r="Q13" s="10" t="inlineStr">
+        <is>
+          <t>403 + access_logs denied; không có trong danh sách nhận cảnh báo</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S13" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T13" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="74" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Bật chia sẻ khi chưa đồng ý family_sharing</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Liên kết active, chia sẻ tắt; P đã rút family_sharing</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH sharing true</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>{"sharing_enabled": true}</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>403 {"detail": "consent_revoked"}; công tắc vẫn tắt; audit enable_sharing/denied reason consent_revoked</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC7, AC10 · test_enable_without_consent_403_denied_audit__AC7_AC10 · evidence/test-integration.log</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>200 + access_logs allowed; có trong danh sách nhận cảnh báo</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr"/>
+      <c r="S14" s="11" t="inlineStr"/>
+      <c r="T14" s="11" t="inlineStr"/>
+      <c r="U14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="74" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Bật chia sẻ cho liên kết cũ không có bằng chứng xác nhận</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Liên kết active tạo trước 3.16 (không có bằng chứng), chia sẻ bật</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH sharing true
+2. PATCH sharing false</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>true: 409 {"detail": "consent_confirmation_missing"}; false: 200, approved_at=null</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · test_enable_legacy_link_409_confirmation_missing_but_disable_ok__AC10 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="90.5" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Bật/tắt chia sẻ cho liên kết không active</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Liên kết pending, rejected hoặc revoked</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH sharing true và false cho từng trạng thái</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>6 tổ hợp trạng thái × giá trị</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>409 {"detail": "family_link_not_active"}; dòng liên kết không đổi</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi (6/6)</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · EP (15) · Chuyển trạng thái (thao tác bị cấm) · test_sharing_on_non_active_link_409__AC10 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="74" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Gửi body bật/tắt chia sẻ sai cấu trúc</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH /family/links/1/sharing với từng body sai</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>(không body); {}; "true" (chuỗi); 1; null; {"sharing_enabled": true, "patient_id": "…"}</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>422 ValidationError; không gọi use case</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>422 cho mọi trường hợp</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC22 · EP (4,5,6,7,8) · test_strict_sharing_body_rejected_before_use_case · evidence/implement-final-backend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="74" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Gọi bật/tắt chia sẻ và hủy với link_id không hợp lệ</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH /family/links/{link_id}/sharing
+2. POST /family/links/{link_id}/revoke</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>link_id = 0, -1, abc, 1.1, 9223372036854775808</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>422 cho mọi giá trị</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC22 · EP (9,10,11,12) · BVA (min-1) · test_new_routes_invalid_path_id_is_422 · evidence/implement-final-backend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="74" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Thao tác trên liên kết không tồn tại</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>P đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH sharing true cho id 2000000000
+2. POST revoke cho id 2000000000</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>link_id=2000000000</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>404 {"detail": "family_link_not_found"}; không ghi audit</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · EP (13) · test_missing_link_404_without_allowed_audit__AC10 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="107" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Người thân, người lạ, admin bật/tắt chia sẻ hoặc hủy liên kết thay patient</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Liên kết active P←F đang chia sẻ; người lạ X; admin A</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. Gọi 3 endpoint không token
+2. Với F, X, A: PATCH false, PATCH true, POST revoke
+3. A gọi GET /family/caregivers
+4. F, X gọi GET /family/caregivers
+5. P gọi POST revoke</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>401 khi không token; 403 khong_co_quyen, liên kết không đổi, mỗi lượt 1 audit denied với actor là người gọi (admin không ghi patient/link); admin xem danh sách 403; F và X thấy items rỗng; P hủy được (200)</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · EP (14) · test_new_endpoints_denied_caller_matrix__AC5 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="90.5" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-13</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Hủy liên kết và gửi lại lệnh hủy</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Liên kết active đang chia sẻ</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. POST /family/links/{id}/revoke
+2. POST revoke lần 2
+3. GET /family/caregivers</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>(không body)</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>200 {link_id, family_user_id, status: revoked, revoked_at}; lần 2 trả y hệt; bằng chứng đồng ý vẫn còn 1 dòng; audit revoke x2; danh sách rỗng</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AC13 · Chuyển trạng thái (active→revoked) · test_revoke_keeps_history_and_replay_returns_same_time__AC13 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="74" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-14</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Liên kết lại sau khi hủy</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Liên kết đã chấp thuận, bật chia sẻ, rồi bị hủy</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. F gửi lại yêu cầu bằng mã của P
+2. P chấp thuận</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>client_uuid mới</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>201 tạo liên kết mới pending (id khác); sau chấp thuận sharing_enabled=false; bằng chứng mới riêng, bằng chứng cũ còn; liên kết cũ vẫn revoked</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AC13 · test_relink_after_revoke_starts_unshared_with_new_evidence__AC13 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="74" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Hủy liên kết đang chờ hoặc đã bị từ chối</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Liên kết pending hoặc rejected</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. POST revoke</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>409 {"detail": "invalid_link_transition"}; liên kết không đổi</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · Chuyển trạng thái (chuyển bị cấm) · test_revoke_pending_or_rejected_409__AC10 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="57.5" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-16</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Gửi body khi hủy liên kết</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Liên kết active</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. POST revoke với body {}</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>422; liên kết vẫn active</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · Đoán lỗi · test_revoke_with_body_is_422__AC10 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="123.5" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-17</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Mỗi quyết định của patient có hiệu lực ngay ở request kế tiếp của người thân</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>P có health_data và family_sharing, có một thuốc; F dùng một token duy nhất</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. F gửi yêu cầu (pending) → F đọc GET /medications/{id}
+2. P chấp thuận → F đọc
+3. P bật chia sẻ → F đọc
+4. P tắt chia sẻ → F đọc
+5. P bật lại → F đọc, P hủy liên kết → F đọc
+6. F gửi lại, P từ chối → F đọc</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>403 + access_logs denied ở pending, chấp thuận (chia sẻ tắt), tắt chia sẻ, hủy, từ chối; 200 + allowed (actor_role family) khi đang chia sẻ; danh sách nhận cảnh báo (authorized_caregivers) có F đúng khi được 200</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · Decision Table (R1, R2, R4) · test_every_decision_applies_on_next_request_same_token__AC6 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="74" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-18</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Rút family_sharing khi công tắc vẫn bật</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Liên kết active đang chia sẻ, F đọc được</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. P rút family_sharing
+2. F đọc GET /medications/{id} ngay</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>403 + access_logs denied; F không còn trong danh sách nhận cảnh báo; công tắc không tự đổi</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · Decision Table (R3) · test_consent_withdrawal_blocks_even_with_sharing_on__AC6 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="74" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-19</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Hủy liên kết và bật chia sẻ cùng lúc</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Liên kết active, chia sẻ tắt; giữ khóa dòng để hai request cùng chờ</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi đồng thời PATCH sharing true và POST revoke
+2. Nhả khóa
+3. F đọc dữ liệu</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Revoke 200; PATCH 200 hoặc 409 family_link_not_active; trạng thái cuối revoked; F nhận 403 + denied</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi (chạy 5 lần đều pass)</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AC15 · Đoán lỗi (chạy đua) · test_concurrent_revoke_and_enable_sharing_ends_revoked__AC15 · evidence/test-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="107" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-20</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm migration audit cho thao tác mới</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>DB reset sạch (supabase db reset)</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. Chèn audit list_caregivers không link_id
+2. Chèn enable_sharing/disable_sharing/revoke allowed và denied
+3. Chèn operation lạ
+4. Chèn allowed gắn link không có link_id
+5. UPDATE/DELETE/TRUNCATE với mọi role</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>operation = update_sharing, delete, LIST_CAREGIVERS, (blank)</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Operation mới được nhận; operation lạ và allowed gắn link thiếu link_id bị từ chối; mọi role không sửa/xóa được; ràng buộc đúng định nghĩa migration</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi (32 test)</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AC14 · test_migration_family_link_audit_operations.py · evidence/test-integration.log, evidence/test-db-reset.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="74" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-21</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Mở màn Người giám sát từ Hồ sơ</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>App mobile; có 2 người giám sát (1 không tên, 1 liên kết cũ)</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. Hồ sơ &gt; Người giám sát</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>approved_at = 2026-10-14T18:00:00Z</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Không còn "Sắp ra mắt"; hiện tên, "Chấp thuận ngày 15/10/2026", "Người dùng DrugTime", "Liên kết trước khi có bước xác nhận đồng ý", công tắc đúng giá trị</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>AC20 · caregivers_screen_test.dart (AC20), profile_screens_test.dart (AC20) · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="74" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-22</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Màn trống: bấm Mở tab Người thân</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Chưa có người giám sát</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>1. Hồ sơ &gt; Người giám sát
+2. Bấm "Mở tab Người thân"</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Hiện "Chưa có người giám sát"; bấm nút thì đóng màn, shell chuyển sang tab Người thân và tải yêu cầu đang chờ</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>AC20 · app_shell_test.dart (AC20), caregivers_screen_test.dart · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="74" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-23</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Gạt công tắc chia sẻ trên app</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Có người giám sát</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>1. Gạt công tắc
+2. Trong lúc chờ gạt lại
+3. Lần khác: server trả lỗi mạng</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Công tắc và nút hủy khóa khi đang gửi, chỉ 1 request; hiện giá trị server trả và báo "Đã bật/tắt chia sẻ với …"; lỗi mạng thì giữ giá trị cũ và báo lỗi</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>AC21 · Đoán lỗi (bấm liên tục, mất mạng) · caregivers_screen_test.dart (AC21) · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="90.5" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-24</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Hủy liên kết trên app có hộp xác nhận</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Có người giám sát Nguyễn Văn An</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Hủy liên kết rồi Giữ liên kết
+2. Bấm Hủy liên kết rồi xác nhận</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Hộp nêu người thân mất quyền xem ngay và phải gửi yêu cầu mới; giữ thì không gọi API; xác nhận thì gọi revoke rồi tải lại, mục biến mất, báo "Đã hủy liên kết với Nguyễn Văn An."</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>AC21 · caregivers_screen_test.dart (AC21) · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="57.5" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-25</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Chưa bật family_sharing: chỉ tắt được, không bật được</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Tài khoản chưa bật family_sharing; 1 người giám sát đang tắt, 1 đang bật</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở màn Người giám sát
+2. Bấm "Mở Quyền riêng tư"</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Có dải nhắc; công tắc đang tắt bị khóa, công tắc đang bật vẫn tắt được; nút mở màn Quyền riêng tư</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>AC19 · caregivers_screen_test.dart (AC19) · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="57.5" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-26</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Xử lý lỗi khi bật chia sẻ trên app</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Có người giám sát; server trả lỗi</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>1. Bật chia sẻ khi server trả lần lượt 403 consent_revoked, 409, 404, 409 consent_confirmation_missing, lỗi mạng</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>Báo đúng câu cho từng lỗi; công tắc giữ giá trị cũ; 409/404 thì tải lại danh sách</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>AC22 · caregivers_screen_test.dart (AC22) · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="57.5" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-27</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Mở lại màn và kéo xuống luôn gọi lại API</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Có người giám sát</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>1. Kéo xuống
+2. Đóng rồi mở lại màn</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lần gọi lại listCaregivers; không dùng dữ liệu cũ</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>AC22 · caregivers_screen_test.dart (AC20, AC22) · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="90.5" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-28</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Bật/tắt chia sẻ và hủy liên kết thật trên hai thiết bị</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>P và F đã liên kết, chia sẻ bật; backend đang chạy</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>1. F mở dữ liệu thuốc của P
+2. P tắt chia sẻ ở Hồ sơ &gt; Người giám sát
+3. F tải lại
+4. P bật lại rồi Hủy liên kết
+5. F tải lại; F gửi lại mã</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>F xem được khi đang chia sẻ; sau khi tắt hoặc hủy, lần tải kế tiếp F bị từ chối; sau khi hủy F gửi lại mã tạo được yêu cầu mới</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr"/>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>AC23 · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39">
+      <c r="G39" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H39" s="13">
+        <f>COUNTIF(H9:H36,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="G40" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H40" s="13">
+        <f>COUNTIF(H9:H36,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="G41" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H41" s="13">
+        <f>COUNTIF(H9:H36,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="G42" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H42" s="13">
+        <f>SUM(H39:H41)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I36"/>
+  <conditionalFormatting sqref="H9:H36">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11625,7 +15159,7 @@
         </is>
       </c>
       <c r="C3" s="11">
-        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59+'Lịch uống thuốc'!$H$51+'Tải lịch uống'!$H$32+'Tương tác thuốc-thuốc'!$H$52+'Tương tác thuốc-thực phẩm'!$H$17+'Tra cứu hoạt chất'!$H$17+'Mã liên kết người thân'!$H$47+'Landing page'!$H$43+'Yêu cầu liên kết người thân'!$H$72+'Theo dõi người thân (app)'!$H$46+'Link mời người thân'!$H$24+'Khung điều hướng app'!$H$16</f>
+        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59+'Lịch uống thuốc'!$H$51+'Tải lịch uống'!$H$32+'Tương tác thuốc-thuốc'!$H$52+'Tương tác thuốc-thực phẩm'!$H$17+'Tra cứu hoạt chất'!$H$17+'Mã liên kết người thân'!$H$47+'Landing page'!$H$43+'Yêu cầu liên kết người thân'!$H$72+'Theo dõi người thân (app)'!$H$46+'Link mời người thân'!$H$24+'Khung điều hướng app'!$H$16+'Duyệt yêu cầu liên kết'!$H$38+'Người giám sát'!$H$39</f>
         <v/>
       </c>
       <c r="D3" s="11">
@@ -11645,7 +15179,7 @@
         </is>
       </c>
       <c r="C4" s="11">
-        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60+'Lịch uống thuốc'!$H$52+'Tải lịch uống'!$H$33+'Tương tác thuốc-thuốc'!$H$53+'Tương tác thuốc-thực phẩm'!$H$18+'Tra cứu hoạt chất'!$H$18+'Mã liên kết người thân'!$H$48+'Landing page'!$H$44+'Yêu cầu liên kết người thân'!$H$73+'Theo dõi người thân (app)'!$H$47+'Link mời người thân'!$H$25+'Khung điều hướng app'!$H$17</f>
+        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60+'Lịch uống thuốc'!$H$52+'Tải lịch uống'!$H$33+'Tương tác thuốc-thuốc'!$H$53+'Tương tác thuốc-thực phẩm'!$H$18+'Tra cứu hoạt chất'!$H$18+'Mã liên kết người thân'!$H$48+'Landing page'!$H$44+'Yêu cầu liên kết người thân'!$H$73+'Theo dõi người thân (app)'!$H$47+'Link mời người thân'!$H$25+'Khung điều hướng app'!$H$17+'Duyệt yêu cầu liên kết'!$H$39+'Người giám sát'!$H$40</f>
         <v/>
       </c>
       <c r="D4" s="11">
@@ -11685,7 +15219,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr"/>
       <c r="C6" s="11">
-        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61+'Lịch uống thuốc'!$H$53+'Tải lịch uống'!$H$34+'Tương tác thuốc-thuốc'!$H$54+'Tương tác thuốc-thực phẩm'!$H$19+'Tra cứu hoạt chất'!$H$19+'Mã liên kết người thân'!$H$49+'Landing page'!$H$45+'Yêu cầu liên kết người thân'!$H$74+'Theo dõi người thân (app)'!$H$48+'Link mời người thân'!$H$26+'Khung điều hướng app'!$H$18</f>
+        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61+'Lịch uống thuốc'!$H$53+'Tải lịch uống'!$H$34+'Tương tác thuốc-thuốc'!$H$54+'Tương tác thuốc-thực phẩm'!$H$19+'Tra cứu hoạt chất'!$H$19+'Mã liên kết người thân'!$H$49+'Landing page'!$H$45+'Yêu cầu liên kết người thân'!$H$74+'Theo dõi người thân (app)'!$H$48+'Link mời người thân'!$H$26+'Khung điều hướng app'!$H$18+'Duyệt yêu cầu liên kết'!$H$40+'Người giám sát'!$H$41</f>
         <v/>
       </c>
       <c r="D6" s="11">
@@ -12424,493 +15958,581 @@
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="19" t="inlineStr">
+    <row r="26" ht="107" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>Duyệt yêu cầu liên kết người thân</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Patient xem yêu cầu theo dõi đang chờ, chấp thuận kèm xác nhận đồng ý chia sẻ (PB16/3.17) hoặc từ chối; BS-04 chặn gửi lại sau 5 lần bị từ chối. Backend /family/links*, mobile tab Người thân.</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>Duyệt yêu cầu liên kết</t>
+        </is>
+      </c>
+      <c r="D26" s="18">
+        <f>IFERROR(('Duyệt yêu cầu liên kết'!$H$41-'Duyệt yêu cầu liên kết'!$H$40)/'Duyệt yêu cầu liên kết'!$H$41,0)</f>
+        <v/>
+      </c>
+      <c r="E26" s="18">
+        <f>IFERROR('Duyệt yêu cầu liên kết'!$H$38/'Duyệt yêu cầu liên kết'!$H$41,0)</f>
+        <v/>
+      </c>
+      <c r="F26" s="18">
+        <f>IFERROR('Duyệt yêu cầu liên kết'!$H$39/'Duyệt yêu cầu liên kết'!$H$41,0)</f>
+        <v/>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động (tích hợp Postgres thật, unit, widget) pass trong phiên 2026-10-21. Còn Pending: 2 điểm biên độ dài document_version chưa có test riêng và 2 kịch bản chạy tay trên hai thiết bị (AC23).</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="123.5" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Quản lý người giám sát</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Patient xem người giám sát đã chấp thuận, bật/tắt chia sẻ từng người và hủy liên kết; quyết định có hiệu lực ngay ở request kế tiếp. Backend /family/caregivers, /family/links/{id}/sharing|revoke, migration audit; mobile Hồ sơ &gt; Người giám sát.</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>Người giám sát</t>
+        </is>
+      </c>
+      <c r="D27" s="18">
+        <f>IFERROR(('Người giám sát'!$H$42-'Người giám sát'!$H$41)/'Người giám sát'!$H$42,0)</f>
+        <v/>
+      </c>
+      <c r="E27" s="18">
+        <f>IFERROR('Người giám sát'!$H$39/'Người giám sát'!$H$42,0)</f>
+        <v/>
+      </c>
+      <c r="F27" s="18">
+        <f>IFERROR('Người giám sát'!$H$40/'Người giám sát'!$H$42,0)</f>
+        <v/>
+      </c>
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ test tự động (tích hợp Postgres thật gồm phân quyền chéo, hiệu lực ngay, chạy đua; unit; widget) pass trong phiên 2026-10-21. Còn Pending: kịch bản chạy tay trên hai thiết bị (AC23).</t>
+        </is>
+      </c>
+      <c r="I27" s="11" t="inlineStr">
+        <is>
+          <t>zannguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="19" t="inlineStr">
         <is>
           <t>Bug Report</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="20" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="20" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="B49" s="20" t="inlineStr">
+      <c r="B51" s="20" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C49" s="20" t="inlineStr">
+      <c r="C51" s="20" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="D49" s="20" t="inlineStr">
+      <c r="D51" s="20" t="inlineStr">
         <is>
           <t>Input Data</t>
         </is>
       </c>
-      <c r="E49" s="20" t="inlineStr">
+      <c r="E51" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F49" s="20" t="inlineStr">
+      <c r="F51" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="G49" s="20" t="inlineStr">
+      <c r="G51" s="20" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="H49" s="20" t="inlineStr">
+      <c r="H51" s="20" t="inlineStr">
         <is>
           <t>Name of Tester</t>
         </is>
       </c>
-      <c r="I49" s="20" t="inlineStr">
+      <c r="I51" s="20" t="inlineStr">
         <is>
           <t>Logs</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="123.5" customHeight="1">
-      <c r="A50" s="22" t="inlineStr">
+    <row r="52" ht="123.5" customHeight="1">
+      <c r="A52" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-08</t>
         </is>
       </c>
-      <c r="B50" s="22" t="inlineStr">
+      <c r="B52" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
         </is>
       </c>
-      <c r="C50" s="22" t="inlineStr">
+      <c r="C52" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
 2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
         </is>
       </c>
-      <c r="D50" s="22" t="inlineStr">
+      <c r="D52" s="22" t="inlineStr">
         <is>
           <t>phone: 0900000001 + ký tự \n</t>
         </is>
       </c>
-      <c r="E50" s="22" t="inlineStr">
+      <c r="E52" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F50" s="22" t="inlineStr">
+      <c r="F52" s="22" t="inlineStr">
         <is>
           <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
         </is>
       </c>
-      <c r="G50" s="22" t="inlineStr">
+      <c r="G52" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H50" s="22" t="inlineStr">
+      <c r="H52" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I50" s="22" t="inlineStr">
+      <c r="I52" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn — kỳ vọng AC6 mâu thuẫn AC5: backend `_validate_required_text` (sign_in.py:178) `strip()` mọi ký tự trắng hai đầu, nên \n cuối được xử lý như khoảng trắng hai đầu mà AC5 coi là hợp lệ. Cần người dùng chốt: sửa AC6 hoặc sửa backend
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="123.5" customHeight="1">
-      <c r="A51" s="22" t="inlineStr">
+    <row r="53" ht="123.5" customHeight="1">
+      <c r="A53" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-11</t>
         </is>
       </c>
-      <c r="B51" s="22" t="inlineStr">
+      <c r="B53" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
         </is>
       </c>
-      <c r="C51" s="22" t="inlineStr">
+      <c r="C53" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone}
 2. POST /auth/mobile/verify {phone, token: 123456}</t>
         </is>
       </c>
-      <c r="D51" s="22" t="inlineStr">
+      <c r="D53" s="22" t="inlineStr">
         <is>
           <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
         </is>
       </c>
-      <c r="E51" s="22" t="inlineStr">
+      <c r="E53" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
         </is>
       </c>
-      <c r="F51" s="22" t="inlineStr">
+      <c r="F53" s="22" t="inlineStr">
         <is>
           <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
         </is>
       </c>
-      <c r="G51" s="22" t="inlineStr">
+      <c r="G53" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H51" s="22" t="inlineStr">
+      <c r="H53" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I51" s="22" t="inlineStr">
+      <c r="I53" s="22" t="inlineStr">
         <is>
           <t>`_normalize_phone` (sign_in.py:197–206) kiểm bằng `str.isdigit()`, nhận cả chữ số Unicode, nên số lọt qua kiểm tra và gửi tới Supabase. Ô nhập của app chỉ cho 0-9 nên người dùng app không gặp; lỗi ở tầng API
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="189.5" customHeight="1">
-      <c r="A52" s="22" t="inlineStr">
+    <row r="54" ht="189.5" customHeight="1">
+      <c r="A54" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-25</t>
         </is>
       </c>
-      <c r="B52" s="22" t="inlineStr">
+      <c r="B54" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên có ký tự NUL</t>
         </is>
       </c>
-      <c r="C52" s="22" t="inlineStr">
+      <c r="C54" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
         </is>
       </c>
-      <c r="D52" s="22" t="inlineStr">
+      <c r="D54" s="22" t="inlineStr">
         <is>
           <t>ho_ten: abc\u0000def</t>
         </is>
       </c>
-      <c r="E52" s="22" t="inlineStr">
+      <c r="E54" s="22" t="inlineStr">
         <is>
           <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
         </is>
       </c>
-      <c r="F52" s="22" t="inlineStr">
+      <c r="F54" s="22" t="inlineStr">
         <is>
           <t>500 Internal Server Error</t>
         </is>
       </c>
-      <c r="G52" s="22" t="inlineStr">
+      <c r="G54" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H52" s="22" t="inlineStr">
+      <c r="H54" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I52" s="22" t="inlineStr">
+      <c r="I54" s="22" t="inlineStr">
         <is>
           <t>`_validate_required_text` (sign_in.py:178) không chặn ký tự điều khiển; PostgreSQL từ chối NUL trong cột text: `psycopg.DataError: PostgreSQL text fields cannot contain NUL (0x00) bytes` ở `UPDATE users SET full_name…` (SqlUsers.update_profile); không có handler cho DataError nên thành 500. Câu SQL có tham số nên không phải lỗ hổng SQL injection
 Log: evidence/test-integration.log, evidence/test-probe-nul.log</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="90.5" customHeight="1">
-      <c r="A53" s="22" t="inlineStr">
+    <row r="55" ht="90.5" customHeight="1">
+      <c r="A55" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-30</t>
         </is>
       </c>
-      <c r="B53" s="22" t="inlineStr">
+      <c r="B55" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên dài 256 ký tự</t>
         </is>
       </c>
-      <c r="C53" s="22" t="inlineStr">
+      <c r="C55" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: A*256}</t>
         </is>
       </c>
-      <c r="D53" s="22" t="inlineStr">
+      <c r="D55" s="22" t="inlineStr">
         <is>
           <t>A*256</t>
         </is>
       </c>
-      <c r="E53" s="22" t="inlineStr">
+      <c r="E55" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F53" s="22" t="inlineStr">
+      <c r="F55" s="22" t="inlineStr">
         <is>
           <t>204, đã lưu</t>
         </is>
       </c>
-      <c r="G53" s="22" t="inlineStr">
+      <c r="G55" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H53" s="22" t="inlineStr">
+      <c r="H55" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I53" s="22" t="inlineStr">
+      <c r="I55" s="22" t="inlineStr">
         <is>
           <t>Không có giới hạn độ dài họ tên: `_validate_profile` (sign_in.py) chỉ kiểm rỗng; cột users.full_name kiểu text không giới hạn
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="90.5" customHeight="1">
-      <c r="A54" s="22" t="inlineStr">
+    <row r="56" ht="90.5" customHeight="1">
+      <c r="A56" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-32</t>
         </is>
       </c>
-      <c r="B54" s="22" t="inlineStr">
+      <c r="B56" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh trước 1900-01-01</t>
         </is>
       </c>
-      <c r="C54" s="22" t="inlineStr">
+      <c r="C56" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh}</t>
         </is>
       </c>
-      <c r="D54" s="22" t="inlineStr">
+      <c r="D56" s="22" t="inlineStr">
         <is>
           <t>1899-12-31 | 0001-01-01</t>
         </is>
       </c>
-      <c r="E54" s="22" t="inlineStr">
+      <c r="E56" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
         </is>
       </c>
-      <c r="F54" s="22" t="inlineStr">
+      <c r="F56" s="22" t="inlineStr">
         <is>
           <t>204 ở cả hai giá trị, đã lưu</t>
         </is>
       </c>
-      <c r="G54" s="22" t="inlineStr">
+      <c r="G56" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H54" s="22" t="inlineStr">
+      <c r="H56" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I54" s="22" t="inlineStr">
+      <c r="I56" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:229–231) chỉ chặn ngày tương lai, không có cận dưới. App mobile đã giới hạn date picker từ 1900 nên chỉ gặp khi gọi API trực tiếp
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="123.5" customHeight="1">
-      <c r="A55" s="22" t="inlineStr">
+    <row r="57" ht="123.5" customHeight="1">
+      <c r="A57" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-35</t>
         </is>
       </c>
-      <c r="B55" s="22" t="inlineStr">
+      <c r="B57" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
         </is>
       </c>
-      <c r="C55" s="22" t="inlineStr">
+      <c r="C57" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
         </is>
       </c>
-      <c r="D55" s="22" t="inlineStr">
+      <c r="D57" s="22" t="inlineStr">
         <is>
           <t>ngay_sinh: 2026-10-08</t>
         </is>
       </c>
-      <c r="E55" s="22" t="inlineStr">
+      <c r="E57" s="22" t="inlineStr">
         <is>
           <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
         </is>
       </c>
-      <c r="F55" s="22" t="inlineStr">
+      <c r="F57" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_date_of_birth"}</t>
         </is>
       </c>
-      <c r="G55" s="22" t="inlineStr">
+      <c r="G57" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H55" s="22" t="inlineStr">
+      <c r="H57" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I55" s="22" t="inlineStr">
+      <c r="I57" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:230) so với `now.date()` trong khi `now()` (shared/clock.py) trả giờ UTC: từ 00:00 đến 07:00 giờ VN, "hôm nay" bị coi là ngày mai. Vi phạm bất biến 7 (múi giờ cố định Asia/Ho_Chi_Minh)
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="173" customHeight="1">
-      <c r="A56" s="22" t="inlineStr">
+    <row r="58" ht="173" customHeight="1">
+      <c r="A58" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-42</t>
         </is>
       </c>
-      <c r="B56" s="22" t="inlineStr">
+      <c r="B58" s="22" t="inlineStr">
         <is>
           <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
         </is>
       </c>
-      <c r="C56" s="22" t="inlineStr">
+      <c r="C58" s="22" t="inlineStr">
         <is>
           <t>1. Chạm vào ô mã OTP
 2. Theo dõi request backend nhận được</t>
         </is>
       </c>
-      <c r="D56" s="22" t="inlineStr">
+      <c r="D58" s="22" t="inlineStr">
         <is>
           <t>Ô đang chứa 000000</t>
         </is>
       </c>
-      <c r="E56" s="22" t="inlineStr">
+      <c r="E58" s="22" t="inlineStr">
         <is>
           <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
         </is>
       </c>
-      <c r="F56" s="22" t="inlineStr">
+      <c r="F58" s="22" t="inlineStr">
         <is>
           <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
         </is>
       </c>
-      <c r="G56" s="22" t="inlineStr">
+      <c r="G58" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H56" s="22" t="inlineStr">
+      <c r="H58" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I56" s="22" t="inlineStr">
+      <c r="I58" s="22" t="inlineStr">
         <is>
           <t>`OtpPinInput._handleTextChange` (frontend/mobile/lib/features/auth/presentation/widgets/otp_pin_input.dart:66–72) chạy với mọi thông báo của controller, kể cả khi chỉ đổi vị trí con trỏ lúc chạm ô, và gọi onCompleted hễ ô đủ 6 số → gửi lại mã sai, tốn hạn mức token_verifications
 Log: evidence/test-e2e.log (mục "request backend trong pha 2"), evidence/implement-P10-run-phase2-requests.log</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="222.5" customHeight="1">
-      <c r="A57" s="22" t="inlineStr">
+    <row r="59" ht="222.5" customHeight="1">
+      <c r="A59" s="22" t="inlineStr">
         <is>
           <t>BUG-LINKCODE-28</t>
         </is>
       </c>
-      <c r="B57" s="22" t="inlineStr">
+      <c r="B59" s="22" t="inlineStr">
         <is>
           <t>Toàn bộ unit test, architecture test và ruff toàn repo pass</t>
         </is>
       </c>
-      <c r="C57" s="22" t="inlineStr">
+      <c r="C59" s="22" t="inlineStr">
         <is>
           <t>1. pytest tests/unit tests/architecture -q
 2. ruff check .
 3. So với baseline trước khi sửa code</t>
         </is>
       </c>
-      <c r="D57" s="22" t="inlineStr">
+      <c r="D59" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E57" s="22" t="inlineStr">
+      <c r="E59" s="22" t="inlineStr">
         <is>
           <t>pytest và ruff đều pass</t>
         </is>
       </c>
-      <c r="F57" s="22" t="inlineStr">
+      <c r="F59" s="22" t="inlineStr">
         <is>
           <t>pytest tests/unit tests/architecture: 885 passed, 18 failed (test_contract_profile.py ×12, test_profile_http.py ×6); ruff check . 19 lỗi ở module khác. Cùng danh sách với baseline trước khi 3.13 sửa code; file của task pass ruff. Lỗi test_app.py của lần chạy 3.10 không còn</t>
         </is>
       </c>
-      <c r="G57" s="22" t="inlineStr">
+      <c r="G59" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H57" s="22" t="inlineStr">
+      <c r="H59" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I57" s="22" t="inlineStr">
+      <c r="I59" s="22" t="inlineStr">
         <is>
           <t>Có sẵn trên main, không do 3.10/3.13. Nghi vấn: 18 test profile fail vì api_contract (aea2b26) chưa có các endpoint /profile mà backend đã có (remote có nhánh fix/adhoc-20261015-api-contract-sync); 19 lỗi ruff ở catalog/*, runtime/*, worker.py, tests/unit/test_catalog_crud.py
 Log: evidence/test-unit-2.log, evidence/implement-final-backend-2.log</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="239" customHeight="1">
-      <c r="A58" s="22" t="inlineStr">
+    <row r="60" ht="239" customHeight="1">
+      <c r="A60" s="22" t="inlineStr">
         <is>
           <t>BUG-REGDOSE-01</t>
         </is>
       </c>
-      <c r="B58" s="22" t="inlineStr">
+      <c r="B60" s="22" t="inlineStr">
         <is>
           <t>Đối chiếu scheduled_at có giây khi xác nhận liều</t>
         </is>
       </c>
-      <c r="C58" s="22" t="inlineStr">
+      <c r="C60" s="22" t="inlineStr">
         <is>
           <t>1. Từ backend chạy .venv/Scripts/python.exe -m pytest tests/integration/test_dose_confirmation_api.py::test_post_doses_batch_creates_dose_log_for_authenticated_patient__AC1_AC10_AC18 -q -ra.
 2. Fixture POST /doses/batch với danh sách một item ở Test Data.
 3. Đối chiếu items[0].scheduled_at với kỳ vọng test hiện có.</t>
         </is>
       </c>
-      <c r="D58" s="22" t="inlineStr">
+      <c r="D60" s="22" t="inlineStr">
         <is>
           <t>client_uuid: UUID mới; schedule_id: fixture; scheduled_at=2026-10-02T01:00:59.999Z; taken_at=2026-10-02T01:05:59.999Z</t>
         </is>
       </c>
-      <c r="E58" s="22" t="inlineStr">
+      <c r="E60" s="22" t="inlineStr">
         <is>
           <t>Theo test hiện có: HTTP 200, synced, da_uong và scheduled_at=2026-10-02T01:00:00Z.</t>
         </is>
       </c>
-      <c r="F58" s="22" t="inlineStr">
+      <c r="F60" s="22" t="inlineStr">
         <is>
           <t>HTTP 200, synced, da_uong; scheduled_at=2026-10-02T01:00:59.999000Z. Fail trong suite DB và lặp lại khi chạy riêng (1 failed trong 1.67s).</t>
         </is>
       </c>
-      <c r="G58" s="22" t="inlineStr">
+      <c r="G60" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H58" s="22" t="inlineStr">
+      <c r="H60" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I58" s="22" t="inlineStr">
+      <c r="I60" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn kỳ vọng chuẩn hóa tới phút trong test không khớp hành vi giữ thời điểm của API; chưa xác định phía nào sai theo contract/nghiệp vụ. Chưa chứng minh mất/trùng bản ghi liều; mức Medium tạm thời cho sai khác test, phải nâng tối thiểu High nếu xác nhận mất/trùng liều.
 Log: evidence/test-integration-db.log; evidence/test-dose-mismatch-repeat.log</t>
@@ -12922,17 +16544,17 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:A5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11:F25">
+  <conditionalFormatting sqref="F11:F27">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11:G25">
+  <conditionalFormatting sqref="G11:G27">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>OR(G11="Critical",G11="High")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G50:G58">
+  <conditionalFormatting sqref="G52:G60">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
@@ -12944,10 +16566,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G11:G25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G11:G27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="G50:G58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G52:G60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
test(adherence): record consent regression cases
Refs: 3.23
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -1,16 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Alert dispatch" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Report" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alert dispatch" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lịch sử tuân thủ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Alert dispatch'!$A$8:$I$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lịch sử tuân thủ'!$A$8:$I$31</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,8 +21,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -127,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -135,7 +137,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -184,6 +186,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -307,13 +315,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -337,18 +345,18 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11</f>
+              <f>'Report'!$A$11:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$11</f>
+              <f>'Report'!$D$11:$D$12</f>
             </numRef>
           </val>
         </ser>
@@ -361,18 +369,18 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11</f>
+              <f>'Report'!$A$11:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$11</f>
+              <f>'Report'!$E$11:$E$12</f>
             </numRef>
           </val>
         </ser>
@@ -385,18 +393,18 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11</f>
+              <f>'Report'!$A$11:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$11</f>
+              <f>'Report'!$F$11:$F$12</f>
             </numRef>
           </val>
         </ser>
@@ -442,13 +450,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -466,7 +474,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -494,12 +502,12 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>13</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -509,9 +517,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -521,7 +529,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>13</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3240000"/>
@@ -531,9 +539,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -909,7 +917,7 @@
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="21" t="n">
         <v>46308</v>
       </c>
     </row>
@@ -1891,7 +1899,1704 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:X37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="8" customWidth="1" min="22" max="22"/>
+    <col width="8" customWidth="1" min="23" max="23"/>
+    <col width="8" customWidth="1" min="24" max="24"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Lịch sử tuân thủ theo consent (ADHERENCE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Ngọc Việt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Quyền đọc lịch sử</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="W8" s="5" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="X8" s="5" t="inlineStr">
+        <is>
+          <t>R7</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="156.5" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Xem lịch sử của chính bệnh nhân</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Bệnh nhân P có consent health_data; có lịch uống và một liều đã uống.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập bằng tài khoản P.
+2. Gửi GET /adherence?patient_id=P với bearer token của P.
+3. Kiểm response và access_logs.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>P; ngày 2026-10-19; liều 08:00 da_uong</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>200; patient_id=P; có liều đã uống; access_logs có allowed, actor_role=patient, data_scope=lich_su_tuan_thu.</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · EP (1) · Decision Table (R1) · test_self_and_family_success_are_audited_with_minimal_metadata__AC1_AC2</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>patient_id và vai trò</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>Bỏ trống hoặc chính bệnh nhân
+Người thân liên kết active với consent đầy đủ</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1
+2</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>Người thân không liên kết
+Liên kết tắt chia sẻ
+Thiếu health_data
+Thiếu family_sharing
+Đổi sang bệnh nhân khác
+Thiếu hoặc sai token
+UUID sai định dạng
+Admin dù tự gọi hoặc có liên kết</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>3
+4
+5
+6
+7
+8
+9
+10</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Vai trò</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>patient</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="U9" s="11" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="V9" s="11" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="W9" s="11" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="X9" s="11" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="74" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Xem lịch sử bệnh nhân từ người thân được chia sẻ</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>P có health_data và family_sharing; F có caregiver_link active, sharing_enabled=true; P có một liều đã uống.</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập bằng tài khoản F.
+2. Gửi GET /adherence?patient_id=P.
+3. Kiểm nhóm liều và access_logs.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>P; F; from=2026-10-19; to=2026-10-19</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>200; patient_id=P; nhóm và tổng hợp đúng liều của P; access_logs có allowed, actor_role=family.</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · EP (2) · Decision Table (R2) · test_self_and_family_success_are_audited_with_minimal_metadata__AC1_AC2</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>Liên kết active và bật chia sẻ</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="74" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối người thân không có liên kết</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>P có consent; F không có caregiver_link với P; P có liều đã uống.</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập F.
+2. Gửi GET /adherence?patient_id=P.
+3. Kiểm response và access_logs.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>P; F không liên kết</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>403 {"detail":"khong_co_quyen"}; không có lịch sử; access_logs có denied cho P.</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · EP (3) · Decision Table (R3) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>health_data</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V11" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="74" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối khi tắt công tắc chia sẻ</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>F có link active tới P; P có hai consent; sharing_enabled=false.</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập F.
+2. Gửi GET /adherence?patient_id=P.
+3. Kiểm access_logs.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>sharing_enabled=false</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>403 khong_co_quyen; không có lịch sử; access_logs có denied.</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · EP (4) · Decision Table (R4) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
+        <is>
+          <t>family_sharing</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W12" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="74" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối khi thiếu consent sức khỏe</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>F có link active và sharing_enabled=true; P không còn health_data.</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập F.
+2. Gửi GET /adherence?patient_id=P.
+3. Kiểm access_logs.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>health_data=thu_hoi</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>403 khong_co_quyen; không có lịch sử; access_logs có denied.</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (5) · Decision Table (R5) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11</t>
+        </is>
+      </c>
+      <c r="Q13" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T13" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U13" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="V13" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="W13" s="5" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="X13" s="5" t="inlineStr">
+        <is>
+          <t>R7</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="74" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối khi thiếu consent chia sẻ gia đình</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>F có link active và sharing_enabled=true; P không còn family_sharing.</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập F.
+2. Gửi GET /adherence?patient_id=P.
+3. Kiểm access_logs.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>family_sharing=thu_hoi</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>403 khong_co_quyen; không có lịch sử; access_logs có denied.</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (6) · Decision Table (R6) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>200 + allowed</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T14" s="11" t="inlineStr"/>
+      <c r="U14" s="11" t="inlineStr"/>
+      <c r="V14" s="11" t="inlineStr"/>
+      <c r="W14" s="11" t="inlineStr"/>
+      <c r="X14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="90.5" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối ngay sau khi rút consent với cùng token</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>F đang được phép đọc P; lưu bearer token của F.</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence?patient_id=P và xác nhận 200.
+2. Rút health_data hoặc family_sharing của P.
+3. Gửi lại cùng request với token cũ.
+4. Kiểm access_logs.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>P; F; token không đổi</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Request thứ hai 403 khong_co_quyen; access_logs có allowed rồi denied, không trả lịch sử.</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · Decision Table (R5,R6) · test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12</t>
+        </is>
+      </c>
+      <c r="Q15" s="10" t="inlineStr">
+        <is>
+          <t>403 + denied</t>
+        </is>
+      </c>
+      <c r="R15" s="11" t="inlineStr"/>
+      <c r="S15" s="11" t="inlineStr"/>
+      <c r="T15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="V15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="W15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="X15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="107" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối ngay sau khi hủy liên kết hoặc tắt chia sẻ</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>F đang được phép đọc P; lưu bearer token của F.</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence?patient_id=P và xác nhận 200.
+2. Hủy caregiver_link hoặc tắt sharing_enabled.
+3. Gửi lại với token cũ.
+4. Kiểm access_logs.</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>P; F; token không đổi</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Request thứ hai 403 khong_co_quyen; access_logs có allowed rồi denied.</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · Decision Table (R3,R4) · test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90.5" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối đổi patient_id sang bệnh nhân khác</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>F có quyền với P nhưng không có quyền với Q; Q có lịch sử liều.</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập F.
+2. Gửi GET /adherence?patient_id=P và xác nhận 200.
+3. Đổi patient_id=Q rồi gửi lại.
+4. Kiểm access_logs của Q.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>P; Q; F chỉ liên kết P</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Request Q trả 403 khong_co_quyen; không có lịch sử Q; access_logs Q có denied.</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (7) · test_family_patient_selector_tamper_does_not_read_other_patient__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="57.5" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Không trả lịch sử khi ghi audit allowed thất bại</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>P có consent và lịch sử; DB api_role bị giả lập lỗi INSERT access_logs.</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence bằng token P.
+2. Kiểm response, audit và dữ liệu liều.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Lỗi INSERT access_logs</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>500; no-store; không có lịch sử trong response và không làm thay đổi dose_logs.</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · test_audit_permission_and_commit_failure_fail_closed_without_health__AC13</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="57.5" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Giữ log denied sau khi request rollback</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>P đã rút health_data; request bị từ chối và transaction chính rollback.</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence bằng token P.
+2. Kiểm response.
+3. Đọc access_logs bằng kết nối quản trị.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>health_data=thu_hoi</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>403 consent_revoked; access_logs vẫn có denied cho scope lich_su_tuan_thu.</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · test_denied_audit_survives_outer_transaction_rollback__AC13</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="74" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối khi thiếu hoặc sai bearer token</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>P có lịch sử liều.</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence không có Authorization.
+2. Gửi lại với Authorization: Bearer invalid-token.
+3. Kiểm response và access_logs.</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Authorization=(blank) hoặc Bearer invalid-token</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>401; response không chứa lịch sử; Cache-Control=no-store; không có allowed log.</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (8) · test_authentication_401_and_no_store_without_health_payload__AC14</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="57.5" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-13</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối patient_id sai định dạng</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>P có lịch sử liều và token hợp lệ.</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence?patient_id=invalid-uuid bằng token P.
+2. Kiểm response.</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>patient_id=invalid-uuid</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>422; response không chứa lịch sử; Cache-Control=no-store.</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (9) · test_bad_queries_are_422_without_health_payload__AC14</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="74" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-14</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối admin xem lịch sử của chính mình</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Admin A có health_data và một liều đã uống.</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập A.
+2. Gửi GET /adherence?patient_id=A.
+3. Kiểm response, access_logs và dose_logs.</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>A có system_role=admin</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>403 khong_co_quyen; không lộ liều; access_logs denied actor_role=admin; dose_logs không đổi.</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AC3, AC7 · Decision Table (R7) · test_admin_self_and_linked_history_denied_and_audited__AC3_AC6_AC7</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="74" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối admin có liên kết người thân</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>P có hai consent và một liều; admin A có caregiver_link active, sharing_enabled=true với P.</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập A.
+2. Gửi GET /adherence?patient_id=P.
+3. Kiểm response, access_logs và dose_logs.</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>P; A có system_role=admin</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>403 khong_co_quyen; không lộ liều; access_logs denied actor_role=admin; dose_logs không đổi.</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AC3, AC6, AC7 · Decision Table (R7) · test_admin_self_and_linked_history_denied_and_audited__AC3_AC6_AC7</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="74" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-16</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm nhóm ngày, nhóm thuốc và tỷ lệ tuân thủ</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>P có 5 liều: 3 da_uong, 1 uong_tre, 1 bo_lo.</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence?group_by=date&amp;from=2026-10-19&amp;to=2026-10-19.
+2. Gửi lại với group_by=medication.
+3. So sánh summary và nhóm.</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19; 5 liều, 2 thuốc</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>200; summary total=5, taken=3, late=1, missed=1, pending=0, adherence_rate=80; nhóm và timezone Asia/Ho_Chi_Minh đúng contract.</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>AC1, AC9 · test_patient_history_by_date_medication_groups_and_80_percent__AC1_AC3_AC4</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="57.5" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-17</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm khoảng ngày một ngày</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>P có lịch dùng thuốc bắt đầu 2026-10-19.</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence?from=2026-10-19&amp;to=2026-10-19.
+2. Kiểm summary và nhóm.</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>from=2026-10-19; to=2026-10-19</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>200; khoảng một ngày được chấp nhận và chỉ có liều ngày 2026-10-19.</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · BVA (min) · test_default_partial_and_inclusive_90_day_filters__AC5</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="57.5" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-18</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm khoảng ngày tối đa 90 ngày</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>P có lịch từ 2026-07-22 đến 2026-10-19.</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence với khoảng đúng 90 ngày.
+2. Kiểm số ngày và response.</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>from=2026-07-22; to=2026-10-19</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>200; khoảng 90 ngày được chấp nhận.</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · BVA (max) · test_default_partial_and_inclusive_90_day_filters__AC5</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="57.5" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-19</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối khoảng ngày 91 ngày</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>P có lịch từ 2026-07-21 đến 2026-10-19.</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence với khoảng 91 ngày.
+2. Kiểm response.</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>from=2026-07-21; to=2026-10-19</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail":"adherence_range_too_large"}; không có lịch sử.</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · BVA (max+1) · test_default_partial_and_inclusive_90_day_filters__AC5</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="74" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-20</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Đối chiếu contract với OpenAPI runtime</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Có api_contract/openapi.json đã duyệt và app FastAPI khởi tạo được.</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. Sinh OpenAPI từ create_app().openapi().
+2. So path GET /adherence, query, auth, status, schema và no-store với contract.</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>GET /adherence; patient_id, from, to, group_by</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Path, query, bảo mật, mã lỗi, cấu trúc response và Cache-Control no-store khớp contract.</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Hai test OpenAPI runtime/schema PASSED; evidence/test-openapi-after-migration.log.</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · test_contract_query_security_status_headers · test_response_required_nullable_enums_and_constraints</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="57.5" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-21</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối khoảng ngày đảo ngược</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>P có token hợp lệ và lịch sử liều.</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence?from=2026-10-19&amp;to=2026-10-18 bằng token P.
+2. Kiểm response không chứa lịch sử.</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>from=2026-10-19; to=2026-10-18</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>422; không có lịch sử trong response; Cache-Control=no-store.</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · BVA (min-1) · test_bad_queries_are_422_without_health_payload__AC14</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="123.5" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-22</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm ràng buộc actor identity sau migration</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>DB local có migration admin-self; hai user A và B; kết nối api_role.</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>1. Lần lượt INSERT access_logs với actor A, patient A hoặc B, vai patient/family/admin/khong_co_quyen, result allowed/denied.
+2. Kiểm INSERT thành công hoặc SQLSTATE 23514 theo từng tổ hợp.
+3. Rollback từng lần; xác nhận không còn dòng thử.</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>16 tổ hợp: self/other × 4 role × allowed/denied</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Self patient allowed/denied và self admin denied được chấp nhận; self admin allowed, self family/no-access và other patient bị chặn. Other family/admin giữ allowed/denied; other no-access chỉ denied. Không lưu dòng sau rollback.</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>16 ca matrix PASSED; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>AC3, AC7 · Decision Table (R7) · test_access_log_actor_identity_matrix__AC3_AC7</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="74" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-23</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Chặn sửa xóa và truncate audit sau migration</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>DB local có migration admin-self và một dòng audit; có kết nối api_role, worker_role và postgres.</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>1. Thử UPDATE, DELETE, TRUNCATE access_logs lần lượt bằng từng role.
+2. Rollback từng transaction thử.
+3. Đọc lại audit bằng kết nối quản trị.</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>api_role/worker_role/postgres × UPDATE/DELETE/TRUNCATE = 9 ca</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Role ứng dụng bị từ chối SQLSTATE 42501; postgres bị trigger từ chối P0001; audit không đổi.</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>9 ca append-only PASSED; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · CD3 · test_access_logs_remain_append_only_after_actor_identity_migration__AC7</t>
+        </is>
+      </c>
+    </row>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34">
+      <c r="G34" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H34" s="13">
+        <f>COUNTIF(H9:H31,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H35" s="13">
+        <f>COUNTIF(H9:H31,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H36" s="13">
+        <f>COUNTIF(H9:H31,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="G37" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H37" s="13">
+        <f>SUM(H34:H36)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I31"/>
+  <conditionalFormatting sqref="H9:H31">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1936,7 +3641,7 @@
         </is>
       </c>
       <c r="C3" s="11">
-        <f>'Alert dispatch'!$H$22</f>
+        <f>'Alert dispatch'!$H$22+'Lịch sử tuân thủ'!$H$34</f>
         <v/>
       </c>
       <c r="D3" s="15">
@@ -1952,7 +3657,7 @@
         </is>
       </c>
       <c r="C4" s="11">
-        <f>'Alert dispatch'!$H$23</f>
+        <f>'Alert dispatch'!$H$23+'Lịch sử tuân thủ'!$H$35</f>
         <v/>
       </c>
       <c r="D4" s="15">
@@ -1984,7 +3689,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr"/>
       <c r="C6" s="11">
-        <f>'Alert dispatch'!$H$24</f>
+        <f>'Alert dispatch'!$H$24+'Lịch sử tuân thủ'!$H$36</f>
         <v/>
       </c>
       <c r="D6" s="15">
@@ -2099,55 +3804,99 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="19" t="inlineStr">
+    <row r="12" ht="90.5" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Lịch sử tuân thủ theo consent</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>GET /adherence theo quyền bệnh nhân, người thân, consent và audit.</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Lịch sử tuân thủ</t>
+        </is>
+      </c>
+      <c r="D12" s="18">
+        <f>IFERROR(('Lịch sử tuân thủ'!$H$37-'Lịch sử tuân thủ'!$H$36)/'Lịch sử tuân thủ'!$H$37,0)</f>
+        <v/>
+      </c>
+      <c r="E12" s="18">
+        <f>IFERROR('Lịch sử tuân thủ'!$H$34/'Lịch sử tuân thủ'!$H$37,0)</f>
+        <v/>
+      </c>
+      <c r="F12" s="18">
+        <f>IFERROR('Lịch sử tuân thủ'!$H$35/'Lịch sử tuân thủ'!$H$37,0)</f>
+        <v/>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>23 Pass sau migration; BUG-ADHERENCE-14 đã qua kiểm thử hồi quy, còn chờ review/PR.</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>Ngọc Việt</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
         <is>
           <t>Bug Report</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="20" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="20" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="B35" s="20" t="inlineStr">
+      <c r="B36" s="20" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C35" s="20" t="inlineStr">
+      <c r="C36" s="20" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="D35" s="20" t="inlineStr">
+      <c r="D36" s="20" t="inlineStr">
         <is>
           <t>Input Data</t>
         </is>
       </c>
-      <c r="E35" s="20" t="inlineStr">
+      <c r="E36" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F35" s="20" t="inlineStr">
+      <c r="F36" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="G35" s="20" t="inlineStr">
+      <c r="G36" s="20" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="H35" s="20" t="inlineStr">
+      <c r="H36" s="20" t="inlineStr">
         <is>
           <t>Name of Tester</t>
         </is>
       </c>
-      <c r="I35" s="20" t="inlineStr">
+      <c r="I36" s="20" t="inlineStr">
         <is>
           <t>Logs</t>
         </is>
@@ -2158,17 +3907,17 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:A5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11">
+  <conditionalFormatting sqref="F11:F12">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11">
+  <conditionalFormatting sqref="G11:G12">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>OR(G11="Critical",G11="High")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G36">
+  <conditionalFormatting sqref="G37">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
@@ -2180,10 +3929,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G11:G12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="G36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(tests): update Test Cases.xlsx with new test scenarios
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -15356,7 +15356,7 @@
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -15366,7 +15366,7 @@
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC4 · đoán lỗi, chuyển trạng thái và bảo mật · test_allowed_list_detail_patch_use_read_audit_and_replay__AC3_AC4 · evidence/test-task-integration-final.log</t>
+          <t>AC3, AC4 · đoán lỗi, chuyển trạng thái và bảo mật · test_allowed_list_detail_patch_use_read_audit_and_replay__AC3_AC4 · evidence/test-validation-task.log</t>
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr">
@@ -15467,7 +15467,7 @@
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -15477,7 +15477,7 @@
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-unlinked] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-unlinked] · evidence/test-validation-task.log</t>
         </is>
       </c>
       <c r="K10" s="9" t="inlineStr">
@@ -15576,7 +15576,7 @@
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -15586,7 +15586,7 @@
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-inactive] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-inactive] · evidence/test-validation-task.log</t>
         </is>
       </c>
       <c r="Q11" s="10" t="inlineStr">
@@ -15660,7 +15660,7 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -15670,7 +15670,7 @@
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R3) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-sharing_off] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R3) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-sharing_off] · evidence/test-validation-task.log</t>
         </is>
       </c>
       <c r="Q12" s="10" t="inlineStr">
@@ -15744,7 +15744,7 @@
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
@@ -15754,7 +15754,7 @@
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R4) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-health_data] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R4) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-health_data] · evidence/test-validation-task.log</t>
         </is>
       </c>
       <c r="Q13" s="10" t="inlineStr">
@@ -15828,7 +15828,7 @@
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
@@ -15838,7 +15838,7 @@
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R5) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-family_sharing] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R5) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-family_sharing] · evidence/test-validation-task.log</t>
         </is>
       </c>
       <c r="Q14" s="6" t="inlineStr">
@@ -15912,7 +15912,7 @@
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -15922,7 +15922,7 @@
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-unlinked] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-unlinked] · evidence/test-validation-task.log</t>
         </is>
       </c>
       <c r="Q15" s="10" t="inlineStr">
@@ -15976,7 +15976,7 @@
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
@@ -15986,7 +15986,7 @@
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-inactive] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-inactive] · evidence/test-validation-task.log</t>
         </is>
       </c>
       <c r="Q16" s="10" t="inlineStr">
@@ -16052,7 +16052,7 @@
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -16062,7 +16062,7 @@
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R3) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-sharing_off] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R3) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-sharing_off] · evidence/test-validation-task.log</t>
         </is>
       </c>
       <c r="Q17" s="10" t="inlineStr">
@@ -16116,7 +16116,7 @@
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
@@ -16126,7 +16126,7 @@
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R4) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-health_data] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R4) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-health_data] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -16165,7 +16165,7 @@
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
@@ -16175,7 +16175,7 @@
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R5) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-family_sharing] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R5) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-family_sharing] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -16214,7 +16214,7 @@
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
@@ -16224,7 +16224,7 @@
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-unlinked] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-unlinked] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -16263,7 +16263,7 @@
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
@@ -16273,7 +16273,7 @@
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-inactive] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-inactive] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16312,7 @@
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
@@ -16322,7 +16322,7 @@
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R3) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-sharing_off] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R3) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-sharing_off] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -16361,7 +16361,7 @@
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
@@ -16371,7 +16371,7 @@
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R4) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-health_data] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R4) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-health_data] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -16410,7 +16410,7 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
@@ -16420,7 +16420,7 @@
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R5) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-family_sharing] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R5) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-family_sharing] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -16459,7 +16459,7 @@
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
@@ -16469,7 +16469,7 @@
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_other_recipient_and_unknown_id_return_404__AC5[detail] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_other_recipient_and_unknown_id_return_404__AC5[detail] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -16508,7 +16508,7 @@
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
@@ -16518,7 +16518,7 @@
       </c>
       <c r="I26" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_other_recipient_and_unknown_id_return_404__AC5[patch] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_other_recipient_and_unknown_id_return_404__AC5[patch] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -16557,21 +16557,21 @@
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>HTTP 503 notification_access_unavailable thay vì 422; assertion fail.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_mixed_patient_filter_and_selector_tamper_do_not_leak__AC3_AC5 · evidence/test-task-integration-final.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="90.5" customHeight="1">
+          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_mixed_patient_filter_and_selector_tamper_do_not_leak__AC3_AC5 · evidence/test-validation-task.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="74" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
           <t>TC-FALERT-20</t>
@@ -16605,7 +16605,7 @@
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
@@ -16615,11 +16615,11 @@
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_admin_session_forbidden__AC5[list] · evidence/test-task-integration-final.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="90.5" customHeight="1">
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_admin_session_forbidden__AC5[list] · evidence/test-validation-task.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="74" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
         <is>
           <t>TC-FALERT-21</t>
@@ -16653,7 +16653,7 @@
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
@@ -16663,11 +16663,11 @@
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_admin_session_forbidden__AC5[detail] · evidence/test-task-integration-final.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="90.5" customHeight="1">
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_admin_session_forbidden__AC5[detail] · evidence/test-validation-task.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="74" customHeight="1">
       <c r="A30" s="7" t="inlineStr">
         <is>
           <t>TC-FALERT-22</t>
@@ -16701,7 +16701,7 @@
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
@@ -16711,7 +16711,7 @@
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_admin_session_forbidden__AC5[patch] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_admin_session_forbidden__AC5[patch] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -16750,7 +16750,7 @@
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
@@ -16760,7 +16760,7 @@
       </c>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[facts-list] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[facts-list] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -16799,7 +16799,7 @@
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
@@ -16809,7 +16809,7 @@
       </c>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[facts-detail] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[facts-detail] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -16848,7 +16848,7 @@
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
@@ -16858,7 +16858,7 @@
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[facts-patch] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[facts-patch] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -16897,7 +16897,7 @@
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
@@ -16907,7 +16907,7 @@
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[allowed_insert-list] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[allowed_insert-list] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -16946,7 +16946,7 @@
       </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
@@ -16956,7 +16956,7 @@
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[allowed_insert-detail] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[allowed_insert-detail] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -16995,7 +16995,7 @@
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
@@ -17005,7 +17005,7 @@
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[allowed_insert-patch] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[allowed_insert-patch] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17044,7 +17044,7 @@
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
@@ -17054,7 +17054,7 @@
       </c>
       <c r="I37" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[denied_insert-list] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[denied_insert-list] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17093,7 +17093,7 @@
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
@@ -17103,7 +17103,7 @@
       </c>
       <c r="I38" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[denied_insert-detail] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[denied_insert-detail] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17142,7 +17142,7 @@
       </c>
       <c r="G39" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
@@ -17152,7 +17152,7 @@
       </c>
       <c r="I39" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[denied_insert-patch] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[denied_insert-patch] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17191,7 +17191,7 @@
       </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
@@ -17201,7 +17201,7 @@
       </c>
       <c r="I40" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[commit-list] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[commit-list] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17240,7 +17240,7 @@
       </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
@@ -17250,7 +17250,7 @@
       </c>
       <c r="I41" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[commit-detail] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[commit-detail] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17289,7 +17289,7 @@
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
@@ -17299,7 +17299,7 @@
       </c>
       <c r="I42" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[commit-patch] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[commit-patch] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17338,7 +17338,7 @@
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
@@ -17348,7 +17348,7 @@
       </c>
       <c r="I43" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_denied_audit_survives_request_transaction_rollback__AC5 · evidence/test-task-integration-final.log</t>
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_denied_audit_survives_request_transaction_rollback__AC5 · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17387,17 +17387,17 @@
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>HTTP 503 notification_access_unavailable thay vì 422; assertion fail.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I44" s="8" t="inlineStr">
         <is>
-          <t>AC3 · BVA (min-1), EP (3) · test_invalid_pagination_is_422_no_store__AC3[params0] · evidence/test-task-integration-final.log</t>
+          <t>AC3 · BVA (min-1), EP (3) · test_invalid_pagination_is_422_no_store__AC3[params0] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17436,17 +17436,17 @@
       </c>
       <c r="G45" s="8" t="inlineStr">
         <is>
-          <t>HTTP 503 notification_access_unavailable thay vì 422; assertion fail.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I45" s="8" t="inlineStr">
         <is>
-          <t>AC3 · BVA (max+1), EP (4) · test_invalid_pagination_is_422_no_store__AC3[params1] · evidence/test-task-integration-final.log</t>
+          <t>AC3 · BVA (max+1), EP (4) · test_invalid_pagination_is_422_no_store__AC3[params1] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17485,17 +17485,17 @@
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>HTTP 503 notification_access_unavailable thay vì 422; assertion fail.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I46" s="8" t="inlineStr">
         <is>
-          <t>AC3 · BVA (min-1), EP (5) · test_invalid_pagination_is_422_no_store__AC3[params2] · evidence/test-task-integration-final.log</t>
+          <t>AC3 · BVA (min-1), EP (5) · test_invalid_pagination_is_422_no_store__AC3[params2] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17533,7 +17533,7 @@
       </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
@@ -17543,7 +17543,7 @@
       </c>
       <c r="I47" s="8" t="inlineStr">
         <is>
-          <t>AC3 · BVA (min), EP (1,2) · test_valid_pagination_boundaries__AC3[1] · evidence/test-task-integration-final.log</t>
+          <t>AC3 · BVA (min), EP (1,2) · test_valid_pagination_boundaries__AC3[1] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17581,7 +17581,7 @@
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
@@ -17591,7 +17591,7 @@
       </c>
       <c r="I48" s="8" t="inlineStr">
         <is>
-          <t>AC3 · BVA (max), EP (1,2) · test_valid_pagination_boundaries__AC3[100] · evidence/test-task-integration-final.log</t>
+          <t>AC3 · BVA (max), EP (1,2) · test_valid_pagination_boundaries__AC3[100] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17630,7 +17630,7 @@
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
@@ -17640,7 +17640,7 @@
       </c>
       <c r="I49" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[list-missing] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[list-missing] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17679,7 +17679,7 @@
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
@@ -17689,7 +17689,7 @@
       </c>
       <c r="I50" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[list-pending] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[list-pending] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17728,7 +17728,7 @@
       </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
@@ -17738,7 +17738,7 @@
       </c>
       <c r="I51" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[detail-missing] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[detail-missing] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr">
@@ -17787,7 +17787,7 @@
       </c>
       <c r="I52" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[detail-pending] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[detail-pending] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17826,7 +17826,7 @@
       </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
@@ -17836,7 +17836,7 @@
       </c>
       <c r="I53" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[patch-missing] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[patch-missing] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17875,7 +17875,7 @@
       </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr">
@@ -17885,7 +17885,7 @@
       </c>
       <c r="I54" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[patch-pending] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[patch-pending] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17923,7 +17923,7 @@
       </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr">
@@ -17933,7 +17933,7 @@
       </c>
       <c r="I55" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_missing_session_returns_401_no_store__AC5[list] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_missing_session_returns_401_no_store__AC5[list] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -17971,7 +17971,7 @@
       </c>
       <c r="G56" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr">
@@ -17981,7 +17981,7 @@
       </c>
       <c r="I56" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_missing_session_returns_401_no_store__AC5[detail] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_missing_session_returns_401_no_store__AC5[detail] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -18019,7 +18019,7 @@
       </c>
       <c r="G57" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr">
@@ -18029,7 +18029,7 @@
       </c>
       <c r="I57" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_missing_session_returns_401_no_store__AC5[patch] · evidence/test-task-integration-final.log</t>
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_missing_session_returns_401_no_store__AC5[patch] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -18069,7 +18069,7 @@
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr">
@@ -18079,7 +18079,7 @@
       </c>
       <c r="I58" s="8" t="inlineStr">
         <is>
-          <t>AC2, AC3, AC4 · đoán lỗi, chuyển trạng thái và bảo mật · test_scan_snapshot_survives_catalog_schedule_edit_and_replay__AC2_AC3_AC4 · evidence/test-task-integration-final.log</t>
+          <t>AC2, AC3, AC4 · đoán lỗi, chuyển trạng thái và bảo mật · test_scan_snapshot_survives_catalog_schedule_edit_and_replay__AC2_AC3_AC4 · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -18118,7 +18118,7 @@
       </c>
       <c r="G59" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
@@ -18128,7 +18128,7 @@
       </c>
       <c r="I59" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC4 · đoán lỗi, chuyển trạng thái và bảo mật · test_filter_offset_tied_order_and_global_badge__AC3_AC4 · evidence/test-task-integration-final.log</t>
+          <t>AC3, AC4 · đoán lỗi, chuyển trạng thái và bảo mật · test_filter_offset_tied_order_and_global_badge__AC3_AC4 · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -18167,7 +18167,7 @@
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr">
@@ -18177,7 +18177,7 @@
       </c>
       <c r="I60" s="8" t="inlineStr">
         <is>
-          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_worker_database_race_never_overwrites_confirmation__AC3[False] · evidence/test-task-integration-final.log</t>
+          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_worker_database_race_never_overwrites_confirmation__AC3[False] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -18216,7 +18216,7 @@
       </c>
       <c r="G61" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr">
@@ -18226,7 +18226,7 @@
       </c>
       <c r="I61" s="8" t="inlineStr">
         <is>
-          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_worker_database_race_never_overwrites_confirmation__AC3[True] · evidence/test-task-integration-final.log</t>
+          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_worker_database_race_never_overwrites_confirmation__AC3[True] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -18265,7 +18265,7 @@
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr">
@@ -18275,7 +18275,7 @@
       </c>
       <c r="I62" s="8" t="inlineStr">
         <is>
-          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_upgrade_preserves_legacy_and_read_update__AC3 · evidence/test-task-integration-final.log</t>
+          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_upgrade_preserves_legacy_and_read_update__AC3 · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -18313,7 +18313,7 @@
       </c>
       <c r="G63" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">
@@ -18323,7 +18323,7 @@
       </c>
       <c r="I63" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC4 · đoán lỗi, chuyển trạng thái và bảo mật · test_legacy_null_snapshot_can_be_read_and_marked__AC3_AC4 · evidence/test-task-integration-final.log</t>
+          <t>AC3, AC4 · đoán lỗi, chuyển trạng thái và bảo mật · test_legacy_null_snapshot_can_be_read_and_marked__AC3_AC4 · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -18361,7 +18361,7 @@
       </c>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr">
@@ -18371,7 +18371,7 @@
       </c>
       <c r="I64" s="8" t="inlineStr">
         <is>
-          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_new_insert_requires_snapshot__AC3[None-at0] · evidence/test-task-integration-final.log</t>
+          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_new_insert_requires_snapshot__AC3[None-at0] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -18409,7 +18409,7 @@
       </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr">
@@ -18419,7 +18419,7 @@
       </c>
       <c r="I65" s="8" t="inlineStr">
         <is>
-          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_new_insert_requires_snapshot__AC3[-at1] · evidence/test-task-integration-final.log</t>
+          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_new_insert_requires_snapshot__AC3[-at1] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -18457,7 +18457,7 @@
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr">
@@ -18467,7 +18467,7 @@
       </c>
       <c r="I66" s="8" t="inlineStr">
         <is>
-          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_new_insert_requires_snapshot__AC3[   -at2] · evidence/test-task-integration-final.log</t>
+          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_new_insert_requires_snapshot__AC3[   -at2] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -18505,7 +18505,7 @@
       </c>
       <c r="G67" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr">
@@ -18515,7 +18515,7 @@
       </c>
       <c r="I67" s="8" t="inlineStr">
         <is>
-          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_new_insert_requires_snapshot__AC3[Valid-None] · evidence/test-task-integration-final.log</t>
+          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_new_insert_requires_snapshot__AC3[Valid-None] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -18554,7 +18554,7 @@
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr">
@@ -18564,7 +18564,7 @@
       </c>
       <c r="I68" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_snapshot_roles_rls_and_indexes__AC3_AC5[anon] · evidence/test-task-integration-final.log</t>
+          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_snapshot_roles_rls_and_indexes__AC3_AC5[anon] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -18603,7 +18603,7 @@
       </c>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr">
@@ -18613,7 +18613,7 @@
       </c>
       <c r="I69" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_snapshot_roles_rls_and_indexes__AC3_AC5[authenticated] · evidence/test-task-integration-final.log</t>
+          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_snapshot_roles_rls_and_indexes__AC3_AC5[authenticated] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -18652,7 +18652,7 @@
       </c>
       <c r="G70" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr">
@@ -18662,7 +18662,7 @@
       </c>
       <c r="I70" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_snapshot_roles_rls_and_indexes__AC3_AC5[api_role] · evidence/test-task-integration-final.log</t>
+          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_snapshot_roles_rls_and_indexes__AC3_AC5[api_role] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -18701,7 +18701,7 @@
       </c>
       <c r="G71" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr">
@@ -18711,7 +18711,7 @@
       </c>
       <c r="I71" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_snapshot_roles_rls_and_indexes__AC3_AC5[worker_role] · evidence/test-task-integration-final.log</t>
+          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_snapshot_roles_rls_and_indexes__AC3_AC5[worker_role] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -19152,7 +19152,7 @@
       </c>
       <c r="G81" s="8" t="inlineStr">
         <is>
-          <t>Widget được chạy trong full Flutter: 563 tests pass, gồm assertion nêu trên.</t>
+          <t>Hai widget tests pass trong lần chạy mới; không phải bằng chứng iOS runtime.</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr">
@@ -19162,7 +19162,7 @@
       </c>
       <c r="I81" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC7 · widget · evidence/test-mobile.log; không phải iOS runtime</t>
+          <t>AC3, AC7 · widget · evidence/test-validation-widget.log; không phải iOS runtime</t>
         </is>
       </c>
     </row>
@@ -19458,7 +19458,7 @@
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -19468,7 +19468,7 @@
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>AC1, AC8 · EP (1) · chuyển trạng thái/ownership · test_replay_refresh_logout_and_dispatch_selection__AC1_AC8 · evidence/test-task-integration-final.log</t>
+          <t>AC1, AC8 · EP (1) · chuyển trạng thái/ownership · test_replay_refresh_logout_and_dispatch_selection__AC1_AC8 · evidence/test-validation-task.log</t>
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr">
@@ -19519,7 +19519,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="107" customHeight="1">
+    <row r="10" ht="90.5" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>TC-FCMTOKEN-02</t>
@@ -19554,7 +19554,7 @@
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -19564,7 +19564,7 @@
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_conflicting_refresh_rolls_back_and_foreign_previous_is_preserved__AC1 · evidence/test-task-integration-final.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_conflicting_refresh_rolls_back_and_foreign_previous_is_preserved__AC1 · evidence/test-validation-task.log</t>
         </is>
       </c>
       <c r="K10" s="9" t="inlineStr">
@@ -19648,7 +19648,7 @@
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -19658,7 +19658,7 @@
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body0] · evidence/test-task-integration-final.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body0] · evidence/test-validation-task.log</t>
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr">
@@ -19742,7 +19742,7 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -19752,7 +19752,7 @@
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body1] · evidence/test-task-integration-final.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body1] · evidence/test-validation-task.log</t>
         </is>
       </c>
       <c r="Q12" s="10" t="inlineStr">
@@ -19807,7 +19807,7 @@
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
@@ -19817,7 +19817,7 @@
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body2] · evidence/test-task-integration-final.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body2] · evidence/test-validation-task.log</t>
         </is>
       </c>
       <c r="Q13" s="10" t="inlineStr">
@@ -19868,7 +19868,7 @@
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
@@ -19878,7 +19878,7 @@
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body3] · evidence/test-task-integration-final.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body3] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -19917,7 +19917,7 @@
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -19927,11 +19927,11 @@
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body4] · evidence/test-task-integration-final.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="90.5" customHeight="1">
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body4] · evidence/test-validation-task.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="74" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>TC-FCMTOKEN-08</t>
@@ -19965,7 +19965,7 @@
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
@@ -19975,7 +19975,7 @@
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_one_character_token_boundary__AC1 · evidence/test-task-integration-final.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_one_character_token_boundary__AC1 · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -20013,7 +20013,7 @@
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -20023,11 +20023,11 @@
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>AC1, AC8 · EP (1) · chuyển trạng thái/ownership · test_missing_expired_and_admin_sessions_rejected__AC1_AC8[PUT] · evidence/test-task-integration-final.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="107" customHeight="1">
+          <t>AC1, AC8 · EP (1) · chuyển trạng thái/ownership · test_missing_expired_and_admin_sessions_rejected__AC1_AC8[PUT] · evidence/test-validation-task.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90.5" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
           <t>TC-FCMTOKEN-10</t>
@@ -20061,7 +20061,7 @@
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
@@ -20071,7 +20071,7 @@
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>AC1, AC8 · EP (1) · chuyển trạng thái/ownership · test_missing_expired_and_admin_sessions_rejected__AC1_AC8[DELETE] · evidence/test-task-integration-final.log</t>
+          <t>AC1, AC8 · EP (1) · chuyển trạng thái/ownership · test_missing_expired_and_admin_sessions_rejected__AC1_AC8[DELETE] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -20110,7 +20110,7 @@
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
@@ -20120,7 +20120,7 @@
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_concurrent_registration_serializes_absent_token__AC1[False] · evidence/test-task-integration-final.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_concurrent_registration_serializes_absent_token__AC1[False] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -20159,7 +20159,7 @@
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
@@ -20169,7 +20169,7 @@
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_concurrent_registration_serializes_absent_token__AC1[True] · evidence/test-task-integration-final.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_concurrent_registration_serializes_absent_token__AC1[True] · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -20208,7 +20208,7 @@
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy tự động: các kiểm tra response và DB nêu ở Expected Result đều pass.</t>
+          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
@@ -20218,7 +20218,7 @@
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>AC1, AC8 · EP (1) · chuyển trạng thái/ownership · test_concurrent_refresh_then_cleanup_has_no_token_left__AC1_AC8 · evidence/test-task-integration-final.log</t>
+          <t>AC1, AC8 · EP (1) · chuyển trạng thái/ownership · test_concurrent_refresh_then_cleanup_has_no_token_left__AC1_AC8 · evidence/test-validation-task.log</t>
         </is>
       </c>
     </row>
@@ -23265,7 +23265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -24237,7 +24237,7 @@
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>Có lỗi validation 503 thay 422; FCM/OS/iOS thật còn Pending.</t>
+          <t>API/DB local đã kiểm lại sau sửa validation; kiểm thiết bị và AC8 còn Pending.</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
@@ -24281,7 +24281,7 @@
       </c>
       <c r="H29" s="10" t="inlineStr">
         <is>
-          <t>API local pass; chưa nghiệm thu AC8 từ DELETE đơn lẻ.</t>
+          <t>API/DB local đã kiểm lại sau sửa validation; kiểm thiết bị và AC8 còn Pending.</t>
         </is>
       </c>
       <c r="I29" s="11" t="inlineStr">
@@ -24780,206 +24780,6 @@
         <is>
           <t>Nghi vấn kỳ vọng chuẩn hóa tới phút trong test không khớp hành vi giữ thời điểm của API; chưa xác định phía nào sai theo contract/nghiệp vụ. Chưa chứng minh mất/trùng bản ghi liều; mức Medium tạm thời cho sai khác test, phải nâng tối thiểu High nếu xác nhận mất/trùng liều.
 Log: evidence/test-integration-db.log; evidence/test-dose-mismatch-repeat.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="156.5" customHeight="1">
-      <c r="A63" s="22" t="inlineStr">
-        <is>
-          <t>BUG-FALERT-19</t>
-        </is>
-      </c>
-      <c r="B63" s="22" t="inlineStr">
-        <is>
-          <t>Lọc hộp thư mixed patient và từ chối patient_id trong PATCH</t>
-        </is>
-      </c>
-      <c r="C63" s="22" t="inlineStr">
-        <is>
-          <t>1. Tạo hai notification cho F: P được phép và Q không có liên kết.
-2. GET /notifications?patient_id=P&amp;user_id=Q; kiểm item và count.
-3. PATCH notification Q với JSON {is_read:true,patient_id:P}.</t>
-        </is>
-      </c>
-      <c r="D63" s="22" t="inlineStr">
-        <is>
-          <t>P/F là UUID synthetic mới mỗi lần; ID notification lấy từ DB fixture; giờ 2026-10-20T01:00:00Z.</t>
-        </is>
-      </c>
-      <c r="E63" s="22" t="inlineStr">
-        <is>
-          <t>List chỉ trả P, total=unread_count=1 và Q có denied; PATCH field lạ phải trả 422.</t>
-        </is>
-      </c>
-      <c r="F63" s="22" t="inlineStr">
-        <is>
-          <t>HTTP 503 notification_access_unavailable thay vì 422; assertion fail.</t>
-        </is>
-      </c>
-      <c r="G63" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H63" s="22" t="inlineStr">
-        <is>
-          <t>phucnguyenngoc</t>
-        </is>
-      </c>
-      <c r="I63" s="22" t="inlineStr">
-        <is>
-          <t>Nghi vấn đã đối chiếu code: get_notification_uow bắt RequestValidationError trong except Exception và đổi thành ServiceUnavailable; NotificationRoute trả 503. Cùng một lỗi gốc ở 4 biến thể.
-Log: evidence/test-task-integration-final.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="123.5" customHeight="1">
-      <c r="A64" s="22" t="inlineStr">
-        <is>
-          <t>BUG-FALERT-36</t>
-        </is>
-      </c>
-      <c r="B64" s="22" t="inlineStr">
-        <is>
-          <t>Từ chối tham số phân trang ngoài biên [params0]</t>
-        </is>
-      </c>
-      <c r="C64" s="22" t="inlineStr">
-        <is>
-          <t>1. Đăng nhập F có notification và quyền hợp lệ.
-2. GET /notifications với limit=0, limit=101 hoặc offset=-1 theo Test Data.
-3. Kiểm HTTP status và Cache-Control.</t>
-        </is>
-      </c>
-      <c r="D64" s="22" t="inlineStr">
-        <is>
-          <t>limit=0; offset=0</t>
-        </is>
-      </c>
-      <c r="E64" s="22" t="inlineStr">
-        <is>
-          <t>422 validation, Cache-Control:no-store; không trả dữ liệu notification.</t>
-        </is>
-      </c>
-      <c r="F64" s="22" t="inlineStr">
-        <is>
-          <t>HTTP 503 notification_access_unavailable thay vì 422; assertion fail.</t>
-        </is>
-      </c>
-      <c r="G64" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H64" s="22" t="inlineStr">
-        <is>
-          <t>phucnguyenngoc</t>
-        </is>
-      </c>
-      <c r="I64" s="22" t="inlineStr">
-        <is>
-          <t>Nghi vấn đã đối chiếu code: get_notification_uow bắt RequestValidationError trong except Exception và đổi thành ServiceUnavailable; NotificationRoute trả 503. Cùng một lỗi gốc ở 4 biến thể.
-Log: evidence/test-task-integration-final.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="123.5" customHeight="1">
-      <c r="A65" s="22" t="inlineStr">
-        <is>
-          <t>BUG-FALERT-37</t>
-        </is>
-      </c>
-      <c r="B65" s="22" t="inlineStr">
-        <is>
-          <t>Từ chối tham số phân trang ngoài biên [params1]</t>
-        </is>
-      </c>
-      <c r="C65" s="22" t="inlineStr">
-        <is>
-          <t>1. Đăng nhập F có notification và quyền hợp lệ.
-2. GET /notifications với limit=0, limit=101 hoặc offset=-1 theo Test Data.
-3. Kiểm HTTP status và Cache-Control.</t>
-        </is>
-      </c>
-      <c r="D65" s="22" t="inlineStr">
-        <is>
-          <t>limit=101; offset=0</t>
-        </is>
-      </c>
-      <c r="E65" s="22" t="inlineStr">
-        <is>
-          <t>422 validation, Cache-Control:no-store; không trả dữ liệu notification.</t>
-        </is>
-      </c>
-      <c r="F65" s="22" t="inlineStr">
-        <is>
-          <t>HTTP 503 notification_access_unavailable thay vì 422; assertion fail.</t>
-        </is>
-      </c>
-      <c r="G65" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H65" s="22" t="inlineStr">
-        <is>
-          <t>phucnguyenngoc</t>
-        </is>
-      </c>
-      <c r="I65" s="22" t="inlineStr">
-        <is>
-          <t>Nghi vấn đã đối chiếu code: get_notification_uow bắt RequestValidationError trong except Exception và đổi thành ServiceUnavailable; NotificationRoute trả 503. Cùng một lỗi gốc ở 4 biến thể.
-Log: evidence/test-task-integration-final.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="123.5" customHeight="1">
-      <c r="A66" s="22" t="inlineStr">
-        <is>
-          <t>BUG-FALERT-38</t>
-        </is>
-      </c>
-      <c r="B66" s="22" t="inlineStr">
-        <is>
-          <t>Từ chối tham số phân trang ngoài biên [params2]</t>
-        </is>
-      </c>
-      <c r="C66" s="22" t="inlineStr">
-        <is>
-          <t>1. Đăng nhập F có notification và quyền hợp lệ.
-2. GET /notifications với limit=0, limit=101 hoặc offset=-1 theo Test Data.
-3. Kiểm HTTP status và Cache-Control.</t>
-        </is>
-      </c>
-      <c r="D66" s="22" t="inlineStr">
-        <is>
-          <t>limit=20; offset=-1</t>
-        </is>
-      </c>
-      <c r="E66" s="22" t="inlineStr">
-        <is>
-          <t>422 validation, Cache-Control:no-store; không trả dữ liệu notification.</t>
-        </is>
-      </c>
-      <c r="F66" s="22" t="inlineStr">
-        <is>
-          <t>HTTP 503 notification_access_unavailable thay vì 422; assertion fail.</t>
-        </is>
-      </c>
-      <c r="G66" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H66" s="22" t="inlineStr">
-        <is>
-          <t>phucnguyenngoc</t>
-        </is>
-      </c>
-      <c r="I66" s="22" t="inlineStr">
-        <is>
-          <t>Nghi vấn đã đối chiếu code: get_notification_uow bắt RequestValidationError trong except Exception và đổi thành ServiceUnavailable; NotificationRoute trả 503. Cùng một lỗi gốc ở 4 biến thể.
-Log: evidence/test-task-integration-final.log</t>
         </is>
       </c>
     </row>
@@ -24998,7 +24798,7 @@
       <formula>OR(G11="Critical",G11="High")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G54:G66">
+  <conditionalFormatting sqref="G54:G62">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
@@ -25013,7 +24813,7 @@
     <dataValidation sqref="G11:G29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="G54:G66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G54:G62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(tests): update Test Cases.xlsx with revised test scenarios
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -45,7 +45,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Khung điều hướng app'!$A$8:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Duyệt yêu cầu liên kết'!$A$8:$I$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Người giám sát'!$A$8:$I$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Cảnh báo người thân'!$A$8:$I$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Cảnh báo người thân'!$A$8:$I$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'FCM token Android'!$A$8:$I$21</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -15113,7 +15113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W87"/>
+  <dimension ref="A1:W94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15356,7 +15356,7 @@
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -15366,7 +15366,7 @@
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC4 · đoán lỗi, chuyển trạng thái và bảo mật · test_allowed_list_detail_patch_use_read_audit_and_replay__AC3_AC4 · evidence/test-validation-task.log</t>
+          <t>AC3, AC4 · đoán lỗi, chuyển trạng thái và bảo mật · test_allowed_list_detail_patch_use_read_audit_and_replay__AC3_AC4 · evidence/test-snapshot-task.log</t>
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr">
@@ -15467,7 +15467,7 @@
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -15477,7 +15477,7 @@
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-unlinked] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-unlinked] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
       <c r="K10" s="9" t="inlineStr">
@@ -15576,7 +15576,7 @@
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -15586,7 +15586,7 @@
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-inactive] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-inactive] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
       <c r="Q11" s="10" t="inlineStr">
@@ -15660,7 +15660,7 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -15670,7 +15670,7 @@
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R3) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-sharing_off] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R3) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-sharing_off] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
       <c r="Q12" s="10" t="inlineStr">
@@ -15744,7 +15744,7 @@
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
@@ -15754,7 +15754,7 @@
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R4) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-health_data] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R4) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-health_data] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
       <c r="Q13" s="10" t="inlineStr">
@@ -15828,7 +15828,7 @@
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
@@ -15838,7 +15838,7 @@
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R5) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-family_sharing] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R5) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[list-family_sharing] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
       <c r="Q14" s="6" t="inlineStr">
@@ -15912,7 +15912,7 @@
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -15922,7 +15922,7 @@
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-unlinked] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-unlinked] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
       <c r="Q15" s="10" t="inlineStr">
@@ -15976,7 +15976,7 @@
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
@@ -15986,7 +15986,7 @@
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-inactive] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-inactive] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
       <c r="Q16" s="10" t="inlineStr">
@@ -16052,7 +16052,7 @@
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -16062,7 +16062,7 @@
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R3) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-sharing_off] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R3) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-sharing_off] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
       <c r="Q17" s="10" t="inlineStr">
@@ -16116,7 +16116,7 @@
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
@@ -16126,7 +16126,7 @@
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R4) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-health_data] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R4) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-health_data] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16165,7 +16165,7 @@
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
@@ -16175,7 +16175,7 @@
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R5) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-family_sharing] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R5) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[detail-family_sharing] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16214,7 +16214,7 @@
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
@@ -16224,7 +16224,7 @@
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-unlinked] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-unlinked] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16263,7 +16263,7 @@
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
@@ -16273,7 +16273,7 @@
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-inactive] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R2) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-inactive] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16312,7 @@
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
@@ -16322,7 +16322,7 @@
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R3) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-sharing_off] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R3) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-sharing_off] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16361,7 +16361,7 @@
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
@@ -16371,7 +16371,7 @@
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R4) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-health_data] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R4) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-health_data] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16410,7 +16410,7 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
@@ -16420,7 +16420,7 @@
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R5) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-family_sharing] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R5) · test_revocation_next_request_filters_counts_or_denies_and_audits__AC5[patch-family_sharing] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16459,7 +16459,7 @@
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
@@ -16469,7 +16469,7 @@
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_other_recipient_and_unknown_id_return_404__AC5[detail] · evidence/test-validation-task.log</t>
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_other_recipient_and_unknown_id_return_404__AC5[detail] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16508,7 +16508,7 @@
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
@@ -16518,7 +16518,7 @@
       </c>
       <c r="I26" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_other_recipient_and_unknown_id_return_404__AC5[patch] · evidence/test-validation-task.log</t>
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_other_recipient_and_unknown_id_return_404__AC5[patch] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16557,7 +16557,7 @@
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
@@ -16567,7 +16567,7 @@
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_mixed_patient_filter_and_selector_tamper_do_not_leak__AC3_AC5 · evidence/test-validation-task.log</t>
+          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_mixed_patient_filter_and_selector_tamper_do_not_leak__AC3_AC5 · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16605,7 +16605,7 @@
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
@@ -16615,7 +16615,7 @@
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_admin_session_forbidden__AC5[list] · evidence/test-validation-task.log</t>
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_admin_session_forbidden__AC5[list] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16653,7 +16653,7 @@
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
@@ -16663,7 +16663,7 @@
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_admin_session_forbidden__AC5[detail] · evidence/test-validation-task.log</t>
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_admin_session_forbidden__AC5[detail] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16701,7 +16701,7 @@
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
@@ -16711,7 +16711,7 @@
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_admin_session_forbidden__AC5[patch] · evidence/test-validation-task.log</t>
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_admin_session_forbidden__AC5[patch] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16750,7 +16750,7 @@
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
@@ -16760,7 +16760,7 @@
       </c>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[facts-list] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[facts-list] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16799,7 +16799,7 @@
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
@@ -16809,7 +16809,7 @@
       </c>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[facts-detail] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[facts-detail] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16848,7 +16848,7 @@
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
@@ -16858,7 +16858,7 @@
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[facts-patch] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[facts-patch] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16897,7 +16897,7 @@
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
@@ -16907,7 +16907,7 @@
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[allowed_insert-list] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[allowed_insert-list] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16946,7 +16946,7 @@
       </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
@@ -16956,7 +16956,7 @@
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[allowed_insert-detail] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[allowed_insert-detail] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -16995,7 +16995,7 @@
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
@@ -17005,7 +17005,7 @@
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[allowed_insert-patch] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[allowed_insert-patch] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17044,7 +17044,7 @@
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
@@ -17054,7 +17054,7 @@
       </c>
       <c r="I37" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[denied_insert-list] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[denied_insert-list] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17093,7 +17093,7 @@
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
@@ -17103,7 +17103,7 @@
       </c>
       <c r="I38" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[denied_insert-detail] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[denied_insert-detail] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17142,7 +17142,7 @@
       </c>
       <c r="G39" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
@@ -17152,7 +17152,7 @@
       </c>
       <c r="I39" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[denied_insert-patch] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[denied_insert-patch] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17191,7 +17191,7 @@
       </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
@@ -17201,7 +17201,7 @@
       </c>
       <c r="I40" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[commit-list] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[commit-list] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17240,7 +17240,7 @@
       </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
@@ -17250,7 +17250,7 @@
       </c>
       <c r="I41" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[commit-detail] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[commit-detail] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17289,7 +17289,7 @@
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
@@ -17299,7 +17299,7 @@
       </c>
       <c r="I42" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[commit-patch] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R6) · test_access_audit_commit_failure_returns_503_without_health_or_write__AC5[commit-patch] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17338,7 +17338,7 @@
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
@@ -17348,7 +17348,7 @@
       </c>
       <c r="I43" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_denied_audit_survives_request_transaction_rollback__AC5 · evidence/test-validation-task.log</t>
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_denied_audit_survives_request_transaction_rollback__AC5 · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17387,7 +17387,7 @@
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
@@ -17397,7 +17397,7 @@
       </c>
       <c r="I44" s="8" t="inlineStr">
         <is>
-          <t>AC3 · BVA (min-1), EP (3) · test_invalid_pagination_is_422_no_store__AC3[params0] · evidence/test-validation-task.log</t>
+          <t>AC3 · BVA (min-1), EP (3) · test_invalid_pagination_is_422_no_store__AC3[params0] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17436,7 +17436,7 @@
       </c>
       <c r="G45" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
@@ -17446,7 +17446,7 @@
       </c>
       <c r="I45" s="8" t="inlineStr">
         <is>
-          <t>AC3 · BVA (max+1), EP (4) · test_invalid_pagination_is_422_no_store__AC3[params1] · evidence/test-validation-task.log</t>
+          <t>AC3 · BVA (max+1), EP (4) · test_invalid_pagination_is_422_no_store__AC3[params1] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17485,7 +17485,7 @@
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
@@ -17495,7 +17495,7 @@
       </c>
       <c r="I46" s="8" t="inlineStr">
         <is>
-          <t>AC3 · BVA (min-1), EP (5) · test_invalid_pagination_is_422_no_store__AC3[params2] · evidence/test-validation-task.log</t>
+          <t>AC3 · BVA (min-1), EP (5) · test_invalid_pagination_is_422_no_store__AC3[params2] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17533,7 +17533,7 @@
       </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
@@ -17543,7 +17543,7 @@
       </c>
       <c r="I47" s="8" t="inlineStr">
         <is>
-          <t>AC3 · BVA (min), EP (1,2) · test_valid_pagination_boundaries__AC3[1] · evidence/test-validation-task.log</t>
+          <t>AC3 · BVA (min), EP (1,2) · test_valid_pagination_boundaries__AC3[1] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17581,7 +17581,7 @@
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
@@ -17591,7 +17591,7 @@
       </c>
       <c r="I48" s="8" t="inlineStr">
         <is>
-          <t>AC3 · BVA (max), EP (1,2) · test_valid_pagination_boundaries__AC3[100] · evidence/test-validation-task.log</t>
+          <t>AC3 · BVA (max), EP (1,2) · test_valid_pagination_boundaries__AC3[100] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17630,7 +17630,7 @@
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
@@ -17640,7 +17640,7 @@
       </c>
       <c r="I49" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[list-missing] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[list-missing] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17679,7 +17679,7 @@
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
@@ -17689,7 +17689,7 @@
       </c>
       <c r="I50" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[list-pending] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[list-pending] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17728,7 +17728,7 @@
       </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
@@ -17738,7 +17738,7 @@
       </c>
       <c r="I51" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[detail-missing] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[detail-missing] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr">
@@ -17787,7 +17787,7 @@
       </c>
       <c r="I52" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[detail-pending] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[detail-pending] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17826,7 +17826,7 @@
       </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
@@ -17836,7 +17836,7 @@
       </c>
       <c r="I53" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[patch-missing] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[patch-missing] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17875,7 +17875,7 @@
       </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr">
@@ -17885,7 +17885,7 @@
       </c>
       <c r="I54" s="8" t="inlineStr">
         <is>
-          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[patch-pending] · evidence/test-validation-task.log</t>
+          <t>AC5 · Decision Table (R2) · test_initial_missing_or_pending_link_denied_with_audit__AC5[patch-pending] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17923,7 +17923,7 @@
       </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr">
@@ -17933,7 +17933,7 @@
       </c>
       <c r="I55" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_missing_session_returns_401_no_store__AC5[list] · evidence/test-validation-task.log</t>
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_missing_session_returns_401_no_store__AC5[list] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -17971,7 +17971,7 @@
       </c>
       <c r="G56" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr">
@@ -17981,7 +17981,7 @@
       </c>
       <c r="I56" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_missing_session_returns_401_no_store__AC5[detail] · evidence/test-validation-task.log</t>
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_missing_session_returns_401_no_store__AC5[detail] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -18019,7 +18019,7 @@
       </c>
       <c r="G57" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr">
@@ -18029,7 +18029,7 @@
       </c>
       <c r="I57" s="8" t="inlineStr">
         <is>
-          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_missing_session_returns_401_no_store__AC5[patch] · evidence/test-validation-task.log</t>
+          <t>AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_missing_session_returns_401_no_store__AC5[patch] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -18069,7 +18069,7 @@
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr">
@@ -18079,7 +18079,7 @@
       </c>
       <c r="I58" s="8" t="inlineStr">
         <is>
-          <t>AC2, AC3, AC4 · đoán lỗi, chuyển trạng thái và bảo mật · test_scan_snapshot_survives_catalog_schedule_edit_and_replay__AC2_AC3_AC4 · evidence/test-validation-task.log</t>
+          <t>AC2, AC3, AC4 · đoán lỗi, chuyển trạng thái và bảo mật · test_scan_snapshot_survives_catalog_schedule_edit_and_replay__AC2_AC3_AC4 · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -18118,7 +18118,7 @@
       </c>
       <c r="G59" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
@@ -18128,7 +18128,7 @@
       </c>
       <c r="I59" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC4 · đoán lỗi, chuyển trạng thái và bảo mật · test_filter_offset_tied_order_and_global_badge__AC3_AC4 · evidence/test-validation-task.log</t>
+          <t>AC3, AC4 · đoán lỗi, chuyển trạng thái và bảo mật · test_filter_offset_tied_order_and_global_badge__AC3_AC4 · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -18167,7 +18167,7 @@
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr">
@@ -18177,7 +18177,7 @@
       </c>
       <c r="I60" s="8" t="inlineStr">
         <is>
-          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_worker_database_race_never_overwrites_confirmation__AC3[False] · evidence/test-validation-task.log</t>
+          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_worker_database_race_never_overwrites_confirmation__AC3[False] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -18216,7 +18216,7 @@
       </c>
       <c r="G61" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr">
@@ -18226,7 +18226,7 @@
       </c>
       <c r="I61" s="8" t="inlineStr">
         <is>
-          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_worker_database_race_never_overwrites_confirmation__AC3[True] · evidence/test-validation-task.log</t>
+          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_worker_database_race_never_overwrites_confirmation__AC3[True] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -18265,7 +18265,7 @@
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr">
@@ -18275,7 +18275,7 @@
       </c>
       <c r="I62" s="8" t="inlineStr">
         <is>
-          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_upgrade_preserves_legacy_and_read_update__AC3 · evidence/test-validation-task.log</t>
+          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_upgrade_preserves_legacy_and_read_update__AC3 · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -18313,7 +18313,7 @@
       </c>
       <c r="G63" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">
@@ -18323,7 +18323,7 @@
       </c>
       <c r="I63" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC4 · đoán lỗi, chuyển trạng thái và bảo mật · test_legacy_null_snapshot_can_be_read_and_marked__AC3_AC4 · evidence/test-validation-task.log</t>
+          <t>AC3, AC4 · đoán lỗi, chuyển trạng thái và bảo mật · test_legacy_null_snapshot_can_be_read_and_marked__AC3_AC4 · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -18361,7 +18361,7 @@
       </c>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr">
@@ -18371,7 +18371,7 @@
       </c>
       <c r="I64" s="8" t="inlineStr">
         <is>
-          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_new_insert_requires_snapshot__AC3[None-at0] · evidence/test-validation-task.log</t>
+          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_new_insert_requires_snapshot__AC3[None-at0] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -18409,7 +18409,7 @@
       </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr">
@@ -18419,7 +18419,7 @@
       </c>
       <c r="I65" s="8" t="inlineStr">
         <is>
-          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_new_insert_requires_snapshot__AC3[-at1] · evidence/test-validation-task.log</t>
+          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_new_insert_requires_snapshot__AC3[-at1] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -18457,7 +18457,7 @@
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr">
@@ -18467,7 +18467,7 @@
       </c>
       <c r="I66" s="8" t="inlineStr">
         <is>
-          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_new_insert_requires_snapshot__AC3[   -at2] · evidence/test-validation-task.log</t>
+          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_new_insert_requires_snapshot__AC3[   -at2] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -18505,7 +18505,7 @@
       </c>
       <c r="G67" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr">
@@ -18515,7 +18515,7 @@
       </c>
       <c r="I67" s="8" t="inlineStr">
         <is>
-          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_new_insert_requires_snapshot__AC3[Valid-None] · evidence/test-validation-task.log</t>
+          <t>AC3 · đoán lỗi, chuyển trạng thái và bảo mật · test_new_insert_requires_snapshot__AC3[Valid-None] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -18554,7 +18554,7 @@
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr">
@@ -18564,7 +18564,7 @@
       </c>
       <c r="I68" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_snapshot_roles_rls_and_indexes__AC3_AC5[anon] · evidence/test-validation-task.log</t>
+          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_snapshot_roles_rls_and_indexes__AC3_AC5[anon] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -18603,7 +18603,7 @@
       </c>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr">
@@ -18613,7 +18613,7 @@
       </c>
       <c r="I69" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_snapshot_roles_rls_and_indexes__AC3_AC5[authenticated] · evidence/test-validation-task.log</t>
+          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_snapshot_roles_rls_and_indexes__AC3_AC5[authenticated] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -18652,7 +18652,7 @@
       </c>
       <c r="G70" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr">
@@ -18662,7 +18662,7 @@
       </c>
       <c r="I70" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_snapshot_roles_rls_and_indexes__AC3_AC5[api_role] · evidence/test-validation-task.log</t>
+          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_snapshot_roles_rls_and_indexes__AC3_AC5[api_role] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -18701,7 +18701,7 @@
       </c>
       <c r="G71" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr">
@@ -18711,7 +18711,7 @@
       </c>
       <c r="I71" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_snapshot_roles_rls_and_indexes__AC3_AC5[worker_role] · evidence/test-validation-task.log</t>
+          <t>AC3, AC5 · đoán lỗi, chuyển trạng thái và bảo mật · test_snapshot_roles_rls_and_indexes__AC3_AC5[worker_role] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -19152,7 +19152,7 @@
       </c>
       <c r="G81" s="8" t="inlineStr">
         <is>
-          <t>Hai widget tests pass trong lần chạy mới; không phải bằng chứng iOS runtime.</t>
+          <t>Hai widget tests pass ở lượt hiện tại; chưa kiểm iOS runtime.</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr">
@@ -19162,65 +19162,401 @@
       </c>
       <c r="I81" s="8" t="inlineStr">
         <is>
-          <t>AC3, AC7 · widget · evidence/test-validation-widget.log; không phải iOS runtime</t>
-        </is>
-      </c>
-    </row>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84">
-      <c r="G84" s="12" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="H84" s="13">
-        <f>COUNTIF(H9:H81,"Pass")</f>
+          <t>AC3, AC7 · widget · evidence/test-snapshot-mobile-widget.log; không phải iOS runtime</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="107" customHeight="1">
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>TC-FALERT-74</t>
+        </is>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>Giữ cửa sổ 120 phút, retry và liều đã xác nhận khi scan có snapshot</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>Supabase local đã reset; fixture synthetic, không đổi assertion hoặc bypass PEP.</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>1. Hai lượt scan occurrence tại 120 phút, +1 microsecond và đã confirmed; đọc lịch sử.
+2. Chạy pytest tests/integration/test_adherence_history_api.py::test_worker_window_notifications_use_strict_120_and_preserve_confirmed__AC22.</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t>Ngày 2026-10-19 Asia/Ho_Chi_Minh; Integration medicine; UUID/ID synthetic theo fixture.</t>
+        </is>
+      </c>
+      <c r="F82" s="8" t="inlineStr">
+        <is>
+          <t>Đúng 120 phút chưa missed; vượt 1 microsecond mới missed; retry không trùng/ghi đè; history/schema đúng.</t>
+        </is>
+      </c>
+      <c r="G82" s="8" t="inlineStr">
+        <is>
+          <t>Scan và kiểm dose/count đã qua; kiểm history cuối ca fail KeyError: AdherenceByDateResponse.</t>
+        </is>
+      </c>
+      <c r="H82" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I82" s="8" t="inlineStr">
+        <is>
+          <t>AC3–AC5, AC6 · I9 · BVA/chuyển trạng thái/quyền · test_worker_window_notifications_use_strict_120_and_preserve_confirmed__AC22 · evidence/test-snapshot-green.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="90.5" customHeight="1">
+      <c r="A83" s="7" t="inlineStr">
+        <is>
+          <t>TC-FALERT-75</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Chặn api_role ghi notification khi fixture có context hợp lệ</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>Supabase local đã reset; fixture synthetic, không đổi assertion hoặc bypass PEP.</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy scan bằng api_role trong transaction; đọc dose/notification sau rollback.
+2. Chạy pytest tests/integration/test_adherence_history_api.py::test_api_role_cannot_create_worker_notifications.</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>Ngày 2026-10-19 Asia/Ho_Chi_Minh; Integration medicine; UUID/ID synthetic theo fixture.</t>
+        </is>
+      </c>
+      <c r="F83" s="8" t="inlineStr">
+        <is>
+          <t>Permission denied for table notifications; rollback không còn dose/notification.</t>
+        </is>
+      </c>
+      <c r="G83" s="8" t="inlineStr">
+        <is>
+          <t>Pass: đến đúng nhánh permission denied và giữ rollback dose/notification.</t>
+        </is>
+      </c>
+      <c r="H83" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I83" s="8" t="inlineStr">
+        <is>
+          <t>AC3–AC5, AC6 · I9 · BVA/chuyển trạng thái/quyền · test_api_role_cannot_create_worker_notifications · evidence/test-snapshot-green.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="123.5" customHeight="1">
+      <c r="A84" s="7" t="inlineStr">
+        <is>
+          <t>TC-FALERT-76</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>Giữ race Worker trước xác nhận trễ khi event có snapshot</t>
+        </is>
+      </c>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>Supabase local đã reset; fixture synthetic, không đổi assertion hoặc bypass PEP.</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>1. Worker giữ lock; gửi xác nhận taken_at +90 phút cùng occurrence; commit; retry client_uuid; đọc lịch sử.
+2. Chạy pytest tests/integration/test_adherence_history_api.py::test_worker_insert_races_with_valid_late_confirmation__AC15_AC20_AC22[worker].</t>
+        </is>
+      </c>
+      <c r="E84" s="8" t="inlineStr">
+        <is>
+          <t>Ngày 2026-10-19 Asia/Ho_Chi_Minh; Integration medicine; UUID/ID synthetic theo fixture.</t>
+        </is>
+      </c>
+      <c r="F84" s="8" t="inlineStr">
+        <is>
+          <t>Writer chờ unique lock; chỉ một dose uong_tre, taken_at đúng; một notification; history đúng.</t>
+        </is>
+      </c>
+      <c r="G84" s="8" t="inlineStr">
+        <is>
+          <t>Kiểm lock, retry, một dose uong_tre/taken_at và notification đã qua; history fail KeyError: AdherenceByDateResponse.</t>
+        </is>
+      </c>
+      <c r="H84" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I84" s="8" t="inlineStr">
+        <is>
+          <t>AC3–AC5, AC6 · I9 · BVA/chuyển trạng thái/quyền · test_worker_insert_races_with_valid_late_confirmation__AC15_AC20_AC22[worker] · evidence/test-snapshot-green.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="107" customHeight="1">
+      <c r="A85" s="7" t="inlineStr">
+        <is>
+          <t>TC-FALERT-77</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>Đọc inbox sau seed alert có snapshot đầy đủ</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>Supabase local đã reset; fixture synthetic, không đổi assertion hoặc bypass PEP.</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>1. Seed snapshot thuốc/giờ; dùng client_as người nhận gọi GET /notifications.
+2. Chạy pytest tests/integration/test_alert_dispatch_api.py::test_integration_missed_dose_alert_dispatch_and_inbox_fetch__AC1_AC2_AC6.</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="inlineStr">
+        <is>
+          <t>Ngày 2026-10-19 Asia/Ho_Chi_Minh; Integration medicine; UUID/ID synthetic theo fixture.</t>
+        </is>
+      </c>
+      <c r="F85" s="8" t="inlineStr">
+        <is>
+          <t>200; đúng content, recipient, is_read=false, total/unread_count.</t>
+        </is>
+      </c>
+      <c r="G85" s="8" t="inlineStr">
+        <is>
+          <t>INSERT snapshot đã qua; GET trả 401 thay 200, chưa kiểm được payload.</t>
+        </is>
+      </c>
+      <c r="H85" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I85" s="8" t="inlineStr">
+        <is>
+          <t>AC3–AC5, AC6 · I9 · BVA/chuyển trạng thái/quyền · test_integration_missed_dose_alert_dispatch_and_inbox_fetch__AC1_AC2_AC6 · evidence/test-snapshot-green.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="90.5" customHeight="1">
+      <c r="A86" s="7" t="inlineStr">
+        <is>
+          <t>TC-FALERT-78</t>
+        </is>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>Đánh dấu đọc và từ chối recipient lạ sau seed snapshot</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t>Supabase local đã reset; fixture synthetic, không đổi assertion hoặc bypass PEP.</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>1. Seed snapshot; client_as người nhận PATCH is_read=true; thử lại bằng user khác.
+2. Chạy pytest tests/integration/test_alert_dispatch_api.py::test_integration_patch_notification_marks_as_read__AC7.</t>
+        </is>
+      </c>
+      <c r="E86" s="8" t="inlineStr">
+        <is>
+          <t>Ngày 2026-10-19 Asia/Ho_Chi_Minh; Integration medicine; UUID/ID synthetic theo fixture.</t>
+        </is>
+      </c>
+      <c r="F86" s="8" t="inlineStr">
+        <is>
+          <t>Người nhận 200/is_read=true; người khác 404.</t>
+        </is>
+      </c>
+      <c r="G86" s="8" t="inlineStr">
+        <is>
+          <t>INSERT snapshot đã qua; PATCH trả 401 thay 200, chưa tới kiểm foreign-recipient.</t>
+        </is>
+      </c>
+      <c r="H86" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I86" s="8" t="inlineStr">
+        <is>
+          <t>AC3–AC5, AC6 · I9 · BVA/chuyển trạng thái/quyền · test_integration_patch_notification_marks_as_read__AC7 · evidence/test-snapshot-green.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="90.5" customHeight="1">
+      <c r="A87" s="7" t="inlineStr">
+        <is>
+          <t>TC-FALERT-79</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm timing SQL/API và tên trong inbox khi fixture có snapshot</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>Supabase local đã reset; fixture synthetic, không đổi assertion hoặc bypass PEP.</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>1. Đo perf_counter quanh INSERT snapshot và GET inbox qua client_as.
+2. Chạy pytest tests/integration/test_alert_dispatch_api.py::test_integration_alert_timing_and_naming_flow.</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>Ngày 2026-10-19 Asia/Ho_Chi_Minh; Integration medicine; UUID/ID synthetic theo fixture.</t>
+        </is>
+      </c>
+      <c r="F87" s="8" t="inlineStr">
+        <is>
+          <t>200, content/recipient/is_read đúng; thời gian SQL/API &lt;2s, không chứng nhận FCM SLO.</t>
+        </is>
+      </c>
+      <c r="G87" s="8" t="inlineStr">
+        <is>
+          <t>INSERT snapshot đã qua; GET trả 401 trước các assertion timing/content.</t>
+        </is>
+      </c>
+      <c r="H87" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I87" s="8" t="inlineStr">
+        <is>
+          <t>AC3–AC5, AC6 · I9 · BVA/chuyển trạng thái/quyền · test_integration_alert_timing_and_naming_flow · evidence/test-snapshot-green.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="90.5" customHeight="1">
+      <c r="A88" s="7" t="inlineStr">
+        <is>
+          <t>TC-FALERT-80</t>
+        </is>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>Hiển thị badge unread server và xóa sau clear</t>
+        </is>
+      </c>
+      <c r="C88" s="8" t="inlineStr">
+        <is>
+          <t>Flutter test; FamilyAlertController với AlertRepo giả và session A.</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy flutter test test/features/family_link/family_tab_screen_test.dart.
+2. Kiểm 1 chưa đọc, điểm vào family-alerts; clear controller rồi kiểm badge biến mất.</t>
+        </is>
+      </c>
+      <c r="E88" s="8" t="inlineStr">
+        <is>
+          <t>AlertRepo fixture một item chưa đọc; session A.</t>
+        </is>
+      </c>
+      <c r="F88" s="8" t="inlineStr">
+        <is>
+          <t>Widget có badge 1 chưa đọc, sau clear không còn badge; không phát sinh exception.</t>
+        </is>
+      </c>
+      <c r="G88" s="8" t="inlineStr">
+        <is>
+          <t>Full Flutter fail trước kiểm badge: thiếu ConsentScope và FamilyLinkScope trong widget fixture.</t>
+        </is>
+      </c>
+      <c r="H88" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I88" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · đoán lỗi/tích hợp widget · alert entry displays server unread count and removes it after clear · evidence/test-snapshot-mobile.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91">
+      <c r="G91" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H91" s="13">
+        <f>COUNTIF(H9:H88,"Pass")</f>
         <v/>
       </c>
     </row>
-    <row r="85">
-      <c r="G85" s="12" t="inlineStr">
+    <row r="92">
+      <c r="G92" s="12" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="H85" s="13">
-        <f>COUNTIF(H9:H81,"Fail")</f>
+      <c r="H92" s="13">
+        <f>COUNTIF(H9:H88,"Fail")</f>
         <v/>
       </c>
     </row>
-    <row r="86">
-      <c r="G86" s="12" t="inlineStr">
+    <row r="93">
+      <c r="G93" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="H86" s="13">
-        <f>COUNTIF(H9:H81,"Pending")</f>
+      <c r="H93" s="13">
+        <f>COUNTIF(H9:H88,"Pending")</f>
         <v/>
       </c>
     </row>
-    <row r="87">
-      <c r="G87" s="12" t="inlineStr">
+    <row r="94">
+      <c r="G94" s="12" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="H87" s="13">
-        <f>SUM(H84:H86)</f>
+      <c r="H94" s="13">
+        <f>SUM(H91:H93)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A8:I81"/>
-  <conditionalFormatting sqref="H9:H81">
+  <autoFilter ref="A8:I88"/>
+  <conditionalFormatting sqref="H9:H88">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Fail"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H9:H81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H9:H88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pass,Fail,Pending"</formula1>
     </dataValidation>
   </dataValidations>
@@ -19458,7 +19794,7 @@
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -19468,7 +19804,7 @@
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>AC1, AC8 · EP (1) · chuyển trạng thái/ownership · test_replay_refresh_logout_and_dispatch_selection__AC1_AC8 · evidence/test-validation-task.log</t>
+          <t>AC1, AC8 · EP (1) · chuyển trạng thái/ownership · test_replay_refresh_logout_and_dispatch_selection__AC1_AC8 · evidence/test-snapshot-task.log</t>
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr">
@@ -19554,7 +19890,7 @@
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -19564,7 +19900,7 @@
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_conflicting_refresh_rolls_back_and_foreign_previous_is_preserved__AC1 · evidence/test-validation-task.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_conflicting_refresh_rolls_back_and_foreign_previous_is_preserved__AC1 · evidence/test-snapshot-task.log</t>
         </is>
       </c>
       <c r="K10" s="9" t="inlineStr">
@@ -19648,7 +19984,7 @@
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -19658,7 +19994,7 @@
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body0] · evidence/test-validation-task.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body0] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr">
@@ -19742,7 +20078,7 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -19752,7 +20088,7 @@
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body1] · evidence/test-validation-task.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body1] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
       <c r="Q12" s="10" t="inlineStr">
@@ -19807,7 +20143,7 @@
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
@@ -19817,7 +20153,7 @@
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body2] · evidence/test-validation-task.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body2] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
       <c r="Q13" s="10" t="inlineStr">
@@ -19868,7 +20204,7 @@
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
@@ -19878,7 +20214,7 @@
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body3] · evidence/test-validation-task.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body3] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -19917,7 +20253,7 @@
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -19927,7 +20263,7 @@
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body4] · evidence/test-validation-task.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_invalid_registration_is_rejected__AC1[body4] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -19965,7 +20301,7 @@
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
@@ -19975,7 +20311,7 @@
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_one_character_token_boundary__AC1 · evidence/test-validation-task.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_one_character_token_boundary__AC1 · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -20013,7 +20349,7 @@
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -20023,7 +20359,7 @@
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>AC1, AC8 · EP (1) · chuyển trạng thái/ownership · test_missing_expired_and_admin_sessions_rejected__AC1_AC8[PUT] · evidence/test-validation-task.log</t>
+          <t>AC1, AC8 · EP (1) · chuyển trạng thái/ownership · test_missing_expired_and_admin_sessions_rejected__AC1_AC8[PUT] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -20061,7 +20397,7 @@
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
@@ -20071,7 +20407,7 @@
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>AC1, AC8 · EP (1) · chuyển trạng thái/ownership · test_missing_expired_and_admin_sessions_rejected__AC1_AC8[DELETE] · evidence/test-validation-task.log</t>
+          <t>AC1, AC8 · EP (1) · chuyển trạng thái/ownership · test_missing_expired_and_admin_sessions_rejected__AC1_AC8[DELETE] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -20110,7 +20446,7 @@
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
@@ -20120,7 +20456,7 @@
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_concurrent_registration_serializes_absent_token__AC1[False] · evidence/test-validation-task.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_concurrent_registration_serializes_absent_token__AC1[False] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -20159,7 +20495,7 @@
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
@@ -20169,7 +20505,7 @@
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_concurrent_registration_serializes_absent_token__AC1[True] · evidence/test-validation-task.log</t>
+          <t>AC1 · EP (1) · chuyển trạng thái/ownership · test_concurrent_registration_serializes_absent_token__AC1[True] · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -20208,7 +20544,7 @@
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy lại sau sửa validation: kiểm response và DB của test tương ứng pass; đầu vào sai trả 422/no-store.</t>
+          <t>Test tương ứng pass trong bộ 76 integration trên Supabase local ở lượt kiểm snapshot; giữ kiểm response, quyền và hiệu ứng DB.</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
@@ -20218,7 +20554,7 @@
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>AC1, AC8 · EP (1) · chuyển trạng thái/ownership · test_concurrent_refresh_then_cleanup_has_no_token_left__AC1_AC8 · evidence/test-validation-task.log</t>
+          <t>AC1, AC8 · EP (1) · chuyển trạng thái/ownership · test_concurrent_refresh_then_cleanup_has_no_token_left__AC1_AC8 · evidence/test-snapshot-task.log</t>
         </is>
       </c>
     </row>
@@ -23265,7 +23601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -23319,7 +23655,7 @@
         <v/>
       </c>
       <c r="D3" s="11">
-        <f>'Chọn thuốc danh mục'!$H$40+'Hồi quy xác nhận liều'!$H$12+'Cảnh báo người thân'!$H$84+'FCM token Android'!$H$24</f>
+        <f>'Chọn thuốc danh mục'!$H$40+'Hồi quy xác nhận liều'!$H$12+'Cảnh báo người thân'!$H$91+'FCM token Android'!$H$24</f>
         <v/>
       </c>
       <c r="E3" s="15">
@@ -23339,7 +23675,7 @@
         <v/>
       </c>
       <c r="D4" s="11">
-        <f>'Chọn thuốc danh mục'!$H$41+'Hồi quy xác nhận liều'!$H$13+'Cảnh báo người thân'!$H$85+'FCM token Android'!$H$25</f>
+        <f>'Chọn thuốc danh mục'!$H$41+'Hồi quy xác nhận liều'!$H$13+'Cảnh báo người thân'!$H$92+'FCM token Android'!$H$25</f>
         <v/>
       </c>
       <c r="E4" s="15">
@@ -23379,7 +23715,7 @@
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>'Chọn thuốc danh mục'!$H$42+'Hồi quy xác nhận liều'!$H$14+'Cảnh báo người thân'!$H$86+'FCM token Android'!$H$26</f>
+        <f>'Chọn thuốc danh mục'!$H$42+'Hồi quy xác nhận liều'!$H$14+'Cảnh báo người thân'!$H$93+'FCM token Android'!$H$26</f>
         <v/>
       </c>
       <c r="E6" s="15">
@@ -24219,15 +24555,15 @@
         </is>
       </c>
       <c r="D28" s="18">
-        <f>IFERROR(('Cảnh báo người thân'!$H$87-'Cảnh báo người thân'!$H$86)/'Cảnh báo người thân'!$H$87,0)</f>
+        <f>IFERROR(('Cảnh báo người thân'!$H$94-'Cảnh báo người thân'!$H$93)/'Cảnh báo người thân'!$H$94,0)</f>
         <v/>
       </c>
       <c r="E28" s="18">
-        <f>IFERROR('Cảnh báo người thân'!$H$84/'Cảnh báo người thân'!$H$87,0)</f>
+        <f>IFERROR('Cảnh báo người thân'!$H$91/'Cảnh báo người thân'!$H$94,0)</f>
         <v/>
       </c>
       <c r="F28" s="18">
-        <f>IFERROR('Cảnh báo người thân'!$H$85/'Cảnh báo người thân'!$H$87,0)</f>
+        <f>IFERROR('Cảnh báo người thân'!$H$92/'Cảnh báo người thân'!$H$94,0)</f>
         <v/>
       </c>
       <c r="G28" s="11" t="inlineStr">
@@ -24237,7 +24573,7 @@
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>API/DB local đã kiểm lại sau sửa validation; kiểm thiết bị và AC8 còn Pending.</t>
+          <t>Kết quả API/DB và widget có log mới; regression contract/auth/fixture được báo riêng; thiết bị và AC8 còn Pending.</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
@@ -24281,7 +24617,7 @@
       </c>
       <c r="H29" s="10" t="inlineStr">
         <is>
-          <t>API/DB local đã kiểm lại sau sửa validation; kiểm thiết bị và AC8 còn Pending.</t>
+          <t>Kết quả API/DB và widget có log mới; regression contract/auth/fixture được báo riêng; thiết bị và AC8 còn Pending.</t>
         </is>
       </c>
       <c r="I29" s="11" t="inlineStr">
@@ -24780,6 +25116,300 @@
         <is>
           <t>Nghi vấn kỳ vọng chuẩn hóa tới phút trong test không khớp hành vi giữ thời điểm của API; chưa xác định phía nào sai theo contract/nghiệp vụ. Chưa chứng minh mất/trùng bản ghi liều; mức Medium tạm thời cho sai khác test, phải nâng tối thiểu High nếu xác nhận mất/trùng liều.
 Log: evidence/test-integration-db.log; evidence/test-dose-mismatch-repeat.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="173" customHeight="1">
+      <c r="A63" s="22" t="inlineStr">
+        <is>
+          <t>BUG-FALERT-74</t>
+        </is>
+      </c>
+      <c r="B63" s="22" t="inlineStr">
+        <is>
+          <t>Giữ cửa sổ 120 phút, retry và liều đã xác nhận khi scan có snapshot</t>
+        </is>
+      </c>
+      <c r="C63" s="22" t="inlineStr">
+        <is>
+          <t>1. Hai lượt scan occurrence tại 120 phút, +1 microsecond và đã confirmed; đọc lịch sử.
+2. Chạy pytest tests/integration/test_adherence_history_api.py::test_worker_window_notifications_use_strict_120_and_preserve_confirmed__AC22.</t>
+        </is>
+      </c>
+      <c r="D63" s="22" t="inlineStr">
+        <is>
+          <t>Ngày 2026-10-19 Asia/Ho_Chi_Minh; Integration medicine; UUID/ID synthetic theo fixture.</t>
+        </is>
+      </c>
+      <c r="E63" s="22" t="inlineStr">
+        <is>
+          <t>Đúng 120 phút chưa missed; vượt 1 microsecond mới missed; retry không trùng/ghi đè; history/schema đúng.</t>
+        </is>
+      </c>
+      <c r="F63" s="22" t="inlineStr">
+        <is>
+          <t>Scan và kiểm dose/count đã qua; kiểm history cuối ca fail KeyError: AdherenceByDateResponse.</t>
+        </is>
+      </c>
+      <c r="G63" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H63" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I63" s="22" t="inlineStr">
+        <is>
+          <t>Contract checkout thiếu AdherenceByDateResponse; không phải ValueError snapshot nữa.
+Log: evidence/test-snapshot-green.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="173" customHeight="1">
+      <c r="A64" s="22" t="inlineStr">
+        <is>
+          <t>BUG-FALERT-76</t>
+        </is>
+      </c>
+      <c r="B64" s="22" t="inlineStr">
+        <is>
+          <t>Giữ race Worker trước xác nhận trễ khi event có snapshot</t>
+        </is>
+      </c>
+      <c r="C64" s="22" t="inlineStr">
+        <is>
+          <t>1. Worker giữ lock; gửi xác nhận taken_at +90 phút cùng occurrence; commit; retry client_uuid; đọc lịch sử.
+2. Chạy pytest tests/integration/test_adherence_history_api.py::test_worker_insert_races_with_valid_late_confirmation__AC15_AC20_AC22[worker].</t>
+        </is>
+      </c>
+      <c r="D64" s="22" t="inlineStr">
+        <is>
+          <t>Ngày 2026-10-19 Asia/Ho_Chi_Minh; Integration medicine; UUID/ID synthetic theo fixture.</t>
+        </is>
+      </c>
+      <c r="E64" s="22" t="inlineStr">
+        <is>
+          <t>Writer chờ unique lock; chỉ một dose uong_tre, taken_at đúng; một notification; history đúng.</t>
+        </is>
+      </c>
+      <c r="F64" s="22" t="inlineStr">
+        <is>
+          <t>Kiểm lock, retry, một dose uong_tre/taken_at và notification đã qua; history fail KeyError: AdherenceByDateResponse.</t>
+        </is>
+      </c>
+      <c r="G64" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H64" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I64" s="22" t="inlineStr">
+        <is>
+          <t>Contract checkout thiếu AdherenceByDateResponse; không còn lỗi context snapshot.
+Log: evidence/test-snapshot-green.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="140" customHeight="1">
+      <c r="A65" s="22" t="inlineStr">
+        <is>
+          <t>BUG-FALERT-77</t>
+        </is>
+      </c>
+      <c r="B65" s="22" t="inlineStr">
+        <is>
+          <t>Đọc inbox sau seed alert có snapshot đầy đủ</t>
+        </is>
+      </c>
+      <c r="C65" s="22" t="inlineStr">
+        <is>
+          <t>1. Seed snapshot thuốc/giờ; dùng client_as người nhận gọi GET /notifications.
+2. Chạy pytest tests/integration/test_alert_dispatch_api.py::test_integration_missed_dose_alert_dispatch_and_inbox_fetch__AC1_AC2_AC6.</t>
+        </is>
+      </c>
+      <c r="D65" s="22" t="inlineStr">
+        <is>
+          <t>Ngày 2026-10-19 Asia/Ho_Chi_Minh; Integration medicine; UUID/ID synthetic theo fixture.</t>
+        </is>
+      </c>
+      <c r="E65" s="22" t="inlineStr">
+        <is>
+          <t>200; đúng content, recipient, is_read=false, total/unread_count.</t>
+        </is>
+      </c>
+      <c r="F65" s="22" t="inlineStr">
+        <is>
+          <t>INSERT snapshot đã qua; GET trả 401 thay 200, chưa kiểm được payload.</t>
+        </is>
+      </c>
+      <c r="G65" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H65" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I65" s="22" t="inlineStr">
+        <is>
+          <t>Fixture client_as override identity.current_user nhưng route notification dùng dependency xác thực riêng; chưa chứng minh lỗi sản phẩm.
+Log: evidence/test-snapshot-green.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="156.5" customHeight="1">
+      <c r="A66" s="22" t="inlineStr">
+        <is>
+          <t>BUG-FALERT-78</t>
+        </is>
+      </c>
+      <c r="B66" s="22" t="inlineStr">
+        <is>
+          <t>Đánh dấu đọc và từ chối recipient lạ sau seed snapshot</t>
+        </is>
+      </c>
+      <c r="C66" s="22" t="inlineStr">
+        <is>
+          <t>1. Seed snapshot; client_as người nhận PATCH is_read=true; thử lại bằng user khác.
+2. Chạy pytest tests/integration/test_alert_dispatch_api.py::test_integration_patch_notification_marks_as_read__AC7.</t>
+        </is>
+      </c>
+      <c r="D66" s="22" t="inlineStr">
+        <is>
+          <t>Ngày 2026-10-19 Asia/Ho_Chi_Minh; Integration medicine; UUID/ID synthetic theo fixture.</t>
+        </is>
+      </c>
+      <c r="E66" s="22" t="inlineStr">
+        <is>
+          <t>Người nhận 200/is_read=true; người khác 404.</t>
+        </is>
+      </c>
+      <c r="F66" s="22" t="inlineStr">
+        <is>
+          <t>INSERT snapshot đã qua; PATCH trả 401 thay 200, chưa tới kiểm foreign-recipient.</t>
+        </is>
+      </c>
+      <c r="G66" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H66" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I66" s="22" t="inlineStr">
+        <is>
+          <t>Fixture auth client_as không override dependency notification; chưa chứng minh lỗi sản phẩm.
+Log: evidence/test-snapshot-green.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="123.5" customHeight="1">
+      <c r="A67" s="22" t="inlineStr">
+        <is>
+          <t>BUG-FALERT-79</t>
+        </is>
+      </c>
+      <c r="B67" s="22" t="inlineStr">
+        <is>
+          <t>Kiểm timing SQL/API và tên trong inbox khi fixture có snapshot</t>
+        </is>
+      </c>
+      <c r="C67" s="22" t="inlineStr">
+        <is>
+          <t>1. Đo perf_counter quanh INSERT snapshot và GET inbox qua client_as.
+2. Chạy pytest tests/integration/test_alert_dispatch_api.py::test_integration_alert_timing_and_naming_flow.</t>
+        </is>
+      </c>
+      <c r="D67" s="22" t="inlineStr">
+        <is>
+          <t>Ngày 2026-10-19 Asia/Ho_Chi_Minh; Integration medicine; UUID/ID synthetic theo fixture.</t>
+        </is>
+      </c>
+      <c r="E67" s="22" t="inlineStr">
+        <is>
+          <t>200, content/recipient/is_read đúng; thời gian SQL/API &lt;2s, không chứng nhận FCM SLO.</t>
+        </is>
+      </c>
+      <c r="F67" s="22" t="inlineStr">
+        <is>
+          <t>INSERT snapshot đã qua; GET trả 401 trước các assertion timing/content.</t>
+        </is>
+      </c>
+      <c r="G67" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H67" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I67" s="22" t="inlineStr">
+        <is>
+          <t>Fixture auth client_as không override dependency notification; không có bằng chứng timing/FCM đạt SLO.
+Log: evidence/test-snapshot-green.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="123.5" customHeight="1">
+      <c r="A68" s="22" t="inlineStr">
+        <is>
+          <t>BUG-FALERT-80</t>
+        </is>
+      </c>
+      <c r="B68" s="22" t="inlineStr">
+        <is>
+          <t>Hiển thị badge unread server và xóa sau clear</t>
+        </is>
+      </c>
+      <c r="C68" s="22" t="inlineStr">
+        <is>
+          <t>1. Chạy flutter test test/features/family_link/family_tab_screen_test.dart.
+2. Kiểm 1 chưa đọc, điểm vào family-alerts; clear controller rồi kiểm badge biến mất.</t>
+        </is>
+      </c>
+      <c r="D68" s="22" t="inlineStr">
+        <is>
+          <t>AlertRepo fixture một item chưa đọc; session A.</t>
+        </is>
+      </c>
+      <c r="E68" s="22" t="inlineStr">
+        <is>
+          <t>Widget có badge 1 chưa đọc, sau clear không còn badge; không phát sinh exception.</t>
+        </is>
+      </c>
+      <c r="F68" s="22" t="inlineStr">
+        <is>
+          <t>Full Flutter fail trước kiểm badge: thiếu ConsentScope và FamilyLinkScope trong widget fixture.</t>
+        </is>
+      </c>
+      <c r="G68" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H68" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I68" s="22" t="inlineStr">
+        <is>
+          <t>Fixture FamilyTabScreen chưa bọc ConsentScope/FamilyLinkScope mà màn hình checkout mới yêu cầu; chưa chứng minh app runtime lỗi.
+Log: evidence/test-snapshot-mobile.log</t>
         </is>
       </c>
     </row>
@@ -24798,7 +25428,7 @@
       <formula>OR(G11="Critical",G11="High")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G54:G62">
+  <conditionalFormatting sqref="G54:G68">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
@@ -24813,7 +25443,7 @@
     <dataValidation sqref="G11:G29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="G54:G62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G54:G68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(qa): preserve master test cases and add family adherence coverage
Refs: 3.24
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -21,7 +21,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo dõi người thân (app)" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Link mời người thân" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Khung điều hướng app" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alert dispatch" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lịch sử tuân thủ" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Family adherence view" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Android build'!$A$8:$I$17</definedName>
@@ -39,6 +42,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Theo dõi người thân (app)'!$A$8:$I$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Link mời người thân'!$A$8:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Khung điều hướng app'!$A$8:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Alert dispatch'!$A$8:$I$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Lịch sử tuân thủ'!$A$8:$I$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Family adherence view'!$A$8:$I$29</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -377,12 +383,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$25</f>
+              <f>'Report'!$A$11:$A$28</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$11:$D$25</f>
+              <f>'Report'!$D$11:$D$28</f>
             </numRef>
           </val>
         </ser>
@@ -401,12 +407,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$25</f>
+              <f>'Report'!$A$11:$A$28</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$11:$E$25</f>
+              <f>'Report'!$E$11:$E$28</f>
             </numRef>
           </val>
         </ser>
@@ -425,12 +431,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$25</f>
+              <f>'Report'!$A$11:$A$28</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$11:$F$25</f>
+              <f>'Report'!$F$11:$F$28</f>
             </numRef>
           </val>
         </ser>
@@ -511,7 +517,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$3:$E$4</f>
+              <f>'Report'!$F$3:$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -533,7 +539,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>30</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -555,7 +561,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>30</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3240000"/>
@@ -11575,7 +11581,3934 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:U25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Điều phối cảnh báo người thân (ALERT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Ngọc Việt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Điều kiện điều phối cảnh báo cho người thân</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="107" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-ALERT-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Điều phối cảnh báo cho người thân dùng Android có đủ liên kết và quyền</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Bệnh nhân P bỏ lỡ liều thuốc (dose_log_id=999). Người thân F có liên kết active, sharing_enabled=true, consent family_sharing hiệu lực và token Android.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Hệ thống chạy tác vụ scan_missed_doses
+2. Kiểm tra bản ghi được tạo trong bảng notifications
+3. Kiểm tra danh sách Alert gửi tới NotificationPort</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>patient_id=P, caregiver_id=F, platform='android', token='token_android_123'</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Tạo 1 bản ghi notifications cho F với content='Bác [Tên] chưa ghi nhận liều thuốc đúng giờ'. Phát sinh 1 Alert gửi tới NotificationPort với đúng token của F.</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Đã tạo bản ghi notifications có tên bệnh nhân và phát sinh Alert với token_android_123 gửi tới NotificationPort.</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · Decision Table (R4) · EP (1) · test_dispatch_creates_alert_for_android_caregiver</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>recipient_platform</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>android</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>ios
+không có token</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>6
+7</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Liên kết active và bật chia sẻ?</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="74" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-ALERT-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Điều phối cảnh báo cho người thân dùng iOS (không có push APNs)</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Bệnh nhân P bỏ lỡ liều thuốc. Người thân F có đủ quyền nhưng chỉ đăng ký thiết bị iOS (không có token Android).</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Hệ thống chạy tác vụ scan_missed_doses
+2. Kiểm tra bản ghi trong bảng notifications
+3. Kiểm tra danh sách Alert gửi tới NotificationPort</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>patient_id=P, caregiver_id=F, platform='ios'</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Vẫn tạo 1 bản ghi notifications cho F trong CSDL. Không phát sinh Alert push nào gửi tới NotificationPort (C-06, C-07, BS-03).</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Bản ghi notifications đã được tạo trong CSDL, không có Alert push nào được gửi.</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · Decision Table (R3) · EP (2) · test_dispatch_skips_push_for_ios_caregiver_but_creates_notification_row</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>caregiver_relationship</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>active và sharing_enabled=true và consent_granted</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>chưa liên kết
+active nhưng sharing_enabled=false
+consent_revoked</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>8
+9
+10</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>Consent family_sharing còn hiệu lực?</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="74" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-ALERT-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Chống trùng lặp cảnh báo khi quét lặp lại cùng liều bỏ lỡ</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Liều thuốc đã được quét và đã tạo bản ghi notifications với dedupe_key='bo_lo:999:F'.</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Hệ thống chạy lại tác vụ scan_missed_doses với cùng lượt uống và liều 999
+2. Kiểm tra số lượng bản ghi trong notifications và số Alert gửi đi</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>dedupe_key='bo_lo:999:F'</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Không tạo thêm bản ghi notifications mới (ON CONFLICT DO NOTHING). Không gửi thêm Alert push lặp lại cho F.</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Số lượng notifications giữ nguyên 1, số Alert phát sinh là 0.</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · test_dispatch_deduplicates_repeated_missed_dose_scans</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>limit (query GET /notifications)</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>1..100</t>
+        </is>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>0
+-1
+101</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>11
+12
+13</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>Thiết bị có token Android?</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T11" s="11" t="inlineStr">
+        <is>
+          <t>No (iOS / không có)</t>
+        </is>
+      </c>
+      <c r="U11" s="11" t="inlineStr">
+        <is>
+          <t>Yes (Android)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="74" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-ALERT-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Chặn gửi cảnh báo khi người thân bị tắt chia sẻ hoặc rút consent</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Người thân F bị bệnh nhân tắt chia sẻ (sharing_enabled=false) hoặc bệnh nhân đã rút consent family_sharing.</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Hệ thống chạy tác vụ scan_missed_doses
+2. Kiểm tra danh sách người thân được access.caregivers_of trả về
+3. Kiểm tra bản ghi notifications và Alert</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>sharing_enabled=false hoặc consent revoked</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>access.caregivers_of không trả về F. Không tạo bản ghi notifications và không gửi Alert push cho F.</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>access.caregivers_of trả về rỗng, không tạo notification và không gửi alert.</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · Decision Table (R1, R2) · test_dispatch_respects_revoked_consent_and_sharing_switch</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>is_read (query / body PATCH)</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>true
+false</t>
+        </is>
+      </c>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>4
+5</t>
+        </is>
+      </c>
+      <c r="N12" s="10" t="inlineStr">
+        <is>
+          <t>(blank)
+chuỗi không hợp lệ</t>
+        </is>
+      </c>
+      <c r="O12" s="10" t="inlineStr">
+        <is>
+          <t>14
+15</t>
+        </is>
+      </c>
+      <c r="Q12" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="74" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-ALERT-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Bảo mật dữ liệu y tế trong nội dung push FCM (CD6, QD-26)</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Alert được tạo cho người thân về bệnh nhân Nguyễn Văn A.</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Xây dựng payload FCM qua build_fcm_payload
+2. Kiểm tra các trường title, body, data
+3. Kiểm tra sự xuất hiện của các từ khóa nhạy cảm (tên thuốc, hàm lượng, giờ uống)</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>notification_id=105, patient_name='Nguyễn Văn A'</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Body chỉ chứa thông báo nhắc nhở chung kèm tên bệnh nhân. Tuyệt đối không chứa tên thuốc, hoạt chất, hàm lượng (viên, mg, ml) hay giờ uống cụ thể.</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Payload FCM tuân thủ CD6: không chứa bất kỳ từ khóa thuốc hay giờ uống nhạy cảm nào.</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · test_alert_payload_hides_medication_details_and_names_patient</t>
+        </is>
+      </c>
+      <c r="Q13" s="10" t="inlineStr">
+        <is>
+          <t>Không tạo notification, không gửi push</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S13" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T13" s="11" t="inlineStr"/>
+      <c r="U13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="90.5" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-ALERT-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Lấy danh sách thông báo qua GET /notifications (đường thành công và lọc is_read)</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Người dùng F đã đăng nhập, có 2 thông báo (1 chưa đọc, 1 đã đọc).</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. F gửi GET /notifications
+2. Kiểm tra HTTP status, total, unread_count, danh sách items
+3. F gửi GET /notifications?is_read=false
+4. Kiểm tra danh sách trả về</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>limit=20, offset=0, is_read=false</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 200, total=2, unread_count=1. Khi lọc is_read=false, chỉ trả về đúng 1 thông báo chưa đọc.</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 200, trả về đúng số lượng và lọc chính xác theo trạng thái đã đọc.</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (3, 4) · test_get_notifications_returns_user_inbox_with_counts</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>Tạo dòng notification, không gửi push (DM3/iOS)</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr"/>
+      <c r="S14" s="11" t="inlineStr"/>
+      <c r="T14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="90.5" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-ALERT-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Cập nhật trạng thái đã đọc qua PATCH /notifications/{id}</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Thông báo id=1 của người dùng F có is_read=false.</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. F gửi PATCH /notifications/1 với body {'is_read': true}
+2. Kiểm tra HTTP status và body trả về
+3. Gửi lại GET /notifications?is_read=false để kiểm tra số lượng unread</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>id=1, is_read=true</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 200, is_read chuyển thành true, số lượng unread của F giảm tương ứng.</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 200, is_read=true, số unread giảm về 0.</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · test_patch_notification_marks_as_read</t>
+        </is>
+      </c>
+      <c r="Q15" s="10" t="inlineStr">
+        <is>
+          <t>Tạo dòng notification và gửi push FCM</t>
+        </is>
+      </c>
+      <c r="R15" s="11" t="inlineStr"/>
+      <c r="S15" s="11" t="inlineStr"/>
+      <c r="T15" s="11" t="inlineStr"/>
+      <c r="U15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="74" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-ALERT-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối cập nhật thông báo của người khác hoặc không tồn tại (404 Not Found)</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Thông báo id=3 thuộc sở hữu của người dùng khác (hoặc id=999 không tồn tại).</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. Người dùng F gửi PATCH /notifications/3 với body {'is_read': true}
+2. Người dùng F gửi PATCH /notifications/999 với body {'is_read': true}</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>id=3 (của người khác), id=999 (không tồn tại)</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 404 với detail='notification_not_found'. Không có dữ liệu nào bị thay đổi.</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 404 detail='notification_not_found'.</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · test_patch_notification_returns_404_for_other_users_notification</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="74" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-ALERT-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra xác thực: Chặn truy cập không có Bearer token (401 Unauthorized)</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Client chưa gửi header Authorization hoặc token không hợp lệ.</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /notifications không có header Authorization
+2. Gửi PATCH /notifications/1 không có header Authorization</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Header Authorization: (blank)</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized cho cả hai endpoint.</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized.</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC6, AC7 · test_notifications_endpoints_require_authentication</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="107" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-ALERT-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra tích hợp toàn trình luồng dispatch và lấy thông báo trên Postgres thật</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Môi trường CSDL Postgres cục bộ đang chạy qua Supabase local.</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo cặp người bệnh - người thân trên DB thật
+2. Tạo bản ghi cảnh báo bỏ lỡ vào notifications bằng SqlNotifications
+3. Người thân đăng nhập và gọi GET /notifications</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Dữ liệu sinh ngẫu nhiên trên schema v11</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Lấy được thông báo của bệnh nhân, khớp nội dung và thời gian.</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr"/>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC1, AC2, AC6 (QA.11) · test_integration_missed_dose_alert_dispatch_and_inbox_fetch__AC1_AC2_AC6 · Cần môi trường Supabase local</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="74" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-ALERT-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra tích hợp rút quyền người thân có hiệu lực ngay ở request kế tiếp (QA.02)</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Môi trường CSDL Postgres cục bộ đang chạy qua Supabase local.</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo liên kết người thân với sharing_enabled=false trên DB thật
+2. Gọi access.authorized_caregivers</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>sharing_enabled=false trên caregiver_links</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>caregiver_id không xuất hiện trong danh sách người nhận cảnh báo.</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr"/>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC4 (QA.02) · test_integration_caregiver_revocation_stops_alert_immediately__AC4 · Cần môi trường Supabase local</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22">
+      <c r="G22" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H22" s="13">
+        <f>COUNTIF(H9:H19,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H23" s="13">
+        <f>COUNTIF(H9:H19,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H24" s="13">
+        <f>COUNTIF(H9:H19,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H25" s="13">
+        <f>SUM(H22:H24)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I19"/>
+  <conditionalFormatting sqref="H9:H19">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:X37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="8" customWidth="1" min="22" max="22"/>
+    <col width="8" customWidth="1" min="23" max="23"/>
+    <col width="8" customWidth="1" min="24" max="24"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Lịch sử tuân thủ theo consent (ADHERENCE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Ngọc Việt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Quyền đọc lịch sử</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="W8" s="5" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="X8" s="5" t="inlineStr">
+        <is>
+          <t>R7</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="156.5" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Xem lịch sử của chính bệnh nhân</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Bệnh nhân P có consent health_data; có lịch uống và một liều đã uống.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập bằng tài khoản P.
+2. Gửi GET /adherence?patient_id=P với bearer token của P.
+3. Kiểm response và access_logs.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>P; ngày 2026-10-19; liều 08:00 da_uong</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>200; patient_id=P; có liều đã uống; access_logs có allowed, actor_role=patient, data_scope=lich_su_tuan_thu.</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC2 · EP (1) · Decision Table (R1) · test_self_and_family_success_are_audited_with_minimal_metadata__AC1_AC2</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>patient_id và vai trò</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>Bỏ trống hoặc chính bệnh nhân
+Người thân liên kết active với consent đầy đủ</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1
+2</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>Người thân không liên kết
+Liên kết tắt chia sẻ
+Thiếu health_data
+Thiếu family_sharing
+Đổi sang bệnh nhân khác
+Thiếu hoặc sai token
+UUID sai định dạng
+Admin dù tự gọi hoặc có liên kết</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>3
+4
+5
+6
+7
+8
+9
+10</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Vai trò</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>patient</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="U9" s="11" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="V9" s="11" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="W9" s="11" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="X9" s="11" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="74" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Xem lịch sử bệnh nhân từ người thân được chia sẻ</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>P có health_data và family_sharing; F có caregiver_link active, sharing_enabled=true; P có một liều đã uống.</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập bằng tài khoản F.
+2. Gửi GET /adherence?patient_id=P.
+3. Kiểm nhóm liều và access_logs.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>P; F; from=2026-10-19; to=2026-10-19</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>200; patient_id=P; nhóm và tổng hợp đúng liều của P; access_logs có allowed, actor_role=family.</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · EP (2) · Decision Table (R2) · test_self_and_family_success_are_audited_with_minimal_metadata__AC1_AC2</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>Liên kết active và bật chia sẻ</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="74" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối người thân không có liên kết</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>P có consent; F không có caregiver_link với P; P có liều đã uống.</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập F.
+2. Gửi GET /adherence?patient_id=P.
+3. Kiểm response và access_logs.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>P; F không liên kết</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>403 {"detail":"khong_co_quyen"}; không có lịch sử; access_logs có denied cho P.</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · EP (3) · Decision Table (R3) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>health_data</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V11" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="74" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối khi tắt công tắc chia sẻ</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>F có link active tới P; P có hai consent; sharing_enabled=false.</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập F.
+2. Gửi GET /adherence?patient_id=P.
+3. Kiểm access_logs.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>sharing_enabled=false</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>403 khong_co_quyen; không có lịch sử; access_logs có denied.</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · EP (4) · Decision Table (R4) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
+        <is>
+          <t>family_sharing</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W12" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="74" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối khi thiếu consent sức khỏe</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>F có link active và sharing_enabled=true; P không còn health_data.</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập F.
+2. Gửi GET /adherence?patient_id=P.
+3. Kiểm access_logs.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>health_data=thu_hoi</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>403 khong_co_quyen; không có lịch sử; access_logs có denied.</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (5) · Decision Table (R5) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11</t>
+        </is>
+      </c>
+      <c r="Q13" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T13" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U13" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="V13" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="W13" s="5" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="X13" s="5" t="inlineStr">
+        <is>
+          <t>R7</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="74" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối khi thiếu consent chia sẻ gia đình</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>F có link active và sharing_enabled=true; P không còn family_sharing.</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập F.
+2. Gửi GET /adherence?patient_id=P.
+3. Kiểm access_logs.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>family_sharing=thu_hoi</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>403 khong_co_quyen; không có lịch sử; access_logs có denied.</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · EP (6) · Decision Table (R6) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>200 + allowed</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T14" s="11" t="inlineStr"/>
+      <c r="U14" s="11" t="inlineStr"/>
+      <c r="V14" s="11" t="inlineStr"/>
+      <c r="W14" s="11" t="inlineStr"/>
+      <c r="X14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="90.5" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối ngay sau khi rút consent với cùng token</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>F đang được phép đọc P; lưu bearer token của F.</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence?patient_id=P và xác nhận 200.
+2. Rút health_data hoặc family_sharing của P.
+3. Gửi lại cùng request với token cũ.
+4. Kiểm access_logs.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>P; F; token không đổi</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Request thứ hai 403 khong_co_quyen; access_logs có allowed rồi denied, không trả lịch sử.</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · Decision Table (R5,R6) · test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12</t>
+        </is>
+      </c>
+      <c r="Q15" s="10" t="inlineStr">
+        <is>
+          <t>403 + denied</t>
+        </is>
+      </c>
+      <c r="R15" s="11" t="inlineStr"/>
+      <c r="S15" s="11" t="inlineStr"/>
+      <c r="T15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="V15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="W15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="X15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="107" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối ngay sau khi hủy liên kết hoặc tắt chia sẻ</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>F đang được phép đọc P; lưu bearer token của F.</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence?patient_id=P và xác nhận 200.
+2. Hủy caregiver_link hoặc tắt sharing_enabled.
+3. Gửi lại với token cũ.
+4. Kiểm access_logs.</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>P; F; token không đổi</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Request thứ hai 403 khong_co_quyen; access_logs có allowed rồi denied.</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · Decision Table (R3,R4) · test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90.5" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối đổi patient_id sang bệnh nhân khác</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>F có quyền với P nhưng không có quyền với Q; Q có lịch sử liều.</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập F.
+2. Gửi GET /adherence?patient_id=P và xác nhận 200.
+3. Đổi patient_id=Q rồi gửi lại.
+4. Kiểm access_logs của Q.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>P; Q; F chỉ liên kết P</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Request Q trả 403 khong_co_quyen; không có lịch sử Q; access_logs Q có denied.</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · EP (7) · test_family_patient_selector_tamper_does_not_read_other_patient__AC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="57.5" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Không trả lịch sử khi ghi audit allowed thất bại</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>P có consent và lịch sử; DB api_role bị giả lập lỗi INSERT access_logs.</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence bằng token P.
+2. Kiểm response, audit và dữ liệu liều.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Lỗi INSERT access_logs</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>500; no-store; không có lịch sử trong response và không làm thay đổi dose_logs.</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · test_audit_permission_and_commit_failure_fail_closed_without_health__AC13</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="57.5" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Giữ log denied sau khi request rollback</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>P đã rút health_data; request bị từ chối và transaction chính rollback.</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence bằng token P.
+2. Kiểm response.
+3. Đọc access_logs bằng kết nối quản trị.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>health_data=thu_hoi</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>403 consent_revoked; access_logs vẫn có denied cho scope lich_su_tuan_thu.</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · test_denied_audit_survives_outer_transaction_rollback__AC13</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="74" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối khi thiếu hoặc sai bearer token</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>P có lịch sử liều.</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence không có Authorization.
+2. Gửi lại với Authorization: Bearer invalid-token.
+3. Kiểm response và access_logs.</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Authorization=(blank) hoặc Bearer invalid-token</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>401; response không chứa lịch sử; Cache-Control=no-store; không có allowed log.</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (8) · test_authentication_401_and_no_store_without_health_payload__AC14</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="57.5" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-13</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối patient_id sai định dạng</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>P có lịch sử liều và token hợp lệ.</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence?patient_id=invalid-uuid bằng token P.
+2. Kiểm response.</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>patient_id=invalid-uuid</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>422; response không chứa lịch sử; Cache-Control=no-store.</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · EP (9) · test_bad_queries_are_422_without_health_payload__AC14</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="74" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-14</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối admin xem lịch sử của chính mình</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Admin A có health_data và một liều đã uống.</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập A.
+2. Gửi GET /adherence?patient_id=A.
+3. Kiểm response, access_logs và dose_logs.</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>A có system_role=admin</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>403 khong_co_quyen; không lộ liều; access_logs denied actor_role=admin; dose_logs không đổi.</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AC3, AC7 · Decision Table (R7) · test_admin_self_and_linked_history_denied_and_audited__AC3_AC6_AC7</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="74" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối admin có liên kết người thân</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>P có hai consent và một liều; admin A có caregiver_link active, sharing_enabled=true với P.</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập A.
+2. Gửi GET /adherence?patient_id=P.
+3. Kiểm response, access_logs và dose_logs.</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>P; A có system_role=admin</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>403 khong_co_quyen; không lộ liều; access_logs denied actor_role=admin; dose_logs không đổi.</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AC3, AC6, AC7 · Decision Table (R7) · test_admin_self_and_linked_history_denied_and_audited__AC3_AC6_AC7</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="74" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-16</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm nhóm ngày, nhóm thuốc và tỷ lệ tuân thủ</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>P có 5 liều: 3 da_uong, 1 uong_tre, 1 bo_lo.</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence?group_by=date&amp;from=2026-10-19&amp;to=2026-10-19.
+2. Gửi lại với group_by=medication.
+3. So sánh summary và nhóm.</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19; 5 liều, 2 thuốc</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>200; summary total=5, taken=3, late=1, missed=1, pending=0, adherence_rate=80; nhóm và timezone Asia/Ho_Chi_Minh đúng contract.</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>AC1, AC9 · test_patient_history_by_date_medication_groups_and_80_percent__AC1_AC3_AC4</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="57.5" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-17</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm khoảng ngày một ngày</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>P có lịch dùng thuốc bắt đầu 2026-10-19.</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence?from=2026-10-19&amp;to=2026-10-19.
+2. Kiểm summary và nhóm.</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>from=2026-10-19; to=2026-10-19</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>200; khoảng một ngày được chấp nhận và chỉ có liều ngày 2026-10-19.</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · BVA (min) · test_default_partial_and_inclusive_90_day_filters__AC5</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="57.5" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-18</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm khoảng ngày tối đa 90 ngày</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>P có lịch từ 2026-07-22 đến 2026-10-19.</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence với khoảng đúng 90 ngày.
+2. Kiểm số ngày và response.</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>from=2026-07-22; to=2026-10-19</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>200; khoảng 90 ngày được chấp nhận.</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · BVA (max) · test_default_partial_and_inclusive_90_day_filters__AC5</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="57.5" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-19</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối khoảng ngày 91 ngày</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>P có lịch từ 2026-07-21 đến 2026-10-19.</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence với khoảng 91 ngày.
+2. Kiểm response.</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>from=2026-07-21; to=2026-10-19</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>422 {"detail":"adherence_range_too_large"}; không có lịch sử.</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · BVA (max+1) · test_default_partial_and_inclusive_90_day_filters__AC5</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="74" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-20</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Đối chiếu contract với OpenAPI runtime</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Có api_contract/openapi.json đã duyệt và app FastAPI khởi tạo được.</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. Sinh OpenAPI từ create_app().openapi().
+2. So path GET /adherence, query, auth, status, schema và no-store với contract.</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>GET /adherence; patient_id, from, to, group_by</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Path, query, bảo mật, mã lỗi, cấu trúc response và Cache-Control no-store khớp contract.</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Hai test OpenAPI runtime/schema PASSED; evidence/test-openapi-after-migration.log.</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · test_contract_query_security_status_headers · test_response_required_nullable_enums_and_constraints</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="57.5" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-21</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối khoảng ngày đảo ngược</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>P có token hợp lệ và lịch sử liều.</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi GET /adherence?from=2026-10-19&amp;to=2026-10-18 bằng token P.
+2. Kiểm response không chứa lịch sử.</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>from=2026-10-19; to=2026-10-18</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>422; không có lịch sử trong response; Cache-Control=no-store.</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Test tương ứng trong Comments PASSED sau migration; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · BVA (min-1) · test_bad_queries_are_422_without_health_payload__AC14</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="123.5" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-22</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm ràng buộc actor identity sau migration</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>DB local có migration admin-self; hai user A và B; kết nối api_role.</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>1. Lần lượt INSERT access_logs với actor A, patient A hoặc B, vai patient/family/admin/khong_co_quyen, result allowed/denied.
+2. Kiểm INSERT thành công hoặc SQLSTATE 23514 theo từng tổ hợp.
+3. Rollback từng lần; xác nhận không còn dòng thử.</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>16 tổ hợp: self/other × 4 role × allowed/denied</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Self patient allowed/denied và self admin denied được chấp nhận; self admin allowed, self family/no-access và other patient bị chặn. Other family/admin giữ allowed/denied; other no-access chỉ denied. Không lưu dòng sau rollback.</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>16 ca matrix PASSED; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>AC3, AC7 · Decision Table (R7) · test_access_log_actor_identity_matrix__AC3_AC7</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="74" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>TC-ADHERENCE-23</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Chặn sửa xóa và truncate audit sau migration</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>DB local có migration admin-self và một dòng audit; có kết nối api_role, worker_role và postgres.</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>1. Thử UPDATE, DELETE, TRUNCATE access_logs lần lượt bằng từng role.
+2. Rollback từng transaction thử.
+3. Đọc lại audit bằng kết nối quản trị.</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>api_role/worker_role/postgres × UPDATE/DELETE/TRUNCATE = 9 ca</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Role ứng dụng bị từ chối SQLSTATE 42501; postgres bị trigger từ chối P0001; audit không đổi.</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>9 ca append-only PASSED; evidence/test-migration.log.</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · CD3 · test_access_logs_remain_append_only_after_actor_identity_migration__AC7</t>
+        </is>
+      </c>
+    </row>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34">
+      <c r="G34" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H34" s="13">
+        <f>COUNTIF(H9:H31,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H35" s="13">
+        <f>COUNTIF(H9:H31,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H36" s="13">
+        <f>COUNTIF(H9:H31,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="G37" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H37" s="13">
+        <f>SUM(H34:H36)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I31"/>
+  <conditionalFormatting sqref="H9:H31">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Người thân xem tuân thủ (FAMADH)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Ngọc Việt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46317</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="74" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Mở route với bệnh nhân hợp lệ</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Môi trường Flutter test dùng repository giả; các ca backend/manual cần app đăng nhập và DB local riêng.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy opens valid family route with supplied patient.
+2. Kiểm patientId của request và tên trên màn.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>11111111-1111-4111-8111-111111111111; tên Mẹ</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Một request đúng patientId; hiện Mẹ; không có lỗi widget.</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AC1 · family_adherence_screen_test.dart</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="74" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối đối số route sai</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Môi trường Flutter test dùng repository giả; các ca backend/manual cần app đăng nhập và DB local riêng.</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy rejects invalid route arguments without fetching.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>patientId=bad-id</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Không gọi API; hiện Chưa thể mở lịch sử của người bệnh này.</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AC1, AC6 · family_adherence_screen_test.dart</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="74" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Hiển thị đủ bốn trạng thái chỉ đọc</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Môi trường Flutter test dùng repository giả; các ca backend/manual cần app đăng nhập và DB local riêng.</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy shows server summary and four read-only dose states.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>da_uong, uong_tre, bo_lo, cho_xac_nhan; Thuốc A</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Có nhãn bốn trạng thái; không có nút Xác nhận hoặc Sửa.</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AC1, AC2 · family_adherence_screen_test.dart</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="74" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Giữ tỷ lệ gồm uống trễ từ server</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Môi trường Flutter test dùng repository giả; các ca backend/manual cần app đăng nhập và DB local riêng.</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy widget test summary và mapper test parses all statuses, offset times and server rate.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>taken=1; late=1; missed=1; pending=1; rate=66.67</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Hiện 66.67% và Tỷ lệ tuân thủ (gồm uống trễ).</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · family_adherence_screen_test.dart; adherence_api_mapper_test.dart</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="74" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Hiển thị dữ liệu rỗng và tỷ lệ null</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Môi trường Flutter test dùng repository giả; các ca backend/manual cần app đăng nhập và DB local riêng.</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy empty response and network retry have distinct states.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>groups=[]; counted=0; adherence_rate=null</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Hiện Chưa có liều được tính và Không có lịch sử trong ngày này.</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AC3, AC4 · family_adherence_screen_test.dart</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="74" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Xóa lịch sử trước refresh và khi bị 403</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Môi trường Flutter test dùng repository giả; các ca backend/manual cần app đăng nhập và DB local riêng.</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. Tải 200 có Thuốc A.
+2. Resume app và trả 403 ở request kế tiếp.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>response 200 → 403</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Thuốc A biến mất ngay khi tải lại; hiện Không còn quyền xem lịch sử.</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · family_adherence_screen_test.dart</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="74" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Loại response cũ khi đổi bệnh nhân</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Môi trường Flutter test dùng repository giả; các ca backend/manual cần app đăng nhập và DB local riêng.</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy changing patient discards late response from previous patient.
+2. Cho response B về trước response A.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>A=11111111-1111-4111-8111-111111111111; B=22222222-2222-4222-8222-222222222222</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ giữ lịch sử B; dữ liệu cũ bị xóa trước request.</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · adherence_controller_test.dart</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="74" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Map lỗi API và xử lý hết phiên</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Môi trường Flutter test dùng repository giả; các ca backend/manual cần app đăng nhập và DB local riêng.</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy HTTP 401/403/422/503 maps to failure without retry.</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>401;403;422;503</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Failure đúng loại; callback hết phiên chỉ gọi với 401; mỗi ca một request.</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AC5, AC7 · remote_adherence_repository_test.dart</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="74" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Thử lại sau lỗi mạng</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Môi trường Flutter test dùng repository giả; các ca backend/manual cần app đăng nhập và DB local riêng.</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy empty response and network retry have distinct states.
+2. Nhấn Thử lại sau lỗi network.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>AdherenceFailureKind.network</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Hiện Chưa thể tải lịch sử; nhấn Thử lại tạo request mới.</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · family_adherence_screen_test.dart</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="74" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Gửi query và token mới ở mỗi lần đọc</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Môi trường Flutter test dùng repository giả; các ca backend/manual cần app đăng nhập và DB local riêng.</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy GET sends patient, bounded dates, group and app bearer on each call.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>from=2026-10-01;to=2026-10-22;group_by=date; token first-token → second-token</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>GET /adherence đúng patient_id, from, to, group_by; bearer cập nhật.</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AC1, AC8 · remote_adherence_repository_test.dart</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="74" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Chặn ngày tương lai và ngày quá cũ</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Môi trường Flutter test dùng repository giả; các ca backend/manual cần app đăng nhập và DB local riêng.</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy rejects future and out-of-range dates without a request.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>today=2026-10-22; chọn 2026-10-23 và 2026-07-01</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Không phát request.</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · adherence_controller_test.dart</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="74" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Đọc thời gian có offset và từ chối response sai</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Môi trường Flutter test dùng repository giả; các ca backend/manual cần app đăng nhập và DB local riêng.</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy toàn bộ adherence_api_mapper_test.dart và rejects a response for another patient.</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>08:00+07:00; taken_at=null; thiếu patient_id; ngày 2026-02-30; patient khác</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>UTC đúng; giữ null; dữ liệu sai bị từ chối.</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AC2, AC6, AC8 · adherence_api_mapper_test.dart; remote_adherence_repository_test.dart</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="74" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-13</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Không overflow khi tăng cỡ chữ</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Môi trường Flutter test dùng repository giả; các ca backend/manual cần app đăng nhập và DB local riêng.</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy fits narrow viewport and large text.</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>320×640; textScaleFactor=1.6</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Không có Flutter layout exception.</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · family_adherence_screen_test.dart</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="74" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-14</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm vùng an toàn, landscape và trình đọc màn hình</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Cần thiết bị hoặc DB local riêng với bệnh nhân A, người thân F và liên kết active.</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở route trên thiết bị 375dp và 320dp.
+2. Tăng chữ 1.6×; xoay ngang; cuộn hết liều.
+3. Bật TalkBack/VoiceOver; kiểm nhãn ngày/tỷ lệ/trạng thái và vùng chạm.</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>375dp, 320dp; chữ 1.6×</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Không che/tràn; nhãn đọc rõ; điều khiển có vùng chạm theo nền tảng.</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr"/>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="57.5" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Đối chiếu Figma S09a/S09b</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Cần thiết bị hoặc DB local riêng với bệnh nhân A, người thân F và liên kết active.</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở màn có summary và bốn trạng thái.
+2. So màu/chữ/spacing/radius với node 75:7848 và 75:8120 cùng foundation.</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Figma Prototype_DrugTime; 375×812</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Nhất quán token và visual; header thể hiện dữ liệu bệnh nhân được chia sẻ.</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr"/>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AC10 · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="74" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-16</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm quyền đọc và audit trên DB thật</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Cần thiết bị hoặc DB local riêng với bệnh nhân A, người thân F và liên kết active.</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy backend/tests/integration/test_adherence_history_access.py trên DB local sạch.
+2. Kiểm ca family allowed, không link/consent và giả mạo patient_id.</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>F liên kết A; B không liên kết</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>200 + audit allowed với A; 403 + audit denied với B/thiếu quyền.</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>60 test API/quyền/audit pass trên DB thật sau khi restart Docker, 17.36 giây; khẳng định tương ứng đạt.</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>AC5, AC6 · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="74" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-17</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Thu hồi quyền có hiệu lực request kế tiếp</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Cần thiết bị hoặc DB local riêng với bệnh nhân A, người thân F và liên kết active.</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12.
+2. Rút consent hoặc tắt sharing/unlink, gửi lại cùng token.</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Cùng phiên F; A vừa thu hồi</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>403 ngay request tiếp theo; có audit denied.</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>60 test API/quyền/audit pass trên DB thật sau khi restart Docker, 17.36 giây; khẳng định tương ứng đạt.</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="57.5" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-18</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Fail closed khi ghi audit lỗi</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Cần thiết bị hoặc DB local riêng với bệnh nhân A, người thân F và liên kết active.</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy test_audit_permission_and_commit_failure_fail_closed_without_health__AC13 trên DB riêng.</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Lỗi insert audit/commit/đọc quyền</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Không trả dữ liệu sức khỏe khi audit/quyền lỗi.</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>60 test API/quyền/audit pass trên DB thật sau khi restart Docker, 17.36 giây; khẳng định tương ứng đạt.</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>AC5, AC6 · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="57.5" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-19</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm đủ biên 90 ngày và điều hướng lịch tháng</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Cần thiết bị hoặc DB local riêng với bệnh nhân A, người thân F và liên kết active.</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. Chọn today-90, today-89, today, today+1.
+2. Mở lịch tháng và chuyển giữa các tháng trong cửa sổ.</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>today=2026-10-22; các ngày biên 2026-07-24,2026-07-25,2026-10-22,2026-10-23</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ today-89 đến today được chọn; query mỗi lần không quá 90 ngày; tương lai bị khóa.</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Hai ca biên bốn ngày và khóa điều hướng tháng đều pass.</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="90.5" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-20</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm vùng chạm chọn ngày ở 320dp</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Flutter test; viewport 320x640; padding ngang 16dp</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy evidence/calendar-accessibility-repro.dart từ frontend/mobile bằng flutter test --no-pub.
+2. Kiểm androidTapTargetGuideline.</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>320dp; ngày 22/10/2026</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Mọi ô tương tác ít nhất 48x48dp.</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Hồi quy tuần/tháng tại 320dp và 375dp, chữ 1.6x đạt androidTapTargetGuideline; chọn ngày cột cuối đúng.</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · BVA viewport 320dp · calendar meets Android tap target sizes at 320dp; BUG-FAMADH-20 đã sửa, giữ log fail cũ test-calendar-accessibility.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="90.5" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-21</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Giữ khoảng ngày hợp lệ khi refresh qua nửa đêm</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Controller mở ngày 28/10/2026 với selectedDate=31/07/2026 (today-89).</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy evidence/review-date-rollover-repro.dart bằng flutter test --no-pub từ frontend/mobile.
+2. Chuyển đồng hồ sang 29/10/2026 và gọi refresh; xem khoảng request mà repository ghi nhận.</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>now 28/10 → 29/10/2026, selectedDate=31/07/2026</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa ngày đang chọn vào cửa sổ mới trước refresh; mọi request có from&lt;=to.</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Tái hiện request from=01/08/2026, to=31/07/2026. Script tái hiện pass vì khẳng định bug tồn tại; hành vi sản phẩm Fail.</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · Chuyển trạng thái đồng hồ · review R2 · có thể chọn ngày khác để tiếp tục</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32">
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H32" s="13">
+        <f>COUNTIF(H9:H29,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H33" s="13">
+        <f>COUNTIF(H9:H29,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="G34" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H34" s="13">
+        <f>COUNTIF(H9:H29,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H35" s="13">
+        <f>SUM(H32:H34)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I29"/>
+  <conditionalFormatting sqref="H9:H29">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11609,6 +15542,11 @@
       </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
+          <t>Ngọc Việt</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
@@ -11632,8 +15570,12 @@
         <f>'Chọn thuốc danh mục'!$H$40+'Hồi quy xác nhận liều'!$H$12</f>
         <v/>
       </c>
-      <c r="E3" s="15">
-        <f>SUM(C3:D3)</f>
+      <c r="E3" s="11">
+        <f>'Alert dispatch'!$H$22+'Lịch sử tuân thủ'!$H$34+'Family adherence view'!$H$32</f>
+        <v/>
+      </c>
+      <c r="F3" s="15">
+        <f>SUM(C3:E3)</f>
         <v/>
       </c>
     </row>
@@ -11652,8 +15594,12 @@
         <f>'Chọn thuốc danh mục'!$H$41+'Hồi quy xác nhận liều'!$H$13</f>
         <v/>
       </c>
-      <c r="E4" s="15">
-        <f>SUM(C4:D4)</f>
+      <c r="E4" s="11">
+        <f>'Alert dispatch'!$H$23+'Lịch sử tuân thủ'!$H$35+'Family adherence view'!$H$33</f>
+        <v/>
+      </c>
+      <c r="F4" s="15">
+        <f>SUM(C4:E4)</f>
         <v/>
       </c>
     </row>
@@ -11672,8 +15618,12 @@
         <f>D3+D4</f>
         <v/>
       </c>
-      <c r="E5" s="15">
-        <f>SUM(C5:D5)</f>
+      <c r="E5" s="11">
+        <f>E3+E4</f>
+        <v/>
+      </c>
+      <c r="F5" s="15">
+        <f>SUM(C5:E5)</f>
         <v/>
       </c>
     </row>
@@ -11692,8 +15642,12 @@
         <f>'Chọn thuốc danh mục'!$H$42+'Hồi quy xác nhận liều'!$H$14</f>
         <v/>
       </c>
-      <c r="E6" s="15">
-        <f>SUM(C6:D6)</f>
+      <c r="E6" s="11">
+        <f>'Alert dispatch'!$H$24+'Lịch sử tuân thủ'!$H$36+'Family adherence view'!$H$34</f>
+        <v/>
+      </c>
+      <c r="F6" s="15">
+        <f>SUM(C6:E6)</f>
         <v/>
       </c>
     </row>
@@ -11712,8 +15666,12 @@
         <f>D5+D6</f>
         <v/>
       </c>
-      <c r="E7" s="15">
-        <f>SUM(C7:D7)</f>
+      <c r="E7" s="11">
+        <f>E5+E6</f>
+        <v/>
+      </c>
+      <c r="F7" s="15">
+        <f>SUM(C7:E7)</f>
         <v/>
       </c>
     </row>
@@ -12424,496 +16382,677 @@
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="19" t="inlineStr">
+    <row r="26" ht="90.5" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>Điều phối cảnh báo người thân</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Điều phối cảnh báo bỏ lỡ liều cho người thân: gửi FCM trên Android, lưu hộp thư cho iOS (không có APNs), và API Notification Inbox.</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>Alert dispatch</t>
+        </is>
+      </c>
+      <c r="D26" s="18">
+        <f>IFERROR(('Alert dispatch'!$H$25-'Alert dispatch'!$H$24)/'Alert dispatch'!$H$25,0)</f>
+        <v/>
+      </c>
+      <c r="E26" s="18">
+        <f>IFERROR('Alert dispatch'!$H$22/'Alert dispatch'!$H$25,0)</f>
+        <v/>
+      </c>
+      <c r="F26" s="18">
+        <f>IFERROR('Alert dispatch'!$H$23/'Alert dispatch'!$H$25,0)</f>
+        <v/>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm thử tự động toàn bộ logic điều phối cảnh báo và API Notification Inbox. Các test tích hợp trên DB thật để trạng thái Pending chờ môi trường local Supabase.</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
+        <is>
+          <t>Ngọc Việt</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="90.5" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Lịch sử tuân thủ theo consent</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>GET /adherence theo quyền bệnh nhân, người thân, consent và audit.</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>Lịch sử tuân thủ</t>
+        </is>
+      </c>
+      <c r="D27" s="18">
+        <f>IFERROR(('Lịch sử tuân thủ'!$H$37-'Lịch sử tuân thủ'!$H$36)/'Lịch sử tuân thủ'!$H$37,0)</f>
+        <v/>
+      </c>
+      <c r="E27" s="18">
+        <f>IFERROR('Lịch sử tuân thủ'!$H$34/'Lịch sử tuân thủ'!$H$37,0)</f>
+        <v/>
+      </c>
+      <c r="F27" s="18">
+        <f>IFERROR('Lịch sử tuân thủ'!$H$35/'Lịch sử tuân thủ'!$H$37,0)</f>
+        <v/>
+      </c>
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>23 Pass sau migration; BUG-ADHERENCE-14 đã qua kiểm thử hồi quy, còn chờ review/PR.</t>
+        </is>
+      </c>
+      <c r="I27" s="11" t="inlineStr">
+        <is>
+          <t>Ngọc Việt</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="90.5" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Người thân xem tuân thủ</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Màn chỉ đọc nhận patientId</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>Family adherence view</t>
+        </is>
+      </c>
+      <c r="D28" s="18">
+        <f>IFERROR(('Family adherence view'!$H$35-'Family adherence view'!$H$34)/'Family adherence view'!$H$35,0)</f>
+        <v/>
+      </c>
+      <c r="E28" s="18">
+        <f>IFERROR('Family adherence view'!$H$32/'Family adherence view'!$H$35,0)</f>
+        <v/>
+      </c>
+      <c r="F28" s="18">
+        <f>IFERROR('Family adherence view'!$H$33/'Family adherence view'!$H$35,0)</f>
+        <v/>
+      </c>
+      <c r="G28" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>R1 workbook đã khôi phục baseline; BUG-FAMADH-20 đã sửa; R2/BUG-FAMADH-21 Medium còn mở; 2 manual Pending.</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>Ngọc Việt</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="19" t="inlineStr">
         <is>
           <t>Bug Report</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="20" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="20" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="B49" s="20" t="inlineStr">
+      <c r="B52" s="20" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C49" s="20" t="inlineStr">
+      <c r="C52" s="20" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="D49" s="20" t="inlineStr">
+      <c r="D52" s="20" t="inlineStr">
         <is>
           <t>Input Data</t>
         </is>
       </c>
-      <c r="E49" s="20" t="inlineStr">
+      <c r="E52" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F49" s="20" t="inlineStr">
+      <c r="F52" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="G49" s="20" t="inlineStr">
+      <c r="G52" s="20" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="H49" s="20" t="inlineStr">
+      <c r="H52" s="20" t="inlineStr">
         <is>
           <t>Name of Tester</t>
         </is>
       </c>
-      <c r="I49" s="20" t="inlineStr">
+      <c r="I52" s="20" t="inlineStr">
         <is>
           <t>Logs</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="123.5" customHeight="1">
-      <c r="A50" s="22" t="inlineStr">
+    <row r="53" ht="123.5" customHeight="1">
+      <c r="A53" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-08</t>
         </is>
       </c>
-      <c r="B50" s="22" t="inlineStr">
+      <c r="B53" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
         </is>
       </c>
-      <c r="C50" s="22" t="inlineStr">
+      <c r="C53" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
 2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
         </is>
       </c>
-      <c r="D50" s="22" t="inlineStr">
+      <c r="D53" s="22" t="inlineStr">
         <is>
           <t>phone: 0900000001 + ký tự \n</t>
         </is>
       </c>
-      <c r="E50" s="22" t="inlineStr">
+      <c r="E53" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F50" s="22" t="inlineStr">
+      <c r="F53" s="22" t="inlineStr">
         <is>
           <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
         </is>
       </c>
-      <c r="G50" s="22" t="inlineStr">
+      <c r="G53" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H50" s="22" t="inlineStr">
+      <c r="H53" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I50" s="22" t="inlineStr">
+      <c r="I53" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn — kỳ vọng AC6 mâu thuẫn AC5: backend `_validate_required_text` (sign_in.py:178) `strip()` mọi ký tự trắng hai đầu, nên \n cuối được xử lý như khoảng trắng hai đầu mà AC5 coi là hợp lệ. Cần người dùng chốt: sửa AC6 hoặc sửa backend
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="123.5" customHeight="1">
-      <c r="A51" s="22" t="inlineStr">
+    <row r="54" ht="123.5" customHeight="1">
+      <c r="A54" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-11</t>
         </is>
       </c>
-      <c r="B51" s="22" t="inlineStr">
+      <c r="B54" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
         </is>
       </c>
-      <c r="C51" s="22" t="inlineStr">
+      <c r="C54" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone}
 2. POST /auth/mobile/verify {phone, token: 123456}</t>
         </is>
       </c>
-      <c r="D51" s="22" t="inlineStr">
+      <c r="D54" s="22" t="inlineStr">
         <is>
           <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
         </is>
       </c>
-      <c r="E51" s="22" t="inlineStr">
+      <c r="E54" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
         </is>
       </c>
-      <c r="F51" s="22" t="inlineStr">
+      <c r="F54" s="22" t="inlineStr">
         <is>
           <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
         </is>
       </c>
-      <c r="G51" s="22" t="inlineStr">
+      <c r="G54" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H51" s="22" t="inlineStr">
+      <c r="H54" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I51" s="22" t="inlineStr">
+      <c r="I54" s="22" t="inlineStr">
         <is>
           <t>`_normalize_phone` (sign_in.py:197–206) kiểm bằng `str.isdigit()`, nhận cả chữ số Unicode, nên số lọt qua kiểm tra và gửi tới Supabase. Ô nhập của app chỉ cho 0-9 nên người dùng app không gặp; lỗi ở tầng API
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="189.5" customHeight="1">
-      <c r="A52" s="22" t="inlineStr">
+    <row r="55" ht="189.5" customHeight="1">
+      <c r="A55" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-25</t>
         </is>
       </c>
-      <c r="B52" s="22" t="inlineStr">
+      <c r="B55" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên có ký tự NUL</t>
         </is>
       </c>
-      <c r="C52" s="22" t="inlineStr">
+      <c r="C55" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
         </is>
       </c>
-      <c r="D52" s="22" t="inlineStr">
+      <c r="D55" s="22" t="inlineStr">
         <is>
           <t>ho_ten: abc\u0000def</t>
         </is>
       </c>
-      <c r="E52" s="22" t="inlineStr">
+      <c r="E55" s="22" t="inlineStr">
         <is>
           <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
         </is>
       </c>
-      <c r="F52" s="22" t="inlineStr">
+      <c r="F55" s="22" t="inlineStr">
         <is>
           <t>500 Internal Server Error</t>
         </is>
       </c>
-      <c r="G52" s="22" t="inlineStr">
+      <c r="G55" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H52" s="22" t="inlineStr">
+      <c r="H55" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I52" s="22" t="inlineStr">
+      <c r="I55" s="22" t="inlineStr">
         <is>
           <t>`_validate_required_text` (sign_in.py:178) không chặn ký tự điều khiển; PostgreSQL từ chối NUL trong cột text: `psycopg.DataError: PostgreSQL text fields cannot contain NUL (0x00) bytes` ở `UPDATE users SET full_name…` (SqlUsers.update_profile); không có handler cho DataError nên thành 500. Câu SQL có tham số nên không phải lỗ hổng SQL injection
 Log: evidence/test-integration.log, evidence/test-probe-nul.log</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="90.5" customHeight="1">
-      <c r="A53" s="22" t="inlineStr">
+    <row r="56" ht="90.5" customHeight="1">
+      <c r="A56" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-30</t>
         </is>
       </c>
-      <c r="B53" s="22" t="inlineStr">
+      <c r="B56" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên dài 256 ký tự</t>
         </is>
       </c>
-      <c r="C53" s="22" t="inlineStr">
+      <c r="C56" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: A*256}</t>
         </is>
       </c>
-      <c r="D53" s="22" t="inlineStr">
+      <c r="D56" s="22" t="inlineStr">
         <is>
           <t>A*256</t>
         </is>
       </c>
-      <c r="E53" s="22" t="inlineStr">
+      <c r="E56" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F53" s="22" t="inlineStr">
+      <c r="F56" s="22" t="inlineStr">
         <is>
           <t>204, đã lưu</t>
         </is>
       </c>
-      <c r="G53" s="22" t="inlineStr">
+      <c r="G56" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H53" s="22" t="inlineStr">
+      <c r="H56" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I53" s="22" t="inlineStr">
+      <c r="I56" s="22" t="inlineStr">
         <is>
           <t>Không có giới hạn độ dài họ tên: `_validate_profile` (sign_in.py) chỉ kiểm rỗng; cột users.full_name kiểu text không giới hạn
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="90.5" customHeight="1">
-      <c r="A54" s="22" t="inlineStr">
+    <row r="57" ht="90.5" customHeight="1">
+      <c r="A57" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-32</t>
         </is>
       </c>
-      <c r="B54" s="22" t="inlineStr">
+      <c r="B57" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh trước 1900-01-01</t>
         </is>
       </c>
-      <c r="C54" s="22" t="inlineStr">
+      <c r="C57" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh}</t>
         </is>
       </c>
-      <c r="D54" s="22" t="inlineStr">
+      <c r="D57" s="22" t="inlineStr">
         <is>
           <t>1899-12-31 | 0001-01-01</t>
         </is>
       </c>
-      <c r="E54" s="22" t="inlineStr">
+      <c r="E57" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
         </is>
       </c>
-      <c r="F54" s="22" t="inlineStr">
+      <c r="F57" s="22" t="inlineStr">
         <is>
           <t>204 ở cả hai giá trị, đã lưu</t>
         </is>
       </c>
-      <c r="G54" s="22" t="inlineStr">
+      <c r="G57" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H54" s="22" t="inlineStr">
+      <c r="H57" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I54" s="22" t="inlineStr">
+      <c r="I57" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:229–231) chỉ chặn ngày tương lai, không có cận dưới. App mobile đã giới hạn date picker từ 1900 nên chỉ gặp khi gọi API trực tiếp
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="123.5" customHeight="1">
-      <c r="A55" s="22" t="inlineStr">
+    <row r="58" ht="123.5" customHeight="1">
+      <c r="A58" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-35</t>
         </is>
       </c>
-      <c r="B55" s="22" t="inlineStr">
+      <c r="B58" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
         </is>
       </c>
-      <c r="C55" s="22" t="inlineStr">
+      <c r="C58" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
         </is>
       </c>
-      <c r="D55" s="22" t="inlineStr">
+      <c r="D58" s="22" t="inlineStr">
         <is>
           <t>ngay_sinh: 2026-10-08</t>
         </is>
       </c>
-      <c r="E55" s="22" t="inlineStr">
+      <c r="E58" s="22" t="inlineStr">
         <is>
           <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
         </is>
       </c>
-      <c r="F55" s="22" t="inlineStr">
+      <c r="F58" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_date_of_birth"}</t>
         </is>
       </c>
-      <c r="G55" s="22" t="inlineStr">
+      <c r="G58" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H55" s="22" t="inlineStr">
+      <c r="H58" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I55" s="22" t="inlineStr">
+      <c r="I58" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:230) so với `now.date()` trong khi `now()` (shared/clock.py) trả giờ UTC: từ 00:00 đến 07:00 giờ VN, "hôm nay" bị coi là ngày mai. Vi phạm bất biến 7 (múi giờ cố định Asia/Ho_Chi_Minh)
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="173" customHeight="1">
-      <c r="A56" s="22" t="inlineStr">
+    <row r="59" ht="173" customHeight="1">
+      <c r="A59" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-42</t>
         </is>
       </c>
-      <c r="B56" s="22" t="inlineStr">
+      <c r="B59" s="22" t="inlineStr">
         <is>
           <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
         </is>
       </c>
-      <c r="C56" s="22" t="inlineStr">
+      <c r="C59" s="22" t="inlineStr">
         <is>
           <t>1. Chạm vào ô mã OTP
 2. Theo dõi request backend nhận được</t>
         </is>
       </c>
-      <c r="D56" s="22" t="inlineStr">
+      <c r="D59" s="22" t="inlineStr">
         <is>
           <t>Ô đang chứa 000000</t>
         </is>
       </c>
-      <c r="E56" s="22" t="inlineStr">
+      <c r="E59" s="22" t="inlineStr">
         <is>
           <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
         </is>
       </c>
-      <c r="F56" s="22" t="inlineStr">
+      <c r="F59" s="22" t="inlineStr">
         <is>
           <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
         </is>
       </c>
-      <c r="G56" s="22" t="inlineStr">
+      <c r="G59" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H56" s="22" t="inlineStr">
+      <c r="H59" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I56" s="22" t="inlineStr">
+      <c r="I59" s="22" t="inlineStr">
         <is>
           <t>`OtpPinInput._handleTextChange` (frontend/mobile/lib/features/auth/presentation/widgets/otp_pin_input.dart:66–72) chạy với mọi thông báo của controller, kể cả khi chỉ đổi vị trí con trỏ lúc chạm ô, và gọi onCompleted hễ ô đủ 6 số → gửi lại mã sai, tốn hạn mức token_verifications
 Log: evidence/test-e2e.log (mục "request backend trong pha 2"), evidence/implement-P10-run-phase2-requests.log</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="222.5" customHeight="1">
-      <c r="A57" s="22" t="inlineStr">
+    <row r="60" ht="222.5" customHeight="1">
+      <c r="A60" s="22" t="inlineStr">
         <is>
           <t>BUG-LINKCODE-28</t>
         </is>
       </c>
-      <c r="B57" s="22" t="inlineStr">
+      <c r="B60" s="22" t="inlineStr">
         <is>
           <t>Toàn bộ unit test, architecture test và ruff toàn repo pass</t>
         </is>
       </c>
-      <c r="C57" s="22" t="inlineStr">
+      <c r="C60" s="22" t="inlineStr">
         <is>
           <t>1. pytest tests/unit tests/architecture -q
 2. ruff check .
 3. So với baseline trước khi sửa code</t>
         </is>
       </c>
-      <c r="D57" s="22" t="inlineStr">
+      <c r="D60" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E57" s="22" t="inlineStr">
+      <c r="E60" s="22" t="inlineStr">
         <is>
           <t>pytest và ruff đều pass</t>
         </is>
       </c>
-      <c r="F57" s="22" t="inlineStr">
+      <c r="F60" s="22" t="inlineStr">
         <is>
           <t>pytest tests/unit tests/architecture: 885 passed, 18 failed (test_contract_profile.py ×12, test_profile_http.py ×6); ruff check . 19 lỗi ở module khác. Cùng danh sách với baseline trước khi 3.13 sửa code; file của task pass ruff. Lỗi test_app.py của lần chạy 3.10 không còn</t>
         </is>
       </c>
-      <c r="G57" s="22" t="inlineStr">
+      <c r="G60" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H57" s="22" t="inlineStr">
+      <c r="H60" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I57" s="22" t="inlineStr">
+      <c r="I60" s="22" t="inlineStr">
         <is>
           <t>Có sẵn trên main, không do 3.10/3.13. Nghi vấn: 18 test profile fail vì api_contract (aea2b26) chưa có các endpoint /profile mà backend đã có (remote có nhánh fix/adhoc-20261015-api-contract-sync); 19 lỗi ruff ở catalog/*, runtime/*, worker.py, tests/unit/test_catalog_crud.py
 Log: evidence/test-unit-2.log, evidence/implement-final-backend-2.log</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="239" customHeight="1">
-      <c r="A58" s="22" t="inlineStr">
+    <row r="61" ht="239" customHeight="1">
+      <c r="A61" s="22" t="inlineStr">
         <is>
           <t>BUG-REGDOSE-01</t>
         </is>
       </c>
-      <c r="B58" s="22" t="inlineStr">
+      <c r="B61" s="22" t="inlineStr">
         <is>
           <t>Đối chiếu scheduled_at có giây khi xác nhận liều</t>
         </is>
       </c>
-      <c r="C58" s="22" t="inlineStr">
+      <c r="C61" s="22" t="inlineStr">
         <is>
           <t>1. Từ backend chạy .venv/Scripts/python.exe -m pytest tests/integration/test_dose_confirmation_api.py::test_post_doses_batch_creates_dose_log_for_authenticated_patient__AC1_AC10_AC18 -q -ra.
 2. Fixture POST /doses/batch với danh sách một item ở Test Data.
 3. Đối chiếu items[0].scheduled_at với kỳ vọng test hiện có.</t>
         </is>
       </c>
-      <c r="D58" s="22" t="inlineStr">
+      <c r="D61" s="22" t="inlineStr">
         <is>
           <t>client_uuid: UUID mới; schedule_id: fixture; scheduled_at=2026-10-02T01:00:59.999Z; taken_at=2026-10-02T01:05:59.999Z</t>
         </is>
       </c>
-      <c r="E58" s="22" t="inlineStr">
+      <c r="E61" s="22" t="inlineStr">
         <is>
           <t>Theo test hiện có: HTTP 200, synced, da_uong và scheduled_at=2026-10-02T01:00:00Z.</t>
         </is>
       </c>
-      <c r="F58" s="22" t="inlineStr">
+      <c r="F61" s="22" t="inlineStr">
         <is>
           <t>HTTP 200, synced, da_uong; scheduled_at=2026-10-02T01:00:59.999000Z. Fail trong suite DB và lặp lại khi chạy riêng (1 failed trong 1.67s).</t>
         </is>
       </c>
-      <c r="G58" s="22" t="inlineStr">
+      <c r="G61" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H58" s="22" t="inlineStr">
+      <c r="H61" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I58" s="22" t="inlineStr">
+      <c r="I61" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn kỳ vọng chuẩn hóa tới phút trong test không khớp hành vi giữ thời điểm của API; chưa xác định phía nào sai theo contract/nghiệp vụ. Chưa chứng minh mất/trùng bản ghi liều; mức Medium tạm thời cho sai khác test, phải nâng tối thiểu High nếu xác nhận mất/trùng liều.
 Log: evidence/test-integration-db.log; evidence/test-dose-mismatch-repeat.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="140" customHeight="1">
+      <c r="A62" s="22" t="inlineStr">
+        <is>
+          <t>BUG-FAMADH-21</t>
+        </is>
+      </c>
+      <c r="B62" s="22" t="inlineStr">
+        <is>
+          <t>Giữ khoảng ngày hợp lệ khi refresh qua nửa đêm</t>
+        </is>
+      </c>
+      <c r="C62" s="22" t="inlineStr">
+        <is>
+          <t>1. Chạy evidence/review-date-rollover-repro.dart bằng flutter test --no-pub từ frontend/mobile.
+2. Chuyển đồng hồ sang 29/10/2026 và gọi refresh; xem khoảng request mà repository ghi nhận.</t>
+        </is>
+      </c>
+      <c r="D62" s="22" t="inlineStr">
+        <is>
+          <t>now 28/10 → 29/10/2026, selectedDate=31/07/2026</t>
+        </is>
+      </c>
+      <c r="E62" s="22" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa ngày đang chọn vào cửa sổ mới trước refresh; mọi request có from&lt;=to.</t>
+        </is>
+      </c>
+      <c r="F62" s="22" t="inlineStr">
+        <is>
+          <t>Tái hiện request from=01/08/2026, to=31/07/2026. Script tái hiện pass vì khẳng định bug tồn tại; hành vi sản phẩm Fail.</t>
+        </is>
+      </c>
+      <c r="G62" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H62" s="22" t="inlineStr">
+        <is>
+          <t>Ngọc Việt</t>
+        </is>
+      </c>
+      <c r="I62" s="22" t="inlineStr">
+        <is>
+          <t>selectedDate không được clamp khi earliestDate thay đổi theo đồng hồ; rangeFrom động nhưng rangeTo dựa tháng cũ.
+Log: evidence/test-rollover-known-issue.log</t>
         </is>
       </c>
     </row>
@@ -12922,17 +17061,17 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:A5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11:F25">
+  <conditionalFormatting sqref="F11:F28">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11:G25">
+  <conditionalFormatting sqref="G11:G28">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>OR(G11="Critical",G11="High")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G50:G58">
+  <conditionalFormatting sqref="G53:G62">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
@@ -12944,10 +17083,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G11:G25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G11:G28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="G50:G58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G53:G62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(testing): update CAREGIVER test cases for remove-link UI and cache revocation
Refs: 3.27
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -44,7 +44,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Link mời người thân'!$A$8:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Khung điều hướng app'!$A$8:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Duyệt yêu cầu liên kết'!$A$8:$I$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Người giám sát'!$A$8:$I$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Người giám sát'!$A$8:$I$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Cảnh báo người thân'!$A$8:$I$81</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'FCM token Android'!$A$8:$I$21</definedName>
   </definedNames>
@@ -519,7 +519,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$3:$E$4</f>
+              <f>'Report'!$F$3:$F$4</f>
             </numRef>
           </val>
         </ser>
@@ -13297,7 +13297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -13353,7 +13353,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>zannguyen</t>
+          <t>DrugTime Team</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13364,7 @@
         </is>
       </c>
       <c r="B4" s="21" t="n">
-        <v>46316</v>
+        <v>46319</v>
       </c>
     </row>
     <row r="5">
@@ -13391,7 +13391,7 @@
       </c>
       <c r="Q7" s="4" t="inlineStr">
         <is>
-          <t>Người thân đọc dữ liệu sức khỏe / nhận cảnh báo của patient</t>
+          <t>Quyền xem dữ liệu và thao tác gỡ liên kết của Patient</t>
         </is>
       </c>
     </row>
@@ -13567,36 +13567,36 @@
       </c>
       <c r="O9" s="10" t="inlineStr">
         <is>
-          <t>4
-5
-6
-7
-8</t>
+          <t>8
+9
+10
+11
+12</t>
         </is>
       </c>
       <c r="Q9" s="10" t="inlineStr">
         <is>
-          <t>Liên kết active?</t>
+          <t>Người gọi là Patient sở hữu liên kết?</t>
         </is>
       </c>
       <c r="R9" s="11" t="inlineStr">
         <is>
-          <t>Không</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="S9" s="11" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="T9" s="11" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U9" s="11" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -13674,38 +13674,38 @@
       </c>
       <c r="O10" s="10" t="inlineStr">
         <is>
-          <t>9
-10
-11
-12
-13
+          <t>13
 14
-15</t>
+15
+16
+17
+18
+19</t>
         </is>
       </c>
       <c r="Q10" s="10" t="inlineStr">
         <is>
-          <t>Công tắc chia sẻ bật?</t>
+          <t>Trạng thái liên kết trước khi gỡ?</t>
         </is>
       </c>
       <c r="R10" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>active</t>
         </is>
       </c>
       <c r="S10" s="11" t="inlineStr">
         <is>
-          <t>Không</t>
+          <t>active</t>
         </is>
       </c>
       <c r="T10" s="11" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>revoked</t>
         </is>
       </c>
       <c r="U10" s="11" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>active</t>
         </is>
       </c>
     </row>
@@ -13755,29 +13755,58 @@
           <t>AC5 · Đoán lỗi (truy cập dữ liệu người khác) · test_caregivers_rejects_query_parameters__AC11 · evidence/test-integration.log</t>
         </is>
       </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>action_dialog (thao tác hộp thoại gỡ liên kết)</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>Bấm "Gỡ liên kết" (xác nhận gọi API)
+Bấm "Hủy" (đóng hộp thoại)</t>
+        </is>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>4
+5</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>Bấm ngoài dialog khi đang loading
+Gửi request trùng khi đang busy</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>20
+21</t>
+        </is>
+      </c>
       <c r="Q11" s="10" t="inlineStr">
         <is>
-          <t>Patient còn đồng ý family_sharing?</t>
+          <t>Xác nhận trên hộp thoại gỡ liên kết?</t>
         </is>
       </c>
       <c r="R11" s="11" t="inlineStr">
         <is>
+          <t>Yes (Gỡ)</t>
+        </is>
+      </c>
+      <c r="S11" s="11" t="inlineStr">
+        <is>
+          <t>No (Hủy)</t>
+        </is>
+      </c>
+      <c r="T11" s="11" t="inlineStr">
+        <is>
+          <t>Yes (Gỡ)</t>
+        </is>
+      </c>
+      <c r="U11" s="11" t="inlineStr">
+        <is>
           <t>-</t>
-        </is>
-      </c>
-      <c r="S11" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T11" s="11" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
-      <c r="U11" s="11" t="inlineStr">
-        <is>
-          <t>Có</t>
         </is>
       </c>
     </row>
@@ -13829,6 +13858,35 @@
           <t>AC12 · EP (1,2,3) · Đoán lỗi (gửi trùng) · test_enable_disable_idempotent_and_audit__AC12 · evidence/test-integration.log</t>
         </is>
       </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>revocation_event (nguồn phát hiện thu hồi quyền ở Family Member)</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden khi truy cập dữ liệu
+Đồng bộ danh sách liên kết mới thiếu Patient</t>
+        </is>
+      </c>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>6
+7</t>
+        </is>
+      </c>
+      <c r="N12" s="10" t="inlineStr">
+        <is>
+          <t>Lỗi mạng tạm thời hoặc 5xx
+Token hết hạn 401</t>
+        </is>
+      </c>
+      <c r="O12" s="10" t="inlineStr">
+        <is>
+          <t>22
+23</t>
+        </is>
+      </c>
       <c r="Q12" s="6" t="inlineStr">
         <is>
           <t>Action</t>
@@ -13903,7 +13961,7 @@
       </c>
       <c r="Q13" s="10" t="inlineStr">
         <is>
-          <t>403 + access_logs denied; không có trong danh sách nhận cảnh báo</t>
+          <t>DELETE /family/links/{id} -&gt; 204 No Content, gỡ khỏi UI, SnackBar</t>
         </is>
       </c>
       <c r="R13" s="11" t="inlineStr">
@@ -13911,11 +13969,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="S13" s="11" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="S13" s="11" t="inlineStr"/>
       <c r="T13" s="11" t="inlineStr">
         <is>
           <t>X</t>
@@ -13971,17 +14025,17 @@
       </c>
       <c r="Q14" s="10" t="inlineStr">
         <is>
-          <t>200 + access_logs allowed; có trong danh sách nhận cảnh báo</t>
+          <t>Đóng dialog, giữ nguyên liên kết, không gọi API</t>
         </is>
       </c>
       <c r="R14" s="11" t="inlineStr"/>
-      <c r="S14" s="11" t="inlineStr"/>
+      <c r="S14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="T14" s="11" t="inlineStr"/>
-      <c r="U14" s="11" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="U14" s="11" t="inlineStr"/>
     </row>
     <row r="15" ht="74" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
@@ -14030,6 +14084,19 @@
           <t>AC10 · test_enable_legacy_link_409_confirmation_missing_but_disable_ok__AC10 · evidence/test-integration.log</t>
         </is>
       </c>
+      <c r="Q15" s="10" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden khong_co_quyen</t>
+        </is>
+      </c>
+      <c r="R15" s="11" t="inlineStr"/>
+      <c r="S15" s="11" t="inlineStr"/>
+      <c r="T15" s="11" t="inlineStr"/>
+      <c r="U15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="90.5" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
@@ -14172,6 +14239,11 @@
           <t>AC22 · EP (9,10,11,12) · BVA (min-1) · test_new_routes_invalid_path_id_is_422 · evidence/implement-final-backend.log</t>
         </is>
       </c>
+      <c r="Q18" s="4" t="inlineStr">
+        <is>
+          <t>Xử lý cache &amp; state khi Family Member bị thu hồi quyền truy cập</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="74" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
@@ -14218,6 +14290,26 @@
       <c r="I19" s="8" t="inlineStr">
         <is>
           <t>AC10 · EP (13) · test_missing_link_404_without_allowed_audit__AC10 · evidence/test-integration.log</t>
+        </is>
+      </c>
+      <c r="Q19" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T19" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
         </is>
       </c>
     </row>
@@ -14271,6 +14363,26 @@
           <t>AC5 · EP (14) · test_new_endpoints_denied_caller_matrix__AC5 · evidence/test-integration.log</t>
         </is>
       </c>
+      <c r="Q20" s="10" t="inlineStr">
+        <is>
+          <t>Nhận HTTP 403 Forbidden do bị thu hồi liên kết?</t>
+        </is>
+      </c>
+      <c r="R20" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S20" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T20" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="90.5" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
@@ -14320,6 +14432,26 @@
           <t>AC13 · Chuyển trạng thái (active→revoked) · test_revoke_keeps_history_and_replay_returns_same_time__AC13 · evidence/test-integration.log</t>
         </is>
       </c>
+      <c r="Q21" s="10" t="inlineStr">
+        <is>
+          <t>Dữ liệu/cache thuộc phạm vi Patient bị thu hồi?</t>
+        </is>
+      </c>
+      <c r="R21" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S21" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T21" s="11" t="inlineStr">
+        <is>
+          <t>No (Patient khác)</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="74" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
@@ -14368,6 +14500,26 @@
           <t>AC13 · test_relink_after_revoke_starts_unshared_with_new_evidence__AC13 · evidence/test-integration.log</t>
         </is>
       </c>
+      <c r="Q22" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R22" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S22" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T22" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="74" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
@@ -14415,6 +14567,18 @@
           <t>AC10 · Chuyển trạng thái (chuyển bị cấm) · test_revoke_pending_or_rejected_409__AC10 · evidence/test-integration.log</t>
         </is>
       </c>
+      <c r="Q23" s="10" t="inlineStr">
+        <is>
+          <t>Xóa Patient khỏi state &amp; xóa SQLite cache &amp; xóa RAM history &amp; dọn alert</t>
+        </is>
+      </c>
+      <c r="R23" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S23" s="11" t="inlineStr"/>
+      <c r="T23" s="11" t="inlineStr"/>
     </row>
     <row r="24" ht="57.5" customHeight="1">
       <c r="A24" s="7" t="inlineStr">
@@ -14460,6 +14624,22 @@
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>AC10 · Đoán lỗi · test_revoke_with_body_is_422__AC10 · evidence/test-integration.log</t>
+        </is>
+      </c>
+      <c r="Q24" s="10" t="inlineStr">
+        <is>
+          <t>Giữ nguyên dữ liệu &amp; cache, không xóa nhầm</t>
+        </is>
+      </c>
+      <c r="R24" s="11" t="inlineStr"/>
+      <c r="S24" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T24" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -14807,7 +14987,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="90.5" customHeight="1">
+    <row r="32" ht="123.5" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
         <is>
           <t>TC-CAREGIVER-24</t>
@@ -14815,33 +14995,35 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Hủy liên kết trên app có hộp xác nhận</t>
+          <t>Gỡ liên kết trên app với hộp thoại xác nhận</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Có người giám sát Nguyễn Văn An</t>
+          <t>Có người giám sát trong danh sách liên kết active (ví dụ Bác An)</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>1. Bấm Hủy liên kết rồi Giữ liên kết
-2. Bấm Hủy liên kết rồi xác nhận</t>
+          <t>1. Mở màn Người thân đã liên kết (CaregiversScreen)
+2. Bấm nút Gỡ liên kết tại mục Bác An
+3. Tại hộp thoại Gỡ liên kết với người thân?, bấm Hủy
+4. Bấm lại Gỡ liên kết và chọn Gỡ liên kết (xác nhận)</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>linkId=1, name='Bác An'</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>Hộp nêu người thân mất quyền xem ngay và phải gửi yêu cầu mới; giữ thì không gọi API; xác nhận thì gọi revoke rồi tải lại, mục biến mất, báo "Đã hủy liên kết với Nguyễn Văn An."</t>
+          <t>Hộp thoại nêu rõ người thân mất quyền xem ngay; chọn Hủy thì đóng hộp thoại không gọi API; xác nhận thì gọi DELETE /family/links/{id}, nút chuyển loading, gỡ mục khỏi danh sách và hiện SnackBar 'Đã gỡ liên kết với Bác An.'</t>
         </is>
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>Đúng như mong đợi</t>
+          <t>Đúng như mong đợi (hộp thoại chuẩn, nút Hủy đóng dialog, xác nhận gọi DELETE 204 và hiện SnackBar)</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
@@ -14851,7 +15033,7 @@
       </c>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>AC21 · caregivers_screen_test.dart (AC21) · evidence/implement-final-frontend.log</t>
+          <t>AC1, AC2, AC3 · caregivers_screen_test.dart · evidence/implement-final-frontend.log</t>
         </is>
       </c>
     </row>
@@ -15045,61 +15227,453 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39">
-      <c r="G39" s="12" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="H39" s="13">
-        <f>COUNTIF(H9:H36,"Pass")</f>
+    <row r="37" ht="90.5" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-29</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Màn hình Người thân đã liên kết hiển thị danh sách và nút Gỡ liên kết cho từng người; bấm Hủy không đổi dữ liệu</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Patient đã đăng nhập, có ít nhất một người thân liên kết hợp lệ</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở màn hình Hồ sơ &gt; Người thân đã liên kết
+2. Kiểm tra danh sách hiển thị và sự xuất hiện của nút Gỡ liên kết
+3. Bấm Gỡ liên kết, sau đó bấm Hủy trên dialog xác nhận</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>caregiver: Bác An (linkId=1)</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Hiển thị đúng tên, ngày liên kết; mỗi item có nút Gỡ liên kết; khi bấm Hủy, dialog đóng lại, không gọi API DELETE và giữ nguyên danh sách.</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi (CaregiversScreen render đủ thông tin, dialog đóng khi hủy, không gọi API)</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>AC1, AC2 · caregivers_screen_test.dart · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="90.5" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-30</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Xác nhận gỡ liên kết gọi đúng API DELETE /family/links/{id} nhận 204 No Content và cập nhật UI</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Patient đang mở dialog xác nhận gỡ liên kết với Bác An</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm nút Gỡ liên kết trên dialog xác nhận
+2. Theo dõi request gửi đi từ RemoteCaregiverRepository
+3. Kiểm tra phản hồi HTTP 204 No Content và cập nhật state/UI</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>linkId=1, method=DELETE, url=/family/links/1</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>Gửi đúng DELETE /family/links/1 (không body), nhận 204 No Content; mục Bác An biến mất khỏi danh sách và hiển thị SnackBar: Đã gỡ liên kết với Bác An.</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi (gọi DELETE 204, item được gỡ và SnackBar hiển thị chuẩn)</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>AC3 · remote_caregiver_repository_test.dart, caregivers_screen_test.dart · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="74" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-31</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Xử lý khi API gỡ liên kết thất bại (lỗi mạng hoặc server)</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Patient xác nhận gỡ liên kết nhưng backend trả lỗi (ví dụ lỗi mạng hoặc 500)</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm nút Gỡ liên kết trên dialog xác nhận
+2. Backend giả lập ném CaregiverFailureKind.network
+3. Quan sát giao diện và danh sách hiển thị</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>linkId=1, failure=network</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>Giữ nguyên danh sách người thân, không xóa nhầm dữ liệu; hiển thị thông báo lỗi phù hợp trên SnackBar và cho phép người dùng thử lại.</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi (danh sách giữ nguyên, SnackBar báo lỗi và cho phép thử lại)</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>AC4 · caregivers_screen_test.dart · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="90.5" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-32</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Khóa nút và hiển thị loading spinner chống bấm trùng; tự động tải lại nếu link đã bị gỡ từ trước</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Patient bấm nút Gỡ liên kết</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm xác nhận gỡ liên kết
+2. Trong khi request đang pending, cố gắng bấm nút lần nữa
+3. Kiểm tra trường hợp server trả 404 (đã bị gỡ từ trước)</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>linkId=1</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Nút chuyển sang CircularProgressIndicator và bị khóa không cho bấm trùng; nếu server báo link không tồn tại (404), tự động gọi load() làm mới danh sách.</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi (loading spinner hiển thị, nút bị khóa, tự reload khi gặp lỗi transition/not found)</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>AC5 · caregivers_screen_test.dart · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="107" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-33</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Family Member gặp HTTP 403 Forbidden khi truy cập dữ liệu Patient bị gỡ: xóa khỏi state và dọn dẹp cache</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Family Member đang liên kết với Patient A và Patient B; Patient A đã gỡ liên kết</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>1. Family Member gửi request truy cập lịch sử tuân thủ hoặc cảnh báo của Patient A
+2. API trả về HTTP 403 Forbidden (AdherenceFailureKind.denied)
+3. LinkedPatientsController và AdherenceController xử lý phản hồi 403</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>patientId=patient-A-uuid</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>Patient A bị xóa khỏi danh sách linked patients; SQLite cache lịch uống của Patient A bị dọn sạch (clearPatientData); history trên RAM bị xóa (history=null); alerts của Patient A bị loại bỏ.</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi (state loại bỏ patientA, clearPatientData được gọi, history reset null, alert bị dọn)</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="inlineStr">
+        <is>
+          <t>AC6 · linked_patients_controller_test.dart, adherence_controller_test.dart · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="90.5" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-34</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Family Member đồng bộ danh sách liên kết mới từ backend: xóa bỏ các Patient không còn trong danh sách</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Family Member có state cục bộ gồm Patient A, Patient B, Patient C</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>1. Backend trả về danh sách liên kết mới chỉ gồm Patient B và Patient C
+2. LinkedPatientsController.syncPatients được kích hoạt
+3. Kiểm tra danh sách hiển thị và cache cục bộ</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>newActivePatients=[Patient B, Patient C]</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>Patient A tự động bị xóa khỏi state hiển thị; toàn bộ cache SQLite và alert của Patient A được dọn sạch; dữ liệu của Patient B và C giữ nguyên.</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi (Patient A bị loại bỏ, cache SQLite được dọn, Patient B và C còn nguyên)</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I42" s="8" t="inlineStr">
+        <is>
+          <t>AC7 · linked_patients_controller_test.dart · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="90.5" customHeight="1">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-35</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Độc lập dữ liệu giữa các bệnh nhân khi gỡ liên kết</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Local database và alert store đang lưu dữ liệu của cả Patient A và Patient B</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>1. Kích hoạt thu hồi quyền truy cập đối với Patient A (clearPatientData và removePatient)
+2. Truy vấn dữ liệu SQLite của schedulesTable
+3. Kiểm tra danh sách alerts trong FamilyAlertController</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>patientA, patientB</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>Toàn bộ bản ghi của Patient A bị xóa sạch; toàn bộ bản ghi của Patient B được bảo toàn 100%, không bị ảnh hưởng.</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi (bản ghi Patient A bị xóa, Patient B còn nguyên vẹn)</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="inlineStr">
+        <is>
+          <t>AC8 · local_medication_store_test.dart, linked_patients_controller_test.dart · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="90.5" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>TC-CAREGIVER-36</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>An toàn khi nhiều request 403 thu hồi quyền diễn ra đồng thời hoặc lặp lại (concurrency &amp; idempotency)</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>LinkedPatientsController đang quản lý Patient A</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>1. Gửi đồng thời 5 lời gọi handleRevocation cho cùng Patient A
+2. Chờ toàn bộ các lời gọi hoàn tất
+3. Gửi thêm một lời gọi handleRevocation lặp lại khi Patient A đã bị gỡ</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>5 concurrent calls for patientA</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>Các lời gọi hoàn thành an toàn, không ném exception; patientA bị xóa sạch và không bị nhân bản hay hồi phục dữ liệu trái phép.</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi (5 concurrent calls hoàn thành an toàn, không có race condition)</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I44" s="8" t="inlineStr">
+        <is>
+          <t>AC9 · linked_patients_controller_test.dart · evidence/implement-final-frontend.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47">
+      <c r="G47" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H47" s="13">
+        <f>COUNTIF(H9:H44,"Pass")</f>
         <v/>
       </c>
     </row>
-    <row r="40">
-      <c r="G40" s="12" t="inlineStr">
+    <row r="48">
+      <c r="G48" s="12" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="H40" s="13">
-        <f>COUNTIF(H9:H36,"Fail")</f>
+      <c r="H48" s="13">
+        <f>COUNTIF(H9:H44,"Fail")</f>
         <v/>
       </c>
     </row>
-    <row r="41">
-      <c r="G41" s="12" t="inlineStr">
+    <row r="49">
+      <c r="G49" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="H41" s="13">
-        <f>COUNTIF(H9:H36,"Pending")</f>
+      <c r="H49" s="13">
+        <f>COUNTIF(H9:H44,"Pending")</f>
         <v/>
       </c>
     </row>
-    <row r="42">
-      <c r="G42" s="12" t="inlineStr">
+    <row r="50">
+      <c r="G50" s="12" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="H42" s="13">
-        <f>SUM(H39:H41)</f>
+      <c r="H50" s="13">
+        <f>SUM(H47:H49)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A8:I36"/>
-  <conditionalFormatting sqref="H9:H36">
+  <autoFilter ref="A8:I44"/>
+  <conditionalFormatting sqref="H9:H44">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Fail"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H9:H36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H9:H44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pass,Fail,Pending"</formula1>
     </dataValidation>
   </dataValidations>
@@ -23299,6 +23873,11 @@
       </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
+          <t>DrugTime Team</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
@@ -23315,15 +23894,19 @@
         </is>
       </c>
       <c r="C3" s="11">
-        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59+'Lịch uống thuốc'!$H$51+'Tải lịch uống'!$H$32+'Tương tác thuốc-thuốc'!$H$52+'Tương tác thuốc-thực phẩm'!$H$17+'Tra cứu hoạt chất'!$H$17+'Mã liên kết người thân'!$H$47+'Landing page'!$H$43+'Yêu cầu liên kết người thân'!$H$72+'Theo dõi người thân (app)'!$H$46+'Link mời người thân'!$H$24+'Khung điều hướng app'!$H$16+'Duyệt yêu cầu liên kết'!$H$38+'Người giám sát'!$H$39</f>
+        <f>'Android build'!$H$20+'Đăng nhập người dùng'!$H$59+'Lịch uống thuốc'!$H$51+'Tải lịch uống'!$H$32+'Tương tác thuốc-thuốc'!$H$52+'Tương tác thuốc-thực phẩm'!$H$17+'Tra cứu hoạt chất'!$H$17+'Mã liên kết người thân'!$H$47+'Landing page'!$H$43+'Yêu cầu liên kết người thân'!$H$72+'Theo dõi người thân (app)'!$H$46+'Link mời người thân'!$H$24+'Khung điều hướng app'!$H$16+'Duyệt yêu cầu liên kết'!$H$38</f>
         <v/>
       </c>
       <c r="D3" s="11">
         <f>'Chọn thuốc danh mục'!$H$40+'Hồi quy xác nhận liều'!$H$12+'Cảnh báo người thân'!$H$84+'FCM token Android'!$H$24</f>
         <v/>
       </c>
-      <c r="E3" s="15">
-        <f>SUM(C3:D3)</f>
+      <c r="E3" s="11">
+        <f>'Người giám sát'!$H$47</f>
+        <v/>
+      </c>
+      <c r="F3" s="15">
+        <f>SUM(C3:E3)</f>
         <v/>
       </c>
     </row>
@@ -23335,15 +23918,19 @@
         </is>
       </c>
       <c r="C4" s="11">
-        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60+'Lịch uống thuốc'!$H$52+'Tải lịch uống'!$H$33+'Tương tác thuốc-thuốc'!$H$53+'Tương tác thuốc-thực phẩm'!$H$18+'Tra cứu hoạt chất'!$H$18+'Mã liên kết người thân'!$H$48+'Landing page'!$H$44+'Yêu cầu liên kết người thân'!$H$73+'Theo dõi người thân (app)'!$H$47+'Link mời người thân'!$H$25+'Khung điều hướng app'!$H$17+'Duyệt yêu cầu liên kết'!$H$39+'Người giám sát'!$H$40</f>
+        <f>'Android build'!$H$21+'Đăng nhập người dùng'!$H$60+'Lịch uống thuốc'!$H$52+'Tải lịch uống'!$H$33+'Tương tác thuốc-thuốc'!$H$53+'Tương tác thuốc-thực phẩm'!$H$18+'Tra cứu hoạt chất'!$H$18+'Mã liên kết người thân'!$H$48+'Landing page'!$H$44+'Yêu cầu liên kết người thân'!$H$73+'Theo dõi người thân (app)'!$H$47+'Link mời người thân'!$H$25+'Khung điều hướng app'!$H$17+'Duyệt yêu cầu liên kết'!$H$39</f>
         <v/>
       </c>
       <c r="D4" s="11">
         <f>'Chọn thuốc danh mục'!$H$41+'Hồi quy xác nhận liều'!$H$13+'Cảnh báo người thân'!$H$85+'FCM token Android'!$H$25</f>
         <v/>
       </c>
-      <c r="E4" s="15">
-        <f>SUM(C4:D4)</f>
+      <c r="E4" s="11">
+        <f>'Người giám sát'!$H$48</f>
+        <v/>
+      </c>
+      <c r="F4" s="15">
+        <f>SUM(C4:E4)</f>
         <v/>
       </c>
     </row>
@@ -23362,8 +23949,12 @@
         <f>D3+D4</f>
         <v/>
       </c>
-      <c r="E5" s="15">
-        <f>SUM(C5:D5)</f>
+      <c r="E5" s="11">
+        <f>E3+E4</f>
+        <v/>
+      </c>
+      <c r="F5" s="15">
+        <f>SUM(C5:E5)</f>
         <v/>
       </c>
     </row>
@@ -23375,15 +23966,19 @@
       </c>
       <c r="B6" s="10" t="inlineStr"/>
       <c r="C6" s="11">
-        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61+'Lịch uống thuốc'!$H$53+'Tải lịch uống'!$H$34+'Tương tác thuốc-thuốc'!$H$54+'Tương tác thuốc-thực phẩm'!$H$19+'Tra cứu hoạt chất'!$H$19+'Mã liên kết người thân'!$H$49+'Landing page'!$H$45+'Yêu cầu liên kết người thân'!$H$74+'Theo dõi người thân (app)'!$H$48+'Link mời người thân'!$H$26+'Khung điều hướng app'!$H$18+'Duyệt yêu cầu liên kết'!$H$40+'Người giám sát'!$H$41</f>
+        <f>'Android build'!$H$22+'Đăng nhập người dùng'!$H$61+'Lịch uống thuốc'!$H$53+'Tải lịch uống'!$H$34+'Tương tác thuốc-thuốc'!$H$54+'Tương tác thuốc-thực phẩm'!$H$19+'Tra cứu hoạt chất'!$H$19+'Mã liên kết người thân'!$H$49+'Landing page'!$H$45+'Yêu cầu liên kết người thân'!$H$74+'Theo dõi người thân (app)'!$H$48+'Link mời người thân'!$H$26+'Khung điều hướng app'!$H$18+'Duyệt yêu cầu liên kết'!$H$40</f>
         <v/>
       </c>
       <c r="D6" s="11">
         <f>'Chọn thuốc danh mục'!$H$42+'Hồi quy xác nhận liều'!$H$14+'Cảnh báo người thân'!$H$86+'FCM token Android'!$H$26</f>
         <v/>
       </c>
-      <c r="E6" s="15">
-        <f>SUM(C6:D6)</f>
+      <c r="E6" s="11">
+        <f>'Người giám sát'!$H$49</f>
+        <v/>
+      </c>
+      <c r="F6" s="15">
+        <f>SUM(C6:E6)</f>
         <v/>
       </c>
     </row>
@@ -23402,8 +23997,12 @@
         <f>D5+D6</f>
         <v/>
       </c>
-      <c r="E7" s="15">
-        <f>SUM(C7:D7)</f>
+      <c r="E7" s="11">
+        <f>E5+E6</f>
+        <v/>
+      </c>
+      <c r="F7" s="15">
+        <f>SUM(C7:E7)</f>
         <v/>
       </c>
     </row>
@@ -24158,7 +24757,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="123.5" customHeight="1">
+    <row r="27" ht="74" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Quản lý người giám sát</t>
@@ -24166,7 +24765,7 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>Patient xem người giám sát đã chấp thuận, bật/tắt chia sẻ từng người và hủy liên kết; quyết định có hiệu lực ngay ở request kế tiếp. Backend /family/caregivers, /family/links/{id}/sharing|revoke, migration audit; mobile Hồ sơ &gt; Người giám sát.</t>
+          <t>Quản lý người giám sát và gỡ liên kết người thân trên mobile (task 3.27)</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
@@ -24175,15 +24774,15 @@
         </is>
       </c>
       <c r="D27" s="18">
-        <f>IFERROR(('Người giám sát'!$H$42-'Người giám sát'!$H$41)/'Người giám sát'!$H$42,0)</f>
+        <f>IFERROR(('Người giám sát'!$H$50-'Người giám sát'!$H$49)/'Người giám sát'!$H$50,0)</f>
         <v/>
       </c>
       <c r="E27" s="18">
-        <f>IFERROR('Người giám sát'!$H$39/'Người giám sát'!$H$42,0)</f>
+        <f>IFERROR('Người giám sát'!$H$47/'Người giám sát'!$H$50,0)</f>
         <v/>
       </c>
       <c r="F27" s="18">
-        <f>IFERROR('Người giám sát'!$H$40/'Người giám sát'!$H$42,0)</f>
+        <f>IFERROR('Người giám sát'!$H$48/'Người giám sát'!$H$50,0)</f>
         <v/>
       </c>
       <c r="G27" s="11" t="inlineStr">
@@ -24193,12 +24792,12 @@
       </c>
       <c r="H27" s="10" t="inlineStr">
         <is>
-          <t>Toàn bộ test tự động (tích hợp Postgres thật gồm phân quyền chéo, hiệu lực ngay, chạy đua; unit; widget) pass trong phiên 2026-10-21. Còn Pending: kịch bản chạy tay trên hai thiết bị (AC23).</t>
+          <t>Hoàn thành 100% kiểm thử unit, widget và tích hợp controller. 35/36 test cases pass (1 manual pending trên 2 thiết bị thật).</t>
         </is>
       </c>
       <c r="I27" s="11" t="inlineStr">
         <is>
-          <t>zannguyen</t>
+          <t>DrugTime Team</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(adherence): record PB21 cases and results
Refs: 3.25
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -26,7 +26,8 @@
     <sheet name="Cảnh báo người thân" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="FCM token Android" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="Redeem flow E2E" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Report" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Lịch sử tuân thủ người thân" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Report" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Android build'!$A$8:$I$17</definedName>
@@ -49,6 +50,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Cảnh báo người thân'!$A$8:$I$81</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'FCM token Android'!$A$8:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Redeem flow E2E'!$A$8:$I$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Lịch sử tuân thủ người thân'!$A$8:$I$53</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -387,12 +389,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$30</f>
+              <f>'Report'!$A$11:$A$31</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$11:$D$30</f>
+              <f>'Report'!$D$11:$D$31</f>
             </numRef>
           </val>
         </ser>
@@ -411,12 +413,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$30</f>
+              <f>'Report'!$A$11:$A$31</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$11:$E$30</f>
+              <f>'Report'!$E$11:$E$31</f>
             </numRef>
           </val>
         </ser>
@@ -435,12 +437,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$11:$A$30</f>
+              <f>'Report'!$A$11:$A$31</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$11:$F$30</f>
+              <f>'Report'!$F$11:$F$31</f>
             </numRef>
           </val>
         </ser>
@@ -543,7 +545,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>32</row>
+      <row>33</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -565,7 +567,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>32</row>
+      <row>33</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3240000"/>
@@ -24866,7 +24868,2637 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I68"/>
+  <dimension ref="A1:V59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="8" customWidth="1" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>DrugTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Module Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Lịch sử tuân thủ cho người thân (FADH)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>46319</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed Date</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Quyền xem lịch sử PB21</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Comments(if any)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="123.5" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-01</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Xem cùng lịch sử bằng patient và người thân</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
+3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19 08:00 +07; status=da_uong</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>200; payload đúng contract, hai response giống nhau; mỗi caller có allowed; audit không chứa nội dung thuốc/liều.</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr"/>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC1,AC9 · Decision Table (R1) · EP (1) · test_self_and_family_success_are_audited · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>Quyền người thân</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>Link active + sharing + hai consent</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>Không liên kết hoặc patient khác
+Thiếu health_data
+Thiếu family_sharing
+Sharing tắt</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>4
+5
+6
+7</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Link active</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V9" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="123.5" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-02</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Chặn người thân chưa liên kết</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực. F tồn tại, không có caregiver_link với P</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
+3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>case=unlinked; patient_id=P</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>403 {detail: khong_co_quyen}; Cache-Control: no-store; có denied và dose_logs không đổi.</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC4 · Decision Table (R2) · EP (4) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11[unlinked] · evidence/test-history.log</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>Mẫu số tỷ lệ</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>Liều xác nhận hợp lệ hoặc chưa xác nhận đã quá +120
+Không có liều đủ điều kiện</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>2
+3</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr"/>
+      <c r="O10" s="10" t="inlineStr"/>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>health_data</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="123.5" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Chặn khi thiếu consent sức khỏe</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực. Thu hồi health_data của P</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
+3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>case=health_consent; patient_id=P</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>403 {detail: khong_co_quyen}; Cache-Control: no-store; có denied và dose_logs không đổi.</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC4 · Decision Table (R3) · EP (5) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11[health_consent] · evidence/test-history.log</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>family_sharing</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U11" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="123.5" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Chặn khi thiếu consent chia sẻ</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực. Thu hồi family_sharing của P</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
+3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>case=family_consent; patient_id=P</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>403 {detail: khong_co_quyen}; Cache-Control: no-store; có denied và dose_logs không đổi.</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC4 · Decision Table (R4) · EP (6) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11[family_consent] · evidence/test-history.log</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
+        <is>
+          <t>sharing_enabled</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V12" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="123.5" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Chặn khi bệnh nhân tắt chia sẻ</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực. Đặt sharing_enabled=false</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
+3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>case=sharing_off; patient_id=P</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>403 {detail: khong_co_quyen}; Cache-Control: no-store; có denied và dose_logs không đổi.</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC4 · Decision Table (R5) · EP (7) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11[sharing_off] · evidence/test-history.log</t>
+        </is>
+      </c>
+      <c r="Q13" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="T13" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="U13" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="V13" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="123.5" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-06</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Chặn sửa patient_id sang bệnh nhân khác</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực. Thêm patient Q không liên kết với F.</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
+3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>patient_id=Q</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>403; denied cho Q; không trả dữ liệu Q; request P trước đó có allowed.</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr"/>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC4 · EP (4) · kiểm truy cập chéo · test_family_patient_selector_tamper · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>200 + allowed</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S14" s="11" t="inlineStr"/>
+      <c r="T14" s="11" t="inlineStr"/>
+      <c r="U14" s="11" t="inlineStr"/>
+      <c r="V14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="156.5" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-07</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Mất quyền ngay sau thay đổi health_consent</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
+3. Giữ nguyên token; thực hiện health_consent.
+4. Gửi GET /adherence ngay bằng cùng token và kiểm denied.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>change=health_consent; cùng bearer session</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Request đầu 200, request kế tiếp 403 {detail: khong_co_quyen}; audit lần lượt allowed, denied.</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC5 · Chuyển trạng thái (allowed → denied) · test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12[health_consent] · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
+        </is>
+      </c>
+      <c r="Q15" s="10" t="inlineStr">
+        <is>
+          <t>403 + denied</t>
+        </is>
+      </c>
+      <c r="R15" s="11" t="inlineStr"/>
+      <c r="S15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="V15" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="156.5" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-08</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Mất quyền ngay sau thay đổi family_consent</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
+3. Giữ nguyên token; thực hiện family_consent.
+4. Gửi GET /adherence ngay bằng cùng token và kiểm denied.</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>change=family_consent; cùng bearer session</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Request đầu 200, request kế tiếp 403 {detail: khong_co_quyen}; audit lần lượt allowed, denied.</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr"/>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC5 · Chuyển trạng thái (allowed → denied) · test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12[family_consent] · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="156.5" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-09</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Mất quyền ngay sau thay đổi sharing_off</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
+3. Giữ nguyên token; thực hiện sharing_off.
+4. Gửi GET /adherence ngay bằng cùng token và kiểm denied.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>change=sharing_off; cùng bearer session</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Request đầu 200, request kế tiếp 403 {detail: khong_co_quyen}; audit lần lượt allowed, denied.</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr"/>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC5 · Chuyển trạng thái (allowed → denied) · test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12[sharing_off] · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="156.5" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-10</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Mất quyền ngay sau thay đổi unlink</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
+3. Giữ nguyên token; thực hiện unlink.
+4. Gửi GET /adherence ngay bằng cùng token và kiểm denied.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>change=unlink; cùng bearer session</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Request đầu 200, request kế tiếp 403 {detail: khong_co_quyen}; audit lần lượt allowed, denied.</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr"/>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC5 · Chuyển trạng thái (allowed → denied) · test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12[unlink] · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="107" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Chặn lịch sử khi lỗi allowed_insert</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gắn fault injection allowed_insert theo test access.
+3. GET /adherence, kiểm status/body, log, SQL history read và snapshot DB.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>failure=allowed_insert</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>500 {detail: Internal server error}; no-store; không trả dữ liệu sức khỏe; không thay dose_logs; lỗi quyền/audit trước đọc thì không SELECT lịch sử.</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC7 · Đoán lỗi (fail-closed) · test_audit_permission_and_commit_failure_fail_closed_without_health__AC13[allowed_insert] · evidence/test-history.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="107" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Chặn lịch sử khi lỗi commit</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gắn fault injection commit theo test access.
+3. GET /adherence, kiểm status/body, log, SQL history read và snapshot DB.</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>failure=commit</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>500 {detail: Internal server error}; no-store; không trả dữ liệu sức khỏe; không thay dose_logs; lỗi quyền/audit trước đọc thì không SELECT lịch sử.</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC7 · Đoán lỗi (fail-closed) · test_audit_permission_and_commit_failure_fail_closed_without_health__AC13[commit] · evidence/test-history.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="107" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-13</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Chặn lịch sử khi lỗi denied_insert</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gắn fault injection denied_insert theo test access.
+3. GET /adherence, kiểm status/body, log, SQL history read và snapshot DB.</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>failure=denied_insert</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>500 {detail: Internal server error}; no-store; không trả dữ liệu sức khỏe; không thay dose_logs; lỗi quyền/audit trước đọc thì không SELECT lịch sử.</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC7 · Đoán lỗi (fail-closed) · test_audit_permission_and_commit_failure_fail_closed_without_health__AC13[denied_insert] · evidence/test-history.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="107" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-14</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Chặn lịch sử khi lỗi permission_read</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gắn fault injection permission_read theo test access.
+3. GET /adherence, kiểm status/body, log, SQL history read và snapshot DB.</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>failure=permission_read</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>500 {detail: Internal server error}; no-store; không trả dữ liệu sức khỏe; không thay dose_logs; lỗi quyền/audit trước đọc thì không SELECT lịch sử.</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC7 · Đoán lỗi (fail-closed) · test_audit_permission_and_commit_failure_fail_closed_without_health__AC13[permission_read] · evidence/test-history.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="123.5" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Giữ denied audit sau rollback nghiệp vụ</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực. Thu hồi health_data.</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>1. Gắn context theo dõi rollback như test.
+2. GET /adherence bằng patient P.
+3. Sau rollback đọc access_logs bằng kết nối DB riêng.</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>health_data=thu_hoi</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>403; outer transaction đã rollback; denied consent_revoked còn bền.</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC7 · Đoán lỗi (rollback) · test_denied_audit_survives_outer_transaction_rollback · evidence/test-history.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="107" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-16</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối phiên missing</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>1. Chuẩn bị auth theo kind của test (không in token).
+2. GET /adherence.
+3. Kiểm 401, no-store, body chỉ có detail và không ghi allowed.</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>kind=missing</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>401; no-store; không trả dữ liệu sức khỏe; không có access_logs.</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC4 · Đoán lỗi (xác thực) · test_authentication_401_and_no_store_without_health_payload__AC14[missing] · evidence/test-history.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="107" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-17</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối phiên invalid</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1. Chuẩn bị auth theo kind của test (không in token).
+2. GET /adherence.
+3. Kiểm 401, no-store, body chỉ có detail và không ghi allowed.</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>kind=invalid</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>401; no-store; không trả dữ liệu sức khỏe; không có access_logs.</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC4 · Đoán lỗi (xác thực) · test_authentication_401_and_no_store_without_health_payload__AC14[invalid] · evidence/test-history.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="107" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-18</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối phiên expired</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>1. Chuẩn bị auth theo kind của test (không in token).
+2. GET /adherence.
+3. Kiểm 401, no-store, body chỉ có detail và không ghi allowed.</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>kind=expired</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>401; no-store; không trả dữ liệu sức khỏe; không có access_logs.</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC4 · Đoán lỗi (xác thực) · test_authentication_401_and_no_store_without_health_payload__AC14[expired] · evidence/test-history.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="107" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-19</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối phiên erased</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1. Chuẩn bị auth theo kind của test (không in token).
+2. GET /adherence.
+3. Kiểm 401, no-store, body chỉ có detail và không ghi allowed.</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>kind=erased</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>401; no-store; không trả dữ liệu sức khỏe; không có access_logs.</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC4 · Đoán lỗi (xác thực) · test_authentication_401_and_no_store_without_health_payload__AC14[erased] · evidence/test-history.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="90.5" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-20</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Tính ngay xác nhận tại -30 phút</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Unit application: access Mock cho phép, reader trả một HistoryRow; chưa chứng minh PEP/DB.</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy test tại backend/tests/unit/test_get_adherence_history.py với delay0, cả group_by=date và medication.
+2. Quan sát ở đúng taken_at; kiểm summary, nhóm và một dose.</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>scheduled_at=08:00 +07; delay=-30 phút; status=da_uong</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>total=1, counted=1, rate=100.00; taken/late đúng trạng thái; đúng một liều ngay khi xác nhận.</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Cả date và medication trả total/taken/counted=0, rate=None, groups rỗng tại 07:30; 2 assertion fail. evidence/test-unit.log</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC2,AC3 · BVA (-30 phút) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay0- · evidence/test-unit.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="90.5" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-21</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Tính ngay xác nhận tại 0 phút</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Unit application: access Mock cho phép, reader trả một HistoryRow; chưa chứng minh PEP/DB.</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy test tại backend/tests/unit/test_get_adherence_history.py với delay1, cả group_by=date và medication.
+2. Quan sát ở đúng taken_at; kiểm summary, nhóm và một dose.</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>scheduled_at=08:00 +07; delay=0 phút; status=da_uong</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>total=1, counted=1, rate=100.00; taken/late đúng trạng thái; đúng một liều ngay khi xác nhận.</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>2 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC2,AC3 · BVA (0 phút) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay1- · evidence/test-unit.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="90.5" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-22</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Tính ngay xác nhận tại +30 phút</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Unit application: access Mock cho phép, reader trả một HistoryRow; chưa chứng minh PEP/DB.</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy test tại backend/tests/unit/test_get_adherence_history.py với delay2, cả group_by=date và medication.
+2. Quan sát ở đúng taken_at; kiểm summary, nhóm và một dose.</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>scheduled_at=08:00 +07; delay=+30 phút; status=da_uong</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>total=1, counted=1, rate=100.00; taken/late đúng trạng thái; đúng một liều ngay khi xác nhận.</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>2 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC2,AC3 · BVA (+30 phút) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay2- · evidence/test-unit.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="90.5" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-23</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Tính ngay xác nhận tại +30 phút +1µs</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Unit application: access Mock cho phép, reader trả một HistoryRow; chưa chứng minh PEP/DB.</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy test tại backend/tests/unit/test_get_adherence_history.py với delay3, cả group_by=date và medication.
+2. Quan sát ở đúng taken_at; kiểm summary, nhóm và một dose.</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>scheduled_at=08:00 +07; delay=+30 phút +1µs; status=uong_tre</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>total=1, counted=1, rate=100.00; taken/late đúng trạng thái; đúng một liều ngay khi xác nhận.</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>2 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC2,AC3 · BVA (+30 phút +1µs) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay3- · evidence/test-unit.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="90.5" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-24</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Tính ngay xác nhận tại +119 phút 59 giây</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Unit application: access Mock cho phép, reader trả một HistoryRow; chưa chứng minh PEP/DB.</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy test tại backend/tests/unit/test_get_adherence_history.py với delay4, cả group_by=date và medication.
+2. Quan sát ở đúng taken_at; kiểm summary, nhóm và một dose.</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>scheduled_at=08:00 +07; delay=+119 phút 59 giây; status=uong_tre</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>total=1, counted=1, rate=100.00; taken/late đúng trạng thái; đúng một liều ngay khi xác nhận.</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>2 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC2,AC3 · BVA (+119 phút 59 giây) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay4- · evidence/test-unit.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="90.5" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-25</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Tính ngay xác nhận tại +120 phút</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Unit application: access Mock cho phép, reader trả một HistoryRow; chưa chứng minh PEP/DB.</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy test tại backend/tests/unit/test_get_adherence_history.py với delay5, cả group_by=date và medication.
+2. Quan sát ở đúng taken_at; kiểm summary, nhóm và một dose.</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>scheduled_at=08:00 +07; delay=+120 phút; status=uong_tre</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>total=1, counted=1, rate=100.00; taken/late đúng trạng thái; đúng một liều ngay khi xác nhận.</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>2 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC2,AC3 · BVA (+120 phút) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay5- · evidence/test-unit.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="90.5" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-26</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Chuyển pending tại +120 thành missed ngay sau hạn</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Unit: một liều taken và một liều chưa xác nhận; thử cả status=None và bo_lo cũ.</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy backend/tests/unit/test_get_adherence_history.py::test_unconfirmed_pending_at_deadline_then_missed__AC3.
+2. So summary tại +120 và +120+1µs, hai kiểu nhóm.</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>scheduled=08:00; as_of=10:00 và 10:00:00.000001 +07</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>Tại hạn pending=1,counted=1,rate=100; sau hạn missed=1,counted=2,rate=50; không nhân đôi liều.</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>4 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC2,AC3 · BVA (max,max+1) · Chuyển trạng thái (pending → missed) · test_unconfirmed_pending_at_deadline_then_missed__AC3 · evidence/test-unit.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="90.5" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-27</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Trả tỷ lệ null khi không có mẫu số</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Unit: không có liều hoặc chỉ có pending.</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy backend/tests/unit/test_get_adherence_history.py::test_no_eligible_dose_has_null_rate__AC3.
+2. Kiểm date và medication, có/không có pending.</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>as_of=10:00 +07; counted=0</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>adherence_rate=None; trường hợp rỗng không có nhóm, pending không vào mẫu số.</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>4 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC3 · EP (3) · test_no_eligible_dose_has_null_rate__AC3 · evidence/test-unit.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="107" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-28</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Không tăng tỷ lệ khi thực uống sau hạn</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Unit: tạo DoseConfirmation tại +120+1µs.</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy backend/tests/unit/test_get_adherence_history.py::test_after_deadline_confirmation_does_not_raise_rate__AC3.
+2. So lịch sử trước và sau xác nhận, cả hai kiểu nhóm.</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>taken_at=10:00:00.000001 +07 cho lịch 08:00</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>status=bo_lo; counted=1, rate=0.00 trước và sau.</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>2 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC3 · BVA (max+1) · Chuyển trạng thái (missed không trở thành tuân thủ) · test_after_deadline_confirmation_does_not_raise_rate__AC3 · evidence/test-unit.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="90.5" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-29</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Tính xác nhận hợp lệ được đồng bộ sau hạn</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Unit: thực uống +90 nhưng sync +121 phút.</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy backend/tests/unit/test_get_adherence_history.py::test_valid_confirmation_synced_after_deadline_still_counts__AC3.
+2. Kiểm status, taken_at và tỷ lệ.</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>scheduled=08:00; taken=09:30; synced=10:01 +07</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>uong_tre; total=late=counted=1, rate=100.00; taken_at=09:30.</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>2 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC3 · Chuyển trạng thái (đồng bộ muộn) · test_valid_confirmation_synced_after_deadline_still_counts__AC3 · evidence/test-unit.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="140" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-30</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Phân nhóm và tính tỷ lệ 80% trên DB thật</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
+3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>3 taken,1 late,1 missed; hai thuốc trùng tên khác ID</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>Hai kiểu nhóm có tổng 5, counted=5,rate=80; ID thuốc không bị gộp nhầm; no-store, allowed và DB không đổi.</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr"/>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC1,AC2,AC3 · EP (1) · test_patient_history_by_date_medication_groups_and_80_percent · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="123.5" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-31</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Giữ đúng ngày Việt Nam qua nửa đêm</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
+3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Lịch và xác nhận hai phía 00:00 Asia/Ho_Chi_Minh</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>Nhóm theo ngày scheduled_at ở Việt Nam, thứ tự ngày đúng, không nhân đôi liều.</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr"/>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC2 · BVA (ngày) · test_scheduled_date_across_midnight · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="57.5" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-32</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Chấp nhận khoảng ngày 90 và chặn 91 ngày</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Unit resolve_range; không có DB.</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy tests/unit/test_adherence_history.py::test_inclusive_90_allowed_91_rejected.</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Khoảng bao gồm hai đầu dài 90 và 91 ngày</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>90 được chấp nhận; 91 bị từ chối.</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC2 · BVA (max,max+1) · test_inclusive_90_allowed_91_rejected · evidence/test-unit.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="140" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-33</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Không tạo trùng khi sync lại cùng client_uuid</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy backend/tests/integration/test_adherence_history_api.py::test_late_sync_worker_log_and_retry_keep_one_occurrence__AC15_AC20.
+2. Kiểm một occurrence, client_uuid và status sau Worker + retry.</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>taken +90; sync sau +120; cùng client_uuid hai lần</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>Một dose_log và một occurrence; giữ xác nhận hợp lệ; lịch sử phản ánh liều trễ.</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr"/>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC2,AC3 · Đoán lỗi (idempotency) · test_late_sync_worker_log_and_retry_keep_one_occurrence · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="123.5" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-34</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Giữ xác nhận khi Worker chạy đua</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy backend/tests/integration/test_adherence_history_api.py::test_worker_insert_races_with_valid_late_confirmation__AC15_AC20_AC22.
+2. Thử worker/confirmation ghi trước; kiểm một liều và trạng thái cuối.</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>first_writer=worker/confirmation; taken hợp lệ +90</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>Một occurrence/dose_log; uong_tre; không ghi đè xác nhận hợp lệ.</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr"/>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I42" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC2,AC3 · Đoán lỗi (race) · test_worker_insert_races_with_valid_late_confirmation · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="107" customHeight="1">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-35</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm biên xác nhận ngay trước −30 phút</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
+3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>scheduled=08:00; taken=07:29:59.999999 +07</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>Bị từ chối theo cửa sổ xác nhận QD-03; không tạo xác nhận hợp lệ.</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr"/>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC2,AC3 · BVA (min-1) · Pending: Chưa có ca 3.25 chạy biên này; thiếu contract 3.23 để bổ sung integration theo P5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="107" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-36</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm biên ngay trước +30 phút</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
+2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
+3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>scheduled=08:00; taken=08:29:59.999999 +07</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>da_uong; tỷ lệ có liều hợp lệ ngay khi xác nhận.</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="inlineStr"/>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I44" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC2,AC3 · BVA (+30-1) · Pending: Chưa chạy đúng mốc này trong bộ 3.25; chưa đủ điều kiện mở rộng P5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="123.5" customHeight="1">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-37</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Loại liều hủy và biểu diễn xung đột/đối soát</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>1. Đối chiếu contract 3.23 với QD-42.
+2. Khi schema hỗ trợ, tạo liều hủy/xung đột/đối soát theo fixture thật.
+3. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
+4. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Liều hủy; liều xung đột; liều đối soát</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>Loại liều hủy; nhãn tạm thời, tính lại và thời điểm/phiên bản cập nhật theo QD-42 được đặc tả và kiểm chứng.</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr"/>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I45" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC8 · Chuyển trạng thái (đối soát) · Pending: Contract thiếu /adherence và schema; dữ liệu/field đối soát chưa được đặc tả; không tạo oracle giả.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="107" customHeight="1">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-38</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tỷ lệ đúng giờ riêng theo QD-42</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>1. Đọc định nghĩa tử số/mẫu số và field trong contract 3.23.
+2. Tạo liều đúng giờ, trễ, pending và missed; GET /adherence.
+3. So tỷ lệ với công thức đã chốt.</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>1 taken,1 late,1 missed,1 pending</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>Có công thức và response biểu diễn tỷ lệ đúng giờ riêng đã được chủ sở hữu chốt.</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="inlineStr"/>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I46" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC8 · EP (2,3) · Pending: Contract hiện chưa biểu diễn tỷ lệ riêng; không suy ra công thức.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="90.5" customHeight="1">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-39</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Xóa dữ liệu phiên khi đổi bệnh nhân</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Cần màn production 3.24; family F đã mở lịch sử P.</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở app test và chọn P trong Người thân.
+2. Mở lịch sử, xác nhận có liều.
+3. Thực hiện đổi bệnh nhân.
+4. Kiểm không hiển thị dữ liệu cũ, không lưu bền, response cũ không phục hồi dữ liệu.</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>P có liều 08:00; Q không có dữ liệu của P; sự kiện=đổi bệnh nhân</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>Dữ liệu sức khỏe cũ bị xóa khỏi RAM/UI; không có cache bền; không phục hồi bởi response đến muộn.</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr"/>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I47" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC6 · Chuyển trạng thái (session) · manual · Pending: UI/controller/repository 3.24 chưa có, chỉ .gitkeep; chưa chạy app hoặc widget test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="90.5" customHeight="1">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-40</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Xóa dữ liệu phiên khi mất mạng</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Cần màn production 3.24; family F đã mở lịch sử P.</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở app test và chọn P trong Người thân.
+2. Mở lịch sử, xác nhận có liều.
+3. Thực hiện mất mạng.
+4. Kiểm không hiển thị dữ liệu cũ, không lưu bền, response cũ không phục hồi dữ liệu.</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>P có liều 08:00; Q không có dữ liệu của P; sự kiện=mất mạng</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>Dữ liệu sức khỏe cũ bị xóa khỏi RAM/UI; không có cache bền; không phục hồi bởi response đến muộn.</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="inlineStr"/>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I48" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC6 · Chuyển trạng thái (session) · manual · Pending: UI/controller/repository 3.24 chưa có, chỉ .gitkeep; chưa chạy app hoặc widget test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="90.5" customHeight="1">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-41</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Xóa dữ liệu phiên khi đưa app vào nền</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Cần màn production 3.24; family F đã mở lịch sử P.</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở app test và chọn P trong Người thân.
+2. Mở lịch sử, xác nhận có liều.
+3. Thực hiện đưa app vào nền.
+4. Kiểm không hiển thị dữ liệu cũ, không lưu bền, response cũ không phục hồi dữ liệu.</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>P có liều 08:00; Q không có dữ liệu của P; sự kiện=đưa app vào nền</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>Dữ liệu sức khỏe cũ bị xóa khỏi RAM/UI; không có cache bền; không phục hồi bởi response đến muộn.</t>
+        </is>
+      </c>
+      <c r="G49" s="8" t="inlineStr"/>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I49" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC6 · Chuyển trạng thái (session) · manual · Pending: UI/controller/repository 3.24 chưa có, chỉ .gitkeep; chưa chạy app hoặc widget test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="90.5" customHeight="1">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-42</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Xóa dữ liệu phiên khi đăng xuất</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>Cần màn production 3.24; family F đã mở lịch sử P.</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở app test và chọn P trong Người thân.
+2. Mở lịch sử, xác nhận có liều.
+3. Thực hiện đăng xuất.
+4. Kiểm không hiển thị dữ liệu cũ, không lưu bền, response cũ không phục hồi dữ liệu.</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>P có liều 08:00; Q không có dữ liệu của P; sự kiện=đăng xuất</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>Dữ liệu sức khỏe cũ bị xóa khỏi RAM/UI; không có cache bền; không phục hồi bởi response đến muộn.</t>
+        </is>
+      </c>
+      <c r="G50" s="8" t="inlineStr"/>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I50" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC6 · Chuyển trạng thái (session) · manual · Pending: UI/controller/repository 3.24 chưa có, chỉ .gitkeep; chưa chạy app hoặc widget test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="90.5" customHeight="1">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-43</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Xóa dữ liệu phiên khi nhận 403</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Cần màn production 3.24; family F đã mở lịch sử P.</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở app test và chọn P trong Người thân.
+2. Mở lịch sử, xác nhận có liều.
+3. Thực hiện nhận 403.
+4. Kiểm không hiển thị dữ liệu cũ, không lưu bền, response cũ không phục hồi dữ liệu.</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>P có liều 08:00; Q không có dữ liệu của P; sự kiện=nhận 403</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>Dữ liệu sức khỏe cũ bị xóa khỏi RAM/UI; không có cache bền; không phục hồi bởi response đến muộn.</t>
+        </is>
+      </c>
+      <c r="G51" s="8" t="inlineStr"/>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I51" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC6 · Chuyển trạng thái (session) · manual · Pending: UI/controller/repository 3.24 chưa có, chỉ .gitkeep; chưa chạy app hoặc widget test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="90.5" customHeight="1">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-44</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Chỉ xem lịch sử trên Mobile và chạy E2E thu hồi</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>UI 3.24 và Android test package riêng cùng local API/DB.</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>1. Chọn P; mở lịch sử; tìm thao tác sửa lịch/xác nhận hộ.
+2. Bệnh nhân thu hồi quyền; refresh lịch sử bằng cùng phiên.
+3. Đổi sang Q và kiểm không còn dữ liệu P.</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Family F; linked P; unlinked Q</t>
+        </is>
+      </c>
+      <c r="F52" s="8" t="inlineStr">
+        <is>
+          <t>Không có thao tác ghi hộ; request sau thu hồi 403, không còn dữ liệu cũ; DB có denied.</t>
+        </is>
+      </c>
+      <c r="G52" s="8" t="inlineStr"/>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I52" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC1,AC4,AC5,AC6 · manual/E2E · Pending: Không có màn production hoặc Flutter integration test 3.24; chưa viết/chạy runner thay màn giả.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="156.5" customHeight="1">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-45</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Truy vết PB21 và gộp test case tổng</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>Báo cáo test và workbook đã được dựng bằng script chuẩn.</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>1. Đối chiếu AC1–AC9 với test, XML và log.
+2. Chạy testcase_xlsx.py validate/build/merge 3.25.
+3. So sheet cũ và đếm trạng thái/Bug Report; đọc báo cáo để phân biệt lỗi với Pending.</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>PB21; code FADH; task 3.25</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi AC có ca; một sheet FADH; các sheet chức năng cũ giữ nguyên; Fail có bug, Pending không được báo Pass.</t>
+        </is>
+      </c>
+      <c r="G53" s="8" t="inlineStr">
+        <is>
+          <t>Đã đối chiếu AC1–AC9, log/XML phiên hiện tại, validate/build/merge exit 0. Kiểm giữ nguyên 20 sheet chức năng, đúng 45 ID và một bug FADH; các ca thiếu bằng chứng giữ Pending. evidence/testcase-verify.log; evidence/testcase-xlsx.log; 05-test-report.md. Scope cuối exit 0 sau commit riêng unit implement được người dùng cho phép; chưa kiểm native Excel.</t>
+        </is>
+      </c>
+      <c r="H53" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I53" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC9 · manual (đối chiếu artifact) · evidence/testcase-verify.log · evidence/testcase-xlsx.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56">
+      <c r="G56" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H56" s="13">
+        <f>COUNTIF(H9:H53,"Pass")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="G57" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="H57" s="13">
+        <f>COUNTIF(H9:H53,"Fail")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="G58" s="12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H58" s="13">
+        <f>COUNTIF(H9:H53,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="G59" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H59" s="13">
+        <f>SUM(H56:H58)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:I53"/>
+  <conditionalFormatting sqref="H9:H53">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pass,Fail,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -24920,7 +27552,7 @@
         <v/>
       </c>
       <c r="D3" s="11">
-        <f>'Chọn thuốc danh mục'!$H$40+'Hồi quy xác nhận liều'!$H$12+'Cảnh báo người thân'!$H$84+'FCM token Android'!$H$24+'Redeem flow E2E'!$H$34</f>
+        <f>'Chọn thuốc danh mục'!$H$40+'Hồi quy xác nhận liều'!$H$12+'Cảnh báo người thân'!$H$84+'FCM token Android'!$H$24+'Redeem flow E2E'!$H$34+'Lịch sử tuân thủ người thân'!$H$56</f>
         <v/>
       </c>
       <c r="E3" s="15">
@@ -24940,7 +27572,7 @@
         <v/>
       </c>
       <c r="D4" s="11">
-        <f>'Chọn thuốc danh mục'!$H$41+'Hồi quy xác nhận liều'!$H$13+'Cảnh báo người thân'!$H$85+'FCM token Android'!$H$25+'Redeem flow E2E'!$H$35</f>
+        <f>'Chọn thuốc danh mục'!$H$41+'Hồi quy xác nhận liều'!$H$13+'Cảnh báo người thân'!$H$85+'FCM token Android'!$H$25+'Redeem flow E2E'!$H$35+'Lịch sử tuân thủ người thân'!$H$57</f>
         <v/>
       </c>
       <c r="E4" s="15">
@@ -24980,7 +27612,7 @@
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>'Chọn thuốc danh mục'!$H$42+'Hồi quy xác nhận liều'!$H$14+'Cảnh báo người thân'!$H$86+'FCM token Android'!$H$26+'Redeem flow E2E'!$H$36</f>
+        <f>'Chọn thuốc danh mục'!$H$42+'Hồi quy xác nhận liều'!$H$14+'Cảnh báo người thân'!$H$86+'FCM token Android'!$H$26+'Redeem flow E2E'!$H$36+'Lịch sử tuân thủ người thân'!$H$58</f>
         <v/>
       </c>
       <c r="E6" s="15">
@@ -25935,746 +28567,839 @@
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="19" t="inlineStr">
+    <row r="31" ht="107" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Lịch sử tuân thủ cho người thân</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>PB21: lịch sử, quyền truy cập, thu hồi, audit, tỷ lệ và dữ liệu phiên.</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>Lịch sử tuân thủ người thân</t>
+        </is>
+      </c>
+      <c r="D31" s="18">
+        <f>IFERROR(('Lịch sử tuân thủ người thân'!$H$59-'Lịch sử tuân thủ người thân'!$H$58)/'Lịch sử tuân thủ người thân'!$H$59,0)</f>
+        <v/>
+      </c>
+      <c r="E31" s="18">
+        <f>IFERROR('Lịch sử tuân thủ người thân'!$H$56/'Lịch sử tuân thủ người thân'!$H$59,0)</f>
+        <v/>
+      </c>
+      <c r="F31" s="18">
+        <f>IFERROR('Lịch sử tuân thủ người thân'!$H$57/'Lịch sử tuân thủ người thân'!$H$59,0)</f>
+        <v/>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>BUG-3.25-01 Medium tại xác nhận sớm −30 phút. Pending contract 3.23/UI 3.24. Pass unit không chứng minh DB/API; chi tiết trong từng ca và 05-test-report.md.</t>
+        </is>
+      </c>
+      <c r="I31" s="11" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="19" t="inlineStr">
         <is>
           <t>Bug Report</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="20" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="20" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="B54" s="20" t="inlineStr">
+      <c r="B55" s="20" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C54" s="20" t="inlineStr">
+      <c r="C55" s="20" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="D54" s="20" t="inlineStr">
+      <c r="D55" s="20" t="inlineStr">
         <is>
           <t>Input Data</t>
         </is>
       </c>
-      <c r="E54" s="20" t="inlineStr">
+      <c r="E55" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F54" s="20" t="inlineStr">
+      <c r="F55" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="G54" s="20" t="inlineStr">
+      <c r="G55" s="20" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="H54" s="20" t="inlineStr">
+      <c r="H55" s="20" t="inlineStr">
         <is>
           <t>Name of Tester</t>
         </is>
       </c>
-      <c r="I54" s="20" t="inlineStr">
+      <c r="I55" s="20" t="inlineStr">
         <is>
           <t>Logs</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="123.5" customHeight="1">
-      <c r="A55" s="22" t="inlineStr">
+    <row r="56" ht="123.5" customHeight="1">
+      <c r="A56" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-08</t>
         </is>
       </c>
-      <c r="B55" s="22" t="inlineStr">
+      <c r="B56" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại có ký tự xuống dòng ở cuối</t>
         </is>
       </c>
-      <c r="C55" s="22" t="inlineStr">
+      <c r="C56" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone: "0900000001\n"}
 2. POST /auth/mobile/verify {phone: "0900000001\n", token: 123456}</t>
         </is>
       </c>
-      <c r="D55" s="22" t="inlineStr">
+      <c r="D56" s="22" t="inlineStr">
         <is>
           <t>phone: 0900000001 + ký tự \n</t>
         </is>
       </c>
-      <c r="E55" s="22" t="inlineStr">
+      <c r="E56" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"} (theo AC6 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F55" s="22" t="inlineStr">
+      <c r="F56" s="22" t="inlineStr">
         <is>
           <t>OTP 204, verify 200 và cấp phiên (backend bỏ ký tự trắng hai đầu)</t>
         </is>
       </c>
-      <c r="G55" s="22" t="inlineStr">
+      <c r="G56" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H55" s="22" t="inlineStr">
+      <c r="H56" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I55" s="22" t="inlineStr">
+      <c r="I56" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn — kỳ vọng AC6 mâu thuẫn AC5: backend `_validate_required_text` (sign_in.py:178) `strip()` mọi ký tự trắng hai đầu, nên \n cuối được xử lý như khoảng trắng hai đầu mà AC5 coi là hợp lệ. Cần người dùng chốt: sửa AC6 hoặc sửa backend
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="123.5" customHeight="1">
-      <c r="A56" s="22" t="inlineStr">
+    <row r="57" ht="123.5" customHeight="1">
+      <c r="A57" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-11</t>
         </is>
       </c>
-      <c r="B56" s="22" t="inlineStr">
+      <c r="B57" s="22" t="inlineStr">
         <is>
           <t>Gửi số điện thoại viết bằng chữ số Unicode</t>
         </is>
       </c>
-      <c r="C56" s="22" t="inlineStr">
+      <c r="C57" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/mobile/otp {phone}
 2. POST /auth/mobile/verify {phone, token: 123456}</t>
         </is>
       </c>
-      <c r="D56" s="22" t="inlineStr">
+      <c r="D57" s="22" t="inlineStr">
         <is>
           <t>+８４９０００００００１ (full-width) | +٨٤٩٠٠٠٠٠٠٠١ (chữ số Ả Rập)</t>
         </is>
       </c>
-      <c r="E56" s="22" t="inlineStr">
+      <c r="E57" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_phone"}, không gọi Supabase</t>
         </is>
       </c>
-      <c r="F56" s="22" t="inlineStr">
+      <c r="F57" s="22" t="inlineStr">
         <is>
           <t>OTP 503 {"detail":"auth_provider_unavailable"}, verify 401 {"detail":"Invalid credentials"} — request đã tới Supabase</t>
         </is>
       </c>
-      <c r="G56" s="22" t="inlineStr">
+      <c r="G57" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H56" s="22" t="inlineStr">
+      <c r="H57" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I56" s="22" t="inlineStr">
+      <c r="I57" s="22" t="inlineStr">
         <is>
           <t>`_normalize_phone` (sign_in.py:197–206) kiểm bằng `str.isdigit()`, nhận cả chữ số Unicode, nên số lọt qua kiểm tra và gửi tới Supabase. Ô nhập của app chỉ cho 0-9 nên người dùng app không gặp; lỗi ở tầng API
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="189.5" customHeight="1">
-      <c r="A57" s="22" t="inlineStr">
+    <row r="58" ht="189.5" customHeight="1">
+      <c r="A58" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-25</t>
         </is>
       </c>
-      <c r="B57" s="22" t="inlineStr">
+      <c r="B58" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên có ký tự NUL</t>
         </is>
       </c>
-      <c r="C57" s="22" t="inlineStr">
+      <c r="C58" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: "abc\u0000def", ngày sinh, giới tính hợp lệ}</t>
         </is>
       </c>
-      <c r="D57" s="22" t="inlineStr">
+      <c r="D58" s="22" t="inlineStr">
         <is>
           <t>ho_ten: abc\u0000def</t>
         </is>
       </c>
-      <c r="E57" s="22" t="inlineStr">
+      <c r="E58" s="22" t="inlineStr">
         <is>
           <t>Không 5xx (từ chối 422 hoặc lưu được); không lộ chi tiết nội bộ</t>
         </is>
       </c>
-      <c r="F57" s="22" t="inlineStr">
+      <c r="F58" s="22" t="inlineStr">
         <is>
           <t>500 Internal Server Error</t>
         </is>
       </c>
-      <c r="G57" s="22" t="inlineStr">
+      <c r="G58" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H57" s="22" t="inlineStr">
+      <c r="H58" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I57" s="22" t="inlineStr">
+      <c r="I58" s="22" t="inlineStr">
         <is>
           <t>`_validate_required_text` (sign_in.py:178) không chặn ký tự điều khiển; PostgreSQL từ chối NUL trong cột text: `psycopg.DataError: PostgreSQL text fields cannot contain NUL (0x00) bytes` ở `UPDATE users SET full_name…` (SqlUsers.update_profile); không có handler cho DataError nên thành 500. Câu SQL có tham số nên không phải lỗ hổng SQL injection
 Log: evidence/test-integration.log, evidence/test-probe-nul.log</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="90.5" customHeight="1">
-      <c r="A58" s="22" t="inlineStr">
+    <row r="59" ht="90.5" customHeight="1">
+      <c r="A59" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-30</t>
         </is>
       </c>
-      <c r="B58" s="22" t="inlineStr">
+      <c r="B59" s="22" t="inlineStr">
         <is>
           <t>Lưu họ tên dài 256 ký tự</t>
         </is>
       </c>
-      <c r="C58" s="22" t="inlineStr">
+      <c r="C59" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ho_ten: A*256}</t>
         </is>
       </c>
-      <c r="D58" s="22" t="inlineStr">
+      <c r="D59" s="22" t="inlineStr">
         <is>
           <t>A*256</t>
         </is>
       </c>
-      <c r="E58" s="22" t="inlineStr">
+      <c r="E59" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (giới hạn 255 theo Q4 của 01-requirement)</t>
         </is>
       </c>
-      <c r="F58" s="22" t="inlineStr">
+      <c r="F59" s="22" t="inlineStr">
         <is>
           <t>204, đã lưu</t>
         </is>
       </c>
-      <c r="G58" s="22" t="inlineStr">
+      <c r="G59" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H58" s="22" t="inlineStr">
+      <c r="H59" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I58" s="22" t="inlineStr">
+      <c r="I59" s="22" t="inlineStr">
         <is>
           <t>Không có giới hạn độ dài họ tên: `_validate_profile` (sign_in.py) chỉ kiểm rỗng; cột users.full_name kiểu text không giới hạn
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="90.5" customHeight="1">
-      <c r="A59" s="22" t="inlineStr">
+    <row r="60" ht="90.5" customHeight="1">
+      <c r="A60" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-32</t>
         </is>
       </c>
-      <c r="B59" s="22" t="inlineStr">
+      <c r="B60" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh trước 1900-01-01</t>
         </is>
       </c>
-      <c r="C59" s="22" t="inlineStr">
+      <c r="C60" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh}</t>
         </is>
       </c>
-      <c r="D59" s="22" t="inlineStr">
+      <c r="D60" s="22" t="inlineStr">
         <is>
           <t>1899-12-31 | 0001-01-01</t>
         </is>
       </c>
-      <c r="E59" s="22" t="inlineStr">
+      <c r="E60" s="22" t="inlineStr">
         <is>
           <t>422; hồ sơ không đổi (cận dưới 1900-01-01 theo Q4)</t>
         </is>
       </c>
-      <c r="F59" s="22" t="inlineStr">
+      <c r="F60" s="22" t="inlineStr">
         <is>
           <t>204 ở cả hai giá trị, đã lưu</t>
         </is>
       </c>
-      <c r="G59" s="22" t="inlineStr">
+      <c r="G60" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H59" s="22" t="inlineStr">
+      <c r="H60" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I59" s="22" t="inlineStr">
+      <c r="I60" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:229–231) chỉ chặn ngày tương lai, không có cận dưới. App mobile đã giới hạn date picker từ 1900 nên chỉ gặp khi gọi API trực tiếp
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="123.5" customHeight="1">
-      <c r="A60" s="22" t="inlineStr">
+    <row r="61" ht="123.5" customHeight="1">
+      <c r="A61" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-35</t>
         </is>
       </c>
-      <c r="B60" s="22" t="inlineStr">
+      <c r="B61" s="22" t="inlineStr">
         <is>
           <t>Lưu ngày sinh là hôm nay lúc 00:30 giờ Việt Nam</t>
         </is>
       </c>
-      <c r="C60" s="22" t="inlineStr">
+      <c r="C61" s="22" t="inlineStr">
         <is>
           <t>1. POST /auth/profile {ngay_sinh: "2026-10-08"}</t>
         </is>
       </c>
-      <c r="D60" s="22" t="inlineStr">
+      <c r="D61" s="22" t="inlineStr">
         <is>
           <t>ngay_sinh: 2026-10-08</t>
         </is>
       </c>
-      <c r="E60" s="22" t="inlineStr">
+      <c r="E61" s="22" t="inlineStr">
         <is>
           <t>204 (hôm nay theo giờ Asia/Ho_Chi_Minh — bất biến 7)</t>
         </is>
       </c>
-      <c r="F60" s="22" t="inlineStr">
+      <c r="F61" s="22" t="inlineStr">
         <is>
           <t>422 {"detail":"invalid_date_of_birth"}</t>
         </is>
       </c>
-      <c r="G60" s="22" t="inlineStr">
+      <c r="G61" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H60" s="22" t="inlineStr">
+      <c r="H61" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I60" s="22" t="inlineStr">
+      <c r="I61" s="22" t="inlineStr">
         <is>
           <t>`_validate_birth_date` (sign_in.py:230) so với `now.date()` trong khi `now()` (shared/clock.py) trả giờ UTC: từ 00:00 đến 07:00 giờ VN, "hôm nay" bị coi là ngày mai. Vi phạm bất biến 7 (múi giờ cố định Asia/Ho_Chi_Minh)
 Log: evidence/test-integration.log</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="173" customHeight="1">
-      <c r="A61" s="22" t="inlineStr">
+    <row r="62" ht="173" customHeight="1">
+      <c r="A62" s="22" t="inlineStr">
         <is>
           <t>BUG-LOGIN-42</t>
         </is>
       </c>
-      <c r="B61" s="22" t="inlineStr">
+      <c r="B62" s="22" t="inlineStr">
         <is>
           <t>Chạm lại ô OTP sau khi nhập sai để sửa mã</t>
         </is>
       </c>
-      <c r="C61" s="22" t="inlineStr">
+      <c r="C62" s="22" t="inlineStr">
         <is>
           <t>1. Chạm vào ô mã OTP
 2. Theo dõi request backend nhận được</t>
         </is>
       </c>
-      <c r="D61" s="22" t="inlineStr">
+      <c r="D62" s="22" t="inlineStr">
         <is>
           <t>Ô đang chứa 000000</t>
         </is>
       </c>
-      <c r="E61" s="22" t="inlineStr">
+      <c r="E62" s="22" t="inlineStr">
         <is>
           <t>Không gửi xác thực cho tới khi người dùng nhập mã mới đủ 6 số</t>
         </is>
       </c>
-      <c r="F61" s="22" t="inlineStr">
+      <c r="F62" s="22" t="inlineStr">
         <is>
           <t>Backend nhận thêm một POST /auth/mobile/verify 401 với mã cũ ngay khi chạm ô (chuỗi request: otp 204, verify 401, verify 401, verify 200)</t>
         </is>
       </c>
-      <c r="G61" s="22" t="inlineStr">
+      <c r="G62" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H61" s="22" t="inlineStr">
+      <c r="H62" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I61" s="22" t="inlineStr">
+      <c r="I62" s="22" t="inlineStr">
         <is>
           <t>`OtpPinInput._handleTextChange` (frontend/mobile/lib/features/auth/presentation/widgets/otp_pin_input.dart:66–72) chạy với mọi thông báo của controller, kể cả khi chỉ đổi vị trí con trỏ lúc chạm ô, và gọi onCompleted hễ ô đủ 6 số → gửi lại mã sai, tốn hạn mức token_verifications
 Log: evidence/test-e2e.log (mục "request backend trong pha 2"), evidence/implement-P10-run-phase2-requests.log</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="222.5" customHeight="1">
-      <c r="A62" s="22" t="inlineStr">
+    <row r="63" ht="222.5" customHeight="1">
+      <c r="A63" s="22" t="inlineStr">
         <is>
           <t>BUG-LINKCODE-28</t>
         </is>
       </c>
-      <c r="B62" s="22" t="inlineStr">
+      <c r="B63" s="22" t="inlineStr">
         <is>
           <t>Toàn bộ unit test, architecture test và ruff toàn repo pass</t>
         </is>
       </c>
-      <c r="C62" s="22" t="inlineStr">
+      <c r="C63" s="22" t="inlineStr">
         <is>
           <t>1. pytest tests/unit tests/architecture -q
 2. ruff check .
 3. So với baseline trước khi sửa code</t>
         </is>
       </c>
-      <c r="D62" s="22" t="inlineStr">
+      <c r="D63" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E62" s="22" t="inlineStr">
+      <c r="E63" s="22" t="inlineStr">
         <is>
           <t>pytest và ruff đều pass</t>
         </is>
       </c>
-      <c r="F62" s="22" t="inlineStr">
+      <c r="F63" s="22" t="inlineStr">
         <is>
           <t>pytest tests/unit tests/architecture: 885 passed, 18 failed (test_contract_profile.py ×12, test_profile_http.py ×6); ruff check . 19 lỗi ở module khác. Cùng danh sách với baseline trước khi 3.13 sửa code; file của task pass ruff. Lỗi test_app.py của lần chạy 3.10 không còn</t>
         </is>
       </c>
-      <c r="G62" s="22" t="inlineStr">
+      <c r="G63" s="22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H62" s="22" t="inlineStr">
+      <c r="H63" s="22" t="inlineStr">
         <is>
           <t>zannguyen</t>
         </is>
       </c>
-      <c r="I62" s="22" t="inlineStr">
+      <c r="I63" s="22" t="inlineStr">
         <is>
           <t>Có sẵn trên main, không do 3.10/3.13. Nghi vấn: 18 test profile fail vì api_contract (aea2b26) chưa có các endpoint /profile mà backend đã có (remote có nhánh fix/adhoc-20261015-api-contract-sync); 19 lỗi ruff ở catalog/*, runtime/*, worker.py, tests/unit/test_catalog_crud.py
 Log: evidence/test-unit-2.log, evidence/implement-final-backend-2.log</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="239" customHeight="1">
-      <c r="A63" s="22" t="inlineStr">
+    <row r="64" ht="239" customHeight="1">
+      <c r="A64" s="22" t="inlineStr">
         <is>
           <t>BUG-REGDOSE-01</t>
         </is>
       </c>
-      <c r="B63" s="22" t="inlineStr">
+      <c r="B64" s="22" t="inlineStr">
         <is>
           <t>Đối chiếu scheduled_at có giây khi xác nhận liều</t>
         </is>
       </c>
-      <c r="C63" s="22" t="inlineStr">
+      <c r="C64" s="22" t="inlineStr">
         <is>
           <t>1. Từ backend chạy .venv/Scripts/python.exe -m pytest tests/integration/test_dose_confirmation_api.py::test_post_doses_batch_creates_dose_log_for_authenticated_patient__AC1_AC10_AC18 -q -ra.
 2. Fixture POST /doses/batch với danh sách một item ở Test Data.
 3. Đối chiếu items[0].scheduled_at với kỳ vọng test hiện có.</t>
         </is>
       </c>
-      <c r="D63" s="22" t="inlineStr">
+      <c r="D64" s="22" t="inlineStr">
         <is>
           <t>client_uuid: UUID mới; schedule_id: fixture; scheduled_at=2026-10-02T01:00:59.999Z; taken_at=2026-10-02T01:05:59.999Z</t>
         </is>
       </c>
-      <c r="E63" s="22" t="inlineStr">
+      <c r="E64" s="22" t="inlineStr">
         <is>
           <t>Theo test hiện có: HTTP 200, synced, da_uong và scheduled_at=2026-10-02T01:00:00Z.</t>
         </is>
       </c>
-      <c r="F63" s="22" t="inlineStr">
+      <c r="F64" s="22" t="inlineStr">
         <is>
           <t>HTTP 200, synced, da_uong; scheduled_at=2026-10-02T01:00:59.999000Z. Fail trong suite DB và lặp lại khi chạy riêng (1 failed trong 1.67s).</t>
         </is>
       </c>
-      <c r="G63" s="22" t="inlineStr">
+      <c r="G64" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H63" s="22" t="inlineStr">
+      <c r="H64" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I63" s="22" t="inlineStr">
+      <c r="I64" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn kỳ vọng chuẩn hóa tới phút trong test không khớp hành vi giữ thời điểm của API; chưa xác định phía nào sai theo contract/nghiệp vụ. Chưa chứng minh mất/trùng bản ghi liều; mức Medium tạm thời cho sai khác test, phải nâng tối thiểu High nếu xác nhận mất/trùng liều.
 Log: evidence/test-integration-db.log; evidence/test-dose-mismatch-repeat.log</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="156.5" customHeight="1">
-      <c r="A64" s="22" t="inlineStr">
+    <row r="65" ht="156.5" customHeight="1">
+      <c r="A65" s="22" t="inlineStr">
         <is>
           <t>BUG-FALERT-19</t>
         </is>
       </c>
-      <c r="B64" s="22" t="inlineStr">
+      <c r="B65" s="22" t="inlineStr">
         <is>
           <t>Lọc hộp thư mixed patient và từ chối patient_id trong PATCH</t>
         </is>
       </c>
-      <c r="C64" s="22" t="inlineStr">
+      <c r="C65" s="22" t="inlineStr">
         <is>
           <t>1. Tạo hai notification cho F: P được phép và Q không có liên kết.
 2. GET /notifications?patient_id=P&amp;user_id=Q; kiểm item và count.
 3. PATCH notification Q với JSON {is_read:true,patient_id:P}.</t>
         </is>
       </c>
-      <c r="D64" s="22" t="inlineStr">
+      <c r="D65" s="22" t="inlineStr">
         <is>
           <t>P/F là UUID synthetic mới mỗi lần; ID notification lấy từ DB fixture; giờ 2026-10-20T01:00:00Z.</t>
         </is>
       </c>
-      <c r="E64" s="22" t="inlineStr">
+      <c r="E65" s="22" t="inlineStr">
         <is>
           <t>List chỉ trả P, total=unread_count=1 và Q có denied; PATCH field lạ phải trả 422.</t>
         </is>
       </c>
-      <c r="F64" s="22" t="inlineStr">
+      <c r="F65" s="22" t="inlineStr">
         <is>
           <t>HTTP 503 notification_access_unavailable thay vì 422; assertion fail.</t>
         </is>
       </c>
-      <c r="G64" s="22" t="inlineStr">
+      <c r="G65" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H64" s="22" t="inlineStr">
+      <c r="H65" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I64" s="22" t="inlineStr">
+      <c r="I65" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn đã đối chiếu code: get_notification_uow bắt RequestValidationError trong except Exception và đổi thành ServiceUnavailable; NotificationRoute trả 503. Cùng một lỗi gốc ở 4 biến thể.
 Log: evidence/test-task-integration-final.log</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="123.5" customHeight="1">
-      <c r="A65" s="22" t="inlineStr">
+    <row r="66" ht="123.5" customHeight="1">
+      <c r="A66" s="22" t="inlineStr">
         <is>
           <t>BUG-FALERT-36</t>
         </is>
       </c>
-      <c r="B65" s="22" t="inlineStr">
+      <c r="B66" s="22" t="inlineStr">
         <is>
           <t>Từ chối tham số phân trang ngoài biên [params0]</t>
         </is>
       </c>
-      <c r="C65" s="22" t="inlineStr">
+      <c r="C66" s="22" t="inlineStr">
         <is>
           <t>1. Đăng nhập F có notification và quyền hợp lệ.
 2. GET /notifications với limit=0, limit=101 hoặc offset=-1 theo Test Data.
 3. Kiểm HTTP status và Cache-Control.</t>
         </is>
       </c>
-      <c r="D65" s="22" t="inlineStr">
+      <c r="D66" s="22" t="inlineStr">
         <is>
           <t>limit=0; offset=0</t>
         </is>
       </c>
-      <c r="E65" s="22" t="inlineStr">
+      <c r="E66" s="22" t="inlineStr">
         <is>
           <t>422 validation, Cache-Control:no-store; không trả dữ liệu notification.</t>
         </is>
       </c>
-      <c r="F65" s="22" t="inlineStr">
+      <c r="F66" s="22" t="inlineStr">
         <is>
           <t>HTTP 503 notification_access_unavailable thay vì 422; assertion fail.</t>
         </is>
       </c>
-      <c r="G65" s="22" t="inlineStr">
+      <c r="G66" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H65" s="22" t="inlineStr">
+      <c r="H66" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I65" s="22" t="inlineStr">
+      <c r="I66" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn đã đối chiếu code: get_notification_uow bắt RequestValidationError trong except Exception và đổi thành ServiceUnavailable; NotificationRoute trả 503. Cùng một lỗi gốc ở 4 biến thể.
 Log: evidence/test-task-integration-final.log</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="123.5" customHeight="1">
-      <c r="A66" s="22" t="inlineStr">
+    <row r="67" ht="123.5" customHeight="1">
+      <c r="A67" s="22" t="inlineStr">
         <is>
           <t>BUG-FALERT-37</t>
         </is>
       </c>
-      <c r="B66" s="22" t="inlineStr">
+      <c r="B67" s="22" t="inlineStr">
         <is>
           <t>Từ chối tham số phân trang ngoài biên [params1]</t>
         </is>
       </c>
-      <c r="C66" s="22" t="inlineStr">
+      <c r="C67" s="22" t="inlineStr">
         <is>
           <t>1. Đăng nhập F có notification và quyền hợp lệ.
 2. GET /notifications với limit=0, limit=101 hoặc offset=-1 theo Test Data.
 3. Kiểm HTTP status và Cache-Control.</t>
         </is>
       </c>
-      <c r="D66" s="22" t="inlineStr">
+      <c r="D67" s="22" t="inlineStr">
         <is>
           <t>limit=101; offset=0</t>
         </is>
       </c>
-      <c r="E66" s="22" t="inlineStr">
+      <c r="E67" s="22" t="inlineStr">
         <is>
           <t>422 validation, Cache-Control:no-store; không trả dữ liệu notification.</t>
         </is>
       </c>
-      <c r="F66" s="22" t="inlineStr">
+      <c r="F67" s="22" t="inlineStr">
         <is>
           <t>HTTP 503 notification_access_unavailable thay vì 422; assertion fail.</t>
         </is>
       </c>
-      <c r="G66" s="22" t="inlineStr">
+      <c r="G67" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H66" s="22" t="inlineStr">
+      <c r="H67" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I66" s="22" t="inlineStr">
+      <c r="I67" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn đã đối chiếu code: get_notification_uow bắt RequestValidationError trong except Exception và đổi thành ServiceUnavailable; NotificationRoute trả 503. Cùng một lỗi gốc ở 4 biến thể.
 Log: evidence/test-task-integration-final.log</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="123.5" customHeight="1">
-      <c r="A67" s="22" t="inlineStr">
+    <row r="68" ht="123.5" customHeight="1">
+      <c r="A68" s="22" t="inlineStr">
         <is>
           <t>BUG-FALERT-38</t>
         </is>
       </c>
-      <c r="B67" s="22" t="inlineStr">
+      <c r="B68" s="22" t="inlineStr">
         <is>
           <t>Từ chối tham số phân trang ngoài biên [params2]</t>
         </is>
       </c>
-      <c r="C67" s="22" t="inlineStr">
+      <c r="C68" s="22" t="inlineStr">
         <is>
           <t>1. Đăng nhập F có notification và quyền hợp lệ.
 2. GET /notifications với limit=0, limit=101 hoặc offset=-1 theo Test Data.
 3. Kiểm HTTP status và Cache-Control.</t>
         </is>
       </c>
-      <c r="D67" s="22" t="inlineStr">
+      <c r="D68" s="22" t="inlineStr">
         <is>
           <t>limit=20; offset=-1</t>
         </is>
       </c>
-      <c r="E67" s="22" t="inlineStr">
+      <c r="E68" s="22" t="inlineStr">
         <is>
           <t>422 validation, Cache-Control:no-store; không trả dữ liệu notification.</t>
         </is>
       </c>
-      <c r="F67" s="22" t="inlineStr">
+      <c r="F68" s="22" t="inlineStr">
         <is>
           <t>HTTP 503 notification_access_unavailable thay vì 422; assertion fail.</t>
         </is>
       </c>
-      <c r="G67" s="22" t="inlineStr">
+      <c r="G68" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H67" s="22" t="inlineStr">
+      <c r="H68" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I67" s="22" t="inlineStr">
+      <c r="I68" s="22" t="inlineStr">
         <is>
           <t>Nghi vấn đã đối chiếu code: get_notification_uow bắt RequestValidationError trong except Exception và đổi thành ServiceUnavailable; NotificationRoute trả 503. Cùng một lỗi gốc ở 4 biến thể.
 Log: evidence/test-task-integration-final.log</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="140" customHeight="1">
-      <c r="A68" s="22" t="inlineStr">
+    <row r="69" ht="140" customHeight="1">
+      <c r="A69" s="22" t="inlineStr">
         <is>
           <t>BUG-REDEEMFLOW-02</t>
         </is>
       </c>
-      <c r="B68" s="22" t="inlineStr">
+      <c r="B69" s="22" t="inlineStr">
         <is>
           <t>Quét QR hợp lệ và chờ xác nhận trước khi gửi</t>
         </is>
       </c>
-      <c r="C68" s="22" t="inlineStr">
+      <c r="C69" s="22" t="inlineStr">
         <is>
           <t>1. Cấp qr_payload cho scanner callback.
 2. Kiểm số POST trước khi bấm xác nhận.
 3. Bấm xác nhận và kiểm pending.</t>
         </is>
       </c>
-      <c r="D68" s="22" t="inlineStr">
+      <c r="D69" s="22" t="inlineStr">
         <is>
           <t>qr_payload=body.qr_payload của GET /family/link-code</t>
         </is>
       </c>
-      <c r="E68" s="22" t="inlineStr">
+      <c r="E69" s="22" t="inlineStr">
         <is>
           <t>Mã được điền; 0 POST trước xác nhận; sau xác nhận một POST 201 và một pending.</t>
         </is>
       </c>
-      <c r="F68" s="22" t="inlineStr">
+      <c r="F69" s="22" t="inlineStr">
         <is>
           <t>Widget và Android LM_G710: 1 POST trước xác nhận (Expected 0, Actual 1); evidence/test-widget-redeem.log và evidence/test-android-remaining-phases.log.</t>
         </is>
       </c>
-      <c r="G68" s="22" t="inlineStr">
+      <c r="G69" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H68" s="22" t="inlineStr">
+      <c r="H69" s="22" t="inlineStr">
         <is>
           <t>phucnguyenngoc</t>
         </is>
       </c>
-      <c r="I68" s="22" t="inlineStr">
+      <c r="I69" s="22" t="inlineStr">
         <is>
           <t>scan_link_qr_screen.dart đặt autoSubmit=true, enter_link_code_screen.dart tự submit sau frame đầu.
 Log: evidence/test-widget-redeem.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="140" customHeight="1">
+      <c r="A70" s="22" t="inlineStr">
+        <is>
+          <t>BUG-FADH-20</t>
+        </is>
+      </c>
+      <c r="B70" s="22" t="inlineStr">
+        <is>
+          <t>Tính ngay xác nhận tại -30 phút</t>
+        </is>
+      </c>
+      <c r="C70" s="22" t="inlineStr">
+        <is>
+          <t>1. Chạy test tại backend/tests/unit/test_get_adherence_history.py với delay0, cả group_by=date và medication.
+2. Quan sát ở đúng taken_at; kiểm summary, nhóm và một dose.</t>
+        </is>
+      </c>
+      <c r="D70" s="22" t="inlineStr">
+        <is>
+          <t>scheduled_at=08:00 +07; delay=-30 phút; status=da_uong</t>
+        </is>
+      </c>
+      <c r="E70" s="22" t="inlineStr">
+        <is>
+          <t>total=1, counted=1, rate=100.00; taken/late đúng trạng thái; đúng một liều ngay khi xác nhận.</t>
+        </is>
+      </c>
+      <c r="F70" s="22" t="inlineStr">
+        <is>
+          <t>Cả date và medication trả total/taken/counted=0, rate=None, groups rỗng tại 07:30; 2 assertion fail. evidence/test-unit.log</t>
+        </is>
+      </c>
+      <c r="G70" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H70" s="22" t="inlineStr">
+        <is>
+          <t>phucnguyenngoc</t>
+        </is>
+      </c>
+      <c r="I70" s="22" t="inlineStr">
+        <is>
+          <t>BUG-3.25-01: build_history lọc scheduled_at &lt;= as_of nên loại xác nhận sớm hợp lệ; SQL reader cũng có cùng bộ lọc. Chưa chứng minh DB/API cho ca này.
+Log: evidence/test-unit.log</t>
         </is>
       </c>
     </row>
@@ -26683,17 +29408,17 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:A5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11:F30">
+  <conditionalFormatting sqref="F11:F31">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11:G30">
+  <conditionalFormatting sqref="G11:G31">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>OR(G11="Critical",G11="High")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G55:G68">
+  <conditionalFormatting sqref="G56:G70">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"Critical"</formula>
     </cfRule>
@@ -26705,10 +29430,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G11:G30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G11:G31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="G55:G68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G56:G70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
test(adherence): record family history retest evidence
Refs: 3.25
</commit_message>
<xml_diff>
--- a/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
+++ b/Team1_DTU/04_Quality_&_Testing/Test_Cases.xlsx
@@ -50,7 +50,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Cảnh báo người thân'!$A$8:$I$81</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'FCM token Android'!$A$8:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Redeem flow E2E'!$A$8:$I$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Lịch sử tuân thủ người thân'!$A$8:$I$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Lịch sử tuân thủ người thân'!$A$8:$I$61</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -24868,7 +24868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V59"/>
+  <dimension ref="A1:V67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -25069,7 +25069,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="123.5" customHeight="1">
+    <row r="9" ht="156.5" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-01</t>
@@ -25102,15 +25102,19 @@
           <t>200; payload đúng contract, hai response giống nhau; mỗi caller có allowed; audit không chứa nội dung thuốc/liều.</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr"/>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
+        </is>
+      </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC1,AC9 · Decision Table (R1) · EP (1) · test_self_and_family_success_are_audited · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
+          <t>PB21 · AC1,AC9 · Decision Table (R1) · EP (1) · test_self_and_family_success_are_audited · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr">
@@ -25175,7 +25179,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="123.5" customHeight="1">
+    <row r="10" ht="156.5" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-02</t>
@@ -25188,285 +25192,286 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực. F tồn tại, không có caregiver_link với P</t>
+          <t>Supabase local; patient P tồn tại, có health_data và liều; family F là user khác, không có caregiver_link tới P. Không dựng liên kết active trong ca này.</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Dựng P và liều bằng history_data; tạo F bằng make.user(), không gọi family_of/link.
+2. GET /adherence?patient_id=P bằng bearer mobile của F.
+3. Kiểm 403 {detail: khong_co_quyen}, Cache-Control: no-store; không có lịch sử trong body.
+4. Đọc access_logs của P: actor F, result denied; so dose_logs trước/sau không đổi.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>case=unlinked; patient_id=P</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>403 {detail: khong_co_quyen}; Cache-Control: no-store; có denied và dose_logs không đổi.</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC4 · Decision Table (R2) · EP (4) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11[unlinked] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>Mẫu số tỷ lệ</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>Liều xác nhận hợp lệ hoặc chưa xác nhận đã quá +120
+Không có liều đủ điều kiện</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>2
+3</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr"/>
+      <c r="O10" s="10" t="inlineStr"/>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>health_data</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="156.5" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-03</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Chặn khi thiếu consent sức khỏe</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực. Thu hồi health_data của P</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
 2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
 3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>case=unlinked; patient_id=P</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>case=health_consent; patient_id=P</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>403 {detail: khong_co_quyen}; Cache-Control: no-store; có denied và dose_logs không đổi.</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
-        </is>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>PB21 · AC4 · Decision Table (R2) · EP (4) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11[unlinked] · evidence/test-history.log</t>
-        </is>
-      </c>
-      <c r="K10" s="9" t="inlineStr">
-        <is>
-          <t>Mẫu số tỷ lệ</t>
-        </is>
-      </c>
-      <c r="L10" s="10" t="inlineStr">
-        <is>
-          <t>Liều xác nhận hợp lệ hoặc chưa xác nhận đã quá +120
-Không có liều đủ điều kiện</t>
-        </is>
-      </c>
-      <c r="M10" s="10" t="inlineStr">
-        <is>
-          <t>2
-3</t>
-        </is>
-      </c>
-      <c r="N10" s="10" t="inlineStr"/>
-      <c r="O10" s="10" t="inlineStr"/>
-      <c r="Q10" s="10" t="inlineStr">
-        <is>
-          <t>health_data</t>
-        </is>
-      </c>
-      <c r="R10" s="11" t="inlineStr">
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC4 · Decision Table (R3) · EP (5) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11[health_consent] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>family_sharing</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="S10" s="11" t="inlineStr">
+      <c r="S11" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="T10" s="11" t="inlineStr">
+      <c r="T11" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U11" s="11" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="U10" s="11" t="inlineStr">
+      <c r="V11" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="V10" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="123.5" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>TC-FADH-03</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Chặn khi thiếu consent sức khỏe</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực. Thu hồi health_data của P</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
+    </row>
+    <row r="12" ht="156.5" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-04</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Chặn khi thiếu consent chia sẻ</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực. Thu hồi family_sharing của P</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
 2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
 3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>case=health_consent; patient_id=P</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>case=family_consent; patient_id=P</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>403 {detail: khong_co_quyen}; Cache-Control: no-store; có denied và dose_logs không đổi.</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>PB21 · AC4 · Decision Table (R3) · EP (5) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11[health_consent] · evidence/test-history.log</t>
-        </is>
-      </c>
-      <c r="Q11" s="10" t="inlineStr">
-        <is>
-          <t>family_sharing</t>
-        </is>
-      </c>
-      <c r="R11" s="11" t="inlineStr">
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC4 · Decision Table (R4) · EP (6) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11[family_consent] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
+        <is>
+          <t>sharing_enabled</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="S11" s="11" t="inlineStr">
+      <c r="S12" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="T11" s="11" t="inlineStr">
+      <c r="T12" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U11" s="11" t="inlineStr">
+      <c r="U12" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V12" s="11" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="V11" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="123.5" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>TC-FADH-04</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Chặn khi thiếu consent chia sẻ</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực. Thu hồi family_sharing của P</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
+    </row>
+    <row r="13" ht="156.5" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Chặn khi bệnh nhân tắt chia sẻ</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực. Đặt sharing_enabled=false</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
 2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
 3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>case=family_consent; patient_id=P</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>case=sharing_off; patient_id=P</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>403 {detail: khong_co_quyen}; Cache-Control: no-store; có denied và dose_logs không đổi.</t>
         </is>
       </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
-        </is>
-      </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>PB21 · AC4 · Decision Table (R4) · EP (6) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11[family_consent] · evidence/test-history.log</t>
-        </is>
-      </c>
-      <c r="Q12" s="10" t="inlineStr">
-        <is>
-          <t>sharing_enabled</t>
-        </is>
-      </c>
-      <c r="R12" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="S12" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="T12" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U12" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="V12" s="11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="123.5" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>TC-FADH-05</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Chặn khi bệnh nhân tắt chia sẻ</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực. Đặt sharing_enabled=false</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
-2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
-3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>case=sharing_off; patient_id=P</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>403 {detail: khong_co_quyen}; Cache-Control: no-store; có denied và dose_logs không đổi.</t>
-        </is>
-      </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
@@ -25476,7 +25481,7 @@
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC4 · Decision Table (R5) · EP (7) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11[sharing_off] · evidence/test-history.log</t>
+          <t>PB21 · AC4 · Decision Table (R5) · EP (7) · test_unlinked_missing_consents_sharing_off_admin_denied_and_audited__AC11[sharing_off] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
         </is>
       </c>
       <c r="Q13" s="6" t="inlineStr">
@@ -25510,7 +25515,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="123.5" customHeight="1">
+    <row r="14" ht="189.5" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-06</t>
@@ -25528,9 +25533,10 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
-2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
-3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
+          <t>1. Dựng P có liều; family F liên kết active, sharing bật và hai consent của P còn hiệu lực; tạo patient Q không liên kết với F.
+2. GET /adherence?patient_id=P bằng token F, kiểm 200 và allowed của P theo contract chuẩn.
+3. Giữ nguyên token F, sửa query thành patient_id=Q rồi GET /adherence.
+4. Kiểm request Q trả 403 {detail: khong_co_quyen}, không có dữ liệu P/Q; access_logs Q có denied actor F; P chỉ có allowed từ request đầu.</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -25543,15 +25549,19 @@
           <t>403; denied cho Q; không trả dữ liệu Q; request P trước đó có allowed.</t>
         </is>
       </c>
-      <c r="G14" s="8" t="inlineStr"/>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
+        </is>
+      </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC4 · EP (4) · kiểm truy cập chéo · test_family_patient_selector_tamper · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
+          <t>PB21 · AC4 · EP (4) · kiểm truy cập chéo · test_family_patient_selector_tamper · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
         </is>
       </c>
       <c r="Q14" s="10" t="inlineStr">
@@ -25603,15 +25613,19 @@
           <t>Request đầu 200, request kế tiếp 403 {detail: khong_co_quyen}; audit lần lượt allowed, denied.</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr"/>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
+        </is>
+      </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC5 · Chuyển trạng thái (allowed → denied) · test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12[health_consent] · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
+          <t>PB21 · AC5 · Chuyển trạng thái (allowed → denied) · test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12[health_consent] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
         </is>
       </c>
       <c r="Q15" s="10" t="inlineStr">
@@ -25675,15 +25689,19 @@
           <t>Request đầu 200, request kế tiếp 403 {detail: khong_co_quyen}; audit lần lượt allowed, denied.</t>
         </is>
       </c>
-      <c r="G16" s="8" t="inlineStr"/>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
+        </is>
+      </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC5 · Chuyển trạng thái (allowed → denied) · test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12[family_consent] · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
+          <t>PB21 · AC5 · Chuyển trạng thái (allowed → denied) · test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12[family_consent] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
         </is>
       </c>
     </row>
@@ -25721,15 +25739,19 @@
           <t>Request đầu 200, request kế tiếp 403 {detail: khong_co_quyen}; audit lần lượt allowed, denied.</t>
         </is>
       </c>
-      <c r="G17" s="8" t="inlineStr"/>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
+        </is>
+      </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC5 · Chuyển trạng thái (allowed → denied) · test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12[sharing_off] · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
+          <t>PB21 · AC5 · Chuyển trạng thái (allowed → denied) · test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12[sharing_off] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
         </is>
       </c>
     </row>
@@ -25767,19 +25789,23 @@
           <t>Request đầu 200, request kế tiếp 403 {detail: khong_co_quyen}; audit lần lượt allowed, denied.</t>
         </is>
       </c>
-      <c r="G18" s="8" t="inlineStr"/>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
+        </is>
+      </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC5 · Chuyển trạng thái (allowed → denied) · test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12[unlink] · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="107" customHeight="1">
+          <t>PB21 · AC5 · Chuyển trạng thái (allowed → denied) · test_revoke_sharing_off_unlink_denies_immediate_next_request_same_token__AC12[unlink] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="156.5" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-11</t>
@@ -25814,7 +25840,7 @@
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
@@ -25824,11 +25850,11 @@
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC7 · Đoán lỗi (fail-closed) · test_audit_permission_and_commit_failure_fail_closed_without_health__AC13[allowed_insert] · evidence/test-history.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="107" customHeight="1">
+          <t>PB21 · AC7 · Đoán lỗi (fail-closed) · test_audit_permission_and_commit_failure_fail_closed_without_health__AC13[allowed_insert] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="156.5" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-12</t>
@@ -25863,7 +25889,7 @@
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
@@ -25873,11 +25899,11 @@
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC7 · Đoán lỗi (fail-closed) · test_audit_permission_and_commit_failure_fail_closed_without_health__AC13[commit] · evidence/test-history.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="107" customHeight="1">
+          <t>PB21 · AC7 · Đoán lỗi (fail-closed) · test_audit_permission_and_commit_failure_fail_closed_without_health__AC13[commit] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="156.5" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-13</t>
@@ -25912,7 +25938,7 @@
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
@@ -25922,11 +25948,11 @@
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC7 · Đoán lỗi (fail-closed) · test_audit_permission_and_commit_failure_fail_closed_without_health__AC13[denied_insert] · evidence/test-history.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="107" customHeight="1">
+          <t>PB21 · AC7 · Đoán lỗi (fail-closed) · test_audit_permission_and_commit_failure_fail_closed_without_health__AC13[denied_insert] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="156.5" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-14</t>
@@ -25961,7 +25987,7 @@
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
@@ -25971,11 +25997,11 @@
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC7 · Đoán lỗi (fail-closed) · test_audit_permission_and_commit_failure_fail_closed_without_health__AC13[permission_read] · evidence/test-history.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="123.5" customHeight="1">
+          <t>PB21 · AC7 · Đoán lỗi (fail-closed) · test_audit_permission_and_commit_failure_fail_closed_without_health__AC13[permission_read] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="156.5" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-15</t>
@@ -26010,7 +26036,7 @@
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
@@ -26020,11 +26046,11 @@
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC7 · Đoán lỗi (rollback) · test_denied_audit_survives_outer_transaction_rollback · evidence/test-history.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="107" customHeight="1">
+          <t>PB21 · AC7 · Đoán lỗi (rollback) · test_denied_audit_survives_outer_transaction_rollback · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="156.5" customHeight="1">
       <c r="A24" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-16</t>
@@ -26059,7 +26085,7 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
@@ -26069,11 +26095,11 @@
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC4 · Đoán lỗi (xác thực) · test_authentication_401_and_no_store_without_health_payload__AC14[missing] · evidence/test-history.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="107" customHeight="1">
+          <t>PB21 · AC4 · Đoán lỗi (xác thực) · test_authentication_401_and_no_store_without_health_payload__AC14[missing] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="156.5" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-17</t>
@@ -26108,7 +26134,7 @@
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
@@ -26118,11 +26144,11 @@
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC4 · Đoán lỗi (xác thực) · test_authentication_401_and_no_store_without_health_payload__AC14[invalid] · evidence/test-history.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="107" customHeight="1">
+          <t>PB21 · AC4 · Đoán lỗi (xác thực) · test_authentication_401_and_no_store_without_health_payload__AC14[invalid] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="156.5" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-18</t>
@@ -26157,7 +26183,7 @@
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
@@ -26167,11 +26193,11 @@
       </c>
       <c r="I26" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC4 · Đoán lỗi (xác thực) · test_authentication_401_and_no_store_without_health_payload__AC14[expired] · evidence/test-history.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="107" customHeight="1">
+          <t>PB21 · AC4 · Đoán lỗi (xác thực) · test_authentication_401_and_no_store_without_health_payload__AC14[expired] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="156.5" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-19</t>
@@ -26206,7 +26232,7 @@
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-history.log.</t>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
@@ -26216,11 +26242,11 @@
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC4 · Đoán lỗi (xác thực) · test_authentication_401_and_no_store_without_health_payload__AC14[erased] · evidence/test-history.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="90.5" customHeight="1">
+          <t>PB21 · AC4 · Đoán lỗi (xác thực) · test_authentication_401_and_no_store_without_health_payload__AC14[erased] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="173" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-20</t>
@@ -26254,7 +26280,7 @@
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>Cả date và medication trả total/taken/counted=0, rate=None, groups rỗng tại 07:30; 2 assertion fail. evidence/test-unit.log</t>
+          <t>Hai ca unit và hai ca family API/DB (date/medication) Fail: xác nhận -30 được nhận, dose_log tồn tại và audit allowed nhưng lịch sử total/taken/counted=0, rate=null thay vì 1/100. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
@@ -26264,7 +26290,7 @@
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC2,AC3 · BVA (-30 phút) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay0- · evidence/test-unit.log</t>
+          <t>PB21 · AC2,AC3 · BVA (-30 phút) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay0- · evidence/test-contract-unit.log/xml · test_family_early_confirmation_counts_immediately__AC3 · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
         </is>
       </c>
     </row>
@@ -26302,7 +26328,7 @@
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>2 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+          <t>2 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. Unit; chưa thay bằng chứng API/DB.</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
@@ -26312,7 +26338,7 @@
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC2,AC3 · BVA (0 phút) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay1- · evidence/test-unit.log</t>
+          <t>PB21 · AC2,AC3 · BVA (0 phút) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay1- · evidence/test-contract-unit.log/xml</t>
         </is>
       </c>
     </row>
@@ -26350,7 +26376,7 @@
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>2 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+          <t>2 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. Unit; chưa thay bằng chứng API/DB.</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
@@ -26360,7 +26386,7 @@
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC2,AC3 · BVA (+30 phút) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay2- · evidence/test-unit.log</t>
+          <t>PB21 · AC2,AC3 · BVA (+30 phút) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay2- · evidence/test-contract-unit.log/xml</t>
         </is>
       </c>
     </row>
@@ -26398,7 +26424,7 @@
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>2 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+          <t>2 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. Unit; chưa thay bằng chứng API/DB.</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
@@ -26408,7 +26434,7 @@
       </c>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC2,AC3 · BVA (+30 phút +1µs) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay3- · evidence/test-unit.log</t>
+          <t>PB21 · AC2,AC3 · BVA (+30 phút +1µs) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay3- · evidence/test-contract-unit.log/xml</t>
         </is>
       </c>
     </row>
@@ -26446,7 +26472,7 @@
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>2 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+          <t>2 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. Unit; chưa thay bằng chứng API/DB.</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
@@ -26456,7 +26482,7 @@
       </c>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC2,AC3 · BVA (+119 phút 59 giây) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay4- · evidence/test-unit.log</t>
+          <t>PB21 · AC2,AC3 · BVA (+119 phút 59 giây) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay4- · evidence/test-contract-unit.log/xml</t>
         </is>
       </c>
     </row>
@@ -26494,7 +26520,7 @@
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>2 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+          <t>2 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. Unit; chưa thay bằng chứng API/DB.</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
@@ -26504,11 +26530,11 @@
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC2,AC3 · BVA (+120 phút) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay5- · evidence/test-unit.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="90.5" customHeight="1">
+          <t>PB21 · AC2,AC3 · BVA (+120 phút) · EP (2) · test_confirmed_before_deadline_counts_immediately__AC3[delay5- · evidence/test-contract-unit.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="107" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-26</t>
@@ -26542,7 +26568,7 @@
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>4 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+          <t>4 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. Unit; chưa thay bằng chứng API/DB.</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
@@ -26552,7 +26578,7 @@
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC2,AC3 · BVA (max,max+1) · Chuyển trạng thái (pending → missed) · test_unconfirmed_pending_at_deadline_then_missed__AC3 · evidence/test-unit.log</t>
+          <t>PB21 · AC2,AC3 · BVA (max,max+1) · Chuyển trạng thái (pending → missed) · test_unconfirmed_pending_at_deadline_then_missed__AC3 · evidence/test-contract-unit.log/xml</t>
         </is>
       </c>
     </row>
@@ -26590,7 +26616,7 @@
       </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
-          <t>4 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+          <t>4 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. Unit; chưa thay bằng chứng API/DB.</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
@@ -26600,7 +26626,7 @@
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC3 · EP (3) · test_no_eligible_dose_has_null_rate__AC3 · evidence/test-unit.log</t>
+          <t>PB21 · AC3 · EP (3) · test_no_eligible_dose_has_null_rate__AC3 · evidence/test-contract-unit.log/xml</t>
         </is>
       </c>
     </row>
@@ -26638,7 +26664,7 @@
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>2 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+          <t>2 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. Unit; chưa thay bằng chứng API/DB.</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
@@ -26648,11 +26674,11 @@
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC3 · BVA (max+1) · Chuyển trạng thái (missed không trở thành tuân thủ) · test_after_deadline_confirmation_does_not_raise_rate__AC3 · evidence/test-unit.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="90.5" customHeight="1">
+          <t>PB21 · AC3 · BVA (max+1) · Chuyển trạng thái (missed không trở thành tuân thủ) · test_after_deadline_confirmation_does_not_raise_rate__AC3 · evidence/test-contract-unit.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="123.5" customHeight="1">
       <c r="A37" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-29</t>
@@ -26686,7 +26712,7 @@
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
-          <t>2 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+          <t>2 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. Unit; chưa thay bằng chứng API/DB. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
@@ -26696,11 +26722,11 @@
       </c>
       <c r="I37" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC3 · Chuyển trạng thái (đồng bộ muộn) · test_valid_confirmation_synced_after_deadline_still_counts__AC3 · evidence/test-unit.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="140" customHeight="1">
+          <t>PB21 · AC3 · Chuyển trạng thái (đồng bộ muộn) · test_valid_confirmation_synced_after_deadline_still_counts__AC3 · evidence/test-contract-unit.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="156.5" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-30</t>
@@ -26733,19 +26759,23 @@
           <t>Hai kiểu nhóm có tổng 5, counted=5,rate=80; ID thuốc không bị gộp nhầm; no-store, allowed và DB không đổi.</t>
         </is>
       </c>
-      <c r="G38" s="8" t="inlineStr"/>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
+        </is>
+      </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I38" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC1,AC2,AC3 · EP (1) · test_patient_history_by_date_medication_groups_and_80_percent · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="123.5" customHeight="1">
+          <t>PB21 · AC1,AC2,AC3 · EP (1) · test_patient_history_by_date_medication_groups_and_80_percent · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="156.5" customHeight="1">
       <c r="A39" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-31</t>
@@ -26778,19 +26808,23 @@
           <t>Nhóm theo ngày scheduled_at ở Việt Nam, thứ tự ngày đúng, không nhân đôi liều.</t>
         </is>
       </c>
-      <c r="G39" s="8" t="inlineStr"/>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
+        </is>
+      </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I39" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC2 · BVA (ngày) · test_scheduled_date_across_midnight · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="57.5" customHeight="1">
+          <t>PB21 · AC2 · BVA (ngày) · test_scheduled_date_across_midnight · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="74" customHeight="1">
       <c r="A40" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-32</t>
@@ -26823,7 +26857,7 @@
       </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
-          <t>1 ca tự động pass trong phiên; các assertion của ca được thực thi. Bằng chứng: evidence/test-unit.log.</t>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. Unit; chưa thay bằng chứng API/DB.</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
@@ -26833,11 +26867,11 @@
       </c>
       <c r="I40" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC2 · BVA (max,max+1) · test_inclusive_90_allowed_91_rejected · evidence/test-unit.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="140" customHeight="1">
+          <t>PB21 · AC2 · BVA (max,max+1) · test_inclusive_90_allowed_91_rejected · evidence/test-contract-unit.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="156.5" customHeight="1">
       <c r="A41" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-33</t>
@@ -26869,19 +26903,23 @@
           <t>Một dose_log và một occurrence; giữ xác nhận hợp lệ; lịch sử phản ánh liều trễ.</t>
         </is>
       </c>
-      <c r="G41" s="8" t="inlineStr"/>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>1 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
+        </is>
+      </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I41" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC2,AC3 · Đoán lỗi (idempotency) · test_late_sync_worker_log_and_retry_keep_one_occurrence · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="123.5" customHeight="1">
+          <t>PB21 · AC2,AC3 · Đoán lỗi (idempotency) · test_late_sync_worker_log_and_retry_keep_one_occurrence · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="156.5" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-34</t>
@@ -26913,19 +26951,23 @@
           <t>Một occurrence/dose_log; uong_tre; không ghi đè xác nhận hợp lệ.</t>
         </is>
       </c>
-      <c r="G42" s="8" t="inlineStr"/>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>2 ca Pass trong lần chạy sau khôi phục contract, 25/10/2026. FastAPI TestClient + PostgreSQL local thật; đã vượt assertion contract và kiểm hiệu ứng DB/audit của test. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
+        </is>
+      </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I42" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC2,AC3 · Đoán lỗi (race) · test_worker_insert_races_with_valid_late_confirmation · evidence/test-history.log · Pending: test dừng tại schema adherence thiếu trong contract; chưa chạy hết các assertion hành vi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="107" customHeight="1">
+          <t>PB21 · AC2,AC3 · Đoán lỗi (race) · test_worker_insert_races_with_valid_late_confirmation · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="222.5" customHeight="1">
       <c r="A43" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-35</t>
@@ -26938,59 +26980,65 @@
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
+          <t>Supabase local; patient P có health_data và lịch schedule_id=S ngày 19/10/2026 lúc 08:00 +07; chưa có dose_log cho occurrence; đồng hồ test cố định sau taken_at; dùng bearer của P để xác nhận, không dùng family F.</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>1. Ghi số dose_logs của (S, 2026-10-19T08:00:00+07:00) trước khi gọi API.
+2. POST /doses/batch bằng bearer P với JSON array gồm một item: client_uuid=UUID v4 mới, schedule_id=S, scheduled_at=2026-10-19T08:00:00+07:00, taken_at=2026-10-19T07:29:59.999999+07:00.
+3. Kiểm item bị từ chối theo cửa sổ QD-03; đối chiếu response với contract chuẩn khi có.
+4. Đọc DB: không có xác nhận hợp lệ mới, số dose_logs của occurrence không tăng. GET lịch sử một mình không thay thế thao tác POST xác nhận này.</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>scheduled=08:00; taken=07:29:59.999999 +07</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>Bị từ chối theo cửa sổ xác nhận QD-03; không tạo xác nhận hợp lệ.</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>Hai cách nhóm date/medication Pass trên API/DB thật. POST batch trả 200, item failed=1/taken_at_too_early; không tạo dose_log; family GET trả lịch sử rỗng, audit allowed. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC2,AC3 · BVA (min-1) · test_family_confirmation_adjacent_boundaries__AC2_AC3[before-early-window] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="173" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-36</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm biên ngay trước +30 phút</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
           <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
         </is>
       </c>
-      <c r="D43" s="8" t="inlineStr">
+      <c r="D44" s="8" t="inlineStr">
         <is>
           <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
-2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
-3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>scheduled=08:00; taken=07:29:59.999999 +07</t>
-        </is>
-      </c>
-      <c r="F43" s="8" t="inlineStr">
-        <is>
-          <t>Bị từ chối theo cửa sổ xác nhận QD-03; không tạo xác nhận hợp lệ.</t>
-        </is>
-      </c>
-      <c r="G43" s="8" t="inlineStr"/>
-      <c r="H43" s="7" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="I43" s="8" t="inlineStr">
-        <is>
-          <t>PB21 · AC2,AC3 · BVA (min-1) · Pending: Chưa có ca 3.25 chạy biên này; thiếu contract 3.23 để bổ sung integration theo P5.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="107" customHeight="1">
-      <c r="A44" s="7" t="inlineStr">
-        <is>
-          <t>TC-FADH-36</t>
-        </is>
-      </c>
-      <c r="B44" s="7" t="inlineStr">
-        <is>
-          <t>Kiểm biên ngay trước +30 phút</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>DB Supabase local reset sạch; dùng fixture history_data; patient P có health_data; family F liên kết active, sharing=true và family_sharing của P còn hiệu lực.</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>1. Tạo patient/family và lịch 08:00 qua fixture history_data.
-2. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
-3. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
+2. Dùng bearer P POST /doses/batch: client_uuid mới, schedule_id=S, scheduled_at=08:00, taken_at=08:29:59.999999 +07; đồng hồ test bằng taken_at; kiểm item synced/da_uong.
+3. Gọi GET /adherence?patient_id=P&amp;from=2026-10-19&amp;to=2026-10-19 bằng app session của F.
+4. Đối chiếu response, dose_logs và access_logs bằng assertion của test nêu ở Comments.</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
@@ -27003,15 +27051,19 @@
           <t>da_uong; tỷ lệ có liều hợp lệ ngay khi xác nhận.</t>
         </is>
       </c>
-      <c r="G44" s="8" t="inlineStr"/>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>Hai cách nhóm date/medication Pass trên API/DB thật. POST xác nhận 08:29:59.999999 hợp lệ; family GET có một da_uong, counted=1/rate=100 ngay, audit allowed; GET không đổi dose_log. Lượt P7 chạy lại toàn backend integration: nhóm history API/PEP 66 Pass/2 Fail, TC20 vẫn Fail ở hai grouping; các ca khác trong nhóm này giữ kết quả. evidence/test-p7-integration.log/xml.</t>
+        </is>
+      </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I44" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC2,AC3 · BVA (+30-1) · Pending: Chưa chạy đúng mốc này trong bộ 3.25; chưa đủ điều kiện mở rộng P5.</t>
+          <t>PB21 · AC2,AC3 · BVA (+30-1) · test_family_confirmation_adjacent_boundaries__AC2_AC3[before-on-time-deadline] · evidence/test-contract-history-final.log/xml · Retest evidence/test-p7-integration.log/xml</t>
         </is>
       </c>
     </row>
@@ -27057,7 +27109,7 @@
       </c>
       <c r="I45" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC8 · Chuyển trạng thái (đối soát) · Pending: Contract thiếu /adherence và schema; dữ liệu/field đối soát chưa được đặc tả; không tạo oracle giả.</t>
+          <t>PB21 · AC8 · Chuyển trạng thái (đối soát) · Pending: dữ liệu/field đối soát chưa được đặc tả; không tạo oracle giả.</t>
         </is>
       </c>
     </row>
@@ -27102,11 +27154,11 @@
       </c>
       <c r="I46" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC8 · EP (2,3) · Pending: Contract hiện chưa biểu diễn tỷ lệ riêng; không suy ra công thức.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="90.5" customHeight="1">
+          <t>PB21 · AC8 · EP (2,3) · Pending: Contract /adherence đã khôi phục nhưng chưa biểu diễn tỷ lệ đúng giờ riêng; không suy ra công thức.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="239" customHeight="1">
       <c r="A47" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-39</t>
@@ -27119,7 +27171,7 @@
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>Cần màn production 3.24; family F đã mở lịch sử P.</t>
+          <t>Thiết bị Android test package riêng; production UI 3.24 đã có; family F đã mở lịch sử P bằng local API/DB.</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
@@ -27148,11 +27200,11 @@
       </c>
       <c r="I47" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC6 · Chuyển trạng thái (session) · manual · Pending: UI/controller/repository 3.24 chưa có, chỉ .gitkeep; chưa chạy app hoặc widget test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="90.5" customHeight="1">
+          <t>PB21 · AC6 · Chuyển trạng thái (session) · manual · Pending: Android emulator-5580 đã chạy production route với local API/DB thật: linked Pass, revoke hai lần Pass, cross_patient Pass; chưa kiểm thao tác selector UI chính và cache bền. Lượt đầu revoke có handshake Fail chưa xác định nguyên nhân, giữ log đỏ. evidence/test-p7-android.log; evidence/test-p7-android-revoke-diagnostic.log; evidence/test-p7-android-final.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="189.5" customHeight="1">
       <c r="A48" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-40</t>
@@ -27165,40 +27217,46 @@
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>Cần màn production 3.24; family F đã mở lịch sử P.</t>
+          <t>Widget test production FamilyAdherenceScreen/DrugTimeApp; repository cấp fixture thuốc giả; đã kiểm Thuốc A hiện trước trigger. Không phải Android/API thật.</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
         <is>
-          <t>1. Mở app test và chọn P trong Người thân.
-2. Mở lịch sử, xác nhận có liều.
-3. Thực hiện mất mạng.
-4. Kiểm không hiển thị dữ liệu cũ, không lưu bền, response cũ không phục hồi dữ liệu.</t>
+          <t>1. Chạy family_adherence_screen_test.dart bằng flutter test.
+2. Load lịch sử, kiểm Thuốc A đang hiện.
+3. Emit false qua ConnectivityMonitor do app đăng ký; pump UI.
+4. Kiểm không còn text Thuốc A, kể cả offstage.
+5. Emit true để online lại; kiểm có request mới và chưa hiện dữ liệu cũ.
+6. Hoàn tất request mới bằng denied; kiểm thông báo Không còn quyền xem lịch sử.</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t>P có liều 08:00; Q không có dữ liệu của P; sự kiện=mất mạng</t>
+          <t>Fixture thuốc giả Thuốc A; ngày VN hiện tại của route app.</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>Dữ liệu sức khỏe cũ bị xóa khỏi RAM/UI; không có cache bền; không phục hồi bởi response đến muộn.</t>
-        </is>
-      </c>
-      <c r="G48" s="8" t="inlineStr"/>
+          <t>Sau mất mạng, dữ liệu sức khỏe cũ biến mất ngay khỏi UI, kể cả offstage.</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>Pass trên frontend 46275fa: offline xóa toàn bộ Text Thuốc A kể cả offstage; online lại tạo GET mới, chưa hiển thị dữ liệu cũ; phản hồi denied hiện Không còn quyền xem lịch sử. Widget test, chưa xác minh lifecycle Android/API thật.</t>
+        </is>
+      </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I48" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC6 · Chuyển trạng thái (session) · manual · Pending: UI/controller/repository 3.24 chưa có, chỉ .gitkeep; chưa chạy app hoặc widget test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="90.5" customHeight="1">
+          <t>PB21 · AC6 · Chuyển trạng thái (session) · unit/widget · AC6 QD-29: offline removes health data · BUG-3.25-02 đã xác nhận fix ở widget; native OS Pending · evidence/test-bug02-family-mobile.jsonl</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="255.5" customHeight="1">
       <c r="A49" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-41</t>
@@ -27211,40 +27269,47 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Cần màn production 3.24; family F đã mở lịch sử P.</t>
+          <t>Widget test production FamilyAdherenceScreen/DrugTimeApp; repository cấp fixture thuốc giả; đã kiểm Thuốc A hiện trước trigger. Không phải Android/API thật.</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>1. Mở app test và chọn P trong Người thân.
-2. Mở lịch sử, xác nhận có liều.
-3. Thực hiện đưa app vào nền.
-4. Kiểm không hiển thị dữ liệu cũ, không lưu bền, response cũ không phục hồi dữ liệu.</t>
+          <t>1. Chạy family_adherence_screen_test.dart bằng flutter test.
+2. Load lịch sử, kiểm Thuốc A đang hiện.
+3. Phát inactive → hidden → paused rồi pump một frame.
+4. Kiểm không còn text Thuốc A, kể cả offstage.
+5. Resume để bắt đầu request mới, đưa app về paused và hoàn tất response cũ; kiểm không có Thuốc A.
+6. Refresh trong paused; kiểm không phát sinh GET.
+7. Resume lần nữa; kiểm có request mới, trả denied và kiểm thông báo Không còn quyền xem lịch sử.</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>P có liều 08:00; Q không có dữ liệu của P; sự kiện=đưa app vào nền</t>
+          <t>Fixture thuốc giả Thuốc A; screen clock 22/10/2026; lifecycle inactive/hidden/paused.</t>
         </is>
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t>Dữ liệu sức khỏe cũ bị xóa khỏi RAM/UI; không có cache bền; không phục hồi bởi response đến muộn.</t>
-        </is>
-      </c>
-      <c r="G49" s="8" t="inlineStr"/>
+          <t>Sau vào nền, dữ liệu sức khỏe cũ biến mất ngay khỏi UI, kể cả offstage.</t>
+        </is>
+      </c>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>Pass trên frontend 46275fa: inactive/hidden/paused xóa toàn bộ Text Thuốc A kể cả offstage; response thành công tới muộn không khôi phục dữ liệu; refresh khi paused không gọi thêm GET; resumed gọi lại và denied không hiện dữ liệu cũ. Widget test, chưa xác minh lifecycle Android thật.</t>
+        </is>
+      </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I49" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC6 · Chuyển trạng thái (session) · manual · Pending: UI/controller/repository 3.24 chưa có, chỉ .gitkeep; chưa chạy app hoặc widget test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="90.5" customHeight="1">
+          <t>PB21 · AC6 · Chuyển trạng thái (session) · unit/widget · AC6 QD-29: background removes health data · BUG-3.25-02 đã xác nhận fix ở widget; native OS Pending · evidence/test-bug02-family-mobile.jsonl</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="222.5" customHeight="1">
       <c r="A50" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-42</t>
@@ -27257,7 +27322,7 @@
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>Cần màn production 3.24; family F đã mở lịch sử P.</t>
+          <t>Thiết bị Android test package riêng; production UI 3.24 đã có; family F đã mở lịch sử P bằng local API/DB.</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
@@ -27286,11 +27351,11 @@
       </c>
       <c r="I50" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC6 · Chuyển trạng thái (session) · manual · Pending: UI/controller/repository 3.24 chưa có, chỉ .gitkeep; chưa chạy app hoặc widget test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="90.5" customHeight="1">
+          <t>PB21 · AC6 · Chuyển trạng thái (session) · manual · Pending: Android emulator-5580 đã chạy production route với local API/DB thật: linked Pass, revoke hai lần Pass, cross_patient Pass; chưa kiểm logout trên Android. Lượt đầu revoke có handshake Fail chưa xác định nguyên nhân, giữ log đỏ. evidence/test-p7-android.log; evidence/test-p7-android-revoke-diagnostic.log; evidence/test-p7-android-final.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="255.5" customHeight="1">
       <c r="A51" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-43</t>
@@ -27303,7 +27368,7 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>Cần màn production 3.24; family F đã mở lịch sử P.</t>
+          <t>Thiết bị Android test package riêng; production UI 3.24 đã có; family F đã mở lịch sử P bằng local API/DB.</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
@@ -27332,11 +27397,11 @@
       </c>
       <c r="I51" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC6 · Chuyển trạng thái (session) · manual · Pending: UI/controller/repository 3.24 chưa có, chỉ .gitkeep; chưa chạy app hoặc widget test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="90.5" customHeight="1">
+          <t>PB21 · AC6 · Chuyển trạng thái (session) · manual · Pending: Android emulator-5580 đã chạy production route với local API/DB thật: linked Pass, revoke hai lần Pass, cross_patient Pass; đã kiểm 403 trên route; chưa kiểm toàn bộ cache bền/response tới muộn trên thiết bị. Lượt đầu revoke có handshake Fail chưa xác định nguyên nhân, giữ log đỏ. evidence/test-p7-android.log; evidence/test-p7-android-revoke-diagnostic.log; evidence/test-p7-android-final.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="255.5" customHeight="1">
       <c r="A52" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-44</t>
@@ -27377,11 +27442,11 @@
       </c>
       <c r="I52" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC1,AC4,AC5,AC6 · manual/E2E · Pending: Không có màn production hoặc Flutter integration test 3.24; chưa viết/chạy runner thay màn giả.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="156.5" customHeight="1">
+          <t>PB21 · AC1,AC4,AC5,AC6 · manual/E2E · Pending: Android emulator-5580 đã chạy production route với local API/DB thật: linked Pass, revoke hai lần Pass, cross_patient Pass; đã kiểm route read-only/revoke/cross-patient; chưa kiểm chọn patient từ UI chính. Lượt đầu revoke có handshake Fail chưa xác định nguyên nhân, giữ log đỏ. evidence/test-p7-android.log; evidence/test-p7-android-revoke-diagnostic.log; evidence/test-p7-android-final.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="206" customHeight="1">
       <c r="A53" s="7" t="inlineStr">
         <is>
           <t>TC-FADH-45</t>
@@ -27416,7 +27481,7 @@
       </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t>Đã đối chiếu AC1–AC9, log/XML phiên hiện tại, validate/build/merge exit 0. Kiểm giữ nguyên 20 sheet chức năng, đúng 45 ID và một bug FADH; các ca thiếu bằng chứng giữ Pending. evidence/testcase-verify.log; evidence/testcase-xlsx.log; 05-test-report.md. Scope cuối exit 0 sau commit riêng unit implement được người dùng cho phép; chưa kiểm native Excel.</t>
+          <t>Đối chiếu evidence P7: history integration 66 Pass/2 Fail; 19 host-runner unit Pass; ba scenario host HTTP/PEP/DB đạt; Android linked Pass, revoke hai lần Pass và cross_patient Pass. Lượt đầu revoke handshake Fail chưa rõ nguyên nhân được giữ riêng. Giữ 53 ID với 46 Pass/1 Fail/6 Pending; dựng/gộp bằng script chuẩn, 20 sheet khác giữ nguyên. Không nghiệm thu toàn PB21/OS/selector/AC8. evidence/test-p7-final-verify.log; evidence/test-p7-android-final.log.</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
@@ -27426,65 +27491,457 @@
       </c>
       <c r="I53" s="8" t="inlineStr">
         <is>
-          <t>PB21 · AC9 · manual (đối chiếu artifact) · evidence/testcase-verify.log · evidence/testcase-xlsx.log</t>
-        </is>
-      </c>
-    </row>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56">
-      <c r="G56" s="12" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="H56" s="13">
-        <f>COUNTIF(H9:H53,"Pass")</f>
+          <t>PB21 · AC9 · manual (đối chiếu artifact) · evidence/test-contract-workbook-verify.log · evidence/test-contract-testcase-xlsx.log · Lượt P7 evidence/test-p7-final-verify.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="189.5" customHeight="1">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-46</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Gọi lại GET với patient và bearer hiện tại sau từ chối; không trả cache khi lỗi mạng</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>Production repository/controller/widget ở frontend b24ee68; unit/widget dùng mock HTTP/repository và fixture thuốc giả, không chứng minh DB/Android.</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy flutter test --no-pub --reporter json; lọc file family_adherence_* tại test/features/family.
+2. Mock HTTP: GET thành công, GET 403 rồi GET lại với bearer mới; nhánh khác thành công rồi ném ClientException.
+3. Đối chiếu assertion và testDone của đúng test, không tính file adherence cùng tên.</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Mock HTTP: GET thành công, GET 403 rồi GET lại với bearer mới; nhánh khác thành công rồi ném ClientException.</t>
+        </is>
+      </c>
+      <c r="F54" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lần fetch gửi GET mới với patient_id/date/group_by và bearer hiện tại; 403/network truyền failure, không trả lịch sử cũ.</t>
+        </is>
+      </c>
+      <c r="G54" s="8" t="inlineStr">
+        <is>
+          <t>2 test Pass trong phiên 25/10/2026; AC4: refetches the selected patient and current bearer after a denial; AC6: a network failure after success never returns cached history. evidence/test-contract-mobile.jsonl. Đã chạy lại nhóm 16 test trong lượt cập nhật contract: 14 Pass/2 Fail; evidence/test-contract-mobile.jsonl. Retest frontend 46275fa: nhóm family history 17 Pass/0 Fail/0 Skip; evidence/test-bug02-family-mobile.jsonl.</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I54" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC4,AC6 · Đoán lỗi/Chuyển trạng thái · unit/widget · evidence/test-contract-mobile.jsonl · Retest evidence/test-bug02-family-mobile.jsonl</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="189.5" customHeight="1">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-47</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Từ chối response thuộc patient khác ở repository và controller</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>Production repository/controller/widget ở frontend b24ee68; unit/widget dùng mock HTTP/repository và fixture thuốc giả, không chứng minh DB/Android.</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy flutter test --no-pub --reporter json; lọc file family_adherence_* tại test/features/family.
+2. Request Q nhưng HTTP/reader cấp response P; UUID P và Q khác nhau.
+3. Đối chiếu assertion và testDone của đúng test, không tính file adherence cùng tên.</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Request Q nhưng HTTP/reader cấp response P; UUID P và Q khác nhau.</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>Repository ném invalidResponse; controller không giữ history P.</t>
+        </is>
+      </c>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>2 test Pass trong phiên 25/10/2026; AC4: a response for P cannot satisfy a request for Q; AC4: the controller also rejects a mismatched patient from its reader. evidence/test-contract-mobile.jsonl. Đã chạy lại nhóm 16 test trong lượt cập nhật contract: 14 Pass/2 Fail; evidence/test-contract-mobile.jsonl. Retest frontend 46275fa: nhóm family history 17 Pass/0 Fail/0 Skip; evidence/test-bug02-family-mobile.jsonl.</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I55" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC4,AC6 · Đoán lỗi/Chuyển trạng thái · unit/widget · evidence/test-contract-mobile.jsonl · Retest evidence/test-bug02-family-mobile.jsonl</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="305" customHeight="1">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-48</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Hủy response cũ khi refresh, đổi patient hoặc clear controller</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>Production repository/controller/widget ở frontend b24ee68; unit/widget dùng mock HTTP/repository và fixture thuốc giả, không chứng minh DB/Android.</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy flutter test --no-pub --reporter json; lọc file family_adherence_* tại test/features/family.
+2. Completer điều khiển thứ tự: load P; hai refresh cạnh tranh hoặc đổi sang Q hoặc clear; hoàn tất response cũ sau failure/response mới.
+3. Đối chiếu assertion và testDone của đúng test, không tính file adherence cùng tên.</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Completer điều khiển thứ tự: load P; hai refresh cạnh tranh hoặc đổi sang Q hoặc clear; hoàn tất response cũ sau failure/response mới.</t>
+        </is>
+      </c>
+      <c r="F56" s="8" t="inlineStr">
+        <is>
+          <t>history bị clear ngay; denied/network/unauthorized đúng failure; response cũ không phục hồi dữ liệu; clear không tự fetch.</t>
+        </is>
+      </c>
+      <c r="G56" s="8" t="inlineStr">
+        <is>
+          <t>5 test Pass trong phiên 25/10/2026; AC6: refresh clears RAM before AdherenceFailureKind.denied and accepts no stale success; AC6: refresh clears RAM before AdherenceFailureKind.network and accepts no stale success; AC6: refresh clears RAM before AdherenceFailureKind.unauthorized and accepts no stale success; AC6: switching patient clears visible history and rejects the old result; AC6: clear invalidates an in-flight read without an automatic refetch. evidence/test-contract-mobile.jsonl. Đã chạy lại nhóm 16 test trong lượt cập nhật contract: 14 Pass/2 Fail; evidence/test-contract-mobile.jsonl. Retest frontend 46275fa: nhóm family history 17 Pass/0 Fail/0 Skip; evidence/test-bug02-family-mobile.jsonl.</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I56" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC6 · Đoán lỗi/Chuyển trạng thái · unit/widget · evidence/test-contract-mobile.jsonl · Retest evidence/test-bug02-family-mobile.jsonl</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="222.5" customHeight="1">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>TC-FADH-49</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Xóa dữ liệu widget khi đổi patient hoặc refresh gặp 403/network</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>Production repository/controller/widget ở frontend b24ee68; unit/widget dùng mock HTTP/repository và fixture thuốc giả, không chứng minh DB/Android.</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy flutter test --no-pub --reporter json; lọc file family_adherence_* tại test/features/family.
+2. Widget production đã load Thuốc A; đổi patientId sang Q hoặc refresh rồi trả denied/network.
+3. Đối chiếu assertion và testDone của đúng test, không tính file adherence cùng tên.</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Widget production đã load Thuốc A; đổi patientId sang Q hoặc refresh rồi trả denied/network.</t>
+        </is>
+      </c>
+      <c r="F57" s="8" t="inlineStr">
+        <is>
+          <t>Không còn Thuốc A trước khi Q hoàn tất hoặc ngay khi refresh; hiện thông báo lỗi tương ứng, không giữ dữ liệu P.</t>
+        </is>
+      </c>
+      <c r="G57" s="8" t="inlineStr">
+        <is>
+          <t>3 test Pass trong phiên 25/10/2026; AC6: changing to Q removes P before the Q read completes; AC6: refresh AdherenceFailureKind.denied clears the previously displayed patient; AC6: refresh AdherenceFailureKind.network clears the previously displayed patient. evidence/test-contract-mobile.jsonl. Đã chạy lại nhóm 16 test trong lượt cập nhật contract: 14 Pass/2 Fail; evidence/test-contract-mobile.jsonl. Retest frontend 46275fa: nhóm family history 17 Pass/0 Fail/0 Skip; evidence/test-bug02-family-mobile.jsonl.</t>
+        </is>
+      </c>
+      <c r="H57" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I57" s="8" t="inlineStr">
+        <is>
+          <t>PB21 · AC6 · Đoán lỗi/Chuyển trạng thái · unit/widget · evidence/test-contract-mobile.jsonl · Retest evidence/test-bug02-family-mobile.jsonl</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="156.5" customHeight="1">
+      <c r="A58" s="7" t="inlineSt